<commit_message>
🔪 Slice france_travail 2026-07-10
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseFranceTravail" displayName="BaseFranceTravail" ref="A1:W17" headerRowCount="1">
-  <autoFilter ref="A1:W17"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseFranceTravail" displayName="BaseFranceTravail" ref="A1:W27" headerRowCount="1">
+  <autoFilter ref="A1:W27"/>
   <tableColumns count="23">
     <tableColumn id="1" name="zone"/>
     <tableColumn id="2" name="formation"/>
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5">
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W17"/>
+  <dimension ref="A1:W27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -577,7 +577,7 @@
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
-    <col width="31" customWidth="1" min="9" max="9"/>
+    <col width="35" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="17" customWidth="1" min="12" max="12"/>
@@ -714,17 +714,17 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Préparation au concours d'adjoint administratif d'État principal de 2ème classe</t>
+          <t>Titre professionnel secrétaire assistant médico-administratif (FOAD)</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school)</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Durée de 335 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 1084 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>foad@skillandyou.com</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>foad@skillandyou.com</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -774,15 +774,19 @@
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>0146006878</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>0146006878</t>
-        </is>
-      </c>
-      <c r="O2" s="5" t="inlineStr"/>
+          <t>0180888030</t>
+        </is>
+      </c>
+      <c r="O2" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -796,18 +800,22 @@
       <c r="R2" s="5" t="inlineStr"/>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>Votre intégration - Guide d'intégration - Bienvenue dans votre formation - Guide Métier Adjoint administratif d'État principal de 2ème classe - Guide de la formation - Guide des épreuves - Le concours d'adjoint administratif d'État principal de 2ème classe Aide à la réalisation de vos documents professionnels Compléter votre livret de suivi des compétences professionnelles Retranscrire et ordonner les idées principales d'un texte Annales corrigées Épreuves blanches Solliciter les connaissances fondamentales pour le concours Comprendre l'administration française Comprendre le fonctionnement des institutions françaises Acquérir des connaissances en français Acquérir une bonne culture générale Mathématiques Les tests d'aptitudes verbales Annales corrigées Épreuves blanches Mobiliser les compétences professionnelles de l'adjoint administratif d'État Bureautique Épreuves blanches Techniques et recherche d'emploi/stage Sensibilisation au développement durable | Organisme | Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school) | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T2" s="5" t="inlineStr"/>
+          <t>7 projets professionnalisants vous permettront d'acquérir les compétences citées au dessus par la pratique.Vous réaliserez les projets suivants :P1 - Démarrez votre formation de secrétaire assistant médico-administratifP2 - Niveau 1 : Maîtrisez l'accueil et la gestion administrative en milieu médicalP3 - Niveau 2 : Développez vos compétences en rédaction, communication et outils numériques en milieuP4 - Réalisez votre mission en entrepriseP5 - Niveau 3 : Optimisez l'organisation, la sécuritéet la gestion des données sensibles en milieu médicalP6 - Niveau 4 : Améliorez la gestion des communications, données et environnements sanitairesP7 - Préparez votre fin de formation de secrétaire assistant médico-administratif | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel secrétaire assistant médico-administratif</t>
+        </is>
+      </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11205913/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/true</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -819,17 +827,17 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Certification CLOE français langue étrangère - spécialité hôtellerie Restauration niveau A2 vers B1 (FOAD)</t>
+          <t>Formation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Nepsod Evolution</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
@@ -844,7 +852,7 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Durée de 331 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 346 heures</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -859,12 +867,12 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>accueil@nepsod.com</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>accueil@nepsod.com</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
@@ -879,19 +887,15 @@
       </c>
       <c r="M3" s="7" t="inlineStr">
         <is>
-          <t>0474639587</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr">
         <is>
-          <t>0474639587</t>
-        </is>
-      </c>
-      <c r="O3" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0180888030</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="inlineStr"/>
       <c r="P3" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -905,22 +909,18 @@
       <c r="R3" s="7" t="inlineStr"/>
       <c r="S3" s="7" t="inlineStr">
         <is>
-          <t>Accueil et initiation à la formation (1h30) - Module FLE visée insertion professionnelle : chercher un emploi, présenter son métier, présenter ses projets, interagir avec ses collègues, manipuler les outils numériques (120h30) - Module FOS Hôtellerie Restauration :découvrir la cuisine, travailler en cuisine, identifier les besoins d'un client, présenter des produits et services, gérer les réclamations (50h) Module environnement social et culturel : vie quotidienne et relations sociales, loisirs, patrimoine, citoyenneté et engagement (43h) Module Préparation et recherche de stage en entreprise (14h) Période de stage en entreprise (35 h) Module remise à niveau numérique (35 h maximum) Module accompagnement à l'après-formation (21h maximum) Module Préparation et passage de la certification CLOE (10h) Bilan final (1h) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T3" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Certification CLOE français langue étrangère</t>
-        </is>
-      </c>
+          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T3" s="7" t="inlineStr"/>
       <c r="U3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11576792/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/true</t>
         </is>
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,32 +932,32 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière) - DEI</t>
+          <t>Concours d'atsem (FOAD)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -972,12 +972,12 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -992,48 +992,40 @@
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr"/>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q4" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R4" s="5" t="inlineStr"/>
       <c r="S4" s="5" t="inlineStr">
         <is>
-          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail (bureautique,recherche documentaire, rédaction de documents écrits, communication, anglais) La formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de1 800h, sous la forme de cours magistraux (750 h) travaux dirigés (1 050 h) le travail personnel guidé (suivi pédagogique, temps personnel guidé, supervision, travaux entre étudiants- 300 h) la formation clinique de 2 100 h le travail personnel complémentaire est estimé à 900 heures environ, soit 300 h par an. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T4" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
-        </is>
-      </c>
+          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr"/>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11533526/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
         </is>
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1045,32 +1037,32 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État de technicien de laboratoire médical</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Association des Fondateurs et Protecteurs de l'Institut Catholique de Lyon (AFPICL) (UCLy - Institut Catholique de Lyon)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>69002 Lyon 2e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>10 place des Archives | 69002 Lyon 2e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1120 heures</t>
+          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1085,12 +1077,12 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>fp@univ-catholyon.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>fp@univ-catholyon.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
@@ -1105,12 +1097,12 @@
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>0472325134</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>0472325134</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="O5" s="7" t="inlineStr">
@@ -1120,29 +1112,33 @@
       </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R5" s="7" t="inlineStr"/>
-      <c r="S5" s="7" t="inlineStr"/>
+      <c r="S5" s="7" t="inlineStr">
+        <is>
+          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État de technicien de laboratoire médical</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11026378/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
         </is>
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1154,32 +1150,32 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'ambulancier</t>
+          <t>Préparation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+          <t>AFEC (Siège)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Durée de 801 heures (dont 245 heures en entreprise)</t>
+          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -1194,12 +1190,12 @@
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -1214,48 +1210,40 @@
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>0472117903</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>0472117903</t>
-        </is>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0153368844</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr"/>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R6" s="5" t="inlineStr"/>
       <c r="S6" s="5" t="inlineStr">
         <is>
-          <t>Non renseigne | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T6" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'ambulancier</t>
-        </is>
-      </c>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC (Siège) | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr"/>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11871421/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1267,32 +1255,32 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Agent de prévention et de sécurité - Titre à finalité professionnelle (TFP APS)</t>
+          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Global pro formation (Global pro formation (GPF))</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Blue Concept | 16 Rue Marcel Dutartre | 69100 Villeurbanne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Durée de 379 heures (dont 70 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1307,12 +1295,12 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>globalproformation@gmail.com</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>globalproformation@gmail.com</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
@@ -1327,19 +1315,15 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>0666139535</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>0666139535</t>
-        </is>
-      </c>
-      <c r="O7" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -1347,28 +1331,24 @@
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr"/>
       <c r="S7" s="7" t="inlineStr">
         <is>
-          <t>Théorie : SST : Protéger, Examiner (saignement, étouffement, conscience et respiration) et alerter (alerte et message d'accueil) La déontologie de l'agent de sécurité Les services publics de police et gendarmerie, le CNAPS Le cadre légal de la profession, le code pénal et le code de procédure pénale La sûreté de l'État Les armes Mise en sûreté et neutralisation des armes Prévention et actes terrorisme L'accueil, le contrôle d'accès, le contrôle visuel et la palpation de sécurité La prise en compte d'un poste de contrôle de sécurité et les consignes La protection du travailleur Isolé Le circuit de vérification La gestion des alarmes intrusion et incendie, la vidéo et la télésurveillance (surveillance et gardiennage) Les techniques d'information, de communication et la gestion des conflits L'incendie et les risques majeurs Le risque électrique (initiation) Le cadre légal et la problématique de l'activité d'événementiel La définition du terrorisme (historique, mécanisme, méthodologie et modes opératoires) Les différentes menaces terroristes et les niveaux de risque associés La prévention des actes de terrorisme par la reconnaissance des comportements suspects (profiling) et de la radicalisation violente L'action en cas d'attaque et suivant le type d'attaque (actes réflexes, mesures de mise en sécurité immédiate) Le combat en dernier recours L'alerte et la facilitation de l'intervention des forces de l'ordre La sécurisation d'une zone dans l'urgence, risque de sur-attentat et post-attentat. Pratique : Mise en pratique SST CQP APS: Code de la sécurité intérieure Code pénal et libertés publiques Déontologie professionnelle Secours à personnes (SST) Situations conflictuelles et résolution de conflit Consignes, compte rendu et rapport Gestion des risques majeurs, électriques, incendie Gestion d'alarmes Technique d'information et de communication Préparation d'une mission Gestion de conflit Contrôle d'accès Poste de contrôle de sécurité Rondes Palpation de sécurité et inspection de bagages Télésurveillance et vidéo protection Sensibilisation aux risques terroristes Examen : en cours de formation UV 1 (secourisme) : le candidat sera déclaré apte ou inapte en fonction des résultats de la grille d'évaluation conforme aux procédures de validation de l'INRS. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
-        </is>
-      </c>
-      <c r="T7" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Agent de prévention et de sécurité</t>
-        </is>
-      </c>
+          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T7" s="7" t="inlineStr"/>
       <c r="U7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11870188/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
         </is>
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1380,32 +1360,32 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'Etat de la Jeunesse de l'Education Populaire et du Sport spécialité "animation socio-éducative ou culturelle mention "coordination de projets" - RNCP 39930 spécialité "animation socio-éducative ou culturel mention "coordination de projets</t>
+          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -1415,17 +1395,17 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>https://arfatsema.catalogueformpro.com/3/dejeps-17/2857880/diplome-detat-de-la-jeunesse-de-leducation-populaire-et-du-sport-dejeps-17-specialite-animation-soci/registration?session_id=2846144</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1440,48 +1420,40 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>0478031711</t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr"/>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q8" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>BC1: Animer et accompagner une équipe dans le champ du sport ou de l'animation Animer une équipe en structure d'éducation populaire : enjeux éthiques, valeurs et spécificités Réaliser un diagnostic des ressources humaines de son périmètre d'intervention Animer une équipe en structure d'éducation populaire : organisation, cadre légal, réglementation et procédures Diversité et inclusion : analyser les besoins et mettre en place une organisation adaptée Management participatif : développer le pouvoir d'agir d'une équipe Management participatif : outils et pratiques Accompagner une équipe: médiation et gestion de conflits Accompagner une équipe : émancipation et développement de l'autonomie Dynamique de groupe Animer un processus démocratique Projet d'action formative et conception de séance formative Droit du travail/Droit social Communication non violente Outils d'animation collective Outils d'accompagnement individuel Accompagner la vulnérabilité Dialogue social et syndical Responsabilité du coordinateur Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? BC2: Concevoir un projet d'action dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Education Populaire Rapport de domination Le numérique comme un fait social Esprit critique Culture politique Démocratie et contre pouvoir Pouvoir d'agir ou devoir d'agir? Diagnostic et enjeux De l'attribution d'une place à une culture de la participation Famille et éducation Connaissance des institutions publics et relation aux association ingéniérie sociale Portrait de territoire Mesure de l'impact social BC3 : Mettre en oeuvre et évaluer un projet d'action Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie de projet Mesure de l'impact social Accompagner la vulnérabilité La protection de l'Enfance en France Outils participatifs Intelligence artificielle et fonction de coordination BC4 : Développer les partenariats opérationnelles et contribuer aux dynamiques institutionnelles dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Connaissance des institutions publics et relation aux associations Démocratie et contre pouvoir Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie sociale Outils participatifs | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T8" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | DEJEPS spécialité animation socio-éducative ou culturelle mention coordination de projets</t>
-        </is>
-      </c>
+          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880827/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
         </is>
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1493,32 +1465,32 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Créez votre vignoble bio de raisin de table, rentable et résilient - Devenez autonome pour produire et vendre votre propre raisin de table bio</t>
+          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>SARL Agri-learn éditions</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>69001 Lyon</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 69001 Lyon | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Durée de 9 heures</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1533,12 +1505,12 @@
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
@@ -1553,18 +1525,18 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="O9" s="7" t="inlineStr"/>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q9" s="7" t="inlineStr">
@@ -1575,18 +1547,18 @@
       <c r="R9" s="7" t="inlineStr"/>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>1. Taille de la vigne Principes de taille (formation et production) Techniques de taille douce Entretien et corrections2. Modes de conduite Choix du système (lyre, gable, plan vertical. Comparaison des conduites Adaptation au contexte pédoclimatique3. Fertilité des sols Gestion du sol (travail / non-travail) Irrigation Maintien de la fertilité en bio4. Travaux du vignoble Protection contre maladies et ravageurs Calendrier des interventions Conduite sous abri (tunnel)5. Choix des plants Sélection des variétés Choix du porte-greffe Adaptation au marché et au terroir6. Plantation Préparation du sol Étapes de plantation Coûts et organisation7. Récolte et commercialisation Récolte et conservation Organisation du travail Valorisation et vente8. Protection du vignoble en bio Biocontrôle et PNPP Réduction des intrants Stratégies alternatives9. Gestion des maladies et ravageurs Identification des principaux risques Prévention et lutte adaptée10. Pilotage des traitements Stratégie cuivre / soufre Optimisation des doses11. Approche agroécologique Biodiversité fonctionnelle Variétés résistantes | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr"/>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11870193/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/true</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1598,32 +1570,32 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
+          <t>BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>UCPA Formation</t>
+          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>69200 Vénissieux</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>16 Avenue Dr Georges Levy | 69200 Vénissieux | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1267 heures (dont 637 heures en entreprise)</t>
+          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1638,12 +1610,12 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>ucpa-formation@ucpa.asso.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>ucpa-formation@ucpa.asso.fr | fgehant@ucpa.asso.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr | cecile.iribarne@educagri.fr</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1658,12 +1630,12 @@
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>0642833617</t>
+          <t>0479264427</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>0642833617</t>
+          <t>0479264427</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -1673,33 +1645,33 @@
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q10" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>Unité capitalisable (UC) - 1. Encadrer tout public dans tout lieu et toute structureUnité capitalisable (UC) - 2. Mettre en œuvre un projet d'animation s'inscrivant dans le projet de la structureUnité capitalisable (UC) - 3. Conduire une séance, un cycle d'animation ou d'apprentissage dans le champ des activités aquatiques et de la natationUnité capitalisable (UC) - 4. Mobiliser les techniques des activités aquatiques et de la natation pour mettre en œuvre une séance ou un cycle d'apprentissage | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11447001/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/true</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1711,32 +1683,32 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'aide-soignant - DEAS</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1540 heures (dont 770 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1746,17 +1718,17 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=aide-soignant</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1771,12 +1743,12 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="O11" s="7" t="inlineStr">
@@ -1786,33 +1758,33 @@
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>La formation conduisant au diplôme d'État d'aide-soignant, 17 semaines d'enseignement théoriques organisées autour de 8 modules : Accompagnement d'une personne dans les activités de la vie quotidienne L'état clinique d'une personne Les soins Ergonomie Relation Communication Hygiène des locaux hospitaliers Transmission des informations Organisation du travail Les titulaires du DE d'auxiliaire de puériculture, du DE d'aide médico-psychologique, du DE d'auxiliaire de vie sociale ou de la MC aide à domicile, sont dispensés de certaines unités de formation. La formation comprend également 6 stages d'une durée totale de 24 semaines en milieu hospitalier ou extra-hospitalier. Possibilité d'effectuer la formation en initial ou en apprentissage. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'aide-soignant</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11533549/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1829,27 +1801,27 @@
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>Préparation au concours d'adjoint administratif d'État principal de 2ème classe</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+          <t>Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 335 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1864,12 +1836,12 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>foad@skillandyou.com</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>foad@skillandyou.com</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1884,44 +1856,40 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>0472117979</t>
+          <t>0146006878</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>0472117979</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0146006878</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr"/>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q12" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R12" s="5" t="inlineStr"/>
-      <c r="S12" s="5" t="inlineStr"/>
-      <c r="T12" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
-        </is>
-      </c>
+      <c r="S12" s="5" t="inlineStr">
+        <is>
+          <t>Votre intégration - Guide d'intégration - Bienvenue dans votre formation - Guide Métier Adjoint administratif d'État principal de 2ème classe - Guide de la formation - Guide des épreuves - Le concours d'adjoint administratif d'État principal de 2ème classe Aide à la réalisation de vos documents professionnels Compléter votre livret de suivi des compétences professionnelles Retranscrire et ordonner les idées principales d'un texte Annales corrigées Épreuves blanches Solliciter les connaissances fondamentales pour le concours Comprendre l'administration française Comprendre le fonctionnement des institutions françaises Acquérir des connaissances en français Acquérir une bonne culture générale Mathématiques Les tests d'aptitudes verbales Annales corrigées Épreuves blanches Mobiliser les compétences professionnelles de l'adjoint administratif d'État Bureautique Épreuves blanches Techniques et recherche d'emploi/stage Sensibilisation au développement durable | Organisme | Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school) | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr"/>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11817055/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11205913/true/false/true/true</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -1938,27 +1906,27 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'assistant de service social - DE ASS</t>
+          <t>Certification CLOE français langue étrangère - spécialité hôtellerie Restauration niveau A2 vers B1 (FOAD)</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Nepsod Evolution</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 avenue Lacassagne | Croix Rouge francaise | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Durée de 3420 heures (dont 1680 heures en entreprise)</t>
+          <t>Durée de 331 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1968,17 +1936,17 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=assistant%20de%20service%20social</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>accueil@nepsod.com</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>accueil@nepsod.com</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
@@ -1993,12 +1961,12 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0474639587</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0474639587</t>
         </is>
       </c>
       <c r="O13" s="7" t="inlineStr">
@@ -2008,29 +1976,33 @@
       </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R13" s="7" t="inlineStr"/>
-      <c r="S13" s="7" t="inlineStr"/>
+      <c r="S13" s="7" t="inlineStr">
+        <is>
+          <t>Accueil et initiation à la formation (1h30) - Module FLE visée insertion professionnelle : chercher un emploi, présenter son métier, présenter ses projets, interagir avec ses collègues, manipuler les outils numériques (120h30) - Module FOS Hôtellerie Restauration :découvrir la cuisine, travailler en cuisine, identifier les besoins d'un client, présenter des produits et services, gérer les réclamations (50h) Module environnement social et culturel : vie quotidienne et relations sociales, loisirs, patrimoine, citoyenneté et engagement (43h) Module Préparation et recherche de stage en entreprise (14h) Période de stage en entreprise (35 h) Module remise à niveau numérique (35 h maximum) Module accompagnement à l'après-formation (21h maximum) Module Préparation et passage de la certification CLOE (10h) Bilan final (1h) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Certification CLOE français langue étrangère</t>
         </is>
       </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11672249/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11576792/true/false/true/false</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W13" s="7" t="inlineStr">
@@ -2047,27 +2019,27 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'éducateur spécialisé</t>
+          <t>Diplôme d'État d'infirmier(ière) - DEI</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales (ARFRIPS - Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales)</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>69009 Lyon 9e</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>10 Impasse Pierre Baizet | 69009 Lyon 9e | France</t>
+          <t>115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Durée de 3442 heures (dont 1925 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -2082,12 +2054,12 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>info@arfrips.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>info@arfrips.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -2102,12 +2074,12 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>0478699090</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>0478699090</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -2126,15 +2098,19 @@
         </is>
       </c>
       <c r="R14" s="5" t="inlineStr"/>
-      <c r="S14" s="5" t="inlineStr"/>
+      <c r="S14" s="5" t="inlineStr">
+        <is>
+          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail (bureautique,recherche documentaire, rédaction de documents écrits, communication, anglais) La formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de1 800h, sous la forme de cours magistraux (750 h) travaux dirigés (1 050 h) le travail personnel guidé (suivi pédagogique, temps personnel guidé, supervision, travaux entre étudiants- 300 h) la formation clinique de 2 100 h le travail personnel complémentaire est estimé à 900 heures environ, soit 300 h par an. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur spécialisé</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11737248/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11533526/true/false/false/false</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
@@ -2156,27 +2132,27 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet - RNCP 39931 - spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+          <t>Diplôme d'État de technicien de laboratoire médical</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+          <t>Association des Fondateurs et Protecteurs de l'Institut Catholique de Lyon (AFPICL) (UCLy - Institut Catholique de Lyon)</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>69002 Lyon 2e</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+          <t>10 place des Archives | 69002 Lyon 2e | France</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 1120 heures</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2186,17 +2162,17 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>https://arfatsema.catalogueformpro.com/2/desjeps-17/2858060/desjeps-17-diplome-detat-superieur-de-la-jeunesse-de-leducation-populaire-et-du-sport-specialite-ani</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>fp@univ-catholyon.fr</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>fp@univ-catholyon.fr</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -2211,12 +2187,12 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0472325134</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0472325134</t>
         </is>
       </c>
       <c r="O15" s="7" t="inlineStr">
@@ -2226,7 +2202,7 @@
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q15" s="7" t="inlineStr">
@@ -2235,19 +2211,15 @@
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr"/>
-      <c r="S15" s="7" t="inlineStr">
-        <is>
-          <t>BC1 : Construire, avec les instances de gouvernance, la stratégie de développement d'une structure dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Éducation Populaire Culture Politique Rapport de domination Pouvoir d'Agir et Vulnérabilité Esprit critique Transformation social/rapport sociaux Le numérique comme un fait social Nouvel esprit du capitalisme Laicité et valeurs de la République Violence sexiste violences sexuelles Ingénierie social en lien avec la structure Réaliser un diagnostic RH et financier Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Elaboration de la stratégie de développement en lien avec les instances de gouvernance Animer un processus démocratique Démocratie et contre pouvoir BC2 : Concevoir et diriger un projet de développement de la structure Cartographie des relations et l'environnement de son association Ingénierie du projet Processus d'évaluation dans une démarche partagée et participative Outils participatifs Outils de communication Utilité sociale BC3 : Manager l'équipe et gérer les ressources humaines ( et la démarche Qualité, Sécurité, Santé au Travail et Environnement d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Gestion des ressources humaines en structures d'éducation populaire : enjeux, éthique et complexités associative Articulation employeur bénévole - direction dans la gestion des ressources humaines : définition d'une politique RH et organisation des délégations de pouvoir Gérer l'équipe au quotidien : accompagnement, régulation et gestion conflits Analyse des pratiques en co-développement Développer le pouvoir d'agir des salariés Attractivité, recrutement, intégration et fidélisation des salariés Diversité, inclusion et égalité professionnelle au sein de son organisation Assurer la GPEC, la formation et la gestion des carrières dans un alignement éthique Le financement de la formation professionnelle Qualité de vie Santé sécurité au travail Droit du travail/Droit social Dialogue social/dialogue syndical Cadre général des RPS Démarche prévention et outils BC4 : Assurer la gestion financière, matérielle et administrative d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Comprendre les fondamentaux de la situation financière Initiation à l'analyse financière associative ou de structure d'intérêt général Identifier les leviers de financement Construire des scénarios budgétaires et faire des arbitrages Élaborer un plan d'action financier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
+      <c r="S15" s="7" t="inlineStr"/>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État de technicien de laboratoire médical</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880835/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11026378/true/false/false/false</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
@@ -2269,27 +2241,27 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Créer sa ferme en circuit court : transformation, commercialisation et communication</t>
+          <t>Diplôme d'État d'ambulancier</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>SARL Agri-learn éditions</t>
+          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>69001 Lyon</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 69001 Lyon | France</t>
+          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Durée de 20 heures</t>
+          <t>Durée de 801 heures (dont 245 heures en entreprise)</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2304,12 +2276,12 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -2324,40 +2296,48 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0472117903</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>0620021214</t>
-        </is>
-      </c>
-      <c r="O16" s="5" t="inlineStr"/>
+          <t>0472117903</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P16" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q16" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R16" s="5" t="inlineStr"/>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>Cette formation s'appuie sur plusieurs compétences essentielles : Stratégie commerciale et étude de marché : définir son offre, ses volumes, ses prix et ses circuits de vente Techniques de vente : maîtriser les étapes clés pour convaincre et fidéliser les clients Transformation des produits agricoles : valoriser ses matières premières pour créer de la valeur ajoutée Hygiène et réglementation : garantir la sécurité sanitaire dans les ateliers de transformation Communication et prospection : développer sa clientèle et promouvoir ses produits Valorisation des produits : savoir parler de ses produits et les mettre en avant (ex : dégustation) L'ensemble permet d'acquérir une vision globale du fonctionnement d'une ferme en circuit court, de la production jusqu'à la vente. 3 heures de visio avec les experts sont prévues dans le cursus. | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T16" s="5" t="inlineStr"/>
+          <t>Non renseigne | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T16" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'ambulancier</t>
+        </is>
+      </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880868/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11871421/true/false/false/false</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
         </is>
       </c>
       <c r="W16" s="5" t="inlineStr">
@@ -2374,27 +2354,27 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Titre professionnel administrateur d'infrastructures sécurisées (FOAD)</t>
+          <t>Agent de prévention et de sécurité - Titre à finalité professionnelle (TFP APS)</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>STUDI</t>
+          <t>Global pro formation (Global pro formation (GPF))</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>69100 Villeurbanne</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Blue Concept | 16 Rue Marcel Dutartre | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Durée de 947 heures (dont 350 heures en entreprise)</t>
+          <t>Durée de 379 heures (dont 70 heures en entreprise)</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2409,12 +2389,12 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>contact@studi.fr</t>
+          <t>globalproformation@gmail.com</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>contact@studi.fr | conseiller-formation.aoft@studi.fr</t>
+          <t>globalproformation@gmail.com</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -2429,12 +2409,12 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>0174888555</t>
+          <t>0666139535</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>0174888555</t>
+          <t>0666139535</t>
         </is>
       </c>
       <c r="O17" s="7" t="inlineStr">
@@ -2449,31 +2429,1133 @@
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="7" t="inlineStr">
         <is>
+          <t>Théorie : SST : Protéger, Examiner (saignement, étouffement, conscience et respiration) et alerter (alerte et message d'accueil) La déontologie de l'agent de sécurité Les services publics de police et gendarmerie, le CNAPS Le cadre légal de la profession, le code pénal et le code de procédure pénale La sûreté de l'État Les armes Mise en sûreté et neutralisation des armes Prévention et actes terrorisme L'accueil, le contrôle d'accès, le contrôle visuel et la palpation de sécurité La prise en compte d'un poste de contrôle de sécurité et les consignes La protection du travailleur Isolé Le circuit de vérification La gestion des alarmes intrusion et incendie, la vidéo et la télésurveillance (surveillance et gardiennage) Les techniques d'information, de communication et la gestion des conflits L'incendie et les risques majeurs Le risque électrique (initiation) Le cadre légal et la problématique de l'activité d'événementiel La définition du terrorisme (historique, mécanisme, méthodologie et modes opératoires) Les différentes menaces terroristes et les niveaux de risque associés La prévention des actes de terrorisme par la reconnaissance des comportements suspects (profiling) et de la radicalisation violente L'action en cas d'attaque et suivant le type d'attaque (actes réflexes, mesures de mise en sécurité immédiate) Le combat en dernier recours L'alerte et la facilitation de l'intervention des forces de l'ordre La sécurisation d'une zone dans l'urgence, risque de sur-attentat et post-attentat. Pratique : Mise en pratique SST CQP APS: Code de la sécurité intérieure Code pénal et libertés publiques Déontologie professionnelle Secours à personnes (SST) Situations conflictuelles et résolution de conflit Consignes, compte rendu et rapport Gestion des risques majeurs, électriques, incendie Gestion d'alarmes Technique d'information et de communication Préparation d'une mission Gestion de conflit Contrôle d'accès Poste de contrôle de sécurité Rondes Palpation de sécurité et inspection de bagages Télésurveillance et vidéo protection Sensibilisation aux risques terroristes Examen : en cours de formation UV 1 (secourisme) : le candidat sera déclaré apte ou inapte en fonction des résultats de la grille d'évaluation conforme aux procédures de validation de l'INRS. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
+        </is>
+      </c>
+      <c r="T17" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Agent de prévention et de sécurité</t>
+        </is>
+      </c>
+      <c r="U17" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11870188/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V17" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W17" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Diplôme d'Etat de la Jeunesse de l'Education Populaire et du Sport spécialité "animation socio-éducative ou culturelle mention "coordination de projets" - RNCP 39930 spécialité "animation socio-éducative ou culturel mention "coordination de projets</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>69100 Villeurbanne</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>https://arfatsema.catalogueformpro.com/3/dejeps-17/2857880/diplome-detat-de-la-jeunesse-de-leducation-populaire-et-du-sport-dejeps-17-specialite-animation-soci/registration?session_id=2846144</t>
+        </is>
+      </c>
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>arfatsema.direction@orange.fr</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>arfatsema.direction@orange.fr</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M18" s="5" t="inlineStr">
+        <is>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R18" s="5" t="inlineStr"/>
+      <c r="S18" s="5" t="inlineStr">
+        <is>
+          <t>BC1: Animer et accompagner une équipe dans le champ du sport ou de l'animation Animer une équipe en structure d'éducation populaire : enjeux éthiques, valeurs et spécificités Réaliser un diagnostic des ressources humaines de son périmètre d'intervention Animer une équipe en structure d'éducation populaire : organisation, cadre légal, réglementation et procédures Diversité et inclusion : analyser les besoins et mettre en place une organisation adaptée Management participatif : développer le pouvoir d'agir d'une équipe Management participatif : outils et pratiques Accompagner une équipe: médiation et gestion de conflits Accompagner une équipe : émancipation et développement de l'autonomie Dynamique de groupe Animer un processus démocratique Projet d'action formative et conception de séance formative Droit du travail/Droit social Communication non violente Outils d'animation collective Outils d'accompagnement individuel Accompagner la vulnérabilité Dialogue social et syndical Responsabilité du coordinateur Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? BC2: Concevoir un projet d'action dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Education Populaire Rapport de domination Le numérique comme un fait social Esprit critique Culture politique Démocratie et contre pouvoir Pouvoir d'agir ou devoir d'agir? Diagnostic et enjeux De l'attribution d'une place à une culture de la participation Famille et éducation Connaissance des institutions publics et relation aux association ingéniérie sociale Portrait de territoire Mesure de l'impact social BC3 : Mettre en oeuvre et évaluer un projet d'action Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie de projet Mesure de l'impact social Accompagner la vulnérabilité La protection de l'Enfance en France Outils participatifs Intelligence artificielle et fonction de coordination BC4 : Développer les partenariats opérationnelles et contribuer aux dynamiques institutionnelles dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Connaissance des institutions publics et relation aux associations Démocratie et contre pouvoir Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie sociale Outils participatifs | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T18" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | DEJEPS spécialité animation socio-éducative ou culturelle mention coordination de projets</t>
+        </is>
+      </c>
+      <c r="U18" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11880827/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V18" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W18" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Créez votre vignoble bio de raisin de table, rentable et résilient - Devenez autonome pour produire et vendre votre propre raisin de table bio</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>SARL Agri-learn éditions</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>69001 Lyon</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Formation a distance | 69001 Lyon | France</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 9 heures</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>fanny@agrilearn.fr</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>fanny@agrilearn.fr</t>
+        </is>
+      </c>
+      <c r="K19" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="inlineStr">
+        <is>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="N19" s="7" t="inlineStr">
+        <is>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr"/>
+      <c r="P19" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+        </is>
+      </c>
+      <c r="Q19" s="7" t="inlineStr">
+        <is>
+          <t>À distance</t>
+        </is>
+      </c>
+      <c r="R19" s="7" t="inlineStr"/>
+      <c r="S19" s="7" t="inlineStr">
+        <is>
+          <t>1. Taille de la vigne Principes de taille (formation et production) Techniques de taille douce Entretien et corrections2. Modes de conduite Choix du système (lyre, gable, plan vertical. Comparaison des conduites Adaptation au contexte pédoclimatique3. Fertilité des sols Gestion du sol (travail / non-travail) Irrigation Maintien de la fertilité en bio4. Travaux du vignoble Protection contre maladies et ravageurs Calendrier des interventions Conduite sous abri (tunnel)5. Choix des plants Sélection des variétés Choix du porte-greffe Adaptation au marché et au terroir6. Plantation Préparation du sol Étapes de plantation Coûts et organisation7. Récolte et commercialisation Récolte et conservation Organisation du travail Valorisation et vente8. Protection du vignoble en bio Biocontrôle et PNPP Réduction des intrants Stratégies alternatives9. Gestion des maladies et ravageurs Identification des principaux risques Prévention et lutte adaptée10. Pilotage des traitements Stratégie cuivre / soufre Optimisation des doses11. Approche agroécologique Biodiversité fonctionnelle Variétés résistantes | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T19" s="7" t="inlineStr"/>
+      <c r="U19" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11870193/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V19" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W19" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>UCPA Formation</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>69200 Vénissieux</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>16 Avenue Dr Georges Levy | 69200 Vénissieux | France</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 1267 heures (dont 637 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>ucpa-formation@ucpa.asso.fr</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>ucpa-formation@ucpa.asso.fr | fgehant@ucpa.asso.fr</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>0642833617</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>0642833617</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="inlineStr"/>
+      <c r="S20" s="5" t="inlineStr">
+        <is>
+          <t>Unité capitalisable (UC) - 1. Encadrer tout public dans tout lieu et toute structureUnité capitalisable (UC) - 2. Mettre en œuvre un projet d'animation s'inscrivant dans le projet de la structureUnité capitalisable (UC) - 3. Conduire une séance, un cycle d'animation ou d'apprentissage dans le champ des activités aquatiques et de la natationUnité capitalisable (UC) - 4. Mobiliser les techniques des activités aquatiques et de la natation pour mettre en œuvre une séance ou un cycle d'apprentissage | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T20" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
+        </is>
+      </c>
+      <c r="U20" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11447001/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V20" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W20" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Diplôme d'État d'aide-soignant - DEAS</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>69003 Lyon 3e</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 1540 heures (dont 770 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=aide-soignant</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>competence.ara@croix-rouge.fr</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+        </is>
+      </c>
+      <c r="K21" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>0472115560</t>
+        </is>
+      </c>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>0472115560</t>
+        </is>
+      </c>
+      <c r="O21" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P21" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q21" s="7" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R21" s="7" t="inlineStr"/>
+      <c r="S21" s="7" t="inlineStr">
+        <is>
+          <t>La formation conduisant au diplôme d'État d'aide-soignant, 17 semaines d'enseignement théoriques organisées autour de 8 modules : Accompagnement d'une personne dans les activités de la vie quotidienne L'état clinique d'une personne Les soins Ergonomie Relation Communication Hygiène des locaux hospitaliers Transmission des informations Organisation du travail Les titulaires du DE d'auxiliaire de puériculture, du DE d'aide médico-psychologique, du DE d'auxiliaire de vie sociale ou de la MC aide à domicile, sont dispensés de certaines unités de formation. La formation comprend également 6 stages d'une durée totale de 24 semaines en milieu hospitalier ou extra-hospitalier. Possibilité d'effectuer la formation en initial ou en apprentissage. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T21" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'aide-soignant</t>
+        </is>
+      </c>
+      <c r="U21" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11533549/true/false/false/true</t>
+        </is>
+      </c>
+      <c r="V21" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W21" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Diplôme d'État d'infirmier(ière)</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>69003 Lyon 3e</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>magaly.lebrat@chu-lyon.fr</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>magaly.lebrat@chu-lyon.fr</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>0472117979</t>
+        </is>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>0472117979</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P22" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q22" s="5" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R22" s="5" t="inlineStr"/>
+      <c r="S22" s="5" t="inlineStr"/>
+      <c r="T22" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+        </is>
+      </c>
+      <c r="U22" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11817055/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V22" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W22" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Diplôme d'État d'assistant de service social - DE ASS</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>69003 Lyon 3e</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 avenue Lacassagne | Croix Rouge francaise | 69003 Lyon 3e | France</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 3420 heures (dont 1680 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=assistant%20de%20service%20social</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>competence.ara@croix-rouge.fr</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+        </is>
+      </c>
+      <c r="K23" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L23" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>0472115560</t>
+        </is>
+      </c>
+      <c r="N23" s="7" t="inlineStr">
+        <is>
+          <t>0472115560</t>
+        </is>
+      </c>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P23" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q23" s="7" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R23" s="7" t="inlineStr"/>
+      <c r="S23" s="7" t="inlineStr"/>
+      <c r="T23" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
+        </is>
+      </c>
+      <c r="U23" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11672249/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V23" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W23" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Diplôme d'État d'éducateur spécialisé</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales (ARFRIPS - Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales)</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>69009 Lyon 9e</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>10 Impasse Pierre Baizet | 69009 Lyon 9e | France</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 3442 heures (dont 1925 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>info@arfrips.fr</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>info@arfrips.fr</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>0478699090</t>
+        </is>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>0478699090</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P24" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="inlineStr"/>
+      <c r="S24" s="5" t="inlineStr"/>
+      <c r="T24" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur spécialisé</t>
+        </is>
+      </c>
+      <c r="U24" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11737248/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V24" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W24" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet - RNCP 39931 - spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>69100 Villeurbanne</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>https://arfatsema.catalogueformpro.com/2/desjeps-17/2858060/desjeps-17-diplome-detat-superieur-de-la-jeunesse-de-leducation-populaire-et-du-sport-specialite-ani</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>arfatsema.direction@orange.fr</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>arfatsema.direction@orange.fr</t>
+        </is>
+      </c>
+      <c r="K25" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L25" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M25" s="7" t="inlineStr">
+        <is>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="N25" s="7" t="inlineStr">
+        <is>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="O25" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P25" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+        </is>
+      </c>
+      <c r="Q25" s="7" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R25" s="7" t="inlineStr"/>
+      <c r="S25" s="7" t="inlineStr">
+        <is>
+          <t>BC1 : Construire, avec les instances de gouvernance, la stratégie de développement d'une structure dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Éducation Populaire Culture Politique Rapport de domination Pouvoir d'Agir et Vulnérabilité Esprit critique Transformation social/rapport sociaux Le numérique comme un fait social Nouvel esprit du capitalisme Laicité et valeurs de la République Violence sexiste violences sexuelles Ingénierie social en lien avec la structure Réaliser un diagnostic RH et financier Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Elaboration de la stratégie de développement en lien avec les instances de gouvernance Animer un processus démocratique Démocratie et contre pouvoir BC2 : Concevoir et diriger un projet de développement de la structure Cartographie des relations et l'environnement de son association Ingénierie du projet Processus d'évaluation dans une démarche partagée et participative Outils participatifs Outils de communication Utilité sociale BC3 : Manager l'équipe et gérer les ressources humaines ( et la démarche Qualité, Sécurité, Santé au Travail et Environnement d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Gestion des ressources humaines en structures d'éducation populaire : enjeux, éthique et complexités associative Articulation employeur bénévole - direction dans la gestion des ressources humaines : définition d'une politique RH et organisation des délégations de pouvoir Gérer l'équipe au quotidien : accompagnement, régulation et gestion conflits Analyse des pratiques en co-développement Développer le pouvoir d'agir des salariés Attractivité, recrutement, intégration et fidélisation des salariés Diversité, inclusion et égalité professionnelle au sein de son organisation Assurer la GPEC, la formation et la gestion des carrières dans un alignement éthique Le financement de la formation professionnelle Qualité de vie Santé sécurité au travail Droit du travail/Droit social Dialogue social/dialogue syndical Cadre général des RPS Démarche prévention et outils BC4 : Assurer la gestion financière, matérielle et administrative d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Comprendre les fondamentaux de la situation financière Initiation à l'analyse financière associative ou de structure d'intérêt général Identifier les leviers de financement Construire des scénarios budgétaires et faire des arbitrages Élaborer un plan d'action financier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T25" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+        </is>
+      </c>
+      <c r="U25" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11880835/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V25" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W25" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Créer sa ferme en circuit court : transformation, commercialisation et communication</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>SARL Agri-learn éditions</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>69001 Lyon</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Formation a distance | 69001 Lyon | France</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 20 heures</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>fanny@agrilearn.fr</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>fanny@agrilearn.fr</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="O26" s="5" t="inlineStr"/>
+      <c r="P26" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+        </is>
+      </c>
+      <c r="Q26" s="5" t="inlineStr">
+        <is>
+          <t>À distance</t>
+        </is>
+      </c>
+      <c r="R26" s="5" t="inlineStr"/>
+      <c r="S26" s="5" t="inlineStr">
+        <is>
+          <t>Cette formation s'appuie sur plusieurs compétences essentielles : Stratégie commerciale et étude de marché : définir son offre, ses volumes, ses prix et ses circuits de vente Techniques de vente : maîtriser les étapes clés pour convaincre et fidéliser les clients Transformation des produits agricoles : valoriser ses matières premières pour créer de la valeur ajoutée Hygiène et réglementation : garantir la sécurité sanitaire dans les ateliers de transformation Communication et prospection : développer sa clientèle et promouvoir ses produits Valorisation des produits : savoir parler de ses produits et les mettre en avant (ex : dégustation) L'ensemble permet d'acquérir une vision globale du fonctionnement d'une ferme en circuit court, de la production jusqu'à la vente. 3 heures de visio avec les experts sont prévues dans le cursus. | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T26" s="5" t="inlineStr"/>
+      <c r="U26" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11880868/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V26" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W26" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Titre professionnel administrateur d'infrastructures sécurisées (FOAD)</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>STUDI</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>75004 Paris</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Formation a distance | 75004 Paris | France</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 947 heures (dont 350 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>contact@studi.fr</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>contact@studi.fr | conseiller-formation.aoft@studi.fr</t>
+        </is>
+      </c>
+      <c r="K27" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L27" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M27" s="7" t="inlineStr">
+        <is>
+          <t>0174888555</t>
+        </is>
+      </c>
+      <c r="N27" s="7" t="inlineStr">
+        <is>
+          <t>0174888555</t>
+        </is>
+      </c>
+      <c r="O27" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P27" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par France Travail</t>
+        </is>
+      </c>
+      <c r="Q27" s="7" t="inlineStr">
+        <is>
+          <t>À distance</t>
+        </is>
+      </c>
+      <c r="R27" s="7" t="inlineStr"/>
+      <c r="S27" s="7" t="inlineStr">
+        <is>
           <t>Administrer et sécuriser les infrastructures Les bonnes pratiques dans l'administration des infrastructures Utiliser un logiciel de gestion centralisé : GLPI Configurer le routage Administrer et sécuriser le réseau Automatiser les tâches d'administration Administrer et sécuriser les systèmes Les bases des serveurs virtualisés Administrer et sécuriser une infrastructure de serveurs virtualisée Gérer des containersConcevoir et mettre en œuvre une solution en réponse à un besoin d'évolution Les bases des solutions techniques Proposer une solution informatique répondant à des besoins nouveaux Mettre en production des évolutions de l'infrastructure Les bases de la supervision Superviser la disponibilité de l'infrastructure et en présenter les résultats Mesurer les performances et la disponibilité de l'infrastructureParticiper à la gestion de la cybersécurité Les bases de la cybersécurité Participer à la mesure et à l'analyse du niveau de sécurité de l'infrastructure Participer à l'élaboration et à la mise en œuvre de la politique de sécurité Participer à la détection et au traitement des incidents de sécurité | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
-      <c r="T17" s="7" t="inlineStr">
+      <c r="T27" s="7" t="inlineStr">
         <is>
           <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel administrateur d'infrastructures sécurisées</t>
         </is>
       </c>
-      <c r="U17" s="7" t="inlineStr">
+      <c r="U27" s="7" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/detail/11590088/true/false/true/false</t>
         </is>
       </c>
-      <c r="V17" s="7" t="inlineStr">
+      <c r="V27" s="7" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
-      <c r="W17" s="7" t="inlineStr">
+      <c r="W27" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-07-11
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseFranceTravail" displayName="BaseFranceTravail" ref="A1:W27" headerRowCount="1">
-  <autoFilter ref="A1:W27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseFranceTravail" displayName="BaseFranceTravail" ref="A1:W28" headerRowCount="1">
+  <autoFilter ref="A1:W28"/>
   <tableColumns count="23">
     <tableColumn id="1" name="zone"/>
     <tableColumn id="2" name="formation"/>
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W27"/>
+  <dimension ref="A1:W28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1255,7 +1255,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1360,7 +1360,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,32 +1683,32 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>CAP Fleuriste</t>
+          <t>E2C - Ecole de la Deuxième Chance</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>Ecole de la Deuxième Chance Grand Hainaut</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>02140 Vervins</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Ecole de la deuxième chance - site de VERVINS | 3 Place des Anciens Combattants | 02140 Vervins | France</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 1400 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1723,12 +1723,12 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>c.renaud@e2cgrandhainaut.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>c.renaud@e2cgrandhainaut.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1743,48 +1743,40 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0375310010</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O11" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0375310010</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="inlineStr"/>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T11" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
-        </is>
-      </c>
+          <t>Savoir fondamentauxOrientation et démarches professionnelsSocialisation et développement personnelAlternance en entreprise (près de 30% du temps)Des outils pédagogiques de liaison, d'évaluation et de suivi9 mois maximum + 12 mois de suivi post-parcours | Organisme | Ecole de la Deuxième Chance Grand Hainaut | Lieu de la formation | Ecole de la deuxième chance - site de VERVINS</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr"/>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11072382/true/false/false/true</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1796,17 +1788,17 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Préparation au concours d'adjoint administratif d'État principal de 2ème classe</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1821,7 +1813,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Durée de 335 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1836,12 +1828,12 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>foad@skillandyou.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>foad@skillandyou.com</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1856,15 +1848,19 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>0146006878</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>0146006878</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -1878,18 +1874,22 @@
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>Votre intégration - Guide d'intégration - Bienvenue dans votre formation - Guide Métier Adjoint administratif d'État principal de 2ème classe - Guide de la formation - Guide des épreuves - Le concours d'adjoint administratif d'État principal de 2ème classe Aide à la réalisation de vos documents professionnels Compléter votre livret de suivi des compétences professionnelles Retranscrire et ordonner les idées principales d'un texte Annales corrigées Épreuves blanches Solliciter les connaissances fondamentales pour le concours Comprendre l'administration française Comprendre le fonctionnement des institutions françaises Acquérir des connaissances en français Acquérir une bonne culture générale Mathématiques Les tests d'aptitudes verbales Annales corrigées Épreuves blanches Mobiliser les compétences professionnelles de l'adjoint administratif d'État Bureautique Épreuves blanches Techniques et recherche d'emploi/stage Sensibilisation au développement durable | Organisme | Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school) | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T12" s="5" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+        </is>
+      </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11205913/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -1906,12 +1906,12 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Certification CLOE français langue étrangère - spécialité hôtellerie Restauration niveau A2 vers B1 (FOAD)</t>
+          <t>Préparation au concours d'adjoint administratif d'État principal de 2ème classe</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Nepsod Evolution</t>
+          <t>Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school)</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Durée de 331 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 335 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1941,12 +1941,12 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>accueil@nepsod.com</t>
+          <t>foad@skillandyou.com</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>accueil@nepsod.com</t>
+          <t>foad@skillandyou.com</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
@@ -1961,19 +1961,15 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>0474639587</t>
+          <t>0146006878</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>0474639587</t>
-        </is>
-      </c>
-      <c r="O13" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0146006878</t>
+        </is>
+      </c>
+      <c r="O13" s="7" t="inlineStr"/>
       <c r="P13" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -1987,17 +1983,13 @@
       <c r="R13" s="7" t="inlineStr"/>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>Accueil et initiation à la formation (1h30) - Module FLE visée insertion professionnelle : chercher un emploi, présenter son métier, présenter ses projets, interagir avec ses collègues, manipuler les outils numériques (120h30) - Module FOS Hôtellerie Restauration :découvrir la cuisine, travailler en cuisine, identifier les besoins d'un client, présenter des produits et services, gérer les réclamations (50h) Module environnement social et culturel : vie quotidienne et relations sociales, loisirs, patrimoine, citoyenneté et engagement (43h) Module Préparation et recherche de stage en entreprise (14h) Période de stage en entreprise (35 h) Module remise à niveau numérique (35 h maximum) Module accompagnement à l'après-formation (21h maximum) Module Préparation et passage de la certification CLOE (10h) Bilan final (1h) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T13" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Certification CLOE français langue étrangère</t>
-        </is>
-      </c>
+          <t>Votre intégration - Guide d'intégration - Bienvenue dans votre formation - Guide Métier Adjoint administratif d'État principal de 2ème classe - Guide de la formation - Guide des épreuves - Le concours d'adjoint administratif d'État principal de 2ème classe Aide à la réalisation de vos documents professionnels Compléter votre livret de suivi des compétences professionnelles Retranscrire et ordonner les idées principales d'un texte Annales corrigées Épreuves blanches Solliciter les connaissances fondamentales pour le concours Comprendre l'administration française Comprendre le fonctionnement des institutions françaises Acquérir des connaissances en français Acquérir une bonne culture générale Mathématiques Les tests d'aptitudes verbales Annales corrigées Épreuves blanches Mobiliser les compétences professionnelles de l'adjoint administratif d'État Bureautique Épreuves blanches Techniques et recherche d'emploi/stage Sensibilisation au développement durable | Organisme | Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school) | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T13" s="7" t="inlineStr"/>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11576792/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11205913/true/false/true/true</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
@@ -2019,27 +2011,27 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière) - DEI</t>
+          <t>Certification CLOE français langue étrangère - spécialité hôtellerie Restauration niveau A2 vers B1 (FOAD)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Nepsod Evolution</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 331 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -2054,12 +2046,12 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>accueil@nepsod.com</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>accueil@nepsod.com</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -2074,12 +2066,12 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0474639587</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0474639587</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -2089,28 +2081,28 @@
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q14" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail (bureautique,recherche documentaire, rédaction de documents écrits, communication, anglais) La formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de1 800h, sous la forme de cours magistraux (750 h) travaux dirigés (1 050 h) le travail personnel guidé (suivi pédagogique, temps personnel guidé, supervision, travaux entre étudiants- 300 h) la formation clinique de 2 100 h le travail personnel complémentaire est estimé à 900 heures environ, soit 300 h par an. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Accueil et initiation à la formation (1h30) - Module FLE visée insertion professionnelle : chercher un emploi, présenter son métier, présenter ses projets, interagir avec ses collègues, manipuler les outils numériques (120h30) - Module FOS Hôtellerie Restauration :découvrir la cuisine, travailler en cuisine, identifier les besoins d'un client, présenter des produits et services, gérer les réclamations (50h) Module environnement social et culturel : vie quotidienne et relations sociales, loisirs, patrimoine, citoyenneté et engagement (43h) Module Préparation et recherche de stage en entreprise (14h) Période de stage en entreprise (35 h) Module remise à niveau numérique (35 h maximum) Module accompagnement à l'après-formation (21h maximum) Module Préparation et passage de la certification CLOE (10h) Bilan final (1h) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Certification CLOE français langue étrangère</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11533526/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11576792/true/false/true/false</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
@@ -2132,27 +2124,27 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État de technicien de laboratoire médical</t>
+          <t>Diplôme d'État d'infirmier(ière) - DEI</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Association des Fondateurs et Protecteurs de l'Institut Catholique de Lyon (AFPICL) (UCLy - Institut Catholique de Lyon)</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>69002 Lyon 2e</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>10 place des Archives | 69002 Lyon 2e | France</t>
+          <t>115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1120 heures</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2167,12 +2159,12 @@
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>fp@univ-catholyon.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>fp@univ-catholyon.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -2187,12 +2179,12 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>0472325134</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>0472325134</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O15" s="7" t="inlineStr">
@@ -2211,15 +2203,19 @@
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr"/>
-      <c r="S15" s="7" t="inlineStr"/>
+      <c r="S15" s="7" t="inlineStr">
+        <is>
+          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail (bureautique,recherche documentaire, rédaction de documents écrits, communication, anglais) La formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de1 800h, sous la forme de cours magistraux (750 h) travaux dirigés (1 050 h) le travail personnel guidé (suivi pédagogique, temps personnel guidé, supervision, travaux entre étudiants- 300 h) la formation clinique de 2 100 h le travail personnel complémentaire est estimé à 900 heures environ, soit 300 h par an. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État de technicien de laboratoire médical</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11026378/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11533526/true/false/false/false</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
@@ -2241,27 +2237,27 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'ambulancier</t>
+          <t>Diplôme d'État de technicien de laboratoire médical</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+          <t>Association des Fondateurs et Protecteurs de l'Institut Catholique de Lyon (AFPICL) (UCLy - Institut Catholique de Lyon)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>69002 Lyon 2e</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+          <t>10 place des Archives | 69002 Lyon 2e | France</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Durée de 801 heures (dont 245 heures en entreprise)</t>
+          <t>Durée de 1120 heures</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2276,12 +2272,12 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>fp@univ-catholyon.fr</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>fp@univ-catholyon.fr</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -2296,12 +2292,12 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>0472117903</t>
+          <t>0472325134</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>0472117903</t>
+          <t>0472325134</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr">
@@ -2320,24 +2316,20 @@
         </is>
       </c>
       <c r="R16" s="5" t="inlineStr"/>
-      <c r="S16" s="5" t="inlineStr">
-        <is>
-          <t>Non renseigne | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
+      <c r="S16" s="5" t="inlineStr"/>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'ambulancier</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État de technicien de laboratoire médical</t>
         </is>
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11871421/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11026378/true/false/false/false</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W16" s="5" t="inlineStr">
@@ -2354,27 +2346,27 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Agent de prévention et de sécurité - Titre à finalité professionnelle (TFP APS)</t>
+          <t>Diplôme d'État d'ambulancier</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Global pro formation (Global pro formation (GPF))</t>
+          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Blue Concept | 16 Rue Marcel Dutartre | 69100 Villeurbanne | France</t>
+          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Durée de 379 heures (dont 70 heures en entreprise)</t>
+          <t>Durée de 801 heures (dont 245 heures en entreprise)</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2389,12 +2381,12 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>globalproformation@gmail.com</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>globalproformation@gmail.com</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -2409,12 +2401,12 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>0666139535</t>
+          <t>0472117903</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>0666139535</t>
+          <t>0472117903</t>
         </is>
       </c>
       <c r="O17" s="7" t="inlineStr">
@@ -2424,7 +2416,7 @@
       </c>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q17" s="7" t="inlineStr">
@@ -2435,22 +2427,22 @@
       <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="7" t="inlineStr">
         <is>
-          <t>Théorie : SST : Protéger, Examiner (saignement, étouffement, conscience et respiration) et alerter (alerte et message d'accueil) La déontologie de l'agent de sécurité Les services publics de police et gendarmerie, le CNAPS Le cadre légal de la profession, le code pénal et le code de procédure pénale La sûreté de l'État Les armes Mise en sûreté et neutralisation des armes Prévention et actes terrorisme L'accueil, le contrôle d'accès, le contrôle visuel et la palpation de sécurité La prise en compte d'un poste de contrôle de sécurité et les consignes La protection du travailleur Isolé Le circuit de vérification La gestion des alarmes intrusion et incendie, la vidéo et la télésurveillance (surveillance et gardiennage) Les techniques d'information, de communication et la gestion des conflits L'incendie et les risques majeurs Le risque électrique (initiation) Le cadre légal et la problématique de l'activité d'événementiel La définition du terrorisme (historique, mécanisme, méthodologie et modes opératoires) Les différentes menaces terroristes et les niveaux de risque associés La prévention des actes de terrorisme par la reconnaissance des comportements suspects (profiling) et de la radicalisation violente L'action en cas d'attaque et suivant le type d'attaque (actes réflexes, mesures de mise en sécurité immédiate) Le combat en dernier recours L'alerte et la facilitation de l'intervention des forces de l'ordre La sécurisation d'une zone dans l'urgence, risque de sur-attentat et post-attentat. Pratique : Mise en pratique SST CQP APS: Code de la sécurité intérieure Code pénal et libertés publiques Déontologie professionnelle Secours à personnes (SST) Situations conflictuelles et résolution de conflit Consignes, compte rendu et rapport Gestion des risques majeurs, électriques, incendie Gestion d'alarmes Technique d'information et de communication Préparation d'une mission Gestion de conflit Contrôle d'accès Poste de contrôle de sécurité Rondes Palpation de sécurité et inspection de bagages Télésurveillance et vidéo protection Sensibilisation aux risques terroristes Examen : en cours de formation UV 1 (secourisme) : le candidat sera déclaré apte ou inapte en fonction des résultats de la grille d'évaluation conforme aux procédures de validation de l'INRS. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
+          <t>Non renseigne | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Agent de prévention et de sécurité</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'ambulancier</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11870188/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11871421/true/false/false/false</t>
         </is>
       </c>
       <c r="V17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
         </is>
       </c>
       <c r="W17" s="7" t="inlineStr">
@@ -2467,12 +2459,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'Etat de la Jeunesse de l'Education Populaire et du Sport spécialité "animation socio-éducative ou culturelle mention "coordination de projets" - RNCP 39930 spécialité "animation socio-éducative ou culturel mention "coordination de projets</t>
+          <t>Agent de prévention et de sécurité - Titre à finalité professionnelle (TFP APS)</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+          <t>Global pro formation (Global pro formation (GPF))</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -2482,12 +2474,12 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+          <t>Blue Concept | 16 Rue Marcel Dutartre | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 379 heures (dont 70 heures en entreprise)</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -2497,17 +2489,17 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>https://arfatsema.catalogueformpro.com/3/dejeps-17/2857880/diplome-detat-de-la-jeunesse-de-leducation-populaire-et-du-sport-dejeps-17-specialite-animation-soci/registration?session_id=2846144</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>globalproformation@gmail.com</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>globalproformation@gmail.com</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -2522,12 +2514,12 @@
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0666139535</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0666139535</t>
         </is>
       </c>
       <c r="O18" s="5" t="inlineStr">
@@ -2537,7 +2529,7 @@
       </c>
       <c r="P18" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q18" s="5" t="inlineStr">
@@ -2548,17 +2540,17 @@
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>BC1: Animer et accompagner une équipe dans le champ du sport ou de l'animation Animer une équipe en structure d'éducation populaire : enjeux éthiques, valeurs et spécificités Réaliser un diagnostic des ressources humaines de son périmètre d'intervention Animer une équipe en structure d'éducation populaire : organisation, cadre légal, réglementation et procédures Diversité et inclusion : analyser les besoins et mettre en place une organisation adaptée Management participatif : développer le pouvoir d'agir d'une équipe Management participatif : outils et pratiques Accompagner une équipe: médiation et gestion de conflits Accompagner une équipe : émancipation et développement de l'autonomie Dynamique de groupe Animer un processus démocratique Projet d'action formative et conception de séance formative Droit du travail/Droit social Communication non violente Outils d'animation collective Outils d'accompagnement individuel Accompagner la vulnérabilité Dialogue social et syndical Responsabilité du coordinateur Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? BC2: Concevoir un projet d'action dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Education Populaire Rapport de domination Le numérique comme un fait social Esprit critique Culture politique Démocratie et contre pouvoir Pouvoir d'agir ou devoir d'agir? Diagnostic et enjeux De l'attribution d'une place à une culture de la participation Famille et éducation Connaissance des institutions publics et relation aux association ingéniérie sociale Portrait de territoire Mesure de l'impact social BC3 : Mettre en oeuvre et évaluer un projet d'action Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie de projet Mesure de l'impact social Accompagner la vulnérabilité La protection de l'Enfance en France Outils participatifs Intelligence artificielle et fonction de coordination BC4 : Développer les partenariats opérationnelles et contribuer aux dynamiques institutionnelles dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Connaissance des institutions publics et relation aux associations Démocratie et contre pouvoir Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie sociale Outils participatifs | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Théorie : SST : Protéger, Examiner (saignement, étouffement, conscience et respiration) et alerter (alerte et message d'accueil) La déontologie de l'agent de sécurité Les services publics de police et gendarmerie, le CNAPS Le cadre légal de la profession, le code pénal et le code de procédure pénale La sûreté de l'État Les armes Mise en sûreté et neutralisation des armes Prévention et actes terrorisme L'accueil, le contrôle d'accès, le contrôle visuel et la palpation de sécurité La prise en compte d'un poste de contrôle de sécurité et les consignes La protection du travailleur Isolé Le circuit de vérification La gestion des alarmes intrusion et incendie, la vidéo et la télésurveillance (surveillance et gardiennage) Les techniques d'information, de communication et la gestion des conflits L'incendie et les risques majeurs Le risque électrique (initiation) Le cadre légal et la problématique de l'activité d'événementiel La définition du terrorisme (historique, mécanisme, méthodologie et modes opératoires) Les différentes menaces terroristes et les niveaux de risque associés La prévention des actes de terrorisme par la reconnaissance des comportements suspects (profiling) et de la radicalisation violente L'action en cas d'attaque et suivant le type d'attaque (actes réflexes, mesures de mise en sécurité immédiate) Le combat en dernier recours L'alerte et la facilitation de l'intervention des forces de l'ordre La sécurisation d'une zone dans l'urgence, risque de sur-attentat et post-attentat. Pratique : Mise en pratique SST CQP APS: Code de la sécurité intérieure Code pénal et libertés publiques Déontologie professionnelle Secours à personnes (SST) Situations conflictuelles et résolution de conflit Consignes, compte rendu et rapport Gestion des risques majeurs, électriques, incendie Gestion d'alarmes Technique d'information et de communication Préparation d'une mission Gestion de conflit Contrôle d'accès Poste de contrôle de sécurité Rondes Palpation de sécurité et inspection de bagages Télésurveillance et vidéo protection Sensibilisation aux risques terroristes Examen : en cours de formation UV 1 (secourisme) : le candidat sera déclaré apte ou inapte en fonction des résultats de la grille d'évaluation conforme aux procédures de validation de l'INRS. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
         </is>
       </c>
       <c r="T18" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | DEJEPS spécialité animation socio-éducative ou culturelle mention coordination de projets</t>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Agent de prévention et de sécurité</t>
         </is>
       </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880827/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11870188/true/false/false/false</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
@@ -2580,27 +2572,27 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Créez votre vignoble bio de raisin de table, rentable et résilient - Devenez autonome pour produire et vendre votre propre raisin de table bio</t>
+          <t>Diplôme d'Etat de la Jeunesse de l'Education Populaire et du Sport spécialité "animation socio-éducative ou culturelle mention "coordination de projets" - RNCP 39930 spécialité "animation socio-éducative ou culturel mention "coordination de projets</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>SARL Agri-learn éditions</t>
+          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>69001 Lyon</t>
+          <t>69100 Villeurbanne</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 69001 Lyon | France</t>
+          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Durée de 9 heures</t>
+          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2610,17 +2602,17 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://arfatsema.catalogueformpro.com/3/dejeps-17/2857880/diplome-detat-de-la-jeunesse-de-leducation-populaire-et-du-sport-dejeps-17-specialite-animation-soci/registration?session_id=2846144</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="K19" s="7" t="inlineStr">
@@ -2635,15 +2627,19 @@
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0478031711</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>0620021214</t>
-        </is>
-      </c>
-      <c r="O19" s="7" t="inlineStr"/>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P19" s="7" t="inlineStr">
         <is>
           <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
@@ -2651,24 +2647,28 @@
       </c>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R19" s="7" t="inlineStr"/>
       <c r="S19" s="7" t="inlineStr">
         <is>
-          <t>1. Taille de la vigne Principes de taille (formation et production) Techniques de taille douce Entretien et corrections2. Modes de conduite Choix du système (lyre, gable, plan vertical. Comparaison des conduites Adaptation au contexte pédoclimatique3. Fertilité des sols Gestion du sol (travail / non-travail) Irrigation Maintien de la fertilité en bio4. Travaux du vignoble Protection contre maladies et ravageurs Calendrier des interventions Conduite sous abri (tunnel)5. Choix des plants Sélection des variétés Choix du porte-greffe Adaptation au marché et au terroir6. Plantation Préparation du sol Étapes de plantation Coûts et organisation7. Récolte et commercialisation Récolte et conservation Organisation du travail Valorisation et vente8. Protection du vignoble en bio Biocontrôle et PNPP Réduction des intrants Stratégies alternatives9. Gestion des maladies et ravageurs Identification des principaux risques Prévention et lutte adaptée10. Pilotage des traitements Stratégie cuivre / soufre Optimisation des doses11. Approche agroécologique Biodiversité fonctionnelle Variétés résistantes | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T19" s="7" t="inlineStr"/>
+          <t>BC1: Animer et accompagner une équipe dans le champ du sport ou de l'animation Animer une équipe en structure d'éducation populaire : enjeux éthiques, valeurs et spécificités Réaliser un diagnostic des ressources humaines de son périmètre d'intervention Animer une équipe en structure d'éducation populaire : organisation, cadre légal, réglementation et procédures Diversité et inclusion : analyser les besoins et mettre en place une organisation adaptée Management participatif : développer le pouvoir d'agir d'une équipe Management participatif : outils et pratiques Accompagner une équipe: médiation et gestion de conflits Accompagner une équipe : émancipation et développement de l'autonomie Dynamique de groupe Animer un processus démocratique Projet d'action formative et conception de séance formative Droit du travail/Droit social Communication non violente Outils d'animation collective Outils d'accompagnement individuel Accompagner la vulnérabilité Dialogue social et syndical Responsabilité du coordinateur Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? BC2: Concevoir un projet d'action dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Education Populaire Rapport de domination Le numérique comme un fait social Esprit critique Culture politique Démocratie et contre pouvoir Pouvoir d'agir ou devoir d'agir? Diagnostic et enjeux De l'attribution d'une place à une culture de la participation Famille et éducation Connaissance des institutions publics et relation aux association ingéniérie sociale Portrait de territoire Mesure de l'impact social BC3 : Mettre en oeuvre et évaluer un projet d'action Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie de projet Mesure de l'impact social Accompagner la vulnérabilité La protection de l'Enfance en France Outils participatifs Intelligence artificielle et fonction de coordination BC4 : Développer les partenariats opérationnelles et contribuer aux dynamiques institutionnelles dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Connaissance des institutions publics et relation aux associations Démocratie et contre pouvoir Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie sociale Outils participatifs | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T19" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | DEJEPS spécialité animation socio-éducative ou culturelle mention coordination de projets</t>
+        </is>
+      </c>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11870193/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11880827/true/false/false/false</t>
         </is>
       </c>
       <c r="V19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W19" s="7" t="inlineStr">
@@ -2685,27 +2685,27 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
+          <t>Créez votre vignoble bio de raisin de table, rentable et résilient - Devenez autonome pour produire et vendre votre propre raisin de table bio</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>UCPA Formation</t>
+          <t>SARL Agri-learn éditions</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>69200 Vénissieux</t>
+          <t>69001 Lyon</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>16 Avenue Dr Georges Levy | 69200 Vénissieux | France</t>
+          <t>Formation a distance | 69001 Lyon | France</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1267 heures (dont 637 heures en entreprise)</t>
+          <t>Durée de 9 heures</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -2720,12 +2720,12 @@
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>ucpa-formation@ucpa.asso.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>ucpa-formation@ucpa.asso.fr | fgehant@ucpa.asso.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -2740,43 +2740,35 @@
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>0642833617</t>
+          <t>0620021214</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>0642833617</t>
-        </is>
-      </c>
-      <c r="O20" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr"/>
       <c r="P20" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q20" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>Unité capitalisable (UC) - 1. Encadrer tout public dans tout lieu et toute structureUnité capitalisable (UC) - 2. Mettre en œuvre un projet d'animation s'inscrivant dans le projet de la structureUnité capitalisable (UC) - 3. Conduire une séance, un cycle d'animation ou d'apprentissage dans le champ des activités aquatiques et de la natationUnité capitalisable (UC) - 4. Mobiliser les techniques des activités aquatiques et de la natation pour mettre en œuvre une séance ou un cycle d'apprentissage | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T20" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
-        </is>
-      </c>
+          <t>1. Taille de la vigne Principes de taille (formation et production) Techniques de taille douce Entretien et corrections2. Modes de conduite Choix du système (lyre, gable, plan vertical. Comparaison des conduites Adaptation au contexte pédoclimatique3. Fertilité des sols Gestion du sol (travail / non-travail) Irrigation Maintien de la fertilité en bio4. Travaux du vignoble Protection contre maladies et ravageurs Calendrier des interventions Conduite sous abri (tunnel)5. Choix des plants Sélection des variétés Choix du porte-greffe Adaptation au marché et au terroir6. Plantation Préparation du sol Étapes de plantation Coûts et organisation7. Récolte et commercialisation Récolte et conservation Organisation du travail Valorisation et vente8. Protection du vignoble en bio Biocontrôle et PNPP Réduction des intrants Stratégies alternatives9. Gestion des maladies et ravageurs Identification des principaux risques Prévention et lutte adaptée10. Pilotage des traitements Stratégie cuivre / soufre Optimisation des doses11. Approche agroécologique Biodiversité fonctionnelle Variétés résistantes | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11447001/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11870193/true/false/false/false</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
@@ -2798,27 +2790,27 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'aide-soignant - DEAS</t>
+          <t>BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>UCPA Formation</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>69200 Vénissieux</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+          <t>16 Avenue Dr Georges Levy | 69200 Vénissieux | France</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1540 heures (dont 770 heures en entreprise)</t>
+          <t>Durée de 1267 heures (dont 637 heures en entreprise)</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -2828,17 +2820,17 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=aide-soignant</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>ucpa-formation@ucpa.asso.fr</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>ucpa-formation@ucpa.asso.fr | fgehant@ucpa.asso.fr</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
@@ -2853,12 +2845,12 @@
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0642833617</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0642833617</t>
         </is>
       </c>
       <c r="O21" s="7" t="inlineStr">
@@ -2879,17 +2871,17 @@
       <c r="R21" s="7" t="inlineStr"/>
       <c r="S21" s="7" t="inlineStr">
         <is>
-          <t>La formation conduisant au diplôme d'État d'aide-soignant, 17 semaines d'enseignement théoriques organisées autour de 8 modules : Accompagnement d'une personne dans les activités de la vie quotidienne L'état clinique d'une personne Les soins Ergonomie Relation Communication Hygiène des locaux hospitaliers Transmission des informations Organisation du travail Les titulaires du DE d'auxiliaire de puériculture, du DE d'aide médico-psychologique, du DE d'auxiliaire de vie sociale ou de la MC aide à domicile, sont dispensés de certaines unités de formation. La formation comprend également 6 stages d'une durée totale de 24 semaines en milieu hospitalier ou extra-hospitalier. Possibilité d'effectuer la formation en initial ou en apprentissage. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Unité capitalisable (UC) - 1. Encadrer tout public dans tout lieu et toute structureUnité capitalisable (UC) - 2. Mettre en œuvre un projet d'animation s'inscrivant dans le projet de la structureUnité capitalisable (UC) - 3. Conduire une séance, un cycle d'animation ou d'apprentissage dans le champ des activités aquatiques et de la natationUnité capitalisable (UC) - 4. Mobiliser les techniques des activités aquatiques et de la natation pour mettre en œuvre une séance ou un cycle d'apprentissage | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'aide-soignant</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
         </is>
       </c>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11533549/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11447001/true/false/false/false</t>
         </is>
       </c>
       <c r="V21" s="7" t="inlineStr">
@@ -2911,12 +2903,12 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>Diplôme d'État d'aide-soignant - DEAS</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -2926,12 +2918,12 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 1540 heures (dont 770 heures en entreprise)</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -2941,17 +2933,17 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=aide-soignant</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -2966,12 +2958,12 @@
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>0472117979</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>0472117979</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O22" s="5" t="inlineStr">
@@ -2990,15 +2982,19 @@
         </is>
       </c>
       <c r="R22" s="5" t="inlineStr"/>
-      <c r="S22" s="5" t="inlineStr"/>
+      <c r="S22" s="5" t="inlineStr">
+        <is>
+          <t>La formation conduisant au diplôme d'État d'aide-soignant, 17 semaines d'enseignement théoriques organisées autour de 8 modules : Accompagnement d'une personne dans les activités de la vie quotidienne L'état clinique d'une personne Les soins Ergonomie Relation Communication Hygiène des locaux hospitaliers Transmission des informations Organisation du travail Les titulaires du DE d'auxiliaire de puériculture, du DE d'aide médico-psychologique, du DE d'auxiliaire de vie sociale ou de la MC aide à domicile, sont dispensés de certaines unités de formation. La formation comprend également 6 stages d'une durée totale de 24 semaines en milieu hospitalier ou extra-hospitalier. Possibilité d'effectuer la formation en initial ou en apprentissage. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T22" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'aide-soignant</t>
         </is>
       </c>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11817055/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11533549/true/false/false/true</t>
         </is>
       </c>
       <c r="V22" s="5" t="inlineStr">
@@ -3020,12 +3016,12 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'assistant de service social - DE ASS</t>
+          <t>Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -3035,12 +3031,12 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 avenue Lacassagne | Croix Rouge francaise | 69003 Lyon 3e | France</t>
+          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Durée de 3420 heures (dont 1680 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -3050,17 +3046,17 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=assistant%20de%20service%20social</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -3075,12 +3071,12 @@
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0472117979</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0472117979</t>
         </is>
       </c>
       <c r="O23" s="7" t="inlineStr">
@@ -3102,12 +3098,12 @@
       <c r="S23" s="7" t="inlineStr"/>
       <c r="T23" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11672249/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11817055/true/false/false/false</t>
         </is>
       </c>
       <c r="V23" s="7" t="inlineStr">
@@ -3129,27 +3125,27 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'éducateur spécialisé</t>
+          <t>Diplôme d'État d'assistant de service social - DE ASS</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales (ARFRIPS - Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales)</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>69009 Lyon 9e</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>10 Impasse Pierre Baizet | 69009 Lyon 9e | France</t>
+          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 avenue Lacassagne | Croix Rouge francaise | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Durée de 3442 heures (dont 1925 heures en entreprise)</t>
+          <t>Durée de 3420 heures (dont 1680 heures en entreprise)</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -3159,17 +3155,17 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=assistant%20de%20service%20social</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>info@arfrips.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>info@arfrips.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -3184,12 +3180,12 @@
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>0478699090</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
         <is>
-          <t>0478699090</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O24" s="5" t="inlineStr">
@@ -3211,17 +3207,17 @@
       <c r="S24" s="5" t="inlineStr"/>
       <c r="T24" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur spécialisé</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
         </is>
       </c>
       <c r="U24" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11737248/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11672249/true/false/false/false</t>
         </is>
       </c>
       <c r="V24" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
         </is>
       </c>
       <c r="W24" s="5" t="inlineStr">
@@ -3238,27 +3234,27 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet - RNCP 39931 - spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+          <t>Diplôme d'État d'éducateur spécialisé</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+          <t>Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales (ARFRIPS - Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales)</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>69009 Lyon 9e</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+          <t>10 Impasse Pierre Baizet | 69009 Lyon 9e | France</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 3442 heures (dont 1925 heures en entreprise)</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -3268,17 +3264,17 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>https://arfatsema.catalogueformpro.com/2/desjeps-17/2858060/desjeps-17-diplome-detat-superieur-de-la-jeunesse-de-leducation-populaire-et-du-sport-specialite-ani</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>info@arfrips.fr</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>info@arfrips.fr</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
@@ -3293,12 +3289,12 @@
       </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0478699090</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0478699090</t>
         </is>
       </c>
       <c r="O25" s="7" t="inlineStr">
@@ -3308,7 +3304,7 @@
       </c>
       <c r="P25" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q25" s="7" t="inlineStr">
@@ -3317,19 +3313,15 @@
         </is>
       </c>
       <c r="R25" s="7" t="inlineStr"/>
-      <c r="S25" s="7" t="inlineStr">
-        <is>
-          <t>BC1 : Construire, avec les instances de gouvernance, la stratégie de développement d'une structure dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Éducation Populaire Culture Politique Rapport de domination Pouvoir d'Agir et Vulnérabilité Esprit critique Transformation social/rapport sociaux Le numérique comme un fait social Nouvel esprit du capitalisme Laicité et valeurs de la République Violence sexiste violences sexuelles Ingénierie social en lien avec la structure Réaliser un diagnostic RH et financier Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Elaboration de la stratégie de développement en lien avec les instances de gouvernance Animer un processus démocratique Démocratie et contre pouvoir BC2 : Concevoir et diriger un projet de développement de la structure Cartographie des relations et l'environnement de son association Ingénierie du projet Processus d'évaluation dans une démarche partagée et participative Outils participatifs Outils de communication Utilité sociale BC3 : Manager l'équipe et gérer les ressources humaines ( et la démarche Qualité, Sécurité, Santé au Travail et Environnement d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Gestion des ressources humaines en structures d'éducation populaire : enjeux, éthique et complexités associative Articulation employeur bénévole - direction dans la gestion des ressources humaines : définition d'une politique RH et organisation des délégations de pouvoir Gérer l'équipe au quotidien : accompagnement, régulation et gestion conflits Analyse des pratiques en co-développement Développer le pouvoir d'agir des salariés Attractivité, recrutement, intégration et fidélisation des salariés Diversité, inclusion et égalité professionnelle au sein de son organisation Assurer la GPEC, la formation et la gestion des carrières dans un alignement éthique Le financement de la formation professionnelle Qualité de vie Santé sécurité au travail Droit du travail/Droit social Dialogue social/dialogue syndical Cadre général des RPS Démarche prévention et outils BC4 : Assurer la gestion financière, matérielle et administrative d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Comprendre les fondamentaux de la situation financière Initiation à l'analyse financière associative ou de structure d'intérêt général Identifier les leviers de financement Construire des scénarios budgétaires et faire des arbitrages Élaborer un plan d'action financier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
+      <c r="S25" s="7" t="inlineStr"/>
       <c r="T25" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur spécialisé</t>
         </is>
       </c>
       <c r="U25" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880835/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11737248/true/false/false/false</t>
         </is>
       </c>
       <c r="V25" s="7" t="inlineStr">
@@ -3351,27 +3343,27 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Créer sa ferme en circuit court : transformation, commercialisation et communication</t>
+          <t>DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet - RNCP 39931 - spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>SARL Agri-learn éditions</t>
+          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>69001 Lyon</t>
+          <t>69100 Villeurbanne</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 69001 Lyon | France</t>
+          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Durée de 20 heures</t>
+          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -3381,17 +3373,17 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://arfatsema.catalogueformpro.com/2/desjeps-17/2858060/desjeps-17-diplome-detat-superieur-de-la-jeunesse-de-leducation-populaire-et-du-sport-specialite-ani</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
@@ -3406,15 +3398,19 @@
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0478031711</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
-          <t>0620021214</t>
-        </is>
-      </c>
-      <c r="O26" s="5" t="inlineStr"/>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="O26" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P26" s="5" t="inlineStr">
         <is>
           <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
@@ -3422,19 +3418,23 @@
       </c>
       <c r="Q26" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R26" s="5" t="inlineStr"/>
       <c r="S26" s="5" t="inlineStr">
         <is>
-          <t>Cette formation s'appuie sur plusieurs compétences essentielles : Stratégie commerciale et étude de marché : définir son offre, ses volumes, ses prix et ses circuits de vente Techniques de vente : maîtriser les étapes clés pour convaincre et fidéliser les clients Transformation des produits agricoles : valoriser ses matières premières pour créer de la valeur ajoutée Hygiène et réglementation : garantir la sécurité sanitaire dans les ateliers de transformation Communication et prospection : développer sa clientèle et promouvoir ses produits Valorisation des produits : savoir parler de ses produits et les mettre en avant (ex : dégustation) L'ensemble permet d'acquérir une vision globale du fonctionnement d'une ferme en circuit court, de la production jusqu'à la vente. 3 heures de visio avec les experts sont prévues dans le cursus. | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T26" s="5" t="inlineStr"/>
+          <t>BC1 : Construire, avec les instances de gouvernance, la stratégie de développement d'une structure dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Éducation Populaire Culture Politique Rapport de domination Pouvoir d'Agir et Vulnérabilité Esprit critique Transformation social/rapport sociaux Le numérique comme un fait social Nouvel esprit du capitalisme Laicité et valeurs de la République Violence sexiste violences sexuelles Ingénierie social en lien avec la structure Réaliser un diagnostic RH et financier Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Elaboration de la stratégie de développement en lien avec les instances de gouvernance Animer un processus démocratique Démocratie et contre pouvoir BC2 : Concevoir et diriger un projet de développement de la structure Cartographie des relations et l'environnement de son association Ingénierie du projet Processus d'évaluation dans une démarche partagée et participative Outils participatifs Outils de communication Utilité sociale BC3 : Manager l'équipe et gérer les ressources humaines ( et la démarche Qualité, Sécurité, Santé au Travail et Environnement d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Gestion des ressources humaines en structures d'éducation populaire : enjeux, éthique et complexités associative Articulation employeur bénévole - direction dans la gestion des ressources humaines : définition d'une politique RH et organisation des délégations de pouvoir Gérer l'équipe au quotidien : accompagnement, régulation et gestion conflits Analyse des pratiques en co-développement Développer le pouvoir d'agir des salariés Attractivité, recrutement, intégration et fidélisation des salariés Diversité, inclusion et égalité professionnelle au sein de son organisation Assurer la GPEC, la formation et la gestion des carrières dans un alignement éthique Le financement de la formation professionnelle Qualité de vie Santé sécurité au travail Droit du travail/Droit social Dialogue social/dialogue syndical Cadre général des RPS Démarche prévention et outils BC4 : Assurer la gestion financière, matérielle et administrative d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Comprendre les fondamentaux de la situation financière Initiation à l'analyse financière associative ou de structure d'intérêt général Identifier les leviers de financement Construire des scénarios budgétaires et faire des arbitrages Élaborer un plan d'action financier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T26" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+        </is>
+      </c>
       <c r="U26" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880868/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11880835/true/false/false/false</t>
         </is>
       </c>
       <c r="V26" s="5" t="inlineStr">
@@ -3456,27 +3456,27 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Titre professionnel administrateur d'infrastructures sécurisées (FOAD)</t>
+          <t>Créer sa ferme en circuit court : transformation, commercialisation et communication</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>STUDI</t>
+          <t>SARL Agri-learn éditions</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>69001 Lyon</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Formation a distance | 69001 Lyon | France</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Durée de 947 heures (dont 350 heures en entreprise)</t>
+          <t>Durée de 20 heures</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -3491,12 +3491,12 @@
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>contact@studi.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>contact@studi.fr | conseiller-formation.aoft@studi.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
@@ -3511,22 +3511,18 @@
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>0174888555</t>
+          <t>0620021214</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>0174888555</t>
-        </is>
-      </c>
-      <c r="O27" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="O27" s="7" t="inlineStr"/>
       <c r="P27" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q27" s="7" t="inlineStr">
@@ -3537,25 +3533,134 @@
       <c r="R27" s="7" t="inlineStr"/>
       <c r="S27" s="7" t="inlineStr">
         <is>
+          <t>Cette formation s'appuie sur plusieurs compétences essentielles : Stratégie commerciale et étude de marché : définir son offre, ses volumes, ses prix et ses circuits de vente Techniques de vente : maîtriser les étapes clés pour convaincre et fidéliser les clients Transformation des produits agricoles : valoriser ses matières premières pour créer de la valeur ajoutée Hygiène et réglementation : garantir la sécurité sanitaire dans les ateliers de transformation Communication et prospection : développer sa clientèle et promouvoir ses produits Valorisation des produits : savoir parler de ses produits et les mettre en avant (ex : dégustation) L'ensemble permet d'acquérir une vision globale du fonctionnement d'une ferme en circuit court, de la production jusqu'à la vente. 3 heures de visio avec les experts sont prévues dans le cursus. | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T27" s="7" t="inlineStr"/>
+      <c r="U27" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11880868/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V27" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W27" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Titre professionnel administrateur d'infrastructures sécurisées (FOAD)</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>STUDI</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>75004 Paris</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Formation a distance | 75004 Paris | France</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 947 heures (dont 350 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>contact@studi.fr</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>contact@studi.fr | conseiller-formation.aoft@studi.fr</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M28" s="5" t="inlineStr">
+        <is>
+          <t>0174888555</t>
+        </is>
+      </c>
+      <c r="N28" s="5" t="inlineStr">
+        <is>
+          <t>0174888555</t>
+        </is>
+      </c>
+      <c r="O28" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P28" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par France Travail</t>
+        </is>
+      </c>
+      <c r="Q28" s="5" t="inlineStr">
+        <is>
+          <t>À distance</t>
+        </is>
+      </c>
+      <c r="R28" s="5" t="inlineStr"/>
+      <c r="S28" s="5" t="inlineStr">
+        <is>
           <t>Administrer et sécuriser les infrastructures Les bonnes pratiques dans l'administration des infrastructures Utiliser un logiciel de gestion centralisé : GLPI Configurer le routage Administrer et sécuriser le réseau Automatiser les tâches d'administration Administrer et sécuriser les systèmes Les bases des serveurs virtualisés Administrer et sécuriser une infrastructure de serveurs virtualisée Gérer des containersConcevoir et mettre en œuvre une solution en réponse à un besoin d'évolution Les bases des solutions techniques Proposer une solution informatique répondant à des besoins nouveaux Mettre en production des évolutions de l'infrastructure Les bases de la supervision Superviser la disponibilité de l'infrastructure et en présenter les résultats Mesurer les performances et la disponibilité de l'infrastructureParticiper à la gestion de la cybersécurité Les bases de la cybersécurité Participer à la mesure et à l'analyse du niveau de sécurité de l'infrastructure Participer à l'élaboration et à la mise en œuvre de la politique de sécurité Participer à la détection et au traitement des incidents de sécurité | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
-      <c r="T27" s="7" t="inlineStr">
+      <c r="T28" s="5" t="inlineStr">
         <is>
           <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel administrateur d'infrastructures sécurisées</t>
         </is>
       </c>
-      <c r="U27" s="7" t="inlineStr">
+      <c r="U28" s="5" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/detail/11590088/true/false/true/false</t>
         </is>
       </c>
-      <c r="V27" s="7" t="inlineStr">
+      <c r="V28" s="5" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
-      <c r="W27" s="7" t="inlineStr">
+      <c r="W28" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-07-13
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseFranceTravail" displayName="BaseFranceTravail" ref="A1:W28" headerRowCount="1">
-  <autoFilter ref="A1:W28"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseFranceTravail" displayName="BaseFranceTravail" ref="A1:W38" headerRowCount="1">
+  <autoFilter ref="A1:W38"/>
   <tableColumns count="23">
     <tableColumn id="1" name="zone"/>
     <tableColumn id="2" name="formation"/>
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>27</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5">
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W28"/>
+  <dimension ref="A1:W38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -810,12 +810,12 @@
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/false</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -915,12 +915,12 @@
       <c r="T3" s="7" t="inlineStr"/>
       <c r="U3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/false</t>
         </is>
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1020,12 +1020,12 @@
       <c r="T4" s="5" t="inlineStr"/>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/false</t>
         </is>
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1133,12 +1133,12 @@
       </c>
       <c r="U5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/false</t>
         </is>
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1238,12 +1238,12 @@
       <c r="T6" s="5" t="inlineStr"/>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/false</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1255,7 +1255,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1343,12 +1343,12 @@
       <c r="T7" s="7" t="inlineStr"/>
       <c r="U7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/false</t>
         </is>
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1360,7 +1360,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1448,12 +1448,12 @@
       <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/false</t>
         </is>
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1553,12 +1553,12 @@
       <c r="T9" s="7" t="inlineStr"/>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/false</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1666,12 +1666,12 @@
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/false</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,32 +1683,32 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>E2C - Ecole de la Deuxième Chance</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Ecole de la Deuxième Chance Grand Hainaut</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>02140 Vervins</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Ecole de la deuxième chance - site de VERVINS | 3 Place des Anciens Combattants | 02140 Vervins | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1400 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1723,12 +1723,12 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>c.renaud@e2cgrandhainaut.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>c.renaud@e2cgrandhainaut.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1743,40 +1743,48 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>0375310010</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>0375310010</t>
-        </is>
-      </c>
-      <c r="O11" s="7" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>Savoir fondamentauxOrientation et démarches professionnelsSocialisation et développement personnelAlternance en entreprise (près de 30% du temps)Des outils pédagogiques de liaison, d'évaluation et de suivi9 mois maximum + 12 mois de suivi post-parcours | Organisme | Ecole de la Deuxième Chance Grand Hainaut | Lieu de la formation | Ecole de la deuxième chance - site de VERVINS</t>
-        </is>
-      </c>
-      <c r="T11" s="7" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+        </is>
+      </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11072382/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/false</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1788,17 +1796,17 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>CAP Fleuriste</t>
+          <t>Titre professionnel secrétaire assistant médico-administratif (FOAD)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -1813,7 +1821,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 1084 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1828,12 +1836,12 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1848,12 +1856,12 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr">
@@ -1874,22 +1882,22 @@
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>7 projets professionnalisants vous permettront d'acquérir les compétences citées au dessus par la pratique.Vous réaliserez les projets suivants :P1 - Démarrez votre formation de secrétaire assistant médico-administratifP2 - Niveau 1 : Maîtrisez l'accueil et la gestion administrative en milieu médicalP3 - Niveau 2 : Développez vos compétences en rédaction, communication et outils numériques en milieuP4 - Réalisez votre mission en entrepriseP5 - Niveau 3 : Optimisez l'organisation, la sécuritéet la gestion des données sensibles en milieu médicalP6 - Niveau 4 : Améliorez la gestion des communications, données et environnements sanitairesP7 - Préparez votre fin de formation de secrétaire assistant médico-administratif | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T12" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel secrétaire assistant médico-administratif</t>
         </is>
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/true</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -1901,17 +1909,17 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Préparation au concours d'adjoint administratif d'État principal de 2ème classe</t>
+          <t>Formation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school)</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -1926,7 +1934,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Durée de 335 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 346 heures</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1941,12 +1949,12 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>foad@skillandyou.com</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>foad@skillandyou.com</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
@@ -1961,12 +1969,12 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>0146006878</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>0146006878</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O13" s="7" t="inlineStr"/>
@@ -1983,18 +1991,18 @@
       <c r="R13" s="7" t="inlineStr"/>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>Votre intégration - Guide d'intégration - Bienvenue dans votre formation - Guide Métier Adjoint administratif d'État principal de 2ème classe - Guide de la formation - Guide des épreuves - Le concours d'adjoint administratif d'État principal de 2ème classe Aide à la réalisation de vos documents professionnels Compléter votre livret de suivi des compétences professionnelles Retranscrire et ordonner les idées principales d'un texte Annales corrigées Épreuves blanches Solliciter les connaissances fondamentales pour le concours Comprendre l'administration française Comprendre le fonctionnement des institutions françaises Acquérir des connaissances en français Acquérir une bonne culture générale Mathématiques Les tests d'aptitudes verbales Annales corrigées Épreuves blanches Mobiliser les compétences professionnelles de l'adjoint administratif d'État Bureautique Épreuves blanches Techniques et recherche d'emploi/stage Sensibilisation au développement durable | Organisme | Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school) | Lieu de la formation | Formation a distance</t>
+          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T13" s="7" t="inlineStr"/>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11205913/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/true</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W13" s="7" t="inlineStr">
@@ -2006,17 +2014,17 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Certification CLOE français langue étrangère - spécialité hôtellerie Restauration niveau A2 vers B1 (FOAD)</t>
+          <t>Concours d'atsem (FOAD)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Nepsod Evolution</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -2031,7 +2039,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Durée de 331 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -2046,12 +2054,12 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>accueil@nepsod.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>accueil@nepsod.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -2066,19 +2074,15 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>0474639587</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>0474639587</t>
-        </is>
-      </c>
-      <c r="O14" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr"/>
       <c r="P14" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -2092,22 +2096,18 @@
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>Accueil et initiation à la formation (1h30) - Module FLE visée insertion professionnelle : chercher un emploi, présenter son métier, présenter ses projets, interagir avec ses collègues, manipuler les outils numériques (120h30) - Module FOS Hôtellerie Restauration :découvrir la cuisine, travailler en cuisine, identifier les besoins d'un client, présenter des produits et services, gérer les réclamations (50h) Module environnement social et culturel : vie quotidienne et relations sociales, loisirs, patrimoine, citoyenneté et engagement (43h) Module Préparation et recherche de stage en entreprise (14h) Période de stage en entreprise (35 h) Module remise à niveau numérique (35 h maximum) Module accompagnement à l'après-formation (21h maximum) Module Préparation et passage de la certification CLOE (10h) Bilan final (1h) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T14" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Certification CLOE français langue étrangère</t>
-        </is>
-      </c>
+          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T14" s="5" t="inlineStr"/>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11576792/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
@@ -2119,32 +2119,32 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière) - DEI</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2159,12 +2159,12 @@
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -2179,12 +2179,12 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="O15" s="7" t="inlineStr">
@@ -2194,33 +2194,33 @@
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr"/>
       <c r="S15" s="7" t="inlineStr">
         <is>
-          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail (bureautique,recherche documentaire, rédaction de documents écrits, communication, anglais) La formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de1 800h, sous la forme de cours magistraux (750 h) travaux dirigés (1 050 h) le travail personnel guidé (suivi pédagogique, temps personnel guidé, supervision, travaux entre étudiants- 300 h) la formation clinique de 2 100 h le travail personnel complémentaire est estimé à 900 heures environ, soit 300 h par an. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11533526/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W15" s="7" t="inlineStr">
@@ -2232,32 +2232,32 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État de technicien de laboratoire médical</t>
+          <t>Préparation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Association des Fondateurs et Protecteurs de l'Institut Catholique de Lyon (AFPICL) (UCLy - Institut Catholique de Lyon)</t>
+          <t>AFEC (Siège)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>69002 Lyon 2e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>10 place des Archives | 69002 Lyon 2e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1120 heures</t>
+          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2272,12 +2272,12 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>fp@univ-catholyon.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>fp@univ-catholyon.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -2292,44 +2292,40 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>0472325134</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>0472325134</t>
-        </is>
-      </c>
-      <c r="O16" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0153368844</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr"/>
       <c r="P16" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q16" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R16" s="5" t="inlineStr"/>
-      <c r="S16" s="5" t="inlineStr"/>
-      <c r="T16" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État de technicien de laboratoire médical</t>
-        </is>
-      </c>
+      <c r="S16" s="5" t="inlineStr">
+        <is>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC (Siège) | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T16" s="5" t="inlineStr"/>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11026378/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W16" s="5" t="inlineStr">
@@ -2341,32 +2337,32 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'ambulancier</t>
+          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Durée de 801 heures (dont 245 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2381,12 +2377,12 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -2401,48 +2397,40 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>0472117903</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>0472117903</t>
-        </is>
-      </c>
-      <c r="O17" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="inlineStr"/>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="7" t="inlineStr">
         <is>
-          <t>Non renseigne | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T17" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'ambulancier</t>
-        </is>
-      </c>
+          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T17" s="7" t="inlineStr"/>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11871421/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
         </is>
       </c>
       <c r="V17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W17" s="7" t="inlineStr">
@@ -2454,32 +2442,32 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Agent de prévention et de sécurité - Titre à finalité professionnelle (TFP APS)</t>
+          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Global pro formation (Global pro formation (GPF))</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Blue Concept | 16 Rue Marcel Dutartre | 69100 Villeurbanne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Durée de 379 heures (dont 70 heures en entreprise)</t>
+          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -2494,12 +2482,12 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>globalproformation@gmail.com</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>globalproformation@gmail.com</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -2514,19 +2502,15 @@
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>0666139535</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>0666139535</t>
-        </is>
-      </c>
-      <c r="O18" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr"/>
       <c r="P18" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -2534,28 +2518,24 @@
       </c>
       <c r="Q18" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>Théorie : SST : Protéger, Examiner (saignement, étouffement, conscience et respiration) et alerter (alerte et message d'accueil) La déontologie de l'agent de sécurité Les services publics de police et gendarmerie, le CNAPS Le cadre légal de la profession, le code pénal et le code de procédure pénale La sûreté de l'État Les armes Mise en sûreté et neutralisation des armes Prévention et actes terrorisme L'accueil, le contrôle d'accès, le contrôle visuel et la palpation de sécurité La prise en compte d'un poste de contrôle de sécurité et les consignes La protection du travailleur Isolé Le circuit de vérification La gestion des alarmes intrusion et incendie, la vidéo et la télésurveillance (surveillance et gardiennage) Les techniques d'information, de communication et la gestion des conflits L'incendie et les risques majeurs Le risque électrique (initiation) Le cadre légal et la problématique de l'activité d'événementiel La définition du terrorisme (historique, mécanisme, méthodologie et modes opératoires) Les différentes menaces terroristes et les niveaux de risque associés La prévention des actes de terrorisme par la reconnaissance des comportements suspects (profiling) et de la radicalisation violente L'action en cas d'attaque et suivant le type d'attaque (actes réflexes, mesures de mise en sécurité immédiate) Le combat en dernier recours L'alerte et la facilitation de l'intervention des forces de l'ordre La sécurisation d'une zone dans l'urgence, risque de sur-attentat et post-attentat. Pratique : Mise en pratique SST CQP APS: Code de la sécurité intérieure Code pénal et libertés publiques Déontologie professionnelle Secours à personnes (SST) Situations conflictuelles et résolution de conflit Consignes, compte rendu et rapport Gestion des risques majeurs, électriques, incendie Gestion d'alarmes Technique d'information et de communication Préparation d'une mission Gestion de conflit Contrôle d'accès Poste de contrôle de sécurité Rondes Palpation de sécurité et inspection de bagages Télésurveillance et vidéo protection Sensibilisation aux risques terroristes Examen : en cours de formation UV 1 (secourisme) : le candidat sera déclaré apte ou inapte en fonction des résultats de la grille d'évaluation conforme aux procédures de validation de l'INRS. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
-        </is>
-      </c>
-      <c r="T18" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Agent de prévention et de sécurité</t>
-        </is>
-      </c>
+          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T18" s="5" t="inlineStr"/>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11870188/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W18" s="5" t="inlineStr">
@@ -2567,32 +2547,32 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'Etat de la Jeunesse de l'Education Populaire et du Sport spécialité "animation socio-éducative ou culturelle mention "coordination de projets" - RNCP 39930 spécialité "animation socio-éducative ou culturel mention "coordination de projets</t>
+          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2602,17 +2582,17 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>https://arfatsema.catalogueformpro.com/3/dejeps-17/2857880/diplome-detat-de-la-jeunesse-de-leducation-populaire-et-du-sport-dejeps-17-specialite-animation-soci/registration?session_id=2846144</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K19" s="7" t="inlineStr">
@@ -2627,48 +2607,40 @@
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>0478031711</t>
-        </is>
-      </c>
-      <c r="O19" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O19" s="7" t="inlineStr"/>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R19" s="7" t="inlineStr"/>
       <c r="S19" s="7" t="inlineStr">
         <is>
-          <t>BC1: Animer et accompagner une équipe dans le champ du sport ou de l'animation Animer une équipe en structure d'éducation populaire : enjeux éthiques, valeurs et spécificités Réaliser un diagnostic des ressources humaines de son périmètre d'intervention Animer une équipe en structure d'éducation populaire : organisation, cadre légal, réglementation et procédures Diversité et inclusion : analyser les besoins et mettre en place une organisation adaptée Management participatif : développer le pouvoir d'agir d'une équipe Management participatif : outils et pratiques Accompagner une équipe: médiation et gestion de conflits Accompagner une équipe : émancipation et développement de l'autonomie Dynamique de groupe Animer un processus démocratique Projet d'action formative et conception de séance formative Droit du travail/Droit social Communication non violente Outils d'animation collective Outils d'accompagnement individuel Accompagner la vulnérabilité Dialogue social et syndical Responsabilité du coordinateur Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? BC2: Concevoir un projet d'action dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Education Populaire Rapport de domination Le numérique comme un fait social Esprit critique Culture politique Démocratie et contre pouvoir Pouvoir d'agir ou devoir d'agir? Diagnostic et enjeux De l'attribution d'une place à une culture de la participation Famille et éducation Connaissance des institutions publics et relation aux association ingéniérie sociale Portrait de territoire Mesure de l'impact social BC3 : Mettre en oeuvre et évaluer un projet d'action Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie de projet Mesure de l'impact social Accompagner la vulnérabilité La protection de l'Enfance en France Outils participatifs Intelligence artificielle et fonction de coordination BC4 : Développer les partenariats opérationnelles et contribuer aux dynamiques institutionnelles dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Connaissance des institutions publics et relation aux associations Démocratie et contre pouvoir Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie sociale Outils participatifs | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T19" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | DEJEPS spécialité animation socio-éducative ou culturelle mention coordination de projets</t>
-        </is>
-      </c>
+          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T19" s="7" t="inlineStr"/>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880827/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/true</t>
         </is>
       </c>
       <c r="V19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W19" s="7" t="inlineStr">
@@ -2680,32 +2652,32 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Créez votre vignoble bio de raisin de table, rentable et résilient - Devenez autonome pour produire et vendre votre propre raisin de table bio</t>
+          <t>BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>SARL Agri-learn éditions</t>
+          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>69001 Lyon</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 69001 Lyon | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Durée de 9 heures</t>
+          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -2720,12 +2692,12 @@
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr | cecile.iribarne@educagri.fr</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -2740,18 +2712,22 @@
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0479264427</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>0620021214</t>
-        </is>
-      </c>
-      <c r="O20" s="5" t="inlineStr"/>
+          <t>0479264427</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P20" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q20" s="5" t="inlineStr">
@@ -2762,18 +2738,22 @@
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>1. Taille de la vigne Principes de taille (formation et production) Techniques de taille douce Entretien et corrections2. Modes de conduite Choix du système (lyre, gable, plan vertical. Comparaison des conduites Adaptation au contexte pédoclimatique3. Fertilité des sols Gestion du sol (travail / non-travail) Irrigation Maintien de la fertilité en bio4. Travaux du vignoble Protection contre maladies et ravageurs Calendrier des interventions Conduite sous abri (tunnel)5. Choix des plants Sélection des variétés Choix du porte-greffe Adaptation au marché et au terroir6. Plantation Préparation du sol Étapes de plantation Coûts et organisation7. Récolte et commercialisation Récolte et conservation Organisation du travail Valorisation et vente8. Protection du vignoble en bio Biocontrôle et PNPP Réduction des intrants Stratégies alternatives9. Gestion des maladies et ravageurs Identification des principaux risques Prévention et lutte adaptée10. Pilotage des traitements Stratégie cuivre / soufre Optimisation des doses11. Approche agroécologique Biodiversité fonctionnelle Variétés résistantes | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T20" s="5" t="inlineStr"/>
+          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T20" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
+        </is>
+      </c>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11870193/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/true</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W20" s="5" t="inlineStr">
@@ -2785,32 +2765,32 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
+          <t>E2C - Ecole de la Deuxième Chance</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>UCPA Formation</t>
+          <t>Ecole de la Deuxième Chance Grand Hainaut</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>69200 Vénissieux</t>
+          <t>02140 Vervins</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>16 Avenue Dr Georges Levy | 69200 Vénissieux | France</t>
+          <t>Ecole de la deuxième chance - site de VERVINS | 3 Place des Anciens Combattants | 02140 Vervins | France</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1267 heures (dont 637 heures en entreprise)</t>
+          <t>Durée de 1400 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -2825,12 +2805,12 @@
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>ucpa-formation@ucpa.asso.fr</t>
+          <t>c.renaud@e2cgrandhainaut.fr</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>ucpa-formation@ucpa.asso.fr | fgehant@ucpa.asso.fr</t>
+          <t>c.renaud@e2cgrandhainaut.fr</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
@@ -2845,19 +2825,15 @@
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>0642833617</t>
+          <t>0375310010</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>0642833617</t>
-        </is>
-      </c>
-      <c r="O21" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0375310010</t>
+        </is>
+      </c>
+      <c r="O21" s="7" t="inlineStr"/>
       <c r="P21" s="7" t="inlineStr">
         <is>
           <t>Formation financée par la région</t>
@@ -2871,22 +2847,18 @@
       <c r="R21" s="7" t="inlineStr"/>
       <c r="S21" s="7" t="inlineStr">
         <is>
-          <t>Unité capitalisable (UC) - 1. Encadrer tout public dans tout lieu et toute structureUnité capitalisable (UC) - 2. Mettre en œuvre un projet d'animation s'inscrivant dans le projet de la structureUnité capitalisable (UC) - 3. Conduire une séance, un cycle d'animation ou d'apprentissage dans le champ des activités aquatiques et de la natationUnité capitalisable (UC) - 4. Mobiliser les techniques des activités aquatiques et de la natation pour mettre en œuvre une séance ou un cycle d'apprentissage | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T21" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
-        </is>
-      </c>
+          <t>Savoir fondamentauxOrientation et démarches professionnelsSocialisation et développement personnelAlternance en entreprise (près de 30% du temps)Des outils pédagogiques de liaison, d'évaluation et de suivi9 mois maximum + 12 mois de suivi post-parcours | Organisme | Ecole de la Deuxième Chance Grand Hainaut | Lieu de la formation | Ecole de la deuxième chance - site de VERVINS</t>
+        </is>
+      </c>
+      <c r="T21" s="7" t="inlineStr"/>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11447001/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11072382/true/false/false/true</t>
         </is>
       </c>
       <c r="V21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W21" s="7" t="inlineStr">
@@ -2898,32 +2870,32 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'aide-soignant - DEAS</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1540 heures (dont 770 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -2933,17 +2905,17 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=aide-soignant</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -2958,12 +2930,12 @@
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="O22" s="5" t="inlineStr">
@@ -2973,33 +2945,33 @@
       </c>
       <c r="P22" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q22" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>La formation conduisant au diplôme d'État d'aide-soignant, 17 semaines d'enseignement théoriques organisées autour de 8 modules : Accompagnement d'une personne dans les activités de la vie quotidienne L'état clinique d'une personne Les soins Ergonomie Relation Communication Hygiène des locaux hospitaliers Transmission des informations Organisation du travail Les titulaires du DE d'auxiliaire de puériculture, du DE d'aide médico-psychologique, du DE d'auxiliaire de vie sociale ou de la MC aide à domicile, sont dispensés de certaines unités de formation. La formation comprend également 6 stages d'une durée totale de 24 semaines en milieu hospitalier ou extra-hospitalier. Possibilité d'effectuer la formation en initial ou en apprentissage. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T22" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'aide-soignant</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
         </is>
       </c>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11533549/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
         </is>
       </c>
       <c r="V22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W22" s="5" t="inlineStr">
@@ -3016,27 +2988,27 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>Préparation au concours d'adjoint administratif d'État principal de 2ème classe</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+          <t>Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school)</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 335 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -3051,12 +3023,12 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>foad@skillandyou.com</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>foad@skillandyou.com</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -3071,44 +3043,40 @@
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>0472117979</t>
+          <t>0146006878</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>0472117979</t>
-        </is>
-      </c>
-      <c r="O23" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0146006878</t>
+        </is>
+      </c>
+      <c r="O23" s="7" t="inlineStr"/>
       <c r="P23" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q23" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R23" s="7" t="inlineStr"/>
-      <c r="S23" s="7" t="inlineStr"/>
-      <c r="T23" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
-        </is>
-      </c>
+      <c r="S23" s="7" t="inlineStr">
+        <is>
+          <t>Votre intégration - Guide d'intégration - Bienvenue dans votre formation - Guide Métier Adjoint administratif d'État principal de 2ème classe - Guide de la formation - Guide des épreuves - Le concours d'adjoint administratif d'État principal de 2ème classe Aide à la réalisation de vos documents professionnels Compléter votre livret de suivi des compétences professionnelles Retranscrire et ordonner les idées principales d'un texte Annales corrigées Épreuves blanches Solliciter les connaissances fondamentales pour le concours Comprendre l'administration française Comprendre le fonctionnement des institutions françaises Acquérir des connaissances en français Acquérir une bonne culture générale Mathématiques Les tests d'aptitudes verbales Annales corrigées Épreuves blanches Mobiliser les compétences professionnelles de l'adjoint administratif d'État Bureautique Épreuves blanches Techniques et recherche d'emploi/stage Sensibilisation au développement durable | Organisme | Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school) | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T23" s="7" t="inlineStr"/>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11817055/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11205913/true/false/true/true</t>
         </is>
       </c>
       <c r="V23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W23" s="7" t="inlineStr">
@@ -3125,27 +3093,27 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'assistant de service social - DE ASS</t>
+          <t>Certification CLOE français langue étrangère - spécialité hôtellerie Restauration niveau A2 vers B1 (FOAD)</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Nepsod Evolution</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 avenue Lacassagne | Croix Rouge francaise | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Durée de 3420 heures (dont 1680 heures en entreprise)</t>
+          <t>Durée de 331 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -3155,17 +3123,17 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=assistant%20de%20service%20social</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>accueil@nepsod.com</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>accueil@nepsod.com</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -3180,12 +3148,12 @@
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0474639587</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0474639587</t>
         </is>
       </c>
       <c r="O24" s="5" t="inlineStr">
@@ -3195,29 +3163,33 @@
       </c>
       <c r="P24" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q24" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R24" s="5" t="inlineStr"/>
-      <c r="S24" s="5" t="inlineStr"/>
+      <c r="S24" s="5" t="inlineStr">
+        <is>
+          <t>Accueil et initiation à la formation (1h30) - Module FLE visée insertion professionnelle : chercher un emploi, présenter son métier, présenter ses projets, interagir avec ses collègues, manipuler les outils numériques (120h30) - Module FOS Hôtellerie Restauration :découvrir la cuisine, travailler en cuisine, identifier les besoins d'un client, présenter des produits et services, gérer les réclamations (50h) Module environnement social et culturel : vie quotidienne et relations sociales, loisirs, patrimoine, citoyenneté et engagement (43h) Module Préparation et recherche de stage en entreprise (14h) Période de stage en entreprise (35 h) Module remise à niveau numérique (35 h maximum) Module accompagnement à l'après-formation (21h maximum) Module Préparation et passage de la certification CLOE (10h) Bilan final (1h) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T24" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Certification CLOE français langue étrangère</t>
         </is>
       </c>
       <c r="U24" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11672249/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11576792/true/false/true/false</t>
         </is>
       </c>
       <c r="V24" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W24" s="5" t="inlineStr">
@@ -3234,27 +3206,27 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'éducateur spécialisé</t>
+          <t>Diplôme d'État d'infirmier(ière) - DEI</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales (ARFRIPS - Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales)</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>69009 Lyon 9e</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>10 Impasse Pierre Baizet | 69009 Lyon 9e | France</t>
+          <t>115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Durée de 3442 heures (dont 1925 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -3269,12 +3241,12 @@
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>info@arfrips.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>info@arfrips.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
@@ -3289,12 +3261,12 @@
       </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>0478699090</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>0478699090</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O25" s="7" t="inlineStr">
@@ -3313,15 +3285,19 @@
         </is>
       </c>
       <c r="R25" s="7" t="inlineStr"/>
-      <c r="S25" s="7" t="inlineStr"/>
+      <c r="S25" s="7" t="inlineStr">
+        <is>
+          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail (bureautique,recherche documentaire, rédaction de documents écrits, communication, anglais) La formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de1 800h, sous la forme de cours magistraux (750 h) travaux dirigés (1 050 h) le travail personnel guidé (suivi pédagogique, temps personnel guidé, supervision, travaux entre étudiants- 300 h) la formation clinique de 2 100 h le travail personnel complémentaire est estimé à 900 heures environ, soit 300 h par an. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T25" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur spécialisé</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U25" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11737248/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11533526/true/false/false/false</t>
         </is>
       </c>
       <c r="V25" s="7" t="inlineStr">
@@ -3343,27 +3319,27 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet - RNCP 39931 - spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+          <t>Diplôme d'État de technicien de laboratoire médical</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+          <t>Association des Fondateurs et Protecteurs de l'Institut Catholique de Lyon (AFPICL) (UCLy - Institut Catholique de Lyon)</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>69002 Lyon 2e</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+          <t>10 place des Archives | 69002 Lyon 2e | France</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 1120 heures</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -3373,17 +3349,17 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>https://arfatsema.catalogueformpro.com/2/desjeps-17/2858060/desjeps-17-diplome-detat-superieur-de-la-jeunesse-de-leducation-populaire-et-du-sport-specialite-ani</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>fp@univ-catholyon.fr</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>fp@univ-catholyon.fr</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
@@ -3398,12 +3374,12 @@
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0472325134</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0472325134</t>
         </is>
       </c>
       <c r="O26" s="5" t="inlineStr">
@@ -3413,7 +3389,7 @@
       </c>
       <c r="P26" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q26" s="5" t="inlineStr">
@@ -3422,19 +3398,15 @@
         </is>
       </c>
       <c r="R26" s="5" t="inlineStr"/>
-      <c r="S26" s="5" t="inlineStr">
-        <is>
-          <t>BC1 : Construire, avec les instances de gouvernance, la stratégie de développement d'une structure dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Éducation Populaire Culture Politique Rapport de domination Pouvoir d'Agir et Vulnérabilité Esprit critique Transformation social/rapport sociaux Le numérique comme un fait social Nouvel esprit du capitalisme Laicité et valeurs de la République Violence sexiste violences sexuelles Ingénierie social en lien avec la structure Réaliser un diagnostic RH et financier Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Elaboration de la stratégie de développement en lien avec les instances de gouvernance Animer un processus démocratique Démocratie et contre pouvoir BC2 : Concevoir et diriger un projet de développement de la structure Cartographie des relations et l'environnement de son association Ingénierie du projet Processus d'évaluation dans une démarche partagée et participative Outils participatifs Outils de communication Utilité sociale BC3 : Manager l'équipe et gérer les ressources humaines ( et la démarche Qualité, Sécurité, Santé au Travail et Environnement d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Gestion des ressources humaines en structures d'éducation populaire : enjeux, éthique et complexités associative Articulation employeur bénévole - direction dans la gestion des ressources humaines : définition d'une politique RH et organisation des délégations de pouvoir Gérer l'équipe au quotidien : accompagnement, régulation et gestion conflits Analyse des pratiques en co-développement Développer le pouvoir d'agir des salariés Attractivité, recrutement, intégration et fidélisation des salariés Diversité, inclusion et égalité professionnelle au sein de son organisation Assurer la GPEC, la formation et la gestion des carrières dans un alignement éthique Le financement de la formation professionnelle Qualité de vie Santé sécurité au travail Droit du travail/Droit social Dialogue social/dialogue syndical Cadre général des RPS Démarche prévention et outils BC4 : Assurer la gestion financière, matérielle et administrative d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Comprendre les fondamentaux de la situation financière Initiation à l'analyse financière associative ou de structure d'intérêt général Identifier les leviers de financement Construire des scénarios budgétaires et faire des arbitrages Élaborer un plan d'action financier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
+      <c r="S26" s="5" t="inlineStr"/>
       <c r="T26" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État de technicien de laboratoire médical</t>
         </is>
       </c>
       <c r="U26" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880835/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11026378/true/false/false/false</t>
         </is>
       </c>
       <c r="V26" s="5" t="inlineStr">
@@ -3456,27 +3428,27 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Créer sa ferme en circuit court : transformation, commercialisation et communication</t>
+          <t>Diplôme d'État d'ambulancier</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>SARL Agri-learn éditions</t>
+          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>69001 Lyon</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 69001 Lyon | France</t>
+          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Durée de 20 heures</t>
+          <t>Durée de 801 heures (dont 245 heures en entreprise)</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -3491,12 +3463,12 @@
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
@@ -3511,40 +3483,48 @@
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0472117903</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>0620021214</t>
-        </is>
-      </c>
-      <c r="O27" s="7" t="inlineStr"/>
+          <t>0472117903</t>
+        </is>
+      </c>
+      <c r="O27" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P27" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q27" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R27" s="7" t="inlineStr"/>
       <c r="S27" s="7" t="inlineStr">
         <is>
-          <t>Cette formation s'appuie sur plusieurs compétences essentielles : Stratégie commerciale et étude de marché : définir son offre, ses volumes, ses prix et ses circuits de vente Techniques de vente : maîtriser les étapes clés pour convaincre et fidéliser les clients Transformation des produits agricoles : valoriser ses matières premières pour créer de la valeur ajoutée Hygiène et réglementation : garantir la sécurité sanitaire dans les ateliers de transformation Communication et prospection : développer sa clientèle et promouvoir ses produits Valorisation des produits : savoir parler de ses produits et les mettre en avant (ex : dégustation) L'ensemble permet d'acquérir une vision globale du fonctionnement d'une ferme en circuit court, de la production jusqu'à la vente. 3 heures de visio avec les experts sont prévues dans le cursus. | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T27" s="7" t="inlineStr"/>
+          <t>Non renseigne | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T27" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'ambulancier</t>
+        </is>
+      </c>
       <c r="U27" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880868/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11871421/true/false/false/false</t>
         </is>
       </c>
       <c r="V27" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
         </is>
       </c>
       <c r="W27" s="7" t="inlineStr">
@@ -3561,27 +3541,27 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Titre professionnel administrateur d'infrastructures sécurisées (FOAD)</t>
+          <t>Agent de prévention et de sécurité - Titre à finalité professionnelle (TFP APS)</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>STUDI</t>
+          <t>Global pro formation (Global pro formation (GPF))</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>69100 Villeurbanne</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Blue Concept | 16 Rue Marcel Dutartre | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Durée de 947 heures (dont 350 heures en entreprise)</t>
+          <t>Durée de 379 heures (dont 70 heures en entreprise)</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -3596,12 +3576,12 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>contact@studi.fr</t>
+          <t>globalproformation@gmail.com</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>contact@studi.fr | conseiller-formation.aoft@studi.fr</t>
+          <t>globalproformation@gmail.com</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
@@ -3616,12 +3596,12 @@
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>0174888555</t>
+          <t>0666139535</t>
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>0174888555</t>
+          <t>0666139535</t>
         </is>
       </c>
       <c r="O28" s="5" t="inlineStr">
@@ -3636,31 +3616,1133 @@
       </c>
       <c r="Q28" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R28" s="5" t="inlineStr"/>
       <c r="S28" s="5" t="inlineStr">
         <is>
+          <t>Théorie : SST : Protéger, Examiner (saignement, étouffement, conscience et respiration) et alerter (alerte et message d'accueil) La déontologie de l'agent de sécurité Les services publics de police et gendarmerie, le CNAPS Le cadre légal de la profession, le code pénal et le code de procédure pénale La sûreté de l'État Les armes Mise en sûreté et neutralisation des armes Prévention et actes terrorisme L'accueil, le contrôle d'accès, le contrôle visuel et la palpation de sécurité La prise en compte d'un poste de contrôle de sécurité et les consignes La protection du travailleur Isolé Le circuit de vérification La gestion des alarmes intrusion et incendie, la vidéo et la télésurveillance (surveillance et gardiennage) Les techniques d'information, de communication et la gestion des conflits L'incendie et les risques majeurs Le risque électrique (initiation) Le cadre légal et la problématique de l'activité d'événementiel La définition du terrorisme (historique, mécanisme, méthodologie et modes opératoires) Les différentes menaces terroristes et les niveaux de risque associés La prévention des actes de terrorisme par la reconnaissance des comportements suspects (profiling) et de la radicalisation violente L'action en cas d'attaque et suivant le type d'attaque (actes réflexes, mesures de mise en sécurité immédiate) Le combat en dernier recours L'alerte et la facilitation de l'intervention des forces de l'ordre La sécurisation d'une zone dans l'urgence, risque de sur-attentat et post-attentat. Pratique : Mise en pratique SST CQP APS: Code de la sécurité intérieure Code pénal et libertés publiques Déontologie professionnelle Secours à personnes (SST) Situations conflictuelles et résolution de conflit Consignes, compte rendu et rapport Gestion des risques majeurs, électriques, incendie Gestion d'alarmes Technique d'information et de communication Préparation d'une mission Gestion de conflit Contrôle d'accès Poste de contrôle de sécurité Rondes Palpation de sécurité et inspection de bagages Télésurveillance et vidéo protection Sensibilisation aux risques terroristes Examen : en cours de formation UV 1 (secourisme) : le candidat sera déclaré apte ou inapte en fonction des résultats de la grille d'évaluation conforme aux procédures de validation de l'INRS. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
+        </is>
+      </c>
+      <c r="T28" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Agent de prévention et de sécurité</t>
+        </is>
+      </c>
+      <c r="U28" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11870188/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V28" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W28" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Diplôme d'Etat de la Jeunesse de l'Education Populaire et du Sport spécialité "animation socio-éducative ou culturelle mention "coordination de projets" - RNCP 39930 spécialité "animation socio-éducative ou culturel mention "coordination de projets</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>69100 Villeurbanne</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>https://arfatsema.catalogueformpro.com/3/dejeps-17/2857880/diplome-detat-de-la-jeunesse-de-leducation-populaire-et-du-sport-dejeps-17-specialite-animation-soci/registration?session_id=2846144</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>arfatsema.direction@orange.fr</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>arfatsema.direction@orange.fr</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="inlineStr">
+        <is>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="N29" s="7" t="inlineStr">
+        <is>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="O29" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P29" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+        </is>
+      </c>
+      <c r="Q29" s="7" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R29" s="7" t="inlineStr"/>
+      <c r="S29" s="7" t="inlineStr">
+        <is>
+          <t>BC1: Animer et accompagner une équipe dans le champ du sport ou de l'animation Animer une équipe en structure d'éducation populaire : enjeux éthiques, valeurs et spécificités Réaliser un diagnostic des ressources humaines de son périmètre d'intervention Animer une équipe en structure d'éducation populaire : organisation, cadre légal, réglementation et procédures Diversité et inclusion : analyser les besoins et mettre en place une organisation adaptée Management participatif : développer le pouvoir d'agir d'une équipe Management participatif : outils et pratiques Accompagner une équipe: médiation et gestion de conflits Accompagner une équipe : émancipation et développement de l'autonomie Dynamique de groupe Animer un processus démocratique Projet d'action formative et conception de séance formative Droit du travail/Droit social Communication non violente Outils d'animation collective Outils d'accompagnement individuel Accompagner la vulnérabilité Dialogue social et syndical Responsabilité du coordinateur Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? BC2: Concevoir un projet d'action dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Education Populaire Rapport de domination Le numérique comme un fait social Esprit critique Culture politique Démocratie et contre pouvoir Pouvoir d'agir ou devoir d'agir? Diagnostic et enjeux De l'attribution d'une place à une culture de la participation Famille et éducation Connaissance des institutions publics et relation aux association ingéniérie sociale Portrait de territoire Mesure de l'impact social BC3 : Mettre en oeuvre et évaluer un projet d'action Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie de projet Mesure de l'impact social Accompagner la vulnérabilité La protection de l'Enfance en France Outils participatifs Intelligence artificielle et fonction de coordination BC4 : Développer les partenariats opérationnelles et contribuer aux dynamiques institutionnelles dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Connaissance des institutions publics et relation aux associations Démocratie et contre pouvoir Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie sociale Outils participatifs | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T29" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | DEJEPS spécialité animation socio-éducative ou culturelle mention coordination de projets</t>
+        </is>
+      </c>
+      <c r="U29" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11880827/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V29" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W29" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Créez votre vignoble bio de raisin de table, rentable et résilient - Devenez autonome pour produire et vendre votre propre raisin de table bio</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>SARL Agri-learn éditions</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>69001 Lyon</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Formation a distance | 69001 Lyon | France</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 9 heures</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>fanny@agrilearn.fr</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>fanny@agrilearn.fr</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M30" s="5" t="inlineStr">
+        <is>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="N30" s="5" t="inlineStr">
+        <is>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="O30" s="5" t="inlineStr"/>
+      <c r="P30" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+        </is>
+      </c>
+      <c r="Q30" s="5" t="inlineStr">
+        <is>
+          <t>À distance</t>
+        </is>
+      </c>
+      <c r="R30" s="5" t="inlineStr"/>
+      <c r="S30" s="5" t="inlineStr">
+        <is>
+          <t>1. Taille de la vigne Principes de taille (formation et production) Techniques de taille douce Entretien et corrections2. Modes de conduite Choix du système (lyre, gable, plan vertical. Comparaison des conduites Adaptation au contexte pédoclimatique3. Fertilité des sols Gestion du sol (travail / non-travail) Irrigation Maintien de la fertilité en bio4. Travaux du vignoble Protection contre maladies et ravageurs Calendrier des interventions Conduite sous abri (tunnel)5. Choix des plants Sélection des variétés Choix du porte-greffe Adaptation au marché et au terroir6. Plantation Préparation du sol Étapes de plantation Coûts et organisation7. Récolte et commercialisation Récolte et conservation Organisation du travail Valorisation et vente8. Protection du vignoble en bio Biocontrôle et PNPP Réduction des intrants Stratégies alternatives9. Gestion des maladies et ravageurs Identification des principaux risques Prévention et lutte adaptée10. Pilotage des traitements Stratégie cuivre / soufre Optimisation des doses11. Approche agroécologique Biodiversité fonctionnelle Variétés résistantes | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T30" s="5" t="inlineStr"/>
+      <c r="U30" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11870193/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V30" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W30" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>UCPA Formation</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>69200 Vénissieux</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>16 Avenue Dr Georges Levy | 69200 Vénissieux | France</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 1267 heures (dont 637 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>ucpa-formation@ucpa.asso.fr</t>
+        </is>
+      </c>
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t>ucpa-formation@ucpa.asso.fr | fgehant@ucpa.asso.fr</t>
+        </is>
+      </c>
+      <c r="K31" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L31" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="inlineStr">
+        <is>
+          <t>0642833617</t>
+        </is>
+      </c>
+      <c r="N31" s="7" t="inlineStr">
+        <is>
+          <t>0642833617</t>
+        </is>
+      </c>
+      <c r="O31" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P31" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q31" s="7" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R31" s="7" t="inlineStr"/>
+      <c r="S31" s="7" t="inlineStr">
+        <is>
+          <t>Unité capitalisable (UC) - 1. Encadrer tout public dans tout lieu et toute structureUnité capitalisable (UC) - 2. Mettre en œuvre un projet d'animation s'inscrivant dans le projet de la structureUnité capitalisable (UC) - 3. Conduire une séance, un cycle d'animation ou d'apprentissage dans le champ des activités aquatiques et de la natationUnité capitalisable (UC) - 4. Mobiliser les techniques des activités aquatiques et de la natation pour mettre en œuvre une séance ou un cycle d'apprentissage | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T31" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
+        </is>
+      </c>
+      <c r="U31" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11447001/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V31" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W31" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Diplôme d'État d'aide-soignant - DEAS</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>69003 Lyon 3e</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 1540 heures (dont 770 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=aide-soignant</t>
+        </is>
+      </c>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>competence.ara@croix-rouge.fr</t>
+        </is>
+      </c>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M32" s="5" t="inlineStr">
+        <is>
+          <t>0472115560</t>
+        </is>
+      </c>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t>0472115560</t>
+        </is>
+      </c>
+      <c r="O32" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P32" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q32" s="5" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R32" s="5" t="inlineStr"/>
+      <c r="S32" s="5" t="inlineStr">
+        <is>
+          <t>La formation conduisant au diplôme d'État d'aide-soignant, 17 semaines d'enseignement théoriques organisées autour de 8 modules : Accompagnement d'une personne dans les activités de la vie quotidienne L'état clinique d'une personne Les soins Ergonomie Relation Communication Hygiène des locaux hospitaliers Transmission des informations Organisation du travail Les titulaires du DE d'auxiliaire de puériculture, du DE d'aide médico-psychologique, du DE d'auxiliaire de vie sociale ou de la MC aide à domicile, sont dispensés de certaines unités de formation. La formation comprend également 6 stages d'une durée totale de 24 semaines en milieu hospitalier ou extra-hospitalier. Possibilité d'effectuer la formation en initial ou en apprentissage. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T32" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'aide-soignant</t>
+        </is>
+      </c>
+      <c r="U32" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11533549/true/false/false/true</t>
+        </is>
+      </c>
+      <c r="V32" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W32" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Diplôme d'État d'infirmier(ière)</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>69003 Lyon 3e</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I33" s="6" t="inlineStr">
+        <is>
+          <t>magaly.lebrat@chu-lyon.fr</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>magaly.lebrat@chu-lyon.fr</t>
+        </is>
+      </c>
+      <c r="K33" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L33" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M33" s="7" t="inlineStr">
+        <is>
+          <t>0472117979</t>
+        </is>
+      </c>
+      <c r="N33" s="7" t="inlineStr">
+        <is>
+          <t>0472117979</t>
+        </is>
+      </c>
+      <c r="O33" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P33" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q33" s="7" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R33" s="7" t="inlineStr"/>
+      <c r="S33" s="7" t="inlineStr"/>
+      <c r="T33" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+        </is>
+      </c>
+      <c r="U33" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11817055/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V33" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W33" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Diplôme d'État d'assistant de service social - DE ASS</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>69003 Lyon 3e</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 avenue Lacassagne | Croix Rouge francaise | 69003 Lyon 3e | France</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 3420 heures (dont 1680 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=assistant%20de%20service%20social</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>competence.ara@croix-rouge.fr</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+        </is>
+      </c>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M34" s="5" t="inlineStr">
+        <is>
+          <t>0472115560</t>
+        </is>
+      </c>
+      <c r="N34" s="5" t="inlineStr">
+        <is>
+          <t>0472115560</t>
+        </is>
+      </c>
+      <c r="O34" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P34" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q34" s="5" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R34" s="5" t="inlineStr"/>
+      <c r="S34" s="5" t="inlineStr"/>
+      <c r="T34" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
+        </is>
+      </c>
+      <c r="U34" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11672249/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V34" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W34" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Diplôme d'État d'éducateur spécialisé</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales (ARFRIPS - Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales)</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>69009 Lyon 9e</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>10 Impasse Pierre Baizet | 69009 Lyon 9e | France</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 3442 heures (dont 1925 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>info@arfrips.fr</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>info@arfrips.fr</t>
+        </is>
+      </c>
+      <c r="K35" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L35" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M35" s="7" t="inlineStr">
+        <is>
+          <t>0478699090</t>
+        </is>
+      </c>
+      <c r="N35" s="7" t="inlineStr">
+        <is>
+          <t>0478699090</t>
+        </is>
+      </c>
+      <c r="O35" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P35" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q35" s="7" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R35" s="7" t="inlineStr"/>
+      <c r="S35" s="7" t="inlineStr"/>
+      <c r="T35" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur spécialisé</t>
+        </is>
+      </c>
+      <c r="U35" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11737248/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V35" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W35" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet - RNCP 39931 - spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>69100 Villeurbanne</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>https://arfatsema.catalogueformpro.com/2/desjeps-17/2858060/desjeps-17-diplome-detat-superieur-de-la-jeunesse-de-leducation-populaire-et-du-sport-specialite-ani</t>
+        </is>
+      </c>
+      <c r="I36" s="6" t="inlineStr">
+        <is>
+          <t>arfatsema.direction@orange.fr</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>arfatsema.direction@orange.fr</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M36" s="5" t="inlineStr">
+        <is>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="O36" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P36" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+        </is>
+      </c>
+      <c r="Q36" s="5" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R36" s="5" t="inlineStr"/>
+      <c r="S36" s="5" t="inlineStr">
+        <is>
+          <t>BC1 : Construire, avec les instances de gouvernance, la stratégie de développement d'une structure dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Éducation Populaire Culture Politique Rapport de domination Pouvoir d'Agir et Vulnérabilité Esprit critique Transformation social/rapport sociaux Le numérique comme un fait social Nouvel esprit du capitalisme Laicité et valeurs de la République Violence sexiste violences sexuelles Ingénierie social en lien avec la structure Réaliser un diagnostic RH et financier Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Elaboration de la stratégie de développement en lien avec les instances de gouvernance Animer un processus démocratique Démocratie et contre pouvoir BC2 : Concevoir et diriger un projet de développement de la structure Cartographie des relations et l'environnement de son association Ingénierie du projet Processus d'évaluation dans une démarche partagée et participative Outils participatifs Outils de communication Utilité sociale BC3 : Manager l'équipe et gérer les ressources humaines ( et la démarche Qualité, Sécurité, Santé au Travail et Environnement d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Gestion des ressources humaines en structures d'éducation populaire : enjeux, éthique et complexités associative Articulation employeur bénévole - direction dans la gestion des ressources humaines : définition d'une politique RH et organisation des délégations de pouvoir Gérer l'équipe au quotidien : accompagnement, régulation et gestion conflits Analyse des pratiques en co-développement Développer le pouvoir d'agir des salariés Attractivité, recrutement, intégration et fidélisation des salariés Diversité, inclusion et égalité professionnelle au sein de son organisation Assurer la GPEC, la formation et la gestion des carrières dans un alignement éthique Le financement de la formation professionnelle Qualité de vie Santé sécurité au travail Droit du travail/Droit social Dialogue social/dialogue syndical Cadre général des RPS Démarche prévention et outils BC4 : Assurer la gestion financière, matérielle et administrative d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Comprendre les fondamentaux de la situation financière Initiation à l'analyse financière associative ou de structure d'intérêt général Identifier les leviers de financement Construire des scénarios budgétaires et faire des arbitrages Élaborer un plan d'action financier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T36" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+        </is>
+      </c>
+      <c r="U36" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11880835/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V36" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W36" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Créer sa ferme en circuit court : transformation, commercialisation et communication</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>SARL Agri-learn éditions</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>69001 Lyon</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Formation a distance | 69001 Lyon | France</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 20 heures</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>fanny@agrilearn.fr</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>fanny@agrilearn.fr</t>
+        </is>
+      </c>
+      <c r="K37" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L37" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M37" s="7" t="inlineStr">
+        <is>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="N37" s="7" t="inlineStr">
+        <is>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="O37" s="7" t="inlineStr"/>
+      <c r="P37" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+        </is>
+      </c>
+      <c r="Q37" s="7" t="inlineStr">
+        <is>
+          <t>À distance</t>
+        </is>
+      </c>
+      <c r="R37" s="7" t="inlineStr"/>
+      <c r="S37" s="7" t="inlineStr">
+        <is>
+          <t>Cette formation s'appuie sur plusieurs compétences essentielles : Stratégie commerciale et étude de marché : définir son offre, ses volumes, ses prix et ses circuits de vente Techniques de vente : maîtriser les étapes clés pour convaincre et fidéliser les clients Transformation des produits agricoles : valoriser ses matières premières pour créer de la valeur ajoutée Hygiène et réglementation : garantir la sécurité sanitaire dans les ateliers de transformation Communication et prospection : développer sa clientèle et promouvoir ses produits Valorisation des produits : savoir parler de ses produits et les mettre en avant (ex : dégustation) L'ensemble permet d'acquérir une vision globale du fonctionnement d'une ferme en circuit court, de la production jusqu'à la vente. 3 heures de visio avec les experts sont prévues dans le cursus. | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T37" s="7" t="inlineStr"/>
+      <c r="U37" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11880868/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V37" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W37" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Titre professionnel administrateur d'infrastructures sécurisées (FOAD)</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>STUDI</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>75004 Paris</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Formation a distance | 75004 Paris | France</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 947 heures (dont 350 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I38" s="6" t="inlineStr">
+        <is>
+          <t>contact@studi.fr</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>contact@studi.fr | conseiller-formation.aoft@studi.fr</t>
+        </is>
+      </c>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M38" s="5" t="inlineStr">
+        <is>
+          <t>0174888555</t>
+        </is>
+      </c>
+      <c r="N38" s="5" t="inlineStr">
+        <is>
+          <t>0174888555</t>
+        </is>
+      </c>
+      <c r="O38" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P38" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par France Travail</t>
+        </is>
+      </c>
+      <c r="Q38" s="5" t="inlineStr">
+        <is>
+          <t>À distance</t>
+        </is>
+      </c>
+      <c r="R38" s="5" t="inlineStr"/>
+      <c r="S38" s="5" t="inlineStr">
+        <is>
           <t>Administrer et sécuriser les infrastructures Les bonnes pratiques dans l'administration des infrastructures Utiliser un logiciel de gestion centralisé : GLPI Configurer le routage Administrer et sécuriser le réseau Automatiser les tâches d'administration Administrer et sécuriser les systèmes Les bases des serveurs virtualisés Administrer et sécuriser une infrastructure de serveurs virtualisée Gérer des containersConcevoir et mettre en œuvre une solution en réponse à un besoin d'évolution Les bases des solutions techniques Proposer une solution informatique répondant à des besoins nouveaux Mettre en production des évolutions de l'infrastructure Les bases de la supervision Superviser la disponibilité de l'infrastructure et en présenter les résultats Mesurer les performances et la disponibilité de l'infrastructureParticiper à la gestion de la cybersécurité Les bases de la cybersécurité Participer à la mesure et à l'analyse du niveau de sécurité de l'infrastructure Participer à l'élaboration et à la mise en œuvre de la politique de sécurité Participer à la détection et au traitement des incidents de sécurité | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
-      <c r="T28" s="5" t="inlineStr">
+      <c r="T38" s="5" t="inlineStr">
         <is>
           <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel administrateur d'infrastructures sécurisées</t>
         </is>
       </c>
-      <c r="U28" s="5" t="inlineStr">
+      <c r="U38" s="5" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/detail/11590088/true/false/true/false</t>
         </is>
       </c>
-      <c r="V28" s="5" t="inlineStr">
+      <c r="V38" s="5" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
-      <c r="W28" s="5" t="inlineStr">
+      <c r="W38" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-07-14
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseFranceTravail" displayName="BaseFranceTravail" ref="A1:W38" headerRowCount="1">
-  <autoFilter ref="A1:W38"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseFranceTravail" displayName="BaseFranceTravail" ref="A1:W39" headerRowCount="1">
+  <autoFilter ref="A1:W39"/>
   <tableColumns count="23">
     <tableColumn id="1" name="zone"/>
     <tableColumn id="2" name="formation"/>
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
@@ -566,13 +566,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W38"/>
+  <dimension ref="A1:W39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -810,12 +810,12 @@
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/true</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -915,12 +915,12 @@
       <c r="T3" s="7" t="inlineStr"/>
       <c r="U3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/true</t>
         </is>
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1020,12 +1020,12 @@
       <c r="T4" s="5" t="inlineStr"/>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
         </is>
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1133,12 +1133,12 @@
       </c>
       <c r="U5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
         </is>
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1238,12 +1238,12 @@
       <c r="T6" s="5" t="inlineStr"/>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1255,7 +1255,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1343,12 +1343,12 @@
       <c r="T7" s="7" t="inlineStr"/>
       <c r="U7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
         </is>
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1360,7 +1360,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1448,12 +1448,12 @@
       <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
         </is>
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1553,12 +1553,12 @@
       <c r="T9" s="7" t="inlineStr"/>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/true</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1666,12 +1666,12 @@
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/true</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,32 +1683,32 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>CAP Fleuriste</t>
+          <t>Ecole de la 2ème Chance (E2C)</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>04000 Digne-les-Bains</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>4 avenue de Verdun | https://www.iap.asso.fr/ | 04000 Digne-les-Bains | France</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 1100 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1718,17 +1718,17 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.iap.asso.fr/</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>contact@iap.asso.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>contact@iap.asso.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1743,48 +1743,40 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>04 92 87 46 10</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O11" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>04 92 87 46 10</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="inlineStr"/>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T11" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
-        </is>
-      </c>
+          <t>Programme non communiqué | Organisme | Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04 | https://www.iap.asso.fr/ | Lieu de la formation</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr"/>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10685143/true/false/false/false</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1796,7 +1788,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
@@ -1892,12 +1884,12 @@
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/false</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -1909,7 +1901,7 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -1997,12 +1989,12 @@
       <c r="T13" s="7" t="inlineStr"/>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/false</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W13" s="7" t="inlineStr">
@@ -2014,7 +2006,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -2102,12 +2094,12 @@
       <c r="T14" s="5" t="inlineStr"/>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/false</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
@@ -2119,7 +2111,7 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -2215,12 +2207,12 @@
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/false</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W15" s="7" t="inlineStr">
@@ -2232,7 +2224,7 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -2320,12 +2312,12 @@
       <c r="T16" s="5" t="inlineStr"/>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/false</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W16" s="5" t="inlineStr">
@@ -2337,7 +2329,7 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -2425,12 +2417,12 @@
       <c r="T17" s="7" t="inlineStr"/>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/false</t>
         </is>
       </c>
       <c r="V17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W17" s="7" t="inlineStr">
@@ -2442,7 +2434,7 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -2530,12 +2522,12 @@
       <c r="T18" s="5" t="inlineStr"/>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/false</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W18" s="5" t="inlineStr">
@@ -2547,7 +2539,7 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -2635,12 +2627,12 @@
       <c r="T19" s="7" t="inlineStr"/>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/false</t>
         </is>
       </c>
       <c r="V19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W19" s="7" t="inlineStr">
@@ -2652,7 +2644,7 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -2748,12 +2740,12 @@
       </c>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/false</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W20" s="5" t="inlineStr">
@@ -2765,32 +2757,32 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>E2C - Ecole de la Deuxième Chance</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Ecole de la Deuxième Chance Grand Hainaut</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>02140 Vervins</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Ecole de la deuxième chance - site de VERVINS | 3 Place des Anciens Combattants | 02140 Vervins | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1400 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -2805,12 +2797,12 @@
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>c.renaud@e2cgrandhainaut.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>c.renaud@e2cgrandhainaut.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
@@ -2825,40 +2817,48 @@
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>0375310010</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>0375310010</t>
-        </is>
-      </c>
-      <c r="O21" s="7" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O21" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P21" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q21" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R21" s="7" t="inlineStr"/>
       <c r="S21" s="7" t="inlineStr">
         <is>
-          <t>Savoir fondamentauxOrientation et démarches professionnelsSocialisation et développement personnelAlternance en entreprise (près de 30% du temps)Des outils pédagogiques de liaison, d'évaluation et de suivi9 mois maximum + 12 mois de suivi post-parcours | Organisme | Ecole de la Deuxième Chance Grand Hainaut | Lieu de la formation | Ecole de la deuxième chance - site de VERVINS</t>
-        </is>
-      </c>
-      <c r="T21" s="7" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T21" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+        </is>
+      </c>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11072382/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/false</t>
         </is>
       </c>
       <c r="V21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W21" s="7" t="inlineStr">
@@ -2870,32 +2870,32 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>CAP Fleuriste</t>
+          <t>E2C - Ecole de la Deuxième Chance</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>Ecole de la Deuxième Chance Grand Hainaut</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>02140 Vervins</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Ecole de la deuxième chance - site de VERVINS | 3 Place des Anciens Combattants | 02140 Vervins | France</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 1400 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -2910,12 +2910,12 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>c.renaud@e2cgrandhainaut.fr</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>c.renaud@e2cgrandhainaut.fr</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -2930,48 +2930,40 @@
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0375310010</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O22" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0375310010</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr"/>
       <c r="P22" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q22" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T22" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
-        </is>
-      </c>
+          <t>Savoir fondamentauxOrientation et démarches professionnelsSocialisation et développement personnelAlternance en entreprise (près de 30% du temps)Des outils pédagogiques de liaison, d'évaluation et de suivi9 mois maximum + 12 mois de suivi post-parcours | Organisme | Ecole de la Deuxième Chance Grand Hainaut | Lieu de la formation | Ecole de la deuxième chance - site de VERVINS</t>
+        </is>
+      </c>
+      <c r="T22" s="5" t="inlineStr"/>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11072382/true/false/false/true</t>
         </is>
       </c>
       <c r="V22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W22" s="5" t="inlineStr">
@@ -2983,17 +2975,17 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>01</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Préparation au concours d'adjoint administratif d'État principal de 2ème classe</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -3008,7 +3000,7 @@
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Durée de 335 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -3023,12 +3015,12 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>foad@skillandyou.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>foad@skillandyou.com</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -3043,15 +3035,19 @@
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>0146006878</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>0146006878</t>
-        </is>
-      </c>
-      <c r="O23" s="7" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P23" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -3065,18 +3061,22 @@
       <c r="R23" s="7" t="inlineStr"/>
       <c r="S23" s="7" t="inlineStr">
         <is>
-          <t>Votre intégration - Guide d'intégration - Bienvenue dans votre formation - Guide Métier Adjoint administratif d'État principal de 2ème classe - Guide de la formation - Guide des épreuves - Le concours d'adjoint administratif d'État principal de 2ème classe Aide à la réalisation de vos documents professionnels Compléter votre livret de suivi des compétences professionnelles Retranscrire et ordonner les idées principales d'un texte Annales corrigées Épreuves blanches Solliciter les connaissances fondamentales pour le concours Comprendre l'administration française Comprendre le fonctionnement des institutions françaises Acquérir des connaissances en français Acquérir une bonne culture générale Mathématiques Les tests d'aptitudes verbales Annales corrigées Épreuves blanches Mobiliser les compétences professionnelles de l'adjoint administratif d'État Bureautique Épreuves blanches Techniques et recherche d'emploi/stage Sensibilisation au développement durable | Organisme | Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school) | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T23" s="7" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T23" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+        </is>
+      </c>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11205913/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
         </is>
       </c>
       <c r="V23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W23" s="7" t="inlineStr">
@@ -3093,12 +3093,12 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Certification CLOE français langue étrangère - spécialité hôtellerie Restauration niveau A2 vers B1 (FOAD)</t>
+          <t>Préparation au concours d'adjoint administratif d'État principal de 2ème classe</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Nepsod Evolution</t>
+          <t>Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school)</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -3113,7 +3113,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Durée de 331 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 335 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -3128,12 +3128,12 @@
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>accueil@nepsod.com</t>
+          <t>foad@skillandyou.com</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>accueil@nepsod.com</t>
+          <t>foad@skillandyou.com</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -3148,19 +3148,15 @@
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>0474639587</t>
+          <t>0146006878</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
         <is>
-          <t>0474639587</t>
-        </is>
-      </c>
-      <c r="O24" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0146006878</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr"/>
       <c r="P24" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -3174,17 +3170,13 @@
       <c r="R24" s="5" t="inlineStr"/>
       <c r="S24" s="5" t="inlineStr">
         <is>
-          <t>Accueil et initiation à la formation (1h30) - Module FLE visée insertion professionnelle : chercher un emploi, présenter son métier, présenter ses projets, interagir avec ses collègues, manipuler les outils numériques (120h30) - Module FOS Hôtellerie Restauration :découvrir la cuisine, travailler en cuisine, identifier les besoins d'un client, présenter des produits et services, gérer les réclamations (50h) Module environnement social et culturel : vie quotidienne et relations sociales, loisirs, patrimoine, citoyenneté et engagement (43h) Module Préparation et recherche de stage en entreprise (14h) Période de stage en entreprise (35 h) Module remise à niveau numérique (35 h maximum) Module accompagnement à l'après-formation (21h maximum) Module Préparation et passage de la certification CLOE (10h) Bilan final (1h) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T24" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Certification CLOE français langue étrangère</t>
-        </is>
-      </c>
+          <t>Votre intégration - Guide d'intégration - Bienvenue dans votre formation - Guide Métier Adjoint administratif d'État principal de 2ème classe - Guide de la formation - Guide des épreuves - Le concours d'adjoint administratif d'État principal de 2ème classe Aide à la réalisation de vos documents professionnels Compléter votre livret de suivi des compétences professionnelles Retranscrire et ordonner les idées principales d'un texte Annales corrigées Épreuves blanches Solliciter les connaissances fondamentales pour le concours Comprendre l'administration française Comprendre le fonctionnement des institutions françaises Acquérir des connaissances en français Acquérir une bonne culture générale Mathématiques Les tests d'aptitudes verbales Annales corrigées Épreuves blanches Mobiliser les compétences professionnelles de l'adjoint administratif d'État Bureautique Épreuves blanches Techniques et recherche d'emploi/stage Sensibilisation au développement durable | Organisme | Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school) | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T24" s="5" t="inlineStr"/>
       <c r="U24" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11576792/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11205913/true/false/true/true</t>
         </is>
       </c>
       <c r="V24" s="5" t="inlineStr">
@@ -3206,27 +3198,27 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière) - DEI</t>
+          <t>Certification CLOE français langue étrangère - spécialité hôtellerie Restauration niveau A2 vers B1 (FOAD)</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Nepsod Evolution</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 331 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -3241,12 +3233,12 @@
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>accueil@nepsod.com</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>accueil@nepsod.com</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
@@ -3261,12 +3253,12 @@
       </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0474639587</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0474639587</t>
         </is>
       </c>
       <c r="O25" s="7" t="inlineStr">
@@ -3276,28 +3268,28 @@
       </c>
       <c r="P25" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R25" s="7" t="inlineStr"/>
       <c r="S25" s="7" t="inlineStr">
         <is>
-          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail (bureautique,recherche documentaire, rédaction de documents écrits, communication, anglais) La formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de1 800h, sous la forme de cours magistraux (750 h) travaux dirigés (1 050 h) le travail personnel guidé (suivi pédagogique, temps personnel guidé, supervision, travaux entre étudiants- 300 h) la formation clinique de 2 100 h le travail personnel complémentaire est estimé à 900 heures environ, soit 300 h par an. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Accueil et initiation à la formation (1h30) - Module FLE visée insertion professionnelle : chercher un emploi, présenter son métier, présenter ses projets, interagir avec ses collègues, manipuler les outils numériques (120h30) - Module FOS Hôtellerie Restauration :découvrir la cuisine, travailler en cuisine, identifier les besoins d'un client, présenter des produits et services, gérer les réclamations (50h) Module environnement social et culturel : vie quotidienne et relations sociales, loisirs, patrimoine, citoyenneté et engagement (43h) Module Préparation et recherche de stage en entreprise (14h) Période de stage en entreprise (35 h) Module remise à niveau numérique (35 h maximum) Module accompagnement à l'après-formation (21h maximum) Module Préparation et passage de la certification CLOE (10h) Bilan final (1h) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T25" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Certification CLOE français langue étrangère</t>
         </is>
       </c>
       <c r="U25" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11533526/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11576792/true/false/true/false</t>
         </is>
       </c>
       <c r="V25" s="7" t="inlineStr">
@@ -3319,27 +3311,27 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État de technicien de laboratoire médical</t>
+          <t>Diplôme d'État d'infirmier(ière) - DEI</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Association des Fondateurs et Protecteurs de l'Institut Catholique de Lyon (AFPICL) (UCLy - Institut Catholique de Lyon)</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>69002 Lyon 2e</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>10 place des Archives | 69002 Lyon 2e | France</t>
+          <t>115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1120 heures</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -3354,12 +3346,12 @@
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>fp@univ-catholyon.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>fp@univ-catholyon.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
@@ -3374,12 +3366,12 @@
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>0472325134</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
-          <t>0472325134</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O26" s="5" t="inlineStr">
@@ -3398,15 +3390,19 @@
         </is>
       </c>
       <c r="R26" s="5" t="inlineStr"/>
-      <c r="S26" s="5" t="inlineStr"/>
+      <c r="S26" s="5" t="inlineStr">
+        <is>
+          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail (bureautique,recherche documentaire, rédaction de documents écrits, communication, anglais) La formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de1 800h, sous la forme de cours magistraux (750 h) travaux dirigés (1 050 h) le travail personnel guidé (suivi pédagogique, temps personnel guidé, supervision, travaux entre étudiants- 300 h) la formation clinique de 2 100 h le travail personnel complémentaire est estimé à 900 heures environ, soit 300 h par an. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T26" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État de technicien de laboratoire médical</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U26" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11026378/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11533526/true/false/false/false</t>
         </is>
       </c>
       <c r="V26" s="5" t="inlineStr">
@@ -3428,27 +3424,27 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'ambulancier</t>
+          <t>Diplôme d'État de technicien de laboratoire médical</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+          <t>Association des Fondateurs et Protecteurs de l'Institut Catholique de Lyon (AFPICL) (UCLy - Institut Catholique de Lyon)</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>69002 Lyon 2e</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+          <t>10 place des Archives | 69002 Lyon 2e | France</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Durée de 801 heures (dont 245 heures en entreprise)</t>
+          <t>Durée de 1120 heures</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -3463,12 +3459,12 @@
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>fp@univ-catholyon.fr</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>fp@univ-catholyon.fr</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
@@ -3483,12 +3479,12 @@
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>0472117903</t>
+          <t>0472325134</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>0472117903</t>
+          <t>0472325134</t>
         </is>
       </c>
       <c r="O27" s="7" t="inlineStr">
@@ -3507,24 +3503,20 @@
         </is>
       </c>
       <c r="R27" s="7" t="inlineStr"/>
-      <c r="S27" s="7" t="inlineStr">
-        <is>
-          <t>Non renseigne | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
+      <c r="S27" s="7" t="inlineStr"/>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'ambulancier</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État de technicien de laboratoire médical</t>
         </is>
       </c>
       <c r="U27" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11871421/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11026378/true/false/false/false</t>
         </is>
       </c>
       <c r="V27" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W27" s="7" t="inlineStr">
@@ -3541,27 +3533,27 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Agent de prévention et de sécurité - Titre à finalité professionnelle (TFP APS)</t>
+          <t>Diplôme d'État d'ambulancier</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Global pro formation (Global pro formation (GPF))</t>
+          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Blue Concept | 16 Rue Marcel Dutartre | 69100 Villeurbanne | France</t>
+          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Durée de 379 heures (dont 70 heures en entreprise)</t>
+          <t>Durée de 801 heures (dont 245 heures en entreprise)</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -3576,12 +3568,12 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>globalproformation@gmail.com</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>globalproformation@gmail.com</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
@@ -3596,12 +3588,12 @@
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>0666139535</t>
+          <t>0472117903</t>
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>0666139535</t>
+          <t>0472117903</t>
         </is>
       </c>
       <c r="O28" s="5" t="inlineStr">
@@ -3611,7 +3603,7 @@
       </c>
       <c r="P28" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q28" s="5" t="inlineStr">
@@ -3622,22 +3614,22 @@
       <c r="R28" s="5" t="inlineStr"/>
       <c r="S28" s="5" t="inlineStr">
         <is>
-          <t>Théorie : SST : Protéger, Examiner (saignement, étouffement, conscience et respiration) et alerter (alerte et message d'accueil) La déontologie de l'agent de sécurité Les services publics de police et gendarmerie, le CNAPS Le cadre légal de la profession, le code pénal et le code de procédure pénale La sûreté de l'État Les armes Mise en sûreté et neutralisation des armes Prévention et actes terrorisme L'accueil, le contrôle d'accès, le contrôle visuel et la palpation de sécurité La prise en compte d'un poste de contrôle de sécurité et les consignes La protection du travailleur Isolé Le circuit de vérification La gestion des alarmes intrusion et incendie, la vidéo et la télésurveillance (surveillance et gardiennage) Les techniques d'information, de communication et la gestion des conflits L'incendie et les risques majeurs Le risque électrique (initiation) Le cadre légal et la problématique de l'activité d'événementiel La définition du terrorisme (historique, mécanisme, méthodologie et modes opératoires) Les différentes menaces terroristes et les niveaux de risque associés La prévention des actes de terrorisme par la reconnaissance des comportements suspects (profiling) et de la radicalisation violente L'action en cas d'attaque et suivant le type d'attaque (actes réflexes, mesures de mise en sécurité immédiate) Le combat en dernier recours L'alerte et la facilitation de l'intervention des forces de l'ordre La sécurisation d'une zone dans l'urgence, risque de sur-attentat et post-attentat. Pratique : Mise en pratique SST CQP APS: Code de la sécurité intérieure Code pénal et libertés publiques Déontologie professionnelle Secours à personnes (SST) Situations conflictuelles et résolution de conflit Consignes, compte rendu et rapport Gestion des risques majeurs, électriques, incendie Gestion d'alarmes Technique d'information et de communication Préparation d'une mission Gestion de conflit Contrôle d'accès Poste de contrôle de sécurité Rondes Palpation de sécurité et inspection de bagages Télésurveillance et vidéo protection Sensibilisation aux risques terroristes Examen : en cours de formation UV 1 (secourisme) : le candidat sera déclaré apte ou inapte en fonction des résultats de la grille d'évaluation conforme aux procédures de validation de l'INRS. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
+          <t>Non renseigne | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T28" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Agent de prévention et de sécurité</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'ambulancier</t>
         </is>
       </c>
       <c r="U28" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11870188/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11871421/true/false/false/false</t>
         </is>
       </c>
       <c r="V28" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
         </is>
       </c>
       <c r="W28" s="5" t="inlineStr">
@@ -3654,12 +3646,12 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'Etat de la Jeunesse de l'Education Populaire et du Sport spécialité "animation socio-éducative ou culturelle mention "coordination de projets" - RNCP 39930 spécialité "animation socio-éducative ou culturel mention "coordination de projets</t>
+          <t>Agent de prévention et de sécurité - Titre à finalité professionnelle (TFP APS)</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+          <t>Global pro formation (Global pro formation (GPF))</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
@@ -3669,12 +3661,12 @@
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+          <t>Blue Concept | 16 Rue Marcel Dutartre | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 379 heures (dont 70 heures en entreprise)</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -3684,17 +3676,17 @@
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>https://arfatsema.catalogueformpro.com/3/dejeps-17/2857880/diplome-detat-de-la-jeunesse-de-leducation-populaire-et-du-sport-dejeps-17-specialite-animation-soci/registration?session_id=2846144</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>globalproformation@gmail.com</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>globalproformation@gmail.com</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
@@ -3709,12 +3701,12 @@
       </c>
       <c r="M29" s="7" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0666139535</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0666139535</t>
         </is>
       </c>
       <c r="O29" s="7" t="inlineStr">
@@ -3724,7 +3716,7 @@
       </c>
       <c r="P29" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q29" s="7" t="inlineStr">
@@ -3735,17 +3727,17 @@
       <c r="R29" s="7" t="inlineStr"/>
       <c r="S29" s="7" t="inlineStr">
         <is>
-          <t>BC1: Animer et accompagner une équipe dans le champ du sport ou de l'animation Animer une équipe en structure d'éducation populaire : enjeux éthiques, valeurs et spécificités Réaliser un diagnostic des ressources humaines de son périmètre d'intervention Animer une équipe en structure d'éducation populaire : organisation, cadre légal, réglementation et procédures Diversité et inclusion : analyser les besoins et mettre en place une organisation adaptée Management participatif : développer le pouvoir d'agir d'une équipe Management participatif : outils et pratiques Accompagner une équipe: médiation et gestion de conflits Accompagner une équipe : émancipation et développement de l'autonomie Dynamique de groupe Animer un processus démocratique Projet d'action formative et conception de séance formative Droit du travail/Droit social Communication non violente Outils d'animation collective Outils d'accompagnement individuel Accompagner la vulnérabilité Dialogue social et syndical Responsabilité du coordinateur Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? BC2: Concevoir un projet d'action dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Education Populaire Rapport de domination Le numérique comme un fait social Esprit critique Culture politique Démocratie et contre pouvoir Pouvoir d'agir ou devoir d'agir? Diagnostic et enjeux De l'attribution d'une place à une culture de la participation Famille et éducation Connaissance des institutions publics et relation aux association ingéniérie sociale Portrait de territoire Mesure de l'impact social BC3 : Mettre en oeuvre et évaluer un projet d'action Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie de projet Mesure de l'impact social Accompagner la vulnérabilité La protection de l'Enfance en France Outils participatifs Intelligence artificielle et fonction de coordination BC4 : Développer les partenariats opérationnelles et contribuer aux dynamiques institutionnelles dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Connaissance des institutions publics et relation aux associations Démocratie et contre pouvoir Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie sociale Outils participatifs | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Théorie : SST : Protéger, Examiner (saignement, étouffement, conscience et respiration) et alerter (alerte et message d'accueil) La déontologie de l'agent de sécurité Les services publics de police et gendarmerie, le CNAPS Le cadre légal de la profession, le code pénal et le code de procédure pénale La sûreté de l'État Les armes Mise en sûreté et neutralisation des armes Prévention et actes terrorisme L'accueil, le contrôle d'accès, le contrôle visuel et la palpation de sécurité La prise en compte d'un poste de contrôle de sécurité et les consignes La protection du travailleur Isolé Le circuit de vérification La gestion des alarmes intrusion et incendie, la vidéo et la télésurveillance (surveillance et gardiennage) Les techniques d'information, de communication et la gestion des conflits L'incendie et les risques majeurs Le risque électrique (initiation) Le cadre légal et la problématique de l'activité d'événementiel La définition du terrorisme (historique, mécanisme, méthodologie et modes opératoires) Les différentes menaces terroristes et les niveaux de risque associés La prévention des actes de terrorisme par la reconnaissance des comportements suspects (profiling) et de la radicalisation violente L'action en cas d'attaque et suivant le type d'attaque (actes réflexes, mesures de mise en sécurité immédiate) Le combat en dernier recours L'alerte et la facilitation de l'intervention des forces de l'ordre La sécurisation d'une zone dans l'urgence, risque de sur-attentat et post-attentat. Pratique : Mise en pratique SST CQP APS: Code de la sécurité intérieure Code pénal et libertés publiques Déontologie professionnelle Secours à personnes (SST) Situations conflictuelles et résolution de conflit Consignes, compte rendu et rapport Gestion des risques majeurs, électriques, incendie Gestion d'alarmes Technique d'information et de communication Préparation d'une mission Gestion de conflit Contrôle d'accès Poste de contrôle de sécurité Rondes Palpation de sécurité et inspection de bagages Télésurveillance et vidéo protection Sensibilisation aux risques terroristes Examen : en cours de formation UV 1 (secourisme) : le candidat sera déclaré apte ou inapte en fonction des résultats de la grille d'évaluation conforme aux procédures de validation de l'INRS. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
         </is>
       </c>
       <c r="T29" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | DEJEPS spécialité animation socio-éducative ou culturelle mention coordination de projets</t>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Agent de prévention et de sécurité</t>
         </is>
       </c>
       <c r="U29" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880827/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11870188/true/false/false/false</t>
         </is>
       </c>
       <c r="V29" s="7" t="inlineStr">
@@ -3767,27 +3759,27 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Créez votre vignoble bio de raisin de table, rentable et résilient - Devenez autonome pour produire et vendre votre propre raisin de table bio</t>
+          <t>Diplôme d'Etat de la Jeunesse de l'Education Populaire et du Sport spécialité "animation socio-éducative ou culturelle mention "coordination de projets" - RNCP 39930 spécialité "animation socio-éducative ou culturel mention "coordination de projets</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>SARL Agri-learn éditions</t>
+          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>69001 Lyon</t>
+          <t>69100 Villeurbanne</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 69001 Lyon | France</t>
+          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Durée de 9 heures</t>
+          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -3797,17 +3789,17 @@
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://arfatsema.catalogueformpro.com/3/dejeps-17/2857880/diplome-detat-de-la-jeunesse-de-leducation-populaire-et-du-sport-dejeps-17-specialite-animation-soci/registration?session_id=2846144</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -3822,15 +3814,19 @@
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0478031711</t>
         </is>
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>0620021214</t>
-        </is>
-      </c>
-      <c r="O30" s="5" t="inlineStr"/>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="O30" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P30" s="5" t="inlineStr">
         <is>
           <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
@@ -3838,24 +3834,28 @@
       </c>
       <c r="Q30" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R30" s="5" t="inlineStr"/>
       <c r="S30" s="5" t="inlineStr">
         <is>
-          <t>1. Taille de la vigne Principes de taille (formation et production) Techniques de taille douce Entretien et corrections2. Modes de conduite Choix du système (lyre, gable, plan vertical. Comparaison des conduites Adaptation au contexte pédoclimatique3. Fertilité des sols Gestion du sol (travail / non-travail) Irrigation Maintien de la fertilité en bio4. Travaux du vignoble Protection contre maladies et ravageurs Calendrier des interventions Conduite sous abri (tunnel)5. Choix des plants Sélection des variétés Choix du porte-greffe Adaptation au marché et au terroir6. Plantation Préparation du sol Étapes de plantation Coûts et organisation7. Récolte et commercialisation Récolte et conservation Organisation du travail Valorisation et vente8. Protection du vignoble en bio Biocontrôle et PNPP Réduction des intrants Stratégies alternatives9. Gestion des maladies et ravageurs Identification des principaux risques Prévention et lutte adaptée10. Pilotage des traitements Stratégie cuivre / soufre Optimisation des doses11. Approche agroécologique Biodiversité fonctionnelle Variétés résistantes | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T30" s="5" t="inlineStr"/>
+          <t>BC1: Animer et accompagner une équipe dans le champ du sport ou de l'animation Animer une équipe en structure d'éducation populaire : enjeux éthiques, valeurs et spécificités Réaliser un diagnostic des ressources humaines de son périmètre d'intervention Animer une équipe en structure d'éducation populaire : organisation, cadre légal, réglementation et procédures Diversité et inclusion : analyser les besoins et mettre en place une organisation adaptée Management participatif : développer le pouvoir d'agir d'une équipe Management participatif : outils et pratiques Accompagner une équipe: médiation et gestion de conflits Accompagner une équipe : émancipation et développement de l'autonomie Dynamique de groupe Animer un processus démocratique Projet d'action formative et conception de séance formative Droit du travail/Droit social Communication non violente Outils d'animation collective Outils d'accompagnement individuel Accompagner la vulnérabilité Dialogue social et syndical Responsabilité du coordinateur Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? BC2: Concevoir un projet d'action dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Education Populaire Rapport de domination Le numérique comme un fait social Esprit critique Culture politique Démocratie et contre pouvoir Pouvoir d'agir ou devoir d'agir? Diagnostic et enjeux De l'attribution d'une place à une culture de la participation Famille et éducation Connaissance des institutions publics et relation aux association ingéniérie sociale Portrait de territoire Mesure de l'impact social BC3 : Mettre en oeuvre et évaluer un projet d'action Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie de projet Mesure de l'impact social Accompagner la vulnérabilité La protection de l'Enfance en France Outils participatifs Intelligence artificielle et fonction de coordination BC4 : Développer les partenariats opérationnelles et contribuer aux dynamiques institutionnelles dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Connaissance des institutions publics et relation aux associations Démocratie et contre pouvoir Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie sociale Outils participatifs | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T30" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | DEJEPS spécialité animation socio-éducative ou culturelle mention coordination de projets</t>
+        </is>
+      </c>
       <c r="U30" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11870193/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11880827/true/false/false/false</t>
         </is>
       </c>
       <c r="V30" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W30" s="5" t="inlineStr">
@@ -3872,27 +3872,27 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
+          <t>Créez votre vignoble bio de raisin de table, rentable et résilient - Devenez autonome pour produire et vendre votre propre raisin de table bio</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>UCPA Formation</t>
+          <t>SARL Agri-learn éditions</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>69200 Vénissieux</t>
+          <t>69001 Lyon</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>16 Avenue Dr Georges Levy | 69200 Vénissieux | France</t>
+          <t>Formation a distance | 69001 Lyon | France</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1267 heures (dont 637 heures en entreprise)</t>
+          <t>Durée de 9 heures</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -3907,12 +3907,12 @@
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>ucpa-formation@ucpa.asso.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>ucpa-formation@ucpa.asso.fr | fgehant@ucpa.asso.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
@@ -3927,43 +3927,35 @@
       </c>
       <c r="M31" s="7" t="inlineStr">
         <is>
-          <t>0642833617</t>
+          <t>0620021214</t>
         </is>
       </c>
       <c r="N31" s="7" t="inlineStr">
         <is>
-          <t>0642833617</t>
-        </is>
-      </c>
-      <c r="O31" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="O31" s="7" t="inlineStr"/>
       <c r="P31" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q31" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R31" s="7" t="inlineStr"/>
       <c r="S31" s="7" t="inlineStr">
         <is>
-          <t>Unité capitalisable (UC) - 1. Encadrer tout public dans tout lieu et toute structureUnité capitalisable (UC) - 2. Mettre en œuvre un projet d'animation s'inscrivant dans le projet de la structureUnité capitalisable (UC) - 3. Conduire une séance, un cycle d'animation ou d'apprentissage dans le champ des activités aquatiques et de la natationUnité capitalisable (UC) - 4. Mobiliser les techniques des activités aquatiques et de la natation pour mettre en œuvre une séance ou un cycle d'apprentissage | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T31" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
-        </is>
-      </c>
+          <t>1. Taille de la vigne Principes de taille (formation et production) Techniques de taille douce Entretien et corrections2. Modes de conduite Choix du système (lyre, gable, plan vertical. Comparaison des conduites Adaptation au contexte pédoclimatique3. Fertilité des sols Gestion du sol (travail / non-travail) Irrigation Maintien de la fertilité en bio4. Travaux du vignoble Protection contre maladies et ravageurs Calendrier des interventions Conduite sous abri (tunnel)5. Choix des plants Sélection des variétés Choix du porte-greffe Adaptation au marché et au terroir6. Plantation Préparation du sol Étapes de plantation Coûts et organisation7. Récolte et commercialisation Récolte et conservation Organisation du travail Valorisation et vente8. Protection du vignoble en bio Biocontrôle et PNPP Réduction des intrants Stratégies alternatives9. Gestion des maladies et ravageurs Identification des principaux risques Prévention et lutte adaptée10. Pilotage des traitements Stratégie cuivre / soufre Optimisation des doses11. Approche agroécologique Biodiversité fonctionnelle Variétés résistantes | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T31" s="7" t="inlineStr"/>
       <c r="U31" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11447001/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11870193/true/false/false/false</t>
         </is>
       </c>
       <c r="V31" s="7" t="inlineStr">
@@ -3985,27 +3977,27 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'aide-soignant - DEAS</t>
+          <t>BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>UCPA Formation</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>69200 Vénissieux</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+          <t>16 Avenue Dr Georges Levy | 69200 Vénissieux | France</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1540 heures (dont 770 heures en entreprise)</t>
+          <t>Durée de 1267 heures (dont 637 heures en entreprise)</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
@@ -4015,17 +4007,17 @@
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=aide-soignant</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>ucpa-formation@ucpa.asso.fr</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>ucpa-formation@ucpa.asso.fr | fgehant@ucpa.asso.fr</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
@@ -4040,12 +4032,12 @@
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0642833617</t>
         </is>
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0642833617</t>
         </is>
       </c>
       <c r="O32" s="5" t="inlineStr">
@@ -4066,17 +4058,17 @@
       <c r="R32" s="5" t="inlineStr"/>
       <c r="S32" s="5" t="inlineStr">
         <is>
-          <t>La formation conduisant au diplôme d'État d'aide-soignant, 17 semaines d'enseignement théoriques organisées autour de 8 modules : Accompagnement d'une personne dans les activités de la vie quotidienne L'état clinique d'une personne Les soins Ergonomie Relation Communication Hygiène des locaux hospitaliers Transmission des informations Organisation du travail Les titulaires du DE d'auxiliaire de puériculture, du DE d'aide médico-psychologique, du DE d'auxiliaire de vie sociale ou de la MC aide à domicile, sont dispensés de certaines unités de formation. La formation comprend également 6 stages d'une durée totale de 24 semaines en milieu hospitalier ou extra-hospitalier. Possibilité d'effectuer la formation en initial ou en apprentissage. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Unité capitalisable (UC) - 1. Encadrer tout public dans tout lieu et toute structureUnité capitalisable (UC) - 2. Mettre en œuvre un projet d'animation s'inscrivant dans le projet de la structureUnité capitalisable (UC) - 3. Conduire une séance, un cycle d'animation ou d'apprentissage dans le champ des activités aquatiques et de la natationUnité capitalisable (UC) - 4. Mobiliser les techniques des activités aquatiques et de la natation pour mettre en œuvre une séance ou un cycle d'apprentissage | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T32" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'aide-soignant</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
         </is>
       </c>
       <c r="U32" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11533549/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11447001/true/false/false/false</t>
         </is>
       </c>
       <c r="V32" s="5" t="inlineStr">
@@ -4098,12 +4090,12 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>Diplôme d'État d'aide-soignant - DEAS</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -4113,12 +4105,12 @@
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 1540 heures (dont 770 heures en entreprise)</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -4128,17 +4120,17 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=aide-soignant</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
@@ -4153,12 +4145,12 @@
       </c>
       <c r="M33" s="7" t="inlineStr">
         <is>
-          <t>0472117979</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N33" s="7" t="inlineStr">
         <is>
-          <t>0472117979</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O33" s="7" t="inlineStr">
@@ -4177,15 +4169,19 @@
         </is>
       </c>
       <c r="R33" s="7" t="inlineStr"/>
-      <c r="S33" s="7" t="inlineStr"/>
+      <c r="S33" s="7" t="inlineStr">
+        <is>
+          <t>La formation conduisant au diplôme d'État d'aide-soignant, 17 semaines d'enseignement théoriques organisées autour de 8 modules : Accompagnement d'une personne dans les activités de la vie quotidienne L'état clinique d'une personne Les soins Ergonomie Relation Communication Hygiène des locaux hospitaliers Transmission des informations Organisation du travail Les titulaires du DE d'auxiliaire de puériculture, du DE d'aide médico-psychologique, du DE d'auxiliaire de vie sociale ou de la MC aide à domicile, sont dispensés de certaines unités de formation. La formation comprend également 6 stages d'une durée totale de 24 semaines en milieu hospitalier ou extra-hospitalier. Possibilité d'effectuer la formation en initial ou en apprentissage. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T33" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'aide-soignant</t>
         </is>
       </c>
       <c r="U33" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11817055/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11533549/true/false/false/true</t>
         </is>
       </c>
       <c r="V33" s="7" t="inlineStr">
@@ -4207,12 +4203,12 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'assistant de service social - DE ASS</t>
+          <t>Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -4222,12 +4218,12 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 avenue Lacassagne | Croix Rouge francaise | 69003 Lyon 3e | France</t>
+          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Durée de 3420 heures (dont 1680 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
@@ -4237,17 +4233,17 @@
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=assistant%20de%20service%20social</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
@@ -4262,12 +4258,12 @@
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0472117979</t>
         </is>
       </c>
       <c r="N34" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0472117979</t>
         </is>
       </c>
       <c r="O34" s="5" t="inlineStr">
@@ -4289,12 +4285,12 @@
       <c r="S34" s="5" t="inlineStr"/>
       <c r="T34" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U34" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11672249/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11817055/true/false/false/false</t>
         </is>
       </c>
       <c r="V34" s="5" t="inlineStr">
@@ -4316,27 +4312,27 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'éducateur spécialisé</t>
+          <t>Diplôme d'État d'assistant de service social - DE ASS</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales (ARFRIPS - Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales)</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>69009 Lyon 9e</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>10 Impasse Pierre Baizet | 69009 Lyon 9e | France</t>
+          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 avenue Lacassagne | Croix Rouge francaise | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Durée de 3442 heures (dont 1925 heures en entreprise)</t>
+          <t>Durée de 3420 heures (dont 1680 heures en entreprise)</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -4346,17 +4342,17 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=assistant%20de%20service%20social</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>info@arfrips.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>info@arfrips.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
@@ -4371,12 +4367,12 @@
       </c>
       <c r="M35" s="7" t="inlineStr">
         <is>
-          <t>0478699090</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N35" s="7" t="inlineStr">
         <is>
-          <t>0478699090</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O35" s="7" t="inlineStr">
@@ -4398,17 +4394,17 @@
       <c r="S35" s="7" t="inlineStr"/>
       <c r="T35" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur spécialisé</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
         </is>
       </c>
       <c r="U35" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11737248/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11672249/true/false/false/false</t>
         </is>
       </c>
       <c r="V35" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
         </is>
       </c>
       <c r="W35" s="7" t="inlineStr">
@@ -4425,27 +4421,27 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet - RNCP 39931 - spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+          <t>Diplôme d'État d'éducateur spécialisé</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+          <t>Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales (ARFRIPS - Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales)</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>69009 Lyon 9e</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+          <t>10 Impasse Pierre Baizet | 69009 Lyon 9e | France</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 3442 heures (dont 1925 heures en entreprise)</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
@@ -4455,17 +4451,17 @@
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>https://arfatsema.catalogueformpro.com/2/desjeps-17/2858060/desjeps-17-diplome-detat-superieur-de-la-jeunesse-de-leducation-populaire-et-du-sport-specialite-ani</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>info@arfrips.fr</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>info@arfrips.fr</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
@@ -4480,12 +4476,12 @@
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0478699090</t>
         </is>
       </c>
       <c r="N36" s="5" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0478699090</t>
         </is>
       </c>
       <c r="O36" s="5" t="inlineStr">
@@ -4495,7 +4491,7 @@
       </c>
       <c r="P36" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q36" s="5" t="inlineStr">
@@ -4504,19 +4500,15 @@
         </is>
       </c>
       <c r="R36" s="5" t="inlineStr"/>
-      <c r="S36" s="5" t="inlineStr">
-        <is>
-          <t>BC1 : Construire, avec les instances de gouvernance, la stratégie de développement d'une structure dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Éducation Populaire Culture Politique Rapport de domination Pouvoir d'Agir et Vulnérabilité Esprit critique Transformation social/rapport sociaux Le numérique comme un fait social Nouvel esprit du capitalisme Laicité et valeurs de la République Violence sexiste violences sexuelles Ingénierie social en lien avec la structure Réaliser un diagnostic RH et financier Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Elaboration de la stratégie de développement en lien avec les instances de gouvernance Animer un processus démocratique Démocratie et contre pouvoir BC2 : Concevoir et diriger un projet de développement de la structure Cartographie des relations et l'environnement de son association Ingénierie du projet Processus d'évaluation dans une démarche partagée et participative Outils participatifs Outils de communication Utilité sociale BC3 : Manager l'équipe et gérer les ressources humaines ( et la démarche Qualité, Sécurité, Santé au Travail et Environnement d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Gestion des ressources humaines en structures d'éducation populaire : enjeux, éthique et complexités associative Articulation employeur bénévole - direction dans la gestion des ressources humaines : définition d'une politique RH et organisation des délégations de pouvoir Gérer l'équipe au quotidien : accompagnement, régulation et gestion conflits Analyse des pratiques en co-développement Développer le pouvoir d'agir des salariés Attractivité, recrutement, intégration et fidélisation des salariés Diversité, inclusion et égalité professionnelle au sein de son organisation Assurer la GPEC, la formation et la gestion des carrières dans un alignement éthique Le financement de la formation professionnelle Qualité de vie Santé sécurité au travail Droit du travail/Droit social Dialogue social/dialogue syndical Cadre général des RPS Démarche prévention et outils BC4 : Assurer la gestion financière, matérielle et administrative d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Comprendre les fondamentaux de la situation financière Initiation à l'analyse financière associative ou de structure d'intérêt général Identifier les leviers de financement Construire des scénarios budgétaires et faire des arbitrages Élaborer un plan d'action financier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
+      <c r="S36" s="5" t="inlineStr"/>
       <c r="T36" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur spécialisé</t>
         </is>
       </c>
       <c r="U36" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880835/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11737248/true/false/false/false</t>
         </is>
       </c>
       <c r="V36" s="5" t="inlineStr">
@@ -4538,27 +4530,27 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Créer sa ferme en circuit court : transformation, commercialisation et communication</t>
+          <t>DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet - RNCP 39931 - spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>SARL Agri-learn éditions</t>
+          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>69001 Lyon</t>
+          <t>69100 Villeurbanne</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 69001 Lyon | France</t>
+          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Durée de 20 heures</t>
+          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -4568,17 +4560,17 @@
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://arfatsema.catalogueformpro.com/2/desjeps-17/2858060/desjeps-17-diplome-detat-superieur-de-la-jeunesse-de-leducation-populaire-et-du-sport-specialite-ani</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="K37" s="7" t="inlineStr">
@@ -4593,15 +4585,19 @@
       </c>
       <c r="M37" s="7" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0478031711</t>
         </is>
       </c>
       <c r="N37" s="7" t="inlineStr">
         <is>
-          <t>0620021214</t>
-        </is>
-      </c>
-      <c r="O37" s="7" t="inlineStr"/>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="O37" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P37" s="7" t="inlineStr">
         <is>
           <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
@@ -4609,19 +4605,23 @@
       </c>
       <c r="Q37" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R37" s="7" t="inlineStr"/>
       <c r="S37" s="7" t="inlineStr">
         <is>
-          <t>Cette formation s'appuie sur plusieurs compétences essentielles : Stratégie commerciale et étude de marché : définir son offre, ses volumes, ses prix et ses circuits de vente Techniques de vente : maîtriser les étapes clés pour convaincre et fidéliser les clients Transformation des produits agricoles : valoriser ses matières premières pour créer de la valeur ajoutée Hygiène et réglementation : garantir la sécurité sanitaire dans les ateliers de transformation Communication et prospection : développer sa clientèle et promouvoir ses produits Valorisation des produits : savoir parler de ses produits et les mettre en avant (ex : dégustation) L'ensemble permet d'acquérir une vision globale du fonctionnement d'une ferme en circuit court, de la production jusqu'à la vente. 3 heures de visio avec les experts sont prévues dans le cursus. | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T37" s="7" t="inlineStr"/>
+          <t>BC1 : Construire, avec les instances de gouvernance, la stratégie de développement d'une structure dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Éducation Populaire Culture Politique Rapport de domination Pouvoir d'Agir et Vulnérabilité Esprit critique Transformation social/rapport sociaux Le numérique comme un fait social Nouvel esprit du capitalisme Laicité et valeurs de la République Violence sexiste violences sexuelles Ingénierie social en lien avec la structure Réaliser un diagnostic RH et financier Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Elaboration de la stratégie de développement en lien avec les instances de gouvernance Animer un processus démocratique Démocratie et contre pouvoir BC2 : Concevoir et diriger un projet de développement de la structure Cartographie des relations et l'environnement de son association Ingénierie du projet Processus d'évaluation dans une démarche partagée et participative Outils participatifs Outils de communication Utilité sociale BC3 : Manager l'équipe et gérer les ressources humaines ( et la démarche Qualité, Sécurité, Santé au Travail et Environnement d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Gestion des ressources humaines en structures d'éducation populaire : enjeux, éthique et complexités associative Articulation employeur bénévole - direction dans la gestion des ressources humaines : définition d'une politique RH et organisation des délégations de pouvoir Gérer l'équipe au quotidien : accompagnement, régulation et gestion conflits Analyse des pratiques en co-développement Développer le pouvoir d'agir des salariés Attractivité, recrutement, intégration et fidélisation des salariés Diversité, inclusion et égalité professionnelle au sein de son organisation Assurer la GPEC, la formation et la gestion des carrières dans un alignement éthique Le financement de la formation professionnelle Qualité de vie Santé sécurité au travail Droit du travail/Droit social Dialogue social/dialogue syndical Cadre général des RPS Démarche prévention et outils BC4 : Assurer la gestion financière, matérielle et administrative d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Comprendre les fondamentaux de la situation financière Initiation à l'analyse financière associative ou de structure d'intérêt général Identifier les leviers de financement Construire des scénarios budgétaires et faire des arbitrages Élaborer un plan d'action financier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T37" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+        </is>
+      </c>
       <c r="U37" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880868/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11880835/true/false/false/false</t>
         </is>
       </c>
       <c r="V37" s="7" t="inlineStr">
@@ -4643,27 +4643,27 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Titre professionnel administrateur d'infrastructures sécurisées (FOAD)</t>
+          <t>Créer sa ferme en circuit court : transformation, commercialisation et communication</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>STUDI</t>
+          <t>SARL Agri-learn éditions</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>69001 Lyon</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Formation a distance | 69001 Lyon | France</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Durée de 947 heures (dont 350 heures en entreprise)</t>
+          <t>Durée de 20 heures</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
@@ -4678,12 +4678,12 @@
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>contact@studi.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>contact@studi.fr | conseiller-formation.aoft@studi.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
@@ -4698,22 +4698,18 @@
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
-          <t>0174888555</t>
+          <t>0620021214</t>
         </is>
       </c>
       <c r="N38" s="5" t="inlineStr">
         <is>
-          <t>0174888555</t>
-        </is>
-      </c>
-      <c r="O38" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="O38" s="5" t="inlineStr"/>
       <c r="P38" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q38" s="5" t="inlineStr">
@@ -4724,25 +4720,134 @@
       <c r="R38" s="5" t="inlineStr"/>
       <c r="S38" s="5" t="inlineStr">
         <is>
+          <t>Cette formation s'appuie sur plusieurs compétences essentielles : Stratégie commerciale et étude de marché : définir son offre, ses volumes, ses prix et ses circuits de vente Techniques de vente : maîtriser les étapes clés pour convaincre et fidéliser les clients Transformation des produits agricoles : valoriser ses matières premières pour créer de la valeur ajoutée Hygiène et réglementation : garantir la sécurité sanitaire dans les ateliers de transformation Communication et prospection : développer sa clientèle et promouvoir ses produits Valorisation des produits : savoir parler de ses produits et les mettre en avant (ex : dégustation) L'ensemble permet d'acquérir une vision globale du fonctionnement d'une ferme en circuit court, de la production jusqu'à la vente. 3 heures de visio avec les experts sont prévues dans le cursus. | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T38" s="5" t="inlineStr"/>
+      <c r="U38" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11880868/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V38" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W38" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Titre professionnel administrateur d'infrastructures sécurisées (FOAD)</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>STUDI</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>75004 Paris</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Formation a distance | 75004 Paris | France</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 947 heures (dont 350 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>contact@studi.fr</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>contact@studi.fr | conseiller-formation.aoft@studi.fr</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L39" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M39" s="7" t="inlineStr">
+        <is>
+          <t>0174888555</t>
+        </is>
+      </c>
+      <c r="N39" s="7" t="inlineStr">
+        <is>
+          <t>0174888555</t>
+        </is>
+      </c>
+      <c r="O39" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P39" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par France Travail</t>
+        </is>
+      </c>
+      <c r="Q39" s="7" t="inlineStr">
+        <is>
+          <t>À distance</t>
+        </is>
+      </c>
+      <c r="R39" s="7" t="inlineStr"/>
+      <c r="S39" s="7" t="inlineStr">
+        <is>
           <t>Administrer et sécuriser les infrastructures Les bonnes pratiques dans l'administration des infrastructures Utiliser un logiciel de gestion centralisé : GLPI Configurer le routage Administrer et sécuriser le réseau Automatiser les tâches d'administration Administrer et sécuriser les systèmes Les bases des serveurs virtualisés Administrer et sécuriser une infrastructure de serveurs virtualisée Gérer des containersConcevoir et mettre en œuvre une solution en réponse à un besoin d'évolution Les bases des solutions techniques Proposer une solution informatique répondant à des besoins nouveaux Mettre en production des évolutions de l'infrastructure Les bases de la supervision Superviser la disponibilité de l'infrastructure et en présenter les résultats Mesurer les performances et la disponibilité de l'infrastructureParticiper à la gestion de la cybersécurité Les bases de la cybersécurité Participer à la mesure et à l'analyse du niveau de sécurité de l'infrastructure Participer à l'élaboration et à la mise en œuvre de la politique de sécurité Participer à la détection et au traitement des incidents de sécurité | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
-      <c r="T38" s="5" t="inlineStr">
+      <c r="T39" s="7" t="inlineStr">
         <is>
           <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel administrateur d'infrastructures sécurisées</t>
         </is>
       </c>
-      <c r="U38" s="5" t="inlineStr">
+      <c r="U39" s="7" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/detail/11590088/true/false/true/false</t>
         </is>
       </c>
-      <c r="V38" s="5" t="inlineStr">
+      <c r="V39" s="7" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
-      <c r="W38" s="5" t="inlineStr">
+      <c r="W39" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-07-15
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1255,7 +1255,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1360,7 +1360,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,32 +1683,32 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Ecole de la 2ème Chance (E2C)</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>04000 Digne-les-Bains</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>4 avenue de Verdun | https://www.iap.asso.fr/ | 04000 Digne-les-Bains | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1100 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1718,17 +1718,17 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>https://www.iap.asso.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>contact@iap.asso.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>contact@iap.asso.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1743,40 +1743,48 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>04 92 87 46 10</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>04 92 87 46 10</t>
-        </is>
-      </c>
-      <c r="O11" s="7" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>Programme non communiqué | Organisme | Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04 | https://www.iap.asso.fr/ | Lieu de la formation</t>
-        </is>
-      </c>
-      <c r="T11" s="7" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+        </is>
+      </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10685143/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1788,32 +1796,32 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Titre professionnel secrétaire assistant médico-administratif (FOAD)</t>
+          <t>Ecole de la 2ème Chance (E2C)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>04000 Digne-les-Bains</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>4 avenue de Verdun | https://www.iap.asso.fr/ | 04000 Digne-les-Bains | France</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1084 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 1100 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1823,17 +1831,17 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.iap.asso.fr/</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>contact@iap.asso.fr</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>contact@iap.asso.fr</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1848,48 +1856,40 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>04 92 87 46 10</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>04 92 87 46 10</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr"/>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q12" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>7 projets professionnalisants vous permettront d'acquérir les compétences citées au dessus par la pratique.Vous réaliserez les projets suivants :P1 - Démarrez votre formation de secrétaire assistant médico-administratifP2 - Niveau 1 : Maîtrisez l'accueil et la gestion administrative en milieu médicalP3 - Niveau 2 : Développez vos compétences en rédaction, communication et outils numériques en milieuP4 - Réalisez votre mission en entrepriseP5 - Niveau 3 : Optimisez l'organisation, la sécuritéet la gestion des données sensibles en milieu médicalP6 - Niveau 4 : Améliorez la gestion des communications, données et environnements sanitairesP7 - Préparez votre fin de formation de secrétaire assistant médico-administratif | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T12" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel secrétaire assistant médico-administratif</t>
-        </is>
-      </c>
+          <t>Programme non communiqué | Organisme | Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04 | https://www.iap.asso.fr/ | Lieu de la formation</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr"/>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10685143/true/false/false/false</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -1906,7 +1906,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Formation au concours d'ATSEM</t>
+          <t>Titre professionnel secrétaire assistant médico-administratif (FOAD)</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Durée de 346 heures</t>
+          <t>Durée de 1084 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1969,7 +1969,11 @@
           <t>0180888030</t>
         </is>
       </c>
-      <c r="O13" s="7" t="inlineStr"/>
+      <c r="O13" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -1983,13 +1987,17 @@
       <c r="R13" s="7" t="inlineStr"/>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T13" s="7" t="inlineStr"/>
+          <t>7 projets professionnalisants vous permettront d'acquérir les compétences citées au dessus par la pratique.Vous réaliserez les projets suivants :P1 - Démarrez votre formation de secrétaire assistant médico-administratifP2 - Niveau 1 : Maîtrisez l'accueil et la gestion administrative en milieu médicalP3 - Niveau 2 : Développez vos compétences en rédaction, communication et outils numériques en milieuP4 - Réalisez votre mission en entrepriseP5 - Niveau 3 : Optimisez l'organisation, la sécuritéet la gestion des données sensibles en milieu médicalP6 - Niveau 4 : Améliorez la gestion des communications, données et environnements sanitairesP7 - Préparez votre fin de formation de secrétaire assistant médico-administratif | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T13" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel secrétaire assistant médico-administratif</t>
+        </is>
+      </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/false</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
@@ -2011,12 +2019,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Concours d'atsem (FOAD)</t>
+          <t>Formation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -2031,7 +2039,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
+          <t>Durée de 346 heures</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -2046,12 +2054,12 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -2066,12 +2074,12 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr"/>
@@ -2088,13 +2096,13 @@
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
+          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T14" s="5" t="inlineStr"/>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/false</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
@@ -2116,7 +2124,7 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Concours d'atsem (FOAD)</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
@@ -2136,7 +2144,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2156,7 +2164,7 @@
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -2179,11 +2187,7 @@
           <t>0366060201</t>
         </is>
       </c>
-      <c r="O15" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+      <c r="O15" s="7" t="inlineStr"/>
       <c r="P15" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -2197,17 +2201,13 @@
       <c r="R15" s="7" t="inlineStr"/>
       <c r="S15" s="7" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T15" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
+          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T15" s="7" t="inlineStr"/>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/false</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
@@ -2229,12 +2229,12 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Préparation au concours d'ATSEM</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>AFEC (Siège)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2264,12 +2264,12 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -2284,15 +2284,19 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>0153368844</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>0153368844</t>
-        </is>
-      </c>
-      <c r="O16" s="5" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P16" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -2306,13 +2310,17 @@
       <c r="R16" s="5" t="inlineStr"/>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC (Siège) | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T16" s="5" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T16" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+        </is>
+      </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/false</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
@@ -2334,12 +2342,12 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
+          <t>Préparation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>AFEC (Siège)</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -2354,7 +2362,7 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2369,12 +2377,12 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -2389,12 +2397,12 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="O17" s="7" t="inlineStr"/>
@@ -2411,13 +2419,13 @@
       <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="7" t="inlineStr">
         <is>
-          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC (Siège) | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T17" s="7" t="inlineStr"/>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/false</t>
         </is>
       </c>
       <c r="V17" s="7" t="inlineStr">
@@ -2439,7 +2447,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
+          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -2459,7 +2467,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -2516,13 +2524,13 @@
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T18" s="5" t="inlineStr"/>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/false</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
@@ -2544,7 +2552,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
+          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -2564,7 +2572,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2621,13 +2629,13 @@
       <c r="R19" s="7" t="inlineStr"/>
       <c r="S19" s="7" t="inlineStr">
         <is>
-          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T19" s="7" t="inlineStr"/>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/false</t>
         </is>
       </c>
       <c r="V19" s="7" t="inlineStr">
@@ -2649,12 +2657,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>BP option aménagements paysagers</t>
+          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -2669,7 +2677,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -2684,12 +2692,12 @@
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr | cecile.iribarne@educagri.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -2704,19 +2712,15 @@
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>0479264427</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>0479264427</t>
-        </is>
-      </c>
-      <c r="O20" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr"/>
       <c r="P20" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -2730,17 +2734,13 @@
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T20" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
-        </is>
-      </c>
+          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/false</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
@@ -2762,12 +2762,12 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>CAP Fleuriste</t>
+          <t>BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -2797,12 +2797,12 @@
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr | cecile.iribarne@educagri.fr</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
@@ -2817,12 +2817,12 @@
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0479264427</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0479264427</t>
         </is>
       </c>
       <c r="O21" s="7" t="inlineStr">
@@ -2843,17 +2843,17 @@
       <c r="R21" s="7" t="inlineStr"/>
       <c r="S21" s="7" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/false</t>
         </is>
       </c>
       <c r="V21" s="7" t="inlineStr">
@@ -2870,32 +2870,32 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>E2C - Ecole de la Deuxième Chance</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Ecole de la Deuxième Chance Grand Hainaut</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>02140 Vervins</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Ecole de la deuxième chance - site de VERVINS | 3 Place des Anciens Combattants | 02140 Vervins | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1400 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -2910,12 +2910,12 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>c.renaud@e2cgrandhainaut.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>c.renaud@e2cgrandhainaut.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -2930,40 +2930,48 @@
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>0375310010</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>0375310010</t>
-        </is>
-      </c>
-      <c r="O22" s="5" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P22" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q22" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>Savoir fondamentauxOrientation et démarches professionnelsSocialisation et développement personnelAlternance en entreprise (près de 30% du temps)Des outils pédagogiques de liaison, d'évaluation et de suivi9 mois maximum + 12 mois de suivi post-parcours | Organisme | Ecole de la Deuxième Chance Grand Hainaut | Lieu de la formation | Ecole de la deuxième chance - site de VERVINS</t>
-        </is>
-      </c>
-      <c r="T22" s="5" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T22" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+        </is>
+      </c>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11072382/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/false</t>
         </is>
       </c>
       <c r="V22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W22" s="5" t="inlineStr">
@@ -2975,32 +2983,32 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>CAP Fleuriste</t>
+          <t>E2C - Ecole de la Deuxième Chance</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>Ecole de la Deuxième Chance Grand Hainaut</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>02140 Vervins</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Ecole de la deuxième chance - site de VERVINS | 3 Place des Anciens Combattants | 02140 Vervins | France</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 1400 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -3015,12 +3023,12 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>c.renaud@e2cgrandhainaut.fr</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>c.renaud@e2cgrandhainaut.fr</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -3035,48 +3043,40 @@
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0375310010</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O23" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0375310010</t>
+        </is>
+      </c>
+      <c r="O23" s="7" t="inlineStr"/>
       <c r="P23" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q23" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R23" s="7" t="inlineStr"/>
       <c r="S23" s="7" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T23" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
-        </is>
-      </c>
+          <t>Savoir fondamentauxOrientation et démarches professionnelsSocialisation et développement personnelAlternance en entreprise (près de 30% du temps)Des outils pédagogiques de liaison, d'évaluation et de suivi9 mois maximum + 12 mois de suivi post-parcours | Organisme | Ecole de la Deuxième Chance Grand Hainaut | Lieu de la formation | Ecole de la deuxième chance - site de VERVINS</t>
+        </is>
+      </c>
+      <c r="T23" s="7" t="inlineStr"/>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11072382/true/false/false/true</t>
         </is>
       </c>
       <c r="V23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-01&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W23" s="7" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-07-16
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseFranceTravail" displayName="BaseFranceTravail" ref="A1:W39" headerRowCount="1">
-  <autoFilter ref="A1:W39"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseFranceTravail" displayName="BaseFranceTravail" ref="A1:W40" headerRowCount="1">
+  <autoFilter ref="A1:W40"/>
   <tableColumns count="23">
     <tableColumn id="1" name="zone"/>
     <tableColumn id="2" name="formation"/>
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W39"/>
+  <dimension ref="A1:W40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1255,7 +1255,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1360,7 +1360,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,32 +1683,32 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>CAP Fleuriste</t>
+          <t>Ecole de la 2ème Chance (E2C)</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>Objectif 2ème chance - métropôle nice côte d'azur - ecole de la deuxième chance des alpes maritimes - odc nca - e2c</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>06200 Nice</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>455 Promenade des Anglais | Porte Arenas | 06200 Nice | France</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 1100 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1723,12 +1723,12 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>contact@e2cnicecotedazur.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>contact@e2cnicecotedazur.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1743,48 +1743,40 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>04 12 05 20 05</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O11" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>04 12 05 20 05</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="inlineStr"/>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T11" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
-        </is>
-      </c>
+          <t>Programme non communiqué | Organisme | Objectif 2ème chance - métropôle nice côte d'azur - ecole de la deuxième chance des alpes maritimes - odc nca - e2c | Lieu de la formation | 455 Promenade des Anglais</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr"/>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10681643/true/false/false/false</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1796,32 +1788,32 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>05</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Ecole de la 2ème Chance (E2C)</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>04000 Digne-les-Bains</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>4 avenue de Verdun | https://www.iap.asso.fr/ | 04000 Digne-les-Bains | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1100 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1831,17 +1823,17 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>https://www.iap.asso.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>contact@iap.asso.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>contact@iap.asso.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1856,40 +1848,48 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>04 92 87 46 10</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>04 92 87 46 10</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q12" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>Programme non communiqué | Organisme | Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04 | https://www.iap.asso.fr/ | Lieu de la formation</t>
-        </is>
-      </c>
-      <c r="T12" s="5" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+        </is>
+      </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10685143/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -1901,32 +1901,32 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Titre professionnel secrétaire assistant médico-administratif (FOAD)</t>
+          <t>Ecole de la 2ème Chance (E2C)</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>04000 Digne-les-Bains</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>4 avenue de Verdun | https://www.iap.asso.fr/ | 04000 Digne-les-Bains | France</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1084 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 1100 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1936,17 +1936,17 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.iap.asso.fr/</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>contact@iap.asso.fr</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>contact@iap.asso.fr</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
@@ -1961,48 +1961,40 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>04 92 87 46 10</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="O13" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>04 92 87 46 10</t>
+        </is>
+      </c>
+      <c r="O13" s="7" t="inlineStr"/>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R13" s="7" t="inlineStr"/>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>7 projets professionnalisants vous permettront d'acquérir les compétences citées au dessus par la pratique.Vous réaliserez les projets suivants :P1 - Démarrez votre formation de secrétaire assistant médico-administratifP2 - Niveau 1 : Maîtrisez l'accueil et la gestion administrative en milieu médicalP3 - Niveau 2 : Développez vos compétences en rédaction, communication et outils numériques en milieuP4 - Réalisez votre mission en entrepriseP5 - Niveau 3 : Optimisez l'organisation, la sécuritéet la gestion des données sensibles en milieu médicalP6 - Niveau 4 : Améliorez la gestion des communications, données et environnements sanitairesP7 - Préparez votre fin de formation de secrétaire assistant médico-administratif | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T13" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel secrétaire assistant médico-administratif</t>
-        </is>
-      </c>
+          <t>Programme non communiqué | Organisme | Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04 | https://www.iap.asso.fr/ | Lieu de la formation</t>
+        </is>
+      </c>
+      <c r="T13" s="7" t="inlineStr"/>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10685143/true/false/false/false</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W13" s="7" t="inlineStr">
@@ -2019,7 +2011,7 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Formation au concours d'ATSEM</t>
+          <t>Titre professionnel secrétaire assistant médico-administratif (FOAD)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -2039,7 +2031,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Durée de 346 heures</t>
+          <t>Durée de 1084 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -2082,7 +2074,11 @@
           <t>0180888030</t>
         </is>
       </c>
-      <c r="O14" s="5" t="inlineStr"/>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -2096,13 +2092,17 @@
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T14" s="5" t="inlineStr"/>
+          <t>7 projets professionnalisants vous permettront d'acquérir les compétences citées au dessus par la pratique.Vous réaliserez les projets suivants :P1 - Démarrez votre formation de secrétaire assistant médico-administratifP2 - Niveau 1 : Maîtrisez l'accueil et la gestion administrative en milieu médicalP3 - Niveau 2 : Développez vos compétences en rédaction, communication et outils numériques en milieuP4 - Réalisez votre mission en entrepriseP5 - Niveau 3 : Optimisez l'organisation, la sécuritéet la gestion des données sensibles en milieu médicalP6 - Niveau 4 : Améliorez la gestion des communications, données et environnements sanitairesP7 - Préparez votre fin de formation de secrétaire assistant médico-administratif | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T14" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel secrétaire assistant médico-administratif</t>
+        </is>
+      </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/false</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
@@ -2124,12 +2124,12 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Concours d'atsem (FOAD)</t>
+          <t>Formation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -2144,7 +2144,7 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
+          <t>Durée de 346 heures</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2159,12 +2159,12 @@
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -2179,12 +2179,12 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O15" s="7" t="inlineStr"/>
@@ -2201,13 +2201,13 @@
       <c r="R15" s="7" t="inlineStr"/>
       <c r="S15" s="7" t="inlineStr">
         <is>
-          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
+          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T15" s="7" t="inlineStr"/>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/false</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Concours d'atsem (FOAD)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -2292,11 +2292,7 @@
           <t>0366060201</t>
         </is>
       </c>
-      <c r="O16" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+      <c r="O16" s="5" t="inlineStr"/>
       <c r="P16" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -2310,17 +2306,13 @@
       <c r="R16" s="5" t="inlineStr"/>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T16" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
+          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T16" s="5" t="inlineStr"/>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/false</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
@@ -2342,12 +2334,12 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Préparation au concours d'ATSEM</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>AFEC (Siège)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -2362,7 +2354,7 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2377,12 +2369,12 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -2397,15 +2389,19 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>0153368844</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>0153368844</t>
-        </is>
-      </c>
-      <c r="O17" s="7" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P17" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -2419,13 +2415,17 @@
       <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="7" t="inlineStr">
         <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC (Siège) | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T17" s="7" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T17" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+        </is>
+      </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/false</t>
         </is>
       </c>
       <c r="V17" s="7" t="inlineStr">
@@ -2447,12 +2447,12 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
+          <t>Préparation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>AFEC (Siège)</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -2482,12 +2482,12 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -2502,12 +2502,12 @@
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="O18" s="5" t="inlineStr"/>
@@ -2524,13 +2524,13 @@
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC (Siège) | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T18" s="5" t="inlineStr"/>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/false</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
+          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -2572,7 +2572,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2629,13 +2629,13 @@
       <c r="R19" s="7" t="inlineStr"/>
       <c r="S19" s="7" t="inlineStr">
         <is>
-          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T19" s="7" t="inlineStr"/>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/false</t>
         </is>
       </c>
       <c r="V19" s="7" t="inlineStr">
@@ -2657,7 +2657,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
+          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -2677,7 +2677,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -2734,13 +2734,13 @@
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/false</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
@@ -2762,12 +2762,12 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>BP option aménagements paysagers</t>
+          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -2782,7 +2782,7 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -2797,12 +2797,12 @@
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr | cecile.iribarne@educagri.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
@@ -2817,19 +2817,15 @@
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>0479264427</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>0479264427</t>
-        </is>
-      </c>
-      <c r="O21" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O21" s="7" t="inlineStr"/>
       <c r="P21" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -2843,17 +2839,13 @@
       <c r="R21" s="7" t="inlineStr"/>
       <c r="S21" s="7" t="inlineStr">
         <is>
-          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T21" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
-        </is>
-      </c>
+          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T21" s="7" t="inlineStr"/>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/false</t>
         </is>
       </c>
       <c r="V21" s="7" t="inlineStr">
@@ -2875,12 +2867,12 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>CAP Fleuriste</t>
+          <t>BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -2895,7 +2887,7 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -2910,12 +2902,12 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr | cecile.iribarne@educagri.fr</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -2930,12 +2922,12 @@
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0479264427</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0479264427</t>
         </is>
       </c>
       <c r="O22" s="5" t="inlineStr">
@@ -2956,17 +2948,17 @@
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T22" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/false</t>
         </is>
       </c>
       <c r="V22" s="5" t="inlineStr">
@@ -2983,32 +2975,32 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>E2C - Ecole de la Deuxième Chance</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Ecole de la Deuxième Chance Grand Hainaut</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>02140 Vervins</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Ecole de la deuxième chance - site de VERVINS | 3 Place des Anciens Combattants | 02140 Vervins | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1400 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -3023,12 +3015,12 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>c.renaud@e2cgrandhainaut.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>c.renaud@e2cgrandhainaut.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -3043,40 +3035,48 @@
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>0375310010</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>0375310010</t>
-        </is>
-      </c>
-      <c r="O23" s="7" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P23" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q23" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R23" s="7" t="inlineStr"/>
       <c r="S23" s="7" t="inlineStr">
         <is>
-          <t>Savoir fondamentauxOrientation et démarches professionnelsSocialisation et développement personnelAlternance en entreprise (près de 30% du temps)Des outils pédagogiques de liaison, d'évaluation et de suivi9 mois maximum + 12 mois de suivi post-parcours | Organisme | Ecole de la Deuxième Chance Grand Hainaut | Lieu de la formation | Ecole de la deuxième chance - site de VERVINS</t>
-        </is>
-      </c>
-      <c r="T23" s="7" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T23" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+        </is>
+      </c>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11072382/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/false</t>
         </is>
       </c>
       <c r="V23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W23" s="7" t="inlineStr">
@@ -3088,32 +3088,32 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Préparation au concours d'adjoint administratif d'État principal de 2ème classe</t>
+          <t>E2C - Ecole de la Deuxième Chance</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school)</t>
+          <t>Ecole de la Deuxième Chance Grand Hainaut</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>02140 Vervins</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Ecole de la deuxième chance - site de VERVINS | 3 Place des Anciens Combattants | 02140 Vervins | France</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Durée de 335 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 1400 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -3128,12 +3128,12 @@
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>foad@skillandyou.com</t>
+          <t>c.renaud@e2cgrandhainaut.fr</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>foad@skillandyou.com</t>
+          <t>c.renaud@e2cgrandhainaut.fr</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -3148,40 +3148,40 @@
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>0146006878</t>
+          <t>0375310010</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
         <is>
-          <t>0146006878</t>
+          <t>0375310010</t>
         </is>
       </c>
       <c r="O24" s="5" t="inlineStr"/>
       <c r="P24" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q24" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R24" s="5" t="inlineStr"/>
       <c r="S24" s="5" t="inlineStr">
         <is>
-          <t>Votre intégration - Guide d'intégration - Bienvenue dans votre formation - Guide Métier Adjoint administratif d'État principal de 2ème classe - Guide de la formation - Guide des épreuves - Le concours d'adjoint administratif d'État principal de 2ème classe Aide à la réalisation de vos documents professionnels Compléter votre livret de suivi des compétences professionnelles Retranscrire et ordonner les idées principales d'un texte Annales corrigées Épreuves blanches Solliciter les connaissances fondamentales pour le concours Comprendre l'administration française Comprendre le fonctionnement des institutions françaises Acquérir des connaissances en français Acquérir une bonne culture générale Mathématiques Les tests d'aptitudes verbales Annales corrigées Épreuves blanches Mobiliser les compétences professionnelles de l'adjoint administratif d'État Bureautique Épreuves blanches Techniques et recherche d'emploi/stage Sensibilisation au développement durable | Organisme | Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school) | Lieu de la formation | Formation a distance</t>
+          <t>Savoir fondamentauxOrientation et démarches professionnelsSocialisation et développement personnelAlternance en entreprise (près de 30% du temps)Des outils pédagogiques de liaison, d'évaluation et de suivi9 mois maximum + 12 mois de suivi post-parcours | Organisme | Ecole de la Deuxième Chance Grand Hainaut | Lieu de la formation | Ecole de la deuxième chance - site de VERVINS</t>
         </is>
       </c>
       <c r="T24" s="5" t="inlineStr"/>
       <c r="U24" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11205913/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11072382/true/false/false/true</t>
         </is>
       </c>
       <c r="V24" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W24" s="5" t="inlineStr">
@@ -3198,12 +3198,12 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Certification CLOE français langue étrangère - spécialité hôtellerie Restauration niveau A2 vers B1 (FOAD)</t>
+          <t>Préparation au concours d'adjoint administratif d'État principal de 2ème classe</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Nepsod Evolution</t>
+          <t>Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school)</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -3218,7 +3218,7 @@
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Durée de 331 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 335 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>accueil@nepsod.com</t>
+          <t>foad@skillandyou.com</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>accueil@nepsod.com</t>
+          <t>foad@skillandyou.com</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
@@ -3253,19 +3253,15 @@
       </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>0474639587</t>
+          <t>0146006878</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>0474639587</t>
-        </is>
-      </c>
-      <c r="O25" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0146006878</t>
+        </is>
+      </c>
+      <c r="O25" s="7" t="inlineStr"/>
       <c r="P25" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -3279,17 +3275,13 @@
       <c r="R25" s="7" t="inlineStr"/>
       <c r="S25" s="7" t="inlineStr">
         <is>
-          <t>Accueil et initiation à la formation (1h30) - Module FLE visée insertion professionnelle : chercher un emploi, présenter son métier, présenter ses projets, interagir avec ses collègues, manipuler les outils numériques (120h30) - Module FOS Hôtellerie Restauration :découvrir la cuisine, travailler en cuisine, identifier les besoins d'un client, présenter des produits et services, gérer les réclamations (50h) Module environnement social et culturel : vie quotidienne et relations sociales, loisirs, patrimoine, citoyenneté et engagement (43h) Module Préparation et recherche de stage en entreprise (14h) Période de stage en entreprise (35 h) Module remise à niveau numérique (35 h maximum) Module accompagnement à l'après-formation (21h maximum) Module Préparation et passage de la certification CLOE (10h) Bilan final (1h) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T25" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Certification CLOE français langue étrangère</t>
-        </is>
-      </c>
+          <t>Votre intégration - Guide d'intégration - Bienvenue dans votre formation - Guide Métier Adjoint administratif d'État principal de 2ème classe - Guide de la formation - Guide des épreuves - Le concours d'adjoint administratif d'État principal de 2ème classe Aide à la réalisation de vos documents professionnels Compléter votre livret de suivi des compétences professionnelles Retranscrire et ordonner les idées principales d'un texte Annales corrigées Épreuves blanches Solliciter les connaissances fondamentales pour le concours Comprendre l'administration française Comprendre le fonctionnement des institutions françaises Acquérir des connaissances en français Acquérir une bonne culture générale Mathématiques Les tests d'aptitudes verbales Annales corrigées Épreuves blanches Mobiliser les compétences professionnelles de l'adjoint administratif d'État Bureautique Épreuves blanches Techniques et recherche d'emploi/stage Sensibilisation au développement durable | Organisme | Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school) | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T25" s="7" t="inlineStr"/>
       <c r="U25" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11576792/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11205913/true/false/true/true</t>
         </is>
       </c>
       <c r="V25" s="7" t="inlineStr">
@@ -3311,27 +3303,27 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière) - DEI</t>
+          <t>Certification CLOE français langue étrangère - spécialité hôtellerie Restauration niveau A2 vers B1 (FOAD)</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Nepsod Evolution</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 331 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -3346,12 +3338,12 @@
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>accueil@nepsod.com</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>accueil@nepsod.com</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
@@ -3366,12 +3358,12 @@
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0474639587</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0474639587</t>
         </is>
       </c>
       <c r="O26" s="5" t="inlineStr">
@@ -3381,28 +3373,28 @@
       </c>
       <c r="P26" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q26" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R26" s="5" t="inlineStr"/>
       <c r="S26" s="5" t="inlineStr">
         <is>
-          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail (bureautique,recherche documentaire, rédaction de documents écrits, communication, anglais) La formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de1 800h, sous la forme de cours magistraux (750 h) travaux dirigés (1 050 h) le travail personnel guidé (suivi pédagogique, temps personnel guidé, supervision, travaux entre étudiants- 300 h) la formation clinique de 2 100 h le travail personnel complémentaire est estimé à 900 heures environ, soit 300 h par an. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Accueil et initiation à la formation (1h30) - Module FLE visée insertion professionnelle : chercher un emploi, présenter son métier, présenter ses projets, interagir avec ses collègues, manipuler les outils numériques (120h30) - Module FOS Hôtellerie Restauration :découvrir la cuisine, travailler en cuisine, identifier les besoins d'un client, présenter des produits et services, gérer les réclamations (50h) Module environnement social et culturel : vie quotidienne et relations sociales, loisirs, patrimoine, citoyenneté et engagement (43h) Module Préparation et recherche de stage en entreprise (14h) Période de stage en entreprise (35 h) Module remise à niveau numérique (35 h maximum) Module accompagnement à l'après-formation (21h maximum) Module Préparation et passage de la certification CLOE (10h) Bilan final (1h) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T26" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Certification CLOE français langue étrangère</t>
         </is>
       </c>
       <c r="U26" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11533526/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11576792/true/false/true/false</t>
         </is>
       </c>
       <c r="V26" s="5" t="inlineStr">
@@ -3424,27 +3416,27 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État de technicien de laboratoire médical</t>
+          <t>Diplôme d'État d'infirmier(ière) - DEI</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Association des Fondateurs et Protecteurs de l'Institut Catholique de Lyon (AFPICL) (UCLy - Institut Catholique de Lyon)</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>69002 Lyon 2e</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>10 place des Archives | 69002 Lyon 2e | France</t>
+          <t>115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1120 heures</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -3459,12 +3451,12 @@
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>fp@univ-catholyon.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>fp@univ-catholyon.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
@@ -3479,12 +3471,12 @@
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>0472325134</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>0472325134</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O27" s="7" t="inlineStr">
@@ -3503,15 +3495,19 @@
         </is>
       </c>
       <c r="R27" s="7" t="inlineStr"/>
-      <c r="S27" s="7" t="inlineStr"/>
+      <c r="S27" s="7" t="inlineStr">
+        <is>
+          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail (bureautique,recherche documentaire, rédaction de documents écrits, communication, anglais) La formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de1 800h, sous la forme de cours magistraux (750 h) travaux dirigés (1 050 h) le travail personnel guidé (suivi pédagogique, temps personnel guidé, supervision, travaux entre étudiants- 300 h) la formation clinique de 2 100 h le travail personnel complémentaire est estimé à 900 heures environ, soit 300 h par an. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État de technicien de laboratoire médical</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U27" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11026378/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11533526/true/false/false/false</t>
         </is>
       </c>
       <c r="V27" s="7" t="inlineStr">
@@ -3533,27 +3529,27 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'ambulancier</t>
+          <t>Diplôme d'État de technicien de laboratoire médical</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+          <t>Association des Fondateurs et Protecteurs de l'Institut Catholique de Lyon (AFPICL) (UCLy - Institut Catholique de Lyon)</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>69002 Lyon 2e</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+          <t>10 place des Archives | 69002 Lyon 2e | France</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Durée de 801 heures (dont 245 heures en entreprise)</t>
+          <t>Durée de 1120 heures</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -3568,12 +3564,12 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>fp@univ-catholyon.fr</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>fp@univ-catholyon.fr</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
@@ -3588,12 +3584,12 @@
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>0472117903</t>
+          <t>0472325134</t>
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>0472117903</t>
+          <t>0472325134</t>
         </is>
       </c>
       <c r="O28" s="5" t="inlineStr">
@@ -3612,24 +3608,20 @@
         </is>
       </c>
       <c r="R28" s="5" t="inlineStr"/>
-      <c r="S28" s="5" t="inlineStr">
-        <is>
-          <t>Non renseigne | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
+      <c r="S28" s="5" t="inlineStr"/>
       <c r="T28" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'ambulancier</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État de technicien de laboratoire médical</t>
         </is>
       </c>
       <c r="U28" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11871421/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11026378/true/false/false/false</t>
         </is>
       </c>
       <c r="V28" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W28" s="5" t="inlineStr">
@@ -3646,27 +3638,27 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Agent de prévention et de sécurité - Titre à finalité professionnelle (TFP APS)</t>
+          <t>Diplôme d'État d'ambulancier</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Global pro formation (Global pro formation (GPF))</t>
+          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>Blue Concept | 16 Rue Marcel Dutartre | 69100 Villeurbanne | France</t>
+          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Durée de 379 heures (dont 70 heures en entreprise)</t>
+          <t>Durée de 801 heures (dont 245 heures en entreprise)</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -3681,12 +3673,12 @@
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>globalproformation@gmail.com</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>globalproformation@gmail.com</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
@@ -3701,12 +3693,12 @@
       </c>
       <c r="M29" s="7" t="inlineStr">
         <is>
-          <t>0666139535</t>
+          <t>0472117903</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr">
         <is>
-          <t>0666139535</t>
+          <t>0472117903</t>
         </is>
       </c>
       <c r="O29" s="7" t="inlineStr">
@@ -3716,7 +3708,7 @@
       </c>
       <c r="P29" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q29" s="7" t="inlineStr">
@@ -3727,22 +3719,22 @@
       <c r="R29" s="7" t="inlineStr"/>
       <c r="S29" s="7" t="inlineStr">
         <is>
-          <t>Théorie : SST : Protéger, Examiner (saignement, étouffement, conscience et respiration) et alerter (alerte et message d'accueil) La déontologie de l'agent de sécurité Les services publics de police et gendarmerie, le CNAPS Le cadre légal de la profession, le code pénal et le code de procédure pénale La sûreté de l'État Les armes Mise en sûreté et neutralisation des armes Prévention et actes terrorisme L'accueil, le contrôle d'accès, le contrôle visuel et la palpation de sécurité La prise en compte d'un poste de contrôle de sécurité et les consignes La protection du travailleur Isolé Le circuit de vérification La gestion des alarmes intrusion et incendie, la vidéo et la télésurveillance (surveillance et gardiennage) Les techniques d'information, de communication et la gestion des conflits L'incendie et les risques majeurs Le risque électrique (initiation) Le cadre légal et la problématique de l'activité d'événementiel La définition du terrorisme (historique, mécanisme, méthodologie et modes opératoires) Les différentes menaces terroristes et les niveaux de risque associés La prévention des actes de terrorisme par la reconnaissance des comportements suspects (profiling) et de la radicalisation violente L'action en cas d'attaque et suivant le type d'attaque (actes réflexes, mesures de mise en sécurité immédiate) Le combat en dernier recours L'alerte et la facilitation de l'intervention des forces de l'ordre La sécurisation d'une zone dans l'urgence, risque de sur-attentat et post-attentat. Pratique : Mise en pratique SST CQP APS: Code de la sécurité intérieure Code pénal et libertés publiques Déontologie professionnelle Secours à personnes (SST) Situations conflictuelles et résolution de conflit Consignes, compte rendu et rapport Gestion des risques majeurs, électriques, incendie Gestion d'alarmes Technique d'information et de communication Préparation d'une mission Gestion de conflit Contrôle d'accès Poste de contrôle de sécurité Rondes Palpation de sécurité et inspection de bagages Télésurveillance et vidéo protection Sensibilisation aux risques terroristes Examen : en cours de formation UV 1 (secourisme) : le candidat sera déclaré apte ou inapte en fonction des résultats de la grille d'évaluation conforme aux procédures de validation de l'INRS. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
+          <t>Non renseigne | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T29" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Agent de prévention et de sécurité</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'ambulancier</t>
         </is>
       </c>
       <c r="U29" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11870188/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11871421/true/false/false/false</t>
         </is>
       </c>
       <c r="V29" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
         </is>
       </c>
       <c r="W29" s="7" t="inlineStr">
@@ -3759,12 +3751,12 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'Etat de la Jeunesse de l'Education Populaire et du Sport spécialité "animation socio-éducative ou culturelle mention "coordination de projets" - RNCP 39930 spécialité "animation socio-éducative ou culturel mention "coordination de projets</t>
+          <t>Agent de prévention et de sécurité - Titre à finalité professionnelle (TFP APS)</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+          <t>Global pro formation (Global pro formation (GPF))</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -3774,12 +3766,12 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+          <t>Blue Concept | 16 Rue Marcel Dutartre | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 379 heures (dont 70 heures en entreprise)</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -3789,17 +3781,17 @@
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>https://arfatsema.catalogueformpro.com/3/dejeps-17/2857880/diplome-detat-de-la-jeunesse-de-leducation-populaire-et-du-sport-dejeps-17-specialite-animation-soci/registration?session_id=2846144</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>globalproformation@gmail.com</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>globalproformation@gmail.com</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -3814,12 +3806,12 @@
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0666139535</t>
         </is>
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0666139535</t>
         </is>
       </c>
       <c r="O30" s="5" t="inlineStr">
@@ -3829,7 +3821,7 @@
       </c>
       <c r="P30" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q30" s="5" t="inlineStr">
@@ -3840,17 +3832,17 @@
       <c r="R30" s="5" t="inlineStr"/>
       <c r="S30" s="5" t="inlineStr">
         <is>
-          <t>BC1: Animer et accompagner une équipe dans le champ du sport ou de l'animation Animer une équipe en structure d'éducation populaire : enjeux éthiques, valeurs et spécificités Réaliser un diagnostic des ressources humaines de son périmètre d'intervention Animer une équipe en structure d'éducation populaire : organisation, cadre légal, réglementation et procédures Diversité et inclusion : analyser les besoins et mettre en place une organisation adaptée Management participatif : développer le pouvoir d'agir d'une équipe Management participatif : outils et pratiques Accompagner une équipe: médiation et gestion de conflits Accompagner une équipe : émancipation et développement de l'autonomie Dynamique de groupe Animer un processus démocratique Projet d'action formative et conception de séance formative Droit du travail/Droit social Communication non violente Outils d'animation collective Outils d'accompagnement individuel Accompagner la vulnérabilité Dialogue social et syndical Responsabilité du coordinateur Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? BC2: Concevoir un projet d'action dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Education Populaire Rapport de domination Le numérique comme un fait social Esprit critique Culture politique Démocratie et contre pouvoir Pouvoir d'agir ou devoir d'agir? Diagnostic et enjeux De l'attribution d'une place à une culture de la participation Famille et éducation Connaissance des institutions publics et relation aux association ingéniérie sociale Portrait de territoire Mesure de l'impact social BC3 : Mettre en oeuvre et évaluer un projet d'action Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie de projet Mesure de l'impact social Accompagner la vulnérabilité La protection de l'Enfance en France Outils participatifs Intelligence artificielle et fonction de coordination BC4 : Développer les partenariats opérationnelles et contribuer aux dynamiques institutionnelles dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Connaissance des institutions publics et relation aux associations Démocratie et contre pouvoir Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie sociale Outils participatifs | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Théorie : SST : Protéger, Examiner (saignement, étouffement, conscience et respiration) et alerter (alerte et message d'accueil) La déontologie de l'agent de sécurité Les services publics de police et gendarmerie, le CNAPS Le cadre légal de la profession, le code pénal et le code de procédure pénale La sûreté de l'État Les armes Mise en sûreté et neutralisation des armes Prévention et actes terrorisme L'accueil, le contrôle d'accès, le contrôle visuel et la palpation de sécurité La prise en compte d'un poste de contrôle de sécurité et les consignes La protection du travailleur Isolé Le circuit de vérification La gestion des alarmes intrusion et incendie, la vidéo et la télésurveillance (surveillance et gardiennage) Les techniques d'information, de communication et la gestion des conflits L'incendie et les risques majeurs Le risque électrique (initiation) Le cadre légal et la problématique de l'activité d'événementiel La définition du terrorisme (historique, mécanisme, méthodologie et modes opératoires) Les différentes menaces terroristes et les niveaux de risque associés La prévention des actes de terrorisme par la reconnaissance des comportements suspects (profiling) et de la radicalisation violente L'action en cas d'attaque et suivant le type d'attaque (actes réflexes, mesures de mise en sécurité immédiate) Le combat en dernier recours L'alerte et la facilitation de l'intervention des forces de l'ordre La sécurisation d'une zone dans l'urgence, risque de sur-attentat et post-attentat. Pratique : Mise en pratique SST CQP APS: Code de la sécurité intérieure Code pénal et libertés publiques Déontologie professionnelle Secours à personnes (SST) Situations conflictuelles et résolution de conflit Consignes, compte rendu et rapport Gestion des risques majeurs, électriques, incendie Gestion d'alarmes Technique d'information et de communication Préparation d'une mission Gestion de conflit Contrôle d'accès Poste de contrôle de sécurité Rondes Palpation de sécurité et inspection de bagages Télésurveillance et vidéo protection Sensibilisation aux risques terroristes Examen : en cours de formation UV 1 (secourisme) : le candidat sera déclaré apte ou inapte en fonction des résultats de la grille d'évaluation conforme aux procédures de validation de l'INRS. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
         </is>
       </c>
       <c r="T30" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | DEJEPS spécialité animation socio-éducative ou culturelle mention coordination de projets</t>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Agent de prévention et de sécurité</t>
         </is>
       </c>
       <c r="U30" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880827/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11870188/true/false/false/false</t>
         </is>
       </c>
       <c r="V30" s="5" t="inlineStr">
@@ -3872,27 +3864,27 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Créez votre vignoble bio de raisin de table, rentable et résilient - Devenez autonome pour produire et vendre votre propre raisin de table bio</t>
+          <t>Diplôme d'Etat de la Jeunesse de l'Education Populaire et du Sport spécialité "animation socio-éducative ou culturelle mention "coordination de projets" - RNCP 39930 spécialité "animation socio-éducative ou culturel mention "coordination de projets</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>SARL Agri-learn éditions</t>
+          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>69001 Lyon</t>
+          <t>69100 Villeurbanne</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 69001 Lyon | France</t>
+          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Durée de 9 heures</t>
+          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -3902,17 +3894,17 @@
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://arfatsema.catalogueformpro.com/3/dejeps-17/2857880/diplome-detat-de-la-jeunesse-de-leducation-populaire-et-du-sport-dejeps-17-specialite-animation-soci/registration?session_id=2846144</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
@@ -3927,15 +3919,19 @@
       </c>
       <c r="M31" s="7" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0478031711</t>
         </is>
       </c>
       <c r="N31" s="7" t="inlineStr">
         <is>
-          <t>0620021214</t>
-        </is>
-      </c>
-      <c r="O31" s="7" t="inlineStr"/>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="O31" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P31" s="7" t="inlineStr">
         <is>
           <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
@@ -3943,24 +3939,28 @@
       </c>
       <c r="Q31" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R31" s="7" t="inlineStr"/>
       <c r="S31" s="7" t="inlineStr">
         <is>
-          <t>1. Taille de la vigne Principes de taille (formation et production) Techniques de taille douce Entretien et corrections2. Modes de conduite Choix du système (lyre, gable, plan vertical. Comparaison des conduites Adaptation au contexte pédoclimatique3. Fertilité des sols Gestion du sol (travail / non-travail) Irrigation Maintien de la fertilité en bio4. Travaux du vignoble Protection contre maladies et ravageurs Calendrier des interventions Conduite sous abri (tunnel)5. Choix des plants Sélection des variétés Choix du porte-greffe Adaptation au marché et au terroir6. Plantation Préparation du sol Étapes de plantation Coûts et organisation7. Récolte et commercialisation Récolte et conservation Organisation du travail Valorisation et vente8. Protection du vignoble en bio Biocontrôle et PNPP Réduction des intrants Stratégies alternatives9. Gestion des maladies et ravageurs Identification des principaux risques Prévention et lutte adaptée10. Pilotage des traitements Stratégie cuivre / soufre Optimisation des doses11. Approche agroécologique Biodiversité fonctionnelle Variétés résistantes | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T31" s="7" t="inlineStr"/>
+          <t>BC1: Animer et accompagner une équipe dans le champ du sport ou de l'animation Animer une équipe en structure d'éducation populaire : enjeux éthiques, valeurs et spécificités Réaliser un diagnostic des ressources humaines de son périmètre d'intervention Animer une équipe en structure d'éducation populaire : organisation, cadre légal, réglementation et procédures Diversité et inclusion : analyser les besoins et mettre en place une organisation adaptée Management participatif : développer le pouvoir d'agir d'une équipe Management participatif : outils et pratiques Accompagner une équipe: médiation et gestion de conflits Accompagner une équipe : émancipation et développement de l'autonomie Dynamique de groupe Animer un processus démocratique Projet d'action formative et conception de séance formative Droit du travail/Droit social Communication non violente Outils d'animation collective Outils d'accompagnement individuel Accompagner la vulnérabilité Dialogue social et syndical Responsabilité du coordinateur Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? BC2: Concevoir un projet d'action dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Education Populaire Rapport de domination Le numérique comme un fait social Esprit critique Culture politique Démocratie et contre pouvoir Pouvoir d'agir ou devoir d'agir? Diagnostic et enjeux De l'attribution d'une place à une culture de la participation Famille et éducation Connaissance des institutions publics et relation aux association ingéniérie sociale Portrait de territoire Mesure de l'impact social BC3 : Mettre en oeuvre et évaluer un projet d'action Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie de projet Mesure de l'impact social Accompagner la vulnérabilité La protection de l'Enfance en France Outils participatifs Intelligence artificielle et fonction de coordination BC4 : Développer les partenariats opérationnelles et contribuer aux dynamiques institutionnelles dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Connaissance des institutions publics et relation aux associations Démocratie et contre pouvoir Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie sociale Outils participatifs | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T31" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | DEJEPS spécialité animation socio-éducative ou culturelle mention coordination de projets</t>
+        </is>
+      </c>
       <c r="U31" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11870193/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11880827/true/false/false/false</t>
         </is>
       </c>
       <c r="V31" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W31" s="7" t="inlineStr">
@@ -3977,27 +3977,27 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
+          <t>Créez votre vignoble bio de raisin de table, rentable et résilient - Devenez autonome pour produire et vendre votre propre raisin de table bio</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>UCPA Formation</t>
+          <t>SARL Agri-learn éditions</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>69200 Vénissieux</t>
+          <t>69001 Lyon</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>16 Avenue Dr Georges Levy | 69200 Vénissieux | France</t>
+          <t>Formation a distance | 69001 Lyon | France</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1267 heures (dont 637 heures en entreprise)</t>
+          <t>Durée de 9 heures</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
@@ -4012,12 +4012,12 @@
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>ucpa-formation@ucpa.asso.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>ucpa-formation@ucpa.asso.fr | fgehant@ucpa.asso.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
@@ -4032,43 +4032,35 @@
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>0642833617</t>
+          <t>0620021214</t>
         </is>
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>0642833617</t>
-        </is>
-      </c>
-      <c r="O32" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="O32" s="5" t="inlineStr"/>
       <c r="P32" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q32" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R32" s="5" t="inlineStr"/>
       <c r="S32" s="5" t="inlineStr">
         <is>
-          <t>Unité capitalisable (UC) - 1. Encadrer tout public dans tout lieu et toute structureUnité capitalisable (UC) - 2. Mettre en œuvre un projet d'animation s'inscrivant dans le projet de la structureUnité capitalisable (UC) - 3. Conduire une séance, un cycle d'animation ou d'apprentissage dans le champ des activités aquatiques et de la natationUnité capitalisable (UC) - 4. Mobiliser les techniques des activités aquatiques et de la natation pour mettre en œuvre une séance ou un cycle d'apprentissage | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T32" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
-        </is>
-      </c>
+          <t>1. Taille de la vigne Principes de taille (formation et production) Techniques de taille douce Entretien et corrections2. Modes de conduite Choix du système (lyre, gable, plan vertical. Comparaison des conduites Adaptation au contexte pédoclimatique3. Fertilité des sols Gestion du sol (travail / non-travail) Irrigation Maintien de la fertilité en bio4. Travaux du vignoble Protection contre maladies et ravageurs Calendrier des interventions Conduite sous abri (tunnel)5. Choix des plants Sélection des variétés Choix du porte-greffe Adaptation au marché et au terroir6. Plantation Préparation du sol Étapes de plantation Coûts et organisation7. Récolte et commercialisation Récolte et conservation Organisation du travail Valorisation et vente8. Protection du vignoble en bio Biocontrôle et PNPP Réduction des intrants Stratégies alternatives9. Gestion des maladies et ravageurs Identification des principaux risques Prévention et lutte adaptée10. Pilotage des traitements Stratégie cuivre / soufre Optimisation des doses11. Approche agroécologique Biodiversité fonctionnelle Variétés résistantes | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T32" s="5" t="inlineStr"/>
       <c r="U32" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11447001/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11870193/true/false/false/false</t>
         </is>
       </c>
       <c r="V32" s="5" t="inlineStr">
@@ -4090,27 +4082,27 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'aide-soignant - DEAS</t>
+          <t>BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>UCPA Formation</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>69200 Vénissieux</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+          <t>16 Avenue Dr Georges Levy | 69200 Vénissieux | France</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1540 heures (dont 770 heures en entreprise)</t>
+          <t>Durée de 1267 heures (dont 637 heures en entreprise)</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -4120,17 +4112,17 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=aide-soignant</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>ucpa-formation@ucpa.asso.fr</t>
         </is>
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>ucpa-formation@ucpa.asso.fr | fgehant@ucpa.asso.fr</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
@@ -4145,12 +4137,12 @@
       </c>
       <c r="M33" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0642833617</t>
         </is>
       </c>
       <c r="N33" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0642833617</t>
         </is>
       </c>
       <c r="O33" s="7" t="inlineStr">
@@ -4171,17 +4163,17 @@
       <c r="R33" s="7" t="inlineStr"/>
       <c r="S33" s="7" t="inlineStr">
         <is>
-          <t>La formation conduisant au diplôme d'État d'aide-soignant, 17 semaines d'enseignement théoriques organisées autour de 8 modules : Accompagnement d'une personne dans les activités de la vie quotidienne L'état clinique d'une personne Les soins Ergonomie Relation Communication Hygiène des locaux hospitaliers Transmission des informations Organisation du travail Les titulaires du DE d'auxiliaire de puériculture, du DE d'aide médico-psychologique, du DE d'auxiliaire de vie sociale ou de la MC aide à domicile, sont dispensés de certaines unités de formation. La formation comprend également 6 stages d'une durée totale de 24 semaines en milieu hospitalier ou extra-hospitalier. Possibilité d'effectuer la formation en initial ou en apprentissage. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Unité capitalisable (UC) - 1. Encadrer tout public dans tout lieu et toute structureUnité capitalisable (UC) - 2. Mettre en œuvre un projet d'animation s'inscrivant dans le projet de la structureUnité capitalisable (UC) - 3. Conduire une séance, un cycle d'animation ou d'apprentissage dans le champ des activités aquatiques et de la natationUnité capitalisable (UC) - 4. Mobiliser les techniques des activités aquatiques et de la natation pour mettre en œuvre une séance ou un cycle d'apprentissage | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T33" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'aide-soignant</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
         </is>
       </c>
       <c r="U33" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11533549/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11447001/true/false/false/false</t>
         </is>
       </c>
       <c r="V33" s="7" t="inlineStr">
@@ -4203,12 +4195,12 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>Diplôme d'État d'aide-soignant - DEAS</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -4218,12 +4210,12 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 1540 heures (dont 770 heures en entreprise)</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
@@ -4233,17 +4225,17 @@
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=aide-soignant</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
@@ -4258,12 +4250,12 @@
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>0472117979</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N34" s="5" t="inlineStr">
         <is>
-          <t>0472117979</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O34" s="5" t="inlineStr">
@@ -4282,15 +4274,19 @@
         </is>
       </c>
       <c r="R34" s="5" t="inlineStr"/>
-      <c r="S34" s="5" t="inlineStr"/>
+      <c r="S34" s="5" t="inlineStr">
+        <is>
+          <t>La formation conduisant au diplôme d'État d'aide-soignant, 17 semaines d'enseignement théoriques organisées autour de 8 modules : Accompagnement d'une personne dans les activités de la vie quotidienne L'état clinique d'une personne Les soins Ergonomie Relation Communication Hygiène des locaux hospitaliers Transmission des informations Organisation du travail Les titulaires du DE d'auxiliaire de puériculture, du DE d'aide médico-psychologique, du DE d'auxiliaire de vie sociale ou de la MC aide à domicile, sont dispensés de certaines unités de formation. La formation comprend également 6 stages d'une durée totale de 24 semaines en milieu hospitalier ou extra-hospitalier. Possibilité d'effectuer la formation en initial ou en apprentissage. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T34" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'aide-soignant</t>
         </is>
       </c>
       <c r="U34" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11817055/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11533549/true/false/false/true</t>
         </is>
       </c>
       <c r="V34" s="5" t="inlineStr">
@@ -4312,12 +4308,12 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'assistant de service social - DE ASS</t>
+          <t>Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
@@ -4327,12 +4323,12 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 avenue Lacassagne | Croix Rouge francaise | 69003 Lyon 3e | France</t>
+          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Durée de 3420 heures (dont 1680 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -4342,17 +4338,17 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=assistant%20de%20service%20social</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
@@ -4367,12 +4363,12 @@
       </c>
       <c r="M35" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0472117979</t>
         </is>
       </c>
       <c r="N35" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0472117979</t>
         </is>
       </c>
       <c r="O35" s="7" t="inlineStr">
@@ -4394,12 +4390,12 @@
       <c r="S35" s="7" t="inlineStr"/>
       <c r="T35" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U35" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11672249/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11817055/true/false/false/false</t>
         </is>
       </c>
       <c r="V35" s="7" t="inlineStr">
@@ -4421,27 +4417,27 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'éducateur spécialisé</t>
+          <t>Diplôme d'État d'assistant de service social - DE ASS</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales (ARFRIPS - Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales)</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>69009 Lyon 9e</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>10 Impasse Pierre Baizet | 69009 Lyon 9e | France</t>
+          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 avenue Lacassagne | Croix Rouge francaise | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Durée de 3442 heures (dont 1925 heures en entreprise)</t>
+          <t>Durée de 3420 heures (dont 1680 heures en entreprise)</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
@@ -4451,17 +4447,17 @@
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=assistant%20de%20service%20social</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>info@arfrips.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>info@arfrips.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
@@ -4476,12 +4472,12 @@
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>0478699090</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N36" s="5" t="inlineStr">
         <is>
-          <t>0478699090</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O36" s="5" t="inlineStr">
@@ -4503,17 +4499,17 @@
       <c r="S36" s="5" t="inlineStr"/>
       <c r="T36" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur spécialisé</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
         </is>
       </c>
       <c r="U36" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11737248/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11672249/true/false/false/false</t>
         </is>
       </c>
       <c r="V36" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
         </is>
       </c>
       <c r="W36" s="5" t="inlineStr">
@@ -4530,27 +4526,27 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet - RNCP 39931 - spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+          <t>Diplôme d'État d'éducateur spécialisé</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+          <t>Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales (ARFRIPS - Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales)</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>69009 Lyon 9e</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+          <t>10 Impasse Pierre Baizet | 69009 Lyon 9e | France</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 3442 heures (dont 1925 heures en entreprise)</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -4560,17 +4556,17 @@
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>https://arfatsema.catalogueformpro.com/2/desjeps-17/2858060/desjeps-17-diplome-detat-superieur-de-la-jeunesse-de-leducation-populaire-et-du-sport-specialite-ani</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>info@arfrips.fr</t>
         </is>
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>info@arfrips.fr</t>
         </is>
       </c>
       <c r="K37" s="7" t="inlineStr">
@@ -4585,12 +4581,12 @@
       </c>
       <c r="M37" s="7" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0478699090</t>
         </is>
       </c>
       <c r="N37" s="7" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0478699090</t>
         </is>
       </c>
       <c r="O37" s="7" t="inlineStr">
@@ -4600,7 +4596,7 @@
       </c>
       <c r="P37" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q37" s="7" t="inlineStr">
@@ -4609,19 +4605,15 @@
         </is>
       </c>
       <c r="R37" s="7" t="inlineStr"/>
-      <c r="S37" s="7" t="inlineStr">
-        <is>
-          <t>BC1 : Construire, avec les instances de gouvernance, la stratégie de développement d'une structure dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Éducation Populaire Culture Politique Rapport de domination Pouvoir d'Agir et Vulnérabilité Esprit critique Transformation social/rapport sociaux Le numérique comme un fait social Nouvel esprit du capitalisme Laicité et valeurs de la République Violence sexiste violences sexuelles Ingénierie social en lien avec la structure Réaliser un diagnostic RH et financier Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Elaboration de la stratégie de développement en lien avec les instances de gouvernance Animer un processus démocratique Démocratie et contre pouvoir BC2 : Concevoir et diriger un projet de développement de la structure Cartographie des relations et l'environnement de son association Ingénierie du projet Processus d'évaluation dans une démarche partagée et participative Outils participatifs Outils de communication Utilité sociale BC3 : Manager l'équipe et gérer les ressources humaines ( et la démarche Qualité, Sécurité, Santé au Travail et Environnement d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Gestion des ressources humaines en structures d'éducation populaire : enjeux, éthique et complexités associative Articulation employeur bénévole - direction dans la gestion des ressources humaines : définition d'une politique RH et organisation des délégations de pouvoir Gérer l'équipe au quotidien : accompagnement, régulation et gestion conflits Analyse des pratiques en co-développement Développer le pouvoir d'agir des salariés Attractivité, recrutement, intégration et fidélisation des salariés Diversité, inclusion et égalité professionnelle au sein de son organisation Assurer la GPEC, la formation et la gestion des carrières dans un alignement éthique Le financement de la formation professionnelle Qualité de vie Santé sécurité au travail Droit du travail/Droit social Dialogue social/dialogue syndical Cadre général des RPS Démarche prévention et outils BC4 : Assurer la gestion financière, matérielle et administrative d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Comprendre les fondamentaux de la situation financière Initiation à l'analyse financière associative ou de structure d'intérêt général Identifier les leviers de financement Construire des scénarios budgétaires et faire des arbitrages Élaborer un plan d'action financier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
+      <c r="S37" s="7" t="inlineStr"/>
       <c r="T37" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur spécialisé</t>
         </is>
       </c>
       <c r="U37" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880835/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11737248/true/false/false/false</t>
         </is>
       </c>
       <c r="V37" s="7" t="inlineStr">
@@ -4643,27 +4635,27 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Créer sa ferme en circuit court : transformation, commercialisation et communication</t>
+          <t>DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet - RNCP 39931 - spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>SARL Agri-learn éditions</t>
+          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>69001 Lyon</t>
+          <t>69100 Villeurbanne</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 69001 Lyon | France</t>
+          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Durée de 20 heures</t>
+          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
@@ -4673,17 +4665,17 @@
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://arfatsema.catalogueformpro.com/2/desjeps-17/2858060/desjeps-17-diplome-detat-superieur-de-la-jeunesse-de-leducation-populaire-et-du-sport-specialite-ani</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
@@ -4698,15 +4690,19 @@
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0478031711</t>
         </is>
       </c>
       <c r="N38" s="5" t="inlineStr">
         <is>
-          <t>0620021214</t>
-        </is>
-      </c>
-      <c r="O38" s="5" t="inlineStr"/>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="O38" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P38" s="5" t="inlineStr">
         <is>
           <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
@@ -4714,19 +4710,23 @@
       </c>
       <c r="Q38" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R38" s="5" t="inlineStr"/>
       <c r="S38" s="5" t="inlineStr">
         <is>
-          <t>Cette formation s'appuie sur plusieurs compétences essentielles : Stratégie commerciale et étude de marché : définir son offre, ses volumes, ses prix et ses circuits de vente Techniques de vente : maîtriser les étapes clés pour convaincre et fidéliser les clients Transformation des produits agricoles : valoriser ses matières premières pour créer de la valeur ajoutée Hygiène et réglementation : garantir la sécurité sanitaire dans les ateliers de transformation Communication et prospection : développer sa clientèle et promouvoir ses produits Valorisation des produits : savoir parler de ses produits et les mettre en avant (ex : dégustation) L'ensemble permet d'acquérir une vision globale du fonctionnement d'une ferme en circuit court, de la production jusqu'à la vente. 3 heures de visio avec les experts sont prévues dans le cursus. | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T38" s="5" t="inlineStr"/>
+          <t>BC1 : Construire, avec les instances de gouvernance, la stratégie de développement d'une structure dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Éducation Populaire Culture Politique Rapport de domination Pouvoir d'Agir et Vulnérabilité Esprit critique Transformation social/rapport sociaux Le numérique comme un fait social Nouvel esprit du capitalisme Laicité et valeurs de la République Violence sexiste violences sexuelles Ingénierie social en lien avec la structure Réaliser un diagnostic RH et financier Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Elaboration de la stratégie de développement en lien avec les instances de gouvernance Animer un processus démocratique Démocratie et contre pouvoir BC2 : Concevoir et diriger un projet de développement de la structure Cartographie des relations et l'environnement de son association Ingénierie du projet Processus d'évaluation dans une démarche partagée et participative Outils participatifs Outils de communication Utilité sociale BC3 : Manager l'équipe et gérer les ressources humaines ( et la démarche Qualité, Sécurité, Santé au Travail et Environnement d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Gestion des ressources humaines en structures d'éducation populaire : enjeux, éthique et complexités associative Articulation employeur bénévole - direction dans la gestion des ressources humaines : définition d'une politique RH et organisation des délégations de pouvoir Gérer l'équipe au quotidien : accompagnement, régulation et gestion conflits Analyse des pratiques en co-développement Développer le pouvoir d'agir des salariés Attractivité, recrutement, intégration et fidélisation des salariés Diversité, inclusion et égalité professionnelle au sein de son organisation Assurer la GPEC, la formation et la gestion des carrières dans un alignement éthique Le financement de la formation professionnelle Qualité de vie Santé sécurité au travail Droit du travail/Droit social Dialogue social/dialogue syndical Cadre général des RPS Démarche prévention et outils BC4 : Assurer la gestion financière, matérielle et administrative d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Comprendre les fondamentaux de la situation financière Initiation à l'analyse financière associative ou de structure d'intérêt général Identifier les leviers de financement Construire des scénarios budgétaires et faire des arbitrages Élaborer un plan d'action financier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T38" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+        </is>
+      </c>
       <c r="U38" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880868/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11880835/true/false/false/false</t>
         </is>
       </c>
       <c r="V38" s="5" t="inlineStr">
@@ -4748,27 +4748,27 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Titre professionnel administrateur d'infrastructures sécurisées (FOAD)</t>
+          <t>Créer sa ferme en circuit court : transformation, commercialisation et communication</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>STUDI</t>
+          <t>SARL Agri-learn éditions</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>69001 Lyon</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Formation a distance | 69001 Lyon | France</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Durée de 947 heures (dont 350 heures en entreprise)</t>
+          <t>Durée de 20 heures</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -4783,12 +4783,12 @@
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>contact@studi.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>contact@studi.fr | conseiller-formation.aoft@studi.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="K39" s="7" t="inlineStr">
@@ -4803,22 +4803,18 @@
       </c>
       <c r="M39" s="7" t="inlineStr">
         <is>
-          <t>0174888555</t>
+          <t>0620021214</t>
         </is>
       </c>
       <c r="N39" s="7" t="inlineStr">
         <is>
-          <t>0174888555</t>
-        </is>
-      </c>
-      <c r="O39" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="O39" s="7" t="inlineStr"/>
       <c r="P39" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q39" s="7" t="inlineStr">
@@ -4829,25 +4825,134 @@
       <c r="R39" s="7" t="inlineStr"/>
       <c r="S39" s="7" t="inlineStr">
         <is>
+          <t>Cette formation s'appuie sur plusieurs compétences essentielles : Stratégie commerciale et étude de marché : définir son offre, ses volumes, ses prix et ses circuits de vente Techniques de vente : maîtriser les étapes clés pour convaincre et fidéliser les clients Transformation des produits agricoles : valoriser ses matières premières pour créer de la valeur ajoutée Hygiène et réglementation : garantir la sécurité sanitaire dans les ateliers de transformation Communication et prospection : développer sa clientèle et promouvoir ses produits Valorisation des produits : savoir parler de ses produits et les mettre en avant (ex : dégustation) L'ensemble permet d'acquérir une vision globale du fonctionnement d'une ferme en circuit court, de la production jusqu'à la vente. 3 heures de visio avec les experts sont prévues dans le cursus. | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T39" s="7" t="inlineStr"/>
+      <c r="U39" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11880868/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V39" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W39" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Titre professionnel administrateur d'infrastructures sécurisées (FOAD)</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>STUDI</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>75004 Paris</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Formation a distance | 75004 Paris | France</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 947 heures (dont 350 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I40" s="6" t="inlineStr">
+        <is>
+          <t>contact@studi.fr</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>contact@studi.fr | conseiller-formation.aoft@studi.fr</t>
+        </is>
+      </c>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L40" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>0174888555</t>
+        </is>
+      </c>
+      <c r="N40" s="5" t="inlineStr">
+        <is>
+          <t>0174888555</t>
+        </is>
+      </c>
+      <c r="O40" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P40" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par France Travail</t>
+        </is>
+      </c>
+      <c r="Q40" s="5" t="inlineStr">
+        <is>
+          <t>À distance</t>
+        </is>
+      </c>
+      <c r="R40" s="5" t="inlineStr"/>
+      <c r="S40" s="5" t="inlineStr">
+        <is>
           <t>Administrer et sécuriser les infrastructures Les bonnes pratiques dans l'administration des infrastructures Utiliser un logiciel de gestion centralisé : GLPI Configurer le routage Administrer et sécuriser le réseau Automatiser les tâches d'administration Administrer et sécuriser les systèmes Les bases des serveurs virtualisés Administrer et sécuriser une infrastructure de serveurs virtualisée Gérer des containersConcevoir et mettre en œuvre une solution en réponse à un besoin d'évolution Les bases des solutions techniques Proposer une solution informatique répondant à des besoins nouveaux Mettre en production des évolutions de l'infrastructure Les bases de la supervision Superviser la disponibilité de l'infrastructure et en présenter les résultats Mesurer les performances et la disponibilité de l'infrastructureParticiper à la gestion de la cybersécurité Les bases de la cybersécurité Participer à la mesure et à l'analyse du niveau de sécurité de l'infrastructure Participer à l'élaboration et à la mise en œuvre de la politique de sécurité Participer à la détection et au traitement des incidents de sécurité | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
-      <c r="T39" s="7" t="inlineStr">
+      <c r="T40" s="5" t="inlineStr">
         <is>
           <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel administrateur d'infrastructures sécurisées</t>
         </is>
       </c>
-      <c r="U39" s="7" t="inlineStr">
+      <c r="U40" s="5" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/detail/11590088/true/false/true/false</t>
         </is>
       </c>
-      <c r="V39" s="7" t="inlineStr">
+      <c r="V40" s="5" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
-      <c r="W39" s="7" t="inlineStr">
+      <c r="W40" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-07-17
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1255,7 +1255,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1360,7 +1360,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,32 +1683,32 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>07</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Ecole de la 2ème Chance (E2C)</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Objectif 2ème chance - métropôle nice côte d'azur - ecole de la deuxième chance des alpes maritimes - odc nca - e2c</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>06200 Nice</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>455 Promenade des Anglais | Porte Arenas | 06200 Nice | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1100 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1723,12 +1723,12 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>contact@e2cnicecotedazur.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>contact@e2cnicecotedazur.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1743,40 +1743,48 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>04 12 05 20 05</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>04 12 05 20 05</t>
-        </is>
-      </c>
-      <c r="O11" s="7" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>Programme non communiqué | Organisme | Objectif 2ème chance - métropôle nice côte d'azur - ecole de la deuxième chance des alpes maritimes - odc nca - e2c | Lieu de la formation | 455 Promenade des Anglais</t>
-        </is>
-      </c>
-      <c r="T11" s="7" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+        </is>
+      </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10681643/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1788,32 +1796,32 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>05</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>CAP Fleuriste</t>
+          <t>Ecole de la 2ème Chance (E2C)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>Objectif 2ème chance - métropôle nice côte d'azur - ecole de la deuxième chance des alpes maritimes - odc nca - e2c</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>06200 Nice</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>455 Promenade des Anglais | Porte Arenas | 06200 Nice | France</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 1100 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1828,12 +1836,12 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>contact@e2cnicecotedazur.fr</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>contact@e2cnicecotedazur.fr</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1848,48 +1856,40 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>04 12 05 20 05</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>04 12 05 20 05</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr"/>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q12" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T12" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
-        </is>
-      </c>
+          <t>Programme non communiqué | Organisme | Objectif 2ème chance - métropôle nice côte d'azur - ecole de la deuxième chance des alpes maritimes - odc nca - e2c | Lieu de la formation | 455 Promenade des Anglais</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr"/>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10681643/true/false/false/false</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-05&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-07-20
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>09</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>09</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>09</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>09</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>09</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1255,7 +1255,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>09</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1360,7 +1360,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>09</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>09</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>09</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,7 +1683,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>09</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-07&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-07-21
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1255,7 +1255,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1360,7 +1360,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,7 +1570,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1615,7 +1615,7 @@
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr | cecile.iribarne@educagri.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1630,12 +1630,12 @@
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>0479264427</t>
+          <t>0479254180</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>0479264427</t>
+          <t>0479254180</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -1671,7 +1671,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,7 +1683,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>09</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1728,7 +1728,7 @@
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-09&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-07-23
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,32 +714,32 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Titre professionnel de formateur professionnel d'adultes - Bloc 01 Concevoir et préparer la formation</t>
+          <t>Titre professionnel secrétaire assistant médico-administratif (FOAD)</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>CAMELEON (Caméléon Formation)</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>11000 Carcassonne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>8 bd marcou | 11000 Carcassonne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Durée de 189 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1084 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>cameleonformation@gmail.com</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>cameleonformation@gmail.com</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -774,12 +774,12 @@
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>0554543023</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>0554543023</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
@@ -789,33 +789,33 @@
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R2" s="5" t="inlineStr"/>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>Concevoir et préparer la formation : réalisation d'un cahier des charges- rédactiond'un scénario pédagogique et d'un plan d'accompagnement- conception d'un scénario pédagogique etd'accompagnement en présentiel et multimodal - conception d'activités pédagogiques et d'évaluationutilisant les neurosciences- les apports des neurosciences pour une pédagogie différenciée innovante- lesdifférentes modalités pédagogiques actives selon les objectifs - conception des outils del'individualisation -construire un storyboard, notion de storytelling et de synopsis - les différents LMS etlogiciels pour du e-learning- les IA génératives au service de la formation- intégration des cadresréglementaires à la pratique - la démarche de formateur responsable : réglementation et RSE . | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>7 projets professionnalisants vous permettront d'acquérir les compétences citées au dessus par la pratique.Vous réaliserez les projets suivants :P1 - Démarrez votre formation de secrétaire assistant médico-administratifP2 - Niveau 1 : Maîtrisez l'accueil et la gestion administrative en milieu médicalP3 - Niveau 2 : Développez vos compétences en rédaction, communication et outils numériques en milieuP4 - Réalisez votre mission en entrepriseP5 - Niveau 3 : Optimisez l'organisation, la sécuritéet la gestion des données sensibles en milieu médicalP6 - Niveau 4 : Améliorez la gestion des communications, données et environnements sanitairesP7 - Préparez votre fin de formation de secrétaire assistant médico-administratif | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T2" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel formateur professionnel d'adultes</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel secrétaire assistant médico-administratif</t>
         </is>
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10969948/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/true</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,32 +827,32 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Titre professionnel formateur professionnel d'adultes - Bloc 03 Accomapgner les apprenants en formation</t>
+          <t>Formation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>CAMELEON (Caméléon Formation)</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>11000 Carcassonne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>8 rue Marcou | 11000 Carcassonne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Durée de 35 heures</t>
+          <t>Durée de 346 heures</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -867,12 +867,12 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>cameleonformation@gmail.com</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>cameleonformation@gmail.com</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
@@ -887,48 +887,40 @@
       </c>
       <c r="M3" s="7" t="inlineStr">
         <is>
-          <t>0554543023</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr">
         <is>
-          <t>0554543023</t>
-        </is>
-      </c>
-      <c r="O3" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0180888030</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="inlineStr"/>
       <c r="P3" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q3" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R3" s="7" t="inlineStr"/>
       <c r="S3" s="7" t="inlineStr">
         <is>
-          <t>Accompagner les apprenants enformation : adaptation duparcours et accompagnementdes apprenants - tutorat desapprenants à distance -coacherun apprenant selon les modalités- développer la réflexivité chez les apprenants- la métacognitioninclusivité-accompagnement des apprentissages en entreprise - accompagnement des apprenants à laréussite professionnelle - accompagnement d'un apprenant dans son parcours individuel - création d'undispositif de veille pour la démarche de formateur responsable - l'analyse de ses pratiquesprofessionnelles d'accompagnement | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T3" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel formateur professionnel d'adultes</t>
-        </is>
-      </c>
+          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T3" s="7" t="inlineStr"/>
       <c r="U3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10969957/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/true</t>
         </is>
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -940,32 +932,32 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Titre professionnel de formateur professionnel d'adultes - Bloc 02 Animer une formation et évaluer les acquis des apprenants</t>
+          <t>Concours d'atsem (FOAD)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>CAMELEON (Caméléon Formation)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>11000 Carcassonne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>8 rue Marcou | 11000 Carcassonne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Durée de 161 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -980,12 +972,12 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>cameleonformation@gmail.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>cameleonformation@gmail.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1000,48 +992,40 @@
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>0554543023</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>0554543023</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr"/>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q4" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R4" s="5" t="inlineStr"/>
       <c r="S4" s="5" t="inlineStr">
         <is>
-          <t>Animer une formation et évaluer les acquis des apprenants : animation d'uneformation - évaluation en présentiel - évaluation en multimodalité - repérage des difficultés liées auxapprentissages - animation de situations d'apprentissage en présentiel et à distance - analyse de sespratiques professionnelles d'animation et d'évaluation des acquis - apprendre autrement : des outilspour toutes les typologies d'apprentissage- intelligences multiples- psychologie clinique desapprentissages- la démarche de formateur responsable - les profils neuroatypiques : EHP, DYS, TDAH,TSA, la démarche qualité etresponsabilité sociale del'entreprise . | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T4" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel formateur professionnel d'adultes</t>
-        </is>
-      </c>
+          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr"/>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10969959/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
         </is>
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1053,32 +1037,32 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Hygiène en nologie</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>11100 Narbonne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4 heures</t>
+          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1093,12 +1077,12 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
@@ -1113,40 +1097,48 @@
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>0468410152</t>
-        </is>
-      </c>
-      <c r="O5" s="7" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O5" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R5" s="7" t="inlineStr"/>
       <c r="S5" s="7" t="inlineStr">
         <is>
-          <t>Définition des étapes de l'hygiène agro-alimentaire: détergence, désinfection, rinçageChoix du produit d'hygiène selon le bon "S.E.N.S.Le "T.A.C.T. pour nettoyer et désinfecterElaboration d'un plan d'hygiène | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
-        </is>
-      </c>
-      <c r="T5" s="7" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T5" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+        </is>
+      </c>
       <c r="U5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080125/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
         </is>
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1158,32 +1150,32 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Elevage des vins : choix, durée, contrôle</t>
+          <t>Préparation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
+          <t>AFEC</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>11100 Narbonne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
+          <t>AFEC (Siège) | Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4 heures</t>
+          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -1196,62 +1188,46 @@
           <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>thierry.cassagne@labdejean.fr</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>thierry.cassagne@labdejean.fr</t>
-        </is>
-      </c>
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr"/>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>france_travail</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>0676219742</t>
-        </is>
-      </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>0676219742</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr"/>
+      <c r="N6" s="5" t="inlineStr"/>
       <c r="O6" s="5" t="inlineStr"/>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R6" s="5" t="inlineStr"/>
       <c r="S6" s="5" t="inlineStr">
         <is>
-          <t>Définition de l'élevageRôle des gaz (CO2 et O2)Les différents modes d'élevageLe suivi analytique et microbiologique | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC | Lieu de la formation | AFEC (Siège)</t>
         </is>
       </c>
       <c r="T6" s="5" t="inlineStr"/>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080181/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1263,32 +1239,32 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Vinification en rose : les fondamentaux</t>
+          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>11100 Narbonne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4 heures</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1303,12 +1279,12 @@
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
@@ -1323,40 +1299,40 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="O7" s="7" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr"/>
       <c r="S7" s="7" t="inlineStr">
         <is>
-          <t>Définition du profil de vin souhaitéMaturation des raisins: détermination de la date optimale des vendangesItinéraires techniques généraux (pressurage direct, saignée)Opérations préfermentaires: transport, bioprotection, égrappage, foulage, pressurage,gestion de la couleur, débourbagePilotage de la fermentation alcoolique: SO2, levures, nutrition azotée, gestion O2, gestion profil T°Conservation du vin | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T7" s="7" t="inlineStr"/>
       <c r="U7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080222/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
         </is>
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1368,32 +1344,32 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Vinification en rouge : les fondamentaux</t>
+          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>11100 Narbonne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4 heures</t>
+          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -1408,12 +1384,12 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1428,40 +1404,40 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="O8" s="5" t="inlineStr"/>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q8" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>Définition du profil de vin souhaitéMaturation des raisin: détermination de la date optimale des vendangesItinéraire technique général de la vinification en rougeCuvaison/macérationOpérations préfermentaires: transport, bioprorection, égrappage, foulage, MPFPilotage de la fermentation alcoolique: SO2, levures, nutriments, gestion profil thermique, gestion O2, techniques d'extractionOpérations Post macération:Ecoulage, décuvage, pressurage du marc,FMLElevage | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080224/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
         </is>
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1473,32 +1449,32 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Repérer et identifier les principaux défauts du vin</t>
+          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>11100 Narbonne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4 heures</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1513,12 +1489,12 @@
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
@@ -1533,40 +1509,40 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="O9" s="7" t="inlineStr"/>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R9" s="7" t="inlineStr"/>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>Altérations d'origine microbienne:Contamination bactérienne: acescence, piqûre acétique, piqûre lactique, maladie de la tourne, maladie de l'amer, piqure mannitique, odeur de géranium, diacétyleContamination levurienne: brettanomyces, maladie de la fleur, goût de sourisOxydationRéductionMaladies dues à la qualité des raisins: les GMT, le goût herbacé-véétalAutres origines: goût de bouchon, pinking, goût d'huître, goût de lumière | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr"/>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080227/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/true</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1578,32 +1554,32 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Vinification sans sulfites ajoutes ou à teneur réduite en sulfites</t>
+          <t>BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
+          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>11100 Narbonne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4 heures</t>
+          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1618,12 +1594,12 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1638,40 +1614,48 @@
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0479254180</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>0468410152</t>
-        </is>
-      </c>
-      <c r="O10" s="5" t="inlineStr"/>
+          <t>0479254180</t>
+        </is>
+      </c>
+      <c r="O10" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q10" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>Chimie du SO2Produits de substitution au SO2Gestion O2Itinéraires techniques de vinification alternatifsStabilisation et élevage des vins | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
-        </is>
-      </c>
-      <c r="T10" s="5" t="inlineStr"/>
+          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T10" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
+        </is>
+      </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080266/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/true</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,32 +1667,32 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Vinification en blanc: les fondamentaux</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>11100 Narbonne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4 heures</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1723,12 +1707,12 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1743,40 +1727,48 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>0468410152</t>
-        </is>
-      </c>
-      <c r="O11" s="7" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>Détermination du type de vin souhaitéMaturation du raisin: détermination de la date des vendangesItinéraire technique généralOpérations préfermentaires: transport, bioprotection, tri, éraflage, macération préfermentaire à froid, pressurage, débourbagePilotage de la fermentation alcoolique: SO2, levurage, nutrition azotée, gestion O2, maîtrise T°Elevage: en cuve, en barrique, sur lies fines | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
-        </is>
-      </c>
-      <c r="T11" s="7" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+        </is>
+      </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080272/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1788,32 +1780,32 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Titre professionnel secrétaire assistant médico-administratif (FOAD)</t>
+          <t>Titre professionnel de formateur professionnel d'adultes - Bloc 01 Concevoir et préparer la formation</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>CAMELEON (Caméléon Formation)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>11000 Carcassonne</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>8 bd marcou | 11000 Carcassonne | France</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1084 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 189 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1828,12 +1820,12 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>cameleonformation@gmail.com</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>cameleonformation@gmail.com</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1848,12 +1840,12 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0554543023</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0554543023</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr">
@@ -1863,33 +1855,33 @@
       </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q12" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>7 projets professionnalisants vous permettront d'acquérir les compétences citées au dessus par la pratique.Vous réaliserez les projets suivants :P1 - Démarrez votre formation de secrétaire assistant médico-administratifP2 - Niveau 1 : Maîtrisez l'accueil et la gestion administrative en milieu médicalP3 - Niveau 2 : Développez vos compétences en rédaction, communication et outils numériques en milieuP4 - Réalisez votre mission en entrepriseP5 - Niveau 3 : Optimisez l'organisation, la sécuritéet la gestion des données sensibles en milieu médicalP6 - Niveau 4 : Améliorez la gestion des communications, données et environnements sanitairesP7 - Préparez votre fin de formation de secrétaire assistant médico-administratif | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Concevoir et préparer la formation : réalisation d'un cahier des charges- rédactiond'un scénario pédagogique et d'un plan d'accompagnement- conception d'un scénario pédagogique etd'accompagnement en présentiel et multimodal - conception d'activités pédagogiques et d'évaluationutilisant les neurosciences- les apports des neurosciences pour une pédagogie différenciée innovante- lesdifférentes modalités pédagogiques actives selon les objectifs - conception des outils del'individualisation -construire un storyboard, notion de storytelling et de synopsis - les différents LMS etlogiciels pour du e-learning- les IA génératives au service de la formation- intégration des cadresréglementaires à la pratique - la démarche de formateur responsable : réglementation et RSE . | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T12" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel secrétaire assistant médico-administratif</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel formateur professionnel d'adultes</t>
         </is>
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10969948/true/false/false/false</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -1901,32 +1893,32 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Formation au concours d'ATSEM</t>
+          <t>Titre professionnel formateur professionnel d'adultes - Bloc 03 Accomapgner les apprenants en formation</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>CAMELEON (Caméléon Formation)</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>11000 Carcassonne</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>8 rue Marcou | 11000 Carcassonne | France</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Durée de 346 heures</t>
+          <t>Durée de 35 heures</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1941,12 +1933,12 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>cameleonformation@gmail.com</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>cameleonformation@gmail.com</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
@@ -1961,40 +1953,48 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0554543023</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="O13" s="7" t="inlineStr"/>
+          <t>0554543023</t>
+        </is>
+      </c>
+      <c r="O13" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R13" s="7" t="inlineStr"/>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T13" s="7" t="inlineStr"/>
+          <t>Accompagner les apprenants enformation : adaptation duparcours et accompagnementdes apprenants - tutorat desapprenants à distance -coacherun apprenant selon les modalités- développer la réflexivité chez les apprenants- la métacognitioninclusivité-accompagnement des apprentissages en entreprise - accompagnement des apprenants à laréussite professionnelle - accompagnement d'un apprenant dans son parcours individuel - création d'undispositif de veille pour la démarche de formateur responsable - l'analyse de ses pratiquesprofessionnelles d'accompagnement | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T13" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel formateur professionnel d'adultes</t>
+        </is>
+      </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10969957/true/false/false/false</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W13" s="7" t="inlineStr">
@@ -2006,32 +2006,32 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Concours d'atsem (FOAD)</t>
+          <t>Titre professionnel de formateur professionnel d'adultes - Bloc 02 Animer une formation et évaluer les acquis des apprenants</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>CAMELEON (Caméléon Formation)</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>11000 Carcassonne</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>8 rue Marcou | 11000 Carcassonne | France</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
+          <t>Durée de 161 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -2046,12 +2046,12 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>cameleonformation@gmail.com</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>cameleonformation@gmail.com</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -2066,40 +2066,48 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0554543023</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O14" s="5" t="inlineStr"/>
+          <t>0554543023</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q14" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T14" s="5" t="inlineStr"/>
+          <t>Animer une formation et évaluer les acquis des apprenants : animation d'uneformation - évaluation en présentiel - évaluation en multimodalité - repérage des difficultés liées auxapprentissages - animation de situations d'apprentissage en présentiel et à distance - analyse de sespratiques professionnelles d'animation et d'évaluation des acquis - apprendre autrement : des outilspour toutes les typologies d'apprentissage- intelligences multiples- psychologie clinique desapprentissages- la démarche de formateur responsable - les profils neuroatypiques : EHP, DYS, TDAH,TSA, la démarche qualité etresponsabilité sociale del'entreprise . | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T14" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel formateur professionnel d'adultes</t>
+        </is>
+      </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10969959/true/false/false/false</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
@@ -2111,32 +2119,32 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Hygiène en nologie</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>11100 Narbonne</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 4 heures</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2151,12 +2159,12 @@
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -2171,48 +2179,40 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O15" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0468410152</t>
+        </is>
+      </c>
+      <c r="O15" s="7" t="inlineStr"/>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr"/>
       <c r="S15" s="7" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T15" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
+          <t>Définition des étapes de l'hygiène agro-alimentaire: détergence, désinfection, rinçageChoix du produit d'hygiène selon le bon "S.E.N.S.Le "T.A.C.T. pour nettoyer et désinfecterElaboration d'un plan d'hygiène | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+        </is>
+      </c>
+      <c r="T15" s="7" t="inlineStr"/>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080125/true/false/false/false</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W15" s="7" t="inlineStr">
@@ -2224,32 +2224,32 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Préparation au concours d'ATSEM</t>
+          <t>Elevage des vins : choix, durée, contrôle</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>AFEC (Siège)</t>
+          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>11100 Narbonne</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 4 heures</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2264,12 +2264,12 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -2284,40 +2284,40 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>0153368844</t>
+          <t>0676219742</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>0153368844</t>
+          <t>0676219742</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr"/>
       <c r="P16" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q16" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R16" s="5" t="inlineStr"/>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC (Siège) | Lieu de la formation | Formation a distance</t>
+          <t>Définition de l'élevageRôle des gaz (CO2 et O2)Les différents modes d'élevageLe suivi analytique et microbiologique | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T16" s="5" t="inlineStr"/>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080181/true/false/false/false</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W16" s="5" t="inlineStr">
@@ -2329,32 +2329,32 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
+          <t>Vinification en rose : les fondamentaux</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>11100 Narbonne</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 4 heures</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2369,12 +2369,12 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -2389,40 +2389,40 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="O17" s="7" t="inlineStr"/>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="7" t="inlineStr">
         <is>
-          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Définition du profil de vin souhaitéMaturation des raisins: détermination de la date optimale des vendangesItinéraires techniques généraux (pressurage direct, saignée)Opérations préfermentaires: transport, bioprotection, égrappage, foulage, pressurage,gestion de la couleur, débourbagePilotage de la fermentation alcoolique: SO2, levures, nutrition azotée, gestion O2, gestion profil T°Conservation du vin | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T17" s="7" t="inlineStr"/>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080222/true/false/false/false</t>
         </is>
       </c>
       <c r="V17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W17" s="7" t="inlineStr">
@@ -2434,32 +2434,32 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
+          <t>Vinification en rouge : les fondamentaux</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>11100 Narbonne</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 4 heures</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -2474,12 +2474,12 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -2494,40 +2494,40 @@
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="O18" s="5" t="inlineStr"/>
       <c r="P18" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q18" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Définition du profil de vin souhaitéMaturation des raisin: détermination de la date optimale des vendangesItinéraire technique général de la vinification en rougeCuvaison/macérationOpérations préfermentaires: transport, bioprorection, égrappage, foulage, MPFPilotage de la fermentation alcoolique: SO2, levures, nutriments, gestion profil thermique, gestion O2, techniques d'extractionOpérations Post macération:Ecoulage, décuvage, pressurage du marc,FMLElevage | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T18" s="5" t="inlineStr"/>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080224/true/false/false/false</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W18" s="5" t="inlineStr">
@@ -2539,32 +2539,32 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
+          <t>Repérer et identifier les principaux défauts du vin</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>11100 Narbonne</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 4 heures</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2579,12 +2579,12 @@
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="K19" s="7" t="inlineStr">
@@ -2599,40 +2599,40 @@
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="O19" s="7" t="inlineStr"/>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R19" s="7" t="inlineStr"/>
       <c r="S19" s="7" t="inlineStr">
         <is>
-          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Altérations d'origine microbienne:Contamination bactérienne: acescence, piqûre acétique, piqûre lactique, maladie de la tourne, maladie de l'amer, piqure mannitique, odeur de géranium, diacétyleContamination levurienne: brettanomyces, maladie de la fleur, goût de sourisOxydationRéductionMaladies dues à la qualité des raisins: les GMT, le goût herbacé-véétalAutres origines: goût de bouchon, pinking, goût d'huître, goût de lumière | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T19" s="7" t="inlineStr"/>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080227/true/false/false/false</t>
         </is>
       </c>
       <c r="V19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W19" s="7" t="inlineStr">
@@ -2644,32 +2644,32 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>BP option aménagements paysagers</t>
+          <t>Vinification sans sulfites ajoutes ou à teneur réduite en sulfites</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
+          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>11100 Narbonne</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
+          <t>Durée de 4 heures</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -2684,12 +2684,12 @@
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -2704,48 +2704,40 @@
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>0479254180</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>0479254180</t>
-        </is>
-      </c>
-      <c r="O20" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0468410152</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr"/>
       <c r="P20" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q20" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T20" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
-        </is>
-      </c>
+          <t>Chimie du SO2Produits de substitution au SO2Gestion O2Itinéraires techniques de vinification alternatifsStabilisation et élevage des vins | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+        </is>
+      </c>
+      <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080266/true/false/false/false</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W20" s="5" t="inlineStr">
@@ -2757,32 +2749,32 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>CAP Fleuriste</t>
+          <t>Vinification en blanc: les fondamentaux</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>11100 Narbonne</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 4 heures</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -2797,12 +2789,12 @@
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
@@ -2817,48 +2809,40 @@
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O21" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0468410152</t>
+        </is>
+      </c>
+      <c r="O21" s="7" t="inlineStr"/>
       <c r="P21" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q21" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R21" s="7" t="inlineStr"/>
       <c r="S21" s="7" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T21" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
-        </is>
-      </c>
+          <t>Détermination du type de vin souhaitéMaturation du raisin: détermination de la date des vendangesItinéraire technique généralOpérations préfermentaires: transport, bioprotection, tri, éraflage, macération préfermentaire à froid, pressurage, débourbagePilotage de la fermentation alcoolique: SO2, levurage, nutrition azotée, gestion O2, maîtrise T°Elevage: en cuve, en barrique, sur lies fines | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+        </is>
+      </c>
+      <c r="T21" s="7" t="inlineStr"/>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080272/true/false/false/false</t>
         </is>
       </c>
       <c r="V21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-10&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W21" s="7" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-07-24
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseFranceTravail" displayName="BaseFranceTravail" ref="A1:W50" headerRowCount="1">
-  <autoFilter ref="A1:W50"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseFranceTravail" displayName="BaseFranceTravail" ref="A1:W53" headerRowCount="1">
+  <autoFilter ref="A1:W53"/>
   <tableColumns count="23">
     <tableColumn id="1" name="zone"/>
     <tableColumn id="2" name="formation"/>
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5">
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W50"/>
+  <dimension ref="A1:W53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1239,7 +1239,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1344,7 +1344,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1449,17 +1449,17 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 1350 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1489,12 +1489,12 @@
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
@@ -1509,15 +1509,19 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
-        </is>
-      </c>
-      <c r="O9" s="7" t="inlineStr"/>
+          <t>0180888030</t>
+        </is>
+      </c>
+      <c r="O9" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -1531,18 +1535,22 @@
       <c r="R9" s="7" t="inlineStr"/>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T9" s="7" t="inlineStr"/>
+          <t>11 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 : Démarrez votre formation d'Accompagnement Educatif Petite Enfance ; Projet 2 - Préparez un environnement sécurisé pour le jeune enfant ; Projet 3 - Développez des activités éducatives adaptées à la petite enfance ; Projet 4 - Appliquez les protocoles de santé dans le cadre de la petite enfance ; Projet 5 - Soutenez le personnel enseignant dans un contexte collectif ; Projet 6 - Améliorez les conditions d'accueil en école maternelle ; Projet 7 - Organisez l'accueil individuel au domicile ; Projet 8 - Gérez les tâches domestiques et la préparation des repas pour l'enfant ; Projet 9 : Proposer des solutions de prévention, santé et environnement ; Projet 10 : Remise à niveau scolaire ; Projet 11 : Préparez-vous pour l'examen final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T9" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+        </is>
+      </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120311/true/false/true/true</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1554,17 +1562,17 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>BP option aménagements paysagers</t>
+          <t>Conseiller emploi et accompagnement professionnel</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1579,7 +1587,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
+          <t>Durée de 1140 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1594,12 +1602,12 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1614,12 +1622,12 @@
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>0479254180</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>0479254180</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -1640,22 +1648,22 @@
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>10 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de conseiller emploi et évolution professionnelle ; Projet 2 - Accompagnez en parallèle de nombreuses personnes avec des besoins différents ; Projet 3 - Élaborez une veille et analysez le marché de l'emploi ; Projet 4 - Réalisez un diagnostic et co-construisez un plan d'action avec vos bénéficiaires ; Projet 5 - Adaptez votre posture pour l'accompagnement des bénéficiaires ; Projet 6 - Établissez et validez un projet d'accompagnement professionnel ; Projet 7 - Établissez un plan d'action et un bilan professionnel ; Projet 8 - Concevez un atelier sur les métiers émergents avec l'IA ; Projet 9 - Développez votre projet territorial avec des partenaires ; Projet 10 - Élaborez votre boîte à outils pour accompagner vers l'emploi. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
         </is>
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Conseiller emploi et accompagnement professionnel</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120363/true/false/true/true</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1667,17 +1675,17 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>CAP Fleuriste</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>AFEC (Siège)</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -1692,7 +1700,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1707,12 +1715,12 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1727,12 +1735,12 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="O11" s="7" t="inlineStr">
@@ -1753,22 +1761,22 @@
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant des modules d'enseignement et des prestations d'accompagnement. Modules d'enseignement professionnel : - EP1 Accompagnement du développement du jeune enfant (cadre d'intervention, accompagnement à l'autonomie l'enfant) - EP2 Exercer son activité en accueil collectif - EP3 Exercer son activité en accueil individuel Modules d'enseignements généraux : - Prévention santé environnement - Enseignements généraux (Mathématiques et sciences, Histoire-Géographie-Citoyenneté et français) En complément de la formation : - Remise à niveau numérique - Techniques de recherche d'emploi et de stage - Accompagnement au retour à l'emploi 3 Stages en entreprise 14 semaines | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124191/true/false/true/true</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1780,32 +1788,32 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Titre professionnel de formateur professionnel d'adultes - Bloc 01 Concevoir et préparer la formation</t>
+          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>CAMELEON (Caméléon Formation)</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>11000 Carcassonne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>8 bd marcou | 11000 Carcassonne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Durée de 189 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1820,12 +1828,12 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>cameleonformation@gmail.com</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>cameleonformation@gmail.com</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1840,48 +1848,40 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>0554543023</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>0554543023</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr"/>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q12" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>Concevoir et préparer la formation : réalisation d'un cahier des charges- rédactiond'un scénario pédagogique et d'un plan d'accompagnement- conception d'un scénario pédagogique etd'accompagnement en présentiel et multimodal - conception d'activités pédagogiques et d'évaluationutilisant les neurosciences- les apports des neurosciences pour une pédagogie différenciée innovante- lesdifférentes modalités pédagogiques actives selon les objectifs - conception des outils del'individualisation -construire un storyboard, notion de storytelling et de synopsis - les différents LMS etlogiciels pour du e-learning- les IA génératives au service de la formation- intégration des cadresréglementaires à la pratique - la démarche de formateur responsable : réglementation et RSE . | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T12" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel formateur professionnel d'adultes</t>
-        </is>
-      </c>
+          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr"/>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10969948/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/true</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -1893,32 +1893,32 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Titre professionnel formateur professionnel d'adultes - Bloc 03 Accomapgner les apprenants en formation</t>
+          <t>BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>CAMELEON (Caméléon Formation)</t>
+          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>11000 Carcassonne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>8 rue Marcou | 11000 Carcassonne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Durée de 35 heures</t>
+          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1933,12 +1933,12 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>cameleonformation@gmail.com</t>
+          <t>epl.la-motte-servolex@educagri.fr</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>cameleonformation@gmail.com</t>
+          <t>epl.la-motte-servolex@educagri.fr</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
@@ -1953,12 +1953,12 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>0554543023</t>
+          <t>0479254180</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>0554543023</t>
+          <t>0479254180</t>
         </is>
       </c>
       <c r="O13" s="7" t="inlineStr">
@@ -1968,33 +1968,33 @@
       </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R13" s="7" t="inlineStr"/>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>Accompagner les apprenants enformation : adaptation duparcours et accompagnementdes apprenants - tutorat desapprenants à distance -coacherun apprenant selon les modalités- développer la réflexivité chez les apprenants- la métacognitioninclusivité-accompagnement des apprentissages en entreprise - accompagnement des apprenants à laréussite professionnelle - accompagnement d'un apprenant dans son parcours individuel - création d'undispositif de veille pour la démarche de formateur responsable - l'analyse de ses pratiquesprofessionnelles d'accompagnement | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel formateur professionnel d'adultes</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10969957/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/true</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W13" s="7" t="inlineStr">
@@ -2006,32 +2006,32 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Titre professionnel de formateur professionnel d'adultes - Bloc 02 Animer une formation et évaluer les acquis des apprenants</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>CAMELEON (Caméléon Formation)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>11000 Carcassonne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>8 rue Marcou | 11000 Carcassonne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Durée de 161 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -2046,12 +2046,12 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>cameleonformation@gmail.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>cameleonformation@gmail.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -2066,12 +2066,12 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>0554543023</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>0554543023</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -2081,33 +2081,33 @@
       </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q14" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>Animer une formation et évaluer les acquis des apprenants : animation d'uneformation - évaluation en présentiel - évaluation en multimodalité - repérage des difficultés liées auxapprentissages - animation de situations d'apprentissage en présentiel et à distance - analyse de sespratiques professionnelles d'animation et d'évaluation des acquis - apprendre autrement : des outilspour toutes les typologies d'apprentissage- intelligences multiples- psychologie clinique desapprentissages- la démarche de formateur responsable - les profils neuroatypiques : EHP, DYS, TDAH,TSA, la démarche qualité etresponsabilité sociale del'entreprise . | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel formateur professionnel d'adultes</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10969959/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
@@ -2124,27 +2124,27 @@
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Hygiène en nologie</t>
+          <t>Titre professionnel de formateur professionnel d'adultes - Bloc 01 Concevoir et préparer la formation</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
+          <t>CAMELEON (Caméléon Formation)</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>11100 Narbonne</t>
+          <t>11000 Carcassonne</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
+          <t>8 bd marcou | 11000 Carcassonne | France</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4 heures</t>
+          <t>Durée de 189 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2159,12 +2159,12 @@
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>cameleonformation@gmail.com</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>cameleonformation@gmail.com</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -2179,15 +2179,19 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0554543023</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>0468410152</t>
-        </is>
-      </c>
-      <c r="O15" s="7" t="inlineStr"/>
+          <t>0554543023</t>
+        </is>
+      </c>
+      <c r="O15" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
           <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
@@ -2201,13 +2205,17 @@
       <c r="R15" s="7" t="inlineStr"/>
       <c r="S15" s="7" t="inlineStr">
         <is>
-          <t>Définition des étapes de l'hygiène agro-alimentaire: détergence, désinfection, rinçageChoix du produit d'hygiène selon le bon "S.E.N.S.Le "T.A.C.T. pour nettoyer et désinfecterElaboration d'un plan d'hygiène | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
-        </is>
-      </c>
-      <c r="T15" s="7" t="inlineStr"/>
+          <t>Concevoir et préparer la formation : réalisation d'un cahier des charges- rédactiond'un scénario pédagogique et d'un plan d'accompagnement- conception d'un scénario pédagogique etd'accompagnement en présentiel et multimodal - conception d'activités pédagogiques et d'évaluationutilisant les neurosciences- les apports des neurosciences pour une pédagogie différenciée innovante- lesdifférentes modalités pédagogiques actives selon les objectifs - conception des outils del'individualisation -construire un storyboard, notion de storytelling et de synopsis - les différents LMS etlogiciels pour du e-learning- les IA génératives au service de la formation- intégration des cadresréglementaires à la pratique - la démarche de formateur responsable : réglementation et RSE . | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T15" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel formateur professionnel d'adultes</t>
+        </is>
+      </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080125/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10969948/true/false/false/false</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
@@ -2229,27 +2237,27 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Elevage des vins : choix, durée, contrôle</t>
+          <t>Titre professionnel formateur professionnel d'adultes - Bloc 03 Accomapgner les apprenants en formation</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
+          <t>CAMELEON (Caméléon Formation)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>11100 Narbonne</t>
+          <t>11000 Carcassonne</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
+          <t>8 rue Marcou | 11000 Carcassonne | France</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4 heures</t>
+          <t>Durée de 35 heures</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2264,12 +2272,12 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>cameleonformation@gmail.com</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>cameleonformation@gmail.com</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -2284,15 +2292,19 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>0676219742</t>
+          <t>0554543023</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>0676219742</t>
-        </is>
-      </c>
-      <c r="O16" s="5" t="inlineStr"/>
+          <t>0554543023</t>
+        </is>
+      </c>
+      <c r="O16" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P16" s="5" t="inlineStr">
         <is>
           <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
@@ -2306,13 +2318,17 @@
       <c r="R16" s="5" t="inlineStr"/>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>Définition de l'élevageRôle des gaz (CO2 et O2)Les différents modes d'élevageLe suivi analytique et microbiologique | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
-        </is>
-      </c>
-      <c r="T16" s="5" t="inlineStr"/>
+          <t>Accompagner les apprenants enformation : adaptation duparcours et accompagnementdes apprenants - tutorat desapprenants à distance -coacherun apprenant selon les modalités- développer la réflexivité chez les apprenants- la métacognitioninclusivité-accompagnement des apprentissages en entreprise - accompagnement des apprenants à laréussite professionnelle - accompagnement d'un apprenant dans son parcours individuel - création d'undispositif de veille pour la démarche de formateur responsable - l'analyse de ses pratiquesprofessionnelles d'accompagnement | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T16" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel formateur professionnel d'adultes</t>
+        </is>
+      </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080181/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10969957/true/false/false/false</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
@@ -2334,27 +2350,27 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Vinification en rose : les fondamentaux</t>
+          <t>Titre professionnel de formateur professionnel d'adultes - Bloc 02 Animer une formation et évaluer les acquis des apprenants</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
+          <t>CAMELEON (Caméléon Formation)</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>11100 Narbonne</t>
+          <t>11000 Carcassonne</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
+          <t>8 rue Marcou | 11000 Carcassonne | France</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4 heures</t>
+          <t>Durée de 161 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2369,12 +2385,12 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>cameleonformation@gmail.com</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>cameleonformation@gmail.com</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -2389,15 +2405,19 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0554543023</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>0468410152</t>
-        </is>
-      </c>
-      <c r="O17" s="7" t="inlineStr"/>
+          <t>0554543023</t>
+        </is>
+      </c>
+      <c r="O17" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P17" s="7" t="inlineStr">
         <is>
           <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
@@ -2411,13 +2431,17 @@
       <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="7" t="inlineStr">
         <is>
-          <t>Définition du profil de vin souhaitéMaturation des raisins: détermination de la date optimale des vendangesItinéraires techniques généraux (pressurage direct, saignée)Opérations préfermentaires: transport, bioprotection, égrappage, foulage, pressurage,gestion de la couleur, débourbagePilotage de la fermentation alcoolique: SO2, levures, nutrition azotée, gestion O2, gestion profil T°Conservation du vin | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
-        </is>
-      </c>
-      <c r="T17" s="7" t="inlineStr"/>
+          <t>Animer une formation et évaluer les acquis des apprenants : animation d'uneformation - évaluation en présentiel - évaluation en multimodalité - repérage des difficultés liées auxapprentissages - animation de situations d'apprentissage en présentiel et à distance - analyse de sespratiques professionnelles d'animation et d'évaluation des acquis - apprendre autrement : des outilspour toutes les typologies d'apprentissage- intelligences multiples- psychologie clinique desapprentissages- la démarche de formateur responsable - les profils neuroatypiques : EHP, DYS, TDAH,TSA, la démarche qualité etresponsabilité sociale del'entreprise . | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T17" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel formateur professionnel d'adultes</t>
+        </is>
+      </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080222/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10969959/true/false/false/false</t>
         </is>
       </c>
       <c r="V17" s="7" t="inlineStr">
@@ -2439,7 +2463,7 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Vinification en rouge : les fondamentaux</t>
+          <t>Hygiène en nologie</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -2516,13 +2540,13 @@
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>Définition du profil de vin souhaitéMaturation des raisin: détermination de la date optimale des vendangesItinéraire technique général de la vinification en rougeCuvaison/macérationOpérations préfermentaires: transport, bioprorection, égrappage, foulage, MPFPilotage de la fermentation alcoolique: SO2, levures, nutriments, gestion profil thermique, gestion O2, techniques d'extractionOpérations Post macération:Ecoulage, décuvage, pressurage du marc,FMLElevage | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+          <t>Définition des étapes de l'hygiène agro-alimentaire: détergence, désinfection, rinçageChoix du produit d'hygiène selon le bon "S.E.N.S.Le "T.A.C.T. pour nettoyer et désinfecterElaboration d'un plan d'hygiène | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T18" s="5" t="inlineStr"/>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080224/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080125/true/false/false/false</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
@@ -2544,7 +2568,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Repérer et identifier les principaux défauts du vin</t>
+          <t>Elevage des vins : choix, durée, contrôle</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -2599,12 +2623,12 @@
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0676219742</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0676219742</t>
         </is>
       </c>
       <c r="O19" s="7" t="inlineStr"/>
@@ -2621,13 +2645,13 @@
       <c r="R19" s="7" t="inlineStr"/>
       <c r="S19" s="7" t="inlineStr">
         <is>
-          <t>Altérations d'origine microbienne:Contamination bactérienne: acescence, piqûre acétique, piqûre lactique, maladie de la tourne, maladie de l'amer, piqure mannitique, odeur de géranium, diacétyleContamination levurienne: brettanomyces, maladie de la fleur, goût de sourisOxydationRéductionMaladies dues à la qualité des raisins: les GMT, le goût herbacé-véétalAutres origines: goût de bouchon, pinking, goût d'huître, goût de lumière | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+          <t>Définition de l'élevageRôle des gaz (CO2 et O2)Les différents modes d'élevageLe suivi analytique et microbiologique | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T19" s="7" t="inlineStr"/>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080227/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080181/true/false/false/false</t>
         </is>
       </c>
       <c r="V19" s="7" t="inlineStr">
@@ -2649,7 +2673,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Vinification sans sulfites ajoutes ou à teneur réduite en sulfites</t>
+          <t>Vinification en rose : les fondamentaux</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -2726,13 +2750,13 @@
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>Chimie du SO2Produits de substitution au SO2Gestion O2Itinéraires techniques de vinification alternatifsStabilisation et élevage des vins | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+          <t>Définition du profil de vin souhaitéMaturation des raisins: détermination de la date optimale des vendangesItinéraires techniques généraux (pressurage direct, saignée)Opérations préfermentaires: transport, bioprotection, égrappage, foulage, pressurage,gestion de la couleur, débourbagePilotage de la fermentation alcoolique: SO2, levures, nutrition azotée, gestion O2, gestion profil T°Conservation du vin | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080266/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080222/true/false/false/false</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
@@ -2754,7 +2778,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Vinification en blanc: les fondamentaux</t>
+          <t>Vinification en rouge : les fondamentaux</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -2831,13 +2855,13 @@
       <c r="R21" s="7" t="inlineStr"/>
       <c r="S21" s="7" t="inlineStr">
         <is>
-          <t>Détermination du type de vin souhaitéMaturation du raisin: détermination de la date des vendangesItinéraire technique généralOpérations préfermentaires: transport, bioprotection, tri, éraflage, macération préfermentaire à froid, pressurage, débourbagePilotage de la fermentation alcoolique: SO2, levurage, nutrition azotée, gestion O2, maîtrise T°Elevage: en cuve, en barrique, sur lies fines | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+          <t>Définition du profil de vin souhaitéMaturation des raisin: détermination de la date optimale des vendangesItinéraire technique général de la vinification en rougeCuvaison/macérationOpérations préfermentaires: transport, bioprorection, égrappage, foulage, MPFPilotage de la fermentation alcoolique: SO2, levures, nutriments, gestion profil thermique, gestion O2, techniques d'extractionOpérations Post macération:Ecoulage, décuvage, pressurage du marc,FMLElevage | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T21" s="7" t="inlineStr"/>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080272/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080224/true/false/false/false</t>
         </is>
       </c>
       <c r="V21" s="7" t="inlineStr">
@@ -2854,32 +2878,32 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Ecole de la 2ème Chance (E2C)</t>
+          <t>Repérer et identifier les principaux défauts du vin</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Objectif 2ème chance - métropôle nice côte d'azur - ecole de la deuxième chance des alpes maritimes - odc nca - e2c</t>
+          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>06200 Nice</t>
+          <t>11100 Narbonne</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>455 Promenade des Anglais | Porte Arenas | 06200 Nice | France</t>
+          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1100 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 4 heures</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -2894,12 +2918,12 @@
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>contact@e2cnicecotedazur.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>contact@e2cnicecotedazur.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -2914,18 +2938,18 @@
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>04 12 05 20 05</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>04 12 05 20 05</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="O22" s="5" t="inlineStr"/>
       <c r="P22" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q22" s="5" t="inlineStr">
@@ -2936,18 +2960,18 @@
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>Programme non communiqué | Organisme | Objectif 2ème chance - métropôle nice côte d'azur - ecole de la deuxième chance des alpes maritimes - odc nca - e2c | Lieu de la formation | 455 Promenade des Anglais</t>
+          <t>Altérations d'origine microbienne:Contamination bactérienne: acescence, piqûre acétique, piqûre lactique, maladie de la tourne, maladie de l'amer, piqure mannitique, odeur de géranium, diacétyleContamination levurienne: brettanomyces, maladie de la fleur, goût de sourisOxydationRéductionMaladies dues à la qualité des raisins: les GMT, le goût herbacé-véétalAutres origines: goût de bouchon, pinking, goût d'huître, goût de lumière | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T22" s="5" t="inlineStr"/>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10681643/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080227/true/false/false/false</t>
         </is>
       </c>
       <c r="V22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W22" s="5" t="inlineStr">
@@ -2959,32 +2983,32 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Ecole de la 2ème Chance (E2C)</t>
+          <t>Vinification sans sulfites ajoutes ou à teneur réduite en sulfites</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04</t>
+          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>04000 Digne-les-Bains</t>
+          <t>11100 Narbonne</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>4 avenue de Verdun | https://www.iap.asso.fr/ | 04000 Digne-les-Bains | France</t>
+          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1100 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 4 heures</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -2994,17 +3018,17 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>https://www.iap.asso.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>contact@iap.asso.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>contact@iap.asso.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -3019,18 +3043,18 @@
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>04 92 87 46 10</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>04 92 87 46 10</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="O23" s="7" t="inlineStr"/>
       <c r="P23" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q23" s="7" t="inlineStr">
@@ -3041,18 +3065,18 @@
       <c r="R23" s="7" t="inlineStr"/>
       <c r="S23" s="7" t="inlineStr">
         <is>
-          <t>Programme non communiqué | Organisme | Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04 | https://www.iap.asso.fr/ | Lieu de la formation</t>
+          <t>Chimie du SO2Produits de substitution au SO2Gestion O2Itinéraires techniques de vinification alternatifsStabilisation et élevage des vins | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T23" s="7" t="inlineStr"/>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10685143/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080266/true/false/false/false</t>
         </is>
       </c>
       <c r="V23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W23" s="7" t="inlineStr">
@@ -3064,32 +3088,32 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Titre professionnel secrétaire assistant médico-administratif (FOAD)</t>
+          <t>Vinification en blanc: les fondamentaux</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>11100 Narbonne</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1084 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 4 heures</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -3104,12 +3128,12 @@
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -3124,48 +3148,40 @@
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="O24" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0468410152</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr"/>
       <c r="P24" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q24" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R24" s="5" t="inlineStr"/>
       <c r="S24" s="5" t="inlineStr">
         <is>
-          <t>7 projets professionnalisants vous permettront d'acquérir les compétences citées au dessus par la pratique.Vous réaliserez les projets suivants :P1 - Démarrez votre formation de secrétaire assistant médico-administratifP2 - Niveau 1 : Maîtrisez l'accueil et la gestion administrative en milieu médicalP3 - Niveau 2 : Développez vos compétences en rédaction, communication et outils numériques en milieuP4 - Réalisez votre mission en entrepriseP5 - Niveau 3 : Optimisez l'organisation, la sécuritéet la gestion des données sensibles en milieu médicalP6 - Niveau 4 : Améliorez la gestion des communications, données et environnements sanitairesP7 - Préparez votre fin de formation de secrétaire assistant médico-administratif | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T24" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel secrétaire assistant médico-administratif</t>
-        </is>
-      </c>
+          <t>Détermination du type de vin souhaitéMaturation du raisin: détermination de la date des vendangesItinéraire technique généralOpérations préfermentaires: transport, bioprotection, tri, éraflage, macération préfermentaire à froid, pressurage, débourbagePilotage de la fermentation alcoolique: SO2, levurage, nutrition azotée, gestion O2, maîtrise T°Elevage: en cuve, en barrique, sur lies fines | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+        </is>
+      </c>
+      <c r="T24" s="5" t="inlineStr"/>
       <c r="U24" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080272/true/false/false/false</t>
         </is>
       </c>
       <c r="V24" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W24" s="5" t="inlineStr">
@@ -3177,32 +3193,32 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Formation au concours d'ATSEM</t>
+          <t>Ecole de la 2ème Chance (E2C)</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>Objectif 2ème chance - métropôle nice côte d'azur - ecole de la deuxième chance des alpes maritimes - odc nca - e2c</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>06200 Nice</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>455 Promenade des Anglais | Porte Arenas | 06200 Nice | France</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Durée de 346 heures</t>
+          <t>Durée de 1100 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -3217,12 +3233,12 @@
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>contact@e2cnicecotedazur.fr</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>contact@e2cnicecotedazur.fr</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
@@ -3237,40 +3253,40 @@
       </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>04 12 05 20 05</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>04 12 05 20 05</t>
         </is>
       </c>
       <c r="O25" s="7" t="inlineStr"/>
       <c r="P25" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R25" s="7" t="inlineStr"/>
       <c r="S25" s="7" t="inlineStr">
         <is>
-          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
+          <t>Programme non communiqué | Organisme | Objectif 2ème chance - métropôle nice côte d'azur - ecole de la deuxième chance des alpes maritimes - odc nca - e2c | Lieu de la formation | 455 Promenade des Anglais</t>
         </is>
       </c>
       <c r="T25" s="7" t="inlineStr"/>
       <c r="U25" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10681643/true/false/false/false</t>
         </is>
       </c>
       <c r="V25" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W25" s="7" t="inlineStr">
@@ -3282,32 +3298,32 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Concours d'atsem (FOAD)</t>
+          <t>Ecole de la 2ème Chance (E2C)</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>04000 Digne-les-Bains</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>4 avenue de Verdun | https://www.iap.asso.fr/ | 04000 Digne-les-Bains | France</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
+          <t>Durée de 1100 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -3317,17 +3333,17 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.iap.asso.fr/</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>contact@iap.asso.fr</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>contact@iap.asso.fr</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
@@ -3342,40 +3358,40 @@
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>04 92 87 46 10</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>04 92 87 46 10</t>
         </is>
       </c>
       <c r="O26" s="5" t="inlineStr"/>
       <c r="P26" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q26" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R26" s="5" t="inlineStr"/>
       <c r="S26" s="5" t="inlineStr">
         <is>
-          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
+          <t>Programme non communiqué | Organisme | Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04 | https://www.iap.asso.fr/ | Lieu de la formation</t>
         </is>
       </c>
       <c r="T26" s="5" t="inlineStr"/>
       <c r="U26" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10685143/true/false/false/false</t>
         </is>
       </c>
       <c r="V26" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W26" s="5" t="inlineStr">
@@ -3392,12 +3408,12 @@
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Titre professionnel secrétaire assistant médico-administratif (FOAD)</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -3412,7 +3428,7 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 1084 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -3427,12 +3443,12 @@
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
@@ -3447,12 +3463,12 @@
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O27" s="7" t="inlineStr">
@@ -3473,17 +3489,17 @@
       <c r="R27" s="7" t="inlineStr"/>
       <c r="S27" s="7" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>7 projets professionnalisants vous permettront d'acquérir les compétences citées au dessus par la pratique.Vous réaliserez les projets suivants :P1 - Démarrez votre formation de secrétaire assistant médico-administratifP2 - Niveau 1 : Maîtrisez l'accueil et la gestion administrative en milieu médicalP3 - Niveau 2 : Développez vos compétences en rédaction, communication et outils numériques en milieuP4 - Réalisez votre mission en entrepriseP5 - Niveau 3 : Optimisez l'organisation, la sécuritéet la gestion des données sensibles en milieu médicalP6 - Niveau 4 : Améliorez la gestion des communications, données et environnements sanitairesP7 - Préparez votre fin de formation de secrétaire assistant médico-administratif | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel secrétaire assistant médico-administratif</t>
         </is>
       </c>
       <c r="U27" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/false</t>
         </is>
       </c>
       <c r="V27" s="7" t="inlineStr">
@@ -3505,12 +3521,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Préparation au concours d'ATSEM</t>
+          <t>Formation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>AFEC (Siège)</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -3525,7 +3541,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 346 heures</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -3540,12 +3556,12 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
@@ -3560,12 +3576,12 @@
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>0153368844</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>0153368844</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O28" s="5" t="inlineStr"/>
@@ -3582,13 +3598,13 @@
       <c r="R28" s="5" t="inlineStr"/>
       <c r="S28" s="5" t="inlineStr">
         <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC (Siège) | Lieu de la formation | Formation a distance</t>
+          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T28" s="5" t="inlineStr"/>
       <c r="U28" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/false</t>
         </is>
       </c>
       <c r="V28" s="5" t="inlineStr">
@@ -3610,12 +3626,12 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
+          <t>Concours d'atsem (FOAD)</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
@@ -3630,7 +3646,7 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -3645,12 +3661,12 @@
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
@@ -3665,12 +3681,12 @@
       </c>
       <c r="M29" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="O29" s="7" t="inlineStr"/>
@@ -3687,13 +3703,13 @@
       <c r="R29" s="7" t="inlineStr"/>
       <c r="S29" s="7" t="inlineStr">
         <is>
-          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T29" s="7" t="inlineStr"/>
       <c r="U29" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/false</t>
         </is>
       </c>
       <c r="V29" s="7" t="inlineStr">
@@ -3715,12 +3731,12 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -3735,7 +3751,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -3750,12 +3766,12 @@
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -3770,15 +3786,19 @@
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
-        </is>
-      </c>
-      <c r="O30" s="5" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O30" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P30" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -3792,13 +3812,17 @@
       <c r="R30" s="5" t="inlineStr"/>
       <c r="S30" s="5" t="inlineStr">
         <is>
-          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T30" s="5" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T30" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+        </is>
+      </c>
       <c r="U30" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/false</t>
         </is>
       </c>
       <c r="V30" s="5" t="inlineStr">
@@ -3820,12 +3844,12 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
+          <t>Préparation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>AFEC (Siège)</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -3840,7 +3864,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -3855,12 +3879,12 @@
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
@@ -3875,12 +3899,12 @@
       </c>
       <c r="M31" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="N31" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="O31" s="7" t="inlineStr"/>
@@ -3897,13 +3921,13 @@
       <c r="R31" s="7" t="inlineStr"/>
       <c r="S31" s="7" t="inlineStr">
         <is>
-          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC (Siège) | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T31" s="7" t="inlineStr"/>
       <c r="U31" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/false</t>
         </is>
       </c>
       <c r="V31" s="7" t="inlineStr">
@@ -3925,12 +3949,12 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>BP option aménagements paysagers</t>
+          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -3945,7 +3969,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
@@ -3960,12 +3984,12 @@
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr | cecile.iribarne@educagri.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
@@ -3980,19 +4004,15 @@
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>0479264427</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>0479264427</t>
-        </is>
-      </c>
-      <c r="O32" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O32" s="5" t="inlineStr"/>
       <c r="P32" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -4006,17 +4026,13 @@
       <c r="R32" s="5" t="inlineStr"/>
       <c r="S32" s="5" t="inlineStr">
         <is>
-          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T32" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
-        </is>
-      </c>
+          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T32" s="5" t="inlineStr"/>
       <c r="U32" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/false</t>
         </is>
       </c>
       <c r="V32" s="5" t="inlineStr">
@@ -4038,12 +4054,12 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>CAP Fleuriste</t>
+          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -4058,7 +4074,7 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -4073,12 +4089,12 @@
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
@@ -4093,19 +4109,15 @@
       </c>
       <c r="M33" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N33" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O33" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O33" s="7" t="inlineStr"/>
       <c r="P33" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -4119,17 +4131,13 @@
       <c r="R33" s="7" t="inlineStr"/>
       <c r="S33" s="7" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T33" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
-        </is>
-      </c>
+          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T33" s="7" t="inlineStr"/>
       <c r="U33" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/false</t>
         </is>
       </c>
       <c r="V33" s="7" t="inlineStr">
@@ -4146,32 +4154,32 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>E2C - Ecole de la Deuxième Chance</t>
+          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Ecole de la Deuxième Chance Grand Hainaut</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>02140 Vervins</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Ecole de la deuxième chance - site de VERVINS | 3 Place des Anciens Combattants | 02140 Vervins | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1400 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
@@ -4186,12 +4194,12 @@
       </c>
       <c r="I34" s="6" t="inlineStr">
         <is>
-          <t>c.renaud@e2cgrandhainaut.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>c.renaud@e2cgrandhainaut.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K34" s="5" t="inlineStr">
@@ -4206,40 +4214,40 @@
       </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
-          <t>0375310010</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N34" s="5" t="inlineStr">
         <is>
-          <t>0375310010</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="O34" s="5" t="inlineStr"/>
       <c r="P34" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q34" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R34" s="5" t="inlineStr"/>
       <c r="S34" s="5" t="inlineStr">
         <is>
-          <t>Savoir fondamentauxOrientation et démarches professionnelsSocialisation et développement personnelAlternance en entreprise (près de 30% du temps)Des outils pédagogiques de liaison, d'évaluation et de suivi9 mois maximum + 12 mois de suivi post-parcours | Organisme | Ecole de la Deuxième Chance Grand Hainaut | Lieu de la formation | Ecole de la deuxième chance - site de VERVINS</t>
+          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T34" s="5" t="inlineStr"/>
       <c r="U34" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11072382/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/false</t>
         </is>
       </c>
       <c r="V34" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W34" s="5" t="inlineStr">
@@ -4251,17 +4259,17 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Préparation au concours d'adjoint administratif d'État principal de 2ème classe</t>
+          <t>BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school)</t>
+          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
@@ -4276,7 +4284,7 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Durée de 335 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -4291,12 +4299,12 @@
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>foad@skillandyou.com</t>
+          <t>epl.la-motte-servolex@educagri.fr</t>
         </is>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>foad@skillandyou.com</t>
+          <t>epl.la-motte-servolex@educagri.fr | cecile.iribarne@educagri.fr</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
@@ -4311,15 +4319,19 @@
       </c>
       <c r="M35" s="7" t="inlineStr">
         <is>
-          <t>0146006878</t>
+          <t>0479264427</t>
         </is>
       </c>
       <c r="N35" s="7" t="inlineStr">
         <is>
-          <t>0146006878</t>
-        </is>
-      </c>
-      <c r="O35" s="7" t="inlineStr"/>
+          <t>0479264427</t>
+        </is>
+      </c>
+      <c r="O35" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P35" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -4333,18 +4345,22 @@
       <c r="R35" s="7" t="inlineStr"/>
       <c r="S35" s="7" t="inlineStr">
         <is>
-          <t>Votre intégration - Guide d'intégration - Bienvenue dans votre formation - Guide Métier Adjoint administratif d'État principal de 2ème classe - Guide de la formation - Guide des épreuves - Le concours d'adjoint administratif d'État principal de 2ème classe Aide à la réalisation de vos documents professionnels Compléter votre livret de suivi des compétences professionnelles Retranscrire et ordonner les idées principales d'un texte Annales corrigées Épreuves blanches Solliciter les connaissances fondamentales pour le concours Comprendre l'administration française Comprendre le fonctionnement des institutions françaises Acquérir des connaissances en français Acquérir une bonne culture générale Mathématiques Les tests d'aptitudes verbales Annales corrigées Épreuves blanches Mobiliser les compétences professionnelles de l'adjoint administratif d'État Bureautique Épreuves blanches Techniques et recherche d'emploi/stage Sensibilisation au développement durable | Organisme | Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school) | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T35" s="7" t="inlineStr"/>
+          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T35" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
+        </is>
+      </c>
       <c r="U35" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11205913/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/false</t>
         </is>
       </c>
       <c r="V35" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W35" s="7" t="inlineStr">
@@ -4356,17 +4372,17 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Certification CLOE français langue étrangère - spécialité hôtellerie Restauration niveau A2 vers B1 (FOAD)</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Nepsod Evolution</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -4381,7 +4397,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Durée de 331 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
@@ -4396,12 +4412,12 @@
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>accueil@nepsod.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>accueil@nepsod.com</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
@@ -4416,12 +4432,12 @@
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>0474639587</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N36" s="5" t="inlineStr">
         <is>
-          <t>0474639587</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="O36" s="5" t="inlineStr">
@@ -4442,22 +4458,22 @@
       <c r="R36" s="5" t="inlineStr"/>
       <c r="S36" s="5" t="inlineStr">
         <is>
-          <t>Accueil et initiation à la formation (1h30) - Module FLE visée insertion professionnelle : chercher un emploi, présenter son métier, présenter ses projets, interagir avec ses collègues, manipuler les outils numériques (120h30) - Module FOS Hôtellerie Restauration :découvrir la cuisine, travailler en cuisine, identifier les besoins d'un client, présenter des produits et services, gérer les réclamations (50h) Module environnement social et culturel : vie quotidienne et relations sociales, loisirs, patrimoine, citoyenneté et engagement (43h) Module Préparation et recherche de stage en entreprise (14h) Période de stage en entreprise (35 h) Module remise à niveau numérique (35 h maximum) Module accompagnement à l'après-formation (21h maximum) Module Préparation et passage de la certification CLOE (10h) Bilan final (1h) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T36" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Certification CLOE français langue étrangère</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
         </is>
       </c>
       <c r="U36" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11576792/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/false</t>
         </is>
       </c>
       <c r="V36" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W36" s="5" t="inlineStr">
@@ -4469,32 +4485,32 @@
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière) - DEI</t>
+          <t>E2C - Ecole de la Deuxième Chance</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Ecole de la Deuxième Chance Grand Hainaut</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>02140 Vervins</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+          <t>Ecole de la deuxième chance - site de VERVINS | 3 Place des Anciens Combattants | 02140 Vervins | France</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 1400 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -4509,12 +4525,12 @@
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>c.renaud@e2cgrandhainaut.fr</t>
         </is>
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>c.renaud@e2cgrandhainaut.fr</t>
         </is>
       </c>
       <c r="K37" s="7" t="inlineStr">
@@ -4529,19 +4545,15 @@
       </c>
       <c r="M37" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0375310010</t>
         </is>
       </c>
       <c r="N37" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
-        </is>
-      </c>
-      <c r="O37" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0375310010</t>
+        </is>
+      </c>
+      <c r="O37" s="7" t="inlineStr"/>
       <c r="P37" s="7" t="inlineStr">
         <is>
           <t>Formation financée par la région</t>
@@ -4555,22 +4567,18 @@
       <c r="R37" s="7" t="inlineStr"/>
       <c r="S37" s="7" t="inlineStr">
         <is>
-          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail (bureautique,recherche documentaire, rédaction de documents écrits, communication, anglais) La formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de1 800h, sous la forme de cours magistraux (750 h) travaux dirigés (1 050 h) le travail personnel guidé (suivi pédagogique, temps personnel guidé, supervision, travaux entre étudiants- 300 h) la formation clinique de 2 100 h le travail personnel complémentaire est estimé à 900 heures environ, soit 300 h par an. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T37" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
-        </is>
-      </c>
+          <t>Savoir fondamentauxOrientation et démarches professionnelsSocialisation et développement personnelAlternance en entreprise (près de 30% du temps)Des outils pédagogiques de liaison, d'évaluation et de suivi9 mois maximum + 12 mois de suivi post-parcours | Organisme | Ecole de la Deuxième Chance Grand Hainaut | Lieu de la formation | Ecole de la deuxième chance - site de VERVINS</t>
+        </is>
+      </c>
+      <c r="T37" s="7" t="inlineStr"/>
       <c r="U37" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11533526/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11072382/true/false/false/true</t>
         </is>
       </c>
       <c r="V37" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W37" s="7" t="inlineStr">
@@ -4587,27 +4595,27 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État de technicien de laboratoire médical</t>
+          <t>Préparation au concours d'adjoint administratif d'État principal de 2ème classe</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Association des Fondateurs et Protecteurs de l'Institut Catholique de Lyon (AFPICL) (UCLy - Institut Catholique de Lyon)</t>
+          <t>Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school)</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>69002 Lyon 2e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>10 place des Archives | 69002 Lyon 2e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1120 heures</t>
+          <t>Durée de 335 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
@@ -4622,12 +4630,12 @@
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>fp@univ-catholyon.fr</t>
+          <t>foad@skillandyou.com</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>fp@univ-catholyon.fr</t>
+          <t>foad@skillandyou.com</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
@@ -4642,39 +4650,35 @@
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
-          <t>0472325134</t>
+          <t>0146006878</t>
         </is>
       </c>
       <c r="N38" s="5" t="inlineStr">
         <is>
-          <t>0472325134</t>
-        </is>
-      </c>
-      <c r="O38" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0146006878</t>
+        </is>
+      </c>
+      <c r="O38" s="5" t="inlineStr"/>
       <c r="P38" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q38" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R38" s="5" t="inlineStr"/>
-      <c r="S38" s="5" t="inlineStr"/>
-      <c r="T38" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État de technicien de laboratoire médical</t>
-        </is>
-      </c>
+      <c r="S38" s="5" t="inlineStr">
+        <is>
+          <t>Votre intégration - Guide d'intégration - Bienvenue dans votre formation - Guide Métier Adjoint administratif d'État principal de 2ème classe - Guide de la formation - Guide des épreuves - Le concours d'adjoint administratif d'État principal de 2ème classe Aide à la réalisation de vos documents professionnels Compléter votre livret de suivi des compétences professionnelles Retranscrire et ordonner les idées principales d'un texte Annales corrigées Épreuves blanches Solliciter les connaissances fondamentales pour le concours Comprendre l'administration française Comprendre le fonctionnement des institutions françaises Acquérir des connaissances en français Acquérir une bonne culture générale Mathématiques Les tests d'aptitudes verbales Annales corrigées Épreuves blanches Mobiliser les compétences professionnelles de l'adjoint administratif d'État Bureautique Épreuves blanches Techniques et recherche d'emploi/stage Sensibilisation au développement durable | Organisme | Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school) | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T38" s="5" t="inlineStr"/>
       <c r="U38" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11026378/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11205913/true/false/true/true</t>
         </is>
       </c>
       <c r="V38" s="5" t="inlineStr">
@@ -4696,27 +4700,27 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'ambulancier</t>
+          <t>Certification CLOE français langue étrangère - spécialité hôtellerie Restauration niveau A2 vers B1 (FOAD)</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+          <t>Nepsod Evolution</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Durée de 801 heures (dont 245 heures en entreprise)</t>
+          <t>Durée de 331 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -4731,12 +4735,12 @@
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>accueil@nepsod.com</t>
         </is>
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>accueil@nepsod.com</t>
         </is>
       </c>
       <c r="K39" s="7" t="inlineStr">
@@ -4751,12 +4755,12 @@
       </c>
       <c r="M39" s="7" t="inlineStr">
         <is>
-          <t>0472117903</t>
+          <t>0474639587</t>
         </is>
       </c>
       <c r="N39" s="7" t="inlineStr">
         <is>
-          <t>0472117903</t>
+          <t>0474639587</t>
         </is>
       </c>
       <c r="O39" s="7" t="inlineStr">
@@ -4766,33 +4770,33 @@
       </c>
       <c r="P39" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q39" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R39" s="7" t="inlineStr"/>
       <c r="S39" s="7" t="inlineStr">
         <is>
-          <t>Non renseigne | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Accueil et initiation à la formation (1h30) - Module FLE visée insertion professionnelle : chercher un emploi, présenter son métier, présenter ses projets, interagir avec ses collègues, manipuler les outils numériques (120h30) - Module FOS Hôtellerie Restauration :découvrir la cuisine, travailler en cuisine, identifier les besoins d'un client, présenter des produits et services, gérer les réclamations (50h) Module environnement social et culturel : vie quotidienne et relations sociales, loisirs, patrimoine, citoyenneté et engagement (43h) Module Préparation et recherche de stage en entreprise (14h) Période de stage en entreprise (35 h) Module remise à niveau numérique (35 h maximum) Module accompagnement à l'après-formation (21h maximum) Module Préparation et passage de la certification CLOE (10h) Bilan final (1h) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T39" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'ambulancier</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Certification CLOE français langue étrangère</t>
         </is>
       </c>
       <c r="U39" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11871421/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11576792/true/false/true/false</t>
         </is>
       </c>
       <c r="V39" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W39" s="7" t="inlineStr">
@@ -4809,27 +4813,27 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Agent de prévention et de sécurité - Titre à finalité professionnelle (TFP APS)</t>
+          <t>Diplôme d'État d'infirmier(ière) - DEI</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Global pro formation (Global pro formation (GPF))</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Blue Concept | 16 Rue Marcel Dutartre | 69100 Villeurbanne | France</t>
+          <t>115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Durée de 379 heures (dont 70 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
@@ -4844,12 +4848,12 @@
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>globalproformation@gmail.com</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>globalproformation@gmail.com</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K40" s="5" t="inlineStr">
@@ -4864,12 +4868,12 @@
       </c>
       <c r="M40" s="5" t="inlineStr">
         <is>
-          <t>0666139535</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N40" s="5" t="inlineStr">
         <is>
-          <t>0666139535</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O40" s="5" t="inlineStr">
@@ -4879,7 +4883,7 @@
       </c>
       <c r="P40" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q40" s="5" t="inlineStr">
@@ -4890,17 +4894,17 @@
       <c r="R40" s="5" t="inlineStr"/>
       <c r="S40" s="5" t="inlineStr">
         <is>
-          <t>Théorie : SST : Protéger, Examiner (saignement, étouffement, conscience et respiration) et alerter (alerte et message d'accueil) La déontologie de l'agent de sécurité Les services publics de police et gendarmerie, le CNAPS Le cadre légal de la profession, le code pénal et le code de procédure pénale La sûreté de l'État Les armes Mise en sûreté et neutralisation des armes Prévention et actes terrorisme L'accueil, le contrôle d'accès, le contrôle visuel et la palpation de sécurité La prise en compte d'un poste de contrôle de sécurité et les consignes La protection du travailleur Isolé Le circuit de vérification La gestion des alarmes intrusion et incendie, la vidéo et la télésurveillance (surveillance et gardiennage) Les techniques d'information, de communication et la gestion des conflits L'incendie et les risques majeurs Le risque électrique (initiation) Le cadre légal et la problématique de l'activité d'événementiel La définition du terrorisme (historique, mécanisme, méthodologie et modes opératoires) Les différentes menaces terroristes et les niveaux de risque associés La prévention des actes de terrorisme par la reconnaissance des comportements suspects (profiling) et de la radicalisation violente L'action en cas d'attaque et suivant le type d'attaque (actes réflexes, mesures de mise en sécurité immédiate) Le combat en dernier recours L'alerte et la facilitation de l'intervention des forces de l'ordre La sécurisation d'une zone dans l'urgence, risque de sur-attentat et post-attentat. Pratique : Mise en pratique SST CQP APS: Code de la sécurité intérieure Code pénal et libertés publiques Déontologie professionnelle Secours à personnes (SST) Situations conflictuelles et résolution de conflit Consignes, compte rendu et rapport Gestion des risques majeurs, électriques, incendie Gestion d'alarmes Technique d'information et de communication Préparation d'une mission Gestion de conflit Contrôle d'accès Poste de contrôle de sécurité Rondes Palpation de sécurité et inspection de bagages Télésurveillance et vidéo protection Sensibilisation aux risques terroristes Examen : en cours de formation UV 1 (secourisme) : le candidat sera déclaré apte ou inapte en fonction des résultats de la grille d'évaluation conforme aux procédures de validation de l'INRS. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
+          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail (bureautique,recherche documentaire, rédaction de documents écrits, communication, anglais) La formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de1 800h, sous la forme de cours magistraux (750 h) travaux dirigés (1 050 h) le travail personnel guidé (suivi pédagogique, temps personnel guidé, supervision, travaux entre étudiants- 300 h) la formation clinique de 2 100 h le travail personnel complémentaire est estimé à 900 heures environ, soit 300 h par an. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T40" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Agent de prévention et de sécurité</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U40" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11870188/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11533526/true/false/false/false</t>
         </is>
       </c>
       <c r="V40" s="5" t="inlineStr">
@@ -4922,27 +4926,27 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'Etat de la Jeunesse de l'Education Populaire et du Sport spécialité "animation socio-éducative ou culturelle mention "coordination de projets" - RNCP 39930 spécialité "animation socio-éducative ou culturel mention "coordination de projets</t>
+          <t>Diplôme d'État de technicien de laboratoire médical</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+          <t>Association des Fondateurs et Protecteurs de l'Institut Catholique de Lyon (AFPICL) (UCLy - Institut Catholique de Lyon)</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>69002 Lyon 2e</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+          <t>10 place des Archives | 69002 Lyon 2e | France</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 1120 heures</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -4952,17 +4956,17 @@
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>https://arfatsema.catalogueformpro.com/3/dejeps-17/2857880/diplome-detat-de-la-jeunesse-de-leducation-populaire-et-du-sport-dejeps-17-specialite-animation-soci/registration?session_id=2846144</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>fp@univ-catholyon.fr</t>
         </is>
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>fp@univ-catholyon.fr</t>
         </is>
       </c>
       <c r="K41" s="7" t="inlineStr">
@@ -4977,12 +4981,12 @@
       </c>
       <c r="M41" s="7" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0472325134</t>
         </is>
       </c>
       <c r="N41" s="7" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0472325134</t>
         </is>
       </c>
       <c r="O41" s="7" t="inlineStr">
@@ -4992,7 +4996,7 @@
       </c>
       <c r="P41" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q41" s="7" t="inlineStr">
@@ -5001,19 +5005,15 @@
         </is>
       </c>
       <c r="R41" s="7" t="inlineStr"/>
-      <c r="S41" s="7" t="inlineStr">
-        <is>
-          <t>BC1: Animer et accompagner une équipe dans le champ du sport ou de l'animation Animer une équipe en structure d'éducation populaire : enjeux éthiques, valeurs et spécificités Réaliser un diagnostic des ressources humaines de son périmètre d'intervention Animer une équipe en structure d'éducation populaire : organisation, cadre légal, réglementation et procédures Diversité et inclusion : analyser les besoins et mettre en place une organisation adaptée Management participatif : développer le pouvoir d'agir d'une équipe Management participatif : outils et pratiques Accompagner une équipe: médiation et gestion de conflits Accompagner une équipe : émancipation et développement de l'autonomie Dynamique de groupe Animer un processus démocratique Projet d'action formative et conception de séance formative Droit du travail/Droit social Communication non violente Outils d'animation collective Outils d'accompagnement individuel Accompagner la vulnérabilité Dialogue social et syndical Responsabilité du coordinateur Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? BC2: Concevoir un projet d'action dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Education Populaire Rapport de domination Le numérique comme un fait social Esprit critique Culture politique Démocratie et contre pouvoir Pouvoir d'agir ou devoir d'agir? Diagnostic et enjeux De l'attribution d'une place à une culture de la participation Famille et éducation Connaissance des institutions publics et relation aux association ingéniérie sociale Portrait de territoire Mesure de l'impact social BC3 : Mettre en oeuvre et évaluer un projet d'action Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie de projet Mesure de l'impact social Accompagner la vulnérabilité La protection de l'Enfance en France Outils participatifs Intelligence artificielle et fonction de coordination BC4 : Développer les partenariats opérationnelles et contribuer aux dynamiques institutionnelles dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Connaissance des institutions publics et relation aux associations Démocratie et contre pouvoir Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie sociale Outils participatifs | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
+      <c r="S41" s="7" t="inlineStr"/>
       <c r="T41" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | DEJEPS spécialité animation socio-éducative ou culturelle mention coordination de projets</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État de technicien de laboratoire médical</t>
         </is>
       </c>
       <c r="U41" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880827/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11026378/true/false/false/false</t>
         </is>
       </c>
       <c r="V41" s="7" t="inlineStr">
@@ -5035,27 +5035,27 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Créez votre vignoble bio de raisin de table, rentable et résilient - Devenez autonome pour produire et vendre votre propre raisin de table bio</t>
+          <t>Diplôme d'État d'ambulancier</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>SARL Agri-learn éditions</t>
+          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>69001 Lyon</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 69001 Lyon | France</t>
+          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Durée de 9 heures</t>
+          <t>Durée de 801 heures (dont 245 heures en entreprise)</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
@@ -5070,12 +5070,12 @@
       </c>
       <c r="I42" s="6" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="K42" s="5" t="inlineStr">
@@ -5090,35 +5090,43 @@
       </c>
       <c r="M42" s="5" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0472117903</t>
         </is>
       </c>
       <c r="N42" s="5" t="inlineStr">
         <is>
-          <t>0620021214</t>
-        </is>
-      </c>
-      <c r="O42" s="5" t="inlineStr"/>
+          <t>0472117903</t>
+        </is>
+      </c>
+      <c r="O42" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q42" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R42" s="5" t="inlineStr"/>
       <c r="S42" s="5" t="inlineStr">
         <is>
-          <t>1. Taille de la vigne Principes de taille (formation et production) Techniques de taille douce Entretien et corrections2. Modes de conduite Choix du système (lyre, gable, plan vertical. Comparaison des conduites Adaptation au contexte pédoclimatique3. Fertilité des sols Gestion du sol (travail / non-travail) Irrigation Maintien de la fertilité en bio4. Travaux du vignoble Protection contre maladies et ravageurs Calendrier des interventions Conduite sous abri (tunnel)5. Choix des plants Sélection des variétés Choix du porte-greffe Adaptation au marché et au terroir6. Plantation Préparation du sol Étapes de plantation Coûts et organisation7. Récolte et commercialisation Récolte et conservation Organisation du travail Valorisation et vente8. Protection du vignoble en bio Biocontrôle et PNPP Réduction des intrants Stratégies alternatives9. Gestion des maladies et ravageurs Identification des principaux risques Prévention et lutte adaptée10. Pilotage des traitements Stratégie cuivre / soufre Optimisation des doses11. Approche agroécologique Biodiversité fonctionnelle Variétés résistantes | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T42" s="5" t="inlineStr"/>
+          <t>Non renseigne | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T42" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'ambulancier</t>
+        </is>
+      </c>
       <c r="U42" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11870193/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11871421/true/false/false/false</t>
         </is>
       </c>
       <c r="V42" s="5" t="inlineStr">
@@ -5140,27 +5148,27 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
+          <t>Agent de prévention et de sécurité - Titre à finalité professionnelle (TFP APS)</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>UCPA Formation</t>
+          <t>Global pro formation (Global pro formation (GPF))</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>69200 Vénissieux</t>
+          <t>69100 Villeurbanne</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>16 Avenue Dr Georges Levy | 69200 Vénissieux | France</t>
+          <t>Blue Concept | 16 Rue Marcel Dutartre | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1267 heures (dont 637 heures en entreprise)</t>
+          <t>Durée de 379 heures (dont 70 heures en entreprise)</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -5175,12 +5183,12 @@
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>ucpa-formation@ucpa.asso.fr</t>
+          <t>globalproformation@gmail.com</t>
         </is>
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
-          <t>ucpa-formation@ucpa.asso.fr | fgehant@ucpa.asso.fr</t>
+          <t>globalproformation@gmail.com</t>
         </is>
       </c>
       <c r="K43" s="7" t="inlineStr">
@@ -5195,12 +5203,12 @@
       </c>
       <c r="M43" s="7" t="inlineStr">
         <is>
-          <t>0642833617</t>
+          <t>0666139535</t>
         </is>
       </c>
       <c r="N43" s="7" t="inlineStr">
         <is>
-          <t>0642833617</t>
+          <t>0666139535</t>
         </is>
       </c>
       <c r="O43" s="7" t="inlineStr">
@@ -5210,7 +5218,7 @@
       </c>
       <c r="P43" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q43" s="7" t="inlineStr">
@@ -5221,22 +5229,22 @@
       <c r="R43" s="7" t="inlineStr"/>
       <c r="S43" s="7" t="inlineStr">
         <is>
-          <t>Unité capitalisable (UC) - 1. Encadrer tout public dans tout lieu et toute structureUnité capitalisable (UC) - 2. Mettre en œuvre un projet d'animation s'inscrivant dans le projet de la structureUnité capitalisable (UC) - 3. Conduire une séance, un cycle d'animation ou d'apprentissage dans le champ des activités aquatiques et de la natationUnité capitalisable (UC) - 4. Mobiliser les techniques des activités aquatiques et de la natation pour mettre en œuvre une séance ou un cycle d'apprentissage | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Théorie : SST : Protéger, Examiner (saignement, étouffement, conscience et respiration) et alerter (alerte et message d'accueil) La déontologie de l'agent de sécurité Les services publics de police et gendarmerie, le CNAPS Le cadre légal de la profession, le code pénal et le code de procédure pénale La sûreté de l'État Les armes Mise en sûreté et neutralisation des armes Prévention et actes terrorisme L'accueil, le contrôle d'accès, le contrôle visuel et la palpation de sécurité La prise en compte d'un poste de contrôle de sécurité et les consignes La protection du travailleur Isolé Le circuit de vérification La gestion des alarmes intrusion et incendie, la vidéo et la télésurveillance (surveillance et gardiennage) Les techniques d'information, de communication et la gestion des conflits L'incendie et les risques majeurs Le risque électrique (initiation) Le cadre légal et la problématique de l'activité d'événementiel La définition du terrorisme (historique, mécanisme, méthodologie et modes opératoires) Les différentes menaces terroristes et les niveaux de risque associés La prévention des actes de terrorisme par la reconnaissance des comportements suspects (profiling) et de la radicalisation violente L'action en cas d'attaque et suivant le type d'attaque (actes réflexes, mesures de mise en sécurité immédiate) Le combat en dernier recours L'alerte et la facilitation de l'intervention des forces de l'ordre La sécurisation d'une zone dans l'urgence, risque de sur-attentat et post-attentat. Pratique : Mise en pratique SST CQP APS: Code de la sécurité intérieure Code pénal et libertés publiques Déontologie professionnelle Secours à personnes (SST) Situations conflictuelles et résolution de conflit Consignes, compte rendu et rapport Gestion des risques majeurs, électriques, incendie Gestion d'alarmes Technique d'information et de communication Préparation d'une mission Gestion de conflit Contrôle d'accès Poste de contrôle de sécurité Rondes Palpation de sécurité et inspection de bagages Télésurveillance et vidéo protection Sensibilisation aux risques terroristes Examen : en cours de formation UV 1 (secourisme) : le candidat sera déclaré apte ou inapte en fonction des résultats de la grille d'évaluation conforme aux procédures de validation de l'INRS. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
         </is>
       </c>
       <c r="T43" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Agent de prévention et de sécurité</t>
         </is>
       </c>
       <c r="U43" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11447001/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11870188/true/false/false/false</t>
         </is>
       </c>
       <c r="V43" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W43" s="7" t="inlineStr">
@@ -5253,27 +5261,27 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'aide-soignant - DEAS</t>
+          <t>Diplôme d'Etat de la Jeunesse de l'Education Populaire et du Sport spécialité "animation socio-éducative ou culturelle mention "coordination de projets" - RNCP 39930 spécialité "animation socio-éducative ou culturel mention "coordination de projets</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>69100 Villeurbanne</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1540 heures (dont 770 heures en entreprise)</t>
+          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
@@ -5283,17 +5291,17 @@
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=aide-soignant</t>
+          <t>https://arfatsema.catalogueformpro.com/3/dejeps-17/2857880/diplome-detat-de-la-jeunesse-de-leducation-populaire-et-du-sport-dejeps-17-specialite-animation-soci/registration?session_id=2846144</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="K44" s="5" t="inlineStr">
@@ -5308,12 +5316,12 @@
       </c>
       <c r="M44" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0478031711</t>
         </is>
       </c>
       <c r="N44" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0478031711</t>
         </is>
       </c>
       <c r="O44" s="5" t="inlineStr">
@@ -5323,7 +5331,7 @@
       </c>
       <c r="P44" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q44" s="5" t="inlineStr">
@@ -5334,22 +5342,22 @@
       <c r="R44" s="5" t="inlineStr"/>
       <c r="S44" s="5" t="inlineStr">
         <is>
-          <t>La formation conduisant au diplôme d'État d'aide-soignant, 17 semaines d'enseignement théoriques organisées autour de 8 modules : Accompagnement d'une personne dans les activités de la vie quotidienne L'état clinique d'une personne Les soins Ergonomie Relation Communication Hygiène des locaux hospitaliers Transmission des informations Organisation du travail Les titulaires du DE d'auxiliaire de puériculture, du DE d'aide médico-psychologique, du DE d'auxiliaire de vie sociale ou de la MC aide à domicile, sont dispensés de certaines unités de formation. La formation comprend également 6 stages d'une durée totale de 24 semaines en milieu hospitalier ou extra-hospitalier. Possibilité d'effectuer la formation en initial ou en apprentissage. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>BC1: Animer et accompagner une équipe dans le champ du sport ou de l'animation Animer une équipe en structure d'éducation populaire : enjeux éthiques, valeurs et spécificités Réaliser un diagnostic des ressources humaines de son périmètre d'intervention Animer une équipe en structure d'éducation populaire : organisation, cadre légal, réglementation et procédures Diversité et inclusion : analyser les besoins et mettre en place une organisation adaptée Management participatif : développer le pouvoir d'agir d'une équipe Management participatif : outils et pratiques Accompagner une équipe: médiation et gestion de conflits Accompagner une équipe : émancipation et développement de l'autonomie Dynamique de groupe Animer un processus démocratique Projet d'action formative et conception de séance formative Droit du travail/Droit social Communication non violente Outils d'animation collective Outils d'accompagnement individuel Accompagner la vulnérabilité Dialogue social et syndical Responsabilité du coordinateur Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? BC2: Concevoir un projet d'action dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Education Populaire Rapport de domination Le numérique comme un fait social Esprit critique Culture politique Démocratie et contre pouvoir Pouvoir d'agir ou devoir d'agir? Diagnostic et enjeux De l'attribution d'une place à une culture de la participation Famille et éducation Connaissance des institutions publics et relation aux association ingéniérie sociale Portrait de territoire Mesure de l'impact social BC3 : Mettre en oeuvre et évaluer un projet d'action Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie de projet Mesure de l'impact social Accompagner la vulnérabilité La protection de l'Enfance en France Outils participatifs Intelligence artificielle et fonction de coordination BC4 : Développer les partenariats opérationnelles et contribuer aux dynamiques institutionnelles dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Connaissance des institutions publics et relation aux associations Démocratie et contre pouvoir Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie sociale Outils participatifs | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T44" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'aide-soignant</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | DEJEPS spécialité animation socio-éducative ou culturelle mention coordination de projets</t>
         </is>
       </c>
       <c r="U44" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11533549/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11880827/true/false/false/false</t>
         </is>
       </c>
       <c r="V44" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W44" s="5" t="inlineStr">
@@ -5366,27 +5374,27 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>Créez votre vignoble bio de raisin de table, rentable et résilient - Devenez autonome pour produire et vendre votre propre raisin de table bio</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+          <t>SARL Agri-learn éditions</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>69001 Lyon</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 69001 Lyon | France</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 9 heures</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -5401,12 +5409,12 @@
       </c>
       <c r="I45" s="6" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="K45" s="7" t="inlineStr">
@@ -5421,39 +5429,35 @@
       </c>
       <c r="M45" s="7" t="inlineStr">
         <is>
-          <t>0472117979</t>
+          <t>0620021214</t>
         </is>
       </c>
       <c r="N45" s="7" t="inlineStr">
         <is>
-          <t>0472117979</t>
-        </is>
-      </c>
-      <c r="O45" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="O45" s="7" t="inlineStr"/>
       <c r="P45" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q45" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R45" s="7" t="inlineStr"/>
-      <c r="S45" s="7" t="inlineStr"/>
-      <c r="T45" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
-        </is>
-      </c>
+      <c r="S45" s="7" t="inlineStr">
+        <is>
+          <t>1. Taille de la vigne Principes de taille (formation et production) Techniques de taille douce Entretien et corrections2. Modes de conduite Choix du système (lyre, gable, plan vertical. Comparaison des conduites Adaptation au contexte pédoclimatique3. Fertilité des sols Gestion du sol (travail / non-travail) Irrigation Maintien de la fertilité en bio4. Travaux du vignoble Protection contre maladies et ravageurs Calendrier des interventions Conduite sous abri (tunnel)5. Choix des plants Sélection des variétés Choix du porte-greffe Adaptation au marché et au terroir6. Plantation Préparation du sol Étapes de plantation Coûts et organisation7. Récolte et commercialisation Récolte et conservation Organisation du travail Valorisation et vente8. Protection du vignoble en bio Biocontrôle et PNPP Réduction des intrants Stratégies alternatives9. Gestion des maladies et ravageurs Identification des principaux risques Prévention et lutte adaptée10. Pilotage des traitements Stratégie cuivre / soufre Optimisation des doses11. Approche agroécologique Biodiversité fonctionnelle Variétés résistantes | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T45" s="7" t="inlineStr"/>
       <c r="U45" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11817055/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11870193/true/false/false/false</t>
         </is>
       </c>
       <c r="V45" s="7" t="inlineStr">
@@ -5475,27 +5479,27 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'assistant de service social - DE ASS</t>
+          <t>BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>UCPA Formation</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>69200 Vénissieux</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 avenue Lacassagne | Croix Rouge francaise | 69003 Lyon 3e | France</t>
+          <t>16 Avenue Dr Georges Levy | 69200 Vénissieux | France</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Durée de 3420 heures (dont 1680 heures en entreprise)</t>
+          <t>Durée de 1267 heures (dont 637 heures en entreprise)</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
@@ -5505,17 +5509,17 @@
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=assistant%20de%20service%20social</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>ucpa-formation@ucpa.asso.fr</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>ucpa-formation@ucpa.asso.fr | fgehant@ucpa.asso.fr</t>
         </is>
       </c>
       <c r="K46" s="5" t="inlineStr">
@@ -5530,12 +5534,12 @@
       </c>
       <c r="M46" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0642833617</t>
         </is>
       </c>
       <c r="N46" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0642833617</t>
         </is>
       </c>
       <c r="O46" s="5" t="inlineStr">
@@ -5554,15 +5558,19 @@
         </is>
       </c>
       <c r="R46" s="5" t="inlineStr"/>
-      <c r="S46" s="5" t="inlineStr"/>
+      <c r="S46" s="5" t="inlineStr">
+        <is>
+          <t>Unité capitalisable (UC) - 1. Encadrer tout public dans tout lieu et toute structureUnité capitalisable (UC) - 2. Mettre en œuvre un projet d'animation s'inscrivant dans le projet de la structureUnité capitalisable (UC) - 3. Conduire une séance, un cycle d'animation ou d'apprentissage dans le champ des activités aquatiques et de la natationUnité capitalisable (UC) - 4. Mobiliser les techniques des activités aquatiques et de la natation pour mettre en œuvre une séance ou un cycle d'apprentissage | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T46" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
         </is>
       </c>
       <c r="U46" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11672249/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11447001/true/false/false/false</t>
         </is>
       </c>
       <c r="V46" s="5" t="inlineStr">
@@ -5584,27 +5592,27 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'éducateur spécialisé</t>
+          <t>Diplôme d'État d'aide-soignant - DEAS</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales (ARFRIPS - Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales)</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>69009 Lyon 9e</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>10 Impasse Pierre Baizet | 69009 Lyon 9e | France</t>
+          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>Durée de 3442 heures (dont 1925 heures en entreprise)</t>
+          <t>Durée de 1540 heures (dont 770 heures en entreprise)</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -5614,17 +5622,17 @@
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=aide-soignant</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
         <is>
-          <t>info@arfrips.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
-          <t>info@arfrips.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K47" s="7" t="inlineStr">
@@ -5639,12 +5647,12 @@
       </c>
       <c r="M47" s="7" t="inlineStr">
         <is>
-          <t>0478699090</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N47" s="7" t="inlineStr">
         <is>
-          <t>0478699090</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O47" s="7" t="inlineStr">
@@ -5663,20 +5671,24 @@
         </is>
       </c>
       <c r="R47" s="7" t="inlineStr"/>
-      <c r="S47" s="7" t="inlineStr"/>
+      <c r="S47" s="7" t="inlineStr">
+        <is>
+          <t>La formation conduisant au diplôme d'État d'aide-soignant, 17 semaines d'enseignement théoriques organisées autour de 8 modules : Accompagnement d'une personne dans les activités de la vie quotidienne L'état clinique d'une personne Les soins Ergonomie Relation Communication Hygiène des locaux hospitaliers Transmission des informations Organisation du travail Les titulaires du DE d'auxiliaire de puériculture, du DE d'aide médico-psychologique, du DE d'auxiliaire de vie sociale ou de la MC aide à domicile, sont dispensés de certaines unités de formation. La formation comprend également 6 stages d'une durée totale de 24 semaines en milieu hospitalier ou extra-hospitalier. Possibilité d'effectuer la formation en initial ou en apprentissage. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T47" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur spécialisé</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'aide-soignant</t>
         </is>
       </c>
       <c r="U47" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11737248/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11533549/true/false/false/true</t>
         </is>
       </c>
       <c r="V47" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
         </is>
       </c>
       <c r="W47" s="7" t="inlineStr">
@@ -5693,27 +5705,27 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet - RNCP 39931 - spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+          <t>Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
@@ -5723,17 +5735,17 @@
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>https://arfatsema.catalogueformpro.com/2/desjeps-17/2858060/desjeps-17-diplome-detat-superieur-de-la-jeunesse-de-leducation-populaire-et-du-sport-specialite-ani</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="K48" s="5" t="inlineStr">
@@ -5748,12 +5760,12 @@
       </c>
       <c r="M48" s="5" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0472117979</t>
         </is>
       </c>
       <c r="N48" s="5" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0472117979</t>
         </is>
       </c>
       <c r="O48" s="5" t="inlineStr">
@@ -5763,7 +5775,7 @@
       </c>
       <c r="P48" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q48" s="5" t="inlineStr">
@@ -5772,24 +5784,20 @@
         </is>
       </c>
       <c r="R48" s="5" t="inlineStr"/>
-      <c r="S48" s="5" t="inlineStr">
-        <is>
-          <t>BC1 : Construire, avec les instances de gouvernance, la stratégie de développement d'une structure dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Éducation Populaire Culture Politique Rapport de domination Pouvoir d'Agir et Vulnérabilité Esprit critique Transformation social/rapport sociaux Le numérique comme un fait social Nouvel esprit du capitalisme Laicité et valeurs de la République Violence sexiste violences sexuelles Ingénierie social en lien avec la structure Réaliser un diagnostic RH et financier Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Elaboration de la stratégie de développement en lien avec les instances de gouvernance Animer un processus démocratique Démocratie et contre pouvoir BC2 : Concevoir et diriger un projet de développement de la structure Cartographie des relations et l'environnement de son association Ingénierie du projet Processus d'évaluation dans une démarche partagée et participative Outils participatifs Outils de communication Utilité sociale BC3 : Manager l'équipe et gérer les ressources humaines ( et la démarche Qualité, Sécurité, Santé au Travail et Environnement d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Gestion des ressources humaines en structures d'éducation populaire : enjeux, éthique et complexités associative Articulation employeur bénévole - direction dans la gestion des ressources humaines : définition d'une politique RH et organisation des délégations de pouvoir Gérer l'équipe au quotidien : accompagnement, régulation et gestion conflits Analyse des pratiques en co-développement Développer le pouvoir d'agir des salariés Attractivité, recrutement, intégration et fidélisation des salariés Diversité, inclusion et égalité professionnelle au sein de son organisation Assurer la GPEC, la formation et la gestion des carrières dans un alignement éthique Le financement de la formation professionnelle Qualité de vie Santé sécurité au travail Droit du travail/Droit social Dialogue social/dialogue syndical Cadre général des RPS Démarche prévention et outils BC4 : Assurer la gestion financière, matérielle et administrative d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Comprendre les fondamentaux de la situation financière Initiation à l'analyse financière associative ou de structure d'intérêt général Identifier les leviers de financement Construire des scénarios budgétaires et faire des arbitrages Élaborer un plan d'action financier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
+      <c r="S48" s="5" t="inlineStr"/>
       <c r="T48" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U48" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880835/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11817055/true/false/false/false</t>
         </is>
       </c>
       <c r="V48" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
         </is>
       </c>
       <c r="W48" s="5" t="inlineStr">
@@ -5806,27 +5814,27 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Créer sa ferme en circuit court : transformation, commercialisation et communication</t>
+          <t>Diplôme d'État d'assistant de service social - DE ASS</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>SARL Agri-learn éditions</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>69001 Lyon</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 69001 Lyon | France</t>
+          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 avenue Lacassagne | Croix Rouge francaise | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Durée de 20 heures</t>
+          <t>Durée de 3420 heures (dont 1680 heures en entreprise)</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -5836,17 +5844,17 @@
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=assistant%20de%20service%20social</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K49" s="7" t="inlineStr">
@@ -5861,40 +5869,44 @@
       </c>
       <c r="M49" s="7" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N49" s="7" t="inlineStr">
         <is>
-          <t>0620021214</t>
-        </is>
-      </c>
-      <c r="O49" s="7" t="inlineStr"/>
+          <t>0472115560</t>
+        </is>
+      </c>
+      <c r="O49" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P49" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q49" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R49" s="7" t="inlineStr"/>
-      <c r="S49" s="7" t="inlineStr">
-        <is>
-          <t>Cette formation s'appuie sur plusieurs compétences essentielles : Stratégie commerciale et étude de marché : définir son offre, ses volumes, ses prix et ses circuits de vente Techniques de vente : maîtriser les étapes clés pour convaincre et fidéliser les clients Transformation des produits agricoles : valoriser ses matières premières pour créer de la valeur ajoutée Hygiène et réglementation : garantir la sécurité sanitaire dans les ateliers de transformation Communication et prospection : développer sa clientèle et promouvoir ses produits Valorisation des produits : savoir parler de ses produits et les mettre en avant (ex : dégustation) L'ensemble permet d'acquérir une vision globale du fonctionnement d'une ferme en circuit court, de la production jusqu'à la vente. 3 heures de visio avec les experts sont prévues dans le cursus. | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T49" s="7" t="inlineStr"/>
+      <c r="S49" s="7" t="inlineStr"/>
+      <c r="T49" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
+        </is>
+      </c>
       <c r="U49" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880868/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11672249/true/false/false/false</t>
         </is>
       </c>
       <c r="V49" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
         </is>
       </c>
       <c r="W49" s="7" t="inlineStr">
@@ -5911,106 +5923,433 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
+          <t>Diplôme d'État d'éducateur spécialisé</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales (ARFRIPS - Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales)</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>69009 Lyon 9e</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>10 Impasse Pierre Baizet | 69009 Lyon 9e | France</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 3442 heures (dont 1925 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>info@arfrips.fr</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>info@arfrips.fr</t>
+        </is>
+      </c>
+      <c r="K50" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M50" s="5" t="inlineStr">
+        <is>
+          <t>0478699090</t>
+        </is>
+      </c>
+      <c r="N50" s="5" t="inlineStr">
+        <is>
+          <t>0478699090</t>
+        </is>
+      </c>
+      <c r="O50" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P50" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q50" s="5" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R50" s="5" t="inlineStr"/>
+      <c r="S50" s="5" t="inlineStr"/>
+      <c r="T50" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur spécialisé</t>
+        </is>
+      </c>
+      <c r="U50" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11737248/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V50" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W50" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet - RNCP 39931 - spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>69100 Villeurbanne</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>https://arfatsema.catalogueformpro.com/2/desjeps-17/2858060/desjeps-17-diplome-detat-superieur-de-la-jeunesse-de-leducation-populaire-et-du-sport-specialite-ani</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>arfatsema.direction@orange.fr</t>
+        </is>
+      </c>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
+          <t>arfatsema.direction@orange.fr</t>
+        </is>
+      </c>
+      <c r="K51" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L51" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M51" s="7" t="inlineStr">
+        <is>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="N51" s="7" t="inlineStr">
+        <is>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="O51" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P51" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+        </is>
+      </c>
+      <c r="Q51" s="7" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R51" s="7" t="inlineStr"/>
+      <c r="S51" s="7" t="inlineStr">
+        <is>
+          <t>BC1 : Construire, avec les instances de gouvernance, la stratégie de développement d'une structure dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Éducation Populaire Culture Politique Rapport de domination Pouvoir d'Agir et Vulnérabilité Esprit critique Transformation social/rapport sociaux Le numérique comme un fait social Nouvel esprit du capitalisme Laicité et valeurs de la République Violence sexiste violences sexuelles Ingénierie social en lien avec la structure Réaliser un diagnostic RH et financier Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Elaboration de la stratégie de développement en lien avec les instances de gouvernance Animer un processus démocratique Démocratie et contre pouvoir BC2 : Concevoir et diriger un projet de développement de la structure Cartographie des relations et l'environnement de son association Ingénierie du projet Processus d'évaluation dans une démarche partagée et participative Outils participatifs Outils de communication Utilité sociale BC3 : Manager l'équipe et gérer les ressources humaines ( et la démarche Qualité, Sécurité, Santé au Travail et Environnement d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Gestion des ressources humaines en structures d'éducation populaire : enjeux, éthique et complexités associative Articulation employeur bénévole - direction dans la gestion des ressources humaines : définition d'une politique RH et organisation des délégations de pouvoir Gérer l'équipe au quotidien : accompagnement, régulation et gestion conflits Analyse des pratiques en co-développement Développer le pouvoir d'agir des salariés Attractivité, recrutement, intégration et fidélisation des salariés Diversité, inclusion et égalité professionnelle au sein de son organisation Assurer la GPEC, la formation et la gestion des carrières dans un alignement éthique Le financement de la formation professionnelle Qualité de vie Santé sécurité au travail Droit du travail/Droit social Dialogue social/dialogue syndical Cadre général des RPS Démarche prévention et outils BC4 : Assurer la gestion financière, matérielle et administrative d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Comprendre les fondamentaux de la situation financière Initiation à l'analyse financière associative ou de structure d'intérêt général Identifier les leviers de financement Construire des scénarios budgétaires et faire des arbitrages Élaborer un plan d'action financier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T51" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+        </is>
+      </c>
+      <c r="U51" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11880835/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V51" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W51" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>Créer sa ferme en circuit court : transformation, commercialisation et communication</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>SARL Agri-learn éditions</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>69001 Lyon</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Formation a distance | 69001 Lyon | France</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 20 heures</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I52" s="6" t="inlineStr">
+        <is>
+          <t>fanny@agrilearn.fr</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>fanny@agrilearn.fr</t>
+        </is>
+      </c>
+      <c r="K52" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L52" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M52" s="5" t="inlineStr">
+        <is>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="N52" s="5" t="inlineStr">
+        <is>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="O52" s="5" t="inlineStr"/>
+      <c r="P52" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+        </is>
+      </c>
+      <c r="Q52" s="5" t="inlineStr">
+        <is>
+          <t>À distance</t>
+        </is>
+      </c>
+      <c r="R52" s="5" t="inlineStr"/>
+      <c r="S52" s="5" t="inlineStr">
+        <is>
+          <t>Cette formation s'appuie sur plusieurs compétences essentielles : Stratégie commerciale et étude de marché : définir son offre, ses volumes, ses prix et ses circuits de vente Techniques de vente : maîtriser les étapes clés pour convaincre et fidéliser les clients Transformation des produits agricoles : valoriser ses matières premières pour créer de la valeur ajoutée Hygiène et réglementation : garantir la sécurité sanitaire dans les ateliers de transformation Communication et prospection : développer sa clientèle et promouvoir ses produits Valorisation des produits : savoir parler de ses produits et les mettre en avant (ex : dégustation) L'ensemble permet d'acquérir une vision globale du fonctionnement d'une ferme en circuit court, de la production jusqu'à la vente. 3 heures de visio avec les experts sont prévues dans le cursus. | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T52" s="5" t="inlineStr"/>
+      <c r="U52" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11880868/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V52" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W52" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
           <t>Titre professionnel administrateur d'infrastructures sécurisées (FOAD)</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
+      <c r="C53" s="7" t="inlineStr">
         <is>
           <t>STUDI</t>
         </is>
       </c>
-      <c r="D50" s="5" t="inlineStr">
+      <c r="D53" s="7" t="inlineStr">
         <is>
           <t>75004 Paris</t>
         </is>
       </c>
-      <c r="E50" s="5" t="inlineStr">
+      <c r="E53" s="7" t="inlineStr">
         <is>
           <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
-      <c r="F50" s="5" t="inlineStr">
+      <c r="F53" s="7" t="inlineStr">
         <is>
           <t>Durée de 947 heures (dont 350 heures en entreprise)</t>
         </is>
       </c>
-      <c r="G50" s="5" t="inlineStr">
+      <c r="G53" s="7" t="inlineStr">
         <is>
           <t>Prochaine session</t>
         </is>
       </c>
-      <c r="H50" s="5" t="inlineStr">
+      <c r="H53" s="7" t="inlineStr">
         <is>
           <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
-      <c r="I50" s="6" t="inlineStr">
+      <c r="I53" s="6" t="inlineStr">
         <is>
           <t>contact@studi.fr</t>
         </is>
       </c>
-      <c r="J50" s="5" t="inlineStr">
+      <c r="J53" s="7" t="inlineStr">
         <is>
           <t>contact@studi.fr | conseiller-formation.aoft@studi.fr</t>
         </is>
       </c>
-      <c r="K50" s="5" t="inlineStr">
+      <c r="K53" s="7" t="inlineStr">
         <is>
           <t>france_travail</t>
         </is>
       </c>
-      <c r="L50" s="5" t="inlineStr">
+      <c r="L53" s="7" t="inlineStr">
         <is>
           <t>100</t>
         </is>
       </c>
-      <c r="M50" s="5" t="inlineStr">
+      <c r="M53" s="7" t="inlineStr">
         <is>
           <t>0174888555</t>
         </is>
       </c>
-      <c r="N50" s="5" t="inlineStr">
+      <c r="N53" s="7" t="inlineStr">
         <is>
           <t>0174888555</t>
         </is>
       </c>
-      <c r="O50" s="5" t="inlineStr">
+      <c r="O53" s="7" t="inlineStr">
         <is>
           <t>Certifiante</t>
         </is>
       </c>
-      <c r="P50" s="5" t="inlineStr">
+      <c r="P53" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
         </is>
       </c>
-      <c r="Q50" s="5" t="inlineStr">
+      <c r="Q53" s="7" t="inlineStr">
         <is>
           <t>À distance</t>
         </is>
       </c>
-      <c r="R50" s="5" t="inlineStr"/>
-      <c r="S50" s="5" t="inlineStr">
+      <c r="R53" s="7" t="inlineStr"/>
+      <c r="S53" s="7" t="inlineStr">
         <is>
           <t>Administrer et sécuriser les infrastructures Les bonnes pratiques dans l'administration des infrastructures Utiliser un logiciel de gestion centralisé : GLPI Configurer le routage Administrer et sécuriser le réseau Automatiser les tâches d'administration Administrer et sécuriser les systèmes Les bases des serveurs virtualisés Administrer et sécuriser une infrastructure de serveurs virtualisée Gérer des containersConcevoir et mettre en œuvre une solution en réponse à un besoin d'évolution Les bases des solutions techniques Proposer une solution informatique répondant à des besoins nouveaux Mettre en production des évolutions de l'infrastructure Les bases de la supervision Superviser la disponibilité de l'infrastructure et en présenter les résultats Mesurer les performances et la disponibilité de l'infrastructureParticiper à la gestion de la cybersécurité Les bases de la cybersécurité Participer à la mesure et à l'analyse du niveau de sécurité de l'infrastructure Participer à l'élaboration et à la mise en œuvre de la politique de sécurité Participer à la détection et au traitement des incidents de sécurité | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
-      <c r="T50" s="5" t="inlineStr">
+      <c r="T53" s="7" t="inlineStr">
         <is>
           <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel administrateur d'infrastructures sécurisées</t>
         </is>
       </c>
-      <c r="U50" s="5" t="inlineStr">
+      <c r="U53" s="7" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/detail/11590088/true/false/true/false</t>
         </is>
       </c>
-      <c r="V50" s="5" t="inlineStr">
+      <c r="V53" s="7" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
-      <c r="W50" s="5" t="inlineStr">
+      <c r="W53" s="7" t="inlineStr">
         <is>
           <t>ok</t>
         </is>

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-07-25
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -187,8 +187,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseFranceTravail" displayName="BaseFranceTravail" ref="A1:W53" headerRowCount="1">
-  <autoFilter ref="A1:W53"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="BaseFranceTravail" displayName="BaseFranceTravail" ref="A1:W54" headerRowCount="1">
+  <autoFilter ref="A1:W54"/>
   <tableColumns count="23">
     <tableColumn id="1" name="zone"/>
     <tableColumn id="2" name="formation"/>
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5">
@@ -566,13 +566,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W53"/>
+  <dimension ref="A1:W54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1239,7 +1239,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1344,17 +1344,17 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 1350 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -1384,12 +1384,12 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1404,15 +1404,19 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="inlineStr"/>
+          <t>0180888030</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P8" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -1426,18 +1430,22 @@
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T8" s="5" t="inlineStr"/>
+          <t>11 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 : Démarrez votre formation d'Accompagnement Educatif Petite Enfance ; Projet 2 - Préparez un environnement sécurisé pour le jeune enfant ; Projet 3 - Développez des activités éducatives adaptées à la petite enfance ; Projet 4 - Appliquez les protocoles de santé dans le cadre de la petite enfance ; Projet 5 - Soutenez le personnel enseignant dans un contexte collectif ; Projet 6 - Améliorez les conditions d'accueil en école maternelle ; Projet 7 - Organisez l'accueil individuel au domicile ; Projet 8 - Gérez les tâches domestiques et la préparation des repas pour l'enfant ; Projet 9 : Proposer des solutions de prévention, santé et environnement ; Projet 10 : Remise à niveau scolaire ; Projet 11 : Préparez-vous pour l'examen final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+        </is>
+      </c>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120311/true/false/true/true</t>
         </is>
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1449,12 +1457,12 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Conseiller emploi et accompagnement professionnel</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -1474,7 +1482,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1350 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 1140 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1535,22 +1543,22 @@
       <c r="R9" s="7" t="inlineStr"/>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>11 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 : Démarrez votre formation d'Accompagnement Educatif Petite Enfance ; Projet 2 - Préparez un environnement sécurisé pour le jeune enfant ; Projet 3 - Développez des activités éducatives adaptées à la petite enfance ; Projet 4 - Appliquez les protocoles de santé dans le cadre de la petite enfance ; Projet 5 - Soutenez le personnel enseignant dans un contexte collectif ; Projet 6 - Améliorez les conditions d'accueil en école maternelle ; Projet 7 - Organisez l'accueil individuel au domicile ; Projet 8 - Gérez les tâches domestiques et la préparation des repas pour l'enfant ; Projet 9 : Proposer des solutions de prévention, santé et environnement ; Projet 10 : Remise à niveau scolaire ; Projet 11 : Préparez-vous pour l'examen final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>10 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de conseiller emploi et évolution professionnelle ; Projet 2 - Accompagnez en parallèle de nombreuses personnes avec des besoins différents ; Projet 3 - Élaborez une veille et analysez le marché de l'emploi ; Projet 4 - Réalisez un diagnostic et co-construisez un plan d'action avec vos bénéficiaires ; Projet 5 - Adaptez votre posture pour l'accompagnement des bénéficiaires ; Projet 6 - Établissez et validez un projet d'accompagnement professionnel ; Projet 7 - Établissez un plan d'action et un bilan professionnel ; Projet 8 - Concevez un atelier sur les métiers émergents avec l'IA ; Projet 9 - Développez votre projet territorial avec des partenaires ; Projet 10 - Élaborez votre boîte à outils pour accompagner vers l'emploi. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Conseiller emploi et accompagnement professionnel</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120311/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120363/true/false/true/true</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1562,17 +1570,17 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Conseiller emploi et accompagnement professionnel</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>AFEC (Siège)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1587,7 +1595,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1140 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1602,12 +1610,12 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1622,12 +1630,12 @@
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -1648,22 +1656,22 @@
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>10 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de conseiller emploi et évolution professionnelle ; Projet 2 - Accompagnez en parallèle de nombreuses personnes avec des besoins différents ; Projet 3 - Élaborez une veille et analysez le marché de l'emploi ; Projet 4 - Réalisez un diagnostic et co-construisez un plan d'action avec vos bénéficiaires ; Projet 5 - Adaptez votre posture pour l'accompagnement des bénéficiaires ; Projet 6 - Établissez et validez un projet d'accompagnement professionnel ; Projet 7 - Établissez un plan d'action et un bilan professionnel ; Projet 8 - Concevez un atelier sur les métiers émergents avec l'IA ; Projet 9 - Développez votre projet territorial avec des partenaires ; Projet 10 - Élaborez votre boîte à outils pour accompagner vers l'emploi. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant des modules d'enseignement et des prestations d'accompagnement. Modules d'enseignement professionnel : - EP1 Accompagnement du développement du jeune enfant (cadre d'intervention, accompagnement à l'autonomie l'enfant) - EP2 Exercer son activité en accueil collectif - EP3 Exercer son activité en accueil individuel Modules d'enseignements généraux : - Prévention santé environnement - Enseignements généraux (Mathématiques et sciences, Histoire-Géographie-Citoyenneté et français) En complément de la formation : - Remise à niveau numérique - Techniques de recherche d'emploi et de stage - Accompagnement au retour à l'emploi 3 Stages en entreprise 14 semaines | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Conseiller emploi et accompagnement professionnel</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120363/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124191/true/false/true/true</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1675,32 +1683,32 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Accompagnement vers emploi et vers la formation - Ecole de la 2ème chance</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>AFEC (Siège)</t>
+          <t>1ère Ecole de la Deuxième Chance de Normandie : E2C - Site Herouville-St-Clair (E2C NORMANDIE - Centre de formation d'insertion professionnelle)</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>14200 Hérouville-Saint-Clair</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>717 Boulevard de la Grande Delle | 14200 Hérouville-Saint-Clair | France</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 1210 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1710,17 +1718,17 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.e2cnormandie.fr/</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>contact@e2cnormandie.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>contact@e2cnormandie.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1735,48 +1743,40 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>0153368844</t>
+          <t>0261670985</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>0153368844</t>
-        </is>
-      </c>
-      <c r="O11" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0261670985</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="inlineStr"/>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant des modules d'enseignement et des prestations d'accompagnement. Modules d'enseignement professionnel : - EP1 Accompagnement du développement du jeune enfant (cadre d'intervention, accompagnement à l'autonomie l'enfant) - EP2 Exercer son activité en accueil collectif - EP3 Exercer son activité en accueil individuel Modules d'enseignements généraux : - Prévention santé environnement - Enseignements généraux (Mathématiques et sciences, Histoire-Géographie-Citoyenneté et français) En complément de la formation : - Remise à niveau numérique - Techniques de recherche d'emploi et de stage - Accompagnement au retour à l'emploi 3 Stages en entreprise 14 semaines | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T11" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
+          <t>Ateliers et actions de construction et réalisation du projet professionnel.orientation pro, techniques de recherche d'emploi, réseau, coaching, visite d'entreprise, journées métier, job-dating, forums, plateaux techniques...Ateliers, actions et projets de développement des compétences socioprofessionnelles | employabilité (ouverture social, culturelle et sportive, citoyenneté, communication professionnelle orale, écrite, numérique, raisonnement logique...Alternance : 6 stages de 2 à 4 semaines, toutes les 3 semaines (50% du temps de formation) | Organisme | 1ère Ecole de la Deuxième Chance de Normandie : E2C - Site Herouville-St-Clair (E2C NORMANDIE - Centre de formation d'insertion professionnelle) | Lieu de la formation | 717 Boulevard de la Grande Delle</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr"/>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124191/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10825210/true/false/false/false</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1788,12 +1788,12 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
+          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1813,7 +1813,7 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1870,18 +1870,18 @@
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T12" s="5" t="inlineStr"/>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -1898,12 +1898,12 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>BP option aménagements paysagers</t>
+          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1933,12 +1933,12 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
@@ -1953,19 +1953,15 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>0479254180</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>0479254180</t>
-        </is>
-      </c>
-      <c r="O13" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O13" s="7" t="inlineStr"/>
       <c r="P13" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -1979,17 +1975,13 @@
       <c r="R13" s="7" t="inlineStr"/>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T13" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
-        </is>
-      </c>
+          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T13" s="7" t="inlineStr"/>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/true</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
@@ -2011,12 +2003,12 @@
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>CAP Fleuriste</t>
+          <t>BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -2031,7 +2023,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -2046,12 +2038,12 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -2066,12 +2058,12 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0479254180</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0479254180</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -2092,17 +2084,17 @@
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/true</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
@@ -2119,32 +2111,32 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Titre professionnel de formateur professionnel d'adultes - Bloc 01 Concevoir et préparer la formation</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>CAMELEON (Caméléon Formation)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>11000 Carcassonne</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>8 bd marcou | 11000 Carcassonne | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Durée de 189 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2159,12 +2151,12 @@
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>cameleonformation@gmail.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>cameleonformation@gmail.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -2179,12 +2171,12 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>0554543023</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>0554543023</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="O15" s="7" t="inlineStr">
@@ -2194,33 +2186,33 @@
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr"/>
       <c r="S15" s="7" t="inlineStr">
         <is>
-          <t>Concevoir et préparer la formation : réalisation d'un cahier des charges- rédactiond'un scénario pédagogique et d'un plan d'accompagnement- conception d'un scénario pédagogique etd'accompagnement en présentiel et multimodal - conception d'activités pédagogiques et d'évaluationutilisant les neurosciences- les apports des neurosciences pour une pédagogie différenciée innovante- lesdifférentes modalités pédagogiques actives selon les objectifs - conception des outils del'individualisation -construire un storyboard, notion de storytelling et de synopsis - les différents LMS etlogiciels pour du e-learning- les IA génératives au service de la formation- intégration des cadresréglementaires à la pratique - la démarche de formateur responsable : réglementation et RSE . | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel formateur professionnel d'adultes</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10969948/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/true</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-12&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W15" s="7" t="inlineStr">
@@ -2237,7 +2229,7 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Titre professionnel formateur professionnel d'adultes - Bloc 03 Accomapgner les apprenants en formation</t>
+          <t>Titre professionnel de formateur professionnel d'adultes - Bloc 01 Concevoir et préparer la formation</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -2252,12 +2244,12 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>8 rue Marcou | 11000 Carcassonne | France</t>
+          <t>8 bd marcou | 11000 Carcassonne | France</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Durée de 35 heures</t>
+          <t>Durée de 189 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2318,7 +2310,7 @@
       <c r="R16" s="5" t="inlineStr"/>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>Accompagner les apprenants enformation : adaptation duparcours et accompagnementdes apprenants - tutorat desapprenants à distance -coacherun apprenant selon les modalités- développer la réflexivité chez les apprenants- la métacognitioninclusivité-accompagnement des apprentissages en entreprise - accompagnement des apprenants à laréussite professionnelle - accompagnement d'un apprenant dans son parcours individuel - création d'undispositif de veille pour la démarche de formateur responsable - l'analyse de ses pratiquesprofessionnelles d'accompagnement | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Concevoir et préparer la formation : réalisation d'un cahier des charges- rédactiond'un scénario pédagogique et d'un plan d'accompagnement- conception d'un scénario pédagogique etd'accompagnement en présentiel et multimodal - conception d'activités pédagogiques et d'évaluationutilisant les neurosciences- les apports des neurosciences pour une pédagogie différenciée innovante- lesdifférentes modalités pédagogiques actives selon les objectifs - conception des outils del'individualisation -construire un storyboard, notion de storytelling et de synopsis - les différents LMS etlogiciels pour du e-learning- les IA génératives au service de la formation- intégration des cadresréglementaires à la pratique - la démarche de formateur responsable : réglementation et RSE . | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T16" s="5" t="inlineStr">
@@ -2328,7 +2320,7 @@
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10969957/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10969948/true/false/false/false</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
@@ -2350,7 +2342,7 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Titre professionnel de formateur professionnel d'adultes - Bloc 02 Animer une formation et évaluer les acquis des apprenants</t>
+          <t>Titre professionnel formateur professionnel d'adultes - Bloc 03 Accomapgner les apprenants en formation</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -2370,7 +2362,7 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Durée de 161 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 35 heures</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2431,7 +2423,7 @@
       <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="7" t="inlineStr">
         <is>
-          <t>Animer une formation et évaluer les acquis des apprenants : animation d'uneformation - évaluation en présentiel - évaluation en multimodalité - repérage des difficultés liées auxapprentissages - animation de situations d'apprentissage en présentiel et à distance - analyse de sespratiques professionnelles d'animation et d'évaluation des acquis - apprendre autrement : des outilspour toutes les typologies d'apprentissage- intelligences multiples- psychologie clinique desapprentissages- la démarche de formateur responsable - les profils neuroatypiques : EHP, DYS, TDAH,TSA, la démarche qualité etresponsabilité sociale del'entreprise . | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Accompagner les apprenants enformation : adaptation duparcours et accompagnementdes apprenants - tutorat desapprenants à distance -coacherun apprenant selon les modalités- développer la réflexivité chez les apprenants- la métacognitioninclusivité-accompagnement des apprentissages en entreprise - accompagnement des apprenants à laréussite professionnelle - accompagnement d'un apprenant dans son parcours individuel - création d'undispositif de veille pour la démarche de formateur responsable - l'analyse de ses pratiquesprofessionnelles d'accompagnement | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T17" s="7" t="inlineStr">
@@ -2441,7 +2433,7 @@
       </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10969959/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10969957/true/false/false/false</t>
         </is>
       </c>
       <c r="V17" s="7" t="inlineStr">
@@ -2463,27 +2455,27 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Hygiène en nologie</t>
+          <t>Titre professionnel de formateur professionnel d'adultes - Bloc 02 Animer une formation et évaluer les acquis des apprenants</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
+          <t>CAMELEON (Caméléon Formation)</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>11100 Narbonne</t>
+          <t>11000 Carcassonne</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
+          <t>8 rue Marcou | 11000 Carcassonne | France</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4 heures</t>
+          <t>Durée de 161 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -2498,12 +2490,12 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>cameleonformation@gmail.com</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>thierry.cassagne@labdejean.fr</t>
+          <t>cameleonformation@gmail.com</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -2518,15 +2510,19 @@
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0554543023</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>0468410152</t>
-        </is>
-      </c>
-      <c r="O18" s="5" t="inlineStr"/>
+          <t>0554543023</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P18" s="5" t="inlineStr">
         <is>
           <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
@@ -2540,13 +2536,17 @@
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>Définition des étapes de l'hygiène agro-alimentaire: détergence, désinfection, rinçageChoix du produit d'hygiène selon le bon "S.E.N.S.Le "T.A.C.T. pour nettoyer et désinfecterElaboration d'un plan d'hygiène | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
-        </is>
-      </c>
-      <c r="T18" s="5" t="inlineStr"/>
+          <t>Animer une formation et évaluer les acquis des apprenants : animation d'uneformation - évaluation en présentiel - évaluation en multimodalité - repérage des difficultés liées auxapprentissages - animation de situations d'apprentissage en présentiel et à distance - analyse de sespratiques professionnelles d'animation et d'évaluation des acquis - apprendre autrement : des outilspour toutes les typologies d'apprentissage- intelligences multiples- psychologie clinique desapprentissages- la démarche de formateur responsable - les profils neuroatypiques : EHP, DYS, TDAH,TSA, la démarche qualité etresponsabilité sociale del'entreprise . | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T18" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel formateur professionnel d'adultes</t>
+        </is>
+      </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080125/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10969959/true/false/false/false</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
@@ -2568,7 +2568,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Elevage des vins : choix, durée, contrôle</t>
+          <t>Hygiène en nologie</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -2623,12 +2623,12 @@
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>0676219742</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>0676219742</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="O19" s="7" t="inlineStr"/>
@@ -2645,13 +2645,13 @@
       <c r="R19" s="7" t="inlineStr"/>
       <c r="S19" s="7" t="inlineStr">
         <is>
-          <t>Définition de l'élevageRôle des gaz (CO2 et O2)Les différents modes d'élevageLe suivi analytique et microbiologique | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+          <t>Définition des étapes de l'hygiène agro-alimentaire: détergence, désinfection, rinçageChoix du produit d'hygiène selon le bon "S.E.N.S.Le "T.A.C.T. pour nettoyer et désinfecterElaboration d'un plan d'hygiène | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T19" s="7" t="inlineStr"/>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080181/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080125/true/false/false/false</t>
         </is>
       </c>
       <c r="V19" s="7" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Vinification en rose : les fondamentaux</t>
+          <t>Elevage des vins : choix, durée, contrôle</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -2728,12 +2728,12 @@
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0676219742</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>0468410152</t>
+          <t>0676219742</t>
         </is>
       </c>
       <c r="O20" s="5" t="inlineStr"/>
@@ -2750,13 +2750,13 @@
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>Définition du profil de vin souhaitéMaturation des raisins: détermination de la date optimale des vendangesItinéraires techniques généraux (pressurage direct, saignée)Opérations préfermentaires: transport, bioprotection, égrappage, foulage, pressurage,gestion de la couleur, débourbagePilotage de la fermentation alcoolique: SO2, levures, nutrition azotée, gestion O2, gestion profil T°Conservation du vin | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+          <t>Définition de l'élevageRôle des gaz (CO2 et O2)Les différents modes d'élevageLe suivi analytique et microbiologique | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080222/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080181/true/false/false/false</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Vinification en rouge : les fondamentaux</t>
+          <t>Vinification en rose : les fondamentaux</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -2855,13 +2855,13 @@
       <c r="R21" s="7" t="inlineStr"/>
       <c r="S21" s="7" t="inlineStr">
         <is>
-          <t>Définition du profil de vin souhaitéMaturation des raisin: détermination de la date optimale des vendangesItinéraire technique général de la vinification en rougeCuvaison/macérationOpérations préfermentaires: transport, bioprorection, égrappage, foulage, MPFPilotage de la fermentation alcoolique: SO2, levures, nutriments, gestion profil thermique, gestion O2, techniques d'extractionOpérations Post macération:Ecoulage, décuvage, pressurage du marc,FMLElevage | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+          <t>Définition du profil de vin souhaitéMaturation des raisins: détermination de la date optimale des vendangesItinéraires techniques généraux (pressurage direct, saignée)Opérations préfermentaires: transport, bioprotection, égrappage, foulage, pressurage,gestion de la couleur, débourbagePilotage de la fermentation alcoolique: SO2, levures, nutrition azotée, gestion O2, gestion profil T°Conservation du vin | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T21" s="7" t="inlineStr"/>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080224/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080222/true/false/false/false</t>
         </is>
       </c>
       <c r="V21" s="7" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Repérer et identifier les principaux défauts du vin</t>
+          <t>Vinification en rouge : les fondamentaux</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -2960,13 +2960,13 @@
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>Altérations d'origine microbienne:Contamination bactérienne: acescence, piqûre acétique, piqûre lactique, maladie de la tourne, maladie de l'amer, piqure mannitique, odeur de géranium, diacétyleContamination levurienne: brettanomyces, maladie de la fleur, goût de sourisOxydationRéductionMaladies dues à la qualité des raisins: les GMT, le goût herbacé-véétalAutres origines: goût de bouchon, pinking, goût d'huître, goût de lumière | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+          <t>Définition du profil de vin souhaitéMaturation des raisin: détermination de la date optimale des vendangesItinéraire technique général de la vinification en rougeCuvaison/macérationOpérations préfermentaires: transport, bioprorection, égrappage, foulage, MPFPilotage de la fermentation alcoolique: SO2, levures, nutriments, gestion profil thermique, gestion O2, techniques d'extractionOpérations Post macération:Ecoulage, décuvage, pressurage du marc,FMLElevage | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T22" s="5" t="inlineStr"/>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080227/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080224/true/false/false/false</t>
         </is>
       </c>
       <c r="V22" s="5" t="inlineStr">
@@ -2988,7 +2988,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Vinification sans sulfites ajoutes ou à teneur réduite en sulfites</t>
+          <t>Repérer et identifier les principaux défauts du vin</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -3065,13 +3065,13 @@
       <c r="R23" s="7" t="inlineStr"/>
       <c r="S23" s="7" t="inlineStr">
         <is>
-          <t>Chimie du SO2Produits de substitution au SO2Gestion O2Itinéraires techniques de vinification alternatifsStabilisation et élevage des vins | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+          <t>Altérations d'origine microbienne:Contamination bactérienne: acescence, piqûre acétique, piqûre lactique, maladie de la tourne, maladie de l'amer, piqure mannitique, odeur de géranium, diacétyleContamination levurienne: brettanomyces, maladie de la fleur, goût de sourisOxydationRéductionMaladies dues à la qualité des raisins: les GMT, le goût herbacé-véétalAutres origines: goût de bouchon, pinking, goût d'huître, goût de lumière | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T23" s="7" t="inlineStr"/>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080266/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080227/true/false/false/false</t>
         </is>
       </c>
       <c r="V23" s="7" t="inlineStr">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Vinification en blanc: les fondamentaux</t>
+          <t>Vinification sans sulfites ajoutes ou à teneur réduite en sulfites</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -3170,13 +3170,13 @@
       <c r="R24" s="5" t="inlineStr"/>
       <c r="S24" s="5" t="inlineStr">
         <is>
-          <t>Détermination du type de vin souhaitéMaturation du raisin: détermination de la date des vendangesItinéraire technique généralOpérations préfermentaires: transport, bioprotection, tri, éraflage, macération préfermentaire à froid, pressurage, débourbagePilotage de la fermentation alcoolique: SO2, levurage, nutrition azotée, gestion O2, maîtrise T°Elevage: en cuve, en barrique, sur lies fines | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
+          <t>Chimie du SO2Produits de substitution au SO2Gestion O2Itinéraires techniques de vinification alternatifsStabilisation et élevage des vins | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T24" s="5" t="inlineStr"/>
       <c r="U24" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11080272/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080266/true/false/false/false</t>
         </is>
       </c>
       <c r="V24" s="5" t="inlineStr">
@@ -3193,32 +3193,32 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Ecole de la 2ème Chance (E2C)</t>
+          <t>Vinification en blanc: les fondamentaux</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Objectif 2ème chance - métropôle nice côte d'azur - ecole de la deuxième chance des alpes maritimes - odc nca - e2c</t>
+          <t>SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN)</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>06200 Nice</t>
+          <t>11100 Narbonne</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>455 Promenade des Anglais | Porte Arenas | 06200 Nice | France</t>
+          <t>Impasse Edouard Branly | 11100 Narbonne | France</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1100 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 4 heures</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>contact@e2cnicecotedazur.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>contact@e2cnicecotedazur.fr</t>
+          <t>thierry.cassagne@labdejean.fr</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
@@ -3253,18 +3253,18 @@
       </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>04 12 05 20 05</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>04 12 05 20 05</t>
+          <t>0468410152</t>
         </is>
       </c>
       <c r="O25" s="7" t="inlineStr"/>
       <c r="P25" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q25" s="7" t="inlineStr">
@@ -3275,18 +3275,18 @@
       <c r="R25" s="7" t="inlineStr"/>
       <c r="S25" s="7" t="inlineStr">
         <is>
-          <t>Programme non communiqué | Organisme | Objectif 2ème chance - métropôle nice côte d'azur - ecole de la deuxième chance des alpes maritimes - odc nca - e2c | Lieu de la formation | 455 Promenade des Anglais</t>
+          <t>Détermination du type de vin souhaitéMaturation du raisin: détermination de la date des vendangesItinéraire technique généralOpérations préfermentaires: transport, bioprotection, tri, éraflage, macération préfermentaire à froid, pressurage, débourbagePilotage de la fermentation alcoolique: SO2, levurage, nutrition azotée, gestion O2, maîtrise T°Elevage: en cuve, en barrique, sur lies fines | Organisme | SOCIETE D'EXPLOITATION DES ETABLISSEMENTS DEJEAN (SEE DEJEAN) | Lieu de la formation | Impasse Edouard Branly</t>
         </is>
       </c>
       <c r="T25" s="7" t="inlineStr"/>
       <c r="U25" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10681643/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11080272/true/false/false/false</t>
         </is>
       </c>
       <c r="V25" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-11&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W25" s="7" t="inlineStr">
@@ -3298,7 +3298,7 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>04</t>
+          <t>06</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
@@ -3308,17 +3308,17 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04</t>
+          <t>Objectif 2ème chance - métropôle nice côte d'azur - ecole de la deuxième chance des alpes maritimes - odc nca - e2c</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>04000 Digne-les-Bains</t>
+          <t>06200 Nice</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>4 avenue de Verdun | https://www.iap.asso.fr/ | 04000 Digne-les-Bains | France</t>
+          <t>455 Promenade des Anglais | Porte Arenas | 06200 Nice | France</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -3333,17 +3333,17 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>https://www.iap.asso.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>contact@iap.asso.fr</t>
+          <t>contact@e2cnicecotedazur.fr</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>contact@iap.asso.fr</t>
+          <t>contact@e2cnicecotedazur.fr</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
@@ -3358,12 +3358,12 @@
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>04 92 87 46 10</t>
+          <t>04 12 05 20 05</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
-          <t>04 92 87 46 10</t>
+          <t>04 12 05 20 05</t>
         </is>
       </c>
       <c r="O26" s="5" t="inlineStr"/>
@@ -3380,18 +3380,18 @@
       <c r="R26" s="5" t="inlineStr"/>
       <c r="S26" s="5" t="inlineStr">
         <is>
-          <t>Programme non communiqué | Organisme | Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04 | https://www.iap.asso.fr/ | Lieu de la formation</t>
+          <t>Programme non communiqué | Organisme | Objectif 2ème chance - métropôle nice côte d'azur - ecole de la deuxième chance des alpes maritimes - odc nca - e2c | Lieu de la formation | 455 Promenade des Anglais</t>
         </is>
       </c>
       <c r="T26" s="5" t="inlineStr"/>
       <c r="U26" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10685143/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10681643/true/false/false/false</t>
         </is>
       </c>
       <c r="V26" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-06&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W26" s="5" t="inlineStr">
@@ -3403,32 +3403,32 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>04</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Titre professionnel secrétaire assistant médico-administratif (FOAD)</t>
+          <t>Ecole de la 2ème Chance (E2C)</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>04000 Digne-les-Bains</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>4 avenue de Verdun | https://www.iap.asso.fr/ | 04000 Digne-les-Bains | France</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1084 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 1100 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -3438,17 +3438,17 @@
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.iap.asso.fr/</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>contact@iap.asso.fr</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>contact@iap.asso.fr</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
@@ -3463,48 +3463,40 @@
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>04 92 87 46 10</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="O27" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>04 92 87 46 10</t>
+        </is>
+      </c>
+      <c r="O27" s="7" t="inlineStr"/>
       <c r="P27" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q27" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R27" s="7" t="inlineStr"/>
       <c r="S27" s="7" t="inlineStr">
         <is>
-          <t>7 projets professionnalisants vous permettront d'acquérir les compétences citées au dessus par la pratique.Vous réaliserez les projets suivants :P1 - Démarrez votre formation de secrétaire assistant médico-administratifP2 - Niveau 1 : Maîtrisez l'accueil et la gestion administrative en milieu médicalP3 - Niveau 2 : Développez vos compétences en rédaction, communication et outils numériques en milieuP4 - Réalisez votre mission en entrepriseP5 - Niveau 3 : Optimisez l'organisation, la sécuritéet la gestion des données sensibles en milieu médicalP6 - Niveau 4 : Améliorez la gestion des communications, données et environnements sanitairesP7 - Préparez votre fin de formation de secrétaire assistant médico-administratif | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T27" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel secrétaire assistant médico-administratif</t>
-        </is>
-      </c>
+          <t>Programme non communiqué | Organisme | Institut avenir provence - ecole de la deuxième chance des alpes de haute provence - iap - e2c 04 | https://www.iap.asso.fr/ | Lieu de la formation</t>
+        </is>
+      </c>
+      <c r="T27" s="7" t="inlineStr"/>
       <c r="U27" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10685143/true/false/false/false</t>
         </is>
       </c>
       <c r="V27" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-04&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W27" s="7" t="inlineStr">
@@ -3521,7 +3513,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Formation au concours d'ATSEM</t>
+          <t>Titre professionnel secrétaire assistant médico-administratif (FOAD)</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -3541,7 +3533,7 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Durée de 346 heures</t>
+          <t>Durée de 1084 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -3584,7 +3576,11 @@
           <t>0180888030</t>
         </is>
       </c>
-      <c r="O28" s="5" t="inlineStr"/>
+      <c r="O28" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P28" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -3598,13 +3594,17 @@
       <c r="R28" s="5" t="inlineStr"/>
       <c r="S28" s="5" t="inlineStr">
         <is>
-          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T28" s="5" t="inlineStr"/>
+          <t>7 projets professionnalisants vous permettront d'acquérir les compétences citées au dessus par la pratique.Vous réaliserez les projets suivants :P1 - Démarrez votre formation de secrétaire assistant médico-administratifP2 - Niveau 1 : Maîtrisez l'accueil et la gestion administrative en milieu médicalP3 - Niveau 2 : Développez vos compétences en rédaction, communication et outils numériques en milieuP4 - Réalisez votre mission en entrepriseP5 - Niveau 3 : Optimisez l'organisation, la sécuritéet la gestion des données sensibles en milieu médicalP6 - Niveau 4 : Améliorez la gestion des communications, données et environnements sanitairesP7 - Préparez votre fin de formation de secrétaire assistant médico-administratif | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T28" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel secrétaire assistant médico-administratif</t>
+        </is>
+      </c>
       <c r="U28" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/false</t>
         </is>
       </c>
       <c r="V28" s="5" t="inlineStr">
@@ -3626,12 +3626,12 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Concours d'atsem (FOAD)</t>
+          <t>Formation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
+          <t>Durée de 346 heures</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -3661,12 +3661,12 @@
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
@@ -3681,12 +3681,12 @@
       </c>
       <c r="M29" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O29" s="7" t="inlineStr"/>
@@ -3703,13 +3703,13 @@
       <c r="R29" s="7" t="inlineStr"/>
       <c r="S29" s="7" t="inlineStr">
         <is>
-          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
+          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T29" s="7" t="inlineStr"/>
       <c r="U29" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/false</t>
         </is>
       </c>
       <c r="V29" s="7" t="inlineStr">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Concours d'atsem (FOAD)</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
@@ -3751,7 +3751,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -3771,7 +3771,7 @@
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -3794,11 +3794,7 @@
           <t>0366060201</t>
         </is>
       </c>
-      <c r="O30" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+      <c r="O30" s="5" t="inlineStr"/>
       <c r="P30" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -3812,17 +3808,13 @@
       <c r="R30" s="5" t="inlineStr"/>
       <c r="S30" s="5" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T30" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
+          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T30" s="5" t="inlineStr"/>
       <c r="U30" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/false</t>
         </is>
       </c>
       <c r="V30" s="5" t="inlineStr">
@@ -3844,12 +3836,12 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Préparation au concours d'ATSEM</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>AFEC (Siège)</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -3864,7 +3856,7 @@
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -3879,12 +3871,12 @@
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
@@ -3899,15 +3891,19 @@
       </c>
       <c r="M31" s="7" t="inlineStr">
         <is>
-          <t>0153368844</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N31" s="7" t="inlineStr">
         <is>
-          <t>0153368844</t>
-        </is>
-      </c>
-      <c r="O31" s="7" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O31" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P31" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -3921,13 +3917,17 @@
       <c r="R31" s="7" t="inlineStr"/>
       <c r="S31" s="7" t="inlineStr">
         <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC (Siège) | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T31" s="7" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T31" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+        </is>
+      </c>
       <c r="U31" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/false</t>
         </is>
       </c>
       <c r="V31" s="7" t="inlineStr">
@@ -3949,12 +3949,12 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
+          <t>Préparation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>AFEC (Siège)</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -3969,7 +3969,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
@@ -3984,12 +3984,12 @@
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
@@ -4004,12 +4004,12 @@
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="O32" s="5" t="inlineStr"/>
@@ -4026,13 +4026,13 @@
       <c r="R32" s="5" t="inlineStr"/>
       <c r="S32" s="5" t="inlineStr">
         <is>
-          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC (Siège) | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T32" s="5" t="inlineStr"/>
       <c r="U32" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/false</t>
         </is>
       </c>
       <c r="V32" s="5" t="inlineStr">
@@ -4054,7 +4054,7 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
+          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
@@ -4074,7 +4074,7 @@
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -4131,13 +4131,13 @@
       <c r="R33" s="7" t="inlineStr"/>
       <c r="S33" s="7" t="inlineStr">
         <is>
-          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T33" s="7" t="inlineStr"/>
       <c r="U33" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/false</t>
         </is>
       </c>
       <c r="V33" s="7" t="inlineStr">
@@ -4159,7 +4159,7 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
+          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -4179,7 +4179,7 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
@@ -4236,13 +4236,13 @@
       <c r="R34" s="5" t="inlineStr"/>
       <c r="S34" s="5" t="inlineStr">
         <is>
-          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
         </is>
       </c>
       <c r="T34" s="5" t="inlineStr"/>
       <c r="U34" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/false</t>
         </is>
       </c>
       <c r="V34" s="5" t="inlineStr">
@@ -4264,12 +4264,12 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>BP option aménagements paysagers</t>
+          <t>Préparation à l'entrée en institut de formation d'auxiliaire de puériculture</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
@@ -4284,7 +4284,7 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -4299,12 +4299,12 @@
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>epl.la-motte-servolex@educagri.fr | cecile.iribarne@educagri.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
@@ -4319,19 +4319,15 @@
       </c>
       <c r="M35" s="7" t="inlineStr">
         <is>
-          <t>0479264427</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N35" s="7" t="inlineStr">
         <is>
-          <t>0479264427</t>
-        </is>
-      </c>
-      <c r="O35" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O35" s="7" t="inlineStr"/>
       <c r="P35" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -4345,17 +4341,13 @@
       <c r="R35" s="7" t="inlineStr"/>
       <c r="S35" s="7" t="inlineStr">
         <is>
-          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T35" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
-        </is>
-      </c>
+          <t>MODULE 1 - Remise à niveau numérique préparatoire Objectifs : -Se connecter à une plateforme?de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra MODULE 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter MODULE 3 - Remise à niveau - Mathématiques Objectif : Utiliser les bases des mathématiques dans sa pratique professionnelle MODULE 4 - Remise à niveau - Biologie Objectif : Maîtriser les bases de la biologie nécessaires à l'entrée en école d'auxiliaire de puériculture MODULE 5 - Compétences numériques Objectifs: Être autonome sur l'outil numérique MODULE 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectifs: -Connaître son environnement professionnel -Connaître son futur métier MODULE 7 - La relation d'aide Objectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les enfants et leur famille MODULE 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi MODULE 9 - Aide à l'admission Objectifs : -Anticiper son entrée en école d'auxiliaire de puériculture -Savoir se présenter et présenter son projet professionnel MODULE 10 - Accompagnement à la recherche de stage Objectifs :Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact MODULE 11 - Accompagnement au retour à l'emploi Objectifs : -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entreprise Objectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T35" s="7" t="inlineStr"/>
       <c r="U35" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128426/true/false/true/false</t>
         </is>
       </c>
       <c r="V35" s="7" t="inlineStr">
@@ -4377,12 +4369,12 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>CAP Fleuriste</t>
+          <t>BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>EPLEFPA Chambéry La Motte-Servolex (Savoie) (EPLEFPA - Lycée agricole Reinach)</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -4397,7 +4389,7 @@
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 991 heures (dont 420 heures en entreprise)</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
@@ -4412,12 +4404,12 @@
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
+          <t>epl.la-motte-servolex@educagri.fr | cecile.iribarne@educagri.fr</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
@@ -4432,12 +4424,12 @@
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0479264427</t>
         </is>
       </c>
       <c r="N36" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0479264427</t>
         </is>
       </c>
       <c r="O36" s="5" t="inlineStr">
@@ -4458,17 +4450,17 @@
       <c r="R36" s="5" t="inlineStr"/>
       <c r="S36" s="5" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Référentiel RNCP - Code RNCP 38314 - est organisé autour de 6 blocs de compétences : - C1 - Se situer en tant que professionnel - C2 - Organiser le travail d'un chantier d'aménagement paysager - C3 - Réaliser les interventions de mise en place des végétaux - C4 - Réaliser les interventions d'entretien des végétaux - C5 - Mettre en place les infrastructures - UCARE - Mettre en place un jardin vivrier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T36" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BP option aménagements paysagers</t>
         </is>
       </c>
       <c r="U36" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200732/true/false/true/false</t>
         </is>
       </c>
       <c r="V36" s="5" t="inlineStr">
@@ -4485,32 +4477,32 @@
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>E2C - Ecole de la Deuxième Chance</t>
+          <t>CAP Fleuriste</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Ecole de la Deuxième Chance Grand Hainaut</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>02140 Vervins</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Ecole de la deuxième chance - site de VERVINS | 3 Place des Anciens Combattants | 02140 Vervins | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1400 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 1296 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -4525,12 +4517,12 @@
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>c.renaud@e2cgrandhainaut.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>c.renaud@e2cgrandhainaut.fr</t>
+          <t>info@cenef.fr | service-prise-en-charge@cenef.fr</t>
         </is>
       </c>
       <c r="K37" s="7" t="inlineStr">
@@ -4545,40 +4537,48 @@
       </c>
       <c r="M37" s="7" t="inlineStr">
         <is>
-          <t>0375310010</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N37" s="7" t="inlineStr">
         <is>
-          <t>0375310010</t>
-        </is>
-      </c>
-      <c r="O37" s="7" t="inlineStr"/>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O37" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P37" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q37" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R37" s="7" t="inlineStr"/>
       <c r="S37" s="7" t="inlineStr">
         <is>
-          <t>Savoir fondamentauxOrientation et démarches professionnelsSocialisation et développement personnelAlternance en entreprise (près de 30% du temps)Des outils pédagogiques de liaison, d'évaluation et de suivi9 mois maximum + 12 mois de suivi post-parcours | Organisme | Ecole de la Deuxième Chance Grand Hainaut | Lieu de la formation | Ecole de la deuxième chance - site de VERVINS</t>
-        </is>
-      </c>
-      <c r="T37" s="7" t="inlineStr"/>
+          <t>Le programme obligatoire de la formation est le suivant :BC01 - PREPARER LES PRODUITS, LES VEGETAUX ET REALISER UNE COMPOSITION FLORALEReconnaître les végétauxRéceptionner et conditionner les marchandisesRespecter les règles de sécuritéConnaître les techniques fondamentalesRéaliser des arrangements florauxAppliquer les règles de compositionSavoir harmoniserBC02 - VENDRE, CONSEILLER LE CLIENT ET METTRE EN VALEUR L'OFFREVendre des produits et conseiller le clientProposer des services et fidéliserMaintenir l'attractivité du point de venteCommuniquerConnaitre l'environnement éco juridique et social des activités professionnellesBC03 - PREVENTION SANTE ENVIRONNEMENTPrévention, santé, environnement, tome 1Prévention, santé, environnement, tome 2ANGLAIS (pour les élèves non dispensés)AnglaisMATIERES GENERALES (pour les élèves non dispensés)FrançaisMathématiquesSciencesHistoire - Géographie - Enseignement moral et civiquesDes cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus :Epreuves blanches EP1 , EP2 , PSE , Matières généralesFiches des végétaux | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T37" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP fleuriste</t>
+        </is>
+      </c>
       <c r="U37" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11072382/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11200737/true/false/true/false</t>
         </is>
       </c>
       <c r="V37" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-03&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W37" s="7" t="inlineStr">
@@ -4590,32 +4590,32 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>02</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Préparation au concours d'adjoint administratif d'État principal de 2ème classe</t>
+          <t>E2C - Ecole de la Deuxième Chance</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school)</t>
+          <t>Ecole de la Deuxième Chance Grand Hainaut</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>02140 Vervins</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Ecole de la deuxième chance - site de VERVINS | 3 Place des Anciens Combattants | 02140 Vervins | France</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Durée de 335 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 1400 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
@@ -4630,12 +4630,12 @@
       </c>
       <c r="I38" s="6" t="inlineStr">
         <is>
-          <t>foad@skillandyou.com</t>
+          <t>c.renaud@e2cgrandhainaut.fr</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>foad@skillandyou.com</t>
+          <t>c.renaud@e2cgrandhainaut.fr</t>
         </is>
       </c>
       <c r="K38" s="5" t="inlineStr">
@@ -4650,40 +4650,40 @@
       </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
-          <t>0146006878</t>
+          <t>0375310010</t>
         </is>
       </c>
       <c r="N38" s="5" t="inlineStr">
         <is>
-          <t>0146006878</t>
+          <t>0375310010</t>
         </is>
       </c>
       <c r="O38" s="5" t="inlineStr"/>
       <c r="P38" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q38" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R38" s="5" t="inlineStr"/>
       <c r="S38" s="5" t="inlineStr">
         <is>
-          <t>Votre intégration - Guide d'intégration - Bienvenue dans votre formation - Guide Métier Adjoint administratif d'État principal de 2ème classe - Guide de la formation - Guide des épreuves - Le concours d'adjoint administratif d'État principal de 2ème classe Aide à la réalisation de vos documents professionnels Compléter votre livret de suivi des compétences professionnelles Retranscrire et ordonner les idées principales d'un texte Annales corrigées Épreuves blanches Solliciter les connaissances fondamentales pour le concours Comprendre l'administration française Comprendre le fonctionnement des institutions françaises Acquérir des connaissances en français Acquérir une bonne culture générale Mathématiques Les tests d'aptitudes verbales Annales corrigées Épreuves blanches Mobiliser les compétences professionnelles de l'adjoint administratif d'État Bureautique Épreuves blanches Techniques et recherche d'emploi/stage Sensibilisation au développement durable | Organisme | Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school) | Lieu de la formation | Formation a distance</t>
+          <t>Savoir fondamentauxOrientation et démarches professionnelsSocialisation et développement personnelAlternance en entreprise (près de 30% du temps)Des outils pédagogiques de liaison, d'évaluation et de suivi9 mois maximum + 12 mois de suivi post-parcours | Organisme | Ecole de la Deuxième Chance Grand Hainaut | Lieu de la formation | Ecole de la deuxième chance - site de VERVINS</t>
         </is>
       </c>
       <c r="T38" s="5" t="inlineStr"/>
       <c r="U38" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11205913/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11072382/true/false/false/true</t>
         </is>
       </c>
       <c r="V38" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-02&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W38" s="5" t="inlineStr">
@@ -4700,12 +4700,12 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Certification CLOE français langue étrangère - spécialité hôtellerie Restauration niveau A2 vers B1 (FOAD)</t>
+          <t>Préparation au concours d'adjoint administratif d'État principal de 2ème classe</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Nepsod Evolution</t>
+          <t>Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school)</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
@@ -4720,7 +4720,7 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Durée de 331 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 335 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -4735,12 +4735,12 @@
       </c>
       <c r="I39" s="6" t="inlineStr">
         <is>
-          <t>accueil@nepsod.com</t>
+          <t>foad@skillandyou.com</t>
         </is>
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>accueil@nepsod.com</t>
+          <t>foad@skillandyou.com</t>
         </is>
       </c>
       <c r="K39" s="7" t="inlineStr">
@@ -4755,19 +4755,15 @@
       </c>
       <c r="M39" s="7" t="inlineStr">
         <is>
-          <t>0474639587</t>
+          <t>0146006878</t>
         </is>
       </c>
       <c r="N39" s="7" t="inlineStr">
         <is>
-          <t>0474639587</t>
-        </is>
-      </c>
-      <c r="O39" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0146006878</t>
+        </is>
+      </c>
+      <c r="O39" s="7" t="inlineStr"/>
       <c r="P39" s="7" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -4781,17 +4777,13 @@
       <c r="R39" s="7" t="inlineStr"/>
       <c r="S39" s="7" t="inlineStr">
         <is>
-          <t>Accueil et initiation à la formation (1h30) - Module FLE visée insertion professionnelle : chercher un emploi, présenter son métier, présenter ses projets, interagir avec ses collègues, manipuler les outils numériques (120h30) - Module FOS Hôtellerie Restauration :découvrir la cuisine, travailler en cuisine, identifier les besoins d'un client, présenter des produits et services, gérer les réclamations (50h) Module environnement social et culturel : vie quotidienne et relations sociales, loisirs, patrimoine, citoyenneté et engagement (43h) Module Préparation et recherche de stage en entreprise (14h) Période de stage en entreprise (35 h) Module remise à niveau numérique (35 h maximum) Module accompagnement à l'après-formation (21h maximum) Module Préparation et passage de la certification CLOE (10h) Bilan final (1h) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T39" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Certification CLOE français langue étrangère</t>
-        </is>
-      </c>
+          <t>Votre intégration - Guide d'intégration - Bienvenue dans votre formation - Guide Métier Adjoint administratif d'État principal de 2ème classe - Guide de la formation - Guide des épreuves - Le concours d'adjoint administratif d'État principal de 2ème classe Aide à la réalisation de vos documents professionnels Compléter votre livret de suivi des compétences professionnelles Retranscrire et ordonner les idées principales d'un texte Annales corrigées Épreuves blanches Solliciter les connaissances fondamentales pour le concours Comprendre l'administration française Comprendre le fonctionnement des institutions françaises Acquérir des connaissances en français Acquérir une bonne culture générale Mathématiques Les tests d'aptitudes verbales Annales corrigées Épreuves blanches Mobiliser les compétences professionnelles de l'adjoint administratif d'État Bureautique Épreuves blanches Techniques et recherche d'emploi/stage Sensibilisation au développement durable | Organisme | Skill and you (Skill and You, Be academie, Cours Minerve, Cours Servais, Deficompta, Ecole chez soi, Ecole des pros, Educatel, ESECAD, Fashion skills, IFSA, Karis Formations, Lignes et formations, Naturadis, Eric Kayser school) | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T39" s="7" t="inlineStr"/>
       <c r="U39" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11576792/true/false/true/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11205913/true/false/true/true</t>
         </is>
       </c>
       <c r="V39" s="7" t="inlineStr">
@@ -4813,27 +4805,27 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière) - DEI</t>
+          <t>Certification CLOE français langue étrangère - spécialité hôtellerie Restauration niveau A2 vers B1 (FOAD)</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Nepsod Evolution</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 331 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
@@ -4848,12 +4840,12 @@
       </c>
       <c r="I40" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>accueil@nepsod.com</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>accueil@nepsod.com</t>
         </is>
       </c>
       <c r="K40" s="5" t="inlineStr">
@@ -4868,12 +4860,12 @@
       </c>
       <c r="M40" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0474639587</t>
         </is>
       </c>
       <c r="N40" s="5" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0474639587</t>
         </is>
       </c>
       <c r="O40" s="5" t="inlineStr">
@@ -4883,28 +4875,28 @@
       </c>
       <c r="P40" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q40" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R40" s="5" t="inlineStr"/>
       <c r="S40" s="5" t="inlineStr">
         <is>
-          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail (bureautique,recherche documentaire, rédaction de documents écrits, communication, anglais) La formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de1 800h, sous la forme de cours magistraux (750 h) travaux dirigés (1 050 h) le travail personnel guidé (suivi pédagogique, temps personnel guidé, supervision, travaux entre étudiants- 300 h) la formation clinique de 2 100 h le travail personnel complémentaire est estimé à 900 heures environ, soit 300 h par an. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Accueil et initiation à la formation (1h30) - Module FLE visée insertion professionnelle : chercher un emploi, présenter son métier, présenter ses projets, interagir avec ses collègues, manipuler les outils numériques (120h30) - Module FOS Hôtellerie Restauration :découvrir la cuisine, travailler en cuisine, identifier les besoins d'un client, présenter des produits et services, gérer les réclamations (50h) Module environnement social et culturel : vie quotidienne et relations sociales, loisirs, patrimoine, citoyenneté et engagement (43h) Module Préparation et recherche de stage en entreprise (14h) Période de stage en entreprise (35 h) Module remise à niveau numérique (35 h maximum) Module accompagnement à l'après-formation (21h maximum) Module Préparation et passage de la certification CLOE (10h) Bilan final (1h) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T40" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Certification CLOE français langue étrangère</t>
         </is>
       </c>
       <c r="U40" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11533526/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11576792/true/false/true/false</t>
         </is>
       </c>
       <c r="V40" s="5" t="inlineStr">
@@ -4926,27 +4918,27 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État de technicien de laboratoire médical</t>
+          <t>Diplôme d'État d'infirmier(ière) - DEI</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Association des Fondateurs et Protecteurs de l'Institut Catholique de Lyon (AFPICL) (UCLy - Institut Catholique de Lyon)</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>69002 Lyon 2e</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>10 place des Archives | 69002 Lyon 2e | France</t>
+          <t>115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1120 heures</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
@@ -4961,12 +4953,12 @@
       </c>
       <c r="I41" s="6" t="inlineStr">
         <is>
-          <t>fp@univ-catholyon.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>fp@univ-catholyon.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K41" s="7" t="inlineStr">
@@ -4981,12 +4973,12 @@
       </c>
       <c r="M41" s="7" t="inlineStr">
         <is>
-          <t>0472325134</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N41" s="7" t="inlineStr">
         <is>
-          <t>0472325134</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O41" s="7" t="inlineStr">
@@ -5005,15 +4997,19 @@
         </is>
       </c>
       <c r="R41" s="7" t="inlineStr"/>
-      <c r="S41" s="7" t="inlineStr"/>
+      <c r="S41" s="7" t="inlineStr">
+        <is>
+          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail (bureautique,recherche documentaire, rédaction de documents écrits, communication, anglais) La formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de1 800h, sous la forme de cours magistraux (750 h) travaux dirigés (1 050 h) le travail personnel guidé (suivi pédagogique, temps personnel guidé, supervision, travaux entre étudiants- 300 h) la formation clinique de 2 100 h le travail personnel complémentaire est estimé à 900 heures environ, soit 300 h par an. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T41" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État de technicien de laboratoire médical</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U41" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11026378/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11533526/true/false/false/false</t>
         </is>
       </c>
       <c r="V41" s="7" t="inlineStr">
@@ -5035,27 +5031,27 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'ambulancier</t>
+          <t>Diplôme d'État de technicien de laboratoire médical</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+          <t>Association des Fondateurs et Protecteurs de l'Institut Catholique de Lyon (AFPICL) (UCLy - Institut Catholique de Lyon)</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>69002 Lyon 2e</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+          <t>10 place des Archives | 69002 Lyon 2e | France</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>Durée de 801 heures (dont 245 heures en entreprise)</t>
+          <t>Durée de 1120 heures</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
@@ -5070,12 +5066,12 @@
       </c>
       <c r="I42" s="6" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>fp@univ-catholyon.fr</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>fp@univ-catholyon.fr</t>
         </is>
       </c>
       <c r="K42" s="5" t="inlineStr">
@@ -5090,12 +5086,12 @@
       </c>
       <c r="M42" s="5" t="inlineStr">
         <is>
-          <t>0472117903</t>
+          <t>0472325134</t>
         </is>
       </c>
       <c r="N42" s="5" t="inlineStr">
         <is>
-          <t>0472117903</t>
+          <t>0472325134</t>
         </is>
       </c>
       <c r="O42" s="5" t="inlineStr">
@@ -5114,24 +5110,20 @@
         </is>
       </c>
       <c r="R42" s="5" t="inlineStr"/>
-      <c r="S42" s="5" t="inlineStr">
-        <is>
-          <t>Non renseigne | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
+      <c r="S42" s="5" t="inlineStr"/>
       <c r="T42" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'ambulancier</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État de technicien de laboratoire médical</t>
         </is>
       </c>
       <c r="U42" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11871421/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11026378/true/false/false/false</t>
         </is>
       </c>
       <c r="V42" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W42" s="5" t="inlineStr">
@@ -5148,27 +5140,27 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Agent de prévention et de sécurité - Titre à finalité professionnelle (TFP APS)</t>
+          <t>Diplôme d'État d'ambulancier</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Global pro formation (Global pro formation (GPF))</t>
+          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>Blue Concept | 16 Rue Marcel Dutartre | 69100 Villeurbanne | France</t>
+          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Durée de 379 heures (dont 70 heures en entreprise)</t>
+          <t>Durée de 801 heures (dont 245 heures en entreprise)</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
@@ -5183,12 +5175,12 @@
       </c>
       <c r="I43" s="6" t="inlineStr">
         <is>
-          <t>globalproformation@gmail.com</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
-          <t>globalproformation@gmail.com</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="K43" s="7" t="inlineStr">
@@ -5203,12 +5195,12 @@
       </c>
       <c r="M43" s="7" t="inlineStr">
         <is>
-          <t>0666139535</t>
+          <t>0472117903</t>
         </is>
       </c>
       <c r="N43" s="7" t="inlineStr">
         <is>
-          <t>0666139535</t>
+          <t>0472117903</t>
         </is>
       </c>
       <c r="O43" s="7" t="inlineStr">
@@ -5218,7 +5210,7 @@
       </c>
       <c r="P43" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q43" s="7" t="inlineStr">
@@ -5229,22 +5221,22 @@
       <c r="R43" s="7" t="inlineStr"/>
       <c r="S43" s="7" t="inlineStr">
         <is>
-          <t>Théorie : SST : Protéger, Examiner (saignement, étouffement, conscience et respiration) et alerter (alerte et message d'accueil) La déontologie de l'agent de sécurité Les services publics de police et gendarmerie, le CNAPS Le cadre légal de la profession, le code pénal et le code de procédure pénale La sûreté de l'État Les armes Mise en sûreté et neutralisation des armes Prévention et actes terrorisme L'accueil, le contrôle d'accès, le contrôle visuel et la palpation de sécurité La prise en compte d'un poste de contrôle de sécurité et les consignes La protection du travailleur Isolé Le circuit de vérification La gestion des alarmes intrusion et incendie, la vidéo et la télésurveillance (surveillance et gardiennage) Les techniques d'information, de communication et la gestion des conflits L'incendie et les risques majeurs Le risque électrique (initiation) Le cadre légal et la problématique de l'activité d'événementiel La définition du terrorisme (historique, mécanisme, méthodologie et modes opératoires) Les différentes menaces terroristes et les niveaux de risque associés La prévention des actes de terrorisme par la reconnaissance des comportements suspects (profiling) et de la radicalisation violente L'action en cas d'attaque et suivant le type d'attaque (actes réflexes, mesures de mise en sécurité immédiate) Le combat en dernier recours L'alerte et la facilitation de l'intervention des forces de l'ordre La sécurisation d'une zone dans l'urgence, risque de sur-attentat et post-attentat. Pratique : Mise en pratique SST CQP APS: Code de la sécurité intérieure Code pénal et libertés publiques Déontologie professionnelle Secours à personnes (SST) Situations conflictuelles et résolution de conflit Consignes, compte rendu et rapport Gestion des risques majeurs, électriques, incendie Gestion d'alarmes Technique d'information et de communication Préparation d'une mission Gestion de conflit Contrôle d'accès Poste de contrôle de sécurité Rondes Palpation de sécurité et inspection de bagages Télésurveillance et vidéo protection Sensibilisation aux risques terroristes Examen : en cours de formation UV 1 (secourisme) : le candidat sera déclaré apte ou inapte en fonction des résultats de la grille d'évaluation conforme aux procédures de validation de l'INRS. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
+          <t>Non renseigne | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T43" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Agent de prévention et de sécurité</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'ambulancier</t>
         </is>
       </c>
       <c r="U43" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11870188/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11871421/true/false/false/false</t>
         </is>
       </c>
       <c r="V43" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
         </is>
       </c>
       <c r="W43" s="7" t="inlineStr">
@@ -5261,12 +5253,12 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'Etat de la Jeunesse de l'Education Populaire et du Sport spécialité "animation socio-éducative ou culturelle mention "coordination de projets" - RNCP 39930 spécialité "animation socio-éducative ou culturel mention "coordination de projets</t>
+          <t>Agent de prévention et de sécurité - Titre à finalité professionnelle (TFP APS)</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+          <t>Global pro formation (Global pro formation (GPF))</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
@@ -5276,12 +5268,12 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+          <t>Blue Concept | 16 Rue Marcel Dutartre | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 379 heures (dont 70 heures en entreprise)</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
@@ -5291,17 +5283,17 @@
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>https://arfatsema.catalogueformpro.com/3/dejeps-17/2857880/diplome-detat-de-la-jeunesse-de-leducation-populaire-et-du-sport-dejeps-17-specialite-animation-soci/registration?session_id=2846144</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>globalproformation@gmail.com</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>globalproformation@gmail.com</t>
         </is>
       </c>
       <c r="K44" s="5" t="inlineStr">
@@ -5316,12 +5308,12 @@
       </c>
       <c r="M44" s="5" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0666139535</t>
         </is>
       </c>
       <c r="N44" s="5" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0666139535</t>
         </is>
       </c>
       <c r="O44" s="5" t="inlineStr">
@@ -5331,7 +5323,7 @@
       </c>
       <c r="P44" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q44" s="5" t="inlineStr">
@@ -5342,17 +5334,17 @@
       <c r="R44" s="5" t="inlineStr"/>
       <c r="S44" s="5" t="inlineStr">
         <is>
-          <t>BC1: Animer et accompagner une équipe dans le champ du sport ou de l'animation Animer une équipe en structure d'éducation populaire : enjeux éthiques, valeurs et spécificités Réaliser un diagnostic des ressources humaines de son périmètre d'intervention Animer une équipe en structure d'éducation populaire : organisation, cadre légal, réglementation et procédures Diversité et inclusion : analyser les besoins et mettre en place une organisation adaptée Management participatif : développer le pouvoir d'agir d'une équipe Management participatif : outils et pratiques Accompagner une équipe: médiation et gestion de conflits Accompagner une équipe : émancipation et développement de l'autonomie Dynamique de groupe Animer un processus démocratique Projet d'action formative et conception de séance formative Droit du travail/Droit social Communication non violente Outils d'animation collective Outils d'accompagnement individuel Accompagner la vulnérabilité Dialogue social et syndical Responsabilité du coordinateur Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? BC2: Concevoir un projet d'action dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Education Populaire Rapport de domination Le numérique comme un fait social Esprit critique Culture politique Démocratie et contre pouvoir Pouvoir d'agir ou devoir d'agir? Diagnostic et enjeux De l'attribution d'une place à une culture de la participation Famille et éducation Connaissance des institutions publics et relation aux association ingéniérie sociale Portrait de territoire Mesure de l'impact social BC3 : Mettre en oeuvre et évaluer un projet d'action Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie de projet Mesure de l'impact social Accompagner la vulnérabilité La protection de l'Enfance en France Outils participatifs Intelligence artificielle et fonction de coordination BC4 : Développer les partenariats opérationnelles et contribuer aux dynamiques institutionnelles dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Connaissance des institutions publics et relation aux associations Démocratie et contre pouvoir Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie sociale Outils participatifs | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Théorie : SST : Protéger, Examiner (saignement, étouffement, conscience et respiration) et alerter (alerte et message d'accueil) La déontologie de l'agent de sécurité Les services publics de police et gendarmerie, le CNAPS Le cadre légal de la profession, le code pénal et le code de procédure pénale La sûreté de l'État Les armes Mise en sûreté et neutralisation des armes Prévention et actes terrorisme L'accueil, le contrôle d'accès, le contrôle visuel et la palpation de sécurité La prise en compte d'un poste de contrôle de sécurité et les consignes La protection du travailleur Isolé Le circuit de vérification La gestion des alarmes intrusion et incendie, la vidéo et la télésurveillance (surveillance et gardiennage) Les techniques d'information, de communication et la gestion des conflits L'incendie et les risques majeurs Le risque électrique (initiation) Le cadre légal et la problématique de l'activité d'événementiel La définition du terrorisme (historique, mécanisme, méthodologie et modes opératoires) Les différentes menaces terroristes et les niveaux de risque associés La prévention des actes de terrorisme par la reconnaissance des comportements suspects (profiling) et de la radicalisation violente L'action en cas d'attaque et suivant le type d'attaque (actes réflexes, mesures de mise en sécurité immédiate) Le combat en dernier recours L'alerte et la facilitation de l'intervention des forces de l'ordre La sécurisation d'une zone dans l'urgence, risque de sur-attentat et post-attentat. Pratique : Mise en pratique SST CQP APS: Code de la sécurité intérieure Code pénal et libertés publiques Déontologie professionnelle Secours à personnes (SST) Situations conflictuelles et résolution de conflit Consignes, compte rendu et rapport Gestion des risques majeurs, électriques, incendie Gestion d'alarmes Technique d'information et de communication Préparation d'une mission Gestion de conflit Contrôle d'accès Poste de contrôle de sécurité Rondes Palpation de sécurité et inspection de bagages Télésurveillance et vidéo protection Sensibilisation aux risques terroristes Examen : en cours de formation UV 1 (secourisme) : le candidat sera déclaré apte ou inapte en fonction des résultats de la grille d'évaluation conforme aux procédures de validation de l'INRS. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
         </is>
       </c>
       <c r="T44" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | DEJEPS spécialité animation socio-éducative ou culturelle mention coordination de projets</t>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Agent de prévention et de sécurité</t>
         </is>
       </c>
       <c r="U44" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880827/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11870188/true/false/false/false</t>
         </is>
       </c>
       <c r="V44" s="5" t="inlineStr">
@@ -5374,27 +5366,27 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Créez votre vignoble bio de raisin de table, rentable et résilient - Devenez autonome pour produire et vendre votre propre raisin de table bio</t>
+          <t>Diplôme d'Etat de la Jeunesse de l'Education Populaire et du Sport spécialité "animation socio-éducative ou culturelle mention "coordination de projets" - RNCP 39930 spécialité "animation socio-éducative ou culturel mention "coordination de projets</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>SARL Agri-learn éditions</t>
+          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>69001 Lyon</t>
+          <t>69100 Villeurbanne</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 69001 Lyon | France</t>
+          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Durée de 9 heures</t>
+          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -5404,17 +5396,17 @@
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://arfatsema.catalogueformpro.com/3/dejeps-17/2857880/diplome-detat-de-la-jeunesse-de-leducation-populaire-et-du-sport-dejeps-17-specialite-animation-soci/registration?session_id=2846144</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="K45" s="7" t="inlineStr">
@@ -5429,15 +5421,19 @@
       </c>
       <c r="M45" s="7" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0478031711</t>
         </is>
       </c>
       <c r="N45" s="7" t="inlineStr">
         <is>
-          <t>0620021214</t>
-        </is>
-      </c>
-      <c r="O45" s="7" t="inlineStr"/>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="O45" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P45" s="7" t="inlineStr">
         <is>
           <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
@@ -5445,24 +5441,28 @@
       </c>
       <c r="Q45" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R45" s="7" t="inlineStr"/>
       <c r="S45" s="7" t="inlineStr">
         <is>
-          <t>1. Taille de la vigne Principes de taille (formation et production) Techniques de taille douce Entretien et corrections2. Modes de conduite Choix du système (lyre, gable, plan vertical. Comparaison des conduites Adaptation au contexte pédoclimatique3. Fertilité des sols Gestion du sol (travail / non-travail) Irrigation Maintien de la fertilité en bio4. Travaux du vignoble Protection contre maladies et ravageurs Calendrier des interventions Conduite sous abri (tunnel)5. Choix des plants Sélection des variétés Choix du porte-greffe Adaptation au marché et au terroir6. Plantation Préparation du sol Étapes de plantation Coûts et organisation7. Récolte et commercialisation Récolte et conservation Organisation du travail Valorisation et vente8. Protection du vignoble en bio Biocontrôle et PNPP Réduction des intrants Stratégies alternatives9. Gestion des maladies et ravageurs Identification des principaux risques Prévention et lutte adaptée10. Pilotage des traitements Stratégie cuivre / soufre Optimisation des doses11. Approche agroécologique Biodiversité fonctionnelle Variétés résistantes | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T45" s="7" t="inlineStr"/>
+          <t>BC1: Animer et accompagner une équipe dans le champ du sport ou de l'animation Animer une équipe en structure d'éducation populaire : enjeux éthiques, valeurs et spécificités Réaliser un diagnostic des ressources humaines de son périmètre d'intervention Animer une équipe en structure d'éducation populaire : organisation, cadre légal, réglementation et procédures Diversité et inclusion : analyser les besoins et mettre en place une organisation adaptée Management participatif : développer le pouvoir d'agir d'une équipe Management participatif : outils et pratiques Accompagner une équipe: médiation et gestion de conflits Accompagner une équipe : émancipation et développement de l'autonomie Dynamique de groupe Animer un processus démocratique Projet d'action formative et conception de séance formative Droit du travail/Droit social Communication non violente Outils d'animation collective Outils d'accompagnement individuel Accompagner la vulnérabilité Dialogue social et syndical Responsabilité du coordinateur Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? BC2: Concevoir un projet d'action dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Education Populaire Rapport de domination Le numérique comme un fait social Esprit critique Culture politique Démocratie et contre pouvoir Pouvoir d'agir ou devoir d'agir? Diagnostic et enjeux De l'attribution d'une place à une culture de la participation Famille et éducation Connaissance des institutions publics et relation aux association ingéniérie sociale Portrait de territoire Mesure de l'impact social BC3 : Mettre en oeuvre et évaluer un projet d'action Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie de projet Mesure de l'impact social Accompagner la vulnérabilité La protection de l'Enfance en France Outils participatifs Intelligence artificielle et fonction de coordination BC4 : Développer les partenariats opérationnelles et contribuer aux dynamiques institutionnelles dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Introduction à la sociologie par la pratique : l'oeil et l'oreille vous avez dit posture? Connaissance des institutions publics et relation aux associations Démocratie et contre pouvoir Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Ingéniérie sociale Outils participatifs | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T45" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | DEJEPS spécialité animation socio-éducative ou culturelle mention coordination de projets</t>
+        </is>
+      </c>
       <c r="U45" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11870193/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11880827/true/false/false/false</t>
         </is>
       </c>
       <c r="V45" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
       <c r="W45" s="7" t="inlineStr">
@@ -5479,27 +5479,27 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
+          <t>Créez votre vignoble bio de raisin de table, rentable et résilient - Devenez autonome pour produire et vendre votre propre raisin de table bio</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>UCPA Formation</t>
+          <t>SARL Agri-learn éditions</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>69200 Vénissieux</t>
+          <t>69001 Lyon</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>16 Avenue Dr Georges Levy | 69200 Vénissieux | France</t>
+          <t>Formation a distance | 69001 Lyon | France</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1267 heures (dont 637 heures en entreprise)</t>
+          <t>Durée de 9 heures</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
@@ -5514,12 +5514,12 @@
       </c>
       <c r="I46" s="6" t="inlineStr">
         <is>
-          <t>ucpa-formation@ucpa.asso.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>ucpa-formation@ucpa.asso.fr | fgehant@ucpa.asso.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="K46" s="5" t="inlineStr">
@@ -5534,43 +5534,35 @@
       </c>
       <c r="M46" s="5" t="inlineStr">
         <is>
-          <t>0642833617</t>
+          <t>0620021214</t>
         </is>
       </c>
       <c r="N46" s="5" t="inlineStr">
         <is>
-          <t>0642833617</t>
-        </is>
-      </c>
-      <c r="O46" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="O46" s="5" t="inlineStr"/>
       <c r="P46" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q46" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R46" s="5" t="inlineStr"/>
       <c r="S46" s="5" t="inlineStr">
         <is>
-          <t>Unité capitalisable (UC) - 1. Encadrer tout public dans tout lieu et toute structureUnité capitalisable (UC) - 2. Mettre en œuvre un projet d'animation s'inscrivant dans le projet de la structureUnité capitalisable (UC) - 3. Conduire une séance, un cycle d'animation ou d'apprentissage dans le champ des activités aquatiques et de la natationUnité capitalisable (UC) - 4. Mobiliser les techniques des activités aquatiques et de la natation pour mettre en œuvre une séance ou un cycle d'apprentissage | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T46" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
-        </is>
-      </c>
+          <t>1. Taille de la vigne Principes de taille (formation et production) Techniques de taille douce Entretien et corrections2. Modes de conduite Choix du système (lyre, gable, plan vertical. Comparaison des conduites Adaptation au contexte pédoclimatique3. Fertilité des sols Gestion du sol (travail / non-travail) Irrigation Maintien de la fertilité en bio4. Travaux du vignoble Protection contre maladies et ravageurs Calendrier des interventions Conduite sous abri (tunnel)5. Choix des plants Sélection des variétés Choix du porte-greffe Adaptation au marché et au terroir6. Plantation Préparation du sol Étapes de plantation Coûts et organisation7. Récolte et commercialisation Récolte et conservation Organisation du travail Valorisation et vente8. Protection du vignoble en bio Biocontrôle et PNPP Réduction des intrants Stratégies alternatives9. Gestion des maladies et ravageurs Identification des principaux risques Prévention et lutte adaptée10. Pilotage des traitements Stratégie cuivre / soufre Optimisation des doses11. Approche agroécologique Biodiversité fonctionnelle Variétés résistantes | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T46" s="5" t="inlineStr"/>
       <c r="U46" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11447001/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11870193/true/false/false/false</t>
         </is>
       </c>
       <c r="V46" s="5" t="inlineStr">
@@ -5592,27 +5584,27 @@
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'aide-soignant - DEAS</t>
+          <t>BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>UCPA Formation</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>69003 Lyon 3e</t>
+          <t>69200 Vénissieux</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
+          <t>16 Avenue Dr Georges Levy | 69200 Vénissieux | France</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1540 heures (dont 770 heures en entreprise)</t>
+          <t>Durée de 1267 heures (dont 637 heures en entreprise)</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -5622,17 +5614,17 @@
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=aide-soignant</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>ucpa-formation@ucpa.asso.fr</t>
         </is>
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>ucpa-formation@ucpa.asso.fr | fgehant@ucpa.asso.fr</t>
         </is>
       </c>
       <c r="K47" s="7" t="inlineStr">
@@ -5647,12 +5639,12 @@
       </c>
       <c r="M47" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0642833617</t>
         </is>
       </c>
       <c r="N47" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0642833617</t>
         </is>
       </c>
       <c r="O47" s="7" t="inlineStr">
@@ -5673,17 +5665,17 @@
       <c r="R47" s="7" t="inlineStr"/>
       <c r="S47" s="7" t="inlineStr">
         <is>
-          <t>La formation conduisant au diplôme d'État d'aide-soignant, 17 semaines d'enseignement théoriques organisées autour de 8 modules : Accompagnement d'une personne dans les activités de la vie quotidienne L'état clinique d'une personne Les soins Ergonomie Relation Communication Hygiène des locaux hospitaliers Transmission des informations Organisation du travail Les titulaires du DE d'auxiliaire de puériculture, du DE d'aide médico-psychologique, du DE d'auxiliaire de vie sociale ou de la MC aide à domicile, sont dispensés de certaines unités de formation. La formation comprend également 6 stages d'une durée totale de 24 semaines en milieu hospitalier ou extra-hospitalier. Possibilité d'effectuer la formation en initial ou en apprentissage. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Unité capitalisable (UC) - 1. Encadrer tout public dans tout lieu et toute structureUnité capitalisable (UC) - 2. Mettre en œuvre un projet d'animation s'inscrivant dans le projet de la structureUnité capitalisable (UC) - 3. Conduire une séance, un cycle d'animation ou d'apprentissage dans le champ des activités aquatiques et de la natationUnité capitalisable (UC) - 4. Mobiliser les techniques des activités aquatiques et de la natation pour mettre en œuvre une séance ou un cycle d'apprentissage | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T47" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'aide-soignant</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | BPJEPS spécialité éducateur sportif mention activités aquatiques et de la natation</t>
         </is>
       </c>
       <c r="U47" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11533549/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11447001/true/false/false/false</t>
         </is>
       </c>
       <c r="V47" s="7" t="inlineStr">
@@ -5705,12 +5697,12 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>Diplôme d'État d'aide-soignant - DEAS</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
@@ -5720,12 +5712,12 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
+          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 Avenue Lacassagne | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 1540 heures (dont 770 heures en entreprise)</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
@@ -5735,17 +5727,17 @@
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=aide-soignant</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>magaly.lebrat@chu-lyon.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K48" s="5" t="inlineStr">
@@ -5760,12 +5752,12 @@
       </c>
       <c r="M48" s="5" t="inlineStr">
         <is>
-          <t>0472117979</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N48" s="5" t="inlineStr">
         <is>
-          <t>0472117979</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O48" s="5" t="inlineStr">
@@ -5784,15 +5776,19 @@
         </is>
       </c>
       <c r="R48" s="5" t="inlineStr"/>
-      <c r="S48" s="5" t="inlineStr"/>
+      <c r="S48" s="5" t="inlineStr">
+        <is>
+          <t>La formation conduisant au diplôme d'État d'aide-soignant, 17 semaines d'enseignement théoriques organisées autour de 8 modules : Accompagnement d'une personne dans les activités de la vie quotidienne L'état clinique d'une personne Les soins Ergonomie Relation Communication Hygiène des locaux hospitaliers Transmission des informations Organisation du travail Les titulaires du DE d'auxiliaire de puériculture, du DE d'aide médico-psychologique, du DE d'auxiliaire de vie sociale ou de la MC aide à domicile, sont dispensés de certaines unités de formation. La formation comprend également 6 stages d'une durée totale de 24 semaines en milieu hospitalier ou extra-hospitalier. Possibilité d'effectuer la formation en initial ou en apprentissage. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
       <c r="T48" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'aide-soignant</t>
         </is>
       </c>
       <c r="U48" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11817055/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11533549/true/false/false/true</t>
         </is>
       </c>
       <c r="V48" s="5" t="inlineStr">
@@ -5814,12 +5810,12 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'assistant de service social - DE ASS</t>
+          <t>Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
+          <t>Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (Institut de Formation aux Carrières de Santé - Secteur Est des Hospices civils de Lyon (IFCS - HCL))</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
@@ -5829,12 +5825,12 @@
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 avenue Lacassagne | Croix Rouge francaise | 69003 Lyon 3e | France</t>
+          <t>5 Avenue Esquirol | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Durée de 3420 heures (dont 1680 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -5844,17 +5840,17 @@
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=assistant%20de%20service%20social</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
+          <t>magaly.lebrat@chu-lyon.fr</t>
         </is>
       </c>
       <c r="K49" s="7" t="inlineStr">
@@ -5869,12 +5865,12 @@
       </c>
       <c r="M49" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0472117979</t>
         </is>
       </c>
       <c r="N49" s="7" t="inlineStr">
         <is>
-          <t>0472115560</t>
+          <t>0472117979</t>
         </is>
       </c>
       <c r="O49" s="7" t="inlineStr">
@@ -5896,12 +5892,12 @@
       <c r="S49" s="7" t="inlineStr"/>
       <c r="T49" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U49" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11672249/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11817055/true/false/false/false</t>
         </is>
       </c>
       <c r="V49" s="7" t="inlineStr">
@@ -5923,27 +5919,27 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'éducateur spécialisé</t>
+          <t>Diplôme d'État d'assistant de service social - DE ASS</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales (ARFRIPS - Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales)</t>
+          <t>Croix Rouge Française - Institut Régional de Formation Sanitaire et Sociale Auvergne-Rhône-Alpes (Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site St Etienne)</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>69009 Lyon 9e</t>
+          <t>69003 Lyon 3e</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>10 Impasse Pierre Baizet | 69009 Lyon 9e | France</t>
+          <t>Croix-Rouge Compétence Auvergne-Rhône-Alpes - Site de Lyon | 115 avenue Lacassagne | Croix Rouge francaise | 69003 Lyon 3e | France</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>Durée de 3442 heures (dont 1925 heures en entreprise)</t>
+          <t>Durée de 3420 heures (dont 1680 heures en entreprise)</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
@@ -5953,17 +5949,17 @@
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.croix-rouge.fr/formation-professionnelle?region=auvergne_rhone_alpes&amp;type=formation_diplomante_et_certifiante&amp;search=assistant%20de%20service%20social</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
         <is>
-          <t>info@arfrips.fr</t>
+          <t>competence.ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>info@arfrips.fr</t>
+          <t>competence.ara@croix-rouge.fr | lyon.competence-ara@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K50" s="5" t="inlineStr">
@@ -5978,12 +5974,12 @@
       </c>
       <c r="M50" s="5" t="inlineStr">
         <is>
-          <t>0478699090</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="N50" s="5" t="inlineStr">
         <is>
-          <t>0478699090</t>
+          <t>0472115560</t>
         </is>
       </c>
       <c r="O50" s="5" t="inlineStr">
@@ -6005,17 +6001,17 @@
       <c r="S50" s="5" t="inlineStr"/>
       <c r="T50" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur spécialisé</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
         </is>
       </c>
       <c r="U50" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11737248/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11672249/true/false/false/false</t>
         </is>
       </c>
       <c r="V50" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=0-9&amp;tri=0</t>
         </is>
       </c>
       <c r="W50" s="5" t="inlineStr">
@@ -6032,27 +6028,27 @@
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet - RNCP 39931 - spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+          <t>Diplôme d'État d'éducateur spécialisé</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
+          <t>Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales (ARFRIPS - Association Régionale pour la Formation, la Recherche et l'Innovation en Pratiques Sociales)</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>69100 Villeurbanne</t>
+          <t>69009 Lyon 9e</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
+          <t>10 Impasse Pierre Baizet | 69009 Lyon 9e | France</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
+          <t>Durée de 3442 heures (dont 1925 heures en entreprise)</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -6062,17 +6058,17 @@
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>https://arfatsema.catalogueformpro.com/2/desjeps-17/2858060/desjeps-17-diplome-detat-superieur-de-la-jeunesse-de-leducation-populaire-et-du-sport-specialite-ani</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>info@arfrips.fr</t>
         </is>
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>arfatsema.direction@orange.fr</t>
+          <t>info@arfrips.fr</t>
         </is>
       </c>
       <c r="K51" s="7" t="inlineStr">
@@ -6087,12 +6083,12 @@
       </c>
       <c r="M51" s="7" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0478699090</t>
         </is>
       </c>
       <c r="N51" s="7" t="inlineStr">
         <is>
-          <t>0478031711</t>
+          <t>0478699090</t>
         </is>
       </c>
       <c r="O51" s="7" t="inlineStr">
@@ -6102,7 +6098,7 @@
       </c>
       <c r="P51" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q51" s="7" t="inlineStr">
@@ -6111,19 +6107,15 @@
         </is>
       </c>
       <c r="R51" s="7" t="inlineStr"/>
-      <c r="S51" s="7" t="inlineStr">
-        <is>
-          <t>BC1 : Construire, avec les instances de gouvernance, la stratégie de développement d'une structure dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Éducation Populaire Culture Politique Rapport de domination Pouvoir d'Agir et Vulnérabilité Esprit critique Transformation social/rapport sociaux Le numérique comme un fait social Nouvel esprit du capitalisme Laicité et valeurs de la République Violence sexiste violences sexuelles Ingénierie social en lien avec la structure Réaliser un diagnostic RH et financier Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Elaboration de la stratégie de développement en lien avec les instances de gouvernance Animer un processus démocratique Démocratie et contre pouvoir BC2 : Concevoir et diriger un projet de développement de la structure Cartographie des relations et l'environnement de son association Ingénierie du projet Processus d'évaluation dans une démarche partagée et participative Outils participatifs Outils de communication Utilité sociale BC3 : Manager l'équipe et gérer les ressources humaines ( et la démarche Qualité, Sécurité, Santé au Travail et Environnement d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Gestion des ressources humaines en structures d'éducation populaire : enjeux, éthique et complexités associative Articulation employeur bénévole - direction dans la gestion des ressources humaines : définition d'une politique RH et organisation des délégations de pouvoir Gérer l'équipe au quotidien : accompagnement, régulation et gestion conflits Analyse des pratiques en co-développement Développer le pouvoir d'agir des salariés Attractivité, recrutement, intégration et fidélisation des salariés Diversité, inclusion et égalité professionnelle au sein de son organisation Assurer la GPEC, la formation et la gestion des carrières dans un alignement éthique Le financement de la formation professionnelle Qualité de vie Santé sécurité au travail Droit du travail/Droit social Dialogue social/dialogue syndical Cadre général des RPS Démarche prévention et outils BC4 : Assurer la gestion financière, matérielle et administrative d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Comprendre les fondamentaux de la situation financière Initiation à l'analyse financière associative ou de structure d'intérêt général Identifier les leviers de financement Construire des scénarios budgétaires et faire des arbitrages Élaborer un plan d'action financier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
+      <c r="S51" s="7" t="inlineStr"/>
       <c r="T51" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur spécialisé</t>
         </is>
       </c>
       <c r="U51" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880835/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11737248/true/false/false/false</t>
         </is>
       </c>
       <c r="V51" s="7" t="inlineStr">
@@ -6145,27 +6137,27 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>Créer sa ferme en circuit court : transformation, commercialisation et communication</t>
+          <t>DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet - RNCP 39931 - spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>SARL Agri-learn éditions</t>
+          <t>Association régionale pour la formation au travail socio-éducatif et aux métiers de l'animation</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>69001 Lyon</t>
+          <t>69100 Villeurbanne</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 69001 Lyon | France</t>
+          <t>1 Rue Charny | 69100 Villeurbanne | France</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>Durée de 20 heures</t>
+          <t>Durée de 1200 heures (dont 500 heures en entreprise)</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
@@ -6175,17 +6167,17 @@
       </c>
       <c r="H52" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://arfatsema.catalogueformpro.com/2/desjeps-17/2858060/desjeps-17-diplome-detat-superieur-de-la-jeunesse-de-leducation-populaire-et-du-sport-specialite-ani</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>fanny@agrilearn.fr</t>
+          <t>arfatsema.direction@orange.fr</t>
         </is>
       </c>
       <c r="K52" s="5" t="inlineStr">
@@ -6200,15 +6192,19 @@
       </c>
       <c r="M52" s="5" t="inlineStr">
         <is>
-          <t>0620021214</t>
+          <t>0478031711</t>
         </is>
       </c>
       <c r="N52" s="5" t="inlineStr">
         <is>
-          <t>0620021214</t>
-        </is>
-      </c>
-      <c r="O52" s="5" t="inlineStr"/>
+          <t>0478031711</t>
+        </is>
+      </c>
+      <c r="O52" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P52" s="5" t="inlineStr">
         <is>
           <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
@@ -6216,19 +6212,23 @@
       </c>
       <c r="Q52" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R52" s="5" t="inlineStr"/>
       <c r="S52" s="5" t="inlineStr">
         <is>
-          <t>Cette formation s'appuie sur plusieurs compétences essentielles : Stratégie commerciale et étude de marché : définir son offre, ses volumes, ses prix et ses circuits de vente Techniques de vente : maîtriser les étapes clés pour convaincre et fidéliser les clients Transformation des produits agricoles : valoriser ses matières premières pour créer de la valeur ajoutée Hygiène et réglementation : garantir la sécurité sanitaire dans les ateliers de transformation Communication et prospection : développer sa clientèle et promouvoir ses produits Valorisation des produits : savoir parler de ses produits et les mettre en avant (ex : dégustation) L'ensemble permet d'acquérir une vision globale du fonctionnement d'une ferme en circuit court, de la production jusqu'à la vente. 3 heures de visio avec les experts sont prévues dans le cursus. | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T52" s="5" t="inlineStr"/>
+          <t>BC1 : Construire, avec les instances de gouvernance, la stratégie de développement d'une structure dans le domaine de l'animation socio- éducative, culturelle et/ou sportive Éducation Populaire Culture Politique Rapport de domination Pouvoir d'Agir et Vulnérabilité Esprit critique Transformation social/rapport sociaux Le numérique comme un fait social Nouvel esprit du capitalisme Laicité et valeurs de la République Violence sexiste violences sexuelles Ingénierie social en lien avec la structure Réaliser un diagnostic RH et financier Penser et structurer son action dans la complexité : à la découverte de l'entrainement mental Elaboration de la stratégie de développement en lien avec les instances de gouvernance Animer un processus démocratique Démocratie et contre pouvoir BC2 : Concevoir et diriger un projet de développement de la structure Cartographie des relations et l'environnement de son association Ingénierie du projet Processus d'évaluation dans une démarche partagée et participative Outils participatifs Outils de communication Utilité sociale BC3 : Manager l'équipe et gérer les ressources humaines ( et la démarche Qualité, Sécurité, Santé au Travail et Environnement d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Gestion des ressources humaines en structures d'éducation populaire : enjeux, éthique et complexités associative Articulation employeur bénévole - direction dans la gestion des ressources humaines : définition d'une politique RH et organisation des délégations de pouvoir Gérer l'équipe au quotidien : accompagnement, régulation et gestion conflits Analyse des pratiques en co-développement Développer le pouvoir d'agir des salariés Attractivité, recrutement, intégration et fidélisation des salariés Diversité, inclusion et égalité professionnelle au sein de son organisation Assurer la GPEC, la formation et la gestion des carrières dans un alignement éthique Le financement de la formation professionnelle Qualité de vie Santé sécurité au travail Droit du travail/Droit social Dialogue social/dialogue syndical Cadre général des RPS Démarche prévention et outils BC4 : Assurer la gestion financière, matérielle et administrative d'une structure dans le domaine de l'animation socio-éducative, culturelle et/ou sportive Comprendre les fondamentaux de la situation financière Initiation à l'analyse financière associative ou de structure d'intérêt général Identifier les leviers de financement Construire des scénarios budgétaires et faire des arbitrages Élaborer un plan d'action financier | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T52" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | DESJEPS spécialité animation socio-éducative, culturelle et/ou sportive mention direction de structure et de projet</t>
+        </is>
+      </c>
       <c r="U52" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11880868/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11880835/true/false/false/false</t>
         </is>
       </c>
       <c r="V52" s="5" t="inlineStr">
@@ -6250,27 +6250,27 @@
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Titre professionnel administrateur d'infrastructures sécurisées (FOAD)</t>
+          <t>Créer sa ferme en circuit court : transformation, commercialisation et communication</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>STUDI</t>
+          <t>SARL Agri-learn éditions</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>69001 Lyon</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>Formation a distance | 69001 Lyon | France</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>Durée de 947 heures (dont 350 heures en entreprise)</t>
+          <t>Durée de 20 heures</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -6285,12 +6285,12 @@
       </c>
       <c r="I53" s="6" t="inlineStr">
         <is>
-          <t>contact@studi.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>contact@studi.fr | conseiller-formation.aoft@studi.fr</t>
+          <t>fanny@agrilearn.fr</t>
         </is>
       </c>
       <c r="K53" s="7" t="inlineStr">
@@ -6305,22 +6305,18 @@
       </c>
       <c r="M53" s="7" t="inlineStr">
         <is>
-          <t>0174888555</t>
+          <t>0620021214</t>
         </is>
       </c>
       <c r="N53" s="7" t="inlineStr">
         <is>
-          <t>0174888555</t>
-        </is>
-      </c>
-      <c r="O53" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0620021214</t>
+        </is>
+      </c>
+      <c r="O53" s="7" t="inlineStr"/>
       <c r="P53" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par un Opérateur de Compétences mandaté par les branches professionnelles concernées</t>
         </is>
       </c>
       <c r="Q53" s="7" t="inlineStr">
@@ -6331,25 +6327,134 @@
       <c r="R53" s="7" t="inlineStr"/>
       <c r="S53" s="7" t="inlineStr">
         <is>
+          <t>Cette formation s'appuie sur plusieurs compétences essentielles : Stratégie commerciale et étude de marché : définir son offre, ses volumes, ses prix et ses circuits de vente Techniques de vente : maîtriser les étapes clés pour convaincre et fidéliser les clients Transformation des produits agricoles : valoriser ses matières premières pour créer de la valeur ajoutée Hygiène et réglementation : garantir la sécurité sanitaire dans les ateliers de transformation Communication et prospection : développer sa clientèle et promouvoir ses produits Valorisation des produits : savoir parler de ses produits et les mettre en avant (ex : dégustation) L'ensemble permet d'acquérir une vision globale du fonctionnement d'une ferme en circuit court, de la production jusqu'à la vente. 3 heures de visio avec les experts sont prévues dans le cursus. | Organisme | SARL Agri-learn éditions | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T53" s="7" t="inlineStr"/>
+      <c r="U53" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/11880868/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V53" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W53" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>Titre professionnel administrateur d'infrastructures sécurisées (FOAD)</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>STUDI</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>75004 Paris</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Formation a distance | 75004 Paris | France</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 947 heures (dont 350 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I54" s="6" t="inlineStr">
+        <is>
+          <t>contact@studi.fr</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>contact@studi.fr | conseiller-formation.aoft@studi.fr</t>
+        </is>
+      </c>
+      <c r="K54" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L54" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M54" s="5" t="inlineStr">
+        <is>
+          <t>0174888555</t>
+        </is>
+      </c>
+      <c r="N54" s="5" t="inlineStr">
+        <is>
+          <t>0174888555</t>
+        </is>
+      </c>
+      <c r="O54" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P54" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par France Travail</t>
+        </is>
+      </c>
+      <c r="Q54" s="5" t="inlineStr">
+        <is>
+          <t>À distance</t>
+        </is>
+      </c>
+      <c r="R54" s="5" t="inlineStr"/>
+      <c r="S54" s="5" t="inlineStr">
+        <is>
           <t>Administrer et sécuriser les infrastructures Les bonnes pratiques dans l'administration des infrastructures Utiliser un logiciel de gestion centralisé : GLPI Configurer le routage Administrer et sécuriser le réseau Automatiser les tâches d'administration Administrer et sécuriser les systèmes Les bases des serveurs virtualisés Administrer et sécuriser une infrastructure de serveurs virtualisée Gérer des containersConcevoir et mettre en œuvre une solution en réponse à un besoin d'évolution Les bases des solutions techniques Proposer une solution informatique répondant à des besoins nouveaux Mettre en production des évolutions de l'infrastructure Les bases de la supervision Superviser la disponibilité de l'infrastructure et en présenter les résultats Mesurer les performances et la disponibilité de l'infrastructureParticiper à la gestion de la cybersécurité Les bases de la cybersécurité Participer à la mesure et à l'analyse du niveau de sécurité de l'infrastructure Participer à l'élaboration et à la mise en œuvre de la politique de sécurité Participer à la détection et au traitement des incidents de sécurité | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
-      <c r="T53" s="7" t="inlineStr">
+      <c r="T54" s="5" t="inlineStr">
         <is>
           <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel administrateur d'infrastructures sécurisées</t>
         </is>
       </c>
-      <c r="U53" s="7" t="inlineStr">
+      <c r="U54" s="5" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/detail/11590088/true/false/true/false</t>
         </is>
       </c>
-      <c r="V53" s="7" t="inlineStr">
+      <c r="V54" s="5" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-69&amp;range=10-19&amp;tri=0</t>
         </is>
       </c>
-      <c r="W53" s="7" t="inlineStr">
+      <c r="W54" s="5" t="inlineStr">
         <is>
           <t>ok</t>
         </is>

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-07-27
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1227,7 +1227,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1239,7 +1239,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1344,17 +1344,17 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1350 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -1384,12 +1384,12 @@
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1404,19 +1404,15 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr"/>
       <c r="P8" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -1430,22 +1426,18 @@
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>11 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 : Démarrez votre formation d'Accompagnement Educatif Petite Enfance ; Projet 2 - Préparez un environnement sécurisé pour le jeune enfant ; Projet 3 - Développez des activités éducatives adaptées à la petite enfance ; Projet 4 - Appliquez les protocoles de santé dans le cadre de la petite enfance ; Projet 5 - Soutenez le personnel enseignant dans un contexte collectif ; Projet 6 - Améliorez les conditions d'accueil en école maternelle ; Projet 7 - Organisez l'accueil individuel au domicile ; Projet 8 - Gérez les tâches domestiques et la préparation des repas pour l'enfant ; Projet 9 : Proposer des solutions de prévention, santé et environnement ; Projet 10 : Remise à niveau scolaire ; Projet 11 : Préparez-vous pour l'examen final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T8" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
+          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120311/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
         </is>
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1457,12 +1449,12 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Conseiller emploi et accompagnement professionnel</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -1482,7 +1474,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1140 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 1350 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1543,22 +1535,22 @@
       <c r="R9" s="7" t="inlineStr"/>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>10 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de conseiller emploi et évolution professionnelle ; Projet 2 - Accompagnez en parallèle de nombreuses personnes avec des besoins différents ; Projet 3 - Élaborez une veille et analysez le marché de l'emploi ; Projet 4 - Réalisez un diagnostic et co-construisez un plan d'action avec vos bénéficiaires ; Projet 5 - Adaptez votre posture pour l'accompagnement des bénéficiaires ; Projet 6 - Établissez et validez un projet d'accompagnement professionnel ; Projet 7 - Établissez un plan d'action et un bilan professionnel ; Projet 8 - Concevez un atelier sur les métiers émergents avec l'IA ; Projet 9 - Développez votre projet territorial avec des partenaires ; Projet 10 - Élaborez votre boîte à outils pour accompagner vers l'emploi. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
+          <t>11 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 : Démarrez votre formation d'Accompagnement Educatif Petite Enfance ; Projet 2 - Préparez un environnement sécurisé pour le jeune enfant ; Projet 3 - Développez des activités éducatives adaptées à la petite enfance ; Projet 4 - Appliquez les protocoles de santé dans le cadre de la petite enfance ; Projet 5 - Soutenez le personnel enseignant dans un contexte collectif ; Projet 6 - Améliorez les conditions d'accueil en école maternelle ; Projet 7 - Organisez l'accueil individuel au domicile ; Projet 8 - Gérez les tâches domestiques et la préparation des repas pour l'enfant ; Projet 9 : Proposer des solutions de prévention, santé et environnement ; Projet 10 : Remise à niveau scolaire ; Projet 11 : Préparez-vous pour l'examen final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Conseiller emploi et accompagnement professionnel</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120363/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120311/true/false/true/true</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1570,17 +1562,17 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Conseiller emploi et accompagnement professionnel</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>AFEC (Siège)</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1595,7 +1587,7 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 1140 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1610,12 +1602,12 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1630,12 +1622,12 @@
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>0153368844</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>0153368844</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -1656,22 +1648,22 @@
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant des modules d'enseignement et des prestations d'accompagnement. Modules d'enseignement professionnel : - EP1 Accompagnement du développement du jeune enfant (cadre d'intervention, accompagnement à l'autonomie l'enfant) - EP2 Exercer son activité en accueil collectif - EP3 Exercer son activité en accueil individuel Modules d'enseignements généraux : - Prévention santé environnement - Enseignements généraux (Mathématiques et sciences, Histoire-Géographie-Citoyenneté et français) En complément de la formation : - Remise à niveau numérique - Techniques de recherche d'emploi et de stage - Accompagnement au retour à l'emploi 3 Stages en entreprise 14 semaines | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>10 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de conseiller emploi et évolution professionnelle ; Projet 2 - Accompagnez en parallèle de nombreuses personnes avec des besoins différents ; Projet 3 - Élaborez une veille et analysez le marché de l'emploi ; Projet 4 - Réalisez un diagnostic et co-construisez un plan d'action avec vos bénéficiaires ; Projet 5 - Adaptez votre posture pour l'accompagnement des bénéficiaires ; Projet 6 - Établissez et validez un projet d'accompagnement professionnel ; Projet 7 - Établissez un plan d'action et un bilan professionnel ; Projet 8 - Concevez un atelier sur les métiers émergents avec l'IA ; Projet 9 - Développez votre projet territorial avec des partenaires ; Projet 10 - Élaborez votre boîte à outils pour accompagner vers l'emploi. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
         </is>
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Conseiller emploi et accompagnement professionnel</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124191/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120363/true/false/true/true</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1683,32 +1675,32 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Accompagnement vers emploi et vers la formation - Ecole de la 2ème chance</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>1ère Ecole de la Deuxième Chance de Normandie : E2C - Site Herouville-St-Clair (E2C NORMANDIE - Centre de formation d'insertion professionnelle)</t>
+          <t>AFEC (Siège)</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>14200 Hérouville-Saint-Clair</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>717 Boulevard de la Grande Delle | 14200 Hérouville-Saint-Clair | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1210 heures (dont 560 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1718,17 +1710,17 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>https://www.e2cnormandie.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>contact@e2cnormandie.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>contact@e2cnormandie.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1743,40 +1735,48 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>0261670985</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>0261670985</t>
-        </is>
-      </c>
-      <c r="O11" s="7" t="inlineStr"/>
+          <t>0153368844</t>
+        </is>
+      </c>
+      <c r="O11" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>Ateliers et actions de construction et réalisation du projet professionnel.orientation pro, techniques de recherche d'emploi, réseau, coaching, visite d'entreprise, journées métier, job-dating, forums, plateaux techniques...Ateliers, actions et projets de développement des compétences socioprofessionnelles | employabilité (ouverture social, culturelle et sportive, citoyenneté, communication professionnelle orale, écrite, numérique, raisonnement logique...Alternance : 6 stages de 2 à 4 semaines, toutes les 3 semaines (50% du temps de formation) | Organisme | 1ère Ecole de la Deuxième Chance de Normandie : E2C - Site Herouville-St-Clair (E2C NORMANDIE - Centre de formation d'insertion professionnelle) | Lieu de la formation | 717 Boulevard de la Grande Delle</t>
-        </is>
-      </c>
-      <c r="T11" s="7" t="inlineStr"/>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant des modules d'enseignement et des prestations d'accompagnement. Modules d'enseignement professionnel : - EP1 Accompagnement du développement du jeune enfant (cadre d'intervention, accompagnement à l'autonomie l'enfant) - EP2 Exercer son activité en accueil collectif - EP3 Exercer son activité en accueil individuel Modules d'enseignements généraux : - Prévention santé environnement - Enseignements généraux (Mathématiques et sciences, Histoire-Géographie-Citoyenneté et français) En complément de la formation : - Remise à niveau numérique - Techniques de recherche d'emploi et de stage - Accompagnement au retour à l'emploi 3 Stages en entreprise 14 semaines | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+        </is>
+      </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10825210/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124191/true/false/true/true</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1788,32 +1788,32 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
+          <t>Accompagnement vers emploi et vers la formation - Ecole de la 2ème chance</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>1ère Ecole de la Deuxième Chance de Normandie : E2C - Site Herouville-St-Clair (E2C NORMANDIE - Centre de formation d'insertion professionnelle)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>14200 Hérouville-Saint-Clair</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>717 Boulevard de la Grande Delle | 14200 Hérouville-Saint-Clair | France</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 1210 heures (dont 560 heures en entreprise)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1823,17 +1823,17 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://www.e2cnormandie.fr/</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>contact@e2cnormandie.fr</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>contact@e2cnormandie.fr</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1848,40 +1848,40 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0261670985</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0261670985</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr"/>
       <c r="P12" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q12" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+          <t>Ateliers et actions de construction et réalisation du projet professionnel.orientation pro, techniques de recherche d'emploi, réseau, coaching, visite d'entreprise, journées métier, job-dating, forums, plateaux techniques...Ateliers, actions et projets de développement des compétences socioprofessionnelles | employabilité (ouverture social, culturelle et sportive, citoyenneté, communication professionnelle orale, écrite, numérique, raisonnement logique...Alternance : 6 stages de 2 à 4 semaines, toutes les 3 semaines (50% du temps de formation) | Organisme | 1ère Ecole de la Deuxième Chance de Normandie : E2C - Site Herouville-St-Clair (E2C NORMANDIE - Centre de formation d'insertion professionnelle) | Lieu de la formation | 717 Boulevard de la Grande Delle</t>
         </is>
       </c>
       <c r="T12" s="5" t="inlineStr"/>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10825210/true/false/false/false</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-13&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-14&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-07-30
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,32 +714,32 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Jardinier, Jardinière paysagiste (CAPA) [HSP 1er NQ]</t>
+          <t>Titre professionnel secrétaire assistant médico-administratif (FOAD)</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>CENTRE DE FORMATION PROFESSIONNELLE ET DE PROMOTION AGRICOLES (CFPPA L'OISELLERIE)</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>17100 Saint-Georges-des-Coteaux</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>EPLEFPA DE SAINTONGE - LEGTA GEORGES DESCLAUDE - SAINTES | Rue Georges Desclaude BP 20550 | 17100 Saint-Georges-des-Coteaux | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1220 heures (dont 420 heures en entreprise)</t>
+          <t>Durée de 1084 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
@@ -749,17 +749,17 @@
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>http://www.epl-charente.com/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr">
         <is>
-          <t>cfppa.angouleme@educagri.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>cfppa.angouleme@educagri.fr | sylvie.cousin@educagri.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K2" s="5" t="inlineStr">
@@ -774,12 +774,12 @@
       </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
-          <t>0616662134</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>0616662134</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O2" s="5" t="inlineStr">
@@ -789,33 +789,33 @@
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R2" s="5" t="inlineStr"/>
       <c r="S2" s="5" t="inlineStr">
         <is>
-          <t>Agir dans des situation de la vie courante à l'aide de repères sociaux (CG1) - - Prendre position dans une situation à caractère social et civique- Utiliser des outils dans des situations de la vie courante - 56 hMettre en oeuvre des actions contribuant à la construction personnelle (CG2) - - S'exprimer à travers une réalisation personnelle- Adopter des comportements favorisant son équilibre personnel - 56 hInteragir avec son environnement social (CG3) - - Adapter son langage et son comportement aux situations de communication- S'approprier les normes et cadres de référence d'un collectif - 49 hRéaliser en sécurité des travaux d'entretien paysager (CP4) - - Entretenir la végétation- Réaliser l'entretien des installations et des infrastructures paysagères - 189 hRéaliser en sécurité des travaux d'aménagement paysager (CP5) - - Réaliser des travaux de mise en place des végétaux- Réaliser des travaux de mise en place d'installations et d'infrastructures paysagères - 196 hEffectuer des travaux liés à l'entretien courant des matériels et équipements (CP6) - - Réaliser des opérations de maintenance conditionnelle des matériels et équipements- Réaliser des opérations de maintenance corrective des matériels et équipements - 147 hS'adapter à des enjeux professionnels locaux (CP7) - Pour le département 16, UCARE "Bassin de rétention" : Mettre en oeuvre un bassin de rétention- Entretenir un bassin de rétentionPour le département 17, UCARE "Corridors-Abris Faune" :Réaliser la mise en place de corridors écologiques et abris petite faune ( 70H) - 105 hSensibilisation Priorités Régionales - Identifier les enjeux du dérèglement climatique et proposer des alternatives : - Climat- Renaissance écologiqueSensibilisation aux valeurs de la république (référentiel ANCT) :Valeurs de la république et laïcité-Non discriminationSe questionner sur les impacts environnementaux du numérique, apprendre à mesurer, décrypter et agir, pour trouver sa place de citoyen dans un monde numérique.MOOC-L'identité numérique enjeux pour le citoyen (RGPD, Réseaux sociaux, - 35 hBilans - Intermédiaire et Final - 7 h | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>7 projets professionnalisants vous permettront d'acquérir les compétences citées au dessus par la pratique.Vous réaliserez les projets suivants :P1 - Démarrez votre formation de secrétaire assistant médico-administratifP2 - Niveau 1 : Maîtrisez l'accueil et la gestion administrative en milieu médicalP3 - Niveau 2 : Développez vos compétences en rédaction, communication et outils numériques en milieuP4 - Réalisez votre mission en entrepriseP5 - Niveau 3 : Optimisez l'organisation, la sécuritéet la gestion des données sensibles en milieu médicalP6 - Niveau 4 : Améliorez la gestion des communications, données et environnements sanitairesP7 - Préparez votre fin de formation de secrétaire assistant médico-administratif | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T2" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP agricole jardinier paysagiste</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel secrétaire assistant médico-administratif</t>
         </is>
       </c>
       <c r="U2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910478/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/true</t>
         </is>
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,32 +827,32 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Horticulteur, horticultrice (CAPA) [HSP 1er NQ]</t>
+          <t>Formation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>CENTRE DE FORMATION PROFESSIONNELLE ET DE PROMOTION AGRICOLES (CFPPA L'OISELLERIE)</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>17100 Saintes</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>EPLEFPA DE SAINTONGE - LEGTA GEORGES DESCLAUDE - SAINTES | BP 70528 LYCEE HORTICOLE LE PETIT CHADIGNAC | 17100 Saintes | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1220 heures (dont 420 heures en entreprise)</t>
+          <t>Durée de 346 heures</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
@@ -862,17 +862,17 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>http://www.epl-charente.com/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>cfppa.angouleme@educagri.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>cfppa.angouleme@educagri.fr | sylvie.cousin@educagri.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
@@ -887,48 +887,40 @@
       </c>
       <c r="M3" s="7" t="inlineStr">
         <is>
-          <t>0616662134</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr">
         <is>
-          <t>0616662134</t>
-        </is>
-      </c>
-      <c r="O3" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0180888030</t>
+        </is>
+      </c>
+      <c r="O3" s="7" t="inlineStr"/>
       <c r="P3" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q3" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R3" s="7" t="inlineStr"/>
       <c r="S3" s="7" t="inlineStr">
         <is>
-          <t>Agir dans des situation de la vie courante à l'aide de repères sociaux ( CG1) - - Prendre position dans une situation à caractère social et civique- Utiliser des outils dans des situations de la vie courante - 56 hMettre en oeuvre des actions contribuant à la construction personnelle (CG2) - - S'exprimer à travers une réalisation personnelle- Adopter des comportements favorisant son équilibre personnel - 56 hInteragir avec son environnement social (CG3) - - Adapter son langage et son comportement aux situations decommunication- S'approprier les normes et cadres de référence d'un collectif - 49 hRéaliser des travaux sur les végétaux ( CP4) - - Réaliser des observations et interventions sur le végétal- Réaliser des travaux de mise en place des végétaux - 189 hRéaliser des travaux de suivi des cultures de l'implantation à la récolte et au conditionnement ( CP5) - - Réaliser des observations et opérations techniques liées au cycle de production- Effectuer des travaux de récolte, de conservation et de conditionnement - 196 hEffectuer des travaux liés à l'entretien courant des matériels , équipements, installations et bâtiments (CP6) - - Réaliser des opérations de maintenance conditionnelle des matériels, équipements, installations et bâtiments- Effectuer des travaux simples d'aménagement et de réparation - 147 hS'adapter à des enjeux professionnels locaux (CP7) - Pour le département 16, UCARE "Vente et commercialisation de produits horticoles" : Accueillir les clients- Vendre directement les produits de l'atelierPour le département 17, UCARE "Initiation aux travaux viticoles" : Préparer les principaux travaux liés au vignoble. Réaliser les travaux liés au vignoble - 105 hSensibilisation Priorités Régionales - Identifier les enjeux du dérèglement climatique et proposer des alternatives : - Climat- Renaissance écologiqueSensibilisation aux valeurs de la république (référentiel ANCT) :Valeurs de la république et laïcité-Non discriminationSe questionner sur les impacts environnementaux du numérique, apprendre à mesurer, décrypter et agir, pour trouver sa place de citoyen dans un monde numérique.MOOC-L'identité numérique enjeux pour le citoyen (RGPD, Réseaux sociaux, - 35 hBilans - Intermédiaire et Final - 7 | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T3" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP agricole métiers de l'agriculture</t>
-        </is>
-      </c>
+          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T3" s="7" t="inlineStr"/>
       <c r="U3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910483/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/true</t>
         </is>
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -940,32 +932,32 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Conseiller, Conseillère de vente (TP) [HSP 1er NQ]</t>
+          <t>Concours d'atsem (FOAD)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>17300 Rochefort</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>AFPA ROCHEFORT | 57 Avenue BERNADOTTE | 17300 Rochefort | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -975,17 +967,17 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-rochefort@afpa.fr | lisa.perrotin@afpa.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -1000,48 +992,40 @@
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>0699077417</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>0699077417 | 0616046682</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr"/>
       <c r="P4" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q4" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R4" s="5" t="inlineStr"/>
       <c r="S4" s="5" t="inlineStr">
         <is>
-          <t>Période d'intégration CV - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hM1 - Contribuer à l'efficacité commerciale d'une unité marchande dans un environnement omnicanal - Connaître les différents contextes de la vente de services et de produitsConnaître les fondamentaux de la démarche marketingMener une étude de marché et établir le diagnostic de l'unité marchandeConnaître les différentes techniques et méthodes d'approvisionnementRéaliser des inventairesAppliquer les règles et les obligations légales du recyclage, du tri sélectif des déchets et de la réduction du gaspillageComprendre les règles de merchandisingMettre en place une opération commercialeSuivre et analyser les évolutions et exploiter les résultats pour proposer des ajustements - 245 hPériode en entreprise 1 - Se confronter à la réalité professionnelleMettre en application des acquisDévelopper des compétences transverses Etablir un réseau favorisant l'insertion professionnelle - 140 hM2 - Améliorer l'expérience client dans un environnement omnicanal - Comprendre l'évolution du digital et son impact sur le métierValoriser l'offre de produits et de services de l'unité marchande sur les sites marchands et les médias sociauxAccueillir le client et mettre en oeuvre des conditions favorables à l'accueil des personnes en situation de handicapProcéder à l'enregistrement et à l'encaissementConnaître le cadre juridique de la vente et les enjeux du suivi de la relation commercialeConnaître les fondamentaux de la démarche marketingS'approprier et défendre les principes majeurs de l'écocitoyenneté tout au long de l'expérience d'achat - 210 hPériode en entreprise 2 - Se confronter à la réalité professionnelle Mettre en application des acquis Renforcer ses compétences transverses Développer son réseau professionnel - 140 hPériode de certification - Certification Conseiller de vente - 35 hSensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du dé | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T4" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller de vente</t>
-        </is>
-      </c>
+          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr"/>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910492/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
         </is>
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1053,32 +1037,32 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Conseiller, Conseillère commercial (TP) [HSP 1er NQ]</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>17000 La Rochelle</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>AXYS | 33 Rue DU REMPART ST CLAUDE | 17000 La Rochelle | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1088,17 +1072,17 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | axysetien@orange.fr | axystayeb@orange.fr</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
@@ -1113,12 +1097,12 @@
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>0546411640</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>0546411640 | 0679890571</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="O5" s="7" t="inlineStr">
@@ -1128,33 +1112,33 @@
       </c>
       <c r="P5" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R5" s="7" t="inlineStr"/>
       <c r="S5" s="7" t="inlineStr">
         <is>
-          <t>TP CC - Période d'intégration Conseiller commercial - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hTP CC - Module 1 Prospecter un secteur de vente - Assurer une veille professionnelle et commercialeMettre en oeuvre un plan d'actions commerciales et organiser son activitéProspecter à distanceProspecter physiquementAnalyser ses performances commerciales et en rendre compte - 280 hTP CC - Période Entreprise CCP1 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP CC - Module 2 Vendre en face à face des produits et des services référencés aux entreprises et aux particuliers - Représenter l'entreprise et valoriser son imageConduire un entretien de venteAssurer le suivi de ses ventesFidéliser son portefeuille client - 280 hTP CC - Période Entreprise CCP2 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP CC - Période de synthèse du parcours professionnel - Analyse de ses apprentissagesFinalisation de son dossier professionnelPréparation de la session de validation - 35 hTP CC - Période de certification - Certification Conseiller Commercial - 35 hTP CC - Sensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa propre empreinte écologique / prendre conscience de son propre impact (quiz, impactco2.fr, fresque du climat...Définir les points de progrès individuels et collectifs applicables dans la vie quotidienne, en formation et dans le milieu professionnel (Intervention d'acteurs locaux type ressourcerie, SIVOM, association de facilitation des mobilités douces, ... - 14 hTP CC - Sensibilisation aux enjeux des valeurs de la république.... - APPREHENDERRecontextualisation du principe de laïcité. Présentation : liber | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller commercial</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910495/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
         </is>
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1166,32 +1150,32 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Employé(e) commercial (TP) [HSP 1er NQ]</t>
+          <t>Préparation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>AFEC</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>17300 Rochefort</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>AFPA ROCHEFORT | 57 Avenue BERNADOTTE | 17300 Rochefort | France</t>
+          <t>AFEC (Siège) | Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -1201,73 +1185,49 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-rochefort@afpa.fr | lisa.perrotin@afpa.fr</t>
-        </is>
-      </c>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr"/>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>france_travail</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>0699077417</t>
-        </is>
-      </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>0699077417 | 0616046682</t>
-        </is>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr"/>
+      <c r="N6" s="5" t="inlineStr"/>
+      <c r="O6" s="5" t="inlineStr"/>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R6" s="5" t="inlineStr"/>
       <c r="S6" s="5" t="inlineStr">
         <is>
-          <t>Période d'intégration Employé Commercial - Intégrer son groupe et sa formation J'apprends à apprendreS'approprier les objectifs de la formation et repérer son futur environnement professionnelPréciser ses besoins de formation et contractualiser son parcours personnaliséS'inscrire dans une perspective d'emploi - 35 hModule 1 Mettre à disposition des clients les produits de l'unité marchande dans un environnement omnicanal - Appliquer les règles et les obligations légales du recyclage, du tri sélectif des déchets et de la réduction du gaspillageRéceptionner et stocker la marchandiseComprendre les règles de merchandisingParticiper à la mise en oeuvre d'une opération commercialeVeiller à la mise en oeuvre des mesures de prévention adaptées à l'hygiène et à la sécuritéTraiter les commandes des clients - 140 hPériode d'application en entreprise 1 - Se confronter à la réalité professionnelleMettre en application des acquisDévelopper des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hModule 2 Accueillir et accompagner le client dans un point de vente - Accueillir les clients et mettre en oeuvre des conditions favorables à l'accueil des personnes en situation de handicapProposer les programmes et services de fidélisation de l'unité marchande et conclure l'entretien de venteTenir un poste de caisse et superviser les caisses libre-serviceComprendre l'évolution du digital et les enjeux de la valorisation de l'expérience d'achat dans un contexte omnicanalValoriser l'image de l'unité marchande en s'appropriant les principes majeurs de l'écocitoyenneté tout au long de l'expérience d'achat - 140 hPériode d'application en entreprise 2 (environnement omnicanal) - Se confronter à la réalité professionnelleMettre en application des acquisRenforcer ses compétences transversesDévelopper son réseau professionnel - 140 hPériode de certification - Certification Employé Commercial - 35 hSensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa propre empreinte écologique / prendre conscience de son propre impact (quiz, impactco2.fr, fresque du climat...Définir les points de progrès individuels et collectifs applicables dans la vie quotidie | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T6" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé commercial</t>
-        </is>
-      </c>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC | Lieu de la formation | AFEC (Siège)</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr"/>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910496/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1279,32 +1239,32 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Conseiller, Conseillère de vente (TP) [HSP 1er NQ]</t>
+          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>17000 La Rochelle</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>AXYS | 33 Rue DU REMPART ST CLAUDE | 17000 La Rochelle | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1314,17 +1274,17 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | axysetien@orange.fr | axystayeb@orange.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
@@ -1339,48 +1299,40 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>0546411640</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>0546411640 | 0679890571</t>
-        </is>
-      </c>
-      <c r="O7" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr"/>
       <c r="S7" s="7" t="inlineStr">
         <is>
-          <t>Période d'intégration CV - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hM1 - Contribuer à l'efficacité commerciale d'une unité marchande dans un environnement omnicanal - Connaître les différents contextes de la vente de services et de produitsConnaître les fondamentaux de la démarche marketingMener une étude de marché et établir le diagnostic de l'unité marchandeConnaître les différentes techniques et méthodes d'approvisionnementRéaliser des inventairesAppliquer les règles et les obligations légales du recyclage, du tri sélectif des déchets et de la réduction du gaspillageComprendre les règles de merchandisingMettre en place une opération commercialeSuivre et analyser les évolutions et exploiter les résultats pour proposer des ajustements - 245 hPériode en entreprise 1 - Se confronter à la réalité professionnelleMettre en application des acquisDévelopper des compétences transverses Etablir un réseau favorisant l'insertion professionnelle - 140 hM2 - Améliorer l'expérience client dans un environnement omnicanal - Comprendre l'évolution du digital et son impact sur le métierValoriser l'offre de produits et de services de l'unité marchande sur les sites marchands et les médias sociauxAccueillir le client et mettre en oeuvre des conditions favorables à l'accueil des personnes en situation de handicapProcéder à l'enregistrement et à l'encaissementConnaître le cadre juridique de la vente et les enjeux du suivi de la relation commercialeConnaître les fondamentaux de la démarche marketingS'approprier et défendre les principes majeurs de l'écocitoyenneté tout au long de l'expérience d'achat - 210 hPériode en entreprise 2 - Se confronter à la réalité professionnelle Mettre en application des acquis Renforcer ses compétences transverses Développer son réseau professionnel - 140 hPériode de certification - Certification Conseiller de vente - 35 hSensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du dé | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T7" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller de vente</t>
-        </is>
-      </c>
+          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T7" s="7" t="inlineStr"/>
       <c r="U7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910502/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
         </is>
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1392,32 +1344,32 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Employé(e) commercial (TP) [HSP 1er NQ]</t>
+          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>17000 La Rochelle</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>AXYS | 33 Rue DU REMPART ST CLAUDE | 17000 La Rochelle | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -1427,17 +1379,17 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | axysetien@orange.fr | axystayeb@orange.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1452,48 +1404,40 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>0546411640</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>0546411640 | 0679890571</t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr"/>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q8" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>Période d'intégration Employé Commercial - Intégrer son groupe et sa formation J'apprends à apprendreS'approprier les objectifs de la formation et repérer son futur environnement professionnelPréciser ses besoins de formation et contractualiser son parcours personnaliséS'inscrire dans une perspective d'emploi - 35 hModule 1 Mettre à disposition des clients les produits de l'unité marchande dans un environnement omnicanal - Appliquer les règles et les obligations légales du recyclage, du tri sélectif des déchets et de la réduction du gaspillageRéceptionner et stocker la marchandiseComprendre les règles de merchandisingParticiper à la mise en oeuvre d'une opération commercialeVeiller à la mise en oeuvre des mesures de prévention adaptées à l'hygiène et à la sécuritéTraiter les commandes des clients - 140 hPériode d'application en entreprise 1 - Se confronter à la réalité professionnelleMettre en application des acquisDévelopper des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hModule 2 Accueillir et accompagner le client dans un point de vente - Accueillir les clients et mettre en oeuvre des conditions favorables à l'accueil des personnes en situation de handicapProposer les programmes et services de fidélisation de l'unité marchande et conclure l'entretien de venteTenir un poste de caisse et superviser les caisses libre-serviceComprendre l'évolution du digital et les enjeux de la valorisation de l'expérience d'achat dans un contexte omnicanalValoriser l'image de l'unité marchande en s'appropriant les principes majeurs de l'écocitoyenneté tout au long de l'expérience d'achat - 140 hPériode d'application en entreprise 2 (environnement omnicanal) - Se confronter à la réalité professionnelleMettre en application des acquisRenforcer ses compétences transversesDévelopper son réseau professionnel - 140 hPériode de certification - Certification Employé Commercial - 35 hSensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa propre empreinte écologique / prendre conscience de son propre impact (quiz, impactco2.fr, fresque du climat...Définir les points de progrès individuels et collectifs applicables dans la vie quotidie | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T8" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé commercial</t>
-        </is>
-      </c>
+          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910505/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
         </is>
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1505,32 +1449,32 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Commis de cuisine (TP) [HSP 1er NQ]</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>CENTRE DE FORMATION FARE 16-ROC FLEURI (FARE 16)</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>17300 Rochefort</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>AFPA ROCHEFORT | 57 Avenue BERNADOTTE | 17300 Rochefort | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 1350 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1540,17 +1484,17 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>https://fare16.cneap.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>comptable.fare16@cneap.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>comptable.fare16@cneap.fr | formations-rochefort@afpa.fr | lisa.perrotin@afpa.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
@@ -1565,12 +1509,12 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>0699077417</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>0699077417 | 0616046682</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O9" s="7" t="inlineStr">
@@ -1580,33 +1524,33 @@
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R9" s="7" t="inlineStr"/>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>Positionnement Accompagnement socio-professionnel générique - Réalisation de diagnosticsDéfinition du parcours individualiséIdentification des freins Bilan intermédiaire et final - 63 hCAP Organisation de la production de cuisine UP1 - -Réceptionner, contrôler et stocker les marchandises dans le respect de la réglementation en vigueur et en appliquant les techniques de prévention liées à l'activité- Collecter l'ensemble des informations et organiser sa production culinaire dans le respect des consignes et de temps imparti - 105 hCAP Réalisation de la production de cuisine UP2 - - Préparer, organiser et maintenir en état son poste de travail tout au long de l'activité dans le respect de la réglementation en vigueur- Maîtriser les techniques culinaires de base et réaliser une production dans le respect des consignes et des règles d'hygiène et de sécurité- Analyser, contrôler la qualité de sa production, dresser et participer à la distribution selon le contexte professionnel- Communiquer en fonction du contexte professionnel et en respectant les usages de la profession - 336 hCAP Prévention-santé-environnement UP3 - - Appliquer une méthode d'analyse d'une situation de la vie professionnelle ou quotidienne et d'une documentation- Mettre en relation un phénomène physiologique, un enjeu environnemental, une disposition réglementaire, avec une mesure de prévention- Proposer une solution pour résoudre un problème lié à la santé, l'environnement ou la consommation et argumenter un choix - Communiquer à l'écrit et à l'oral avec une syntaxe claire et un vocabulaire technique adapté- Agir face à une situation d'urgence - 35 hCAP Français et Histoire-géographie Enseignement moral et civique - - Entrer dans l'échange oral et écrit : écouter, réagir, s'exprimer, lire, analyser, écrire- Devenir un lecteur compétent et critique- Confronter des savoirs et des valeurs pour construire son identité culturelle- Histoire-Géographie et Enseignement moral et civique- Appréhender la diversité des sociétés et la richesse des cultures- Repérer la situation étudiée dans le temps et dans l'espace- Relever, classer et hiérarchiser les informations contenues dans un document selon des critères donnés- Acquérir une démarche citoyenne à partir de son environnement quotidien - 56 hCAP Mathématiques - Physique - Chimie - | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>11 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 : Démarrez votre formation d'Accompagnement Educatif Petite Enfance ; Projet 2 - Préparez un environnement sécurisé pour le jeune enfant ; Projet 3 - Développez des activités éducatives adaptées à la petite enfance ; Projet 4 - Appliquez les protocoles de santé dans le cadre de la petite enfance ; Projet 5 - Soutenez le personnel enseignant dans un contexte collectif ; Projet 6 - Améliorez les conditions d'accueil en école maternelle ; Projet 7 - Organisez l'accueil individuel au domicile ; Projet 8 - Gérez les tâches domestiques et la préparation des repas pour l'enfant ; Projet 9 : Proposer des solutions de prévention, santé et environnement ; Projet 10 : Remise à niveau scolaire ; Projet 11 : Préparez-vous pour l'examen final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel commis de cuisine</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10919965/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120311/true/false/true/true</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1618,32 +1562,32 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Serveur, Serveuse en hôtellerie-restauration (TP) [HSP 1er NQ]</t>
+          <t>Conseiller emploi et accompagnement professionnel</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>CENTRE DE FORMATION FARE 16-ROC FLEURI (FARE 16)</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>17300 Rochefort</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>AFPA ROCHEFORT | 57 Avenue BERNADOTTE | 17300 Rochefort | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 1140 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1653,17 +1597,17 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>https://fare16.cneap.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>comptable.fare16@cneap.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>comptable.fare16@cneap.fr | formations-rochefort@afpa.fr | lisa.perrotin@afpa.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1678,12 +1622,12 @@
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>0699077417</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>0699077417 | 0616046682</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -1693,33 +1637,33 @@
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q10" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>TP Positionnement Accompagnement socio-professionnel générique - Réalisation des diagnosticsDéfinition du parcours individualiséIdentification des freinsBilan intermédiaire et final - 63 hTP Réaliser les travaux préalables au service en restauration - - Nettoyer et entretenir les espaces de restauration et les locaux annexes- Mettre en place les espaces de restauration et les locaux annexes- Mettre en place les différents types de buffet - 126 hTP Accueillir, conseiller le client et prendre sa commande - - Accueillir la clientèle et l'accompagner à sa table- Présenter cartes et menus, prendre la commande et la communiquer aux services concernés - 154 hTP Réaliser le service en restauration - - Préparer et servir les boissons en respectant les règles de service- Effectuer les différents types de service à table et au buffet- Préparer, vérifier une addition et l'encaisser - 154 hTP Règles d'hygiène dans la restauration et les commerces alimentaires - Donner à chaque participant les connaissances d'hygiène nécessaires afin: De produire un travail de qualité- De respecter dans chaque secteur de soin les règles d'hygiène en utilisant convenablement le matériel et les produits d'entretien- Situer et valoriser les responsabilités et le rôle du personnel dans la prévention des infections nosocomiales - 14 hTP Gestes et postures - - Acquérir les compétences nécessaires pour contribuer à la mise en oeuvre de la prévention des risques liés à l'activité physique - 14 hTP Sensibilisation au numérique Responsable - Intégrer les enjeux du numérique dans ses pratiques quotidiennes et professionnelles par :L'hygiène numérique compatible avec une pratique responsableLa santé mentale dans l'utilisation d'internetTerritoire numérique responsableBonnes pratiquesLa cybersécurité dans ses pratiques du numériqueLes types d'attaques et conséquencesUtilisateur modérateur et trace numériqueLiberté numérique et l'utilisation des outilsLe règlement général sur la protection des donnéesTraces et e-réputationSources d'information et règlementation CNILDroits d'utilisation, d'auteur et à l'imag - 14 hTP Sensibilisation aux valeurs de la République - - Participer à une meilleure compréhension des enjeux d'une société fondée sur les vale | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>10 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de conseiller emploi et évolution professionnelle ; Projet 2 - Accompagnez en parallèle de nombreuses personnes avec des besoins différents ; Projet 3 - Élaborez une veille et analysez le marché de l'emploi ; Projet 4 - Réalisez un diagnostic et co-construisez un plan d'action avec vos bénéficiaires ; Projet 5 - Adaptez votre posture pour l'accompagnement des bénéficiaires ; Projet 6 - Établissez et validez un projet d'accompagnement professionnel ; Projet 7 - Établissez un plan d'action et un bilan professionnel ; Projet 8 - Concevez un atelier sur les métiers émergents avec l'IA ; Projet 9 - Développez votre projet territorial avec des partenaires ; Projet 10 - Élaborez votre boîte à outils pour accompagner vers l'emploi. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
         </is>
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel serveur en restauration</t>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Conseiller emploi et accompagnement professionnel</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10919967/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120363/true/false/true/true</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1731,32 +1675,32 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Agent(e) de service médico-social (TP) [HSP 1er NQ]</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>GRETA POITOU-CHARENTES - SIÈGE ADMINISTRATIF</t>
+          <t>AFEC (Siège)</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>17300 Rochefort</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>AFPA ROCHEFORT | 57 Avenue BERNADOTTE | 17300 Rochefort | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1766,17 +1710,17 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>http://www.greta-poitou-charentes.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>commercial.greta.agence-poitiers@ac-poitiers.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>commercial.greta.agence-poitiers@ac-poitiers.fr | formations-rochefort@afpa.fr | lisa.perrotin@afpa.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1791,12 +1735,12 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>0699077417</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>0699077417 | 0616046682</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="O11" s="7" t="inlineStr">
@@ -1806,33 +1750,33 @@
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>Bloc de compétences 1 - Réaliser le nettoyage et le bio nettoyage des locaux en s'adaptant à la présence des résidents - Participer à la vie de l'établissementAppliquer les techniques professionnelles d'entretien des locaux dans les espaces communs, la chambre du résident, la salle de bain dans le respect de la présence des résidentsUtiliser les produits, matériels, protocoles, en se protégeant et en protégeant les autres Gérer le temps de son interventionS'organiser et gérer des stocksComprendre la notion de développement durable et l'intégrer dans son activité professionnelle au quotidien - 147 hBloc de compétences 2 - Contribuer aux prestations du service hôtelier en respectant les standards de qualité de l'établissement - Contribuer au service du linge des résidents et de l'établissement, gérer les stocks en lingerieConnaitre et appliquer les moyens de prévention des infections, précautions standards, précautions en cas d'épidémieAssurer la réfection d'un lit inoccupéContribuer au service des repas des résidents, respecter les goûts et consignes, adapter la présentation pour favoriser l'autonomie, préparer la salle à manger dans le respect des normes qualité de l'établissementCommuniquer avec les résidents, respecter leurs habitudes et autonomie - 98 hBloc de compétences 3 - Accompagner le résident dans les gestes de la vie quotidienne en tenant compte du projet - Accompagner le résident dans ses déplacementsAccompagner le résident à prendre son repas et à boireAppréhender les incidences des pathologies, handicaps et déficiences dans la vie quotidienne des résidentsCommuniquer avec l'équipe pluridisciplinaireObserver, écouter et établir des relations avec les résidentsIntervenir dans le respect des gestes de sécurité - 126 hPréparation à la Certification - Accompagner à la rédaction du Dossier ProfessionnelFinaliser les Epreuves en Cours de Formation (ECF)Préparer à l'épreuve finalePréparer à l'entretien final - 35 hLes périodes de formation en milieu professionnel (PFMP) - Les PFMP permettent de mettre en oeuvre ou d'acquérir des compétences sous la responsabilité d'une personne qualifiée (tuteur-trice) et d'apprendre à travailler en situation réelle avec les moyens et contraintes du milieu professionnel.L'alternance centre/entreprise répond à une progression péda | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant des modules d'enseignement et des prestations d'accompagnement. Modules d'enseignement professionnel : - EP1 Accompagnement du développement du jeune enfant (cadre d'intervention, accompagnement à l'autonomie l'enfant) - EP2 Exercer son activité en accueil collectif - EP3 Exercer son activité en accueil individuel Modules d'enseignements généraux : - Prévention santé environnement - Enseignements généraux (Mathématiques et sciences, Histoire-Géographie-Citoyenneté et français) En complément de la formation : - Remise à niveau numérique - Techniques de recherche d'emploi et de stage - Accompagnement au retour à l'emploi 3 Stages en entreprise 14 semaines | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de service médico-social</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10920021/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124191/true/false/true/true</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1844,12 +1788,12 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Action préparatoire aux métiers de l'agriculture [HSP 1er NQ]</t>
+          <t>Jardinier, Jardinière paysagiste (CAPA) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -1859,17 +1803,17 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>16200 Triac-Lautrait</t>
+          <t>17100 Saint-Georges-des-Coteaux</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>MAISON FAMILIALE RURALE D'ÉDUCATION ET D'ORIENTATION TRIAC LAUTRAIT | 16 Route DE COGNAC | 16200 Triac-Lautrait | France</t>
+          <t>EPLEFPA DE SAINTONGE - LEGTA GEORGES DESCLAUDE - SAINTES | Rue Georges Desclaude BP 20550 | 17100 Saint-Georges-des-Coteaux | France</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1220 heures (dont 420 heures en entreprise)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1889,7 +1833,7 @@
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>cfppa.angouleme@educagri.fr | eric.verger@mfr.asso.fr</t>
+          <t>cfppa.angouleme@educagri.fr | sylvie.cousin@educagri.fr</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1904,15 +1848,19 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>0545353771</t>
+          <t>0616662134</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>0545353771</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="inlineStr"/>
+          <t>0616662134</t>
+        </is>
+      </c>
+      <c r="O12" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P12" s="5" t="inlineStr">
         <is>
           <t>Formation financée par la région</t>
@@ -1926,18 +1874,22 @@
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>Découverte des filières et des métiers - Découverte de l'activité professionnelle agricole sur le territoire : Spécificités, filières, métiers... (visites d'exploitations, interventions de professionnels) Les activités agricoles et leur saisonnalité- L'emploi agricole sur le territoire (intervention de partenaires emploi agricole) Les métiers : matériel et risques professionnels - 42 hElaboration du projet professionnel - Définir sa (ses) filière(s) :Le projet initial : Explicitation du projet et ses représentations par chaque candidatDécouvrir et se tester en situation : Visites- Travaux Pratiques en ateliers pédagogiquesChoix de filière : 1 à 3 pour répartir les immersions en stage en entrepriseAccompagnement vers les stages : Cartographie- Mobilité- Candidature (CV, Entretien,LM... Accompagnement personnalisé - 56 hConsolidation et concrétisation du projet professionnel - - Détermination du choix de filière, suite aux immersion : Représentation et explicitation des activités- Consolidation du projet : Projection dans l'activité, besoins (savoir, savoir-être, formations... Technique de Recherche d'Emploi (TRE) et accompagnement vers l'emploi/formation (selon projet personnel) : Présentation de son projet (personnel, professionnel, formation) Identification des compétences (acquises et à acquérir) accompagnement individualisé- Définir son besoin des compétences et les étapes de son projet (formation, emploi) déterminer un "tableau de bord" de projet - 56 hAcquisition des compétences nécessaires à l'intégration professionnelle - - Compétences sociales et civiques : lister les compétences nécessaires, la non discrimination (genre, génération, catégorie socio-pro... intégration en milieu professionnel- Savoir-être, aptitudes professionnelles (attitude et posture) : Communication, savoir explicité son activité, ponctualité, initiative, autonomie, écoute... Santé et sécurité au travail : Identification des facteurs de risques professionnels et adapter/adopter des comportements pour préserver sa santé et celle d'autrui - 49 hIdentification des freins, Accompagnent Socio Pro - Validation par le stagiaire de sa capacité à intégrer une formation/emploiIdentification des freins au projet : mobilité, financiers, handicap, socio, logement, restauration, addiction...Accompagnement personnalisé à la levée des | Organisme | CENTRE DE FORMATION PROFESSIONNELLE ET DE PROMOTION AGRICOLES (CFPPA L'OISELLERIE) | http://www.epl-charente.com | Lieu de la formation</t>
-        </is>
-      </c>
-      <c r="T12" s="5" t="inlineStr"/>
+          <t>Agir dans des situation de la vie courante à l'aide de repères sociaux (CG1) - - Prendre position dans une situation à caractère social et civique- Utiliser des outils dans des situations de la vie courante - 56 hMettre en oeuvre des actions contribuant à la construction personnelle (CG2) - - S'exprimer à travers une réalisation personnelle- Adopter des comportements favorisant son équilibre personnel - 56 hInteragir avec son environnement social (CG3) - - Adapter son langage et son comportement aux situations de communication- S'approprier les normes et cadres de référence d'un collectif - 49 hRéaliser en sécurité des travaux d'entretien paysager (CP4) - - Entretenir la végétation- Réaliser l'entretien des installations et des infrastructures paysagères - 189 hRéaliser en sécurité des travaux d'aménagement paysager (CP5) - - Réaliser des travaux de mise en place des végétaux- Réaliser des travaux de mise en place d'installations et d'infrastructures paysagères - 196 hEffectuer des travaux liés à l'entretien courant des matériels et équipements (CP6) - - Réaliser des opérations de maintenance conditionnelle des matériels et équipements- Réaliser des opérations de maintenance corrective des matériels et équipements - 147 hS'adapter à des enjeux professionnels locaux (CP7) - Pour le département 16, UCARE "Bassin de rétention" : Mettre en oeuvre un bassin de rétention- Entretenir un bassin de rétentionPour le département 17, UCARE "Corridors-Abris Faune" :Réaliser la mise en place de corridors écologiques et abris petite faune ( 70H) - 105 hSensibilisation Priorités Régionales - Identifier les enjeux du dérèglement climatique et proposer des alternatives : - Climat- Renaissance écologiqueSensibilisation aux valeurs de la république (référentiel ANCT) :Valeurs de la république et laïcité-Non discriminationSe questionner sur les impacts environnementaux du numérique, apprendre à mesurer, décrypter et agir, pour trouver sa place de citoyen dans un monde numérique.MOOC-L'identité numérique enjeux pour le citoyen (RGPD, Réseaux sociaux, - 35 hBilans - Intermédiaire et Final - 7 h | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T12" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP agricole jardinier paysagiste</t>
+        </is>
+      </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10904504/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10910478/true/false/false/true</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -1949,12 +1901,12 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Viticulteur, Viticultrice (CAPA) [HSP 1er NQ]</t>
+          <t>Horticulteur, horticultrice (CAPA) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -1964,17 +1916,17 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>16400 La Couronne</t>
+          <t>17100 Saintes</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>28 Allee de l Oisellerie | 16400 La Couronne | France</t>
+          <t>EPLEFPA DE SAINTONGE - LEGTA GEORGES DESCLAUDE - SAINTES | BP 70528 LYCEE HORTICOLE LE PETIT CHADIGNAC | 17100 Saintes | France</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1239 heures (dont 399 heures en entreprise)</t>
+          <t>Durée de 1220 heures (dont 420 heures en entreprise)</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1994,7 +1946,7 @@
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>cfppa.angouleme@educagri.fr | karine.durand@educagri.fr</t>
+          <t>cfppa.angouleme@educagri.fr | sylvie.cousin@educagri.fr</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
@@ -2009,12 +1961,12 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>0545673695</t>
+          <t>0616662134</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>0545673695</t>
+          <t>0616662134</t>
         </is>
       </c>
       <c r="O13" s="7" t="inlineStr">
@@ -2035,7 +1987,7 @@
       <c r="R13" s="7" t="inlineStr"/>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>Agir dans des situation de la vie courante à l'aide de repères sociaux (CG1) - - Prendre position dans une situation à caractère social et civique- Utiliser des outils dans des situations de la vie courante - 56 hMettre en oeuvre des actions contribuant à la construction personnelle (CG2) - - S'exprimer à travers une réalisation personnelle- Adopter des comportements favorisant son équilibre personnel - 56 hInteragir avec son environnement social (CG3) - - Adapter son langage et son comportement aux situations de communication- S'approprier les normes et cadres de référence d'un collectif - 49 hRéaliser des travaux sur les végétaux (CP4) - - Réaliser des observations et interventions sur le végétal- Réaliser des travaux de mise en place des végétaux - 189 hRéaliser des travaux de suivi des cultures de l'implantation à la récolte et au conditionnement (CP5) - - Réaliser des observations et opérations techniques liées au cycle de production- Effectuer des travaux de récolte, de conservation *et de conditionnement* (pour Arboriculture et Horticulture) - 196 hEffectuer des travaux liés à l'entretien courant des matériels, équipements, installations et bâtiments (CP6) - - Réaliser des opérations de maintenance conditionnelle des matériels, équipements, installations et bâtiments- Effectuer des travaux simples d'aménagement et de réparation - 147 hParticiper à la distillation charentaise (CP7) - - Réaliser un vin de chaudière- Participer à la distillation charentaise - 105 hSensibilisation Priorités Régionales - Identifier les enjeux du dérèglement climatique et proposer des alternatives : - Climat- Renaissance écologiqueSensibilisation aux valeurs de la république (référentiel ANCT) :Valeurs de la république et laïcité-Non discriminationSe questionner sur les impacts environnementaux du numérique, apprendre à mesurer, décrypter et agir, pour trouver sa place de citoyen dans un monde numérique.MOOC-L'identité numérique enjeux pour le citoyen (RGPD, Réseaux sociaux, - 35 hBilans - Intermédiaire et Final - 7 h | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Agir dans des situation de la vie courante à l'aide de repères sociaux ( CG1) - - Prendre position dans une situation à caractère social et civique- Utiliser des outils dans des situations de la vie courante - 56 hMettre en oeuvre des actions contribuant à la construction personnelle (CG2) - - S'exprimer à travers une réalisation personnelle- Adopter des comportements favorisant son équilibre personnel - 56 hInteragir avec son environnement social (CG3) - - Adapter son langage et son comportement aux situations decommunication- S'approprier les normes et cadres de référence d'un collectif - 49 hRéaliser des travaux sur les végétaux ( CP4) - - Réaliser des observations et interventions sur le végétal- Réaliser des travaux de mise en place des végétaux - 189 hRéaliser des travaux de suivi des cultures de l'implantation à la récolte et au conditionnement ( CP5) - - Réaliser des observations et opérations techniques liées au cycle de production- Effectuer des travaux de récolte, de conservation et de conditionnement - 196 hEffectuer des travaux liés à l'entretien courant des matériels , équipements, installations et bâtiments (CP6) - - Réaliser des opérations de maintenance conditionnelle des matériels, équipements, installations et bâtiments- Effectuer des travaux simples d'aménagement et de réparation - 147 hS'adapter à des enjeux professionnels locaux (CP7) - Pour le département 16, UCARE "Vente et commercialisation de produits horticoles" : Accueillir les clients- Vendre directement les produits de l'atelierPour le département 17, UCARE "Initiation aux travaux viticoles" : Préparer les principaux travaux liés au vignoble. Réaliser les travaux liés au vignoble - 105 hSensibilisation Priorités Régionales - Identifier les enjeux du dérèglement climatique et proposer des alternatives : - Climat- Renaissance écologiqueSensibilisation aux valeurs de la république (référentiel ANCT) :Valeurs de la république et laïcité-Non discriminationSe questionner sur les impacts environnementaux du numérique, apprendre à mesurer, décrypter et agir, pour trouver sa place de citoyen dans un monde numérique.MOOC-L'identité numérique enjeux pour le citoyen (RGPD, Réseaux sociaux, - 35 hBilans - Intermédiaire et Final - 7 | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T13" s="7" t="inlineStr">
@@ -2045,12 +1997,12 @@
       </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910457/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10910483/true/false/false/true</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W13" s="7" t="inlineStr">
@@ -2062,12 +2014,12 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Conseiller, Conseillère commercial (TP) [HSP 1er NQ]</t>
+          <t>Conseiller, Conseillère de vente (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -2077,12 +2029,12 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>16600 Magnac-sur-Touvre</t>
+          <t>17300 Rochefort</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>ASSOCIATION NATIONALE POUR LA FORMATION PROFESSIONNELLE DES ADULTES | 104 Route Lac Melot Zone la Braconne | 16600 Magnac-sur-Touvre | France</t>
+          <t>AFPA ROCHEFORT | 57 Avenue BERNADOTTE | 17300 Rochefort | France</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -2107,7 +2059,7 @@
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-angouleme@afpa.fr | marion.lesueur@afpa.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-rochefort@afpa.fr | lisa.perrotin@afpa.fr</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -2122,12 +2074,12 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>0648579860</t>
+          <t>0699077417</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>0648579860 | 0545658101</t>
+          <t>0699077417 | 0616046682</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -2148,22 +2100,22 @@
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>TP CC - Période d'intégration Conseiller commercial - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hTP CC - Module 1 Prospecter un secteur de vente - Assurer une veille professionnelle et commercialeMettre en oeuvre un plan d'actions commerciales et organiser son activitéProspecter à distanceProspecter physiquementAnalyser ses performances commerciales et en rendre compte - 280 hTP CC - Période Entreprise CCP1 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP CC - Module 2 Vendre en face à face des produits et des services référencés aux entreprises et aux particuliers - Représenter l'entreprise et valoriser son imageConduire un entretien de venteAssurer le suivi de ses ventesFidéliser son portefeuille client - 280 hTP CC - Période Entreprise CCP2 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP CC - Période de synthèse du parcours professionnel - Analyse de ses apprentissagesFinalisation de son dossier professionnelPréparation de la session de validation - 35 hTP CC - Période de certification - Certification Conseiller Commercial - 35 hTP CC - Sensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa propre empreinte écologique / prendre conscience de son propre impact (quiz, impactco2.fr, fresque du climat...Définir les points de progrès individuels et collectifs applicables dans la vie quotidienne, en formation et dans le milieu professionnel (Intervention d'acteurs locaux type ressourcerie, SIVOM, association de facilitation des mobilités douces, ... - 14 hTP CC - Sensibilisation aux enjeux des valeurs de la république.... - APPREHENDERRecontextualisation du principe de laïcité. Présentation : liber | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Période d'intégration CV - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hM1 - Contribuer à l'efficacité commerciale d'une unité marchande dans un environnement omnicanal - Connaître les différents contextes de la vente de services et de produitsConnaître les fondamentaux de la démarche marketingMener une étude de marché et établir le diagnostic de l'unité marchandeConnaître les différentes techniques et méthodes d'approvisionnementRéaliser des inventairesAppliquer les règles et les obligations légales du recyclage, du tri sélectif des déchets et de la réduction du gaspillageComprendre les règles de merchandisingMettre en place une opération commercialeSuivre et analyser les évolutions et exploiter les résultats pour proposer des ajustements - 245 hPériode en entreprise 1 - Se confronter à la réalité professionnelleMettre en application des acquisDévelopper des compétences transverses Etablir un réseau favorisant l'insertion professionnelle - 140 hM2 - Améliorer l'expérience client dans un environnement omnicanal - Comprendre l'évolution du digital et son impact sur le métierValoriser l'offre de produits et de services de l'unité marchande sur les sites marchands et les médias sociauxAccueillir le client et mettre en oeuvre des conditions favorables à l'accueil des personnes en situation de handicapProcéder à l'enregistrement et à l'encaissementConnaître le cadre juridique de la vente et les enjeux du suivi de la relation commercialeConnaître les fondamentaux de la démarche marketingS'approprier et défendre les principes majeurs de l'écocitoyenneté tout au long de l'expérience d'achat - 210 hPériode en entreprise 2 - Se confronter à la réalité professionnelle Mettre en application des acquis Renforcer ses compétences transverses Développer son réseau professionnel - 140 hPériode de certification - Certification Conseiller de vente - 35 hSensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du dé | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller commercial</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller de vente</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910468/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10910492/true/false/false/true</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
@@ -2175,32 +2127,32 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Serveur, Serveuse en hôtellerie-restauration (TP) [HSP 1er NQ]</t>
+          <t>Conseiller, Conseillère commercial (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>CENTRE DE FORMATION FARE 16-ROC FLEURI (FARE 16)</t>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>16710 Saint-Yrieix-sur-Charente</t>
+          <t>17000 La Rochelle</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>14 Allee PIERRE GAULT | 16710 Saint-Yrieix-sur-Charente | France</t>
+          <t>AXYS | 33 Rue DU REMPART ST CLAUDE | 17000 La Rochelle | France</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2210,17 +2162,17 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>https://fare16.cneap.fr/</t>
+          <t>http://www.afpa.fr/</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>comptable.fare16@cneap.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>comptable.fare16@cneap.fr | accueil.fare16@cneap.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | axysetien@orange.fr | axystayeb@orange.fr</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -2235,12 +2187,12 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>0545315917</t>
+          <t>0546411640</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>0545315917</t>
+          <t>0546411640 | 0679890571</t>
         </is>
       </c>
       <c r="O15" s="7" t="inlineStr">
@@ -2261,22 +2213,22 @@
       <c r="R15" s="7" t="inlineStr"/>
       <c r="S15" s="7" t="inlineStr">
         <is>
-          <t>TP Positionnement Accompagnement socio-professionnel générique - Réalisation des diagnosticsDéfinition du parcours individualiséIdentification des freinsBilan intermédiaire et final - 63 hTP Réaliser les travaux préalables au service en restauration - - Nettoyer et entretenir les espaces de restauration et les locaux annexes- Mettre en place les espaces de restauration et les locaux annexes- Mettre en place les différents types de buffet - 126 hTP Accueillir, conseiller le client et prendre sa commande - - Accueillir la clientèle et l'accompagner à sa table- Présenter cartes et menus, prendre la commande et la communiquer aux services concernés - 154 hTP Réaliser le service en restauration - - Préparer et servir les boissons en respectant les règles de service- Effectuer les différents types de service à table et au buffet- Préparer, vérifier une addition et l'encaisser - 154 hTP Règles d'hygiène dans la restauration et les commerces alimentaires - Donner à chaque participant les connaissances d'hygiène nécessaires afin: De produire un travail de qualité- De respecter dans chaque secteur de soin les règles d'hygiène en utilisant convenablement le matériel et les produits d'entretien- Situer et valoriser les responsabilités et le rôle du personnel dans la prévention des infections nosocomiales - 14 hTP Gestes et postures - - Acquérir les compétences nécessaires pour contribuer à la mise en oeuvre de la prévention des risques liés à l'activité physique - 14 hTP Sensibilisation au numérique Responsable - Intégrer les enjeux du numérique dans ses pratiques quotidiennes et professionnelles par :L'hygiène numérique compatible avec une pratique responsableLa santé mentale dans l'utilisation d'internetTerritoire numérique responsableBonnes pratiquesLa cybersécurité dans ses pratiques du numériqueLes types d'attaques et conséquencesUtilisateur modérateur et trace numériqueLiberté numérique et l'utilisation des outilsLe règlement général sur la protection des donnéesTraces et e-réputationSources d'information et règlementation CNILDroits d'utilisation, d'auteur et à l'imag - 14 hTP Sensibilisation aux valeurs de la République - - Participer à une meilleure compréhension des enjeux d'une société fondée sur les vale | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>TP CC - Période d'intégration Conseiller commercial - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hTP CC - Module 1 Prospecter un secteur de vente - Assurer une veille professionnelle et commercialeMettre en oeuvre un plan d'actions commerciales et organiser son activitéProspecter à distanceProspecter physiquementAnalyser ses performances commerciales et en rendre compte - 280 hTP CC - Période Entreprise CCP1 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP CC - Module 2 Vendre en face à face des produits et des services référencés aux entreprises et aux particuliers - Représenter l'entreprise et valoriser son imageConduire un entretien de venteAssurer le suivi de ses ventesFidéliser son portefeuille client - 280 hTP CC - Période Entreprise CCP2 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP CC - Période de synthèse du parcours professionnel - Analyse de ses apprentissagesFinalisation de son dossier professionnelPréparation de la session de validation - 35 hTP CC - Période de certification - Certification Conseiller Commercial - 35 hTP CC - Sensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa propre empreinte écologique / prendre conscience de son propre impact (quiz, impactco2.fr, fresque du climat...Définir les points de progrès individuels et collectifs applicables dans la vie quotidienne, en formation et dans le milieu professionnel (Intervention d'acteurs locaux type ressourcerie, SIVOM, association de facilitation des mobilités douces, ... - 14 hTP CC - Sensibilisation aux enjeux des valeurs de la république.... - APPREHENDERRecontextualisation du principe de laïcité. Présentation : liber | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel serveur en restauration</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller commercial</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910484/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10910495/true/false/false/true</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W15" s="7" t="inlineStr">
@@ -2288,32 +2240,32 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Commis de cuisine (TP) [HSP 1er NQ]</t>
+          <t>Employé(e) commercial (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>CENTRE DE FORMATION FARE 16-ROC FLEURI (FARE 16)</t>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>16710 Saint-Yrieix-sur-Charente</t>
+          <t>17300 Rochefort</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>14 Allee PIERRE GAULT | 16710 Saint-Yrieix-sur-Charente | France</t>
+          <t>AFPA ROCHEFORT | 57 Avenue BERNADOTTE | 17300 Rochefort | France</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2323,17 +2275,17 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>https://fare16.cneap.fr/</t>
+          <t>http://www.afpa.fr/</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>comptable.fare16@cneap.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>comptable.fare16@cneap.fr | accueil.fare16@cneap.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-rochefort@afpa.fr | lisa.perrotin@afpa.fr</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -2348,12 +2300,12 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>0545315917</t>
+          <t>0699077417</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>0545315917</t>
+          <t>0699077417 | 0616046682</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr">
@@ -2374,22 +2326,22 @@
       <c r="R16" s="5" t="inlineStr"/>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>Positionnement Accompagnement socio-professionnel générique - Réalisation de diagnosticsDéfinition du parcours individualiséIdentification des freins Bilan intermédiaire et final - 63 hCAP Organisation de la production de cuisine UP1 - -Réceptionner, contrôler et stocker les marchandises dans le respect de la réglementation en vigueur et en appliquant les techniques de prévention liées à l'activité- Collecter l'ensemble des informations et organiser sa production culinaire dans le respect des consignes et de temps imparti - 105 hCAP Réalisation de la production de cuisine UP2 - - Préparer, organiser et maintenir en état son poste de travail tout au long de l'activité dans le respect de la réglementation en vigueur- Maîtriser les techniques culinaires de base et réaliser une production dans le respect des consignes et des règles d'hygiène et de sécurité- Analyser, contrôler la qualité de sa production, dresser et participer à la distribution selon le contexte professionnel- Communiquer en fonction du contexte professionnel et en respectant les usages de la profession - 336 hCAP Prévention-santé-environnement UP3 - - Appliquer une méthode d'analyse d'une situation de la vie professionnelle ou quotidienne et d'une documentation- Mettre en relation un phénomène physiologique, un enjeu environnemental, une disposition réglementaire, avec une mesure de prévention- Proposer une solution pour résoudre un problème lié à la santé, l'environnement ou la consommation et argumenter un choix - Communiquer à l'écrit et à l'oral avec une syntaxe claire et un vocabulaire technique adapté- Agir face à une situation d'urgence - 35 hCAP Français et Histoire-géographie Enseignement moral et civique - - Entrer dans l'échange oral et écrit : écouter, réagir, s'exprimer, lire, analyser, écrire- Devenir un lecteur compétent et critique- Confronter des savoirs et des valeurs pour construire son identité culturelle- Histoire-Géographie et Enseignement moral et civique- Appréhender la diversité des sociétés et la richesse des cultures- Repérer la situation étudiée dans le temps et dans l'espace- Relever, classer et hiérarchiser les informations contenues dans un document selon des critères donnés- Acquérir une démarche citoyenne à partir de son environnement quotidien - 56 hCAP Mathématiques - Physique - Chimie - | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Période d'intégration Employé Commercial - Intégrer son groupe et sa formation J'apprends à apprendreS'approprier les objectifs de la formation et repérer son futur environnement professionnelPréciser ses besoins de formation et contractualiser son parcours personnaliséS'inscrire dans une perspective d'emploi - 35 hModule 1 Mettre à disposition des clients les produits de l'unité marchande dans un environnement omnicanal - Appliquer les règles et les obligations légales du recyclage, du tri sélectif des déchets et de la réduction du gaspillageRéceptionner et stocker la marchandiseComprendre les règles de merchandisingParticiper à la mise en oeuvre d'une opération commercialeVeiller à la mise en oeuvre des mesures de prévention adaptées à l'hygiène et à la sécuritéTraiter les commandes des clients - 140 hPériode d'application en entreprise 1 - Se confronter à la réalité professionnelleMettre en application des acquisDévelopper des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hModule 2 Accueillir et accompagner le client dans un point de vente - Accueillir les clients et mettre en oeuvre des conditions favorables à l'accueil des personnes en situation de handicapProposer les programmes et services de fidélisation de l'unité marchande et conclure l'entretien de venteTenir un poste de caisse et superviser les caisses libre-serviceComprendre l'évolution du digital et les enjeux de la valorisation de l'expérience d'achat dans un contexte omnicanalValoriser l'image de l'unité marchande en s'appropriant les principes majeurs de l'écocitoyenneté tout au long de l'expérience d'achat - 140 hPériode d'application en entreprise 2 (environnement omnicanal) - Se confronter à la réalité professionnelleMettre en application des acquisRenforcer ses compétences transversesDévelopper son réseau professionnel - 140 hPériode de certification - Certification Employé Commercial - 35 hSensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa propre empreinte écologique / prendre conscience de son propre impact (quiz, impactco2.fr, fresque du climat...Définir les points de progrès individuels et collectifs applicables dans la vie quotidie | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel commis de cuisine</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé commercial</t>
         </is>
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910486/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10910496/true/false/false/true</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W16" s="5" t="inlineStr">
@@ -2401,32 +2353,32 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Horticulteur, horticultrice (CAPA) [HSP 1er NQ]</t>
+          <t>Conseiller, Conseillère de vente (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>CENTRE DE FORMATION PROFESSIONNELLE ET DE PROMOTION AGRICOLES (CFPPA L'OISELLERIE)</t>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>16400 La Couronne</t>
+          <t>17000 La Rochelle</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>28 Allee de l Oisellerie | 16400 La Couronne | France</t>
+          <t>AXYS | 33 Rue DU REMPART ST CLAUDE | 17000 La Rochelle | France</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1239 heures (dont 399 heures en entreprise)</t>
+          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2436,17 +2388,17 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>http://www.epl-charente.com/</t>
+          <t>http://www.afpa.fr/</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>cfppa.angouleme@educagri.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>cfppa.angouleme@educagri.fr | karine.durand@educagri.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | axysetien@orange.fr | axystayeb@orange.fr</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -2461,12 +2413,12 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>0545673695</t>
+          <t>0546411640</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>0545673695</t>
+          <t>0546411640 | 0679890571</t>
         </is>
       </c>
       <c r="O17" s="7" t="inlineStr">
@@ -2487,22 +2439,22 @@
       <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="7" t="inlineStr">
         <is>
-          <t>Agir dans des situation de la vie courante à l'aide de repères sociaux ( CG1) - - Prendre position dans une situation à caractère social et civique- Utiliser des outils dans des situations de la vie courante - 56 hMettre en oeuvre des actions contribuant à la construction personnelle (CG2) - - S'exprimer à travers une réalisation personnelle- Adopter des comportements favorisant son équilibre personnel - 56 hInteragir avec son environnement social (CG3) - - Adapter son langage et son comportement aux situations decommunication- S'approprier les normes et cadres de référence d'un collectif - 49 hRéaliser des travaux sur les végétaux ( CP4) - - Réaliser des observations et interventions sur le végétal- Réaliser des travaux de mise en place des végétaux - 189 hRéaliser des travaux de suivi des cultures de l'implantation à la récolte et au conditionnement ( CP5) - - Réaliser des observations et opérations techniques liées au cycle de production- Effectuer des travaux de récolte, de conservation et de conditionnement - 196 hEffectuer des travaux liés à l'entretien courant des matériels , équipements, installations et bâtiments (CP6) - - Réaliser des opérations de maintenance conditionnelle des matériels, équipements, installations et bâtiments- Effectuer des travaux simples d'aménagement et de réparation - 147 hS'adapter à des enjeux professionnels locaux (CP7) - Pour le département 16, UCARE "Vente et commercialisation de produits horticoles" : Accueillir les clients- Vendre directement les produits de l'atelierPour le département 17, UCARE "Initiation aux travaux viticoles" : Préparer les principaux travaux liés au vignoble. Réaliser les travaux liés au vignoble - 105 hSensibilisation Priorités Régionales - Identifier les enjeux du dérèglement climatique et proposer des alternatives : - Climat- Renaissance écologiqueSensibilisation aux valeurs de la république (référentiel ANCT) :Valeurs de la république et laïcité-Non discriminationSe questionner sur les impacts environnementaux du numérique, apprendre à mesurer, décrypter et agir, pour trouver sa place de citoyen dans un monde numérique.MOOC-L'identité numérique enjeux pour le citoyen (RGPD, Réseaux sociaux, - 35 hBilans - Intermédiaire et Final - 7 | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Période d'intégration CV - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hM1 - Contribuer à l'efficacité commerciale d'une unité marchande dans un environnement omnicanal - Connaître les différents contextes de la vente de services et de produitsConnaître les fondamentaux de la démarche marketingMener une étude de marché et établir le diagnostic de l'unité marchandeConnaître les différentes techniques et méthodes d'approvisionnementRéaliser des inventairesAppliquer les règles et les obligations légales du recyclage, du tri sélectif des déchets et de la réduction du gaspillageComprendre les règles de merchandisingMettre en place une opération commercialeSuivre et analyser les évolutions et exploiter les résultats pour proposer des ajustements - 245 hPériode en entreprise 1 - Se confronter à la réalité professionnelleMettre en application des acquisDévelopper des compétences transverses Etablir un réseau favorisant l'insertion professionnelle - 140 hM2 - Améliorer l'expérience client dans un environnement omnicanal - Comprendre l'évolution du digital et son impact sur le métierValoriser l'offre de produits et de services de l'unité marchande sur les sites marchands et les médias sociauxAccueillir le client et mettre en oeuvre des conditions favorables à l'accueil des personnes en situation de handicapProcéder à l'enregistrement et à l'encaissementConnaître le cadre juridique de la vente et les enjeux du suivi de la relation commercialeConnaître les fondamentaux de la démarche marketingS'approprier et défendre les principes majeurs de l'écocitoyenneté tout au long de l'expérience d'achat - 210 hPériode en entreprise 2 - Se confronter à la réalité professionnelle Mettre en application des acquis Renforcer ses compétences transverses Développer son réseau professionnel - 140 hPériode de certification - Certification Conseiller de vente - 35 hSensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du dé | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP agricole métiers de l'agriculture</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller de vente</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910500/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10910502/true/false/false/true</t>
         </is>
       </c>
       <c r="V17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W17" s="7" t="inlineStr">
@@ -2514,32 +2466,32 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Jardinier, Jardinière paysagiste (CAPA) [HSP 1er NQ]</t>
+          <t>Employé(e) commercial (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>CENTRE DE FORMATION PROFESSIONNELLE ET DE PROMOTION AGRICOLES (CFPPA L'OISELLERIE)</t>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>16400 La Couronne</t>
+          <t>17000 La Rochelle</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>28 Allee de l Oisellerie | 16400 La Couronne | France</t>
+          <t>AXYS | 33 Rue DU REMPART ST CLAUDE | 17000 La Rochelle | France</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1239 heures (dont 399 heures en entreprise)</t>
+          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -2549,17 +2501,17 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>http://www.epl-charente.com/</t>
+          <t>http://www.afpa.fr/</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>cfppa.angouleme@educagri.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>cfppa.angouleme@educagri.fr | karine.durand@educagri.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | axysetien@orange.fr | axystayeb@orange.fr</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -2574,12 +2526,12 @@
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>0545673695</t>
+          <t>0546411640</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>0545673695</t>
+          <t>0546411640 | 0679890571</t>
         </is>
       </c>
       <c r="O18" s="5" t="inlineStr">
@@ -2600,22 +2552,22 @@
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>Agir dans des situation de la vie courante à l'aide de repères sociaux (CG1) - - Prendre position dans une situation à caractère social et civique- Utiliser des outils dans des situations de la vie courante - 56 hMettre en oeuvre des actions contribuant à la construction personnelle (CG2) - - S'exprimer à travers une réalisation personnelle- Adopter des comportements favorisant son équilibre personnel - 56 hInteragir avec son environnement social (CG3) - - Adapter son langage et son comportement aux situations de communication- S'approprier les normes et cadres de référence d'un collectif - 49 hRéaliser en sécurité des travaux d'entretien paysager (CP4) - - Entretenir la végétation- Réaliser l'entretien des installations et des infrastructures paysagères - 189 hRéaliser en sécurité des travaux d'aménagement paysager (CP5) - - Réaliser des travaux de mise en place des végétaux- Réaliser des travaux de mise en place d'installations et d'infrastructures paysagères - 196 hEffectuer des travaux liés à l'entretien courant des matériels et équipements (CP6) - - Réaliser des opérations de maintenance conditionnelle des matériels et équipements- Réaliser des opérations de maintenance corrective des matériels et équipements - 147 hS'adapter à des enjeux professionnels locaux (CP7) - Pour le département 16, UCARE "Bassin de rétention" : Mettre en oeuvre un bassin de rétention- Entretenir un bassin de rétentionPour le département 17, UCARE "Corridors-Abris Faune" :Réaliser la mise en place de corridors écologiques et abris petite faune ( 70H) - 105 hSensibilisation Priorités Régionales - Identifier les enjeux du dérèglement climatique et proposer des alternatives : - Climat- Renaissance écologiqueSensibilisation aux valeurs de la république (référentiel ANCT) :Valeurs de la république et laïcité-Non discriminationSe questionner sur les impacts environnementaux du numérique, apprendre à mesurer, décrypter et agir, pour trouver sa place de citoyen dans un monde numérique.MOOC-L'identité numérique enjeux pour le citoyen (RGPD, Réseaux sociaux, - 35 hBilans - Intermédiaire et Final - 7 h | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Période d'intégration Employé Commercial - Intégrer son groupe et sa formation J'apprends à apprendreS'approprier les objectifs de la formation et repérer son futur environnement professionnelPréciser ses besoins de formation et contractualiser son parcours personnaliséS'inscrire dans une perspective d'emploi - 35 hModule 1 Mettre à disposition des clients les produits de l'unité marchande dans un environnement omnicanal - Appliquer les règles et les obligations légales du recyclage, du tri sélectif des déchets et de la réduction du gaspillageRéceptionner et stocker la marchandiseComprendre les règles de merchandisingParticiper à la mise en oeuvre d'une opération commercialeVeiller à la mise en oeuvre des mesures de prévention adaptées à l'hygiène et à la sécuritéTraiter les commandes des clients - 140 hPériode d'application en entreprise 1 - Se confronter à la réalité professionnelleMettre en application des acquisDévelopper des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hModule 2 Accueillir et accompagner le client dans un point de vente - Accueillir les clients et mettre en oeuvre des conditions favorables à l'accueil des personnes en situation de handicapProposer les programmes et services de fidélisation de l'unité marchande et conclure l'entretien de venteTenir un poste de caisse et superviser les caisses libre-serviceComprendre l'évolution du digital et les enjeux de la valorisation de l'expérience d'achat dans un contexte omnicanalValoriser l'image de l'unité marchande en s'appropriant les principes majeurs de l'écocitoyenneté tout au long de l'expérience d'achat - 140 hPériode d'application en entreprise 2 (environnement omnicanal) - Se confronter à la réalité professionnelleMettre en application des acquisRenforcer ses compétences transversesDévelopper son réseau professionnel - 140 hPériode de certification - Certification Employé Commercial - 35 hSensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa propre empreinte écologique / prendre conscience de son propre impact (quiz, impactco2.fr, fresque du climat...Définir les points de progrès individuels et collectifs applicables dans la vie quotidie | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T18" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP agricole jardinier paysagiste</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé commercial</t>
         </is>
       </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910501/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10910505/true/false/false/true</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W18" s="5" t="inlineStr">
@@ -2627,32 +2579,32 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Agent(e) de service médico-social (TP) [HSP 1er NQ]</t>
+          <t>Commis de cuisine (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>GRETA POITOU-CHARENTES - SIÈGE ADMINISTRATIF</t>
+          <t>CENTRE DE FORMATION FARE 16-ROC FLEURI (FARE 16)</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>16600 Mornac</t>
+          <t>17300 Rochefort</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>ASSOCIATION NATIONALE POUR LA FORMATION PROFESSIONNELLE DES ADULTES | 104 Route Lac Melot Zone la Braconne | 16600 Mornac | France</t>
+          <t>AFPA ROCHEFORT | 57 Avenue BERNADOTTE | 17300 Rochefort | France</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2662,17 +2614,17 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>http://www.greta-poitou-charentes.fr/</t>
+          <t>https://fare16.cneap.fr/</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>commercial.greta.agence-poitiers@ac-poitiers.fr</t>
+          <t>comptable.fare16@cneap.fr</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>commercial.greta.agence-poitiers@ac-poitiers.fr | formations-angouleme@afpa.fr</t>
+          <t>comptable.fare16@cneap.fr | formations-rochefort@afpa.fr | lisa.perrotin@afpa.fr</t>
         </is>
       </c>
       <c r="K19" s="7" t="inlineStr">
@@ -2687,12 +2639,12 @@
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>0648579860</t>
+          <t>0699077417</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>0648579860</t>
+          <t>0699077417 | 0616046682</t>
         </is>
       </c>
       <c r="O19" s="7" t="inlineStr">
@@ -2713,22 +2665,22 @@
       <c r="R19" s="7" t="inlineStr"/>
       <c r="S19" s="7" t="inlineStr">
         <is>
-          <t>Bloc de compétences 1 - Réaliser le nettoyage et le bio nettoyage des locaux en s'adaptant à la présence des résidents - Participer à la vie de l'établissementAppliquer les techniques professionnelles d'entretien des locaux dans les espaces communs, la chambre du résident, la salle de bain dans le respect de la présence des résidentsUtiliser les produits, matériels, protocoles, en se protégeant et en protégeant les autres Gérer le temps de son interventionS'organiser et gérer des stocksComprendre la notion de développement durable et l'intégrer dans son activité professionnelle au quotidien - 147 hBloc de compétences 2 - Contribuer aux prestations du service hôtelier en respectant les standards de qualité de l'établissement - Contribuer au service du linge des résidents et de l'établissement, gérer les stocks en lingerieConnaitre et appliquer les moyens de prévention des infections, précautions standards, précautions en cas d'épidémieAssurer la réfection d'un lit inoccupéContribuer au service des repas des résidents, respecter les goûts et consignes, adapter la présentation pour favoriser l'autonomie, préparer la salle à manger dans le respect des normes qualité de l'établissementCommuniquer avec les résidents, respecter leurs habitudes et autonomie - 98 hBloc de compétences 3 - Accompagner le résident dans les gestes de la vie quotidienne en tenant compte du projet - Accompagner le résident dans ses déplacementsAccompagner le résident à prendre son repas et à boireAppréhender les incidences des pathologies, handicaps et déficiences dans la vie quotidienne des résidentsCommuniquer avec l'équipe pluridisciplinaireObserver, écouter et établir des relations avec les résidentsIntervenir dans le respect des gestes de sécurité - 126 hPréparation à la Certification - Accompagner à la rédaction du Dossier ProfessionnelFinaliser les Epreuves en Cours de Formation (ECF)Préparer à l'épreuve finalePréparer à l'entretien final - 35 hLes périodes de formation en milieu professionnel (PFMP) - Les PFMP permettent de mettre en oeuvre ou d'acquérir des compétences sous la responsabilité d'une personne qualifiée (tuteur-trice) et d'apprendre à travailler en situation réelle avec les moyens et contraintes du milieu professionnel.L'alternance centre/entreprise répond à une progression péda | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Positionnement Accompagnement socio-professionnel générique - Réalisation de diagnosticsDéfinition du parcours individualiséIdentification des freins Bilan intermédiaire et final - 63 hCAP Organisation de la production de cuisine UP1 - -Réceptionner, contrôler et stocker les marchandises dans le respect de la réglementation en vigueur et en appliquant les techniques de prévention liées à l'activité- Collecter l'ensemble des informations et organiser sa production culinaire dans le respect des consignes et de temps imparti - 105 hCAP Réalisation de la production de cuisine UP2 - - Préparer, organiser et maintenir en état son poste de travail tout au long de l'activité dans le respect de la réglementation en vigueur- Maîtriser les techniques culinaires de base et réaliser une production dans le respect des consignes et des règles d'hygiène et de sécurité- Analyser, contrôler la qualité de sa production, dresser et participer à la distribution selon le contexte professionnel- Communiquer en fonction du contexte professionnel et en respectant les usages de la profession - 336 hCAP Prévention-santé-environnement UP3 - - Appliquer une méthode d'analyse d'une situation de la vie professionnelle ou quotidienne et d'une documentation- Mettre en relation un phénomène physiologique, un enjeu environnemental, une disposition réglementaire, avec une mesure de prévention- Proposer une solution pour résoudre un problème lié à la santé, l'environnement ou la consommation et argumenter un choix - Communiquer à l'écrit et à l'oral avec une syntaxe claire et un vocabulaire technique adapté- Agir face à une situation d'urgence - 35 hCAP Français et Histoire-géographie Enseignement moral et civique - - Entrer dans l'échange oral et écrit : écouter, réagir, s'exprimer, lire, analyser, écrire- Devenir un lecteur compétent et critique- Confronter des savoirs et des valeurs pour construire son identité culturelle- Histoire-Géographie et Enseignement moral et civique- Appréhender la diversité des sociétés et la richesse des cultures- Repérer la situation étudiée dans le temps et dans l'espace- Relever, classer et hiérarchiser les informations contenues dans un document selon des critères donnés- Acquérir une démarche citoyenne à partir de son environnement quotidien - 56 hCAP Mathématiques - Physique - Chimie - | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de service médico-social</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel commis de cuisine</t>
         </is>
       </c>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10919993/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10919965/true/false/false/true</t>
         </is>
       </c>
       <c r="V19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W19" s="7" t="inlineStr">
@@ -2740,47 +2692,1169 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Serveur, Serveuse en hôtellerie-restauration (TP) [HSP 1er NQ]</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>CENTRE DE FORMATION FARE 16-ROC FLEURI (FARE 16)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>17300 Rochefort</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>AFPA ROCHEFORT | 57 Avenue BERNADOTTE | 17300 Rochefort | France</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>https://fare16.cneap.fr/</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
+        <is>
+          <t>comptable.fare16@cneap.fr</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>comptable.fare16@cneap.fr | formations-rochefort@afpa.fr | lisa.perrotin@afpa.fr</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>0699077417</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>0699077417 | 0616046682</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P20" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="inlineStr"/>
+      <c r="S20" s="5" t="inlineStr">
+        <is>
+          <t>TP Positionnement Accompagnement socio-professionnel générique - Réalisation des diagnosticsDéfinition du parcours individualiséIdentification des freinsBilan intermédiaire et final - 63 hTP Réaliser les travaux préalables au service en restauration - - Nettoyer et entretenir les espaces de restauration et les locaux annexes- Mettre en place les espaces de restauration et les locaux annexes- Mettre en place les différents types de buffet - 126 hTP Accueillir, conseiller le client et prendre sa commande - - Accueillir la clientèle et l'accompagner à sa table- Présenter cartes et menus, prendre la commande et la communiquer aux services concernés - 154 hTP Réaliser le service en restauration - - Préparer et servir les boissons en respectant les règles de service- Effectuer les différents types de service à table et au buffet- Préparer, vérifier une addition et l'encaisser - 154 hTP Règles d'hygiène dans la restauration et les commerces alimentaires - Donner à chaque participant les connaissances d'hygiène nécessaires afin: De produire un travail de qualité- De respecter dans chaque secteur de soin les règles d'hygiène en utilisant convenablement le matériel et les produits d'entretien- Situer et valoriser les responsabilités et le rôle du personnel dans la prévention des infections nosocomiales - 14 hTP Gestes et postures - - Acquérir les compétences nécessaires pour contribuer à la mise en oeuvre de la prévention des risques liés à l'activité physique - 14 hTP Sensibilisation au numérique Responsable - Intégrer les enjeux du numérique dans ses pratiques quotidiennes et professionnelles par :L'hygiène numérique compatible avec une pratique responsableLa santé mentale dans l'utilisation d'internetTerritoire numérique responsableBonnes pratiquesLa cybersécurité dans ses pratiques du numériqueLes types d'attaques et conséquencesUtilisateur modérateur et trace numériqueLiberté numérique et l'utilisation des outilsLe règlement général sur la protection des donnéesTraces et e-réputationSources d'information et règlementation CNILDroits d'utilisation, d'auteur et à l'imag - 14 hTP Sensibilisation aux valeurs de la République - - Participer à une meilleure compréhension des enjeux d'une société fondée sur les vale | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T20" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel serveur en restauration</t>
+        </is>
+      </c>
+      <c r="U20" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/10919967/true/false/false/false</t>
+        </is>
+      </c>
+      <c r="V20" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W20" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Agent(e) de service médico-social (TP) [HSP 1er NQ]</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>GRETA POITOU-CHARENTES - SIÈGE ADMINISTRATIF</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>17300 Rochefort</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>AFPA ROCHEFORT | 57 Avenue BERNADOTTE | 17300 Rochefort | France</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>http://www.greta-poitou-charentes.fr/</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>commercial.greta.agence-poitiers@ac-poitiers.fr</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>commercial.greta.agence-poitiers@ac-poitiers.fr | formations-rochefort@afpa.fr | lisa.perrotin@afpa.fr</t>
+        </is>
+      </c>
+      <c r="K21" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="inlineStr">
+        <is>
+          <t>0699077417</t>
+        </is>
+      </c>
+      <c r="N21" s="7" t="inlineStr">
+        <is>
+          <t>0699077417 | 0616046682</t>
+        </is>
+      </c>
+      <c r="O21" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P21" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q21" s="7" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R21" s="7" t="inlineStr"/>
+      <c r="S21" s="7" t="inlineStr">
+        <is>
+          <t>Bloc de compétences 1 - Réaliser le nettoyage et le bio nettoyage des locaux en s'adaptant à la présence des résidents - Participer à la vie de l'établissementAppliquer les techniques professionnelles d'entretien des locaux dans les espaces communs, la chambre du résident, la salle de bain dans le respect de la présence des résidentsUtiliser les produits, matériels, protocoles, en se protégeant et en protégeant les autres Gérer le temps de son interventionS'organiser et gérer des stocksComprendre la notion de développement durable et l'intégrer dans son activité professionnelle au quotidien - 147 hBloc de compétences 2 - Contribuer aux prestations du service hôtelier en respectant les standards de qualité de l'établissement - Contribuer au service du linge des résidents et de l'établissement, gérer les stocks en lingerieConnaitre et appliquer les moyens de prévention des infections, précautions standards, précautions en cas d'épidémieAssurer la réfection d'un lit inoccupéContribuer au service des repas des résidents, respecter les goûts et consignes, adapter la présentation pour favoriser l'autonomie, préparer la salle à manger dans le respect des normes qualité de l'établissementCommuniquer avec les résidents, respecter leurs habitudes et autonomie - 98 hBloc de compétences 3 - Accompagner le résident dans les gestes de la vie quotidienne en tenant compte du projet - Accompagner le résident dans ses déplacementsAccompagner le résident à prendre son repas et à boireAppréhender les incidences des pathologies, handicaps et déficiences dans la vie quotidienne des résidentsCommuniquer avec l'équipe pluridisciplinaireObserver, écouter et établir des relations avec les résidentsIntervenir dans le respect des gestes de sécurité - 126 hPréparation à la Certification - Accompagner à la rédaction du Dossier ProfessionnelFinaliser les Epreuves en Cours de Formation (ECF)Préparer à l'épreuve finalePréparer à l'entretien final - 35 hLes périodes de formation en milieu professionnel (PFMP) - Les PFMP permettent de mettre en oeuvre ou d'acquérir des compétences sous la responsabilité d'une personne qualifiée (tuteur-trice) et d'apprendre à travailler en situation réelle avec les moyens et contraintes du milieu professionnel.L'alternance centre/entreprise répond à une progression péda | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T21" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de service médico-social</t>
+        </is>
+      </c>
+      <c r="U21" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/10920021/true/false/false/true</t>
+        </is>
+      </c>
+      <c r="V21" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-17&amp;range=110-119&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W21" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
           <t>16</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr"/>
-      <c r="C20" s="5" t="inlineStr"/>
-      <c r="D20" s="5" t="inlineStr"/>
-      <c r="E20" s="5" t="inlineStr"/>
-      <c r="F20" s="5" t="inlineStr"/>
-      <c r="G20" s="5" t="inlineStr"/>
-      <c r="H20" s="5" t="inlineStr"/>
-      <c r="I20" s="5" t="inlineStr"/>
-      <c r="J20" s="5" t="inlineStr"/>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Action préparatoire aux métiers de l'agriculture [HSP 1er NQ]</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>CENTRE DE FORMATION PROFESSIONNELLE ET DE PROMOTION AGRICOLES (CFPPA L'OISELLERIE)</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>16200 Triac-Lautrait</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>MAISON FAMILIALE RURALE D'ÉDUCATION ET D'ORIENTATION TRIAC LAUTRAIT | 16 Route DE COGNAC | 16200 Triac-Lautrait | France</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>http://www.epl-charente.com/</t>
+        </is>
+      </c>
+      <c r="I22" s="6" t="inlineStr">
+        <is>
+          <t>cfppa.angouleme@educagri.fr</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>cfppa.angouleme@educagri.fr | eric.verger@mfr.asso.fr</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M22" s="5" t="inlineStr">
+        <is>
+          <t>0545353771</t>
+        </is>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>0545353771</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr"/>
+      <c r="P22" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q22" s="5" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R22" s="5" t="inlineStr"/>
+      <c r="S22" s="5" t="inlineStr">
+        <is>
+          <t>Découverte des filières et des métiers - Découverte de l'activité professionnelle agricole sur le territoire : Spécificités, filières, métiers... (visites d'exploitations, interventions de professionnels) Les activités agricoles et leur saisonnalité- L'emploi agricole sur le territoire (intervention de partenaires emploi agricole) Les métiers : matériel et risques professionnels - 42 hElaboration du projet professionnel - Définir sa (ses) filière(s) :Le projet initial : Explicitation du projet et ses représentations par chaque candidatDécouvrir et se tester en situation : Visites- Travaux Pratiques en ateliers pédagogiquesChoix de filière : 1 à 3 pour répartir les immersions en stage en entrepriseAccompagnement vers les stages : Cartographie- Mobilité- Candidature (CV, Entretien,LM... Accompagnement personnalisé - 56 hConsolidation et concrétisation du projet professionnel - - Détermination du choix de filière, suite aux immersion : Représentation et explicitation des activités- Consolidation du projet : Projection dans l'activité, besoins (savoir, savoir-être, formations... Technique de Recherche d'Emploi (TRE) et accompagnement vers l'emploi/formation (selon projet personnel) : Présentation de son projet (personnel, professionnel, formation) Identification des compétences (acquises et à acquérir) accompagnement individualisé- Définir son besoin des compétences et les étapes de son projet (formation, emploi) déterminer un "tableau de bord" de projet - 56 hAcquisition des compétences nécessaires à l'intégration professionnelle - - Compétences sociales et civiques : lister les compétences nécessaires, la non discrimination (genre, génération, catégorie socio-pro... intégration en milieu professionnel- Savoir-être, aptitudes professionnelles (attitude et posture) : Communication, savoir explicité son activité, ponctualité, initiative, autonomie, écoute... Santé et sécurité au travail : Identification des facteurs de risques professionnels et adapter/adopter des comportements pour préserver sa santé et celle d'autrui - 49 hIdentification des freins, Accompagnent Socio Pro - Validation par le stagiaire de sa capacité à intégrer une formation/emploiIdentification des freins au projet : mobilité, financiers, handicap, socio, logement, restauration, addiction...Accompagnement personnalisé à la levée des | Organisme | CENTRE DE FORMATION PROFESSIONNELLE ET DE PROMOTION AGRICOLES (CFPPA L'OISELLERIE) | http://www.epl-charente.com | Lieu de la formation</t>
+        </is>
+      </c>
+      <c r="T22" s="5" t="inlineStr"/>
+      <c r="U22" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/10904504/true/false/false/true</t>
+        </is>
+      </c>
+      <c r="V22" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W22" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Viticulteur, Viticultrice (CAPA) [HSP 1er NQ]</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>CENTRE DE FORMATION PROFESSIONNELLE ET DE PROMOTION AGRICOLES (CFPPA L'OISELLERIE)</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>16400 La Couronne</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>28 Allee de l Oisellerie | 16400 La Couronne | France</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 1239 heures (dont 399 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>http://www.epl-charente.com/</t>
+        </is>
+      </c>
+      <c r="I23" s="6" t="inlineStr">
+        <is>
+          <t>cfppa.angouleme@educagri.fr</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>cfppa.angouleme@educagri.fr | karine.durand@educagri.fr</t>
+        </is>
+      </c>
+      <c r="K23" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L23" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="inlineStr">
+        <is>
+          <t>0545673695</t>
+        </is>
+      </c>
+      <c r="N23" s="7" t="inlineStr">
+        <is>
+          <t>0545673695</t>
+        </is>
+      </c>
+      <c r="O23" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P23" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q23" s="7" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R23" s="7" t="inlineStr"/>
+      <c r="S23" s="7" t="inlineStr">
+        <is>
+          <t>Agir dans des situation de la vie courante à l'aide de repères sociaux (CG1) - - Prendre position dans une situation à caractère social et civique- Utiliser des outils dans des situations de la vie courante - 56 hMettre en oeuvre des actions contribuant à la construction personnelle (CG2) - - S'exprimer à travers une réalisation personnelle- Adopter des comportements favorisant son équilibre personnel - 56 hInteragir avec son environnement social (CG3) - - Adapter son langage et son comportement aux situations de communication- S'approprier les normes et cadres de référence d'un collectif - 49 hRéaliser des travaux sur les végétaux (CP4) - - Réaliser des observations et interventions sur le végétal- Réaliser des travaux de mise en place des végétaux - 189 hRéaliser des travaux de suivi des cultures de l'implantation à la récolte et au conditionnement (CP5) - - Réaliser des observations et opérations techniques liées au cycle de production- Effectuer des travaux de récolte, de conservation *et de conditionnement* (pour Arboriculture et Horticulture) - 196 hEffectuer des travaux liés à l'entretien courant des matériels, équipements, installations et bâtiments (CP6) - - Réaliser des opérations de maintenance conditionnelle des matériels, équipements, installations et bâtiments- Effectuer des travaux simples d'aménagement et de réparation - 147 hParticiper à la distillation charentaise (CP7) - - Réaliser un vin de chaudière- Participer à la distillation charentaise - 105 hSensibilisation Priorités Régionales - Identifier les enjeux du dérèglement climatique et proposer des alternatives : - Climat- Renaissance écologiqueSensibilisation aux valeurs de la république (référentiel ANCT) :Valeurs de la république et laïcité-Non discriminationSe questionner sur les impacts environnementaux du numérique, apprendre à mesurer, décrypter et agir, pour trouver sa place de citoyen dans un monde numérique.MOOC-L'identité numérique enjeux pour le citoyen (RGPD, Réseaux sociaux, - 35 hBilans - Intermédiaire et Final - 7 h | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T23" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP agricole métiers de l'agriculture</t>
+        </is>
+      </c>
+      <c r="U23" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/10910457/true/false/false/true</t>
+        </is>
+      </c>
+      <c r="V23" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W23" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Conseiller, Conseillère commercial (TP) [HSP 1er NQ]</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>16600 Magnac-sur-Touvre</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>ASSOCIATION NATIONALE POUR LA FORMATION PROFESSIONNELLE DES ADULTES | 104 Route Lac Melot Zone la Braconne | 16600 Magnac-sur-Touvre | France</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>http://www.afpa.fr/</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-angouleme@afpa.fr | marion.lesueur@afpa.fr</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>0648579860</t>
+        </is>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>0648579860 | 0545658101</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P24" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q24" s="5" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R24" s="5" t="inlineStr"/>
+      <c r="S24" s="5" t="inlineStr">
+        <is>
+          <t>TP CC - Période d'intégration Conseiller commercial - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hTP CC - Module 1 Prospecter un secteur de vente - Assurer une veille professionnelle et commercialeMettre en oeuvre un plan d'actions commerciales et organiser son activitéProspecter à distanceProspecter physiquementAnalyser ses performances commerciales et en rendre compte - 280 hTP CC - Période Entreprise CCP1 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP CC - Module 2 Vendre en face à face des produits et des services référencés aux entreprises et aux particuliers - Représenter l'entreprise et valoriser son imageConduire un entretien de venteAssurer le suivi de ses ventesFidéliser son portefeuille client - 280 hTP CC - Période Entreprise CCP2 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP CC - Période de synthèse du parcours professionnel - Analyse de ses apprentissagesFinalisation de son dossier professionnelPréparation de la session de validation - 35 hTP CC - Période de certification - Certification Conseiller Commercial - 35 hTP CC - Sensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa propre empreinte écologique / prendre conscience de son propre impact (quiz, impactco2.fr, fresque du climat...Définir les points de progrès individuels et collectifs applicables dans la vie quotidienne, en formation et dans le milieu professionnel (Intervention d'acteurs locaux type ressourcerie, SIVOM, association de facilitation des mobilités douces, ... - 14 hTP CC - Sensibilisation aux enjeux des valeurs de la république.... - APPREHENDERRecontextualisation du principe de laïcité. Présentation : liber | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T24" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller commercial</t>
+        </is>
+      </c>
+      <c r="U24" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/10910468/true/false/false/true</t>
+        </is>
+      </c>
+      <c r="V24" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W24" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Serveur, Serveuse en hôtellerie-restauration (TP) [HSP 1er NQ]</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>CENTRE DE FORMATION FARE 16-ROC FLEURI (FARE 16)</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>16710 Saint-Yrieix-sur-Charente</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>14 Allee PIERRE GAULT | 16710 Saint-Yrieix-sur-Charente | France</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>https://fare16.cneap.fr/</t>
+        </is>
+      </c>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>comptable.fare16@cneap.fr</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>comptable.fare16@cneap.fr | accueil.fare16@cneap.fr</t>
+        </is>
+      </c>
+      <c r="K25" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L25" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M25" s="7" t="inlineStr">
+        <is>
+          <t>0545315917</t>
+        </is>
+      </c>
+      <c r="N25" s="7" t="inlineStr">
+        <is>
+          <t>0545315917</t>
+        </is>
+      </c>
+      <c r="O25" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P25" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q25" s="7" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R25" s="7" t="inlineStr"/>
+      <c r="S25" s="7" t="inlineStr">
+        <is>
+          <t>TP Positionnement Accompagnement socio-professionnel générique - Réalisation des diagnosticsDéfinition du parcours individualiséIdentification des freinsBilan intermédiaire et final - 63 hTP Réaliser les travaux préalables au service en restauration - - Nettoyer et entretenir les espaces de restauration et les locaux annexes- Mettre en place les espaces de restauration et les locaux annexes- Mettre en place les différents types de buffet - 126 hTP Accueillir, conseiller le client et prendre sa commande - - Accueillir la clientèle et l'accompagner à sa table- Présenter cartes et menus, prendre la commande et la communiquer aux services concernés - 154 hTP Réaliser le service en restauration - - Préparer et servir les boissons en respectant les règles de service- Effectuer les différents types de service à table et au buffet- Préparer, vérifier une addition et l'encaisser - 154 hTP Règles d'hygiène dans la restauration et les commerces alimentaires - Donner à chaque participant les connaissances d'hygiène nécessaires afin: De produire un travail de qualité- De respecter dans chaque secteur de soin les règles d'hygiène en utilisant convenablement le matériel et les produits d'entretien- Situer et valoriser les responsabilités et le rôle du personnel dans la prévention des infections nosocomiales - 14 hTP Gestes et postures - - Acquérir les compétences nécessaires pour contribuer à la mise en oeuvre de la prévention des risques liés à l'activité physique - 14 hTP Sensibilisation au numérique Responsable - Intégrer les enjeux du numérique dans ses pratiques quotidiennes et professionnelles par :L'hygiène numérique compatible avec une pratique responsableLa santé mentale dans l'utilisation d'internetTerritoire numérique responsableBonnes pratiquesLa cybersécurité dans ses pratiques du numériqueLes types d'attaques et conséquencesUtilisateur modérateur et trace numériqueLiberté numérique et l'utilisation des outilsLe règlement général sur la protection des donnéesTraces et e-réputationSources d'information et règlementation CNILDroits d'utilisation, d'auteur et à l'imag - 14 hTP Sensibilisation aux valeurs de la République - - Participer à une meilleure compréhension des enjeux d'une société fondée sur les vale | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T25" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel serveur en restauration</t>
+        </is>
+      </c>
+      <c r="U25" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/10910484/true/false/false/true</t>
+        </is>
+      </c>
+      <c r="V25" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W25" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Commis de cuisine (TP) [HSP 1er NQ]</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>CENTRE DE FORMATION FARE 16-ROC FLEURI (FARE 16)</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>16710 Saint-Yrieix-sur-Charente</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>14 Allee PIERRE GAULT | 16710 Saint-Yrieix-sur-Charente | France</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>https://fare16.cneap.fr/</t>
+        </is>
+      </c>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>comptable.fare16@cneap.fr</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>comptable.fare16@cneap.fr | accueil.fare16@cneap.fr</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>0545315917</t>
+        </is>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>0545315917</t>
+        </is>
+      </c>
+      <c r="O26" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P26" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q26" s="5" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R26" s="5" t="inlineStr"/>
+      <c r="S26" s="5" t="inlineStr">
+        <is>
+          <t>Positionnement Accompagnement socio-professionnel générique - Réalisation de diagnosticsDéfinition du parcours individualiséIdentification des freins Bilan intermédiaire et final - 63 hCAP Organisation de la production de cuisine UP1 - -Réceptionner, contrôler et stocker les marchandises dans le respect de la réglementation en vigueur et en appliquant les techniques de prévention liées à l'activité- Collecter l'ensemble des informations et organiser sa production culinaire dans le respect des consignes et de temps imparti - 105 hCAP Réalisation de la production de cuisine UP2 - - Préparer, organiser et maintenir en état son poste de travail tout au long de l'activité dans le respect de la réglementation en vigueur- Maîtriser les techniques culinaires de base et réaliser une production dans le respect des consignes et des règles d'hygiène et de sécurité- Analyser, contrôler la qualité de sa production, dresser et participer à la distribution selon le contexte professionnel- Communiquer en fonction du contexte professionnel et en respectant les usages de la profession - 336 hCAP Prévention-santé-environnement UP3 - - Appliquer une méthode d'analyse d'une situation de la vie professionnelle ou quotidienne et d'une documentation- Mettre en relation un phénomène physiologique, un enjeu environnemental, une disposition réglementaire, avec une mesure de prévention- Proposer une solution pour résoudre un problème lié à la santé, l'environnement ou la consommation et argumenter un choix - Communiquer à l'écrit et à l'oral avec une syntaxe claire et un vocabulaire technique adapté- Agir face à une situation d'urgence - 35 hCAP Français et Histoire-géographie Enseignement moral et civique - - Entrer dans l'échange oral et écrit : écouter, réagir, s'exprimer, lire, analyser, écrire- Devenir un lecteur compétent et critique- Confronter des savoirs et des valeurs pour construire son identité culturelle- Histoire-Géographie et Enseignement moral et civique- Appréhender la diversité des sociétés et la richesse des cultures- Repérer la situation étudiée dans le temps et dans l'espace- Relever, classer et hiérarchiser les informations contenues dans un document selon des critères donnés- Acquérir une démarche citoyenne à partir de son environnement quotidien - 56 hCAP Mathématiques - Physique - Chimie - | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T26" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel commis de cuisine</t>
+        </is>
+      </c>
+      <c r="U26" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/10910486/true/false/false/true</t>
+        </is>
+      </c>
+      <c r="V26" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W26" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Horticulteur, horticultrice (CAPA) [HSP 1er NQ]</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>CENTRE DE FORMATION PROFESSIONNELLE ET DE PROMOTION AGRICOLES (CFPPA L'OISELLERIE)</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>16400 La Couronne</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>28 Allee de l Oisellerie | 16400 La Couronne | France</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 1239 heures (dont 399 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>http://www.epl-charente.com/</t>
+        </is>
+      </c>
+      <c r="I27" s="6" t="inlineStr">
+        <is>
+          <t>cfppa.angouleme@educagri.fr</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>cfppa.angouleme@educagri.fr | karine.durand@educagri.fr</t>
+        </is>
+      </c>
+      <c r="K27" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L27" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M27" s="7" t="inlineStr">
+        <is>
+          <t>0545673695</t>
+        </is>
+      </c>
+      <c r="N27" s="7" t="inlineStr">
+        <is>
+          <t>0545673695</t>
+        </is>
+      </c>
+      <c r="O27" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P27" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q27" s="7" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R27" s="7" t="inlineStr"/>
+      <c r="S27" s="7" t="inlineStr">
+        <is>
+          <t>Agir dans des situation de la vie courante à l'aide de repères sociaux ( CG1) - - Prendre position dans une situation à caractère social et civique- Utiliser des outils dans des situations de la vie courante - 56 hMettre en oeuvre des actions contribuant à la construction personnelle (CG2) - - S'exprimer à travers une réalisation personnelle- Adopter des comportements favorisant son équilibre personnel - 56 hInteragir avec son environnement social (CG3) - - Adapter son langage et son comportement aux situations decommunication- S'approprier les normes et cadres de référence d'un collectif - 49 hRéaliser des travaux sur les végétaux ( CP4) - - Réaliser des observations et interventions sur le végétal- Réaliser des travaux de mise en place des végétaux - 189 hRéaliser des travaux de suivi des cultures de l'implantation à la récolte et au conditionnement ( CP5) - - Réaliser des observations et opérations techniques liées au cycle de production- Effectuer des travaux de récolte, de conservation et de conditionnement - 196 hEffectuer des travaux liés à l'entretien courant des matériels , équipements, installations et bâtiments (CP6) - - Réaliser des opérations de maintenance conditionnelle des matériels, équipements, installations et bâtiments- Effectuer des travaux simples d'aménagement et de réparation - 147 hS'adapter à des enjeux professionnels locaux (CP7) - Pour le département 16, UCARE "Vente et commercialisation de produits horticoles" : Accueillir les clients- Vendre directement les produits de l'atelierPour le département 17, UCARE "Initiation aux travaux viticoles" : Préparer les principaux travaux liés au vignoble. Réaliser les travaux liés au vignoble - 105 hSensibilisation Priorités Régionales - Identifier les enjeux du dérèglement climatique et proposer des alternatives : - Climat- Renaissance écologiqueSensibilisation aux valeurs de la république (référentiel ANCT) :Valeurs de la république et laïcité-Non discriminationSe questionner sur les impacts environnementaux du numérique, apprendre à mesurer, décrypter et agir, pour trouver sa place de citoyen dans un monde numérique.MOOC-L'identité numérique enjeux pour le citoyen (RGPD, Réseaux sociaux, - 35 hBilans - Intermédiaire et Final - 7 | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T27" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP agricole métiers de l'agriculture</t>
+        </is>
+      </c>
+      <c r="U27" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/10910500/true/false/false/true</t>
+        </is>
+      </c>
+      <c r="V27" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W27" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Jardinier, Jardinière paysagiste (CAPA) [HSP 1er NQ]</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>CENTRE DE FORMATION PROFESSIONNELLE ET DE PROMOTION AGRICOLES (CFPPA L'OISELLERIE)</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>16400 La Couronne</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>28 Allee de l Oisellerie | 16400 La Couronne | France</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Durée de 1239 heures (dont 399 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>http://www.epl-charente.com/</t>
+        </is>
+      </c>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>cfppa.angouleme@educagri.fr</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>cfppa.angouleme@educagri.fr | karine.durand@educagri.fr</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M28" s="5" t="inlineStr">
+        <is>
+          <t>0545673695</t>
+        </is>
+      </c>
+      <c r="N28" s="5" t="inlineStr">
+        <is>
+          <t>0545673695</t>
+        </is>
+      </c>
+      <c r="O28" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P28" s="5" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q28" s="5" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R28" s="5" t="inlineStr"/>
+      <c r="S28" s="5" t="inlineStr">
+        <is>
+          <t>Agir dans des situation de la vie courante à l'aide de repères sociaux (CG1) - - Prendre position dans une situation à caractère social et civique- Utiliser des outils dans des situations de la vie courante - 56 hMettre en oeuvre des actions contribuant à la construction personnelle (CG2) - - S'exprimer à travers une réalisation personnelle- Adopter des comportements favorisant son équilibre personnel - 56 hInteragir avec son environnement social (CG3) - - Adapter son langage et son comportement aux situations de communication- S'approprier les normes et cadres de référence d'un collectif - 49 hRéaliser en sécurité des travaux d'entretien paysager (CP4) - - Entretenir la végétation- Réaliser l'entretien des installations et des infrastructures paysagères - 189 hRéaliser en sécurité des travaux d'aménagement paysager (CP5) - - Réaliser des travaux de mise en place des végétaux- Réaliser des travaux de mise en place d'installations et d'infrastructures paysagères - 196 hEffectuer des travaux liés à l'entretien courant des matériels et équipements (CP6) - - Réaliser des opérations de maintenance conditionnelle des matériels et équipements- Réaliser des opérations de maintenance corrective des matériels et équipements - 147 hS'adapter à des enjeux professionnels locaux (CP7) - Pour le département 16, UCARE "Bassin de rétention" : Mettre en oeuvre un bassin de rétention- Entretenir un bassin de rétentionPour le département 17, UCARE "Corridors-Abris Faune" :Réaliser la mise en place de corridors écologiques et abris petite faune ( 70H) - 105 hSensibilisation Priorités Régionales - Identifier les enjeux du dérèglement climatique et proposer des alternatives : - Climat- Renaissance écologiqueSensibilisation aux valeurs de la république (référentiel ANCT) :Valeurs de la république et laïcité-Non discriminationSe questionner sur les impacts environnementaux du numérique, apprendre à mesurer, décrypter et agir, pour trouver sa place de citoyen dans un monde numérique.MOOC-L'identité numérique enjeux pour le citoyen (RGPD, Réseaux sociaux, - 35 hBilans - Intermédiaire et Final - 7 h | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T28" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP agricole jardinier paysagiste</t>
+        </is>
+      </c>
+      <c r="U28" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/10910501/true/false/false/true</t>
+        </is>
+      </c>
+      <c r="V28" s="5" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W28" s="5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Agent(e) de service médico-social (TP) [HSP 1er NQ]</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>GRETA POITOU-CHARENTES - SIÈGE ADMINISTRATIF</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>16600 Mornac</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>ASSOCIATION NATIONALE POUR LA FORMATION PROFESSIONNELLE DES ADULTES | 104 Route Lac Melot Zone la Braconne | 16600 Mornac | France</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>Prochaine session</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>http://www.greta-poitou-charentes.fr/</t>
+        </is>
+      </c>
+      <c r="I29" s="6" t="inlineStr">
+        <is>
+          <t>commercial.greta.agence-poitiers@ac-poitiers.fr</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>commercial.greta.agence-poitiers@ac-poitiers.fr | formations-angouleme@afpa.fr</t>
+        </is>
+      </c>
+      <c r="K29" s="7" t="inlineStr">
+        <is>
+          <t>france_travail</t>
+        </is>
+      </c>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="inlineStr">
+        <is>
+          <t>0648579860</t>
+        </is>
+      </c>
+      <c r="N29" s="7" t="inlineStr">
+        <is>
+          <t>0648579860</t>
+        </is>
+      </c>
+      <c r="O29" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
+      <c r="P29" s="7" t="inlineStr">
+        <is>
+          <t>Formation financée par la région</t>
+        </is>
+      </c>
+      <c r="Q29" s="7" t="inlineStr">
+        <is>
+          <t>En centre</t>
+        </is>
+      </c>
+      <c r="R29" s="7" t="inlineStr"/>
+      <c r="S29" s="7" t="inlineStr">
+        <is>
+          <t>Bloc de compétences 1 - Réaliser le nettoyage et le bio nettoyage des locaux en s'adaptant à la présence des résidents - Participer à la vie de l'établissementAppliquer les techniques professionnelles d'entretien des locaux dans les espaces communs, la chambre du résident, la salle de bain dans le respect de la présence des résidentsUtiliser les produits, matériels, protocoles, en se protégeant et en protégeant les autres Gérer le temps de son interventionS'organiser et gérer des stocksComprendre la notion de développement durable et l'intégrer dans son activité professionnelle au quotidien - 147 hBloc de compétences 2 - Contribuer aux prestations du service hôtelier en respectant les standards de qualité de l'établissement - Contribuer au service du linge des résidents et de l'établissement, gérer les stocks en lingerieConnaitre et appliquer les moyens de prévention des infections, précautions standards, précautions en cas d'épidémieAssurer la réfection d'un lit inoccupéContribuer au service des repas des résidents, respecter les goûts et consignes, adapter la présentation pour favoriser l'autonomie, préparer la salle à manger dans le respect des normes qualité de l'établissementCommuniquer avec les résidents, respecter leurs habitudes et autonomie - 98 hBloc de compétences 3 - Accompagner le résident dans les gestes de la vie quotidienne en tenant compte du projet - Accompagner le résident dans ses déplacementsAccompagner le résident à prendre son repas et à boireAppréhender les incidences des pathologies, handicaps et déficiences dans la vie quotidienne des résidentsCommuniquer avec l'équipe pluridisciplinaireObserver, écouter et établir des relations avec les résidentsIntervenir dans le respect des gestes de sécurité - 126 hPréparation à la Certification - Accompagner à la rédaction du Dossier ProfessionnelFinaliser les Epreuves en Cours de Formation (ECF)Préparer à l'épreuve finalePréparer à l'entretien final - 35 hLes périodes de formation en milieu professionnel (PFMP) - Les PFMP permettent de mettre en oeuvre ou d'acquérir des compétences sous la responsabilité d'une personne qualifiée (tuteur-trice) et d'apprendre à travailler en situation réelle avec les moyens et contraintes du milieu professionnel.L'alternance centre/entreprise répond à une progression péda | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T29" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de service médico-social</t>
+        </is>
+      </c>
+      <c r="U29" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/detail/10919993/true/false/false/true</t>
+        </is>
+      </c>
+      <c r="V29" s="7" t="inlineStr">
+        <is>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
+        </is>
+      </c>
+      <c r="W29" s="7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr"/>
+      <c r="C30" s="5" t="inlineStr"/>
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="5" t="inlineStr"/>
+      <c r="F30" s="5" t="inlineStr"/>
+      <c r="G30" s="5" t="inlineStr"/>
+      <c r="H30" s="5" t="inlineStr"/>
+      <c r="I30" s="5" t="inlineStr"/>
+      <c r="J30" s="5" t="inlineStr"/>
+      <c r="K30" s="5" t="inlineStr">
         <is>
           <t>introuvable</t>
         </is>
       </c>
-      <c r="L20" s="5" t="inlineStr">
+      <c r="L30" s="5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M20" s="5" t="inlineStr"/>
-      <c r="N20" s="5" t="inlineStr"/>
-      <c r="O20" s="5" t="inlineStr"/>
-      <c r="P20" s="5" t="inlineStr"/>
-      <c r="Q20" s="5" t="inlineStr"/>
-      <c r="R20" s="5" t="inlineStr"/>
-      <c r="S20" s="5" t="inlineStr"/>
-      <c r="T20" s="5" t="inlineStr"/>
-      <c r="U20" s="5" t="inlineStr">
+      <c r="M30" s="5" t="inlineStr"/>
+      <c r="N30" s="5" t="inlineStr"/>
+      <c r="O30" s="5" t="inlineStr"/>
+      <c r="P30" s="5" t="inlineStr"/>
+      <c r="Q30" s="5" t="inlineStr"/>
+      <c r="R30" s="5" t="inlineStr"/>
+      <c r="S30" s="5" t="inlineStr"/>
+      <c r="T30" s="5" t="inlineStr"/>
+      <c r="U30" s="5" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/detail/10921924/true/false/false/true</t>
         </is>
       </c>
-      <c r="V20" s="5" t="inlineStr">
+      <c r="V30" s="5" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
         </is>
       </c>
-      <c r="W20" s="5" t="inlineStr">
+      <c r="W30" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">erreur: Page.goto: Timeout 90000ms exceeded.
 Call log:
@@ -2789,1129 +3863,55 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr"/>
-      <c r="C21" s="7" t="inlineStr"/>
-      <c r="D21" s="7" t="inlineStr"/>
-      <c r="E21" s="7" t="inlineStr"/>
-      <c r="F21" s="7" t="inlineStr"/>
-      <c r="G21" s="7" t="inlineStr"/>
-      <c r="H21" s="7" t="inlineStr"/>
-      <c r="I21" s="7" t="inlineStr"/>
-      <c r="J21" s="7" t="inlineStr"/>
-      <c r="K21" s="7" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr"/>
+      <c r="C31" s="7" t="inlineStr"/>
+      <c r="D31" s="7" t="inlineStr"/>
+      <c r="E31" s="7" t="inlineStr"/>
+      <c r="F31" s="7" t="inlineStr"/>
+      <c r="G31" s="7" t="inlineStr"/>
+      <c r="H31" s="7" t="inlineStr"/>
+      <c r="I31" s="7" t="inlineStr"/>
+      <c r="J31" s="7" t="inlineStr"/>
+      <c r="K31" s="7" t="inlineStr">
         <is>
           <t>introuvable</t>
         </is>
       </c>
-      <c r="L21" s="7" t="inlineStr">
+      <c r="L31" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="M21" s="7" t="inlineStr"/>
-      <c r="N21" s="7" t="inlineStr"/>
-      <c r="O21" s="7" t="inlineStr"/>
-      <c r="P21" s="7" t="inlineStr"/>
-      <c r="Q21" s="7" t="inlineStr"/>
-      <c r="R21" s="7" t="inlineStr"/>
-      <c r="S21" s="7" t="inlineStr"/>
-      <c r="T21" s="7" t="inlineStr"/>
-      <c r="U21" s="7" t="inlineStr">
+      <c r="M31" s="7" t="inlineStr"/>
+      <c r="N31" s="7" t="inlineStr"/>
+      <c r="O31" s="7" t="inlineStr"/>
+      <c r="P31" s="7" t="inlineStr"/>
+      <c r="Q31" s="7" t="inlineStr"/>
+      <c r="R31" s="7" t="inlineStr"/>
+      <c r="S31" s="7" t="inlineStr"/>
+      <c r="T31" s="7" t="inlineStr"/>
+      <c r="U31" s="7" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/detail/10921931/true/false/false/true</t>
         </is>
       </c>
-      <c r="V21" s="7" t="inlineStr">
+      <c r="V31" s="7" t="inlineStr">
         <is>
           <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-16&amp;range=100-109&amp;tri=0</t>
         </is>
       </c>
-      <c r="W21" s="7" t="inlineStr">
+      <c r="W31" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">erreur: Page.goto: Timeout 90000ms exceeded.
 Call log:
   - navigating to "https://candidat.francetravail.fr/formations/detail/10921931/true/false/false/true", waiting until "networkidle"
 </t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Titre professionnel secrétaire assistant médico-administratif (FOAD)</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>OPENCLASSROOMS</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>75004 Paris</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>Formation a distance | 75004 Paris | France</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>Durée de 1084 heures (dont 280 heures en entreprise)</t>
-        </is>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>Prochaine session</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
-        </is>
-      </c>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>inscription@openclassrooms.com</t>
-        </is>
-      </c>
-      <c r="J22" s="5" t="inlineStr">
-        <is>
-          <t>inscription@openclassrooms.com</t>
-        </is>
-      </c>
-      <c r="K22" s="5" t="inlineStr">
-        <is>
-          <t>france_travail</t>
-        </is>
-      </c>
-      <c r="L22" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="M22" s="5" t="inlineStr">
-        <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="N22" s="5" t="inlineStr">
-        <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="O22" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
-      <c r="P22" s="5" t="inlineStr">
-        <is>
-          <t>Formation financée par France Travail</t>
-        </is>
-      </c>
-      <c r="Q22" s="5" t="inlineStr">
-        <is>
-          <t>À distance</t>
-        </is>
-      </c>
-      <c r="R22" s="5" t="inlineStr"/>
-      <c r="S22" s="5" t="inlineStr">
-        <is>
-          <t>7 projets professionnalisants vous permettront d'acquérir les compétences citées au dessus par la pratique.Vous réaliserez les projets suivants :P1 - Démarrez votre formation de secrétaire assistant médico-administratifP2 - Niveau 1 : Maîtrisez l'accueil et la gestion administrative en milieu médicalP3 - Niveau 2 : Développez vos compétences en rédaction, communication et outils numériques en milieuP4 - Réalisez votre mission en entrepriseP5 - Niveau 3 : Optimisez l'organisation, la sécuritéet la gestion des données sensibles en milieu médicalP6 - Niveau 4 : Améliorez la gestion des communications, données et environnements sanitairesP7 - Préparez votre fin de formation de secrétaire assistant médico-administratif | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T22" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel secrétaire assistant médico-administratif</t>
-        </is>
-      </c>
-      <c r="U22" s="5" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120327/true/false/true/true</t>
-        </is>
-      </c>
-      <c r="V22" s="5" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
-        </is>
-      </c>
-      <c r="W22" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Formation au concours d'ATSEM</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
-        <is>
-          <t>OPENCLASSROOMS</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>75004 Paris</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Formation a distance | 75004 Paris | France</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>Durée de 346 heures</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>Prochaine session</t>
-        </is>
-      </c>
-      <c r="H23" s="7" t="inlineStr">
-        <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
-        </is>
-      </c>
-      <c r="I23" s="6" t="inlineStr">
-        <is>
-          <t>inscription@openclassrooms.com</t>
-        </is>
-      </c>
-      <c r="J23" s="7" t="inlineStr">
-        <is>
-          <t>inscription@openclassrooms.com</t>
-        </is>
-      </c>
-      <c r="K23" s="7" t="inlineStr">
-        <is>
-          <t>france_travail</t>
-        </is>
-      </c>
-      <c r="L23" s="7" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="M23" s="7" t="inlineStr">
-        <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="N23" s="7" t="inlineStr">
-        <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="O23" s="7" t="inlineStr"/>
-      <c r="P23" s="7" t="inlineStr">
-        <is>
-          <t>Formation financée par France Travail</t>
-        </is>
-      </c>
-      <c r="Q23" s="7" t="inlineStr">
-        <is>
-          <t>À distance</t>
-        </is>
-      </c>
-      <c r="R23" s="7" t="inlineStr"/>
-      <c r="S23" s="7" t="inlineStr">
-        <is>
-          <t>5 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de préparation au concours ATSEM ; Projet 2 - Comprenez les institutions et le fonctionnement de l'école maternelle ; Projet 3 - Approfondissez le développement et les besoins des enfants de 0 à 6 ans ; Projet 4 - Maîtrisez la santé, la sécurité et les contours du métier d'ATSEM ; Projet 5 - Préparez-vous pour le concours ATSEM. | Organisme | OPENCLASSROOMS | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T23" s="7" t="inlineStr"/>
-      <c r="U23" s="7" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120328/true/false/true/true</t>
-        </is>
-      </c>
-      <c r="V23" s="7" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
-        </is>
-      </c>
-      <c r="W23" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Concours d'atsem (FOAD)</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Centre européen de formation</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>75004 Paris</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>Formation a distance | 75004 Paris | France</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>Prochaine session</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
-        </is>
-      </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>info@cenef.fr</t>
-        </is>
-      </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>info@cenef.fr</t>
-        </is>
-      </c>
-      <c r="K24" s="5" t="inlineStr">
-        <is>
-          <t>france_travail</t>
-        </is>
-      </c>
-      <c r="L24" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="M24" s="5" t="inlineStr">
-        <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="N24" s="5" t="inlineStr">
-        <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O24" s="5" t="inlineStr"/>
-      <c r="P24" s="5" t="inlineStr">
-        <is>
-          <t>Formation financée par France Travail</t>
-        </is>
-      </c>
-      <c r="Q24" s="5" t="inlineStr">
-        <is>
-          <t>À distance</t>
-        </is>
-      </c>
-      <c r="R24" s="5" t="inlineStr"/>
-      <c r="S24" s="5" t="inlineStr">
-        <is>
-          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T24" s="5" t="inlineStr"/>
-      <c r="U24" s="5" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
-        </is>
-      </c>
-      <c r="V24" s="5" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
-        </is>
-      </c>
-      <c r="W24" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
-        <is>
-          <t>Centre européen de formation</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>75004 Paris</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>Formation a distance | 75004 Paris | France</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="inlineStr">
-        <is>
-          <t>Prochaine session</t>
-        </is>
-      </c>
-      <c r="H25" s="7" t="inlineStr">
-        <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
-        </is>
-      </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>info@cenef.fr</t>
-        </is>
-      </c>
-      <c r="J25" s="7" t="inlineStr">
-        <is>
-          <t>info@cenef.fr</t>
-        </is>
-      </c>
-      <c r="K25" s="7" t="inlineStr">
-        <is>
-          <t>france_travail</t>
-        </is>
-      </c>
-      <c r="L25" s="7" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="M25" s="7" t="inlineStr">
-        <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="N25" s="7" t="inlineStr">
-        <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O25" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
-      <c r="P25" s="7" t="inlineStr">
-        <is>
-          <t>Formation financée par France Travail</t>
-        </is>
-      </c>
-      <c r="Q25" s="7" t="inlineStr">
-        <is>
-          <t>À distance</t>
-        </is>
-      </c>
-      <c r="R25" s="7" t="inlineStr"/>
-      <c r="S25" s="7" t="inlineStr">
-        <is>
-          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T25" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
-      <c r="U25" s="7" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
-        </is>
-      </c>
-      <c r="V25" s="7" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
-        </is>
-      </c>
-      <c r="W25" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Préparation au concours d'ATSEM</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>AFEC</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>75004 Paris</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>AFEC (Siège) | Formation a distance | 75004 Paris | France</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>Prochaine session</t>
-        </is>
-      </c>
-      <c r="H26" s="5" t="inlineStr">
-        <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
-        </is>
-      </c>
-      <c r="I26" s="5" t="inlineStr"/>
-      <c r="J26" s="5" t="inlineStr"/>
-      <c r="K26" s="5" t="inlineStr">
-        <is>
-          <t>introuvable</t>
-        </is>
-      </c>
-      <c r="L26" s="5" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M26" s="5" t="inlineStr"/>
-      <c r="N26" s="5" t="inlineStr"/>
-      <c r="O26" s="5" t="inlineStr"/>
-      <c r="P26" s="5" t="inlineStr">
-        <is>
-          <t>Formation financée par France Travail</t>
-        </is>
-      </c>
-      <c r="Q26" s="5" t="inlineStr">
-        <is>
-          <t>À distance</t>
-        </is>
-      </c>
-      <c r="R26" s="5" t="inlineStr"/>
-      <c r="S26" s="5" t="inlineStr">
-        <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC | Lieu de la formation | AFEC (Siège)</t>
-        </is>
-      </c>
-      <c r="T26" s="5" t="inlineStr"/>
-      <c r="U26" s="5" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
-        </is>
-      </c>
-      <c r="V26" s="5" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
-        </is>
-      </c>
-      <c r="W26" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
-        <is>
-          <t>Leo Lagrange Formation</t>
-        </is>
-      </c>
-      <c r="D27" s="7" t="inlineStr">
-        <is>
-          <t>75004 Paris</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>Formation a distance | 75004 Paris | France</t>
-        </is>
-      </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>Prochaine session</t>
-        </is>
-      </c>
-      <c r="H27" s="7" t="inlineStr">
-        <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
-        </is>
-      </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>contact@ifra.fr</t>
-        </is>
-      </c>
-      <c r="J27" s="7" t="inlineStr">
-        <is>
-          <t>contact@ifra.fr</t>
-        </is>
-      </c>
-      <c r="K27" s="7" t="inlineStr">
-        <is>
-          <t>france_travail</t>
-        </is>
-      </c>
-      <c r="L27" s="7" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="M27" s="7" t="inlineStr">
-        <is>
-          <t>0472892042</t>
-        </is>
-      </c>
-      <c r="N27" s="7" t="inlineStr">
-        <is>
-          <t>0472892042</t>
-        </is>
-      </c>
-      <c r="O27" s="7" t="inlineStr"/>
-      <c r="P27" s="7" t="inlineStr">
-        <is>
-          <t>Formation financée par France Travail</t>
-        </is>
-      </c>
-      <c r="Q27" s="7" t="inlineStr">
-        <is>
-          <t>À distance</t>
-        </is>
-      </c>
-      <c r="R27" s="7" t="inlineStr"/>
-      <c r="S27" s="7" t="inlineStr">
-        <is>
-          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T27" s="7" t="inlineStr"/>
-      <c r="U27" s="7" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
-        </is>
-      </c>
-      <c r="V27" s="7" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
-        </is>
-      </c>
-      <c r="W27" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Leo Lagrange Formation</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>75004 Paris</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>Formation a distance | 75004 Paris | France</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>Prochaine session</t>
-        </is>
-      </c>
-      <c r="H28" s="5" t="inlineStr">
-        <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
-        </is>
-      </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>contact@ifra.fr</t>
-        </is>
-      </c>
-      <c r="J28" s="5" t="inlineStr">
-        <is>
-          <t>contact@ifra.fr</t>
-        </is>
-      </c>
-      <c r="K28" s="5" t="inlineStr">
-        <is>
-          <t>france_travail</t>
-        </is>
-      </c>
-      <c r="L28" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="M28" s="5" t="inlineStr">
-        <is>
-          <t>0472892042</t>
-        </is>
-      </c>
-      <c r="N28" s="5" t="inlineStr">
-        <is>
-          <t>0472892042</t>
-        </is>
-      </c>
-      <c r="O28" s="5" t="inlineStr"/>
-      <c r="P28" s="5" t="inlineStr">
-        <is>
-          <t>Formation financée par France Travail</t>
-        </is>
-      </c>
-      <c r="Q28" s="5" t="inlineStr">
-        <is>
-          <t>À distance</t>
-        </is>
-      </c>
-      <c r="R28" s="5" t="inlineStr"/>
-      <c r="S28" s="5" t="inlineStr">
-        <is>
-          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T28" s="5" t="inlineStr"/>
-      <c r="U28" s="5" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
-        </is>
-      </c>
-      <c r="V28" s="5" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
-        </is>
-      </c>
-      <c r="W28" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
-        <is>
-          <t>OPENCLASSROOMS</t>
-        </is>
-      </c>
-      <c r="D29" s="7" t="inlineStr">
-        <is>
-          <t>75004 Paris</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>Formation a distance | 75004 Paris | France</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>Durée de 1350 heures (dont 490 heures en entreprise)</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
-        <is>
-          <t>Prochaine session</t>
-        </is>
-      </c>
-      <c r="H29" s="7" t="inlineStr">
-        <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
-        </is>
-      </c>
-      <c r="I29" s="6" t="inlineStr">
-        <is>
-          <t>inscription@openclassrooms.com</t>
-        </is>
-      </c>
-      <c r="J29" s="7" t="inlineStr">
-        <is>
-          <t>inscription@openclassrooms.com</t>
-        </is>
-      </c>
-      <c r="K29" s="7" t="inlineStr">
-        <is>
-          <t>france_travail</t>
-        </is>
-      </c>
-      <c r="L29" s="7" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="M29" s="7" t="inlineStr">
-        <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="N29" s="7" t="inlineStr">
-        <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="O29" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
-      <c r="P29" s="7" t="inlineStr">
-        <is>
-          <t>Formation financée par France Travail</t>
-        </is>
-      </c>
-      <c r="Q29" s="7" t="inlineStr">
-        <is>
-          <t>À distance</t>
-        </is>
-      </c>
-      <c r="R29" s="7" t="inlineStr"/>
-      <c r="S29" s="7" t="inlineStr">
-        <is>
-          <t>11 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 : Démarrez votre formation d'Accompagnement Educatif Petite Enfance ; Projet 2 - Préparez un environnement sécurisé pour le jeune enfant ; Projet 3 - Développez des activités éducatives adaptées à la petite enfance ; Projet 4 - Appliquez les protocoles de santé dans le cadre de la petite enfance ; Projet 5 - Soutenez le personnel enseignant dans un contexte collectif ; Projet 6 - Améliorez les conditions d'accueil en école maternelle ; Projet 7 - Organisez l'accueil individuel au domicile ; Projet 8 - Gérez les tâches domestiques et la préparation des repas pour l'enfant ; Projet 9 : Proposer des solutions de prévention, santé et environnement ; Projet 10 : Remise à niveau scolaire ; Projet 11 : Préparez-vous pour l'examen final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T29" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
-      <c r="U29" s="7" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120311/true/false/true/true</t>
-        </is>
-      </c>
-      <c r="V29" s="7" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
-        </is>
-      </c>
-      <c r="W29" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Conseiller emploi et accompagnement professionnel</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>OPENCLASSROOMS</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>75004 Paris</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Formation a distance | 75004 Paris | France</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>Durée de 1140 heures (dont 280 heures en entreprise)</t>
-        </is>
-      </c>
-      <c r="G30" s="5" t="inlineStr">
-        <is>
-          <t>Prochaine session</t>
-        </is>
-      </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
-        </is>
-      </c>
-      <c r="I30" s="6" t="inlineStr">
-        <is>
-          <t>inscription@openclassrooms.com</t>
-        </is>
-      </c>
-      <c r="J30" s="5" t="inlineStr">
-        <is>
-          <t>inscription@openclassrooms.com</t>
-        </is>
-      </c>
-      <c r="K30" s="5" t="inlineStr">
-        <is>
-          <t>france_travail</t>
-        </is>
-      </c>
-      <c r="L30" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="M30" s="5" t="inlineStr">
-        <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="N30" s="5" t="inlineStr">
-        <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="O30" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
-      <c r="P30" s="5" t="inlineStr">
-        <is>
-          <t>Formation financée par France Travail</t>
-        </is>
-      </c>
-      <c r="Q30" s="5" t="inlineStr">
-        <is>
-          <t>À distance</t>
-        </is>
-      </c>
-      <c r="R30" s="5" t="inlineStr"/>
-      <c r="S30" s="5" t="inlineStr">
-        <is>
-          <t>10 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de conseiller emploi et évolution professionnelle ; Projet 2 - Accompagnez en parallèle de nombreuses personnes avec des besoins différents ; Projet 3 - Élaborez une veille et analysez le marché de l'emploi ; Projet 4 - Réalisez un diagnostic et co-construisez un plan d'action avec vos bénéficiaires ; Projet 5 - Adaptez votre posture pour l'accompagnement des bénéficiaires ; Projet 6 - Établissez et validez un projet d'accompagnement professionnel ; Projet 7 - Établissez un plan d'action et un bilan professionnel ; Projet 8 - Concevez un atelier sur les métiers émergents avec l'IA ; Projet 9 - Développez votre projet territorial avec des partenaires ; Projet 10 - Élaborez votre boîte à outils pour accompagner vers l'emploi. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
-        </is>
-      </c>
-      <c r="T30" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Conseiller emploi et accompagnement professionnel</t>
-        </is>
-      </c>
-      <c r="U30" s="5" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120363/true/false/true/true</t>
-        </is>
-      </c>
-      <c r="V30" s="5" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
-        </is>
-      </c>
-      <c r="W30" s="5" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
-        <is>
-          <t>AFEC (Siège)</t>
-        </is>
-      </c>
-      <c r="D31" s="7" t="inlineStr">
-        <is>
-          <t>75004 Paris</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>Formation a distance | 75004 Paris | France</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Durée de 1015 heures (dont 490 heures en entreprise)</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="inlineStr">
-        <is>
-          <t>Prochaine session</t>
-        </is>
-      </c>
-      <c r="H31" s="7" t="inlineStr">
-        <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
-        </is>
-      </c>
-      <c r="I31" s="6" t="inlineStr">
-        <is>
-          <t>paris@afec.fr</t>
-        </is>
-      </c>
-      <c r="J31" s="7" t="inlineStr">
-        <is>
-          <t>paris@afec.fr</t>
-        </is>
-      </c>
-      <c r="K31" s="7" t="inlineStr">
-        <is>
-          <t>france_travail</t>
-        </is>
-      </c>
-      <c r="L31" s="7" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="M31" s="7" t="inlineStr">
-        <is>
-          <t>0153368844</t>
-        </is>
-      </c>
-      <c r="N31" s="7" t="inlineStr">
-        <is>
-          <t>0153368844</t>
-        </is>
-      </c>
-      <c r="O31" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
-      <c r="P31" s="7" t="inlineStr">
-        <is>
-          <t>Formation financée par France Travail</t>
-        </is>
-      </c>
-      <c r="Q31" s="7" t="inlineStr">
-        <is>
-          <t>À distance</t>
-        </is>
-      </c>
-      <c r="R31" s="7" t="inlineStr"/>
-      <c r="S31" s="7" t="inlineStr">
-        <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant des modules d'enseignement et des prestations d'accompagnement. Modules d'enseignement professionnel : - EP1 Accompagnement du développement du jeune enfant (cadre d'intervention, accompagnement à l'autonomie l'enfant) - EP2 Exercer son activité en accueil collectif - EP3 Exercer son activité en accueil individuel Modules d'enseignements généraux : - Prévention santé environnement - Enseignements généraux (Mathématiques et sciences, Histoire-Géographie-Citoyenneté et français) En complément de la formation : - Remise à niveau numérique - Techniques de recherche d'emploi et de stage - Accompagnement au retour à l'emploi 3 Stages en entreprise 14 semaines | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T31" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
-      <c r="U31" s="7" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124191/true/false/true/true</t>
-        </is>
-      </c>
-      <c r="V31" s="7" t="inlineStr">
-        <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-15&amp;range=110-119&amp;tri=0</t>
-        </is>
-      </c>
-      <c r="W31" s="7" t="inlineStr">
-        <is>
-          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-08-03
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,17 +932,17 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Concours d'atsem (FOAD)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1350 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -972,12 +972,12 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -992,19 +992,15 @@
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr"/>
       <c r="P4" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -1018,22 +1014,18 @@
       <c r="R4" s="5" t="inlineStr"/>
       <c r="S4" s="5" t="inlineStr">
         <is>
-          <t>11 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 : Démarrez votre formation d'Accompagnement Educatif Petite Enfance ; Projet 2 - Préparez un environnement sécurisé pour le jeune enfant ; Projet 3 - Développez des activités éducatives adaptées à la petite enfance ; Projet 4 - Appliquez les protocoles de santé dans le cadre de la petite enfance ; Projet 5 - Soutenez le personnel enseignant dans un contexte collectif ; Projet 6 - Améliorez les conditions d'accueil en école maternelle ; Projet 7 - Organisez l'accueil individuel au domicile ; Projet 8 - Gérez les tâches domestiques et la préparation des repas pour l'enfant ; Projet 9 : Proposer des solutions de prévention, santé et environnement ; Projet 10 : Remise à niveau scolaire ; Projet 11 : Préparez-vous pour l'examen final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T4" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
+          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr"/>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120311/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
         </is>
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1045,17 +1037,17 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Conseiller emploi et accompagnement professionnel</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -1070,7 +1062,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1140 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1085,12 +1077,12 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
@@ -1105,12 +1097,12 @@
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="O5" s="7" t="inlineStr">
@@ -1131,22 +1123,22 @@
       <c r="R5" s="7" t="inlineStr"/>
       <c r="S5" s="7" t="inlineStr">
         <is>
-          <t>10 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de conseiller emploi et évolution professionnelle ; Projet 2 - Accompagnez en parallèle de nombreuses personnes avec des besoins différents ; Projet 3 - Élaborez une veille et analysez le marché de l'emploi ; Projet 4 - Réalisez un diagnostic et co-construisez un plan d'action avec vos bénéficiaires ; Projet 5 - Adaptez votre posture pour l'accompagnement des bénéficiaires ; Projet 6 - Établissez et validez un projet d'accompagnement professionnel ; Projet 7 - Établissez un plan d'action et un bilan professionnel ; Projet 8 - Concevez un atelier sur les métiers émergents avec l'IA ; Projet 9 - Développez votre projet territorial avec des partenaires ; Projet 10 - Élaborez votre boîte à outils pour accompagner vers l'emploi. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
+          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Conseiller emploi et accompagnement professionnel</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120363/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
         </is>
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1158,32 +1150,32 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Certificat d'aptitude aux fonctions de directeur d'établissement ou de service d'intervention sociale (CAFDES)</t>
+          <t>Préparation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>INSTITUT REGIONAL SUPERIEUR DU TRAVAIL EDUCATIF ET SOCIAL (IRTESS de Dijon)</t>
+          <t>AFEC</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>21000 Dijon</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>2 Rue Professeur Marion | http://www.irtess.fr | 21000 Dijon | France</t>
+          <t>AFEC (Siège) | Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Durée de 700 heures</t>
+          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -1193,73 +1185,49 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>http://www.irtess.fr/</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>contact@irtess.fr</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>contact@irtess.fr</t>
-        </is>
-      </c>
+          <t>https://plmpl.fr/c/zFjGj</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr"/>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>france_travail</t>
+          <t>introuvable</t>
         </is>
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>0380726450</t>
-        </is>
-      </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>0380726450</t>
-        </is>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="inlineStr"/>
+      <c r="N6" s="5" t="inlineStr"/>
+      <c r="O6" s="5" t="inlineStr"/>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R6" s="5" t="inlineStr"/>
       <c r="S6" s="5" t="inlineStr">
         <is>
-          <t>Domaine de formation / modulesDeux possibilités d'envisager le rythme de la formation : Le candidat s'inscrit dans une démarche d'acquisition de la certification globale (4 blocs de compétences) sur 27 mois de septembre de l'année N à novembre de l'année N+2 ; Le candidat s'inscrit dans une démarche d'acquisition de blocs de compétences selon un rythme choisi et négocié avec le centre de formation. La certification sera réputée acquise lorsque le candidat aura validé les 4 blocs de compétences.Rappel : les blocs de compétences sont acquis à titre définitif.Formation théoriqueLa formation théorique de 700 h est organisée en 4 blocs de compétences définissant 4 domaines de formation :BC1/DF1 : Participer à l'élaboration de projets stratégiques en lien avec la mise en uvre des politiques publiques (196 h)BC2/DF2 : Définir et piloter le projet d'établissement ou de service établissement ou service (154 h)BC3/DF3 : Manager et gérer les ressources humaines de l'établissement ou de service (196 h)BC4/DF4 : Gérer les volets économique, financier et logistique de l'établissement ou de service (154 h)Formation pratiqueLa formation pratique de 510 h (allègements possibles de 1/3 à 2/3 selon expérience, statut et fonction) Elle consiste en : 2 stages dans le cadre d'un parcours continu ; 1 stage par blocs de compétences dans le cadre d'un parcours discontinu (par blocs de compétences) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T6" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Certificat d'aptitude aux fonctions de directeur d'établissement ou de service d'intervention sociale</t>
-        </is>
-      </c>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC | Lieu de la formation | AFEC (Siège)</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr"/>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10941347/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1271,32 +1239,32 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>INSTITUT DE FORMATION EN SOINS INFIRMIERS DE BEAUNE (IFSI de Beaune)</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>21200 Beaune</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Avenue Guigone de Salins | https://ifsi.hospices-de-beaune.com/ | 21200 Beaune | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1306,17 +1274,17 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>https://ifsi.hospices-de-beaune.com/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>lst.sec.ifsi@ch-beaune.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>lst.sec.ifsi@ch-beaune.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
@@ -1331,48 +1299,40 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>0380244449</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>0380244449</t>
-        </is>
-      </c>
-      <c r="O7" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr"/>
       <c r="S7" s="7" t="inlineStr">
         <is>
-          <t>La formation en soins infirmiers s'articule autour de l'acquisition de 10 compétences :C1 : Évaluer une situation clinique et établir un diagnostic dans le domaine infirmierC2 : Concevoir et conduire un projet de soins infirmiersC3 : Accompagner la personne dans la réalisation de ses soins quotidiensC4 : Mettre en uvre des actions à visée diagnostique et thérapeutiquesC5 : Initier et mettre en uvre des soins éducatifs et préventifsC6 : Communiquer et conduire une relation dans un contexte de soinsC7 : Analyser la qualité des soins et améliorer sa pratique professionnelleC8 : Rechercher et traiter des données professionnelles et scientifiquesC9 : Organiser et coordonner des interventions soignantesC10 : Informer et former des professionnels et des personnes en formationDes unités d'enseignement en :UG 01. Sciences humaines et socialesUG 02. Sciences biologiques et médicalesUG 03. Sciences et techniques infirmières, fondements et méthodesUG 04. Sciences et techniques infirmières, interventionsUG 05. Intégration des savoirs et posture professionnelle infirmièreUG 06. Méthodes de travail | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T7" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
-        </is>
-      </c>
+          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T7" s="7" t="inlineStr"/>
       <c r="U7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11022070/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
         </is>
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1384,32 +1344,32 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'assistant de service social (DEASS)</t>
+          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>INSTITUT REGIONAL SUPERIEUR DU TRAVAIL EDUCATIF ET SOCIAL (IRTESS de Dijon)</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>21000 Dijon</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>2 Rue Professeur Marion | http://www.irtess.fr | 21000 Dijon | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Durée de 3560 heures (dont 1820 heures en entreprise)</t>
+          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -1419,17 +1379,17 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>http://www.irtess.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>contact@irtess.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>contact@irtess.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1444,48 +1404,40 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>0380726450</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>0380726450</t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr"/>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q8" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>1 740 h de formation théorique et pratique réparties en 8 unités de formation, 12 mois de stage dont 6 mois au moins auprès d'un professionnel assistant de service social. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T8" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
-        </is>
-      </c>
+          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11024875/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
         </is>
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1497,32 +1449,32 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>CROIX ROUGE FRANCAISE (Croix-Rouge Compétence (ex IRFSS) - Site de Quetigny)</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>21800 Quetigny</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>2 Rue du Golf | http://irfss-bourgogne-franche-comte.croix-rouge.fr/ | 21800 Quetigny | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 1350 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1532,17 +1484,17 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>http://irfss-bourgogne-franche-comte.croix-rouge.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>irfss.quetigny@croix-rouge.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>irfss.quetigny@croix-rouge.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
@@ -1557,12 +1509,12 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>0380481735</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>0380481735</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O9" s="7" t="inlineStr">
@@ -1572,33 +1524,33 @@
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R9" s="7" t="inlineStr"/>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>La formation en soins infirmiers s'articule autour de l'acquisition de 10 compétences :C1 : Évaluer une situation clinique et établir un diagnostic dans le domaine infirmierC2 : Concevoir et conduire un projet de soins infirmiersC3 : Accompagner la personne dans la réalisation de ses soins quotidiensC4 : Mettre en uvre des actions à visée diagnostique et thérapeutiquesC5 : Initier et mettre en uvre des soins éducatifs et préventifsC6 : Communiquer et conduire une relation dans un contexte de soinsC7 : Analyser la qualité des soins et améliorer sa pratique professionnelleC8 : Rechercher et traiter des données professionnelles et scientifiquesC9 : Organiser et coordonner des interventions soignantesC10 : Informer et former des professionnels et des personnes en formationDes unités d'enseignement en :UG 01. Sciences humaines et socialesUG 02. Sciences biologiques et médicalesUG 03. Sciences et techniques infirmières, fondements et méthodesUG 04. Sciences et techniques infirmières, interventionsUG 05. Intégration des savoirs et posture professionnelle infirmièreUG 06. Méthodes de travail | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>11 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 : Démarrez votre formation d'Accompagnement Educatif Petite Enfance ; Projet 2 - Préparez un environnement sécurisé pour le jeune enfant ; Projet 3 - Développez des activités éducatives adaptées à la petite enfance ; Projet 4 - Appliquez les protocoles de santé dans le cadre de la petite enfance ; Projet 5 - Soutenez le personnel enseignant dans un contexte collectif ; Projet 6 - Améliorez les conditions d'accueil en école maternelle ; Projet 7 - Organisez l'accueil individuel au domicile ; Projet 8 - Gérez les tâches domestiques et la préparation des repas pour l'enfant ; Projet 9 : Proposer des solutions de prévention, santé et environnement ; Projet 10 : Remise à niveau scolaire ; Projet 11 : Préparez-vous pour l'examen final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11028875/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120311/true/false/true/true</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1610,32 +1562,32 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>Conseiller emploi et accompagnement professionnel</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>INSTITUT DE FORMATION EN SOINS INFIRMIERS ET D'AIDES-SOIGNANTS DE HAUTE COTE-D'OR (IFSI-IFAS de Haute Côte-d'Or)</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>21140 Semur-en-Auxois</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>3bis Avenue Pasteur | http://ifsi-semur-hco.fr | 21140 Semur-en-Auxois | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 1140 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1645,17 +1597,17 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>http://ifsi-semur-hco.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>secretariat.ifsi@ch-semur.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>secretariat.ifsi@ch-semur.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1670,12 +1622,12 @@
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>0380896442</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>0380896442</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -1685,33 +1637,33 @@
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q10" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>La durée est de 3 ans, sur la base de 35 heures / semaine.Soit 6 semestres, pour un total de 4200 heures : 2100 heures de formation théorique 2100 heures de formation cliniqueEnseignements théoriques réalisés sous la forme de : Cours magistraux Travaux dirigés Travaux personnels guidés Travaux de groupes Travaux pratiques Travaux de recherche en groupes ou individuelsEnseignement clinique : Il s'effectue au cours des périodes de stage.Les stages sont à la fois, des lieux d'intégration des connaissances construites par l'étudiant et des lieux d'acquisition de nouvelles connaissances par la voie de : l'observation la contribution aux soins la prise en charge des personnes la participation aux réflexions menées en équipe l'utilisation des savoirs dans la résolution de situation | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>10 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de conseiller emploi et évolution professionnelle ; Projet 2 - Accompagnez en parallèle de nombreuses personnes avec des besoins différents ; Projet 3 - Élaborez une veille et analysez le marché de l'emploi ; Projet 4 - Réalisez un diagnostic et co-construisez un plan d'action avec vos bénéficiaires ; Projet 5 - Adaptez votre posture pour l'accompagnement des bénéficiaires ; Projet 6 - Établissez et validez un projet d'accompagnement professionnel ; Projet 7 - Établissez un plan d'action et un bilan professionnel ; Projet 8 - Concevez un atelier sur les métiers émergents avec l'IA ; Projet 9 - Développez votre projet territorial avec des partenaires ; Projet 10 - Élaborez votre boîte à outils pour accompagner vers l'emploi. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
         </is>
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Conseiller emploi et accompagnement professionnel</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11068856/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120363/true/false/true/true</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1723,32 +1675,32 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>INSTITUT DE FORMATION EN SOINS INFIRMIERS DE DIJON (IFSI de Dijon)</t>
+          <t>AFEC (Siège)</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>21000 Dijon</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>12 Boulevard marechal de Lattre de Tassigny | https://campus-paramedical.chu-dijon.fr/Filiere/infirmiers/ | 21000 Dijon | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1758,17 +1710,17 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>https://campus-paramedical.chu-dijon.fr/Filiere/infirmiers/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>secretariat.ifsi@chu-dijon.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>secretariat.ifsi@chu-dijon.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1783,12 +1735,12 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>0380293502</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>0380293502</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="O11" s="7" t="inlineStr">
@@ -1798,33 +1750,33 @@
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travailLa formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de 2 100 heures, sous la forme de cours magistraux (750 heures) travaux dirigés (1 050 heures) et travail personnel guidé (300 heures) ; la formation clinique de 2 100 heures le travail personnel complémentaire est estimé à 900 heures environ, soit 300 heures par anModules : UG 01. Sciences humaines et sociales UG 02. Sciences biologiques et médicales UG 03. Sciences et techniques infirmières, fondements et méthodes UG 04. Sciences et techniques infirmières, interventions UG 05. Intégration des savoirs et posture professionnelle infirmière UG 06. Méthodes de travail | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant des modules d'enseignement et des prestations d'accompagnement. Modules d'enseignement professionnel : - EP1 Accompagnement du développement du jeune enfant (cadre d'intervention, accompagnement à l'autonomie l'enfant) - EP2 Exercer son activité en accueil collectif - EP3 Exercer son activité en accueil individuel Modules d'enseignements généraux : - Prévention santé environnement - Enseignements généraux (Mathématiques et sciences, Histoire-Géographie-Citoyenneté et français) En complément de la formation : - Remise à niveau numérique - Techniques de recherche d'emploi et de stage - Accompagnement au retour à l'emploi 3 Stages en entreprise 14 semaines | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11119576/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124191/true/false/true/true</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1836,32 +1788,32 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Employé(e) polyvalent(e) en restauration (TP) [HSP 1er NQ]</t>
+          <t>Certificat d'aptitude aux fonctions de directeur d'établissement ou de service d'intervention sociale (CAFDES)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>GRETA DU LIMOUSIN</t>
+          <t>INSTITUT REGIONAL SUPERIEUR DU TRAVAIL EDUCATIF ET SOCIAL (IRTESS de Dijon)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>19100 Brive-la-Gaillarde</t>
+          <t>21000 Dijon</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>AFPA - CENTRE DE BRIVE | 53 Rue MAURICE ROLLINAT | 19100 Brive-la-Gaillarde | France</t>
+          <t>2 Rue Professeur Marion | http://www.irtess.fr | 21000 Dijon | France</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 700 heures</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1871,17 +1823,17 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>https://greta-du-limousin.fr/</t>
+          <t>http://www.irtess.fr/</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr</t>
+          <t>contact@irtess.fr</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr | formations-brive@afpa.fr</t>
+          <t>contact@irtess.fr</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1896,12 +1848,12 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>0685201025</t>
+          <t>0380726450</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>0685201025</t>
+          <t>0380726450</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr">
@@ -1922,22 +1874,22 @@
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>TITRE PRO AGENT DE RESTAURATION Intégration - Entrée en formationPrésentation de l'équipe pédagogique et administrativeVisite des locaux de formation (salles et plateaux techniques)Intégration au groupeFormalisation du parcours de formationInstruction du dossier et sécurisation administrativeExplicitation du calendrier de l'alternance et de l'emploi du temps de formationLecture et explication du Règlement Intérieur - 3 hTITRE PRO AGENT DE RESTAURATION Présentation du métier - Présentation du secteur "Hôtellerie-Restauration-Alimentation" (HRA)Intervention d'un professionnel / témoignage d'anciens stagiaires - 7 hTITRE PRO AGENT DE RESTAURATION Les modalités de certification - Présentation des modalités de certificationLe référentiel de formation et de certification TITRE PROFESSIONNEL Agent de restaurationLe calendrier prévisionnel des épreuves - 4 hTITRE PRO AGENT DES RESTAURATION Diagnostic - Positionnement - Positionnements écritsPositionnements pratiquesEntretien individuel exploratoire de confirmation de projetBilan - exploitation des positionnementsSynthèse et proposition de parcoursSignature du Contrat Pédagogique - 14 hTITRE PRO AGENT DE RESTAURATION Acquisition des connaissances et des compétences culinaires de base - Les principes et règlementation en matière de sécurité alimentaire (Codex alimentarius, GBPH, PMS, méthodologie HACCP,Le vocabulaire culinaire de base et la technologie culinaire : les produits alimentaires (denrées végétales, carnées, condiments, épices, produits dérivés, laitiers... les bases des méthodes de conservation, de cuisson- les principaux matériels et ustensiles culinaires- les préparations de base : fruits, légumes, oeufs, viandes, poissons, entremets, pâtisseries- les principales techniques d'assemblage - 28 hTITRE PRO AGENT DES RESTAURATION Préparer en assemblage des hors d'oeuvre, des desserts et des préparations de type "snacking" (CCP 1) - - Préparer les matières premières alimentaires destinées à la transformation et à l'assemblage - Réaliser l'assemblage et le dressage des hors-d'oeuvre, des desserts et des préparations de type snacking - 56 hTITRE PRO AGENT DE RESTAURATION Réaliser des grillades et remettre en température des PCEA Préparations Culinaires Elaborées à l'Avance) (CCP 2) - - Effectuer la remise en température de préparations culinaire | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Domaine de formation / modulesDeux possibilités d'envisager le rythme de la formation : Le candidat s'inscrit dans une démarche d'acquisition de la certification globale (4 blocs de compétences) sur 27 mois de septembre de l'année N à novembre de l'année N+2 ; Le candidat s'inscrit dans une démarche d'acquisition de blocs de compétences selon un rythme choisi et négocié avec le centre de formation. La certification sera réputée acquise lorsque le candidat aura validé les 4 blocs de compétences.Rappel : les blocs de compétences sont acquis à titre définitif.Formation théoriqueLa formation théorique de 700 h est organisée en 4 blocs de compétences définissant 4 domaines de formation :BC1/DF1 : Participer à l'élaboration de projets stratégiques en lien avec la mise en uvre des politiques publiques (196 h)BC2/DF2 : Définir et piloter le projet d'établissement ou de service établissement ou service (154 h)BC3/DF3 : Manager et gérer les ressources humaines de l'établissement ou de service (196 h)BC4/DF4 : Gérer les volets économique, financier et logistique de l'établissement ou de service (154 h)Formation pratiqueLa formation pratique de 510 h (allègements possibles de 1/3 à 2/3 selon expérience, statut et fonction) Elle consiste en : 2 stages dans le cadre d'un parcours continu ; 1 stage par blocs de compétences dans le cadre d'un parcours discontinu (par blocs de compétences) | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T12" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé polyvalent en restauration</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Certificat d'aptitude aux fonctions de directeur d'établissement ou de service d'intervention sociale</t>
         </is>
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10921927/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10941347/true/false/false/true</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-19&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -1949,32 +1901,32 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Serveur, Serveuse en hôtellerie-restauration (TP) [HSP 1er NQ]</t>
+          <t>Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>GRETA DU LIMOUSIN</t>
+          <t>INSTITUT DE FORMATION EN SOINS INFIRMIERS DE BEAUNE (IFSI de Beaune)</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>19100 Brive-la-Gaillarde</t>
+          <t>21200 Beaune</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>AFPA - CENTRE DE BRIVE | 53 Rue MAURICE ROLLINAT | 19100 Brive-la-Gaillarde | France</t>
+          <t>Avenue Guigone de Salins | https://ifsi.hospices-de-beaune.com/ | 21200 Beaune | France</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1984,17 +1936,17 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>https://greta-du-limousin.fr/</t>
+          <t>https://ifsi.hospices-de-beaune.com/</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr</t>
+          <t>lst.sec.ifsi@ch-beaune.fr</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr | formations-brive@afpa.fr</t>
+          <t>lst.sec.ifsi@ch-beaune.fr</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
@@ -2009,12 +1961,12 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>0685201025</t>
+          <t>0380244449</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>0685201025</t>
+          <t>0380244449</t>
         </is>
       </c>
       <c r="O13" s="7" t="inlineStr">
@@ -2035,22 +1987,22 @@
       <c r="R13" s="7" t="inlineStr"/>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>CAP CS en HCR Intégration - Entrée en formationPrésentation de l'équipe pédagogique et administrativeVisite des locaux de formation (salles et plateaux techniques)Intégration au groupeFormalisation du parcours de formationInstruction du dossier et sécurisation administrativeExplicitation du calendrier de l'alternance et de l'emploi du temps de formationLecture et explication du Règlement Intérieur - 3 hCAP CS en HCR Présentation du métier - Présentation du secteur "Hôtellerie-Restauration-Alimentation" (HRA)Intervention d'un professionnel / témoignage d'anciens stagiaires - 7 hCAP CS en HCR Les modalités de certification - Présentation des modalités de certificationLes modalités de Contrôle en Cours de Formation (CCF) en ponctuel pour l'EIMCL 13 VentsLe référentiel de formation et de certification CAP HCRLe calendrier prévisionnel des épreuves - 4 hCAP CS en HCR Diagnostic - Positionnement - Positionnements écritsPositionnements pratiquesEntretien individuel exploratoire de confirmation de projetBilan - exploitation des positionnementsSynthèse et proposition de parcoursSignature du Contrat Pédagogique - 21 hCAP CS en HCR UP1 - Organisation des prestations en HCR - Réceptionner contrôler et stocker les marchandises1 - Les produits alimentaires et les boissons2 - Les autres produits3 - Les fournisseurs4 - Les mesures d'hygiène et de sécurité dans les locaux professionnels5 - Les stocks et les approvisionnementsCollecter les informations et ordonnancer ses activités6 - L'approche économique7 - Les locaux, les équipements et matériels8 - La prévention des risques liés à l'activité9 - Les différents types de prestations en restauration10 - Les supports et les documents liés aux prestations - 46 hCAP CS en HCR UP2 - Accueil, commercialisation et services en HCR - Accueillir, prendre en charge, renseigner le client et contribuer à la vente des prestations11 - Le client12 - Les points clés de la relation client13 - La réservation14 - Les supports de vente Thème15 - La prise de commande16 - Les étapes de la venteMettre en oeuvre les techniques de mise en place et de préparation17 - Les protocoles de nettoyage et d'entretien18 - La démarche de développement durable19 - Les mises en place20 - Les locaux annexes21 - Les techniques de préparation en restaurant - 137 hCAP CS en HCR UP2 - Accueil, commercialisation et services en HCR - Mettre en | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>La formation en soins infirmiers s'articule autour de l'acquisition de 10 compétences :C1 : Évaluer une situation clinique et établir un diagnostic dans le domaine infirmierC2 : Concevoir et conduire un projet de soins infirmiersC3 : Accompagner la personne dans la réalisation de ses soins quotidiensC4 : Mettre en uvre des actions à visée diagnostique et thérapeutiquesC5 : Initier et mettre en uvre des soins éducatifs et préventifsC6 : Communiquer et conduire une relation dans un contexte de soinsC7 : Analyser la qualité des soins et améliorer sa pratique professionnelleC8 : Rechercher et traiter des données professionnelles et scientifiquesC9 : Organiser et coordonner des interventions soignantesC10 : Informer et former des professionnels et des personnes en formationDes unités d'enseignement en :UG 01. Sciences humaines et socialesUG 02. Sciences biologiques et médicalesUG 03. Sciences et techniques infirmières, fondements et méthodesUG 04. Sciences et techniques infirmières, interventionsUG 05. Intégration des savoirs et posture professionnelle infirmièreUG 06. Méthodes de travail | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel serveur en restauration</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10921937/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11022070/true/false/false/true</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-19&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W13" s="7" t="inlineStr">
@@ -2062,32 +2014,32 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Commis de cuisine (TP) [HSP 1er NQ]</t>
+          <t>Diplôme d'État d'assistant de service social (DEASS)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>GRETA DU LIMOUSIN</t>
+          <t>INSTITUT REGIONAL SUPERIEUR DU TRAVAIL EDUCATIF ET SOCIAL (IRTESS de Dijon)</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>19100 Brive-la-Gaillarde</t>
+          <t>21000 Dijon</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>AFPA - CENTRE DE BRIVE | 53 Rue MAURICE ROLLINAT | 19100 Brive-la-Gaillarde | France</t>
+          <t>2 Rue Professeur Marion | http://www.irtess.fr | 21000 Dijon | France</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 3560 heures (dont 1820 heures en entreprise)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -2097,17 +2049,17 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>https://greta-du-limousin.fr/</t>
+          <t>http://www.irtess.fr/</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr</t>
+          <t>contact@irtess.fr</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr | formations-brive@afpa.fr</t>
+          <t>contact@irtess.fr</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -2122,12 +2074,12 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>0685201025</t>
+          <t>0380726450</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>0685201025</t>
+          <t>0380726450</t>
         </is>
       </c>
       <c r="O14" s="5" t="inlineStr">
@@ -2148,22 +2100,22 @@
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>CAP CUISINE Intégration - Entrée en formationPrésentation de l'équipe pédagogique et administrativeVisite des locaux de formation (salles et plateaux techniques)Intégration au groupeFormalisation du parcours de formationInstruction du dossier et sécurisation administrativeExplicitation du calendrier de l'alternance et de l'emploi du temps de formationLecture et explication du Règlement Intérieur - 3 hCAP CUISINE Présentation du métier - Présentation du secteur "Hôtellerie-Restauration-Alimentation" (HRA)Intervention d'un professionnel / témoignage d'anciens stagiaires - 7 hCAP CUISINE Les modalités de certification - Présentation des modalités de certificationLes modalités de Contrôle en Cours de Formation (CCF)Le référentiel de formation et de certification CAP CuisineLe calendrier prévisionnel des épreuves - 4 hCAP CUISINE Diagnostic - Positionnement - Positionnements écritsPositionnements pratiquesEntretien individuel exploratoire de confirmation de projetBilan - exploitation des positionnementsSynthèse et proposition de parcoursSignature du Contrat Pédagogique - 21 hCAP CUISINE UP 1 - Organisation de la production de cuisine - 1 - Réceptionner, contrôler et stocker les marchandises dans le respect de la réglementation en vigueur et en appliquant les techniques de préventions liées à l'activité2 - Collecter l'ensemble des informations et organiser sa production culinaire dans le respect des consignes et de temps imparti - 63 hCAP CUISINE UP 2 - Préparation et distribution de la production en cuisine - 1 - Préparer, organiser et maintenir en état son poste de travail tout au long de l'activité dans le respect de la réglementation en vigueur2 - Maîtriser les techniques culinaires de base et réaliser une production dans le respect des consignes et des règles d'hygiène et de sécurité3 - Analyser, contrôler la qualité de sa production, dresser et participer à la distribution selon le contexte professionnel4 - Communiquer en fonction du contexte professionnel et en respectant les usages de la profession - 378 hCAP CUISINE Français - Histoire-Géographie - Enseignement Moral et Civique - FRANCAIS- Entrer dans l'échange oral et écrit : écouter, réagir, s'exprimer, lire, analyser, écrire- Devenir un lecteur compétent et critique- Confronter des savoirs et des valeurs pour construire son identité culturelle.HISTOIRE GEOGRAPHI | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>1 740 h de formation théorique et pratique réparties en 8 unités de formation, 12 mois de stage dont 6 mois au moins auprès d'un professionnel assistant de service social. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T14" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel commis de cuisine</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'assistant de service social</t>
         </is>
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10921959/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11024875/true/false/false/true</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-19&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
@@ -2175,32 +2127,32 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Assistant(e) de vie aux familles (TP) [HSP 1er NQ]</t>
+          <t>Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>GRETA DU LIMOUSIN</t>
+          <t>CROIX ROUGE FRANCAISE (Croix-Rouge Compétence (ex IRFSS) - Site de Quetigny)</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>19100 Brive-la-Gaillarde</t>
+          <t>21800 Quetigny</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>AFPA - CENTRE DE BRIVE | 53 Rue MAURICE ROLLINAT | 19100 Brive-la-Gaillarde | France</t>
+          <t>2 Rue du Golf | http://irfss-bourgogne-franche-comte.croix-rouge.fr/ | 21800 Quetigny | France</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2210,17 +2162,17 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>https://greta-du-limousin.fr/</t>
+          <t>http://irfss-bourgogne-franche-comte.croix-rouge.fr/</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr</t>
+          <t>irfss.quetigny@croix-rouge.fr</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr | formations-brive@afpa.fr</t>
+          <t>irfss.quetigny@croix-rouge.fr</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -2235,12 +2187,12 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>0685201025</t>
+          <t>0380481735</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>0685201025</t>
+          <t>0380481735</t>
         </is>
       </c>
       <c r="O15" s="7" t="inlineStr">
@@ -2261,22 +2213,22 @@
       <c r="R15" s="7" t="inlineStr"/>
       <c r="S15" s="7" t="inlineStr">
         <is>
-          <t>Intégration-présentation de la formation - Intégration au groupe et à la formationFormalisation des parcours et sécurisation administrativeFinalisation des dossiers de rémunérationRappel des plannings, emploi du tempsRappel du règlement intérieur - 4 hDiagnostic / Positionnement - Positionnements écritsEntretien individuel exploratoireBilan - synthèse et proposition de parcours - 7 hPrésentation du métier et du secteur - Présentation du secteur santé social Intervention de professionnels Fonctions et place de l'ADVFDroits et devoirs dans l'exercice du métier - 21 hModule Réussir sa formation en centre de formation et en entreprise - Modules sur les savoirs de base appliqués au secteur professionnel : mathématiques, français appliqués au secteur, informatiqueTechniques de recherche de stage, FLIRenforcement de l'acquisition de compétences comportementales. Méthodologie d'apprentissage apprendre à apprendre PAE *Préparation : -Définition des objectifs individuels,choix du type d'entreprise et/ou du service,mise à disposition et aide à la recherche de liste d'adresses et contacts,accompagnement à la démarche de recherche, entretien, négociation.Accompagnement : suivi et bilan en entreprise (stagiai - 63 hCCP 1 : Entretenir le logement et le linge d'un particulier - Relation professionnelle dans le cadre d'une prestation d'entretien chez un particulierCommunication professionnelle et relation avec la personne aidéePrévention des risques domestiques et travail en sécurité au domicile d'un particulierOrganisation du travailEntretien du logement avec les techniques et les gestes professionnels appropriésEntretien du linge (produits et techniques) repassage et initiation à la coutureRespect des règles environnementales/Hygiène et sécuritéEvaluation en cours de formation (mise en situation et écrit) - 126 hCCP 2 : Accompagner la personne dans les actes essentiels du quotidien - La relation avec la personne aidée et son entourageLes besoins fondamentauxLe handicapVieillissement et pathologies associées.Prévention des risques professionnelsL'autonomie physique, intellectuelle et sociale de la personneMobilisation et ergonomie / transferts et déplacementsAide à la toilette, à l'habillage et aux déplacementsAnimation et vie sociale.Aide aux courses, à la préparation et à la prise des repas Diététique et hygiène alimentair | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>La formation en soins infirmiers s'articule autour de l'acquisition de 10 compétences :C1 : Évaluer une situation clinique et établir un diagnostic dans le domaine infirmierC2 : Concevoir et conduire un projet de soins infirmiersC3 : Accompagner la personne dans la réalisation de ses soins quotidiensC4 : Mettre en uvre des actions à visée diagnostique et thérapeutiquesC5 : Initier et mettre en uvre des soins éducatifs et préventifsC6 : Communiquer et conduire une relation dans un contexte de soinsC7 : Analyser la qualité des soins et améliorer sa pratique professionnelleC8 : Rechercher et traiter des données professionnelles et scientifiquesC9 : Organiser et coordonner des interventions soignantesC10 : Informer et former des professionnels et des personnes en formationDes unités d'enseignement en :UG 01. Sciences humaines et socialesUG 02. Sciences biologiques et médicalesUG 03. Sciences et techniques infirmières, fondements et méthodesUG 04. Sciences et techniques infirmières, interventionsUG 05. Intégration des savoirs et posture professionnelle infirmièreUG 06. Méthodes de travail | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel assistant de vie aux familles</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10925822/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11028875/true/false/false/true</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-19&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W15" s="7" t="inlineStr">
@@ -2288,32 +2240,32 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Fraiseur, fraiseuse en réalisation de pièces mécaniques (TP) [HSP 1er NQ]</t>
+          <t>Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>INSTITUT DE FORMATION EN SOINS INFIRMIERS ET D'AIDES-SOIGNANTS DE HAUTE COTE-D'OR (IFSI-IFAS de Haute Côte-d'Or)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>19600 Saint-Pantaléon-de-Larche</t>
+          <t>21140 Semur-en-Auxois</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>AFPA - CENTRE DE BRIVE | 1 Rue de Laumeil | 19600 Saint-Pantaléon-de-Larche | France</t>
+          <t>3bis Avenue Pasteur | http://ifsi-semur-hco.fr | 21140 Semur-en-Auxois | France</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2323,17 +2275,17 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
+          <t>http://ifsi-semur-hco.fr/</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+          <t>secretariat.ifsi@ch-semur.fr</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-brives@afpa.fr</t>
+          <t>secretariat.ifsi@ch-semur.fr</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -2348,12 +2300,12 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>0685201025</t>
+          <t>0380896442</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>0685201025</t>
+          <t>0380896442</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr">
@@ -2374,22 +2326,22 @@
       <c r="R16" s="5" t="inlineStr"/>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>TP FRPM - Période d'intégration - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi S'initier à Métis Développer son autonomie en formation - 35 hTP FRPM - Fraiser des pièces, à l'unité ou en petites séries sur machine conventionnelle - Réaliser des opérations de fraisage broche verticale à partir d'un mode opératoire établiRéaliser des opérations courantes de fraisage , broche verticale, horizontale ou inclinée, de qualité 8, à partir d'un mode opératoire établiRéaliser des opérations spécifiques de fraisage, broche verticale, horizontale ou inclinée, de qualité 8, à partir d'un mode opératoire établiRéaliser des opérations de fraisage broche verticale, horizontale ou inclinée avec une précision de qualité 7 et mode opératoire à établir - 385 hTP FRPM - Régler un centre d'usinage pour produire des séries stabilisées de pièces - Réaliser l'usinage de pièces mécaniques sur un centre d'usinage réglé Préparer hors machine, tous les éléments nécessaires aux réglages d'une production sur centre d'usinage Monter et régler l'outillage nécessaire à l'usinage d'une série de pièces sur un centre d'usinage Mettre au point une production et usiner une pré-série sur un centre d'usinage - 210 hTP FRPM - Réaliser, à partir d'un plan, l'usinage de pièces unitaires ou de petites séries sur centre d'usinage - Réaliser, à partir d'un dossier de fabrication stabilisé, l'usinage de pièces unitaires ou de petites séries sur un centre d'usinagePréparer l'usinage par procédé de fraisage d'une pièce unitaire ou d'une petite série de pièces à partir d'un plan de pièceMettre au point l'usinage d'une nouvelle pièce sur un centre d'usinage - 280 hTP FRPM - Période Entreprise - Contractualiser les objectifs de la période en entreprise Ancrer ses acquis en situation réelle de travail Développer des compétences transversales Accroître son réseau pour une insertion professionnelle - 175 | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>La durée est de 3 ans, sur la base de 35 heures / semaine.Soit 6 semestres, pour un total de 4200 heures : 2100 heures de formation théorique 2100 heures de formation cliniqueEnseignements théoriques réalisés sous la forme de : Cours magistraux Travaux dirigés Travaux personnels guidés Travaux de groupes Travaux pratiques Travaux de recherche en groupes ou individuelsEnseignement clinique : Il s'effectue au cours des périodes de stage.Les stages sont à la fois, des lieux d'intégration des connaissances construites par l'étudiant et des lieux d'acquisition de nouvelles connaissances par la voie de : l'observation la contribution aux soins la prise en charge des personnes la participation aux réflexions menées en équipe l'utilisation des savoirs dans la résolution de situation | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel fraiseur en réalisation de pièces mécaniques</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10926897/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11068856/true/false/false/true</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-19&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W16" s="5" t="inlineStr">
@@ -2401,32 +2353,32 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>19</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Agent(e) de propreté et d'hygiène (TP) [HSP 1er NQ]</t>
+          <t>Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>GRETA DU LIMOUSIN</t>
+          <t>INSTITUT DE FORMATION EN SOINS INFIRMIERS DE DIJON (IFSI de Dijon)</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>19100 Brive-la-Gaillarde</t>
+          <t>21000 Dijon</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>AFPA - CENTRE DE BRIVE | 53 Rue MAURICE ROLLINAT | 19100 Brive-la-Gaillarde | France</t>
+          <t>12 Boulevard marechal de Lattre de Tassigny | https://campus-paramedical.chu-dijon.fr/Filiere/infirmiers/ | 21000 Dijon | France</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2436,17 +2388,17 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>https://greta-du-limousin.fr/</t>
+          <t>https://campus-paramedical.chu-dijon.fr/Filiere/infirmiers/</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr</t>
+          <t>secretariat.ifsi@chu-dijon.fr</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr | formations-brive@afpa.fr</t>
+          <t>secretariat.ifsi@chu-dijon.fr</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -2461,12 +2413,12 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>0685201025</t>
+          <t>0380293502</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>0685201025</t>
+          <t>0380293502</t>
         </is>
       </c>
       <c r="O17" s="7" t="inlineStr">
@@ -2487,22 +2439,22 @@
       <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="7" t="inlineStr">
         <is>
-          <t>INTEGRATION - Intégration au groupe et à la formationFormalisation des parcours et sécurisation administrativeFinalisation des dossiers de rémunérationRappel des plannings, emploi du tempsRappel du règlement intérieur - 2 hDiagnostic / Positionnement - Positionnements écritsPositionnement pratiqueEntretien individuel exploratoireBilan - synthèse et proposition de parcours - 10 hPrésentation du métier et de son contexte - Présentation du "monde de la propreté" Intervention d'un professionnel / témoignage d'anciens stagiairesParticipation à des ateliers pratiques : présentation de produits d'entretien- présentation de matériels de nettoyage- démonstration de techniques d'entretienAteliers connaissance des entreprises du secteur de la propreté - 10 hPrésentation de la formation et la certification - Présentation de la formationIdentification des compétences professionnelles visées par le REAC du TP Agent(e) de Propreté et d'HygièneInformation sur le référentiel et les modalités de certification - 5 hCCP 1 : Prestation de nettoyage manuel - Réalisation d'une prestation de service d'entretien manuel adaptée aux locaux, aux surfaces et à leur utilisation par la mise en oeuvre de modes opératoires en respectant les règles d'hygiène et de sécurité, l'attitude de service et en intégrant les principes du développement durable.Apprentissage des techniques d'organisation des activités, de nettoyage, d'autocontrôle et de communication :1) Réalisation du nettoyage manuel des surfaces2) Réalisation du nettoyage manuel des sanitaires3) Réalisation du bionettoyage en environnement spécifique dans le respect des protocoles - 150 hCCP 2 : Prestation de nettoyage ou de remise en état mécanisés - Réalisation d'une prestation de services d'entretien mécanisé et/ou de remise en état mécanisée adaptée aux locaux et surfaces et à leur utilisation utilisation par la mise en oeuvre de modes opératoires en respectant les règles d'hygiène et de sécurité, l'attitude de service et en intégrant les principes du développement durable.Apprentissage des techniques d'organisation des activités, de nettoyage, d'autocontrôle et de communication :1) Réalisation d'un nettoyage mécanisé2) Réalisation d'une remise en état mécanisée - 175 hCompétenc | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travailLa formation dure trois ans. Les enseignements sont répartis de la manière suivante : la formation théorique de 2 100 heures, sous la forme de cours magistraux (750 heures) travaux dirigés (1 050 heures) et travail personnel guidé (300 heures) ; la formation clinique de 2 100 heures le travail personnel complémentaire est estimé à 900 heures environ, soit 300 heures par anModules : UG 01. Sciences humaines et sociales UG 02. Sciences biologiques et médicales UG 03. Sciences et techniques infirmières, fondements et méthodes UG 04. Sciences et techniques infirmières, interventions UG 05. Intégration des savoirs et posture professionnelle infirmière UG 06. Méthodes de travail | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de propreté et d'hygiène</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10926913/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11119576/true/false/false/true</t>
         </is>
       </c>
       <c r="V17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-19&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-21&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W17" s="7" t="inlineStr">
@@ -2519,27 +2471,27 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Tourneur, tourneuse en réalisation de pièces mécaniques (TP) [HSP 1er NQ]</t>
+          <t>Employé(e) polyvalent(e) en restauration (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>GRETA DU LIMOUSIN</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>19600 Saint-Pantaléon-de-Larche</t>
+          <t>19100 Brive-la-Gaillarde</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>AFPA - CENTRE DE BRIVE | 1 Rue de Laumeil | 19600 Saint-Pantaléon-de-Larche | France</t>
+          <t>AFPA - CENTRE DE BRIVE | 53 Rue MAURICE ROLLINAT | 19100 Brive-la-Gaillarde | France</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -2549,17 +2501,17 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
+          <t>https://greta-du-limousin.fr/</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-brive@afpa.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr | formations-brive@afpa.fr</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -2600,17 +2552,17 @@
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>TP TRPM - Période d'intégration - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi S'initier à Métis Développer son autonomie en formation - 35 hTP TRPM - Tourner des pièces, à l'unité ou en petites séries, sur machine conventionnelle - Réaliser des opérations de tournage en mandrin 3 mors durs en qualité 8 à l'aide d'un mode opératoire établiRéaliser des opérations de tournage en mandrin 3 mors doux, montage en l'air ou mixte en qualité 8 à l'aide d'un mode opératoire établiRéaliser des opérations de tournage dites complexes en qualité 8 à partir d'un mode opératoire établiRéaliser des opérations de tournage en mandrin 3 mors doux, montage en l'air ou mixte en qualité 7 à l'aide d'un mode opératoire à établir - 385 hTP TRPM - Régler un tour à commande numérique pour produire des séries stabilisées de pièces - Réaliser l'usinage de pièces mécaniques sur un TOUR CN régléPréparer hors machine, tous les éléments nécessaires aux réglages d'une production sur un TOUR CNMonter et régler l'outillage nécessaire à l'usinage d'une série de pièces sur un TOUR CNMettre au point une production et usiner une pré-série sur un TOUR CN - 210 hTP TRPM - Réaliser, à partir d'un plan, l'usinage de pièces unitaires ou de petites séries sur tour à commande numérique - Réaliser, à partir d'un dossier de fabrication stabilisé, l'usinage de pièces unitaires ou de petites séries sur tour à commande numériquePréparer l'usinage par procédé de tournage d'une pièce unitaire ou d'une petite série de pièces à partir d'un plan de pièceMettre au point l'usinage d'une nouvelle pièce sur un tour à commande numérique - 280 hTP TRPM - Période Entreprise - Contractualiser les objectifs de la période en entreprise Ancrer ses acquis en situation réelle de travail Développer des compétences transversales Accroître son réseau pour une insertion professionnelle - 105 | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>TITRE PRO AGENT DE RESTAURATION Intégration - Entrée en formationPrésentation de l'équipe pédagogique et administrativeVisite des locaux de formation (salles et plateaux techniques)Intégration au groupeFormalisation du parcours de formationInstruction du dossier et sécurisation administrativeExplicitation du calendrier de l'alternance et de l'emploi du temps de formationLecture et explication du Règlement Intérieur - 3 hTITRE PRO AGENT DE RESTAURATION Présentation du métier - Présentation du secteur "Hôtellerie-Restauration-Alimentation" (HRA)Intervention d'un professionnel / témoignage d'anciens stagiaires - 7 hTITRE PRO AGENT DE RESTAURATION Les modalités de certification - Présentation des modalités de certificationLe référentiel de formation et de certification TITRE PROFESSIONNEL Agent de restaurationLe calendrier prévisionnel des épreuves - 4 hTITRE PRO AGENT DES RESTAURATION Diagnostic - Positionnement - Positionnements écritsPositionnements pratiquesEntretien individuel exploratoire de confirmation de projetBilan - exploitation des positionnementsSynthèse et proposition de parcoursSignature du Contrat Pédagogique - 14 hTITRE PRO AGENT DE RESTAURATION Acquisition des connaissances et des compétences culinaires de base - Les principes et règlementation en matière de sécurité alimentaire (Codex alimentarius, GBPH, PMS, méthodologie HACCP,Le vocabulaire culinaire de base et la technologie culinaire : les produits alimentaires (denrées végétales, carnées, condiments, épices, produits dérivés, laitiers... les bases des méthodes de conservation, de cuisson- les principaux matériels et ustensiles culinaires- les préparations de base : fruits, légumes, oeufs, viandes, poissons, entremets, pâtisseries- les principales techniques d'assemblage - 28 hTITRE PRO AGENT DES RESTAURATION Préparer en assemblage des hors d'oeuvre, des desserts et des préparations de type "snacking" (CCP 1) - - Préparer les matières premières alimentaires destinées à la transformation et à l'assemblage - Réaliser l'assemblage et le dressage des hors-d'oeuvre, des desserts et des préparations de type snacking - 56 hTITRE PRO AGENT DE RESTAURATION Réaliser des grillades et remettre en température des PCEA Préparations Culinaires Elaborées à l'Avance) (CCP 2) - - Effectuer la remise en température de préparations culinaire | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T18" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel tourneur en réalisation de pièces mécaniques</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé polyvalent en restauration</t>
         </is>
       </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10926918/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10921927/true/false/false/true</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
@@ -2632,12 +2584,12 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Conseiller, Conseillère de vente (TP) [HSP 1er NQ]</t>
+          <t>Serveur, Serveuse en hôtellerie-restauration (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>GRETA DU LIMOUSIN</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -2652,7 +2604,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2662,17 +2614,17 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
+          <t>https://greta-du-limousin.fr/</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-brive@afpa.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr | formations-brive@afpa.fr</t>
         </is>
       </c>
       <c r="K19" s="7" t="inlineStr">
@@ -2713,17 +2665,17 @@
       <c r="R19" s="7" t="inlineStr"/>
       <c r="S19" s="7" t="inlineStr">
         <is>
-          <t>TP Conseiller de vente - Période d'intégration CV - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hTP Conseiller de vente - M1 - Contribuer à l'efficacité commerciale d'une unité marchande dans un environnement omnicanal - Connaître les différents contextes de la vente de services et de produitsConnaître les fondamentaux de la démarche marketingMener une étude de marché et établir le diagnostic de l'unité marchandeConnaître les différentes techniques et méthodes d'approvisionnementRéaliser des inventairesAppliquer les règles et les obligations légales du recyclage, du tri sélectif des déchets et de la réduction du gaspillageComprendre les règles de merchandisingMettre en place une opération commercialeSuivre et analyser les évolutions et exploiter les résultats pour proposer des ajustements - 245 hTP Conseiller de vente - Période en entreprise 1 - Se confronter à la réalité professionnelleMettre en application des acquisDévelopper des compétences transverses Etablir un réseau favorisant l'insertion professionnelle - 140 hTP Conseiller de vente - M2 - Améliorer l'expérience client dans un environnement omnicanal - Comprendre l'évolution du digital et son impact sur le métierValoriser l'offre de produits et de services de l'unité marchande sur les sites marchands et les médias sociauxAccueillir le client et mettre en oeuvre des conditions favorables à l'accueil des personnes en situation de handicapProcéder à l'enregistrement et à l'encaissementConnaître le cadre juridique de la vente et les enjeux du suivi de la relation commercialeConnaître les fondamentaux de la démarche marketingS'approprier et défendre les principes majeurs de l'écocitoyenneté tout au long de l'expérience d'achat - 210 hTP Conseiller de vente - Période en entreprise 2 - Se confronter à la réalité professionnelle Mettre en application des acquis Renforcer ses compétences transverses Développer son réseau professionnel - 140 hTP Conseiller de vente - Période de certification - Certification Conseiller de vente - 35 | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>CAP CS en HCR Intégration - Entrée en formationPrésentation de l'équipe pédagogique et administrativeVisite des locaux de formation (salles et plateaux techniques)Intégration au groupeFormalisation du parcours de formationInstruction du dossier et sécurisation administrativeExplicitation du calendrier de l'alternance et de l'emploi du temps de formationLecture et explication du Règlement Intérieur - 3 hCAP CS en HCR Présentation du métier - Présentation du secteur "Hôtellerie-Restauration-Alimentation" (HRA)Intervention d'un professionnel / témoignage d'anciens stagiaires - 7 hCAP CS en HCR Les modalités de certification - Présentation des modalités de certificationLes modalités de Contrôle en Cours de Formation (CCF) en ponctuel pour l'EIMCL 13 VentsLe référentiel de formation et de certification CAP HCRLe calendrier prévisionnel des épreuves - 4 hCAP CS en HCR Diagnostic - Positionnement - Positionnements écritsPositionnements pratiquesEntretien individuel exploratoire de confirmation de projetBilan - exploitation des positionnementsSynthèse et proposition de parcoursSignature du Contrat Pédagogique - 21 hCAP CS en HCR UP1 - Organisation des prestations en HCR - Réceptionner contrôler et stocker les marchandises1 - Les produits alimentaires et les boissons2 - Les autres produits3 - Les fournisseurs4 - Les mesures d'hygiène et de sécurité dans les locaux professionnels5 - Les stocks et les approvisionnementsCollecter les informations et ordonnancer ses activités6 - L'approche économique7 - Les locaux, les équipements et matériels8 - La prévention des risques liés à l'activité9 - Les différents types de prestations en restauration10 - Les supports et les documents liés aux prestations - 46 hCAP CS en HCR UP2 - Accueil, commercialisation et services en HCR - Accueillir, prendre en charge, renseigner le client et contribuer à la vente des prestations11 - Le client12 - Les points clés de la relation client13 - La réservation14 - Les supports de vente Thème15 - La prise de commande16 - Les étapes de la venteMettre en oeuvre les techniques de mise en place et de préparation17 - Les protocoles de nettoyage et d'entretien18 - La démarche de développement durable19 - Les mises en place20 - Les locaux annexes21 - Les techniques de préparation en restaurant - 137 hCAP CS en HCR UP2 - Accueil, commercialisation et services en HCR - Mettre en | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller de vente</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel serveur en restauration</t>
         </is>
       </c>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10926919/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10921937/true/false/false/true</t>
         </is>
       </c>
       <c r="V19" s="7" t="inlineStr">
@@ -2745,12 +2697,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Conseiller, Conseillère commercial (TP) [HSP 1er NQ]</t>
+          <t>Commis de cuisine (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>GRETA DU LIMOUSIN</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -2765,7 +2717,7 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -2775,17 +2727,17 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
+          <t>https://greta-du-limousin.fr/</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-brive@afpa.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr | formations-brive@afpa.fr</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -2826,17 +2778,17 @@
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>TP Conseiller commercial - Période d'intégration Conseiller commercial - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hTP Conseiller commercial - Module 1 Prospecter un secteur de vente - Assurer une veille professionnelle et commercialeMettre en oeuvre un plan d'actions commerciales et organiser son activitéProspecter à distanceProspecter physiquementAnalyser ses performances commerciales et en rendre compte - 280 hTP Conseiller commercial - Période Entreprise CCP1 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP Conseiller commercial - Module 2 Vendre en face à face des produits et des services référencés aux entreprises et aux particuliers - Représenter l'entreprise et valoriser son imageConduire un entretien de venteAssurer le suivi de ses ventesFidéliser son portefeuille client - 280 hTP Conseiller commercial - Période Entreprise CCP2 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP Conseiller commercial - Période de synthèse du parcours professionnel - Analyse de ses apprentissagesFinalisation de son dossier professionnelPréparation de la session de validation - 35 hTP Conseiller commercial - Période de certification - Certification Conseiller Commercial - 35 hTP CC - Sensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa propre empreinte écologique / prendre conscience de son propre impact (quiz, impactco2.fr, fresque du climat...Définir les points de progrès individuels et collectifs applicables dans la vie quotidienne, en formation et dans le milieu professionnel (Intervention d'acteurs locaux type ressourcerie, SIVOM, association de facilitation des mobilités douces, ... - 14 hTP CC - Sensibilisation aux enjeux des v | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>CAP CUISINE Intégration - Entrée en formationPrésentation de l'équipe pédagogique et administrativeVisite des locaux de formation (salles et plateaux techniques)Intégration au groupeFormalisation du parcours de formationInstruction du dossier et sécurisation administrativeExplicitation du calendrier de l'alternance et de l'emploi du temps de formationLecture et explication du Règlement Intérieur - 3 hCAP CUISINE Présentation du métier - Présentation du secteur "Hôtellerie-Restauration-Alimentation" (HRA)Intervention d'un professionnel / témoignage d'anciens stagiaires - 7 hCAP CUISINE Les modalités de certification - Présentation des modalités de certificationLes modalités de Contrôle en Cours de Formation (CCF)Le référentiel de formation et de certification CAP CuisineLe calendrier prévisionnel des épreuves - 4 hCAP CUISINE Diagnostic - Positionnement - Positionnements écritsPositionnements pratiquesEntretien individuel exploratoire de confirmation de projetBilan - exploitation des positionnementsSynthèse et proposition de parcoursSignature du Contrat Pédagogique - 21 hCAP CUISINE UP 1 - Organisation de la production de cuisine - 1 - Réceptionner, contrôler et stocker les marchandises dans le respect de la réglementation en vigueur et en appliquant les techniques de préventions liées à l'activité2 - Collecter l'ensemble des informations et organiser sa production culinaire dans le respect des consignes et de temps imparti - 63 hCAP CUISINE UP 2 - Préparation et distribution de la production en cuisine - 1 - Préparer, organiser et maintenir en état son poste de travail tout au long de l'activité dans le respect de la réglementation en vigueur2 - Maîtriser les techniques culinaires de base et réaliser une production dans le respect des consignes et des règles d'hygiène et de sécurité3 - Analyser, contrôler la qualité de sa production, dresser et participer à la distribution selon le contexte professionnel4 - Communiquer en fonction du contexte professionnel et en respectant les usages de la profession - 378 hCAP CUISINE Français - Histoire-Géographie - Enseignement Moral et Civique - FRANCAIS- Entrer dans l'échange oral et écrit : écouter, réagir, s'exprimer, lire, analyser, écrire- Devenir un lecteur compétent et critique- Confronter des savoirs et des valeurs pour construire son identité culturelle.HISTOIRE GEOGRAPHI | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T20" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller commercial</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel commis de cuisine</t>
         </is>
       </c>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10926920/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10921959/true/false/false/true</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
@@ -2858,7 +2810,7 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Agent(e) de reconditionnement numérique (TP) [HSP 1er NQ]</t>
+          <t>Assistant(e) de vie aux familles (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -2939,17 +2891,17 @@
       <c r="R21" s="7" t="inlineStr"/>
       <c r="S21" s="7" t="inlineStr">
         <is>
-          <t>Période d'intégration IDI - Intégrer son groupe et sa formationS'approprier les objectifs de la formation et repérer son futur environnement professionnelRepérer les risques liés à l'exercice du métier et se sensibiliser au développement durableDévelopper son efficacité personnelleS'inscrire dans une perspective d'emploi - 35 hConnaissances communes IDI - Utilisation Informatique - Internet et bureautiqueAnglais TechniquePosture ProfessionnelleSensibilisation aux règles : Electriques, DEEE, RGPD - 140 hMettre en service des équipements informatiques fixes et mobiles - Installer un système ou déployer une image sur un poste client fixe ou mobileConfigurer, paramétrer et personnaliser un équipement informatique fixe ou mobileRaccorder un équipement fixe ou mobile à un réseauInformer et conseiller le client ou l'utilisateur - 245 hDépanner et reconditionner des équipements informatiques fixes et mobiles - Diagnostiquer et résoudre un dysfonctionnement d'un équipement informatique fixe ou mobileVérifier, identifier, trier un équipement informatique fixe ou mobile d'occasionRevaloriser et intégrer un équipement fixe ou mobile - 175 hPériode d'application en entreprise IDI - Période entreprise IDI - 140 hPériode Certification IDI - Séquence de certification IDI - 35 hSensibilisation aux enjeux du développement durable - Néo terra-Niv 1 - Présentation de la feuille de route NeoTerra et ses 11 ambitionsNotion de développement durableHistoire, causes de l'émergence du conceptEnjeux (Environnement, économie et société)Sensibilisation au développement durable et à la Responsabilité Sociétale de l'Entreprise Diminuer la consommation d'énergie : gestion de l'allumage des lumières et des ordinateurs en salle de formation Identifier les sources d'économie d'énergie dans son activité professionnelle Recycler les déchets : tri et réemploiOptimiser l'envoi des emails (pièces jointes, SharePoint... - 14 hSensibilisation aux enjeux des valeurs de la république - Les institutions.Définitions du Citoyen , de la protection des libertés, de la laïcité, de l'égalité, de la préservation de la paix et des valeurs communes.Explication du règlement intérieur de l'établissement de formation : base pour aborder les valeurs, les principes et les symboles de la | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Intégration-présentation de la formation - Intégration au groupe et à la formationFormalisation des parcours et sécurisation administrativeFinalisation des dossiers de rémunérationRappel des plannings, emploi du tempsRappel du règlement intérieur - 4 hDiagnostic / Positionnement - Positionnements écritsEntretien individuel exploratoireBilan - synthèse et proposition de parcours - 7 hPrésentation du métier et du secteur - Présentation du secteur santé social Intervention de professionnels Fonctions et place de l'ADVFDroits et devoirs dans l'exercice du métier - 21 hModule Réussir sa formation en centre de formation et en entreprise - Modules sur les savoirs de base appliqués au secteur professionnel : mathématiques, français appliqués au secteur, informatiqueTechniques de recherche de stage, FLIRenforcement de l'acquisition de compétences comportementales. Méthodologie d'apprentissage apprendre à apprendre PAE *Préparation : -Définition des objectifs individuels,choix du type d'entreprise et/ou du service,mise à disposition et aide à la recherche de liste d'adresses et contacts,accompagnement à la démarche de recherche, entretien, négociation.Accompagnement : suivi et bilan en entreprise (stagiai - 63 hCCP 1 : Entretenir le logement et le linge d'un particulier - Relation professionnelle dans le cadre d'une prestation d'entretien chez un particulierCommunication professionnelle et relation avec la personne aidéePrévention des risques domestiques et travail en sécurité au domicile d'un particulierOrganisation du travailEntretien du logement avec les techniques et les gestes professionnels appropriésEntretien du linge (produits et techniques) repassage et initiation à la coutureRespect des règles environnementales/Hygiène et sécuritéEvaluation en cours de formation (mise en situation et écrit) - 126 hCCP 2 : Accompagner la personne dans les actes essentiels du quotidien - La relation avec la personne aidée et son entourageLes besoins fondamentauxLe handicapVieillissement et pathologies associées.Prévention des risques professionnelsL'autonomie physique, intellectuelle et sociale de la personneMobilisation et ergonomie / transferts et déplacementsAide à la toilette, à l'habillage et aux déplacementsAnimation et vie sociale.Aide aux courses, à la préparation et à la prise des repas Diététique et hygiène alimentair | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de reconditionnement numérique</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel assistant de vie aux familles</t>
         </is>
       </c>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10926921/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10925822/true/false/false/true</t>
         </is>
       </c>
       <c r="V21" s="7" t="inlineStr">
@@ -2966,32 +2918,32 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Concours d'atsem (FOAD)</t>
+          <t>Fraiseur, fraiseuse en réalisation de pièces mécaniques (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>19600 Saint-Pantaléon-de-Larche</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>AFPA - CENTRE DE BRIVE | 1 Rue de Laumeil | 19600 Saint-Pantaléon-de-Larche | France</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
+          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -3001,17 +2953,17 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>http://www.afpa.fr/</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-brives@afpa.fr</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -3026,40 +2978,48 @@
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0685201025</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O22" s="5" t="inlineStr"/>
+          <t>0685201025</t>
+        </is>
+      </c>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P22" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q22" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T22" s="5" t="inlineStr"/>
+          <t>TP FRPM - Période d'intégration - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi S'initier à Métis Développer son autonomie en formation - 35 hTP FRPM - Fraiser des pièces, à l'unité ou en petites séries sur machine conventionnelle - Réaliser des opérations de fraisage broche verticale à partir d'un mode opératoire établiRéaliser des opérations courantes de fraisage , broche verticale, horizontale ou inclinée, de qualité 8, à partir d'un mode opératoire établiRéaliser des opérations spécifiques de fraisage, broche verticale, horizontale ou inclinée, de qualité 8, à partir d'un mode opératoire établiRéaliser des opérations de fraisage broche verticale, horizontale ou inclinée avec une précision de qualité 7 et mode opératoire à établir - 385 hTP FRPM - Régler un centre d'usinage pour produire des séries stabilisées de pièces - Réaliser l'usinage de pièces mécaniques sur un centre d'usinage réglé Préparer hors machine, tous les éléments nécessaires aux réglages d'une production sur centre d'usinage Monter et régler l'outillage nécessaire à l'usinage d'une série de pièces sur un centre d'usinage Mettre au point une production et usiner une pré-série sur un centre d'usinage - 210 hTP FRPM - Réaliser, à partir d'un plan, l'usinage de pièces unitaires ou de petites séries sur centre d'usinage - Réaliser, à partir d'un dossier de fabrication stabilisé, l'usinage de pièces unitaires ou de petites séries sur un centre d'usinagePréparer l'usinage par procédé de fraisage d'une pièce unitaire ou d'une petite série de pièces à partir d'un plan de pièceMettre au point l'usinage d'une nouvelle pièce sur un centre d'usinage - 280 hTP FRPM - Période Entreprise - Contractualiser les objectifs de la période en entreprise Ancrer ses acquis en situation réelle de travail Développer des compétences transversales Accroître son réseau pour une insertion professionnelle - 175 | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T22" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel fraiseur en réalisation de pièces mécaniques</t>
+        </is>
+      </c>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10926897/true/false/false/true</t>
         </is>
       </c>
       <c r="V22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-19&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W22" s="5" t="inlineStr">
@@ -3071,32 +3031,32 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Agent(e) de propreté et d'hygiène (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>GRETA DU LIMOUSIN</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>19100 Brive-la-Gaillarde</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>AFPA - CENTRE DE BRIVE | 53 Rue MAURICE ROLLINAT | 19100 Brive-la-Gaillarde | France</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -3106,17 +3066,17 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://greta-du-limousin.fr/</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr | formations-brive@afpa.fr</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -3131,12 +3091,12 @@
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0685201025</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0685201025</t>
         </is>
       </c>
       <c r="O23" s="7" t="inlineStr">
@@ -3146,33 +3106,33 @@
       </c>
       <c r="P23" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q23" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R23" s="7" t="inlineStr"/>
       <c r="S23" s="7" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>INTEGRATION - Intégration au groupe et à la formationFormalisation des parcours et sécurisation administrativeFinalisation des dossiers de rémunérationRappel des plannings, emploi du tempsRappel du règlement intérieur - 2 hDiagnostic / Positionnement - Positionnements écritsPositionnement pratiqueEntretien individuel exploratoireBilan - synthèse et proposition de parcours - 10 hPrésentation du métier et de son contexte - Présentation du "monde de la propreté" Intervention d'un professionnel / témoignage d'anciens stagiairesParticipation à des ateliers pratiques : présentation de produits d'entretien- présentation de matériels de nettoyage- démonstration de techniques d'entretienAteliers connaissance des entreprises du secteur de la propreté - 10 hPrésentation de la formation et la certification - Présentation de la formationIdentification des compétences professionnelles visées par le REAC du TP Agent(e) de Propreté et d'HygièneInformation sur le référentiel et les modalités de certification - 5 hCCP 1 : Prestation de nettoyage manuel - Réalisation d'une prestation de service d'entretien manuel adaptée aux locaux, aux surfaces et à leur utilisation par la mise en oeuvre de modes opératoires en respectant les règles d'hygiène et de sécurité, l'attitude de service et en intégrant les principes du développement durable.Apprentissage des techniques d'organisation des activités, de nettoyage, d'autocontrôle et de communication :1) Réalisation du nettoyage manuel des surfaces2) Réalisation du nettoyage manuel des sanitaires3) Réalisation du bionettoyage en environnement spécifique dans le respect des protocoles - 150 hCCP 2 : Prestation de nettoyage ou de remise en état mécanisés - Réalisation d'une prestation de services d'entretien mécanisé et/ou de remise en état mécanisée adaptée aux locaux et surfaces et à leur utilisation utilisation par la mise en oeuvre de modes opératoires en respectant les règles d'hygiène et de sécurité, l'attitude de service et en intégrant les principes du développement durable.Apprentissage des techniques d'organisation des activités, de nettoyage, d'autocontrôle et de communication :1) Réalisation d'un nettoyage mécanisé2) Réalisation d'une remise en état mécanisée - 175 hCompétenc | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T23" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de propreté et d'hygiène</t>
         </is>
       </c>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10926913/true/false/false/false</t>
         </is>
       </c>
       <c r="V23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-19&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W23" s="7" t="inlineStr">
@@ -3184,32 +3144,32 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Préparation au concours d'ATSEM</t>
+          <t>Tourneur, tourneuse en réalisation de pièces mécaniques (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>AFEC</t>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>19600 Saint-Pantaléon-de-Larche</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>AFEC (Siège) | Formation a distance | 75004 Paris | France</t>
+          <t>AFPA - CENTRE DE BRIVE | 1 Rue de Laumeil | 19600 Saint-Pantaléon-de-Larche | France</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -3219,49 +3179,73 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr"/>
-      <c r="J24" s="5" t="inlineStr"/>
+          <t>http://www.afpa.fr/</t>
+        </is>
+      </c>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-brive@afpa.fr</t>
+        </is>
+      </c>
       <c r="K24" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>france_travail</t>
         </is>
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M24" s="5" t="inlineStr"/>
-      <c r="N24" s="5" t="inlineStr"/>
-      <c r="O24" s="5" t="inlineStr"/>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M24" s="5" t="inlineStr">
+        <is>
+          <t>0685201025</t>
+        </is>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>0685201025</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P24" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q24" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R24" s="5" t="inlineStr"/>
       <c r="S24" s="5" t="inlineStr">
         <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC | Lieu de la formation | AFEC (Siège)</t>
-        </is>
-      </c>
-      <c r="T24" s="5" t="inlineStr"/>
+          <t>TP TRPM - Période d'intégration - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi S'initier à Métis Développer son autonomie en formation - 35 hTP TRPM - Tourner des pièces, à l'unité ou en petites séries, sur machine conventionnelle - Réaliser des opérations de tournage en mandrin 3 mors durs en qualité 8 à l'aide d'un mode opératoire établiRéaliser des opérations de tournage en mandrin 3 mors doux, montage en l'air ou mixte en qualité 8 à l'aide d'un mode opératoire établiRéaliser des opérations de tournage dites complexes en qualité 8 à partir d'un mode opératoire établiRéaliser des opérations de tournage en mandrin 3 mors doux, montage en l'air ou mixte en qualité 7 à l'aide d'un mode opératoire à établir - 385 hTP TRPM - Régler un tour à commande numérique pour produire des séries stabilisées de pièces - Réaliser l'usinage de pièces mécaniques sur un TOUR CN régléPréparer hors machine, tous les éléments nécessaires aux réglages d'une production sur un TOUR CNMonter et régler l'outillage nécessaire à l'usinage d'une série de pièces sur un TOUR CNMettre au point une production et usiner une pré-série sur un TOUR CN - 210 hTP TRPM - Réaliser, à partir d'un plan, l'usinage de pièces unitaires ou de petites séries sur tour à commande numérique - Réaliser, à partir d'un dossier de fabrication stabilisé, l'usinage de pièces unitaires ou de petites séries sur tour à commande numériquePréparer l'usinage par procédé de tournage d'une pièce unitaire ou d'une petite série de pièces à partir d'un plan de pièceMettre au point l'usinage d'une nouvelle pièce sur un tour à commande numérique - 280 hTP TRPM - Période Entreprise - Contractualiser les objectifs de la période en entreprise Ancrer ses acquis en situation réelle de travail Développer des compétences transversales Accroître son réseau pour une insertion professionnelle - 105 | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T24" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel tourneur en réalisation de pièces mécaniques</t>
+        </is>
+      </c>
       <c r="U24" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10926918/true/false/false/false</t>
         </is>
       </c>
       <c r="V24" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-19&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W24" s="5" t="inlineStr">
@@ -3273,32 +3257,32 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
+          <t>Conseiller, Conseillère de vente (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>19100 Brive-la-Gaillarde</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>AFPA - CENTRE DE BRIVE | 53 Rue MAURICE ROLLINAT | 19100 Brive-la-Gaillarde | France</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -3308,17 +3292,17 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>http://www.afpa.fr/</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-brive@afpa.fr</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
@@ -3333,40 +3317,48 @@
       </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0685201025</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
-        </is>
-      </c>
-      <c r="O25" s="7" t="inlineStr"/>
+          <t>0685201025</t>
+        </is>
+      </c>
+      <c r="O25" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P25" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R25" s="7" t="inlineStr"/>
       <c r="S25" s="7" t="inlineStr">
         <is>
-          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T25" s="7" t="inlineStr"/>
+          <t>TP Conseiller de vente - Période d'intégration CV - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hTP Conseiller de vente - M1 - Contribuer à l'efficacité commerciale d'une unité marchande dans un environnement omnicanal - Connaître les différents contextes de la vente de services et de produitsConnaître les fondamentaux de la démarche marketingMener une étude de marché et établir le diagnostic de l'unité marchandeConnaître les différentes techniques et méthodes d'approvisionnementRéaliser des inventairesAppliquer les règles et les obligations légales du recyclage, du tri sélectif des déchets et de la réduction du gaspillageComprendre les règles de merchandisingMettre en place une opération commercialeSuivre et analyser les évolutions et exploiter les résultats pour proposer des ajustements - 245 hTP Conseiller de vente - Période en entreprise 1 - Se confronter à la réalité professionnelleMettre en application des acquisDévelopper des compétences transverses Etablir un réseau favorisant l'insertion professionnelle - 140 hTP Conseiller de vente - M2 - Améliorer l'expérience client dans un environnement omnicanal - Comprendre l'évolution du digital et son impact sur le métierValoriser l'offre de produits et de services de l'unité marchande sur les sites marchands et les médias sociauxAccueillir le client et mettre en oeuvre des conditions favorables à l'accueil des personnes en situation de handicapProcéder à l'enregistrement et à l'encaissementConnaître le cadre juridique de la vente et les enjeux du suivi de la relation commercialeConnaître les fondamentaux de la démarche marketingS'approprier et défendre les principes majeurs de l'écocitoyenneté tout au long de l'expérience d'achat - 210 hTP Conseiller de vente - Période en entreprise 2 - Se confronter à la réalité professionnelle Mettre en application des acquis Renforcer ses compétences transverses Développer son réseau professionnel - 140 hTP Conseiller de vente - Période de certification - Certification Conseiller de vente - 35 | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T25" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller de vente</t>
+        </is>
+      </c>
       <c r="U25" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10926919/true/false/false/true</t>
         </is>
       </c>
       <c r="V25" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-19&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W25" s="7" t="inlineStr">
@@ -3378,32 +3370,32 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
+          <t>Conseiller, Conseillère commercial (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>19100 Brive-la-Gaillarde</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>AFPA - CENTRE DE BRIVE | 53 Rue MAURICE ROLLINAT | 19100 Brive-la-Gaillarde | France</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -3413,17 +3405,17 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>http://www.afpa.fr/</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-brive@afpa.fr</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
@@ -3438,40 +3430,48 @@
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0685201025</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
-        </is>
-      </c>
-      <c r="O26" s="5" t="inlineStr"/>
+          <t>0685201025</t>
+        </is>
+      </c>
+      <c r="O26" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P26" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q26" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R26" s="5" t="inlineStr"/>
       <c r="S26" s="5" t="inlineStr">
         <is>
-          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T26" s="5" t="inlineStr"/>
+          <t>TP Conseiller commercial - Période d'intégration Conseiller commercial - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hTP Conseiller commercial - Module 1 Prospecter un secteur de vente - Assurer une veille professionnelle et commercialeMettre en oeuvre un plan d'actions commerciales et organiser son activitéProspecter à distanceProspecter physiquementAnalyser ses performances commerciales et en rendre compte - 280 hTP Conseiller commercial - Période Entreprise CCP1 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP Conseiller commercial - Module 2 Vendre en face à face des produits et des services référencés aux entreprises et aux particuliers - Représenter l'entreprise et valoriser son imageConduire un entretien de venteAssurer le suivi de ses ventesFidéliser son portefeuille client - 280 hTP Conseiller commercial - Période Entreprise CCP2 - Se confronter à la réalité professionnelleMettre en application des acquis Développer des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP Conseiller commercial - Période de synthèse du parcours professionnel - Analyse de ses apprentissagesFinalisation de son dossier professionnelPréparation de la session de validation - 35 hTP Conseiller commercial - Période de certification - Certification Conseiller Commercial - 35 hTP CC - Sensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa propre empreinte écologique / prendre conscience de son propre impact (quiz, impactco2.fr, fresque du climat...Définir les points de progrès individuels et collectifs applicables dans la vie quotidienne, en formation et dans le milieu professionnel (Intervention d'acteurs locaux type ressourcerie, SIVOM, association de facilitation des mobilités douces, ... - 14 hTP CC - Sensibilisation aux enjeux des v | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T26" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller commercial</t>
+        </is>
+      </c>
       <c r="U26" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10926920/true/false/false/false</t>
         </is>
       </c>
       <c r="V26" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-19&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W26" s="5" t="inlineStr">
@@ -3483,32 +3483,32 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Agent(e) de reconditionnement numérique (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>AFEC (Siège)</t>
+          <t>GRETA DU LIMOUSIN</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>19100 Brive-la-Gaillarde</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>AFPA - CENTRE DE BRIVE | 53 Rue MAURICE ROLLINAT | 19100 Brive-la-Gaillarde | France</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -3518,17 +3518,17 @@
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://greta-du-limousin.fr/</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr | formations-brive@afpa.fr</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
@@ -3543,12 +3543,12 @@
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>0153368844</t>
+          <t>0685201025</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>0153368844</t>
+          <t>0685201025</t>
         </is>
       </c>
       <c r="O27" s="7" t="inlineStr">
@@ -3558,33 +3558,33 @@
       </c>
       <c r="P27" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q27" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R27" s="7" t="inlineStr"/>
       <c r="S27" s="7" t="inlineStr">
         <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant des modules d'enseignement et des prestations d'accompagnement. Modules d'enseignement professionnel : - EP1 Accompagnement du développement du jeune enfant (cadre d'intervention, accompagnement à l'autonomie l'enfant) - EP2 Exercer son activité en accueil collectif - EP3 Exercer son activité en accueil individuel Modules d'enseignements généraux : - Prévention santé environnement - Enseignements généraux (Mathématiques et sciences, Histoire-Géographie-Citoyenneté et français) En complément de la formation : - Remise à niveau numérique - Techniques de recherche d'emploi et de stage - Accompagnement au retour à l'emploi 3 Stages en entreprise 14 semaines | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Période d'intégration IDI - Intégrer son groupe et sa formationS'approprier les objectifs de la formation et repérer son futur environnement professionnelRepérer les risques liés à l'exercice du métier et se sensibiliser au développement durableDévelopper son efficacité personnelleS'inscrire dans une perspective d'emploi - 35 hConnaissances communes IDI - Utilisation Informatique - Internet et bureautiqueAnglais TechniquePosture ProfessionnelleSensibilisation aux règles : Electriques, DEEE, RGPD - 140 hMettre en service des équipements informatiques fixes et mobiles - Installer un système ou déployer une image sur un poste client fixe ou mobileConfigurer, paramétrer et personnaliser un équipement informatique fixe ou mobileRaccorder un équipement fixe ou mobile à un réseauInformer et conseiller le client ou l'utilisateur - 245 hDépanner et reconditionner des équipements informatiques fixes et mobiles - Diagnostiquer et résoudre un dysfonctionnement d'un équipement informatique fixe ou mobileVérifier, identifier, trier un équipement informatique fixe ou mobile d'occasionRevaloriser et intégrer un équipement fixe ou mobile - 175 hPériode d'application en entreprise IDI - Période entreprise IDI - 140 hPériode Certification IDI - Séquence de certification IDI - 35 hSensibilisation aux enjeux du développement durable - Néo terra-Niv 1 - Présentation de la feuille de route NeoTerra et ses 11 ambitionsNotion de développement durableHistoire, causes de l'émergence du conceptEnjeux (Environnement, économie et société)Sensibilisation au développement durable et à la Responsabilité Sociétale de l'Entreprise Diminuer la consommation d'énergie : gestion de l'allumage des lumières et des ordinateurs en salle de formation Identifier les sources d'économie d'énergie dans son activité professionnelle Recycler les déchets : tri et réemploiOptimiser l'envoi des emails (pièces jointes, SharePoint... - 14 hSensibilisation aux enjeux des valeurs de la république - Les institutions.Définitions du Citoyen , de la protection des libertés, de la laïcité, de l'égalité, de la préservation de la paix et des valeurs communes.Explication du règlement intérieur de l'établissement de formation : base pour aborder les valeurs, les principes et les symboles de la | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de reconditionnement numérique</t>
         </is>
       </c>
       <c r="U27" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124191/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10926921/true/false/false/true</t>
         </is>
       </c>
       <c r="V27" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-18&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-19&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W27" s="7" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-08-07
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,17 +932,17 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Concours d'atsem (FOAD)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1350 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -972,12 +972,12 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K4" s="5" t="inlineStr">
@@ -992,19 +992,15 @@
       </c>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>0180888030</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0366060201</t>
+        </is>
+      </c>
+      <c r="O4" s="5" t="inlineStr"/>
       <c r="P4" s="5" t="inlineStr">
         <is>
           <t>Formation financée par France Travail</t>
@@ -1018,22 +1014,18 @@
       <c r="R4" s="5" t="inlineStr"/>
       <c r="S4" s="5" t="inlineStr">
         <is>
-          <t>11 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 : Démarrez votre formation d'Accompagnement Educatif Petite Enfance ; Projet 2 - Préparez un environnement sécurisé pour le jeune enfant ; Projet 3 - Développez des activités éducatives adaptées à la petite enfance ; Projet 4 - Appliquez les protocoles de santé dans le cadre de la petite enfance ; Projet 5 - Soutenez le personnel enseignant dans un contexte collectif ; Projet 6 - Améliorez les conditions d'accueil en école maternelle ; Projet 7 - Organisez l'accueil individuel au domicile ; Projet 8 - Gérez les tâches domestiques et la préparation des repas pour l'enfant ; Projet 9 : Proposer des solutions de prévention, santé et environnement ; Projet 10 : Remise à niveau scolaire ; Projet 11 : Préparez-vous pour l'examen final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T4" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
-        </is>
-      </c>
+          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T4" s="5" t="inlineStr"/>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120311/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
         </is>
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1045,17 +1037,17 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Conseiller emploi et accompagnement professionnel</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>OPENCLASSROOMS</t>
+          <t>Centre européen de formation</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -1070,7 +1062,7 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1140 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1085,12 +1077,12 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>inscription@openclassrooms.com</t>
+          <t>info@cenef.fr</t>
         </is>
       </c>
       <c r="K5" s="7" t="inlineStr">
@@ -1105,12 +1097,12 @@
       </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>0180888030</t>
+          <t>0366060201</t>
         </is>
       </c>
       <c r="O5" s="7" t="inlineStr">
@@ -1131,22 +1123,22 @@
       <c r="R5" s="7" t="inlineStr"/>
       <c r="S5" s="7" t="inlineStr">
         <is>
-          <t>10 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de conseiller emploi et évolution professionnelle ; Projet 2 - Accompagnez en parallèle de nombreuses personnes avec des besoins différents ; Projet 3 - Élaborez une veille et analysez le marché de l'emploi ; Projet 4 - Réalisez un diagnostic et co-construisez un plan d'action avec vos bénéficiaires ; Projet 5 - Adaptez votre posture pour l'accompagnement des bénéficiaires ; Projet 6 - Établissez et validez un projet d'accompagnement professionnel ; Projet 7 - Établissez un plan d'action et un bilan professionnel ; Projet 8 - Concevez un atelier sur les métiers émergents avec l'IA ; Projet 9 - Développez votre projet territorial avec des partenaires ; Projet 10 - Élaborez votre boîte à outils pour accompagner vers l'emploi. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
+          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T5" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Conseiller emploi et accompagnement professionnel</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11120363/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
         </is>
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1158,32 +1150,32 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Certificat d'aptitude aux fonctions de directeur d'établissement ou de service d'intervention sociale (CAFDES)</t>
+          <t>Préparation au concours d'ATSEM</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>INSTITUT REGIONAL DU TRAVAIL SOCIAL (IRTS de Besançon)</t>
+          <t>AFEC</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>25000 Besançon</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>1 Rue Alfred de Vigny | http://www.irts-fc.fr | 25000 Besançon | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1210 heures (dont 510 heures en entreprise)</t>
+          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -1193,17 +1185,17 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>http://www.irts-fc.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr">
         <is>
-          <t>irts-fc@irts-fc.fr</t>
+          <t>cergy@afec.fr</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>irts-fc@irts-fc.fr</t>
+          <t>cergy@afec.fr</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
@@ -1218,48 +1210,40 @@
       </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>0381416100</t>
+          <t>0143388881</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
         <is>
-          <t>0381416100</t>
-        </is>
-      </c>
-      <c r="O6" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0143388881</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr"/>
       <c r="P6" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R6" s="5" t="inlineStr"/>
       <c r="S6" s="5" t="inlineStr">
         <is>
-          <t>700 h de formation théorique (formation complète) réparties en 4 Domaines de formation selon 4 blocs de compétences. Allègements possibles d'un à deux tiers selon expérience, statut et formation. 510 h de formation pratique. Allègements possibles d'un à deux tiers selon expérience, statut et formation. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T6" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Certificat d'aptitude aux fonctions de directeur d'établissement ou de service d'intervention sociale</t>
-        </is>
-      </c>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T6" s="5" t="inlineStr"/>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10941346/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1271,32 +1255,32 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>CENTRE HOSPITALIER UNIVERSITAIRE DE BESANCON (CHU Besançon - CESU 25)</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>25000 Besançon</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>INSTITUT DE FORMATION DES PROFESSIONNELS DE SANTE DE BESANCON | 44 chemin du sanatorium | http://www.chu-besancon.fr | 25000 Besançon | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1306,17 +1290,17 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>http://www.chu-besancon.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>drh-formation@chu-besancon.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>drh-formation@chu-besancon.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K7" s="7" t="inlineStr">
@@ -1331,48 +1315,40 @@
       </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>0381415137</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
-          <t>0381415137</t>
-        </is>
-      </c>
-      <c r="O7" s="7" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="inlineStr"/>
       <c r="P7" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>En centre et à distance</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr"/>
       <c r="S7" s="7" t="inlineStr">
         <is>
-          <t>La formation en soins infirmiers s'articule autour de l'acquisition de 10 compétences :C1 : Évaluer une situation clinique et établir un diagnostic dans le domaine infirmierC2 : Concevoir et conduire un projet de soins infirmiersC3 : Accompagner la personne dans la réalisation de ses soins quotidiensC4 : Mettre en uvre des actions à visée diagnostique et thérapeutiquesC5 : Initier et mettre en uvre des soins éducatifs et préventifsC6 : Communiquer et conduire une relation dans un contexte de soinsC7 : Analyser la qualité des soins et améliorer sa pratique professionnelleC8 : Rechercher et traiter des données professionnelles et scientifiquesC9 : Organiser et coordonner des interventions soignantesC10 : Informer et former des professionnels et des personnes en formationDes unités d'enseignement en :UG 01. Sciences humaines et socialesUG 02. Sciences biologiques et médicalesUG 03. Sciences et techniques infirmières, fondements et méthodesUG 04. Sciences et techniques infirmières, interventionsUG 05. Intégration des savoirs et posture professionnelle infirmièreUG 06. Méthodes de travail | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T7" s="7" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
-        </is>
-      </c>
+          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T7" s="7" t="inlineStr"/>
       <c r="U7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10966697/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
         </is>
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1384,32 +1360,32 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'éducateur de jeunes enfants (DEEJE)</t>
+          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>INSTITUT REGIONAL DU TRAVAIL SOCIAL (IRTS de Besançon)</t>
+          <t>Leo Lagrange Formation</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>25000 Besançon</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>1 Rue Alfred de Vigny | http://www.irts-fc.fr | 25000 Besançon | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Durée de 3600 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
@@ -1419,17 +1395,17 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>http://www.irts-fc.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr">
         <is>
-          <t>irts-fc@irts-fc.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>irts-fc@irts-fc.fr</t>
+          <t>contact@ifra.fr</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
@@ -1444,48 +1420,40 @@
       </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>0381416100</t>
+          <t>0472892042</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
         <is>
-          <t>0381416100</t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0472892042</t>
+        </is>
+      </c>
+      <c r="O8" s="5" t="inlineStr"/>
       <c r="P8" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q8" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr">
         <is>
-          <t>La formation d'éducateur de jeunes enfants comprend 2100h de formation pratique et 1500h de formation théorique réparties en 4 domaines de formation : Accueil et accompagnement du jeune enfant et de sa famille 400h- Action éducative en direction du jeune enfant 600h- Travail en équipe pluriprofessionnelle et communication professionnelle 250h- Dynamiques interinstitutionnelles, partenariats et réseaux 250h | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T8" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur de jeunes enfants</t>
-        </is>
-      </c>
+          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
+        </is>
+      </c>
+      <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11068853/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
         </is>
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1497,32 +1465,32 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'Etat d'éducateur technique spécialisé (DEETS)</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>INSTITUT REGIONAL DU TRAVAIL SOCIAL (IRTS de Besançon)</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>25000 Besançon</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>1 Rue Alfred de Vigny | http://www.irts-fc.fr | 25000 Besançon | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>Durée de 3300 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 1350 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1532,17 +1500,17 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>http://www.irts-fc.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>irts-fc@irts-fc.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>irts-fc@irts-fc.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K9" s="7" t="inlineStr">
@@ -1557,12 +1525,12 @@
       </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>0381416100</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
         <is>
-          <t>0381416100</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O9" s="7" t="inlineStr">
@@ -1572,33 +1540,33 @@
       </c>
       <c r="P9" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R9" s="7" t="inlineStr"/>
       <c r="S9" s="7" t="inlineStr">
         <is>
-          <t>La formation d'Educateur Technique spécialisé comprend 2100h de formation pratique et 1200h de formation théorique organisée en 4 Domaines de Formation : Accompagnement social et éducatif spécialisé 450h- Conception et conduite d'un projet éducatif technique spécialisé 350h- Communication professionnelle 200h- Dynamiques interinstitutionnelles partenariats et réseaux 200h | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>11 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 : Démarrez votre formation d'Accompagnement Educatif Petite Enfance ; Projet 2 - Préparez un environnement sécurisé pour le jeune enfant ; Projet 3 - Développez des activités éducatives adaptées à la petite enfance ; Projet 4 - Appliquez les protocoles de santé dans le cadre de la petite enfance ; Projet 5 - Soutenez le personnel enseignant dans un contexte collectif ; Projet 6 - Améliorez les conditions d'accueil en école maternelle ; Projet 7 - Organisez l'accueil individuel au domicile ; Projet 8 - Gérez les tâches domestiques et la préparation des repas pour l'enfant ; Projet 9 : Proposer des solutions de prévention, santé et environnement ; Projet 10 : Remise à niveau scolaire ; Projet 11 : Préparez-vous pour l'examen final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T9" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'Etat d'éducateur technique spécialisé</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11068854/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120311/true/false/true/true</t>
         </is>
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1610,32 +1578,32 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>Conseiller emploi et accompagnement professionnel</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>HOPITAL NORD FRANCHE-COMTE (Hôpital Nord Franche-Comté (HNFC))</t>
+          <t>OPENCLASSROOMS</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>25200 Montbéliard</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>HOPITAL NORD FRANCHE COMTE | 4 Place Lucien Tharradin | http://www.hnfc.fr | 25200 Montbéliard | France</t>
+          <t>Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 1140 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
@@ -1645,17 +1613,17 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>http://www.hnfc.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>dir-generale@hnfc.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>dir-generale@hnfc.fr</t>
+          <t>inscription@openclassrooms.com</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr">
@@ -1670,12 +1638,12 @@
       </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>0381939393</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
         <is>
-          <t>0381939393</t>
+          <t>0180888030</t>
         </is>
       </c>
       <c r="O10" s="5" t="inlineStr">
@@ -1685,33 +1653,33 @@
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q10" s="5" t="inlineStr">
         <is>
-          <t>En centre et à distance</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R10" s="5" t="inlineStr"/>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>10 projets professionnalisants permettront au stagiaire d'acquérir par la pratique les compétences recquises. Chaque livrable enrichira son portfolio qu'il pourra valoriser auprès des recruteurs. Il réalisera les projets suivants : Projet 1 - Démarrez votre formation de conseiller emploi et évolution professionnelle ; Projet 2 - Accompagnez en parallèle de nombreuses personnes avec des besoins différents ; Projet 3 - Élaborez une veille et analysez le marché de l'emploi ; Projet 4 - Réalisez un diagnostic et co-construisez un plan d'action avec vos bénéficiaires ; Projet 5 - Adaptez votre posture pour l'accompagnement des bénéficiaires ; Projet 6 - Établissez et validez un projet d'accompagnement professionnel ; Projet 7 - Établissez un plan d'action et un bilan professionnel ; Projet 8 - Concevez un atelier sur les métiers émergents avec l'IA ; Projet 9 - Développez votre projet territorial avec des partenaires ; Projet 10 - Élaborez votre boîte à outils pour accompagner vers l'emploi. | Validation | Type de validation : | Titre inscrit sur demande au RNCP | Certification :</t>
         </is>
       </c>
       <c r="T10" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Titre inscrit sur demande au RNCP | Certification : | Conseiller emploi et accompagnement professionnel</t>
         </is>
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11075537/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11120363/true/false/true/true</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1723,32 +1691,32 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Diplôme d'État d'infirmier(ière)</t>
+          <t>CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Institut de formation en soins infirmiers de Pontarlier (IFSI de Pontarlier)</t>
+          <t>AFEC (Siège)</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>25300 Pontarlier</t>
+          <t>75004 Paris</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>1 Avenue du General Girod | 25300 Pontarlier | France</t>
+          <t>AFEC | Formation a distance | 75004 Paris | France</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 490 heures en entreprise)</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
@@ -1758,17 +1726,17 @@
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>http://www.ifsi-pontarlier.fr/</t>
+          <t>https://plmpl.fr/c/zFjGj</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>ifp@chi-hc.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>ifp@chi-hc.fr</t>
+          <t>paris@afec.fr</t>
         </is>
       </c>
       <c r="K11" s="7" t="inlineStr">
@@ -1783,12 +1751,12 @@
       </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>0381385329</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>0381385329</t>
+          <t>0153368844</t>
         </is>
       </c>
       <c r="O11" s="7" t="inlineStr">
@@ -1798,33 +1766,33 @@
       </c>
       <c r="P11" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par la région</t>
+          <t>Formation financée par France Travail</t>
         </is>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>À distance</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr"/>
       <c r="S11" s="7" t="inlineStr">
         <is>
-          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : Sciences humaines, sociales et droit, Sciences biologiques et médicales, Sciences et techniques infirmières, fondements et méthodes, Sciences et techniques infirmières, interventions, Intégration des savoirs et posture professionnelle infirmière, Méthodes de travail.La formation dure trois ans. Les enseignements sont répartis de la manière suivante : La formation théorique de 2 100 heures, sous la forme de cours magistraux (750 heures) travaux dirigés (1 050 heures) et travail personnel guidé (300 heures) La formation clinique de 2 100 heures, Le travail personnel complémentaire est estimé à 900 heures environ. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant des modules d'enseignement et des prestations d'accompagnement. Modules d'enseignement professionnel : - EP1 Accompagnement du développement du jeune enfant (cadre d'intervention, accompagnement à l'autonomie l'enfant) - EP2 Exercer son activité en accueil collectif - EP3 Exercer son activité en accueil individuel Modules d'enseignements généraux : - Prévention santé environnement - Enseignements généraux (Mathématiques et sciences, Histoire-Géographie-Citoyenneté et français) En complément de la formation : - Remise à niveau numérique - Techniques de recherche d'emploi et de stage - Accompagnement au retour à l'emploi 3 Stages en entreprise 14 semaines | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T11" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
         </is>
       </c>
       <c r="U11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11115737/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11124191/true/false/true/true</t>
         </is>
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">
@@ -1836,32 +1804,32 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Horticulteur, Horticultrice (CAPA) [HSP 1er NQ]</t>
+          <t>Certificat d'aptitude aux fonctions de directeur d'établissement ou de service d'intervention sociale (CAFDES)</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>CFPPA 47</t>
+          <t>INSTITUT REGIONAL DU TRAVAIL SOCIAL (IRTS de Besançon)</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>24660 Coulounieix-Chamiers</t>
+          <t>25000 Besançon</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>EPLEFPA PERIGORD - LEGTPA PERIGUEUX | Avenue Winston Churchill Domaine Peyrouse | 24660 Coulounieix-Chamiers | France</t>
+          <t>1 Rue Alfred de Vigny | http://www.irts-fc.fr | 25000 Besançon | France</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1220 heures (dont 420 heures en entreprise)</t>
+          <t>Durée de 1210 heures (dont 510 heures en entreprise)</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -1871,17 +1839,17 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>http://www.epl47.educagri.fr/cfppa.html</t>
+          <t>http://www.irts-fc.fr/</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>cfppa.ste-livrade@educagri.fr</t>
+          <t>irts-fc@irts-fc.fr</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>cfppa.ste-livrade@educagri.fr | cfppa.perigueux@educagri.fr</t>
+          <t>irts-fc@irts-fc.fr</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr">
@@ -1896,12 +1864,12 @@
       </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>0553026130</t>
+          <t>0381416100</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>0553026130</t>
+          <t>0381416100</t>
         </is>
       </c>
       <c r="O12" s="5" t="inlineStr">
@@ -1922,22 +1890,22 @@
       <c r="R12" s="5" t="inlineStr"/>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>UC Générale CG 1 : UCG 1 : Agir dans des situations de la vie courante à l'aide de repères sociaux - - Prendre position dans une situation à caractère social et civique- Utiliser des outils dans des situations de la vie courante - 40 hUC Générale CG 2 : UCG 2 : Mettre en oeuvre des actions contribuant à sa construction personnelle - - S'exprimer à travers une réalisation personnelle - Adopter des comportements favorisant son équilibre personnel - 40 hUC Générale CG 3 : UCG 3 : Interagir avec son environnement social - - Adapter son langage et son comportement aux situations de communication - S'approprier les normes et cadres de référence d'un collectif - 40 hUC Professionnelle CP 4 : UCP 1 : Réaliser des travaux sur les végétaux - - Réaliser des observations et interventions sur le végétal - Réaliser des travaux de mise en place des végétaux - 160 hUC Professionnelle CP 5 : UCP 2 : Réaliser des travaux de suivi des cultures de l'implantation à la récolte et au conditionnement - - Réaliser des observations et opérations techniques liées au cycle de production - Effectuer des travaux de récolte, de conservation et de conditionnement - 260 hUC Professionnelle CP 6 : UCP 3 : Effectuer des travaux liés à l'entretien courant des matériels, équipements, installations et bâtiments - - Réaliser des opérations de maintenance conditionnelle des matériels, équipements, installations et bâtiments - Effectuer des travaux simples d'aménagement et de réparation - 91 hUCARE CP 7 : Vente des produits de l'exploitation - - Organisation d'une action de vente- Création d'un support de communication- Aménagement et valorisation du point de vente- Soin et conservation des produits- Conduite de l'entretien de vente - 60 hTechniques à la recherche d'emploi - - Aide à la recherche de stage (CV et lettre de motivation) Suivi individuel de formation - Accompagner et sécuriser la sortie de formation- Favoriser l'insertion professionnelle et assurer la continuité éventuelle du parcours de formation - 70 hCertiphyto Opérateur - - Connaître la réglementation encadrant les produits phytopharmaceutiques- Appliquer les bonnes pratiques de prévention des risques pour la santé et pour l'environnement lors de l'utilisation des produits phytopharmaceutiques. Appliquer les stratégies visant à limit | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>700 h de formation théorique (formation complète) réparties en 4 Domaines de formation selon 4 blocs de compétences. Allègements possibles d'un à deux tiers selon expérience, statut et formation. 510 h de formation pratique. Allègements possibles d'un à deux tiers selon expérience, statut et formation. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T12" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP agricole métiers de l'agriculture</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Certificat d'aptitude aux fonctions de directeur d'établissement ou de service d'intervention sociale</t>
         </is>
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910461/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10941346/true/false/false/true</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-24&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W12" s="5" t="inlineStr">
@@ -1949,32 +1917,32 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Jardinier, Jardinière paysagiste (CAPA) [HSP 1er NQ]</t>
+          <t>Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>CFPPA 47</t>
+          <t>CENTRE HOSPITALIER UNIVERSITAIRE DE BESANCON (CHU Besançon - CESU 25)</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>24660 Coulounieix-Chamiers</t>
+          <t>25000 Besançon</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>EPLEFPA PERIGORD - LEGTPA PERIGUEUX | Avenue Winston Churchill Domaine Peyrouse | 24660 Coulounieix-Chamiers | France</t>
+          <t>INSTITUT DE FORMATION DES PROFESSIONNELS DE SANTE DE BESANCON | 44 chemin du sanatorium | http://www.chu-besancon.fr | 25000 Besançon | France</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1220 heures (dont 420 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1984,17 +1952,17 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>http://www.epl47.educagri.fr/cfppa.html</t>
+          <t>http://www.chu-besancon.fr/</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>cfppa.ste-livrade@educagri.fr</t>
+          <t>drh-formation@chu-besancon.fr</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>cfppa.ste-livrade@educagri.fr | cfppa.perigueux@educagri.fr</t>
+          <t>drh-formation@chu-besancon.fr</t>
         </is>
       </c>
       <c r="K13" s="7" t="inlineStr">
@@ -2009,12 +1977,12 @@
       </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>0553026130</t>
+          <t>0381415137</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>0553026130</t>
+          <t>0381415137</t>
         </is>
       </c>
       <c r="O13" s="7" t="inlineStr">
@@ -2029,28 +1997,28 @@
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>En centre et à distance</t>
         </is>
       </c>
       <c r="R13" s="7" t="inlineStr"/>
       <c r="S13" s="7" t="inlineStr">
         <is>
-          <t>Sensibilsation aux enjeux de développement durable - l'eaule soll'énergie et climat - 21 hSensibilisation aux valeurs de la république, l'éducation citoyenne et à la prévention des violences sexuelles et sexistes - les valeurs de la république,Droits et obligations du citoyenLaïcité Egalité hommes/femmesAlerter et orienter - 7 hSensibilisation aux enjeux numériques - Les outils numériquesLes bons usages du numériques - 7 hCertiphyto - RèglementationPrévention des risques pour l'environnementPrévention des risques pour la santéStratégies visant à limiter le recours aux produits phytosanaitaires - 14 hPositionnement - Test de connaissances et de compétences professionnelles - 35 hUcare : réaliser la taille fruitière - Réalisation des opérations de taille de formationRéalisation des opérations de taille de productionRestructuration des vergers âgés - 70 hEntretien du matériel et des équipements - Préparation du matériel et organisation des tâches en fonction des consignes, du travail en équipe et des aléasRéglage du matériel et ajustement des réglages en cours de travailEntretien courant des matérielsPetites réparations sur le matérielEntretien des protections individuelles et collectivesNettoyage et rangement des outils et matérielsCommunication en situation professionnelle - 105 hCréation d'un espage payasager - Préparation du travail et organisation des tâches en fonction des consignes, du travail en équipe et des aléas,Travaux infrastructure d'un espace en suivant le plan d'exécutionTravaux de plantation des végétauxTravaux de semis et d'engazonnementCommunication professionnelle - 224 hTravaux d'entretien d'un espace paysager - Préparation du travail d'organisation des tâches en fonction des consignes, du travail en équipe et des aléas,Entretien des espaces paysagers et naturelsEntretien des installations et des infrastructures paysagèresCommunication en situation professionnelle - 266 hAgir dans son environnement économique, social et territorial - Prise de position dans une situation à caractère social et civiqueUtilisation d'outils dans des situations de la vie courante,Expression à travers une réalisation personnelleAdoption de comportement favorisant l'équilibre personnelAdaptat | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>La formation en soins infirmiers s'articule autour de l'acquisition de 10 compétences :C1 : Évaluer une situation clinique et établir un diagnostic dans le domaine infirmierC2 : Concevoir et conduire un projet de soins infirmiersC3 : Accompagner la personne dans la réalisation de ses soins quotidiensC4 : Mettre en uvre des actions à visée diagnostique et thérapeutiquesC5 : Initier et mettre en uvre des soins éducatifs et préventifsC6 : Communiquer et conduire une relation dans un contexte de soinsC7 : Analyser la qualité des soins et améliorer sa pratique professionnelleC8 : Rechercher et traiter des données professionnelles et scientifiquesC9 : Organiser et coordonner des interventions soignantesC10 : Informer et former des professionnels et des personnes en formationDes unités d'enseignement en :UG 01. Sciences humaines et socialesUG 02. Sciences biologiques et médicalesUG 03. Sciences et techniques infirmières, fondements et méthodesUG 04. Sciences et techniques infirmières, interventionsUG 05. Intégration des savoirs et posture professionnelle infirmièreUG 06. Méthodes de travail | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T13" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP agricole jardinier paysagiste</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910464/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10966697/true/false/false/true</t>
         </is>
       </c>
       <c r="V13" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-24&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W13" s="7" t="inlineStr">
@@ -2062,32 +2030,32 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Action préparatoire aux métiers de l'agriculture [HSP 1er NQ]</t>
+          <t>Diplôme d'État d'éducateur de jeunes enfants (DEEJE)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>CFPPA 47</t>
+          <t>INSTITUT REGIONAL DU TRAVAIL SOCIAL (IRTS de Besançon)</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>24240 Monbazillac</t>
+          <t>25000 Besançon</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>EPLEFPA PERIGORD - LEGTPA PERIGUEUX | Route du Chateau Domaine de LA BRIE | 24240 Monbazillac | France</t>
+          <t>1 Rue Alfred de Vigny | http://www.irts-fc.fr | 25000 Besançon | France</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 3600 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -2097,17 +2065,17 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>http://www.epl47.educagri.fr/cfppa.html</t>
+          <t>http://www.irts-fc.fr/</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>cfppa.ste-livrade@educagri.fr</t>
+          <t>irts-fc@irts-fc.fr</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>cfppa.ste-livrade@educagri.fr | cfppa.perigueux@educagri.fr</t>
+          <t>irts-fc@irts-fc.fr</t>
         </is>
       </c>
       <c r="K14" s="5" t="inlineStr">
@@ -2122,15 +2090,19 @@
       </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>0553583391</t>
+          <t>0381416100</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
         <is>
-          <t>0553583391</t>
-        </is>
-      </c>
-      <c r="O14" s="5" t="inlineStr"/>
+          <t>0381416100</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P14" s="5" t="inlineStr">
         <is>
           <t>Formation financée par la région</t>
@@ -2144,18 +2116,22 @@
       <c r="R14" s="5" t="inlineStr"/>
       <c r="S14" s="5" t="inlineStr">
         <is>
-          <t>Découverte des filières et des métiers - Les filières, les métiers, les acteursLes spécificités du territoire L'emploi agricole sur le territoireLes types d'entreprises du bassin d'emploi et leur fonctionnement La saisonnalité des travaux Le matériel et les risques professionnels des métiers - 42 hElaboration du projet professionnel - Remobilisation et confiance en soiPréparation immersion en entreprise Se tester en milieu professionnelTRE et coaching vers le stage : Cartographie professionnelle, mobilité, savoir candidater, trouver un stage/emploi (CV Entretien LM) - Accompagnement personnalisé - 56 hConsolidation et concrétisation du projet professionnel - Choix du projet suite aux découvertes et immersionsConsolidation du projet : ciblage activités, d'un l'emploi, savoirs, savoir-être, formations.TRE et coaching vers l'emploi/formation choisi. Accompagnement personnalisé.Accéder à une qualification professionnelle ou à un emploi : définir son besoin de compétences et les étapes de son projet (formation/emploi) tableau de bord du projet, inscription en formation - 56 hAcquisition des compétences nécessaires à l'intégration professionnelle - Compétences sociales et civiques / Savoir-être, aptitudes professionnelles / formation / Communication verbale/non verbale Intégration en milieu professionnel / formationSanté et sécurité au travail - 49 hIdentification des freins, Accompagnent Socio Pro - Validation par le stagiaire de sa capacité à intégrer une formationIdentification des freins à l'entrée en formation : mobilité, Financiers, Handicap, Socio, Logement, restaurationAccompagnement dans la levée des freins : Comportement, Langage, Sociabilisation, Savoir de base, Savoir de base...Possibilités offertes par le HSP et des autres dispositifs d'accompagnement.Si besoin, accompagnement individualisé. - 42 hSensibilisation aux enjeux de développement durable - - Gestion de la ressource en eau en agriculture- Agronomie : Respect des sols et de son vivant en agriculture- Gestion des énergies et impact sur notre climat - 21 hSensibilisation aux valeurs de la république - - Sensibilisation aux valeurs de la république et éducation citoyenne- Prévention des violences sexuelles et sexistes - 7 hSensibilisation aux enjeux du numérique - - Présentation des différents outils numériques accessible au centre de formation- | Organisme | CFPPA 47 | http://www.epl47.educagri.fr/cfppa.html | Lieu de la formation</t>
-        </is>
-      </c>
-      <c r="T14" s="5" t="inlineStr"/>
+          <t>La formation d'éducateur de jeunes enfants comprend 2100h de formation pratique et 1500h de formation théorique réparties en 4 domaines de formation : Accueil et accompagnement du jeune enfant et de sa famille 400h- Action éducative en direction du jeune enfant 600h- Travail en équipe pluriprofessionnelle et communication professionnelle 250h- Dynamiques interinstitutionnelles, partenariats et réseaux 250h | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T14" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'éducateur de jeunes enfants</t>
+        </is>
+      </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10910503/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11068853/true/false/false/true</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-24&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W14" s="5" t="inlineStr">
@@ -2167,32 +2143,32 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Agent(e) des travaux forestiers (BPA) [HSP 1er NQ]</t>
+          <t>Diplôme d'Etat d'éducateur technique spécialisé (DEETS)</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>CFPPA 47</t>
+          <t>INSTITUT REGIONAL DU TRAVAIL SOCIAL (IRTS de Besançon)</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>24300 Nontron</t>
+          <t>25000 Besançon</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>MAISON FAMILIALE RURALE PERIGORD LIMOUSIN - NONTRON | Place DES DROITS DE L HOMME | 24300 Nontron | France</t>
+          <t>1 Rue Alfred de Vigny | http://www.irts-fc.fr | 25000 Besançon | France</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1225 heures (dont 350 heures en entreprise)</t>
+          <t>Durée de 3300 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
@@ -2202,17 +2178,17 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>http://www.epl47.educagri.fr/cfppa.html</t>
+          <t>http://www.irts-fc.fr/</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>cfppa.ste-livrade@educagri.fr</t>
+          <t>irts-fc@irts-fc.fr</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>cfppa.ste-livrade@educagri.fr | mfr.nontron@mfr.asso.fr</t>
+          <t>irts-fc@irts-fc.fr</t>
         </is>
       </c>
       <c r="K15" s="7" t="inlineStr">
@@ -2227,12 +2203,12 @@
       </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>0553603193</t>
+          <t>0381416100</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>0553603193</t>
+          <t>0381416100</t>
         </is>
       </c>
       <c r="O15" s="7" t="inlineStr">
@@ -2253,22 +2229,22 @@
       <c r="R15" s="7" t="inlineStr"/>
       <c r="S15" s="7" t="inlineStr">
         <is>
-          <t>Positionnement BPA Travaux Forestiers - Évaluer le niveau de connaissances pour construire un parcours deformation individualisé qualifiant et/ou diplômant - 14 hConnaissances générales, sociales et économiques intégrant le concept de gestion durable des ressources forestières - UCG1 / UCG 2 - UCG1 Mobiliser les outils nécessaires au traitement de l'information et à la communication dans la vie professionnelle et sociale:Communiquer oralement et à l'écritUtiliser les techniques de collecte et de traitement de l'informationTraiter les mathématiquesUtiliser les outils informatiques et de télécommunicationUCG2 Mobiliser des connaissances relatives aux domaines civique, social etéconomique :Utiliser les règles du droit du travail/protection socialeconnaître les bases de la gestionconnaître la filière dans son ensemble - 223 hConnaissances générales scientifiques intégrant le concept de gestion durable des ressources forestières - UCG 3 : Mobiliser des connaissances pour mettre en oeuvre des pratiques professionnelles respectueuses de l'environnement et de la santé humaineMobiliser des connaissances pour appréhender l'impact environnemental des pratiques professionnellesMobiliser des connaissances pour prévenir les risques et préserver la santé humaine - 40 hConnaissances scientifiques et techniques relatives au domaine forestier intégrant le concept de gestion durable des ressources forestières - UCO1:Mobiliser, en vue de sa pratique professionnelle, les connaissances scientifiques et techniques relatives à la forêtMobiliser des connaissances scientifiques et techniques relatives à l'arbre et à son milieuMobiliser des connaissances scientifiques et techniques relatives à laproduction forestièreUCO2:Mobiliser des connaissances scientifiques et techniques relatives à l'utilisation des matériels et équipements d'exploitation forestièreConnaître le fonctionnement des matériels et installations forestiersConnaître les techniques des matériels et installations forestieres - 198 hConnaissances professionnelles relatives au domaine forestier intégrant le concept de gestion durable des ressources forestières - BPA Travaux de sylvicultureUCS1TS:Effectuer les travaux de régénération forestièrePréparer la mise en place d'un peuplementMettre en place un peuplementProtéger un peuplementUCS2TS:Réaliser les opérations d'entretien d'un jeune peuplementRéaliser le d&amp;eacut | Validation | Type de validation : | Diplôme autres ministères | Certifications :</t>
+          <t>La formation d'Educateur Technique spécialisé comprend 2100h de formation pratique et 1200h de formation théorique organisée en 4 Domaines de Formation : Accompagnement social et éducatif spécialisé 450h- Conception et conduite d'un projet éducatif technique spécialisé 350h- Communication professionnelle 200h- Dynamiques interinstitutionnelles partenariats et réseaux 200h | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T15" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certifications : | BPA option travaux forestiers spécialité travaux de sylviculture</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'Etat d'éducateur technique spécialisé</t>
         </is>
       </c>
       <c r="U15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10913180/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11068854/true/false/false/false</t>
         </is>
       </c>
       <c r="V15" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-24&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W15" s="7" t="inlineStr">
@@ -2280,32 +2256,32 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Employé(e) commercial (TP) [HSP 1er NQ]</t>
+          <t>Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>INFREP DORDOGNE</t>
+          <t>HOPITAL NORD FRANCHE-COMTE (Hôpital Nord Franche-Comté (HNFC))</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>24100 Bergerac</t>
+          <t>25200 Montbéliard</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>TALIS COMPETENCES &amp; CERTIFICATIONS - BERGERAC | 110 Avenue PAULDOUMER | 24100 Bergerac | France</t>
+          <t>HOPITAL NORD FRANCHE COMTE | 4 Place Lucien Tharradin | http://www.hnfc.fr | 25200 Montbéliard | France</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Durée de 980 heures (dont 315 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -2315,17 +2291,17 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>https://www.infrep.org/</t>
+          <t>http://www.hnfc.fr/</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>infrep24@infrep.org</t>
+          <t>dir-generale@hnfc.fr</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>infrep24@infrep.org | v.rousseau@talis-cc.com | patricia.rieupet@talis-bs.com</t>
+          <t>dir-generale@hnfc.fr</t>
         </is>
       </c>
       <c r="K16" s="5" t="inlineStr">
@@ -2340,12 +2316,12 @@
       </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>0553221200</t>
+          <t>0381939393</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
         <is>
-          <t>0553221200</t>
+          <t>0381939393</t>
         </is>
       </c>
       <c r="O16" s="5" t="inlineStr">
@@ -2360,28 +2336,28 @@
       </c>
       <c r="Q16" s="5" t="inlineStr">
         <is>
-          <t>En centre</t>
+          <t>En centre et à distance</t>
         </is>
       </c>
       <c r="R16" s="5" t="inlineStr"/>
       <c r="S16" s="5" t="inlineStr">
         <is>
-          <t>INTEGRATION Communication professionnelle - Accueil des participants et présentation de l'organisme de formation, de l'équipe pédagogique et administrativePrésentation des objectifs du stage, de l'organisation générale de l'action et du cadre de l'action.Diagnostic- positionnement Présentation du livret stagiairePrésentation du règlement intérieur Sensibilisation aux valeurs de la république, à l'éducation citoyenne et à la prévention des violences sexuelles et sexistesDynamique de groupe contrat de formation et annexe pédagogiqueCommunication : Présentation croisée, Brèves de comptoir, Le BlasonI - 21 hCOMPETENCES NUMERIQUES - Etat des lieux des équipements et moyens de connexion pour chaque stagiaire de l'action Prise en main de la plateforme e learning de chaque organisme Utilisation des outils numériques tels que : Le DRIVE- GOOGLE DOCS- GOOGLE SHEETS- GOOGLE SLIDESMobilisation et animation des plateformes numériques en lien avec les CCP du Titre professionnel Les nouvelles technologies de la communication et leurs impactenvironnemental - 14 hModule 1 - METTRE A DISPOSITION DES CLIENTS LES PRODUITS DE L'UNITE MARCHANDE DANS UN ENVIRONNEMENT OMNICANAL - APPROVISIONNER L'UNITE MARCHANDE ASSURER LA PRESENTATION MARCHANDE DES PRODUITS DANS LE MAGASIN CONTRIBUER A LA GESTION ET OPTIMISER LES STOCKS TRAITER LES COMMANDES DE PRODUITS DE CLIENTS - 309 hModule 2 - ACCUEILLIR LES CLIENTS ET REPONDRE A LEUR DEMANDE DANS UN ENVIRONNEMENT OMNICANAL... - ACCUEILLIR, RENSEIGNER ET SERVIR LES CLIENTS CONTRIBUER A L'AMELIORATION DE L'EXPERIENCE D'ACHATTENIR UN POSTE DE CAISSE ET SUPERVISER LES CAISSES LIBRE-SERVICE - 310 hDEVELOPPEMENT DURABLE ET ACTIVITE PROFESSIONNELLE - sensibilisation a la transition énergétique, écologique et sociétale Néo TERRA Niveau 1enjeux mondiaux, nationaux et regionaux ecoresponsabilité au quotidienNEO TERRA Niveau 2 Compétences sectorielles en lien avec la transition energétique, écologique et sociétale sensibilisation aux innovations en lien avec l'activité professionnelle du commerce (commerce équitable, impact du e commerce, achat responsable et solidaire, circuits court, économie circulaire, recyclage et réemploi... - 28 hACCOMPAGNEMENT A LA RECHERCHE D'EMPLOI - Présentation de la plateforme TALENTS D'ICIcréation d'un compte sur le site Création et actualisation d'un CVCréation de compte sur les sites dédiés à la recherche d'emploiMise en relation avec les entreprises pour les recherches | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : sciences humaines, sociales et droit sciences biologiques et médicales sciences et techniques infirmières, fondements et méthodes sciences et techniques infirmières, interventions intégration des savoirs et posture professionnelle infirmière méthodes de travail. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T16" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé commercial</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10913186/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11075537/true/false/false/true</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-24&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W16" s="5" t="inlineStr">
@@ -2393,32 +2369,32 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Conseiller, Conseillère de vente (TP) [HSP 1er NQ]</t>
+          <t>Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>INFREP DORDOGNE</t>
+          <t>Institut de formation en soins infirmiers de Pontarlier (IFSI de Pontarlier)</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>24100 Bergerac</t>
+          <t>25300 Pontarlier</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>TALIS COMPETENCES &amp; CERTIFICATIONS - BERGERAC | 110 Avenue PAULDOUMER | 24100 Bergerac | France</t>
+          <t>1 Avenue du General Girod | 25300 Pontarlier | France</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>Durée de 980 heures (dont 315 heures en entreprise)</t>
+          <t>Durée de 4200 heures (dont 2100 heures en entreprise)</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
@@ -2428,17 +2404,17 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>https://www.infrep.org/</t>
+          <t>http://www.ifsi-pontarlier.fr/</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>infrep24@infrep.org</t>
+          <t>ifp@chi-hc.fr</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>infrep24@infrep.org | v.rousseau@talis-cc.com | patricia.rieupet@talis-bs.com</t>
+          <t>ifp@chi-hc.fr</t>
         </is>
       </c>
       <c r="K17" s="7" t="inlineStr">
@@ -2453,12 +2429,12 @@
       </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>0553221200</t>
+          <t>0381385329</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>0553221200</t>
+          <t>0381385329</t>
         </is>
       </c>
       <c r="O17" s="7" t="inlineStr">
@@ -2479,22 +2455,22 @@
       <c r="R17" s="7" t="inlineStr"/>
       <c r="S17" s="7" t="inlineStr">
         <is>
-          <t>INTEGRATION Communication professionnelle ... - Accueil des participants et présentation de l'organisme de formation, de l'équipe pédagogique et administrativePrésentation des objectifs de la formation, de l'organisation générale de l'action et du cadre de l'action.Diagnostic - positionnement Présentation du livret stagiairePrésentation du règlement intérieur Sensibilisation aux valeurs de la république, à l'éducation citoyenne et à la prévention des violences sexuelles et sexistesDynamique de groupe contrat de formation et de l'annexe pédagogiqueCommunication : Présentation croisée, Brèves de comptoir, Le Blason - 21 hCOMPETENCES NUMERIQUES - Etat des lieux des équipements et moyens de connexion pour chaque stagiaire de l'action Prise en main de la plateforme e learning de chaque organisme Utilisation des outils numériques tels que : Le DRIVE- GOOGLE DOCS- GOOGLE SHEETS- GOOGLE SLIDESMobilisation et animation des plateformes numériques en lien avec lesLes nouvelles technologies de la communication et leurs impactsenvironnementaux (RGPD à inclure) - 28 hCONTRIBUER A L'EFFICACITE COMMERCIALE D'UNE UNITE MARCHANDE DANS UN ENVIRONNEMENT OMNICANAL - ASSURER UNE VIEILLE PROFESSIONNELLE ET COMMERCIALE PARTICIPER A LA GESTION DES FLUX MARCHANDSCONTRIBUER AU MERCHANDISING ANALYSER SES PERFORMANCES COMMERCIALES ET EN RENDRE COMPTE - 442 hAMELIORER L'EXPERIENCE CLIENT DANS UN ENVIRONNEMENT OMNICANAL - REPRESENTER L'UNITE MARCHANDE ET CONTRIBUER A LA VALORISATION DE SON IMAGE CONSEILLER LE CLIENT EN CONDUISANT L'ENTRETIEN DE VENTE ASSURER LE SUIVI DE SES VENTES CONTRIBUER A LA FIDELISATION EN CONSOLIDANT L'EXPERIENCE CLIENT - 443 hDEVELOPPEMENT DURABLE ET ACTIVITE PROFESSIONNELLE - Sensibilisation a la transition énergétique, écologique et sociétale Néo TERRA Niveau 1enjeux mondiaux, nationaux et regionaux ecoresponsabilité au quotidienNEO TERRA Niveau 2 Compétences sectorielles en lien avec la transition energétique, écologique et sociétale sensibilisation aux innovations en lien avec l'activité professionnelle du commerce (commerce équitable, impact du e commerce, achat responsable et solidaire, circuits court, économie circulaire, recyclage et réemploi... - 21 hACOMPAGNEMENT VERS L'EMPLOI - Présentation de la plateforme TALENTS D'ICIcréation d'un compte sur le site Création et actualisation d'un CVCréation de compte sur les sites dédiés à la recherche d'emploiMise en relation avec les entreprises pour les recher | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>La formation comprend 36 matières réparties dans 59 unités d'enseignements. Les unités d'enseignements couvrent 6 champs : Sciences humaines, sociales et droit, Sciences biologiques et médicales, Sciences et techniques infirmières, fondements et méthodes, Sciences et techniques infirmières, interventions, Intégration des savoirs et posture professionnelle infirmière, Méthodes de travail.La formation dure trois ans. Les enseignements sont répartis de la manière suivante : La formation théorique de 2 100 heures, sous la forme de cours magistraux (750 heures) travaux dirigés (1 050 heures) et travail personnel guidé (300 heures) La formation clinique de 2 100 heures, Le travail personnel complémentaire est estimé à 900 heures environ. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T17" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller de vente</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Diplôme d'État d'infirmier(ière)</t>
         </is>
       </c>
       <c r="U17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10913199/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/11115737/true/false/false/true</t>
         </is>
       </c>
       <c r="V17" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-24&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-25&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W17" s="7" t="inlineStr">
@@ -2511,27 +2487,27 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Action Préparatoire aux métiers du BTP [HSP 1er NQ]</t>
+          <t>Horticulteur, Horticultrice (CAPA) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>CFPPA 47</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>24100 Bergerac</t>
+          <t>24660 Coulounieix-Chamiers</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>IDC PRO - CFA CONSTRUCTION SUD DORDOGNE | ZA LE LIBRAIRE | 24100 Bergerac | France</t>
+          <t>EPLEFPA PERIGORD - LEGTPA PERIGUEUX | Avenue Winston Churchill Domaine Peyrouse | 24660 Coulounieix-Chamiers | France</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1220 heures (dont 420 heures en entreprise)</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
@@ -2541,17 +2517,17 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
+          <t>http://www.epl47.educagri.fr/cfppa.html</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+          <t>cfppa.ste-livrade@educagri.fr</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | administratif@idcpro.fr</t>
+          <t>cfppa.ste-livrade@educagri.fr | cfppa.perigueux@educagri.fr</t>
         </is>
       </c>
       <c r="K18" s="5" t="inlineStr">
@@ -2566,15 +2542,19 @@
       </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
-          <t>0553733257</t>
+          <t>0553026130</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>0553733257</t>
-        </is>
-      </c>
-      <c r="O18" s="5" t="inlineStr"/>
+          <t>0553026130</t>
+        </is>
+      </c>
+      <c r="O18" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P18" s="5" t="inlineStr">
         <is>
           <t>Formation financée par la région</t>
@@ -2588,13 +2568,17 @@
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr">
         <is>
-          <t>Période d'intégration - Période d'intégration Intégrer son groupe et sa formationS'approprier le cadre et les objectifs de la formation préparatoire Développer sa culture numérique et prendre en main la plateforme MètisDécouvrir la boîte à outils numériqueDécouvrir Mètis et se repérer dans son parcoursPasser les tests de positionnementPréciser ses besoins de formation et contractualiser son parcours personnaliséS'inscrire dans une continuité de parcours certifiant ou une perspective d'emploi, un contrat en alternanceInitier son portefeuille de compétences - 35 hModule 1 : Découverte des métiers du secteur BTP et de leurs évolutions - Immersions sur les plateaux de formation - Découverte des métiers Les travaux publics : Canalisateur, maçon voirie réseaux divers, conducteur d'engins... Le gros oeuvre : Maçon, charpentier, couvreur zingueur... Le second oeuvre : Peintre, Carreleur, agent de maintenance des bâtiments, plombier, électricien, menuisier...Visites d'entreprises : Préparer, réaliser et exploiter une visite en entreprise Participation à des évènementiels Salons, jobs dating à partir d'une préparation collectiveMatinale entreprise (témoignages professionnels)BILAN INDIVIDUEL D'ORIENTATION - 70 hModule 2 : Acquérir le socle des connaissances nécessaires pour aller vers les métiers de l'industrie - Se remettre à niveau en mathématiquesUtiliser le système métriqueApprendre à lire des documents techniques, des plans....Développer sa communication écrite, son expression orale, comprendre les règles et instructionsTravailler en équipe et adopter la posture professionnelle attendueBILAN INDIVIDUEL D'ORIENTATION - 70 hModule 3 : Acquérir les bases des connaissances techniques et les gestes professionnels d'un métier - Réaliser un ouvrage simple en tenant compte des exigences de sécurité Identifier le matériel et les équipements nécessaires à la réalisation d'un ouvrage simplePréparer la matière nécessaire à la réalisation d'un ouvrage simpleRéaliser un ouvrage simpleMaintenir, l'organisation et la propreté du poste de travailTravailler en sécurité et conformément à la réglementation Repérer les risques liés à l'exercice des métiers de l'industrie Se sensibiliser au développement durable dans les métiers du BTPBILAN INDIVIDUEL D'ORIENTATION - 105 | Organisme | DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE | http://www.afpa.fr | Lieu de la formation</t>
-        </is>
-      </c>
-      <c r="T18" s="5" t="inlineStr"/>
+          <t>UC Générale CG 1 : UCG 1 : Agir dans des situations de la vie courante à l'aide de repères sociaux - - Prendre position dans une situation à caractère social et civique- Utiliser des outils dans des situations de la vie courante - 40 hUC Générale CG 2 : UCG 2 : Mettre en oeuvre des actions contribuant à sa construction personnelle - - S'exprimer à travers une réalisation personnelle - Adopter des comportements favorisant son équilibre personnel - 40 hUC Générale CG 3 : UCG 3 : Interagir avec son environnement social - - Adapter son langage et son comportement aux situations de communication - S'approprier les normes et cadres de référence d'un collectif - 40 hUC Professionnelle CP 4 : UCP 1 : Réaliser des travaux sur les végétaux - - Réaliser des observations et interventions sur le végétal - Réaliser des travaux de mise en place des végétaux - 160 hUC Professionnelle CP 5 : UCP 2 : Réaliser des travaux de suivi des cultures de l'implantation à la récolte et au conditionnement - - Réaliser des observations et opérations techniques liées au cycle de production - Effectuer des travaux de récolte, de conservation et de conditionnement - 260 hUC Professionnelle CP 6 : UCP 3 : Effectuer des travaux liés à l'entretien courant des matériels, équipements, installations et bâtiments - - Réaliser des opérations de maintenance conditionnelle des matériels, équipements, installations et bâtiments - Effectuer des travaux simples d'aménagement et de réparation - 91 hUCARE CP 7 : Vente des produits de l'exploitation - - Organisation d'une action de vente- Création d'un support de communication- Aménagement et valorisation du point de vente- Soin et conservation des produits- Conduite de l'entretien de vente - 60 hTechniques à la recherche d'emploi - - Aide à la recherche de stage (CV et lettre de motivation) Suivi individuel de formation - Accompagner et sécuriser la sortie de formation- Favoriser l'insertion professionnelle et assurer la continuité éventuelle du parcours de formation - 70 hCertiphyto Opérateur - - Connaître la réglementation encadrant les produits phytopharmaceutiques- Appliquer les bonnes pratiques de prévention des risques pour la santé et pour l'environnement lors de l'utilisation des produits phytopharmaceutiques. Appliquer les stratégies visant à limit | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T18" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP agricole métiers de l'agriculture</t>
+        </is>
+      </c>
       <c r="U18" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10921925/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10910461/true/false/false/true</t>
         </is>
       </c>
       <c r="V18" s="5" t="inlineStr">
@@ -2616,27 +2600,27 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Employé(e) polyvalent(e) en restauration (TP) [HSP 1er NQ]</t>
+          <t>Jardinier, Jardinière paysagiste (CAPA) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>GRETA CFA AQUITAINE</t>
+          <t>CFPPA 47</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>24750 Boulazac Isle Manoire</t>
+          <t>24660 Coulounieix-Chamiers</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>AFPA PERIGUEUX | Avenue Ambroise Croizat Z.I de Boulazac | 24750 Boulazac Isle Manoire | France</t>
+          <t>EPLEFPA PERIGORD - LEGTPA PERIGUEUX | Avenue Winston Churchill Domaine Peyrouse | 24660 Coulounieix-Chamiers | France</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 1220 heures (dont 420 heures en entreprise)</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -2646,17 +2630,17 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>https://greta-cfa-aquitaine.fr/</t>
+          <t>http://www.epl47.educagri.fr/cfppa.html</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>contact@greta-cfa-aquitaine.fr</t>
+          <t>cfppa.ste-livrade@educagri.fr</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>contact@greta-cfa-aquitaine.fr | formations-perigueux@afpa.fr</t>
+          <t>cfppa.ste-livrade@educagri.fr | cfppa.perigueux@educagri.fr</t>
         </is>
       </c>
       <c r="K19" s="7" t="inlineStr">
@@ -2671,12 +2655,12 @@
       </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>0617668622</t>
+          <t>0553026130</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>0617668622</t>
+          <t>0553026130</t>
         </is>
       </c>
       <c r="O19" s="7" t="inlineStr">
@@ -2697,17 +2681,17 @@
       <c r="R19" s="7" t="inlineStr"/>
       <c r="S19" s="7" t="inlineStr">
         <is>
-          <t>Accueil / Intégration dans la formation - Intégration au groupe et à la formationS'approprier les objectifs de la formation et repérer son futur environnement professionnelPositionnementsFormalisation des parcours et sécurisation administrative - 7 hRéussir sa formation en centre de formation et en entreprise - Techniques de recherche de stageRenforcement de l'acquisition de compétences comportementales et Soft skills : savoirs être professionnels adaptés aux différents métiers du secteurPAE - Préparation : -définition des objectifs individuels,choix du type d'entreprise et/ou du service,mise à disposition et aide à la recherche de liste d'adresses et contacts,accompagnement à la démarche de recherche, entretien, négociation. Accompagnement : -suivi et bilan en entreprise (stagiaire + formateur référent + tuteur)retour partagé des expériences, travail de réflexivité. - 14 hPréparer en assemblage des hors-d'oeuvre, des desserts et des préparations de type "snacking" - Préparation des matières premières alimentaires destinéesà la transformation et à l'assemblageRéalisation de l'assemblage et du dressage des horsd'oeuvre, des desserts et des préparations de type"snacking"Appliquer les règles d'hygiène et de sécurité alimentaire (haccp) - 154 hRéaliser des grillades et remettre en température des préparations culinaires élaborées à l'avance (PCEA) - Remise en température de préparationsculinaires élaborées à l'avance (PCEA)Réalisation d'une production culinaire au poste grilladeAppliquer les règles d'hygiène et de sécurité alimentaire (haccp) - 154 hAccueillir les clients et distribuer les plats en restauration self-service - Mise en place de la salle à manger du self-serviceRéalisation de la mise en place de la distribution Service aux postes froids et chaudsEnregistrement du contenu des plateaux repas et des préparations de type "snacking"EncaissementRespect des consignes de santé et de sécurité au travail - 147 hRéaliser le nettoyage de la batterie de cuisine et le lavage en machine de la vaisselle - Nettoyage de la "batterie" de cuisineConduite du lavage en machine de lavaisselleAppliquer les consignes du Plan de Maîtrise Sanitaire (P.M.S. - 140 hStage en entreprise - Réception et stockage des marchandisesPlanification, mise en place du matériel e | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Sensibilsation aux enjeux de développement durable - l'eaule soll'énergie et climat - 21 hSensibilisation aux valeurs de la république, l'éducation citoyenne et à la prévention des violences sexuelles et sexistes - les valeurs de la république,Droits et obligations du citoyenLaïcité Egalité hommes/femmesAlerter et orienter - 7 hSensibilisation aux enjeux numériques - Les outils numériquesLes bons usages du numériques - 7 hCertiphyto - RèglementationPrévention des risques pour l'environnementPrévention des risques pour la santéStratégies visant à limiter le recours aux produits phytosanaitaires - 14 hPositionnement - Test de connaissances et de compétences professionnelles - 35 hUcare : réaliser la taille fruitière - Réalisation des opérations de taille de formationRéalisation des opérations de taille de productionRestructuration des vergers âgés - 70 hEntretien du matériel et des équipements - Préparation du matériel et organisation des tâches en fonction des consignes, du travail en équipe et des aléasRéglage du matériel et ajustement des réglages en cours de travailEntretien courant des matérielsPetites réparations sur le matérielEntretien des protections individuelles et collectivesNettoyage et rangement des outils et matérielsCommunication en situation professionnelle - 105 hCréation d'un espage payasager - Préparation du travail et organisation des tâches en fonction des consignes, du travail en équipe et des aléas,Travaux infrastructure d'un espace en suivant le plan d'exécutionTravaux de plantation des végétauxTravaux de semis et d'engazonnementCommunication professionnelle - 224 hTravaux d'entretien d'un espace paysager - Préparation du travail d'organisation des tâches en fonction des consignes, du travail en équipe et des aléas,Entretien des espaces paysagers et naturelsEntretien des installations et des infrastructures paysagèresCommunication en situation professionnelle - 266 hAgir dans son environnement économique, social et territorial - Prise de position dans une situation à caractère social et civiqueUtilisation d'outils dans des situations de la vie courante,Expression à travers une réalisation personnelleAdoption de comportement favorisant l'équilibre personnelAdaptat | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T19" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé polyvalent en restauration</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP agricole jardinier paysagiste</t>
         </is>
       </c>
       <c r="U19" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10921944/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10910464/true/false/false/true</t>
         </is>
       </c>
       <c r="V19" s="7" t="inlineStr">
@@ -2729,27 +2713,27 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Assistant(e) de vie aux familles (TP) [HSP 1er NQ]</t>
+          <t>Action préparatoire aux métiers de l'agriculture [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>GRETA CFA AQUITAINE</t>
+          <t>CFPPA 47</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>24120 Terrasson-Lavilledieu</t>
+          <t>24240 Monbazillac</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Rue Rue Eugene LEROY Pepiniere des Metiers | 24120 Terrasson-Lavilledieu | France</t>
+          <t>EPLEFPA PERIGORD - LEGTPA PERIGUEUX | Route du Chateau Domaine de LA BRIE | 24240 Monbazillac | France</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Durée de 861 heures (dont 301 heures en entreprise)</t>
+          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -2759,17 +2743,17 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>https://greta-cfa-aquitaine.fr/</t>
+          <t>http://www.epl47.educagri.fr/cfppa.html</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>contact@greta-cfa-aquitaine.fr</t>
+          <t>cfppa.ste-livrade@educagri.fr</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>contact@greta-cfa-aquitaine.fr | pole.sante24@greta-cfa-aquitaine.fr</t>
+          <t>cfppa.ste-livrade@educagri.fr | cfppa.perigueux@educagri.fr</t>
         </is>
       </c>
       <c r="K20" s="5" t="inlineStr">
@@ -2784,19 +2768,15 @@
       </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
-          <t>0553027502</t>
+          <t>0553583391</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>0553027502</t>
-        </is>
-      </c>
-      <c r="O20" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0553583391</t>
+        </is>
+      </c>
+      <c r="O20" s="5" t="inlineStr"/>
       <c r="P20" s="5" t="inlineStr">
         <is>
           <t>Formation financée par la région</t>
@@ -2810,17 +2790,13 @@
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr">
         <is>
-          <t>Accueil / Intégration dans la formation - Intégration au groupe et à la formationS'approprier les objectifs de la formation et repérer son futur environnement professionnelPositionnementsFormalisation des parcours et sécurisation administrativeAppropriation des plateformes FOAD mobilisables - 21 hRéussir sa formation en centre - Modules sur les savoirs de base appliqués au secteur professionnel : mathématiques, français appliqués au secteur, informatiqueRenforcement de l'acquisition de compétences comportementales et Soft skills : savoirs être professionnels adaptés aux différents métiers du secteurMéthodologie d'apprentissage apprendre à apprendre - 21 hRéussir sa formation en entreprise - Préparation /Techniques de recherche de stage-Définition des objectifs individuels,choix du type d'entreprise et/ou du service,mise à disposition et aide à la recherche de liste d'adresses et contacts,accompagnement à la démarche de recherche, entretien, négociation.Exploitation des acquis au retour de stage-Retour partagé des expériences, -Travail de réflexivité. - 21 hEntretenir le logement et le linge d'un particulier - Relation professionnelle dans le cadre d'une prestation d'entretien chez un particulierCommunication professionnelle et relation avec la personne aidéePrévention des risques domestiques et travail en sécurité au domicile d'un particulierOrganisation du travailEntretien du logement avec les techniques et les gestes professionnels appropriésEntretien du linge (produits et techniques) repassage et initiation à la coutureRespect des règles environnementales/Hygiène et sécuritéEvaluation en cours de formation (mise en situation et écrit) - 105 hAccompagner la personne dans ses activités essentielles du quotidien et dans ses projets - Relation avec la personne aidée et son entourageBesoins fondamentaux / Handicap / Vieillissement et patho associées.La personne aidée dans son cadre de vie et en lien avec son entourage. Maintien du lien social et accompagnement dans la réalisation de son projet de vie /PAP / outil numériqueAutonomie physique, intellectuelle et sociale de la personneAide à la toilette, à l'habillage, aux déplacements/Aide aux courses, à la préparation et à la prise des repas Mobilisation, ergonomie / transferts, déplacementsBientraitancePrévention risques pro - 161 hSST - Situer son rôle d'acteur de prévention | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T20" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel assistant de vie aux familles</t>
-        </is>
-      </c>
+          <t>Découverte des filières et des métiers - Les filières, les métiers, les acteursLes spécificités du territoire L'emploi agricole sur le territoireLes types d'entreprises du bassin d'emploi et leur fonctionnement La saisonnalité des travaux Le matériel et les risques professionnels des métiers - 42 hElaboration du projet professionnel - Remobilisation et confiance en soiPréparation immersion en entreprise Se tester en milieu professionnelTRE et coaching vers le stage : Cartographie professionnelle, mobilité, savoir candidater, trouver un stage/emploi (CV Entretien LM) - Accompagnement personnalisé - 56 hConsolidation et concrétisation du projet professionnel - Choix du projet suite aux découvertes et immersionsConsolidation du projet : ciblage activités, d'un l'emploi, savoirs, savoir-être, formations.TRE et coaching vers l'emploi/formation choisi. Accompagnement personnalisé.Accéder à une qualification professionnelle ou à un emploi : définir son besoin de compétences et les étapes de son projet (formation/emploi) tableau de bord du projet, inscription en formation - 56 hAcquisition des compétences nécessaires à l'intégration professionnelle - Compétences sociales et civiques / Savoir-être, aptitudes professionnelles / formation / Communication verbale/non verbale Intégration en milieu professionnel / formationSanté et sécurité au travail - 49 hIdentification des freins, Accompagnent Socio Pro - Validation par le stagiaire de sa capacité à intégrer une formationIdentification des freins à l'entrée en formation : mobilité, Financiers, Handicap, Socio, Logement, restaurationAccompagnement dans la levée des freins : Comportement, Langage, Sociabilisation, Savoir de base, Savoir de base...Possibilités offertes par le HSP et des autres dispositifs d'accompagnement.Si besoin, accompagnement individualisé. - 42 hSensibilisation aux enjeux de développement durable - - Gestion de la ressource en eau en agriculture- Agronomie : Respect des sols et de son vivant en agriculture- Gestion des énergies et impact sur notre climat - 21 hSensibilisation aux valeurs de la république - - Sensibilisation aux valeurs de la république et éducation citoyenne- Prévention des violences sexuelles et sexistes - 7 hSensibilisation aux enjeux du numérique - - Présentation des différents outils numériques accessible au centre de formation- | Organisme | CFPPA 47 | http://www.epl47.educagri.fr/cfppa.html | Lieu de la formation</t>
+        </is>
+      </c>
+      <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10921978/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10910503/true/false/false/false</t>
         </is>
       </c>
       <c r="V20" s="5" t="inlineStr">
@@ -2842,27 +2818,27 @@
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Assistant(e) de vie aux familles (TP) [HSP 1er NQ]</t>
+          <t>Agent(e) des travaux forestiers (BPA) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>GRETA CFA AQUITAINE</t>
+          <t>CFPPA 47</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>24100 Bergerac</t>
+          <t>24300 Nontron</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>LEO LAGRANGE FORMATION | 15 Rue Neuve D Argenson | 24100 Bergerac | France</t>
+          <t>MAISON FAMILIALE RURALE PERIGORD LIMOUSIN - NONTRON | Place DES DROITS DE L HOMME | 24300 Nontron | France</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 1225 heures (dont 350 heures en entreprise)</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -2872,17 +2848,17 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>https://greta-cfa-aquitaine.fr/</t>
+          <t>http://www.epl47.educagri.fr/cfppa.html</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>contact@greta-cfa-aquitaine.fr</t>
+          <t>cfppa.ste-livrade@educagri.fr</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>contact@greta-cfa-aquitaine.fr | bergerac@leolagrange-formation.fr</t>
+          <t>cfppa.ste-livrade@educagri.fr | mfr.nontron@mfr.asso.fr</t>
         </is>
       </c>
       <c r="K21" s="7" t="inlineStr">
@@ -2897,12 +2873,12 @@
       </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
-          <t>0553247496</t>
+          <t>0553603193</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>0553247496</t>
+          <t>0553603193</t>
         </is>
       </c>
       <c r="O21" s="7" t="inlineStr">
@@ -2923,17 +2899,17 @@
       <c r="R21" s="7" t="inlineStr"/>
       <c r="S21" s="7" t="inlineStr">
         <is>
-          <t>Accueil / Intégration dans la formation - Intégration au groupe et à la formationS'approprier les objectifs de la formation et repérer son futur environnement professionnelPositionnementsFormalisation des parcours et sécurisation administrativeAppropriation des plateformes FOAD mobilisables - 21 hRéussir sa formation en centre - Modules sur les savoirs de base appliqués au secteur professionnel : mathématiques, français appliqués au secteur, informatiqueRenforcement de l'acquisition de compétences comportementales et Soft skills : savoirs être professionnels adaptés aux différents métiers du secteurMéthodologie d'apprentissage apprendre à apprendre - 21 hRéussir sa formation en entreprise - Préparation /Techniques de recherche de stage-Définition des objectifs individuels,choix du type d'entreprise et/ou du service,mise à disposition et aide à la recherche de liste d'adresses et contacts,accompagnement à la démarche de recherche, entretien, négociation.Exploitation des acquis au retour de stage-Retour partagé des expériences, -Travail de réflexivité. - 21 hEntretenir le logement et le linge d'un particulier - Relation professionnelle dans le cadre d'une prestation d'entretien chez un particulierCommunication professionnelle et relation avec la personne aidéePrévention des risques domestiques et travail en sécurité au domicile d'un particulierOrganisation du travailEntretien du logement avec les techniques et les gestes professionnels appropriésEntretien du linge (produits et techniques) repassage et initiation à la coutureRespect des règles environnementales/Hygiène et sécuritéEvaluation en cours de formation (mise en situation et écrit) - 105 hAccompagner la personne dans ses activités essentielles du quotidien et dans ses projets - Relation avec la personne aidée et son entourageBesoins fondamentaux / Handicap / Vieillissement et patho associées.La personne aidée dans son cadre de vie et en lien avec son entourage. Maintien du lien social et accompagnement dans la réalisation de son projet de vie /PAP / outil numériqueAutonomie physique, intellectuelle et sociale de la personneAide à la toilette, à l'habillage, aux déplacements/Aide aux courses, à la préparation et à la prise des repas Mobilisation, ergonomie / transferts, déplacementsBientraitancePrévention risques pro - 161 hSST - Situer son rôle d'acteur de prévention | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Positionnement BPA Travaux Forestiers - Évaluer le niveau de connaissances pour construire un parcours deformation individualisé qualifiant et/ou diplômant - 14 hConnaissances générales, sociales et économiques intégrant le concept de gestion durable des ressources forestières - UCG1 / UCG 2 - UCG1 Mobiliser les outils nécessaires au traitement de l'information et à la communication dans la vie professionnelle et sociale:Communiquer oralement et à l'écritUtiliser les techniques de collecte et de traitement de l'informationTraiter les mathématiquesUtiliser les outils informatiques et de télécommunicationUCG2 Mobiliser des connaissances relatives aux domaines civique, social etéconomique :Utiliser les règles du droit du travail/protection socialeconnaître les bases de la gestionconnaître la filière dans son ensemble - 223 hConnaissances générales scientifiques intégrant le concept de gestion durable des ressources forestières - UCG 3 : Mobiliser des connaissances pour mettre en oeuvre des pratiques professionnelles respectueuses de l'environnement et de la santé humaineMobiliser des connaissances pour appréhender l'impact environnemental des pratiques professionnellesMobiliser des connaissances pour prévenir les risques et préserver la santé humaine - 40 hConnaissances scientifiques et techniques relatives au domaine forestier intégrant le concept de gestion durable des ressources forestières - UCO1:Mobiliser, en vue de sa pratique professionnelle, les connaissances scientifiques et techniques relatives à la forêtMobiliser des connaissances scientifiques et techniques relatives à l'arbre et à son milieuMobiliser des connaissances scientifiques et techniques relatives à laproduction forestièreUCO2:Mobiliser des connaissances scientifiques et techniques relatives à l'utilisation des matériels et équipements d'exploitation forestièreConnaître le fonctionnement des matériels et installations forestiersConnaître les techniques des matériels et installations forestieres - 198 hConnaissances professionnelles relatives au domaine forestier intégrant le concept de gestion durable des ressources forestières - BPA Travaux de sylvicultureUCS1TS:Effectuer les travaux de régénération forestièrePréparer la mise en place d'un peuplementMettre en place un peuplementProtéger un peuplementUCS2TS:Réaliser les opérations d'entretien d'un jeune peuplementRéaliser le d&amp;eacut | Validation | Type de validation : | Diplôme autres ministères | Certifications :</t>
         </is>
       </c>
       <c r="T21" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel assistant de vie aux familles</t>
+          <t>Type de validation : | Diplôme autres ministères | Certifications : | BPA option travaux forestiers spécialité travaux de sylviculture</t>
         </is>
       </c>
       <c r="U21" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10925800/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10913180/true/false/false/false</t>
         </is>
       </c>
       <c r="V21" s="7" t="inlineStr">
@@ -2950,32 +2926,32 @@
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Agent(e) de service médico-social (TP) [HSP 1er NQ]</t>
+          <t>Employé(e) commercial (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>GRETA DU LIMOUSIN</t>
+          <t>INFREP DORDOGNE</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>23000 Saint-Sulpice-le-Guérétois</t>
+          <t>24100 Bergerac</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>AFPA - CENTRE DE GUÉRET | NC LE CLOCHER | 23000 Saint-Sulpice-le-Guérétois | France</t>
+          <t>TALIS COMPETENCES &amp; CERTIFICATIONS - BERGERAC | 110 Avenue PAULDOUMER | 24100 Bergerac | France</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 980 heures (dont 315 heures en entreprise)</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
@@ -2985,17 +2961,17 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>https://greta-du-limousin.fr/</t>
+          <t>https://www.infrep.org/</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr</t>
+          <t>infrep24@infrep.org</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr | formations-gueret@afpa.fr | jean-philippe.croze@afpa.fr</t>
+          <t>infrep24@infrep.org | v.rousseau@talis-cc.com | patricia.rieupet@talis-bs.com</t>
         </is>
       </c>
       <c r="K22" s="5" t="inlineStr">
@@ -3010,12 +2986,12 @@
       </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
-          <t>0642090687</t>
+          <t>0553221200</t>
         </is>
       </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>0642090687 | 0640895124</t>
+          <t>0553221200</t>
         </is>
       </c>
       <c r="O22" s="5" t="inlineStr">
@@ -3036,22 +3012,22 @@
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr">
         <is>
-          <t>Intégration/ Présentation de la formation - Intégration au groupe et à la formationFormalisation des parcours et sécurisation administrativeFinalisation des dossiers de rémunérationRappel des plannings, emploi du tempsRappel du règlement intérieur - 3 hDiagnostic / Positionnement - Positionnements écritsEntretien individuel exploratoireBilan - synthèse et proposition de parcours - 4 hBloc de compétence 1 - Réaliser le nettoyage et le bio nettoyage des locaux en s'adaptant à la présence des résidents - Participer à la vie de l'établissementAppliquer les techniques professionnelles d'entretien des locaux dans les espaces communs, la chambre du résident, la salle de bain dans le respect de la présence des résidentsUtiliser les produits, matériels, protocoles, en se protégeant et en protégeant les autres Gérer le temps de son interventionS'organiser et gérer des stocksComprendre la notion de développement durable et l'intégrer dans son activité professionnelle au quotidien. - 126 hBloc de compétence 2 - Contribuer aux prestations du service hôtelier en respectant les standards de qualité de l'établissement - Contribuer au service du linge des résidents et de l'établissement, gérer les stocks en lingerieConnaitre et appliquer les moyens de prévention des infections, précautions standards, précautions en cas d'épidémieAssurer la réfection d'un lit inoccupéContribuer au service des repas des résidents, respecter les goûts et consignes, adapter la présentation pour favoriser l'autonomie, préparer la salle à manger dans le respect des normes qualité de l'établissementCommuniquer avec les résidents, respecter leurs habitudes et autonomie - 98 hBloc de compétence 3 - Accompagner le résident dans les gestes de la vie quotidienne en tenant compte du projet - Accompagner le résident dans ses déplacementsAccompagner le résident à prendre son repas et à boireAppréhender les incidences des pathologies, handicaps et déficiences dans la vie quotidienne des résidentsCommuniquer avec l'équipe pluridisciplinaireObserver, écouter et établir des relations avec les résidentsIntervenir dans le respect des gestes de sécurité - 119 hPréparation à la certification - Accompagnement à la réalisation du dossier pro Mise en situation professionnelle.Entretien techniqueEntretien final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>INTEGRATION Communication professionnelle - Accueil des participants et présentation de l'organisme de formation, de l'équipe pédagogique et administrativePrésentation des objectifs du stage, de l'organisation générale de l'action et du cadre de l'action.Diagnostic- positionnement Présentation du livret stagiairePrésentation du règlement intérieur Sensibilisation aux valeurs de la république, à l'éducation citoyenne et à la prévention des violences sexuelles et sexistesDynamique de groupe contrat de formation et annexe pédagogiqueCommunication : Présentation croisée, Brèves de comptoir, Le BlasonI - 21 hCOMPETENCES NUMERIQUES - Etat des lieux des équipements et moyens de connexion pour chaque stagiaire de l'action Prise en main de la plateforme e learning de chaque organisme Utilisation des outils numériques tels que : Le DRIVE- GOOGLE DOCS- GOOGLE SHEETS- GOOGLE SLIDESMobilisation et animation des plateformes numériques en lien avec les CCP du Titre professionnel Les nouvelles technologies de la communication et leurs impactenvironnemental - 14 hModule 1 - METTRE A DISPOSITION DES CLIENTS LES PRODUITS DE L'UNITE MARCHANDE DANS UN ENVIRONNEMENT OMNICANAL - APPROVISIONNER L'UNITE MARCHANDE ASSURER LA PRESENTATION MARCHANDE DES PRODUITS DANS LE MAGASIN CONTRIBUER A LA GESTION ET OPTIMISER LES STOCKS TRAITER LES COMMANDES DE PRODUITS DE CLIENTS - 309 hModule 2 - ACCUEILLIR LES CLIENTS ET REPONDRE A LEUR DEMANDE DANS UN ENVIRONNEMENT OMNICANAL... - ACCUEILLIR, RENSEIGNER ET SERVIR LES CLIENTS CONTRIBUER A L'AMELIORATION DE L'EXPERIENCE D'ACHATTENIR UN POSTE DE CAISSE ET SUPERVISER LES CAISSES LIBRE-SERVICE - 310 hDEVELOPPEMENT DURABLE ET ACTIVITE PROFESSIONNELLE - sensibilisation a la transition énergétique, écologique et sociétale Néo TERRA Niveau 1enjeux mondiaux, nationaux et regionaux ecoresponsabilité au quotidienNEO TERRA Niveau 2 Compétences sectorielles en lien avec la transition energétique, écologique et sociétale sensibilisation aux innovations en lien avec l'activité professionnelle du commerce (commerce équitable, impact du e commerce, achat responsable et solidaire, circuits court, économie circulaire, recyclage et réemploi... - 28 hACCOMPAGNEMENT A LA RECHERCHE D'EMPLOI - Présentation de la plateforme TALENTS D'ICIcréation d'un compte sur le site Création et actualisation d'un CVCréation de compte sur les sites dédiés à la recherche d'emploiMise en relation avec les entreprises pour les recherches | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T22" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de service médico-social</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé commercial</t>
         </is>
       </c>
       <c r="U22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10926927/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10913186/true/false/false/false</t>
         </is>
       </c>
       <c r="V22" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-23&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-24&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W22" s="5" t="inlineStr">
@@ -3063,32 +3039,32 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Employé(e) commercial (TP) [HSP 1er NQ]</t>
+          <t>Conseiller, Conseillère de vente (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>INFREP DORDOGNE</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>23000 Saint-Sulpice-le-Guérétois</t>
+          <t>24100 Bergerac</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>AFPA - CENTRE DE GUÉRET | NC LE CLOCHER | 23000 Saint-Sulpice-le-Guérétois | France</t>
+          <t>TALIS COMPETENCES &amp; CERTIFICATIONS - BERGERAC | 110 Avenue PAULDOUMER | 24100 Bergerac | France</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 980 heures (dont 315 heures en entreprise)</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -3098,17 +3074,17 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
+          <t>https://www.infrep.org/</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+          <t>infrep24@infrep.org</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-gueret@afpa.fr | jean-philippe.croze@afpa.fr</t>
+          <t>infrep24@infrep.org | v.rousseau@talis-cc.com | patricia.rieupet@talis-bs.com</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
@@ -3123,12 +3099,12 @@
       </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
-          <t>0642090687</t>
+          <t>0553221200</t>
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>0642090687 | 0640895124</t>
+          <t>0553221200</t>
         </is>
       </c>
       <c r="O23" s="7" t="inlineStr">
@@ -3149,22 +3125,22 @@
       <c r="R23" s="7" t="inlineStr"/>
       <c r="S23" s="7" t="inlineStr">
         <is>
-          <t>TP Employé commercial - Période d'intégration Employé Commercial - Intégrer son groupe et sa formation J'apprends à apprendreS'approprier les objectifs de la formation et repérer son futur environnement professionnelPréciser ses besoins de formation et contractualiser son parcours personnaliséS'inscrire dans une perspective d'emploi - 35 hTP Employé commercial - Module 1 Mettre à disposition des clients les produits de l'unité marchande dans un environnement omnicanal - - Appliquer les règles et les obligations légales du recyclage, du tri sélectif des déchets et de la réduction du gaspillageRéceptionner et stocker la marchandiseComprendre les règles de merchandisingParticiper à la mise en oeuvre d'une opération commercialeVeiller à la mise en oeuvre des mesures de prévention adaptées à l'hygiène et à la sécuritéTraiter les commandes des clients - 140 hTP Employé commercial - Période d'application en entreprise 1 - Se confronter à la réalité professionnelleMettre en application des acquisDévelopper des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP Employé commercial - Module 2 Accueillir et accompagner le client dans un point de vente - Accueillir les clients et mettre en oeuvre des conditions favorables à l'accueil des personnes en situation de handicapProposer les programmes et services de fidélisation de l'unité marchande et conclure l'entretien de venteTenir un poste de caisse et superviser les caisses libre-serviceComprendre l'évolution du digital et les enjeux de la valorisation de l'expérience d'achat dans un contexte omnicanalValoriser l'image de l'unité marchande en s'appropriant les principes majeurs de l'écocitoyenneté tout au long de l'expérience d'achat - 140 hTP Employé commercial - Période d'application en entreprise 2 (environnement omnicanal) - Se confronter à la réalité professionnelleMettre en application des acquisRenforcer ses compétences transversesDévelopper son réseau professionnel - 140 hTP Employé commercial - Période de certification - Certification Employé Commercial - 35 hTP Employé commercial - Sensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa prop | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>INTEGRATION Communication professionnelle ... - Accueil des participants et présentation de l'organisme de formation, de l'équipe pédagogique et administrativePrésentation des objectifs de la formation, de l'organisation générale de l'action et du cadre de l'action.Diagnostic - positionnement Présentation du livret stagiairePrésentation du règlement intérieur Sensibilisation aux valeurs de la république, à l'éducation citoyenne et à la prévention des violences sexuelles et sexistesDynamique de groupe contrat de formation et de l'annexe pédagogiqueCommunication : Présentation croisée, Brèves de comptoir, Le Blason - 21 hCOMPETENCES NUMERIQUES - Etat des lieux des équipements et moyens de connexion pour chaque stagiaire de l'action Prise en main de la plateforme e learning de chaque organisme Utilisation des outils numériques tels que : Le DRIVE- GOOGLE DOCS- GOOGLE SHEETS- GOOGLE SLIDESMobilisation et animation des plateformes numériques en lien avec lesLes nouvelles technologies de la communication et leurs impactsenvironnementaux (RGPD à inclure) - 28 hCONTRIBUER A L'EFFICACITE COMMERCIALE D'UNE UNITE MARCHANDE DANS UN ENVIRONNEMENT OMNICANAL - ASSURER UNE VIEILLE PROFESSIONNELLE ET COMMERCIALE PARTICIPER A LA GESTION DES FLUX MARCHANDSCONTRIBUER AU MERCHANDISING ANALYSER SES PERFORMANCES COMMERCIALES ET EN RENDRE COMPTE - 442 hAMELIORER L'EXPERIENCE CLIENT DANS UN ENVIRONNEMENT OMNICANAL - REPRESENTER L'UNITE MARCHANDE ET CONTRIBUER A LA VALORISATION DE SON IMAGE CONSEILLER LE CLIENT EN CONDUISANT L'ENTRETIEN DE VENTE ASSURER LE SUIVI DE SES VENTES CONTRIBUER A LA FIDELISATION EN CONSOLIDANT L'EXPERIENCE CLIENT - 443 hDEVELOPPEMENT DURABLE ET ACTIVITE PROFESSIONNELLE - Sensibilisation a la transition énergétique, écologique et sociétale Néo TERRA Niveau 1enjeux mondiaux, nationaux et regionaux ecoresponsabilité au quotidienNEO TERRA Niveau 2 Compétences sectorielles en lien avec la transition energétique, écologique et sociétale sensibilisation aux innovations en lien avec l'activité professionnelle du commerce (commerce équitable, impact du e commerce, achat responsable et solidaire, circuits court, économie circulaire, recyclage et réemploi... - 21 hACOMPAGNEMENT VERS L'EMPLOI - Présentation de la plateforme TALENTS D'ICIcréation d'un compte sur le site Création et actualisation d'un CVCréation de compte sur les sites dédiés à la recherche d'emploiMise en relation avec les entreprises pour les recher | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T23" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé commercial</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller de vente</t>
         </is>
       </c>
       <c r="U23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10926932/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10913199/true/false/false/true</t>
         </is>
       </c>
       <c r="V23" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-23&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-24&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W23" s="7" t="inlineStr">
@@ -3176,32 +3152,32 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Assistant(e) de vie aux familles (TP) [HSP 1er NQ]</t>
+          <t>Action Préparatoire aux métiers du BTP [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>GRETA DU LIMOUSIN</t>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>23000 Saint-Sulpice-le-Guérétois</t>
+          <t>24100 Bergerac</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>AFPA - CENTRE DE GUÉRET | LE CLOCHER | 23000 Saint-Sulpice-le-Guérétois | France</t>
+          <t>IDC PRO - CFA CONSTRUCTION SUD DORDOGNE | ZA LE LIBRAIRE | 24100 Bergerac | France</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -3211,17 +3187,17 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>https://greta-du-limousin.fr/</t>
+          <t>http://www.afpa.fr/</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr | formations-gueret@afpa.fr | jean-philippe.croze@afpa.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | administratif@idcpro.fr</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr">
@@ -3236,19 +3212,15 @@
       </c>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>0642090687</t>
+          <t>0553733257</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
         <is>
-          <t>0642090687 | 0640895124</t>
-        </is>
-      </c>
-      <c r="O24" s="5" t="inlineStr">
-        <is>
-          <t>Certifiante</t>
-        </is>
-      </c>
+          <t>0553733257</t>
+        </is>
+      </c>
+      <c r="O24" s="5" t="inlineStr"/>
       <c r="P24" s="5" t="inlineStr">
         <is>
           <t>Formation financée par la région</t>
@@ -3262,22 +3234,18 @@
       <c r="R24" s="5" t="inlineStr"/>
       <c r="S24" s="5" t="inlineStr">
         <is>
-          <t>Intégration-présentation de la formation - Intégration au groupe et à la formationFormalisation des parcours et sécurisation administrativeFinalisation des dossiers de rémunérationRappel des plannings, emploi du tempsRappel du règlement intérieur - 4 hDiagnostic / Positionnement - Positionnements écritsEntretien individuel exploratoireBilan - synthèse et proposition de parcours - 7 hPrésentation du métier et du secteur - Présentation du secteur santé social Intervention de professionnels Fonctions et place de l'ADVFDroits et devoirs dans l'exercice du métier - 21 hModule Réussir sa formation en centre de formation et en entreprise - Modules sur les savoirs de base appliqués au secteur professionnel : mathématiques, français appliqués au secteur, informatiqueTechniques de recherche de stage, FLIRenforcement de l'acquisition de compétences comportementales. Méthodologie d'apprentissage apprendre à apprendre PAE *Préparation : -Définition des objectifs individuels,choix du type d'entreprise et/ou du service,mise à disposition et aide à la recherche de liste d'adresses et contacts,accompagnement à la démarche de recherche, entretien, négociation.Accompagnement : suivi et bilan en entreprise (stagiai - 63 hCCP 1 : Entretenir le logement et le linge d'un particulier - Relation professionnelle dans le cadre d'une prestation d'entretien chez un particulierCommunication professionnelle et relation avec la personne aidéePrévention des risques domestiques et travail en sécurité au domicile d'un particulierOrganisation du travailEntretien du logement avec les techniques et les gestes professionnels appropriésEntretien du linge (produits et techniques) repassage et initiation à la coutureRespect des règles environnementales/Hygiène et sécuritéEvaluation en cours de formation (mise en situation et écrit) - 126 hCCP 2 : Accompagner la personne dans les actes essentiels du quotidien - La relation avec la personne aidée et son entourageLes besoins fondamentauxLe handicapVieillissement et pathologies associées.Prévention des risques professionnelsL'autonomie physique, intellectuelle et sociale de la personneMobilisation et ergonomie / transferts et déplacementsAide à la toilette, à l'habillage et aux déplacementsAnimation et vie sociale.Aide aux courses, à la préparation et à la prise des repas Diététique et hygiène alimentair | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
-        </is>
-      </c>
-      <c r="T24" s="5" t="inlineStr">
-        <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel assistant de vie aux familles</t>
-        </is>
-      </c>
+          <t>Période d'intégration - Période d'intégration Intégrer son groupe et sa formationS'approprier le cadre et les objectifs de la formation préparatoire Développer sa culture numérique et prendre en main la plateforme MètisDécouvrir la boîte à outils numériqueDécouvrir Mètis et se repérer dans son parcoursPasser les tests de positionnementPréciser ses besoins de formation et contractualiser son parcours personnaliséS'inscrire dans une continuité de parcours certifiant ou une perspective d'emploi, un contrat en alternanceInitier son portefeuille de compétences - 35 hModule 1 : Découverte des métiers du secteur BTP et de leurs évolutions - Immersions sur les plateaux de formation - Découverte des métiers Les travaux publics : Canalisateur, maçon voirie réseaux divers, conducteur d'engins... Le gros oeuvre : Maçon, charpentier, couvreur zingueur... Le second oeuvre : Peintre, Carreleur, agent de maintenance des bâtiments, plombier, électricien, menuisier...Visites d'entreprises : Préparer, réaliser et exploiter une visite en entreprise Participation à des évènementiels Salons, jobs dating à partir d'une préparation collectiveMatinale entreprise (témoignages professionnels)BILAN INDIVIDUEL D'ORIENTATION - 70 hModule 2 : Acquérir le socle des connaissances nécessaires pour aller vers les métiers de l'industrie - Se remettre à niveau en mathématiquesUtiliser le système métriqueApprendre à lire des documents techniques, des plans....Développer sa communication écrite, son expression orale, comprendre les règles et instructionsTravailler en équipe et adopter la posture professionnelle attendueBILAN INDIVIDUEL D'ORIENTATION - 70 hModule 3 : Acquérir les bases des connaissances techniques et les gestes professionnels d'un métier - Réaliser un ouvrage simple en tenant compte des exigences de sécurité Identifier le matériel et les équipements nécessaires à la réalisation d'un ouvrage simplePréparer la matière nécessaire à la réalisation d'un ouvrage simpleRéaliser un ouvrage simpleMaintenir, l'organisation et la propreté du poste de travailTravailler en sécurité et conformément à la réglementation Repérer les risques liés à l'exercice des métiers de l'industrie Se sensibiliser au développement durable dans les métiers du BTPBILAN INDIVIDUEL D'ORIENTATION - 105 | Organisme | DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE | http://www.afpa.fr | Lieu de la formation</t>
+        </is>
+      </c>
+      <c r="T24" s="5" t="inlineStr"/>
       <c r="U24" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10926939/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10921925/true/false/false/true</t>
         </is>
       </c>
       <c r="V24" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-23&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-24&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W24" s="5" t="inlineStr">
@@ -3289,32 +3257,32 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Conseiller, Conseillère de vente (TP) [HSP 1er NQ]</t>
+          <t>Employé(e) polyvalent(e) en restauration (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
+          <t>GRETA CFA AQUITAINE</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>23000 Saint-Sulpice-le-Guérétois</t>
+          <t>24750 Boulazac Isle Manoire</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>AFPA - CENTRE DE GUÉRET | NC LE CLOCHER | 23000 Saint-Sulpice-le-Guérétois | France</t>
+          <t>AFPA PERIGUEUX | Avenue Ambroise Croizat Z.I de Boulazac | 24750 Boulazac Isle Manoire | France</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
+          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
@@ -3324,17 +3292,17 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>http://www.afpa.fr/</t>
+          <t>https://greta-cfa-aquitaine.fr/</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
+          <t>contact@greta-cfa-aquitaine.fr</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-gueret@afpa.fr | jean-philippe.croze@afpa.fr</t>
+          <t>contact@greta-cfa-aquitaine.fr | formations-perigueux@afpa.fr</t>
         </is>
       </c>
       <c r="K25" s="7" t="inlineStr">
@@ -3349,12 +3317,12 @@
       </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>0642090687</t>
+          <t>0617668622</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>0642090687 | 0640895124</t>
+          <t>0617668622</t>
         </is>
       </c>
       <c r="O25" s="7" t="inlineStr">
@@ -3375,22 +3343,22 @@
       <c r="R25" s="7" t="inlineStr"/>
       <c r="S25" s="7" t="inlineStr">
         <is>
-          <t>TP Conseiller de vente - Période d'intégration CV - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hTP Conseiller de vente - M1 - Contribuer à l'efficacité commerciale d'une unité marchande dans un environnement omnicanal - Connaître les différents contextes de la vente de services et de produitsConnaître les fondamentaux de la démarche marketingMener une étude de marché et établir le diagnostic de l'unité marchandeConnaître les différentes techniques et méthodes d'approvisionnementRéaliser des inventairesAppliquer les règles et les obligations légales du recyclage, du tri sélectif des déchets et de la réduction du gaspillageComprendre les règles de merchandisingMettre en place une opération commercialeSuivre et analyser les évolutions et exploiter les résultats pour proposer des ajustements - 245 hTP Conseiller de vente - Période en entreprise 1 - Se confronter à la réalité professionnelleMettre en application des acquisDévelopper des compétences transverses Etablir un réseau favorisant l'insertion professionnelle - 140 hTP Conseiller de vente - M2 - Améliorer l'expérience client dans un environnement omnicanal - Comprendre l'évolution du digital et son impact sur le métierValoriser l'offre de produits et de services de l'unité marchande sur les sites marchands et les médias sociauxAccueillir le client et mettre en oeuvre des conditions favorables à l'accueil des personnes en situation de handicapProcéder à l'enregistrement et à l'encaissementConnaître le cadre juridique de la vente et les enjeux du suivi de la relation commercialeConnaître les fondamentaux de la démarche marketingS'approprier et défendre les principes majeurs de l'écocitoyenneté tout au long de l'expérience d'achat - 210 hTP Conseiller de vente - Période en entreprise 2 - Se confronter à la réalité professionnelle Mettre en application des acquis Renforcer ses compétences transverses Développer son réseau professionnel - 140 hTP Conseiller de vente - Période de certification - Certification Conseiller de vente - 35 | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Accueil / Intégration dans la formation - Intégration au groupe et à la formationS'approprier les objectifs de la formation et repérer son futur environnement professionnelPositionnementsFormalisation des parcours et sécurisation administrative - 7 hRéussir sa formation en centre de formation et en entreprise - Techniques de recherche de stageRenforcement de l'acquisition de compétences comportementales et Soft skills : savoirs être professionnels adaptés aux différents métiers du secteurPAE - Préparation : -définition des objectifs individuels,choix du type d'entreprise et/ou du service,mise à disposition et aide à la recherche de liste d'adresses et contacts,accompagnement à la démarche de recherche, entretien, négociation. Accompagnement : -suivi et bilan en entreprise (stagiaire + formateur référent + tuteur)retour partagé des expériences, travail de réflexivité. - 14 hPréparer en assemblage des hors-d'oeuvre, des desserts et des préparations de type "snacking" - Préparation des matières premières alimentaires destinéesà la transformation et à l'assemblageRéalisation de l'assemblage et du dressage des horsd'oeuvre, des desserts et des préparations de type"snacking"Appliquer les règles d'hygiène et de sécurité alimentaire (haccp) - 154 hRéaliser des grillades et remettre en température des préparations culinaires élaborées à l'avance (PCEA) - Remise en température de préparationsculinaires élaborées à l'avance (PCEA)Réalisation d'une production culinaire au poste grilladeAppliquer les règles d'hygiène et de sécurité alimentaire (haccp) - 154 hAccueillir les clients et distribuer les plats en restauration self-service - Mise en place de la salle à manger du self-serviceRéalisation de la mise en place de la distribution Service aux postes froids et chaudsEnregistrement du contenu des plateaux repas et des préparations de type "snacking"EncaissementRespect des consignes de santé et de sécurité au travail - 147 hRéaliser le nettoyage de la batterie de cuisine et le lavage en machine de la vaisselle - Nettoyage de la "batterie" de cuisineConduite du lavage en machine de lavaisselleAppliquer les consignes du Plan de Maîtrise Sanitaire (P.M.S. - 140 hStage en entreprise - Réception et stockage des marchandisesPlanification, mise en place du matériel e | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T25" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller de vente</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé polyvalent en restauration</t>
         </is>
       </c>
       <c r="U25" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10926944/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10921944/true/false/false/false</t>
         </is>
       </c>
       <c r="V25" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-23&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-24&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W25" s="7" t="inlineStr">
@@ -3402,32 +3370,32 @@
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Employé(e) polyvalent(e) en restauration (TP) [HSP 1er NQ]</t>
+          <t>Assistant(e) de vie aux familles (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>GRETA DU LIMOUSIN</t>
+          <t>GRETA CFA AQUITAINE</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>23000 Saint-Sulpice-le-Guérétois</t>
+          <t>24120 Terrasson-Lavilledieu</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>AFPA - CENTRE DE GUÉRET | LE CLOCHER | 23000 Saint-Sulpice-le-Guérétois | France</t>
+          <t>Rue Rue Eugene LEROY Pepiniere des Metiers | 24120 Terrasson-Lavilledieu | France</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
+          <t>Durée de 861 heures (dont 301 heures en entreprise)</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
@@ -3437,17 +3405,17 @@
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>https://greta-du-limousin.fr/</t>
+          <t>https://greta-cfa-aquitaine.fr/</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr</t>
+          <t>contact@greta-cfa-aquitaine.fr</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr | formations-gueret@afpa.fr | jean-philippe.croze@afpa.fr</t>
+          <t>contact@greta-cfa-aquitaine.fr | pole.sante24@greta-cfa-aquitaine.fr</t>
         </is>
       </c>
       <c r="K26" s="5" t="inlineStr">
@@ -3462,12 +3430,12 @@
       </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
-          <t>0642090687</t>
+          <t>0553027502</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
-          <t>0642090687 | 0640895124</t>
+          <t>0553027502</t>
         </is>
       </c>
       <c r="O26" s="5" t="inlineStr">
@@ -3488,22 +3456,22 @@
       <c r="R26" s="5" t="inlineStr"/>
       <c r="S26" s="5" t="inlineStr">
         <is>
-          <t>TITRE PRO AGENT DE RESTAURATION Intégration - Entrée en formationPrésentation de l'équipe pédagogique et administrativeVisite des locaux de formation (salles et plateaux techniques)Intégration au groupeFormalisation du parcours de formationInstruction du dossier et sécurisation administrativeExplicitation du calendrier de l'alternance et de l'emploi du temps de formationLecture et explication du Règlement Intérieur - 3 hTITRE PRO AGENT DE RESTAURATION Présentation du métier - Présentation du secteur "Hôtellerie-Restauration-Alimentation" (HRA)Intervention d'un professionnel / témoignage d'anciens stagiaires - 7 hTITRE PRO AGENT DE RESTAURATION Les modalités de certification - Présentation des modalités de certificationLe référentiel de formation et de certification TITRE PROFESSIONNEL Agent de restaurationLe calendrier prévisionnel des épreuves - 4 hTITRE PRO AGENT DES RESTAURATION Diagnostic - Positionnement - Positionnements écritsPositionnements pratiquesEntretien individuel exploratoire de confirmation de projetBilan - exploitation des positionnementsSynthèse et proposition de parcoursSignature du Contrat Pédagogique - 14 hTITRE PRO AGENT DE RESTAURATION Acquisition des connaissances et des compétences culinaires de base - Les principes et règlementation en matière de sécurité alimentaire (Codex alimentarius, GBPH, PMS, méthodologie HACCP,Le vocabulaire culinaire de base et la technologie culinaire : les produits alimentaires (denrées végétales, carnées, condiments, épices, produits dérivés, laitiers... les bases des méthodes de conservation, de cuisson- les principaux matériels et ustensiles culinaires- les préparations de base : fruits, légumes, oeufs, viandes, poissons, entremets, pâtisseries- les principales techniques d'assemblage - 28 hTITRE PRO AGENT DES RESTAURATION Préparer en assemblage des hors d'oeuvre, des desserts et des préparations de type "snacking" (CCP 1) - - Préparer les matières premières alimentaires destinées à la transformation et à l'assemblage - Réaliser l'assemblage et le dressage des hors-d'oeuvre, des desserts et des préparations de type snacking - 56 hTITRE PRO AGENT DE RESTAURATION Réaliser des grillades et remettre en température des PCEA Préparations Culinaires Elaborées à l'Avance) (CCP 2) - - Effectuer la remise en température de préparations culinaire | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Accueil / Intégration dans la formation - Intégration au groupe et à la formationS'approprier les objectifs de la formation et repérer son futur environnement professionnelPositionnementsFormalisation des parcours et sécurisation administrativeAppropriation des plateformes FOAD mobilisables - 21 hRéussir sa formation en centre - Modules sur les savoirs de base appliqués au secteur professionnel : mathématiques, français appliqués au secteur, informatiqueRenforcement de l'acquisition de compétences comportementales et Soft skills : savoirs être professionnels adaptés aux différents métiers du secteurMéthodologie d'apprentissage apprendre à apprendre - 21 hRéussir sa formation en entreprise - Préparation /Techniques de recherche de stage-Définition des objectifs individuels,choix du type d'entreprise et/ou du service,mise à disposition et aide à la recherche de liste d'adresses et contacts,accompagnement à la démarche de recherche, entretien, négociation.Exploitation des acquis au retour de stage-Retour partagé des expériences, -Travail de réflexivité. - 21 hEntretenir le logement et le linge d'un particulier - Relation professionnelle dans le cadre d'une prestation d'entretien chez un particulierCommunication professionnelle et relation avec la personne aidéePrévention des risques domestiques et travail en sécurité au domicile d'un particulierOrganisation du travailEntretien du logement avec les techniques et les gestes professionnels appropriésEntretien du linge (produits et techniques) repassage et initiation à la coutureRespect des règles environnementales/Hygiène et sécuritéEvaluation en cours de formation (mise en situation et écrit) - 105 hAccompagner la personne dans ses activités essentielles du quotidien et dans ses projets - Relation avec la personne aidée et son entourageBesoins fondamentaux / Handicap / Vieillissement et patho associées.La personne aidée dans son cadre de vie et en lien avec son entourage. Maintien du lien social et accompagnement dans la réalisation de son projet de vie /PAP / outil numériqueAutonomie physique, intellectuelle et sociale de la personneAide à la toilette, à l'habillage, aux déplacements/Aide aux courses, à la préparation et à la prise des repas Mobilisation, ergonomie / transferts, déplacementsBientraitancePrévention risques pro - 161 hSST - Situer son rôle d'acteur de prévention | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T26" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé polyvalent en restauration</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel assistant de vie aux familles</t>
         </is>
       </c>
       <c r="U26" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10928102/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10921978/true/false/false/true</t>
         </is>
       </c>
       <c r="V26" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-23&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-24&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W26" s="5" t="inlineStr">
@@ -3515,32 +3483,32 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Canalisateur, canalisatrice (TP) [HSP 1er NQ]</t>
+          <t>Assistant(e) de vie aux familles (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>GRETA DU LIMOUSIN</t>
+          <t>GRETA CFA AQUITAINE</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>23300 La Souterraine</t>
+          <t>24100 Bergerac</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>CFIM TP | 29 Rue HENRI PLUYAUD | 23300 La Souterraine | France</t>
+          <t>LEO LAGRANGE FORMATION | 15 Rue Neuve D Argenson | 24100 Bergerac | France</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -3550,17 +3518,17 @@
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>https://greta-du-limousin.fr/</t>
+          <t>https://greta-cfa-aquitaine.fr/</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr</t>
+          <t>contact@greta-cfa-aquitaine.fr</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr | cfimtp.jc@orange.fr</t>
+          <t>contact@greta-cfa-aquitaine.fr | bergerac@leolagrange-formation.fr</t>
         </is>
       </c>
       <c r="K27" s="7" t="inlineStr">
@@ -3575,12 +3543,12 @@
       </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>0555040383</t>
+          <t>0553247496</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>0555040383</t>
+          <t>0553247496</t>
         </is>
       </c>
       <c r="O27" s="7" t="inlineStr">
@@ -3601,22 +3569,22 @@
       <c r="R27" s="7" t="inlineStr"/>
       <c r="S27" s="7" t="inlineStr">
         <is>
-          <t>Accompagnement socio-professionnel - - Diagnostic des besoin sociaux et socio-professionnels- Suivi et réajustement du diagnostic, si nécessaire tout au long du parcours de formation- Accompagnement vers l'emploi, techniques de recherche d'emploi - 35 hPrésentation de la formation et positionnement pédagogique - - Présentation de la formation et de l'environnement socio-professionnel- Confirmation ou affinement du projet professionnel, Positionnement, prise en compte des acquis et de l'expérience- Construction du parcours individualisé prenant appui sur le positionnement, Contractualisation du parcours individualisé dans le contrat de formation - 7 hActions de sensibilisation - Renforcer ses capacités d'agir en faveur de l'écoresponsabilité au quotidien Les bonnes pratiques environnementales dans les entreprises : Tri des déchets, vidéo Youtube de la FNTP sur la présentation du recyclage des déchets dans les TPAuto-formation proposée de 5 modules en ligne recycleur Académie sur la plateforme tp.demain pour des meilleures pratiques et maitriser la réglementationSensibilisation aux valeurs de la République, à l'éducation citoyenne et à la prévention des violences sexuelle et sexistes Sensibilisation à agir en faveur d'un numérique responsable - 35 hModule 1 - réaliser les travaux de préparation et de réfection d'un chantier de canalisations enterrées. - Installer des dispositifs de sécurité pour chantier de voirie et réseauxRéaliser les traçages préparatoires à la pose des réseauxTravailler à proximité des réseaux Déposer et reposer des éléments de voirie : bordures, fontes de voierie, couches superficielles de chausséeSynthèse des apprentissages de l'activité - 112 hModule 2 - construire un réseau d'assainissement en travaux publics - Poser en tranchée un collecteur d'assainissement d'eaux usées ou d'eaux pluvialesRéaliser les branchements particuliers, eaux usées et eaux pluvialesRéaliser les ouvrages coulés en place et maçonnés d'un chantier de canalisationsRéaliser l'enrobage de la canalisation et le remblayage de la tranchéeSynthèse des apprentissages de l'activité - 280 hModule 3 - construire un réseau d'adduction d'eau potable en travaux publics - Construire un réseau d'adduction d'eau potable en PVC et en fonteConstruire un réseau d'adduction d'eau potable en PeHD (Polyéthyl | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Accueil / Intégration dans la formation - Intégration au groupe et à la formationS'approprier les objectifs de la formation et repérer son futur environnement professionnelPositionnementsFormalisation des parcours et sécurisation administrativeAppropriation des plateformes FOAD mobilisables - 21 hRéussir sa formation en centre - Modules sur les savoirs de base appliqués au secteur professionnel : mathématiques, français appliqués au secteur, informatiqueRenforcement de l'acquisition de compétences comportementales et Soft skills : savoirs être professionnels adaptés aux différents métiers du secteurMéthodologie d'apprentissage apprendre à apprendre - 21 hRéussir sa formation en entreprise - Préparation /Techniques de recherche de stage-Définition des objectifs individuels,choix du type d'entreprise et/ou du service,mise à disposition et aide à la recherche de liste d'adresses et contacts,accompagnement à la démarche de recherche, entretien, négociation.Exploitation des acquis au retour de stage-Retour partagé des expériences, -Travail de réflexivité. - 21 hEntretenir le logement et le linge d'un particulier - Relation professionnelle dans le cadre d'une prestation d'entretien chez un particulierCommunication professionnelle et relation avec la personne aidéePrévention des risques domestiques et travail en sécurité au domicile d'un particulierOrganisation du travailEntretien du logement avec les techniques et les gestes professionnels appropriésEntretien du linge (produits et techniques) repassage et initiation à la coutureRespect des règles environnementales/Hygiène et sécuritéEvaluation en cours de formation (mise en situation et écrit) - 105 hAccompagner la personne dans ses activités essentielles du quotidien et dans ses projets - Relation avec la personne aidée et son entourageBesoins fondamentaux / Handicap / Vieillissement et patho associées.La personne aidée dans son cadre de vie et en lien avec son entourage. Maintien du lien social et accompagnement dans la réalisation de son projet de vie /PAP / outil numériqueAutonomie physique, intellectuelle et sociale de la personneAide à la toilette, à l'habillage, aux déplacements/Aide aux courses, à la préparation et à la prise des repas Mobilisation, ergonomie / transferts, déplacementsBientraitancePrévention risques pro - 161 hSST - Situer son rôle d'acteur de prévention | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T27" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel canalisateur</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel assistant de vie aux familles</t>
         </is>
       </c>
       <c r="U27" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10935749/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10925800/true/false/false/true</t>
         </is>
       </c>
       <c r="V27" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-23&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-24&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W27" s="7" t="inlineStr">
@@ -3633,7 +3601,7 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Maçon, maçonne en voirie et réseaux divers (TP) [HSP 1er NQ]</t>
+          <t>Agent(e) de service médico-social (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
@@ -3643,17 +3611,17 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>23300 La Souterraine</t>
+          <t>23000 Saint-Sulpice-le-Guérétois</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>CFIM TP | 29 Rue HENRI PLUYAUD | 23300 La Souterraine | France</t>
+          <t>AFPA - CENTRE DE GUÉRET | NC LE CLOCHER | 23000 Saint-Sulpice-le-Guérétois | France</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
@@ -3673,7 +3641,7 @@
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr | cfimtp.jc@orange.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr | formations-gueret@afpa.fr | jean-philippe.croze@afpa.fr</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
@@ -3688,12 +3656,12 @@
       </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>0555040383</t>
+          <t>0642090687</t>
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>0555040383</t>
+          <t>0642090687 | 0640895124</t>
         </is>
       </c>
       <c r="O28" s="5" t="inlineStr">
@@ -3714,17 +3682,17 @@
       <c r="R28" s="5" t="inlineStr"/>
       <c r="S28" s="5" t="inlineStr">
         <is>
-          <t>Accompagnement socio-professionnel - Diagnostic des besoin sociaux et socio-professionnelsSuivi et réajustement du diagnostic, si nécessaire tout au long du parcours de formationAccompagnement vers l'emploi, techniques de recherche d'emploi - 35 hPrésentation de la formation et positionnement pédagogique - Présentation de la formation et de l'environnement socio-professionnelConfirmation ou affinement du projet professionnel,Positionnement, prise en compte des acquis et de l'expérienceConstruction du parcours individualisé prenant appui sur le positionnement,Contractualisation du parcours individualisé dans le contrat de formation - 7 hActions de sensibilisation - Renforcer ses capacités d'agir en faveur de l'écoresponsabilité au quotidien Les bonnes pratiques environnementales dans les entreprises : Tri des déchets, vidéo Youtube de la FNTP sur la présentation du recyclage des déchets dans les TPAuto-formation proposée de 5 modules en ligne recycleur Académie sur la plateforme tp.demain pour des meilleures pratiques et maitriser la réglementationSensibilisation aux valeurs de la République, à l'éducation citoyenne et à la prévention des violences sexuelle et sexistes Sensibilisation à agir en faveur d'un numérique responsable - 35 hModule 1 - construire des ouvrages de petite maçonnerie et réaliser les couches de surface - Construire des petits ouvrages d'aménagement urbain en maçonnerie ou en béton arméPoser des pavés et des dalles manufacturées Réaliser les dallages en béton pour les ouvrages de voirie en aménagement urbain Effectuer la synthèse des apprentissages de l'activité " Construire des petits ouvrages et réaliser les revêtements de surface"Évaluations de fin d'activité - 204 hModule 2 - Poser des bordures et des caniveaux - Mettre en oeuvre des produits manufacturés de type bordures et caniveaux Sceller les fontes de voirie Connaître les différentes fontes de voirie, leurs spécificités et leurs particularités en matière de mise en oeuvre provisoire et définitiveConnaître les différents produits de scellements et leurs spécificités en matière de temps de séchage et d'ouverture à la circulationEffectuer la synthèse des apprentissages de l'activité "Poser des bordures et des caniveaux"Évaluations ( QCM + Mise en situation professionnelle) - 211 hModule 3 - Construire les réseaux enterr&amp;e | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Intégration/ Présentation de la formation - Intégration au groupe et à la formationFormalisation des parcours et sécurisation administrativeFinalisation des dossiers de rémunérationRappel des plannings, emploi du tempsRappel du règlement intérieur - 3 hDiagnostic / Positionnement - Positionnements écritsEntretien individuel exploratoireBilan - synthèse et proposition de parcours - 4 hBloc de compétence 1 - Réaliser le nettoyage et le bio nettoyage des locaux en s'adaptant à la présence des résidents - Participer à la vie de l'établissementAppliquer les techniques professionnelles d'entretien des locaux dans les espaces communs, la chambre du résident, la salle de bain dans le respect de la présence des résidentsUtiliser les produits, matériels, protocoles, en se protégeant et en protégeant les autres Gérer le temps de son interventionS'organiser et gérer des stocksComprendre la notion de développement durable et l'intégrer dans son activité professionnelle au quotidien. - 126 hBloc de compétence 2 - Contribuer aux prestations du service hôtelier en respectant les standards de qualité de l'établissement - Contribuer au service du linge des résidents et de l'établissement, gérer les stocks en lingerieConnaitre et appliquer les moyens de prévention des infections, précautions standards, précautions en cas d'épidémieAssurer la réfection d'un lit inoccupéContribuer au service des repas des résidents, respecter les goûts et consignes, adapter la présentation pour favoriser l'autonomie, préparer la salle à manger dans le respect des normes qualité de l'établissementCommuniquer avec les résidents, respecter leurs habitudes et autonomie - 98 hBloc de compétence 3 - Accompagner le résident dans les gestes de la vie quotidienne en tenant compte du projet - Accompagner le résident dans ses déplacementsAccompagner le résident à prendre son repas et à boireAppréhender les incidences des pathologies, handicaps et déficiences dans la vie quotidienne des résidentsCommuniquer avec l'équipe pluridisciplinaireObserver, écouter et établir des relations avec les résidentsIntervenir dans le respect des gestes de sécurité - 119 hPréparation à la certification - Accompagnement à la réalisation du dossier pro Mise en situation professionnelle.Entretien techniqueEntretien final. | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T28" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel maçon en voirie et réseaux divers</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de service médico-social</t>
         </is>
       </c>
       <c r="U28" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10935754/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10926927/true/false/false/false</t>
         </is>
       </c>
       <c r="V28" s="5" t="inlineStr">
@@ -3746,27 +3714,27 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Conducteur, Conductrice de transport en commun sur route (TP) [HSP 1er NQ]</t>
+          <t>Employé(e) commercial (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>ECF CENTRE OUEST ATLANTIQUE</t>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>23000 Sainte-Feyre</t>
+          <t>23000 Saint-Sulpice-le-Guérétois</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>LES CHAMPS BLANCS Route de Saint-Laurent | 23000 Sainte-Feyre | France</t>
+          <t>AFPA - CENTRE DE GUÉRET | NC LE CLOCHER | 23000 Saint-Sulpice-le-Guérétois | France</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>Durée de 525 heures (dont 70 heures en entreprise)</t>
+          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
@@ -3776,17 +3744,17 @@
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>http://www.ecf.asso.fr/</t>
+          <t>http://www.afpa.fr/</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>ifp.limoges@ecf-cerca.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>ifp.limoges@ecf-cerca.fr | hsp23@ecf-cerca.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-gueret@afpa.fr | jean-philippe.croze@afpa.fr</t>
         </is>
       </c>
       <c r="K29" s="7" t="inlineStr">
@@ -3801,12 +3769,12 @@
       </c>
       <c r="M29" s="7" t="inlineStr">
         <is>
-          <t>0549089384</t>
+          <t>0642090687</t>
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr">
         <is>
-          <t>0549089384</t>
+          <t>0642090687 | 0640895124</t>
         </is>
       </c>
       <c r="O29" s="7" t="inlineStr">
@@ -3827,17 +3795,17 @@
       <c r="R29" s="7" t="inlineStr"/>
       <c r="S29" s="7" t="inlineStr">
         <is>
-          <t>1-Identifier les objectifs et étapes de la formation - Vérification du respect des prérequis Présentation du centre, de l'équipe pédagogique et des moyens matérielsPrésentation de la formationModalités pratiquesTour de tableEvaluation d'auto-positionnement - 3 h2-Acquérir les connaissances requises pour se préparer à l'épreuve théorique générale - Dispositions légales en matière de circulation routièreLe conducteurLa routeLes autres usagers de la routeRéglementation générale et divers Porter secoursPrécautions nécessaires en quittant le véhiculeEléments mécaniques Eléments liés à la sécuritéEquipements de sécurité des véhiculesUtilisation du véhicule et respect de l'environnement - 23 h3-Acquérir les connaissances requises pour se préparer aux interrogations orales et écrites - "Situations dégradées, accidents Conducteur Equipement véhicules Réglementation sociale européenne, française et transportDocs spécifiquesMasses, dimensions véhicules Règles de circulation, signalisationMécaniqueConduite conditions difficiles Comportement si accident Conduite montagne, zones accidentées Gestes-postures, accident du travail Chargement, surcharge Dépassement Dynamique véhicule Alcool, médicaments, stupéfiants, fatigueEco-conduite, conduite citoyenne Angles morts, porte-à-faux Comportement tunnels, passages à niveau Systèmes de sécurité, aide - 30 h4-Appliquer les consignes d'exploitation et effectuer les contrôles de sécurité dans le cadre d'un transport en commun - "* Respect des différentes réglementations sociale nationale, européenneVérification, utilisation du tachygraphe* Lecture de carte et calculs professionnelsCartes routières, GPS, internet, itinéraire* Contrôles de sécuritéRéglages poste de conduiteÉthylotest anti-démarrageDocuments de bordÉtat intérieur et extérieur véhiculeNiveauxOrganes du véhiculeEquipements dont la plateforme PMRZones du véhicule propices à la criminalitéSignalements* Consignes d'exploitationSystèmes embarquésTableaux de roulement &amp; planchette horaires,RégulationSupports d'enregistrement - 21 h5-Conduire et manoeuvrer en sécurité tout type de véhicule de transport en commun - * Conduite d | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>TP Employé commercial - Période d'intégration Employé Commercial - Intégrer son groupe et sa formation J'apprends à apprendreS'approprier les objectifs de la formation et repérer son futur environnement professionnelPréciser ses besoins de formation et contractualiser son parcours personnaliséS'inscrire dans une perspective d'emploi - 35 hTP Employé commercial - Module 1 Mettre à disposition des clients les produits de l'unité marchande dans un environnement omnicanal - - Appliquer les règles et les obligations légales du recyclage, du tri sélectif des déchets et de la réduction du gaspillageRéceptionner et stocker la marchandiseComprendre les règles de merchandisingParticiper à la mise en oeuvre d'une opération commercialeVeiller à la mise en oeuvre des mesures de prévention adaptées à l'hygiène et à la sécuritéTraiter les commandes des clients - 140 hTP Employé commercial - Période d'application en entreprise 1 - Se confronter à la réalité professionnelleMettre en application des acquisDévelopper des compétences transversesEtablir un réseau favorisant l'insertion professionnelle - 140 hTP Employé commercial - Module 2 Accueillir et accompagner le client dans un point de vente - Accueillir les clients et mettre en oeuvre des conditions favorables à l'accueil des personnes en situation de handicapProposer les programmes et services de fidélisation de l'unité marchande et conclure l'entretien de venteTenir un poste de caisse et superviser les caisses libre-serviceComprendre l'évolution du digital et les enjeux de la valorisation de l'expérience d'achat dans un contexte omnicanalValoriser l'image de l'unité marchande en s'appropriant les principes majeurs de l'écocitoyenneté tout au long de l'expérience d'achat - 140 hTP Employé commercial - Période d'application en entreprise 2 (environnement omnicanal) - Se confronter à la réalité professionnelleMettre en application des acquisRenforcer ses compétences transversesDévelopper son réseau professionnel - 140 hTP Employé commercial - Période de certification - Certification Employé Commercial - 35 hTP Employé commercial - Sensibilisation aux enjeux du développement durable - Néo Terra Niveau 1 - Rappel historique : du développement durable aux transitions énergétique, écologique et sociétale.Évaluer sa prop | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T29" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conducteur de transport en commun sur route</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé commercial</t>
         </is>
       </c>
       <c r="U29" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10935766/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10926932/true/false/false/true</t>
         </is>
       </c>
       <c r="V29" s="7" t="inlineStr">
@@ -3859,27 +3827,27 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Conducteur, Conductrice du transport routier de marchandises sur porteur (TP) [HSP 1er NQ]</t>
+          <t>Assistant(e) de vie aux familles (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>ECF CENTRE OUEST ATLANTIQUE</t>
+          <t>GRETA DU LIMOUSIN</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>23000 Sainte-Feyre</t>
+          <t>23000 Saint-Sulpice-le-Guérétois</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>LES CHAMPS BLANCS | 23000 Sainte-Feyre | France</t>
+          <t>AFPA - CENTRE DE GUÉRET | LE CLOCHER | 23000 Saint-Sulpice-le-Guérétois | France</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Durée de 595 heures (dont 175 heures en entreprise)</t>
+          <t>Durée de 1015 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -3889,17 +3857,17 @@
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>http://www.ecf.asso.fr/</t>
+          <t>https://greta-du-limousin.fr/</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr">
         <is>
-          <t>ifp.limoges@ecf-cerca.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>ifp.limoges@ecf-cerca.fr | hsp23@ecf-cerca.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr | formations-gueret@afpa.fr | jean-philippe.croze@afpa.fr</t>
         </is>
       </c>
       <c r="K30" s="5" t="inlineStr">
@@ -3914,12 +3882,12 @@
       </c>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>0549089384</t>
+          <t>0642090687</t>
         </is>
       </c>
       <c r="N30" s="5" t="inlineStr">
         <is>
-          <t>0549089384</t>
+          <t>0642090687 | 0640895124</t>
         </is>
       </c>
       <c r="O30" s="5" t="inlineStr">
@@ -3940,17 +3908,17 @@
       <c r="R30" s="5" t="inlineStr"/>
       <c r="S30" s="5" t="inlineStr">
         <is>
-          <t>1-Identifier les objectifs et étapes de la formation - "Vérification du respect des prérequis Présentation du centre, de l'équipe pédagogique et des moyens matérielsPrésentation de la formationModalités pratiquesTour de tableEvaluation d'auto-positionnement" - 3 h2-Acquérir les connaissances requises pour se préparer à l'épreuve théorique générale - Dispositions légales en matière de circulation routièreLe conducteurLa routeLes autres usagers de la routeRéglementation générale et divers Porter secoursPrécautions nécessaires en quittant le véhiculeEléments mécaniques Eléments liés à la sécuritéEquipements de sécurité des véhiculesUtilisation du véhicule et respect de l'environnement - 23 h3-Acquérir les connaissances requises pour se préparer aux interrogations orales et écrites - "Situations dégradées, accidents Conducteur Equipement véhicules Réglementation sociale européenne, française et transportDocs spécifiquesMasses, dimensions véhicules Règles de circulation, signalisationMécaniqueConduite conditions difficiles Comportement si accident Conduite montagne, zones accidentées Gestes-postures, accident du travail Chargement, surcharge Dépassement Dynamique véhicule Alcool, médicaments, stupéfiants, fatigueEco-conduite, conduite citoyenne Angles morts, porte-à-faux Comportement tunnels, passages à niveau Systèmes de sécurité, aide - 30 h4-Assurer les contrôles de sécurité et de conformité avant, pendant et après le transport de marchandises - Avant départ Contrôle docs nécessaires au conducteur &amp; à la circulationVérification état du véhicule &amp; ses équipements, validité des visites techniquesContrôles sécurité &amp; fluidesContrôle chargement, répartition, calage, arrimageContrôle indicateurs garantissant le fonctionnement du véhicule Pendant le parcours Contrôle dispositifs d'enregistrements de données sociales, organisationnelles, techniquesContrôle chargement, répartition, calage et arrimageSurveille état du véhicule et absence message d'alerteAprès transportContrôle état du véhiculeRendre compte si anomalie - 4 h5-Conduire et manoeuvrer en sécurité, de façon écologique et &amp;eacu | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Intégration-présentation de la formation - Intégration au groupe et à la formationFormalisation des parcours et sécurisation administrativeFinalisation des dossiers de rémunérationRappel des plannings, emploi du tempsRappel du règlement intérieur - 4 hDiagnostic / Positionnement - Positionnements écritsEntretien individuel exploratoireBilan - synthèse et proposition de parcours - 7 hPrésentation du métier et du secteur - Présentation du secteur santé social Intervention de professionnels Fonctions et place de l'ADVFDroits et devoirs dans l'exercice du métier - 21 hModule Réussir sa formation en centre de formation et en entreprise - Modules sur les savoirs de base appliqués au secteur professionnel : mathématiques, français appliqués au secteur, informatiqueTechniques de recherche de stage, FLIRenforcement de l'acquisition de compétences comportementales. Méthodologie d'apprentissage apprendre à apprendre PAE *Préparation : -Définition des objectifs individuels,choix du type d'entreprise et/ou du service,mise à disposition et aide à la recherche de liste d'adresses et contacts,accompagnement à la démarche de recherche, entretien, négociation.Accompagnement : suivi et bilan en entreprise (stagiai - 63 hCCP 1 : Entretenir le logement et le linge d'un particulier - Relation professionnelle dans le cadre d'une prestation d'entretien chez un particulierCommunication professionnelle et relation avec la personne aidéePrévention des risques domestiques et travail en sécurité au domicile d'un particulierOrganisation du travailEntretien du logement avec les techniques et les gestes professionnels appropriésEntretien du linge (produits et techniques) repassage et initiation à la coutureRespect des règles environnementales/Hygiène et sécuritéEvaluation en cours de formation (mise en situation et écrit) - 126 hCCP 2 : Accompagner la personne dans les actes essentiels du quotidien - La relation avec la personne aidée et son entourageLes besoins fondamentauxLe handicapVieillissement et pathologies associées.Prévention des risques professionnelsL'autonomie physique, intellectuelle et sociale de la personneMobilisation et ergonomie / transferts et déplacementsAide à la toilette, à l'habillage et aux déplacementsAnimation et vie sociale.Aide aux courses, à la préparation et à la prise des repas Diététique et hygiène alimentair | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T30" s="5" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conducteur du transport routier de marchandises sur porteur</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel assistant de vie aux familles</t>
         </is>
       </c>
       <c r="U30" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10935779/true/false/false/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10926939/true/false/false/true</t>
         </is>
       </c>
       <c r="V30" s="5" t="inlineStr">
@@ -3972,27 +3940,27 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>Agent(e) de propreté et d'hygiène (TP) [HSP 1er NQ]</t>
+          <t>Conseiller, Conseillère de vente (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>GRETA DU LIMOUSIN</t>
+          <t>DIRECTION REGIONALE AFPA NOUVELLE-AQUITAINE</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>23320 Saint-Vaury</t>
+          <t>23000 Saint-Sulpice-le-Guérétois</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>NC LA VALETTE | 23320 Saint-Vaury | France</t>
+          <t>AFPA - CENTRE DE GUÉRET | NC LE CLOCHER | 23000 Saint-Sulpice-le-Guérétois | France</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Durée de 735 heures (dont 175 heures en entreprise)</t>
+          <t>Durée de 945 heures (dont 280 heures en entreprise)</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
@@ -4002,17 +3970,17 @@
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>https://greta-du-limousin.fr/</t>
+          <t>http://www.afpa.fr/</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr</t>
         </is>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>ce.gretadulimousin@ac-limoges.fr | angelique.trayaud@ac-limoges.fr | marie.puybras@ac-limoges.fr</t>
+          <t>mc_psr_nouvelle_aquitaine@afpa.fr | formations-gueret@afpa.fr | jean-philippe.croze@afpa.fr</t>
         </is>
       </c>
       <c r="K31" s="7" t="inlineStr">
@@ -4027,12 +3995,12 @@
       </c>
       <c r="M31" s="7" t="inlineStr">
         <is>
-          <t>0555513480</t>
+          <t>0642090687</t>
         </is>
       </c>
       <c r="N31" s="7" t="inlineStr">
         <is>
-          <t>0555513480 | 0555123131</t>
+          <t>0642090687 | 0640895124</t>
         </is>
       </c>
       <c r="O31" s="7" t="inlineStr">
@@ -4053,17 +4021,17 @@
       <c r="R31" s="7" t="inlineStr"/>
       <c r="S31" s="7" t="inlineStr">
         <is>
-          <t>INTEGRATION - Intégration au groupe et à la formationFormalisation des parcours et sécurisation administrativeFinalisation des dossiers de rémunérationRappel des plannings, emploi du tempsRappel du règlement intérieur - 2 hDiagnostic / Positionnement - Positionnements écritsPositionnement pratiqueEntretien individuel exploratoireBilan - synthèse et proposition de parcours - 10 hPrésentation du métier et de son contexte - Présentation du "monde de la propreté" Intervention d'un professionnel / témoignage d'anciens stagiairesParticipation à des ateliers pratiques : présentation de produits d'entretien- présentation de matériels de nettoyage- démonstration de techniques d'entretienAteliers connaissance des entreprises du secteur de la propreté - 10 hPrésentation de la formation et la certification - Présentation de la formationIdentification des compétences professionnelles visées par le REAC du TP Agent(e) de Propreté et d'HygièneInformation sur le référentiel et les modalités de certification - 5 hCCP 1 : Prestation de nettoyage manuel - Réalisation d'une prestation de service d'entretien manuel adaptée aux locaux, aux surfaces et à leur utilisation par la mise en oeuvre de modes opératoires en respectant les règles d'hygiène et de sécurité, l'attitude de service et en intégrant les principes du développement durable.Apprentissage des techniques d'organisation des activités, de nettoyage, d'autocontrôle et de communication :1) Réalisation du nettoyage manuel des surfaces2) Réalisation du nettoyage manuel des sanitaires3) Réalisation du bionettoyage en environnement spécifique dans le respect des protocoles - 150 hCCP 2 : Prestation de nettoyage ou de remise en état mécanisés - Réalisation d'une prestation de services d'entretien mécanisé et/ou de remise en état mécanisée adaptée aux locaux et surfaces et à leur utilisation utilisation par la mise en oeuvre de modes opératoires en respectant les règles d'hygiène et de sécurité, l'attitude de service et en intégrant les principes du développement durable.Apprentissage des techniques d'organisation des activités, de nettoyage, d'autocontrôle et de communication :1) Réalisation d'un nettoyage mécanisé2) Réalisation d'une remise en état mécanisée - 175 hCompétenc | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>TP Conseiller de vente - Période d'intégration CV - Intégrer son groupe et sa formation S'approprier les objectifs de la formation et repérer son futur environnement professionnel Repérer les risques liés à l'exercice du métier et se sensibiliser au développement durable Préciser ses besoins de formation et contractualiser son parcours personnalisé S'inscrire dans une perspective d'emploi - 35 hTP Conseiller de vente - M1 - Contribuer à l'efficacité commerciale d'une unité marchande dans un environnement omnicanal - Connaître les différents contextes de la vente de services et de produitsConnaître les fondamentaux de la démarche marketingMener une étude de marché et établir le diagnostic de l'unité marchandeConnaître les différentes techniques et méthodes d'approvisionnementRéaliser des inventairesAppliquer les règles et les obligations légales du recyclage, du tri sélectif des déchets et de la réduction du gaspillageComprendre les règles de merchandisingMettre en place une opération commercialeSuivre et analyser les évolutions et exploiter les résultats pour proposer des ajustements - 245 hTP Conseiller de vente - Période en entreprise 1 - Se confronter à la réalité professionnelleMettre en application des acquisDévelopper des compétences transverses Etablir un réseau favorisant l'insertion professionnelle - 140 hTP Conseiller de vente - M2 - Améliorer l'expérience client dans un environnement omnicanal - Comprendre l'évolution du digital et son impact sur le métierValoriser l'offre de produits et de services de l'unité marchande sur les sites marchands et les médias sociauxAccueillir le client et mettre en oeuvre des conditions favorables à l'accueil des personnes en situation de handicapProcéder à l'enregistrement et à l'encaissementConnaître le cadre juridique de la vente et les enjeux du suivi de la relation commercialeConnaître les fondamentaux de la démarche marketingS'approprier et défendre les principes majeurs de l'écocitoyenneté tout au long de l'expérience d'achat - 210 hTP Conseiller de vente - Période en entreprise 2 - Se confronter à la réalité professionnelle Mettre en application des acquis Renforcer ses compétences transverses Développer son réseau professionnel - 140 hTP Conseiller de vente - Période de certification - Certification Conseiller de vente - 35 | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T31" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de propreté et d'hygiène</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conseiller de vente</t>
         </is>
       </c>
       <c r="U31" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/10939638/true/false/false/false</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10926944/true/false/false/true</t>
         </is>
       </c>
       <c r="V31" s="7" t="inlineStr">
@@ -4080,32 +4048,32 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Concours d'atsem (FOAD)</t>
+          <t>Employé(e) polyvalent(e) en restauration (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>GRETA DU LIMOUSIN</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>23000 Saint-Sulpice-le-Guérétois</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>AFPA - CENTRE DE GUÉRET | LE CLOCHER | 23000 Saint-Sulpice-le-Guérétois | France</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Durée de 522 heures (dont 261 heures en entreprise)</t>
+          <t>Durée de 1155 heures (dont 455 heures en entreprise)</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
@@ -4115,17 +4083,17 @@
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://greta-du-limousin.fr/</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr | formations-gueret@afpa.fr | jean-philippe.croze@afpa.fr</t>
         </is>
       </c>
       <c r="K32" s="5" t="inlineStr">
@@ -4140,40 +4108,48 @@
       </c>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0642090687</t>
         </is>
       </c>
       <c r="N32" s="5" t="inlineStr">
         <is>
-          <t>0366060201</t>
-        </is>
-      </c>
-      <c r="O32" s="5" t="inlineStr"/>
+          <t>0642090687 | 0640895124</t>
+        </is>
+      </c>
+      <c r="O32" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P32" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q32" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R32" s="5" t="inlineStr"/>
       <c r="S32" s="5" t="inlineStr">
         <is>
-          <t>Programme obligatoire Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Cadre politique et administratif de la France Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Activité d'éveil et de jeux Accueil de la petite enfance Nutrition Préparation des repas Annales Programme complémentaire Le métier d'ATSEM : connaissances techniques Hygiène et Nutrition Développement de l'enfant et jeux Le cadre administratif et juridique de la France" | Organisme | Centre européen de formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T32" s="5" t="inlineStr"/>
+          <t>TITRE PRO AGENT DE RESTAURATION Intégration - Entrée en formationPrésentation de l'équipe pédagogique et administrativeVisite des locaux de formation (salles et plateaux techniques)Intégration au groupeFormalisation du parcours de formationInstruction du dossier et sécurisation administrativeExplicitation du calendrier de l'alternance et de l'emploi du temps de formationLecture et explication du Règlement Intérieur - 3 hTITRE PRO AGENT DE RESTAURATION Présentation du métier - Présentation du secteur "Hôtellerie-Restauration-Alimentation" (HRA)Intervention d'un professionnel / témoignage d'anciens stagiaires - 7 hTITRE PRO AGENT DE RESTAURATION Les modalités de certification - Présentation des modalités de certificationLe référentiel de formation et de certification TITRE PROFESSIONNEL Agent de restaurationLe calendrier prévisionnel des épreuves - 4 hTITRE PRO AGENT DES RESTAURATION Diagnostic - Positionnement - Positionnements écritsPositionnements pratiquesEntretien individuel exploratoire de confirmation de projetBilan - exploitation des positionnementsSynthèse et proposition de parcoursSignature du Contrat Pédagogique - 14 hTITRE PRO AGENT DE RESTAURATION Acquisition des connaissances et des compétences culinaires de base - Les principes et règlementation en matière de sécurité alimentaire (Codex alimentarius, GBPH, PMS, méthodologie HACCP,Le vocabulaire culinaire de base et la technologie culinaire : les produits alimentaires (denrées végétales, carnées, condiments, épices, produits dérivés, laitiers... les bases des méthodes de conservation, de cuisson- les principaux matériels et ustensiles culinaires- les préparations de base : fruits, légumes, oeufs, viandes, poissons, entremets, pâtisseries- les principales techniques d'assemblage - 28 hTITRE PRO AGENT DES RESTAURATION Préparer en assemblage des hors d'oeuvre, des desserts et des préparations de type "snacking" (CCP 1) - - Préparer les matières premières alimentaires destinées à la transformation et à l'assemblage - Réaliser l'assemblage et le dressage des hors-d'oeuvre, des desserts et des préparations de type snacking - 56 hTITRE PRO AGENT DE RESTAURATION Réaliser des grillades et remettre en température des PCEA Préparations Culinaires Elaborées à l'Avance) (CCP 2) - - Effectuer la remise en température de préparations culinaire | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T32" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel employé polyvalent en restauration</t>
+        </is>
+      </c>
       <c r="U32" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122762/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10928102/true/false/false/true</t>
         </is>
       </c>
       <c r="V32" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-23&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W32" s="5" t="inlineStr">
@@ -4185,32 +4161,32 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Canalisateur, canalisatrice (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Centre européen de formation</t>
+          <t>GRETA DU LIMOUSIN</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>23300 La Souterraine</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>CFIM TP | 29 Rue HENRI PLUYAUD | 23300 La Souterraine | France</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1496 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -4220,17 +4196,17 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://greta-du-limousin.fr/</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr</t>
         </is>
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>info@cenef.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr | cfimtp.jc@orange.fr</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
@@ -4245,12 +4221,12 @@
       </c>
       <c r="M33" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0555040383</t>
         </is>
       </c>
       <c r="N33" s="7" t="inlineStr">
         <is>
-          <t>0366060201</t>
+          <t>0555040383</t>
         </is>
       </c>
       <c r="O33" s="7" t="inlineStr">
@@ -4260,33 +4236,33 @@
       </c>
       <c r="P33" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q33" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R33" s="7" t="inlineStr"/>
       <c r="S33" s="7" t="inlineStr">
         <is>
-          <t>Le programme obligatoire de la formation est le suivant : BC01 - ACCOMPAGNER LE DEVELOPPEMENT DU JEUNE ENFANT Développement moteur de l'enfant Développement psychique de l'enfant Anomalies du développement de l'enfant Statut juridique de l'enfant et de la famille Protection sanitaire et sociale de l'enfant et de la famille Anatomie et Physiologie Maintien de l'intégrité de l'organisme Accidents et maladies infantiles Hygiène et confort de l'enfant de 0 à 6 ans BC02 - EXERCER SON ACTIVITE EN MILIEU COLLECTIF Aménagements et équipements des espaces de vie du jeune enfant Hygiène et entretien des équipements Information et communication Activités d'éveil et de jeux BC03 - EXERCER SON ACTIVITE EN ACCUEIL INDIVIDUEL Accueil de la petite enfance Nutrition et préparation des repas BC07 - PREVENTION SANTE ENVIRONNEMENT Prévention, santé, environnement, tome 1 Prévention, santé, environnement, tome 2 MATIERES GENERALES Français Mathématiques Sciences Histoire - Géographie - Enseignement moral et civiques Des cours facultatifs, conçus pour enrichir l'apprentissage de l'élève, sont prévus : Epreuves blanches EP1, EP2, EP3, PSE , Matières générales Livret assistante maternelle | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>Accompagnement socio-professionnel - - Diagnostic des besoin sociaux et socio-professionnels- Suivi et réajustement du diagnostic, si nécessaire tout au long du parcours de formation- Accompagnement vers l'emploi, techniques de recherche d'emploi - 35 hPrésentation de la formation et positionnement pédagogique - - Présentation de la formation et de l'environnement socio-professionnel- Confirmation ou affinement du projet professionnel, Positionnement, prise en compte des acquis et de l'expérience- Construction du parcours individualisé prenant appui sur le positionnement, Contractualisation du parcours individualisé dans le contrat de formation - 7 hActions de sensibilisation - Renforcer ses capacités d'agir en faveur de l'écoresponsabilité au quotidien Les bonnes pratiques environnementales dans les entreprises : Tri des déchets, vidéo Youtube de la FNTP sur la présentation du recyclage des déchets dans les TPAuto-formation proposée de 5 modules en ligne recycleur Académie sur la plateforme tp.demain pour des meilleures pratiques et maitriser la réglementationSensibilisation aux valeurs de la République, à l'éducation citoyenne et à la prévention des violences sexuelle et sexistes Sensibilisation à agir en faveur d'un numérique responsable - 35 hModule 1 - réaliser les travaux de préparation et de réfection d'un chantier de canalisations enterrées. - Installer des dispositifs de sécurité pour chantier de voirie et réseauxRéaliser les traçages préparatoires à la pose des réseauxTravailler à proximité des réseaux Déposer et reposer des éléments de voirie : bordures, fontes de voierie, couches superficielles de chausséeSynthèse des apprentissages de l'activité - 112 hModule 2 - construire un réseau d'assainissement en travaux publics - Poser en tranchée un collecteur d'assainissement d'eaux usées ou d'eaux pluvialesRéaliser les branchements particuliers, eaux usées et eaux pluvialesRéaliser les ouvrages coulés en place et maçonnés d'un chantier de canalisationsRéaliser l'enrobage de la canalisation et le remblayage de la tranchéeSynthèse des apprentissages de l'activité - 280 hModule 3 - construire un réseau d'adduction d'eau potable en travaux publics - Construire un réseau d'adduction d'eau potable en PVC et en fonteConstruire un réseau d'adduction d'eau potable en PeHD (Polyéthyl | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T33" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel canalisateur</t>
         </is>
       </c>
       <c r="U33" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11122788/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10935749/true/false/false/true</t>
         </is>
       </c>
       <c r="V33" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-23&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W33" s="7" t="inlineStr">
@@ -4298,32 +4274,32 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Préparation au concours d'ATSEM</t>
+          <t>Maçon, maçonne en voirie et réseaux divers (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>AFEC</t>
+          <t>GRETA DU LIMOUSIN</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>23300 La Souterraine</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>AFEC (Siège) | Formation a distance | 75004 Paris | France</t>
+          <t>CFIM TP | 29 Rue HENRI PLUYAUD | 23300 La Souterraine | France</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Durée de 385 heures (dont 105 heures en entreprise)</t>
+          <t>Durée de 350 heures (dont 105 heures en entreprise)</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
@@ -4333,49 +4309,73 @@
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
-        </is>
-      </c>
-      <c r="I34" s="5" t="inlineStr"/>
-      <c r="J34" s="5" t="inlineStr"/>
+          <t>https://greta-du-limousin.fr/</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>ce.gretadulimousin@ac-limoges.fr</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>ce.gretadulimousin@ac-limoges.fr | cfimtp.jc@orange.fr</t>
+        </is>
+      </c>
       <c r="K34" s="5" t="inlineStr">
         <is>
-          <t>introuvable</t>
+          <t>france_travail</t>
         </is>
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M34" s="5" t="inlineStr"/>
-      <c r="N34" s="5" t="inlineStr"/>
-      <c r="O34" s="5" t="inlineStr"/>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="M34" s="5" t="inlineStr">
+        <is>
+          <t>0555040383</t>
+        </is>
+      </c>
+      <c r="N34" s="5" t="inlineStr">
+        <is>
+          <t>0555040383</t>
+        </is>
+      </c>
+      <c r="O34" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P34" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q34" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R34" s="5" t="inlineStr"/>
       <c r="S34" s="5" t="inlineStr">
         <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant les modules suivants Modules d'enseignement : - Accompagnement du développement de l'enfant de 2 à 6 ans - Préparation aux épreuves du concours - Examens blancs En complément de la formation : - Remise à niveau numérique - Plan d'action et bilan de formation - Posture professionnelle de l'ATSEM - Techniques de recherche d'emploi et de stage - Accompagnement à la suite de parcours | Organisme | AFEC | Lieu de la formation | AFEC (Siège)</t>
-        </is>
-      </c>
-      <c r="T34" s="5" t="inlineStr"/>
+          <t>Accompagnement socio-professionnel - Diagnostic des besoin sociaux et socio-professionnelsSuivi et réajustement du diagnostic, si nécessaire tout au long du parcours de formationAccompagnement vers l'emploi, techniques de recherche d'emploi - 35 hPrésentation de la formation et positionnement pédagogique - Présentation de la formation et de l'environnement socio-professionnelConfirmation ou affinement du projet professionnel,Positionnement, prise en compte des acquis et de l'expérienceConstruction du parcours individualisé prenant appui sur le positionnement,Contractualisation du parcours individualisé dans le contrat de formation - 7 hActions de sensibilisation - Renforcer ses capacités d'agir en faveur de l'écoresponsabilité au quotidien Les bonnes pratiques environnementales dans les entreprises : Tri des déchets, vidéo Youtube de la FNTP sur la présentation du recyclage des déchets dans les TPAuto-formation proposée de 5 modules en ligne recycleur Académie sur la plateforme tp.demain pour des meilleures pratiques et maitriser la réglementationSensibilisation aux valeurs de la République, à l'éducation citoyenne et à la prévention des violences sexuelle et sexistes Sensibilisation à agir en faveur d'un numérique responsable - 35 hModule 1 - construire des ouvrages de petite maçonnerie et réaliser les couches de surface - Construire des petits ouvrages d'aménagement urbain en maçonnerie ou en béton arméPoser des pavés et des dalles manufacturées Réaliser les dallages en béton pour les ouvrages de voirie en aménagement urbain Effectuer la synthèse des apprentissages de l'activité " Construire des petits ouvrages et réaliser les revêtements de surface"Évaluations de fin d'activité - 204 hModule 2 - Poser des bordures et des caniveaux - Mettre en oeuvre des produits manufacturés de type bordures et caniveaux Sceller les fontes de voirie Connaître les différentes fontes de voirie, leurs spécificités et leurs particularités en matière de mise en oeuvre provisoire et définitiveConnaître les différents produits de scellements et leurs spécificités en matière de temps de séchage et d'ouverture à la circulationEffectuer la synthèse des apprentissages de l'activité "Poser des bordures et des caniveaux"Évaluations ( QCM + Mise en situation professionnelle) - 211 hModule 3 - Construire les réseaux enterr&amp;e | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T34" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel maçon en voirie et réseaux divers</t>
+        </is>
+      </c>
       <c r="U34" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124184/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10935754/true/false/false/true</t>
         </is>
       </c>
       <c r="V34" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-23&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W34" s="5" t="inlineStr">
@@ -4387,32 +4387,32 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'aide-soignant</t>
+          <t>Conducteur, Conductrice de transport en commun sur route (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>ECF CENTRE OUEST ATLANTIQUE</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>23000 Sainte-Feyre</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>LES CHAMPS BLANCS Route de Saint-Laurent | 23000 Sainte-Feyre | France</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>Durée de 207 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 525 heures (dont 70 heures en entreprise)</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
@@ -4422,17 +4422,17 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>http://www.ecf.asso.fr/</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>ifp.limoges@ecf-cerca.fr</t>
         </is>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>ifp.limoges@ecf-cerca.fr | hsp23@ecf-cerca.fr</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
@@ -4447,40 +4447,48 @@
       </c>
       <c r="M35" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0549089384</t>
         </is>
       </c>
       <c r="N35" s="7" t="inlineStr">
         <is>
-          <t>0472892042</t>
-        </is>
-      </c>
-      <c r="O35" s="7" t="inlineStr"/>
+          <t>0549089384</t>
+        </is>
+      </c>
+      <c r="O35" s="7" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P35" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q35" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R35" s="7" t="inlineStr"/>
       <c r="S35" s="7" t="inlineStr">
         <is>
-          <t>Module 1 - Remise à niveau numérique préparatoireObjectifs : -Se connecter à une plateforme?de formation à distance -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - FrançaisObjectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - MathématiquesObjectif: Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - BiologieObjectif: Maîtriser les bases de la biologie nécessaires à l'entrée en école d'aide-soignant Module 5 - Compétences numériquesObjectif : Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire et du métier d'aide-soignantObjectifs :Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aideObjectif: Acquérir les bases de la communication pour bien travailler en équipe et prendre en charge les personnes accompagnées Module 8 - SoftskillsObjectifs: -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service... -Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admissionObjectifs:Anticiper son entrée en école d'aide-soignant -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stageObjectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploiObjectifs:Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétencesModule 12 - Stage en entrepriseObjectif : Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T35" s="7" t="inlineStr"/>
+          <t>1-Identifier les objectifs et étapes de la formation - Vérification du respect des prérequis Présentation du centre, de l'équipe pédagogique et des moyens matérielsPrésentation de la formationModalités pratiquesTour de tableEvaluation d'auto-positionnement - 3 h2-Acquérir les connaissances requises pour se préparer à l'épreuve théorique générale - Dispositions légales en matière de circulation routièreLe conducteurLa routeLes autres usagers de la routeRéglementation générale et divers Porter secoursPrécautions nécessaires en quittant le véhiculeEléments mécaniques Eléments liés à la sécuritéEquipements de sécurité des véhiculesUtilisation du véhicule et respect de l'environnement - 23 h3-Acquérir les connaissances requises pour se préparer aux interrogations orales et écrites - "Situations dégradées, accidents Conducteur Equipement véhicules Réglementation sociale européenne, française et transportDocs spécifiquesMasses, dimensions véhicules Règles de circulation, signalisationMécaniqueConduite conditions difficiles Comportement si accident Conduite montagne, zones accidentées Gestes-postures, accident du travail Chargement, surcharge Dépassement Dynamique véhicule Alcool, médicaments, stupéfiants, fatigueEco-conduite, conduite citoyenne Angles morts, porte-à-faux Comportement tunnels, passages à niveau Systèmes de sécurité, aide - 30 h4-Appliquer les consignes d'exploitation et effectuer les contrôles de sécurité dans le cadre d'un transport en commun - "* Respect des différentes réglementations sociale nationale, européenneVérification, utilisation du tachygraphe* Lecture de carte et calculs professionnelsCartes routières, GPS, internet, itinéraire* Contrôles de sécuritéRéglages poste de conduiteÉthylotest anti-démarrageDocuments de bordÉtat intérieur et extérieur véhiculeNiveauxOrganes du véhiculeEquipements dont la plateforme PMRZones du véhicule propices à la criminalitéSignalements* Consignes d'exploitationSystèmes embarquésTableaux de roulement &amp; planchette horaires,RégulationSupports d'enregistrement - 21 h5-Conduire et manoeuvrer en sécurité tout type de véhicule de transport en commun - * Conduite d | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T35" s="7" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conducteur de transport en commun sur route</t>
+        </is>
+      </c>
       <c r="U35" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128404/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10935766/true/false/false/false</t>
         </is>
       </c>
       <c r="V35" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-23&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W35" s="7" t="inlineStr">
@@ -4492,32 +4500,32 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Préparation à l'entrée en institut de formation d'infirmier</t>
+          <t>Conducteur, Conductrice du transport routier de marchandises sur porteur (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Leo Lagrange Formation</t>
+          <t>ECF CENTRE OUEST ATLANTIQUE</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>23000 Sainte-Feyre</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>LES CHAMPS BLANCS | 23000 Sainte-Feyre | France</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Durée de 228 heures (dont 35 heures en entreprise)</t>
+          <t>Durée de 595 heures (dont 175 heures en entreprise)</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
@@ -4527,17 +4535,17 @@
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>http://www.ecf.asso.fr/</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>ifp.limoges@ecf-cerca.fr</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>contact@ifra.fr</t>
+          <t>ifp.limoges@ecf-cerca.fr | hsp23@ecf-cerca.fr</t>
         </is>
       </c>
       <c r="K36" s="5" t="inlineStr">
@@ -4552,40 +4560,48 @@
       </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
+          <t>0549089384</t>
         </is>
       </c>
       <c r="N36" s="5" t="inlineStr">
         <is>
-          <t>0472892042</t>
-        </is>
-      </c>
-      <c r="O36" s="5" t="inlineStr"/>
+          <t>0549089384</t>
+        </is>
+      </c>
+      <c r="O36" s="5" t="inlineStr">
+        <is>
+          <t>Certifiante</t>
+        </is>
+      </c>
       <c r="P36" s="5" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q36" s="5" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R36" s="5" t="inlineStr"/>
       <c r="S36" s="5" t="inlineStr">
         <is>
-          <t>Module 1- Remise à niveau numérique préparatoire Objectifs:Se connecter à une plateforme de formation -Se repérer et naviguer sur une plateforme de formation -Se connecter à une classe virtuelle avec micro et caméra Module 2 - Remise à niveau - Français Objectif: Améliorer ses capacités rédactionnelles? rédiger, synthétiser, résumer, commenter Module 3 - Remise à niveau - Mathématiques Objectif :Utiliser les bases des mathématiques dans sa pratique professionnelle Module 4 - Remise à niveau - Biologie Objectif :Maîtriser les bases de la biologie nécessaires à l'entrée en école d'infirmier Module 5 - Compétences numériques Objectif:Être autonome sur l'outil numérique Module 6 - Connaissance du secteur sanitaire, de la petite enfance et du métier d'auxiliaire de puériculture Objectif:Connaître son environnement professionnel -Connaître son futur métier Module 7 - La relation d'aide Objectif :Acquérir les bases de la communication pour bien prendre en charge les personnes Module 8 - Softskills Objectifs : -Développer et savoir mobiliser ses savoir-être professionnels? faire preuve d'autonomie, travailler en équipe, organiser son travail, gérer son stress, avoir le sens du service.Acquérir les gestes et postures professionnels en adéquation avec les attentes actuelles du marché de l'emploi Module 9 - Aide à l'admission Objectifs: -Anticiper son entrée en école d'infirmier -Savoir se présenter et présenter son projet professionnel Module 10 - Accompagnement à la recherche de stage Objectifs:Comprendre l'environnement professionnel -Rechercher une offre de stage -Préparer sa prise de contact Module 11 - Accompagnement au retour à l'emploi Objectifs: -Être outillé pour réussir sa recherche d'emploi -Mettre à jour son profil compétences? Stage en entrepriseObjectif: Mieux appréhender l'environnement professionnel de la filière santé et soin | Organisme | Leo Lagrange Formation | Lieu de la formation | Formation a distance</t>
-        </is>
-      </c>
-      <c r="T36" s="5" t="inlineStr"/>
+          <t>1-Identifier les objectifs et étapes de la formation - "Vérification du respect des prérequis Présentation du centre, de l'équipe pédagogique et des moyens matérielsPrésentation de la formationModalités pratiquesTour de tableEvaluation d'auto-positionnement" - 3 h2-Acquérir les connaissances requises pour se préparer à l'épreuve théorique générale - Dispositions légales en matière de circulation routièreLe conducteurLa routeLes autres usagers de la routeRéglementation générale et divers Porter secoursPrécautions nécessaires en quittant le véhiculeEléments mécaniques Eléments liés à la sécuritéEquipements de sécurité des véhiculesUtilisation du véhicule et respect de l'environnement - 23 h3-Acquérir les connaissances requises pour se préparer aux interrogations orales et écrites - "Situations dégradées, accidents Conducteur Equipement véhicules Réglementation sociale européenne, française et transportDocs spécifiquesMasses, dimensions véhicules Règles de circulation, signalisationMécaniqueConduite conditions difficiles Comportement si accident Conduite montagne, zones accidentées Gestes-postures, accident du travail Chargement, surcharge Dépassement Dynamique véhicule Alcool, médicaments, stupéfiants, fatigueEco-conduite, conduite citoyenne Angles morts, porte-à-faux Comportement tunnels, passages à niveau Systèmes de sécurité, aide - 30 h4-Assurer les contrôles de sécurité et de conformité avant, pendant et après le transport de marchandises - Avant départ Contrôle docs nécessaires au conducteur &amp; à la circulationVérification état du véhicule &amp; ses équipements, validité des visites techniquesContrôles sécurité &amp; fluidesContrôle chargement, répartition, calage, arrimageContrôle indicateurs garantissant le fonctionnement du véhicule Pendant le parcours Contrôle dispositifs d'enregistrements de données sociales, organisationnelles, techniquesContrôle chargement, répartition, calage et arrimageSurveille état du véhicule et absence message d'alerteAprès transportContrôle état du véhiculeRendre compte si anomalie - 4 h5-Conduire et manoeuvrer en sécurité, de façon écologique et &amp;eacu | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+        </is>
+      </c>
+      <c r="T36" s="5" t="inlineStr">
+        <is>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel conducteur du transport routier de marchandises sur porteur</t>
+        </is>
+      </c>
       <c r="U36" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11128411/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10935779/true/false/false/true</t>
         </is>
       </c>
       <c r="V36" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-23&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W36" s="5" t="inlineStr">
@@ -4597,32 +4613,32 @@
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>CAP accompagnant éducatif petite enfance</t>
+          <t>Agent(e) de propreté et d'hygiène (TP) [HSP 1er NQ]</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>AFEC (Siège)</t>
+          <t>GRETA DU LIMOUSIN</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>75004 Paris</t>
+          <t>23320 Saint-Vaury</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Formation a distance | 75004 Paris | France</t>
+          <t>NC LA VALETTE | 23320 Saint-Vaury | France</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Durée de 1015 heures (dont 490 heures en entreprise)</t>
+          <t>Durée de 735 heures (dont 175 heures en entreprise)</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -4632,17 +4648,17 @@
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>https://plmpl.fr/c/zFjGj</t>
+          <t>https://greta-du-limousin.fr/</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr</t>
         </is>
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>paris@afec.fr</t>
+          <t>ce.gretadulimousin@ac-limoges.fr | angelique.trayaud@ac-limoges.fr | marie.puybras@ac-limoges.fr</t>
         </is>
       </c>
       <c r="K37" s="7" t="inlineStr">
@@ -4657,12 +4673,12 @@
       </c>
       <c r="M37" s="7" t="inlineStr">
         <is>
-          <t>0153368844</t>
+          <t>0555513480</t>
         </is>
       </c>
       <c r="N37" s="7" t="inlineStr">
         <is>
-          <t>0153368844</t>
+          <t>0555513480 | 0555123131</t>
         </is>
       </c>
       <c r="O37" s="7" t="inlineStr">
@@ -4672,33 +4688,33 @@
       </c>
       <c r="P37" s="7" t="inlineStr">
         <is>
-          <t>Formation financée par France Travail</t>
+          <t>Formation financée par la région</t>
         </is>
       </c>
       <c r="Q37" s="7" t="inlineStr">
         <is>
-          <t>À distance</t>
+          <t>En centre</t>
         </is>
       </c>
       <c r="R37" s="7" t="inlineStr"/>
       <c r="S37" s="7" t="inlineStr">
         <is>
-          <t>Formation individualisée et accompagnée par un formateur coach dédié, comprenant des modules d'enseignement et des prestations d'accompagnement. Modules d'enseignement professionnel : - EP1 Accompagnement du développement du jeune enfant (cadre d'intervention, accompagnement à l'autonomie l'enfant) - EP2 Exercer son activité en accueil collectif - EP3 Exercer son activité en accueil individuel Modules d'enseignements généraux : - Prévention santé environnement - Enseignements généraux (Mathématiques et sciences, Histoire-Géographie-Citoyenneté et français) En complément de la formation : - Remise à niveau numérique - Techniques de recherche d'emploi et de stage - Accompagnement au retour à l'emploi 3 Stages en entreprise 14 semaines | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
+          <t>INTEGRATION - Intégration au groupe et à la formationFormalisation des parcours et sécurisation administrativeFinalisation des dossiers de rémunérationRappel des plannings, emploi du tempsRappel du règlement intérieur - 2 hDiagnostic / Positionnement - Positionnements écritsPositionnement pratiqueEntretien individuel exploratoireBilan - synthèse et proposition de parcours - 10 hPrésentation du métier et de son contexte - Présentation du "monde de la propreté" Intervention d'un professionnel / témoignage d'anciens stagiairesParticipation à des ateliers pratiques : présentation de produits d'entretien- présentation de matériels de nettoyage- démonstration de techniques d'entretienAteliers connaissance des entreprises du secteur de la propreté - 10 hPrésentation de la formation et la certification - Présentation de la formationIdentification des compétences professionnelles visées par le REAC du TP Agent(e) de Propreté et d'HygièneInformation sur le référentiel et les modalités de certification - 5 hCCP 1 : Prestation de nettoyage manuel - Réalisation d'une prestation de service d'entretien manuel adaptée aux locaux, aux surfaces et à leur utilisation par la mise en oeuvre de modes opératoires en respectant les règles d'hygiène et de sécurité, l'attitude de service et en intégrant les principes du développement durable.Apprentissage des techniques d'organisation des activités, de nettoyage, d'autocontrôle et de communication :1) Réalisation du nettoyage manuel des surfaces2) Réalisation du nettoyage manuel des sanitaires3) Réalisation du bionettoyage en environnement spécifique dans le respect des protocoles - 150 hCCP 2 : Prestation de nettoyage ou de remise en état mécanisés - Réalisation d'une prestation de services d'entretien mécanisé et/ou de remise en état mécanisée adaptée aux locaux et surfaces et à leur utilisation utilisation par la mise en oeuvre de modes opératoires en respectant les règles d'hygiène et de sécurité, l'attitude de service et en intégrant les principes du développement durable.Apprentissage des techniques d'organisation des activités, de nettoyage, d'autocontrôle et de communication :1) Réalisation d'un nettoyage mécanisé2) Réalisation d'une remise en état mécanisée - 175 hCompétenc | Validation | Type de validation : | Diplôme autres ministères | Certification :</t>
         </is>
       </c>
       <c r="T37" s="7" t="inlineStr">
         <is>
-          <t>Type de validation : | Diplôme autres ministères | Certification : | CAP accompagnant éducatif petite enfance</t>
+          <t>Type de validation : | Diplôme autres ministères | Certification : | Titre professionnel agent de propreté et d'hygiène</t>
         </is>
       </c>
       <c r="U37" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/detail/11124191/true/false/true/true</t>
+          <t>https://candidat.francetravail.fr/formations/detail/10939638/true/false/false/false</t>
         </is>
       </c>
       <c r="V37" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-22&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-23&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W37" s="7" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-08-08
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1255,7 +1255,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1360,7 +1360,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1578,7 +1578,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1691,7 +1691,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-26&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-08-10
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-28&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W2" s="5" t="inlineStr">
@@ -827,7 +827,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="V3" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-28&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W3" s="7" t="inlineStr">
@@ -932,7 +932,7 @@
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="V4" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-28&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W4" s="5" t="inlineStr">
@@ -1037,7 +1037,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="V5" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-28&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W5" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1243,7 +1243,7 @@
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-28&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W6" s="5" t="inlineStr">
@@ -1255,7 +1255,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="V7" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-28&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W7" s="7" t="inlineStr">
@@ -1360,7 +1360,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
@@ -1453,7 +1453,7 @@
       </c>
       <c r="V8" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-28&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W8" s="5" t="inlineStr">
@@ -1465,7 +1465,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="V9" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-28&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W9" s="7" t="inlineStr">
@@ -1578,7 +1578,7 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-28&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W10" s="5" t="inlineStr">
@@ -1691,7 +1691,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -1792,7 +1792,7 @@
       </c>
       <c r="V11" s="7" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-27&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-28&amp;range=110-119&amp;tri=0</t>
         </is>
       </c>
       <c r="W11" s="7" t="inlineStr">

</xml_diff>

<commit_message>
🔪 Slice france_travail 2026-08-11
</commit_message>
<xml_diff>
--- a/exports/france_travail/francetravail_base.xlsx
+++ b/exports/france_travail/francetravail_base.xlsx
@@ -714,7 +714,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="V2" s="5" t="inlineStr">
         <is>
-          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationTerminee=formEnCours&amp;ou=DEPARTEMENT-28&amp;range=110-119&amp;tri=0</t>
+          <t>https://candidat.francetravail.fr/formations/recherche?filtreEstFormationEnCoursOuAVenir=formEnCours&amp;filtreEstFormationT